<commit_message>
Klinik-Kanal entfernt, alle Artikel in den Webkatalog
Die Klinik hat abgesagt, damit ist der Vertriebsweg "Klinik" gegenstandslos:

- Spalte Kanal bei allen 143 Zeilen geleert. Kanal ist der tatsaechliche
  Verkaufsweg und wird erst beim Verkauf gesetzt; das Rueckeinlesen aus
  WordPress traegt "Webkatalog" ein.
- Auswahlliste fuer Kanal: "Klinik" durch "Webkatalog" ersetzt.
- NU01-12 (Laeufer IKEA Morum) von Im_Katalog=nein auf ja - damit sind
  alle 88 aktiven Positionen im Webkatalog sichtbar.
- Im_Katalog ist jetzt die Wellen-Steuerung: ja = Moebel und grosse Deko
  (Welle 1), nein = Spielzeug und Konvolute (Welle 2). In SKILL.md
  entsprechend beschrieben.
- Artikelstamm, Muster-HTML und katalog_import.json neu erzeugt.

pruefen.py: 0 Fehler, 3 Hinweise.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011yyfqhuiWGsaNy38oaNoGo
</commit_message>
<xml_diff>
--- a/ausgabe/01_Artikelstamm_kikripp.xlsx
+++ b/ausgabe/01_Artikelstamm_kikripp.xlsx
@@ -1385,11 +1385,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z3" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z3" s="19" t="n"/>
       <c r="AA3" s="19" t="n"/>
       <c r="AB3" s="20" t="n"/>
       <c r="AC3" s="21">
@@ -1509,11 +1505,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z4" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z4" s="19" t="n"/>
       <c r="AA4" s="19" t="n"/>
       <c r="AB4" s="20" t="n"/>
       <c r="AC4" s="21">
@@ -1637,11 +1629,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z5" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z5" s="19" t="n"/>
       <c r="AA5" s="19" t="n"/>
       <c r="AB5" s="20" t="n"/>
       <c r="AC5" s="21">
@@ -1761,11 +1749,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z6" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z6" s="19" t="n"/>
       <c r="AA6" s="19" t="n"/>
       <c r="AB6" s="20" t="n"/>
       <c r="AC6" s="21">
@@ -1885,11 +1869,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z7" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z7" s="19" t="n"/>
       <c r="AA7" s="19" t="n"/>
       <c r="AB7" s="20" t="n"/>
       <c r="AC7" s="21">
@@ -2009,11 +1989,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z8" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z8" s="19" t="n"/>
       <c r="AA8" s="19" t="n"/>
       <c r="AB8" s="20" t="n"/>
       <c r="AC8" s="21">
@@ -2133,11 +2109,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z9" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z9" s="19" t="n"/>
       <c r="AA9" s="19" t="n"/>
       <c r="AB9" s="20" t="n"/>
       <c r="AC9" s="21">
@@ -2257,11 +2229,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z10" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z10" s="19" t="n"/>
       <c r="AA10" s="19" t="n"/>
       <c r="AB10" s="20" t="n"/>
       <c r="AC10" s="21">
@@ -2381,11 +2349,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z11" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z11" s="19" t="n"/>
       <c r="AA11" s="19" t="n"/>
       <c r="AB11" s="20" t="n"/>
       <c r="AC11" s="21">
@@ -2509,11 +2473,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z12" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z12" s="19" t="n"/>
       <c r="AA12" s="19" t="n"/>
       <c r="AB12" s="20" t="n"/>
       <c r="AC12" s="21">
@@ -2633,11 +2593,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z13" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z13" s="19" t="n"/>
       <c r="AA13" s="19" t="n"/>
       <c r="AB13" s="20" t="n"/>
       <c r="AC13" s="21">
@@ -2757,11 +2713,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z14" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z14" s="19" t="n"/>
       <c r="AA14" s="19" t="n"/>
       <c r="AB14" s="20" t="n"/>
       <c r="AC14" s="21">
@@ -2881,11 +2833,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z15" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z15" s="19" t="n"/>
       <c r="AA15" s="19" t="n"/>
       <c r="AB15" s="20" t="n"/>
       <c r="AC15" s="21">
@@ -3006,11 +2954,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z16" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z16" s="19" t="n"/>
       <c r="AA16" s="19" t="n"/>
       <c r="AB16" s="20" t="n"/>
       <c r="AC16" s="21">
@@ -3131,11 +3075,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z17" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z17" s="19" t="n"/>
       <c r="AA17" s="19" t="n"/>
       <c r="AB17" s="20" t="n"/>
       <c r="AC17" s="21">
@@ -3255,11 +3195,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z18" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z18" s="19" t="n"/>
       <c r="AA18" s="19" t="n"/>
       <c r="AB18" s="20" t="n"/>
       <c r="AC18" s="21">
@@ -3379,11 +3315,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z19" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z19" s="19" t="n"/>
       <c r="AA19" s="19" t="n"/>
       <c r="AB19" s="20" t="n"/>
       <c r="AC19" s="21">
@@ -3503,11 +3435,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z20" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z20" s="19" t="n"/>
       <c r="AA20" s="19" t="n"/>
       <c r="AB20" s="20" t="n"/>
       <c r="AC20" s="21">
@@ -3627,11 +3555,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z21" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z21" s="19" t="n"/>
       <c r="AA21" s="19" t="n"/>
       <c r="AB21" s="20" t="n"/>
       <c r="AC21" s="21">
@@ -3751,11 +3675,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z22" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z22" s="19" t="n"/>
       <c r="AA22" s="19" t="n"/>
       <c r="AB22" s="20" t="n"/>
       <c r="AC22" s="21">
@@ -3875,11 +3795,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z23" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z23" s="19" t="n"/>
       <c r="AA23" s="19" t="n"/>
       <c r="AB23" s="20" t="n"/>
       <c r="AC23" s="21">
@@ -3999,11 +3915,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z24" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z24" s="19" t="n"/>
       <c r="AA24" s="19" t="n"/>
       <c r="AB24" s="20" t="n"/>
       <c r="AC24" s="21">
@@ -4123,11 +4035,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z25" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z25" s="19" t="n"/>
       <c r="AA25" s="19" t="n"/>
       <c r="AB25" s="20" t="n"/>
       <c r="AC25" s="21">
@@ -4247,11 +4155,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z26" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z26" s="19" t="n"/>
       <c r="AA26" s="19" t="n"/>
       <c r="AB26" s="20" t="n"/>
       <c r="AC26" s="21">
@@ -4371,11 +4275,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z27" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z27" s="19" t="n"/>
       <c r="AA27" s="19" t="n"/>
       <c r="AB27" s="20" t="n"/>
       <c r="AC27" s="21">
@@ -4495,11 +4395,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z28" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z28" s="19" t="n"/>
       <c r="AA28" s="19" t="n"/>
       <c r="AB28" s="20" t="n"/>
       <c r="AC28" s="21">
@@ -4619,11 +4515,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z29" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z29" s="19" t="n"/>
       <c r="AA29" s="19" t="n"/>
       <c r="AB29" s="20" t="n"/>
       <c r="AC29" s="21">
@@ -4743,11 +4635,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z30" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z30" s="19" t="n"/>
       <c r="AA30" s="19" t="n"/>
       <c r="AB30" s="20" t="n"/>
       <c r="AC30" s="21">
@@ -4867,11 +4755,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z31" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z31" s="19" t="n"/>
       <c r="AA31" s="19" t="n"/>
       <c r="AB31" s="20" t="n"/>
       <c r="AC31" s="21">
@@ -4991,11 +4875,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z32" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z32" s="19" t="n"/>
       <c r="AA32" s="19" t="n"/>
       <c r="AB32" s="20" t="n"/>
       <c r="AC32" s="21">
@@ -5115,11 +4995,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z33" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z33" s="19" t="n"/>
       <c r="AA33" s="19" t="n"/>
       <c r="AB33" s="20" t="n"/>
       <c r="AC33" s="21">
@@ -5239,11 +5115,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z34" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z34" s="19" t="n"/>
       <c r="AA34" s="19" t="n"/>
       <c r="AB34" s="20" t="n"/>
       <c r="AC34" s="21">
@@ -5363,11 +5235,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z35" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z35" s="19" t="n"/>
       <c r="AA35" s="19" t="n"/>
       <c r="AB35" s="20" t="n"/>
       <c r="AC35" s="21">
@@ -5487,11 +5355,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z36" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z36" s="19" t="n"/>
       <c r="AA36" s="19" t="n"/>
       <c r="AB36" s="20" t="n"/>
       <c r="AC36" s="21">
@@ -5611,11 +5475,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z37" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z37" s="19" t="n"/>
       <c r="AA37" s="19" t="n"/>
       <c r="AB37" s="20" t="n"/>
       <c r="AC37" s="21">
@@ -5735,11 +5595,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z38" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z38" s="19" t="n"/>
       <c r="AA38" s="19" t="n"/>
       <c r="AB38" s="20" t="n"/>
       <c r="AC38" s="21">
@@ -5859,11 +5715,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z39" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z39" s="19" t="n"/>
       <c r="AA39" s="19" t="n"/>
       <c r="AB39" s="20" t="n"/>
       <c r="AC39" s="21">
@@ -5983,11 +5835,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z40" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z40" s="19" t="n"/>
       <c r="AA40" s="19" t="n"/>
       <c r="AB40" s="20" t="n"/>
       <c r="AC40" s="21">
@@ -6103,11 +5951,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z41" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z41" s="19" t="n"/>
       <c r="AA41" s="19" t="n"/>
       <c r="AB41" s="20" t="n"/>
       <c r="AC41" s="21">
@@ -6223,11 +6067,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z42" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z42" s="19" t="n"/>
       <c r="AA42" s="19" t="n"/>
       <c r="AB42" s="20" t="n"/>
       <c r="AC42" s="21">
@@ -6343,11 +6183,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z43" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z43" s="19" t="n"/>
       <c r="AA43" s="19" t="n"/>
       <c r="AB43" s="20" t="n"/>
       <c r="AC43" s="21">
@@ -6463,11 +6299,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z44" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z44" s="19" t="n"/>
       <c r="AA44" s="19" t="n"/>
       <c r="AB44" s="20" t="n"/>
       <c r="AC44" s="21">
@@ -6583,11 +6415,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z45" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z45" s="19" t="n"/>
       <c r="AA45" s="19" t="n"/>
       <c r="AB45" s="20" t="n"/>
       <c r="AC45" s="21">
@@ -6703,11 +6531,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z46" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z46" s="19" t="n"/>
       <c r="AA46" s="19" t="n"/>
       <c r="AB46" s="20" t="n"/>
       <c r="AC46" s="21">
@@ -6823,11 +6647,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z47" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z47" s="19" t="n"/>
       <c r="AA47" s="19" t="n"/>
       <c r="AB47" s="20" t="n"/>
       <c r="AC47" s="21">
@@ -6943,11 +6763,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z48" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z48" s="19" t="n"/>
       <c r="AA48" s="19" t="n"/>
       <c r="AB48" s="20" t="n"/>
       <c r="AC48" s="21">
@@ -7063,11 +6879,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z49" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z49" s="19" t="n"/>
       <c r="AA49" s="19" t="n"/>
       <c r="AB49" s="20" t="n"/>
       <c r="AC49" s="21">
@@ -7183,11 +6995,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z50" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z50" s="19" t="n"/>
       <c r="AA50" s="19" t="n"/>
       <c r="AB50" s="20" t="n"/>
       <c r="AC50" s="21">
@@ -7303,11 +7111,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z51" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z51" s="19" t="n"/>
       <c r="AA51" s="19" t="n"/>
       <c r="AB51" s="20" t="n"/>
       <c r="AC51" s="21">
@@ -7423,11 +7227,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z52" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z52" s="19" t="n"/>
       <c r="AA52" s="19" t="n"/>
       <c r="AB52" s="20" t="n"/>
       <c r="AC52" s="21">
@@ -7543,11 +7343,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z53" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z53" s="19" t="n"/>
       <c r="AA53" s="19" t="n"/>
       <c r="AB53" s="20" t="n"/>
       <c r="AC53" s="21">
@@ -7663,11 +7459,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z54" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z54" s="19" t="n"/>
       <c r="AA54" s="19" t="n"/>
       <c r="AB54" s="20" t="n"/>
       <c r="AC54" s="21">
@@ -7783,11 +7575,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z55" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z55" s="19" t="n"/>
       <c r="AA55" s="19" t="n"/>
       <c r="AB55" s="20" t="n"/>
       <c r="AC55" s="21">
@@ -7903,11 +7691,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z56" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z56" s="19" t="n"/>
       <c r="AA56" s="19" t="n"/>
       <c r="AB56" s="20" t="n"/>
       <c r="AC56" s="21">
@@ -8023,11 +7807,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z57" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z57" s="19" t="n"/>
       <c r="AA57" s="19" t="n"/>
       <c r="AB57" s="20" t="n"/>
       <c r="AC57" s="21">
@@ -8143,11 +7923,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z58" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z58" s="19" t="n"/>
       <c r="AA58" s="19" t="n"/>
       <c r="AB58" s="20" t="n"/>
       <c r="AC58" s="21">
@@ -8263,11 +8039,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z59" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z59" s="19" t="n"/>
       <c r="AA59" s="19" t="n"/>
       <c r="AB59" s="20" t="n"/>
       <c r="AC59" s="21">
@@ -8383,11 +8155,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z60" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z60" s="19" t="n"/>
       <c r="AA60" s="19" t="n"/>
       <c r="AB60" s="20" t="n"/>
       <c r="AC60" s="21">
@@ -8503,11 +8271,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z61" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z61" s="19" t="n"/>
       <c r="AA61" s="19" t="n"/>
       <c r="AB61" s="20" t="n"/>
       <c r="AC61" s="21">
@@ -8623,11 +8387,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z62" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z62" s="19" t="n"/>
       <c r="AA62" s="19" t="n"/>
       <c r="AB62" s="20" t="n"/>
       <c r="AC62" s="21">
@@ -8743,11 +8503,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z63" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z63" s="19" t="n"/>
       <c r="AA63" s="19" t="n"/>
       <c r="AB63" s="20" t="n"/>
       <c r="AC63" s="21">
@@ -8863,11 +8619,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z64" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z64" s="19" t="n"/>
       <c r="AA64" s="19" t="n"/>
       <c r="AB64" s="20" t="n"/>
       <c r="AC64" s="21">
@@ -8983,11 +8735,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z65" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z65" s="19" t="n"/>
       <c r="AA65" s="19" t="n"/>
       <c r="AB65" s="20" t="n"/>
       <c r="AC65" s="21">
@@ -9103,11 +8851,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z66" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z66" s="19" t="n"/>
       <c r="AA66" s="19" t="n"/>
       <c r="AB66" s="20" t="n"/>
       <c r="AC66" s="21">
@@ -9223,11 +8967,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z67" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z67" s="19" t="n"/>
       <c r="AA67" s="19" t="n"/>
       <c r="AB67" s="20" t="n"/>
       <c r="AC67" s="21">
@@ -9343,11 +9083,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z68" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z68" s="19" t="n"/>
       <c r="AA68" s="19" t="n"/>
       <c r="AB68" s="20" t="n"/>
       <c r="AC68" s="21">
@@ -9463,11 +9199,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z69" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z69" s="19" t="n"/>
       <c r="AA69" s="19" t="n"/>
       <c r="AB69" s="20" t="n"/>
       <c r="AC69" s="21">
@@ -9583,11 +9315,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z70" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z70" s="19" t="n"/>
       <c r="AA70" s="19" t="n"/>
       <c r="AB70" s="20" t="n"/>
       <c r="AC70" s="21">
@@ -9703,11 +9431,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z71" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z71" s="19" t="n"/>
       <c r="AA71" s="19" t="n"/>
       <c r="AB71" s="20" t="n"/>
       <c r="AC71" s="21">
@@ -9823,11 +9547,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z72" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z72" s="19" t="n"/>
       <c r="AA72" s="19" t="n"/>
       <c r="AB72" s="20" t="n"/>
       <c r="AC72" s="21">
@@ -9943,11 +9663,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z73" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z73" s="19" t="n"/>
       <c r="AA73" s="19" t="n"/>
       <c r="AB73" s="20" t="n"/>
       <c r="AC73" s="21">
@@ -10063,11 +9779,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z74" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z74" s="19" t="n"/>
       <c r="AA74" s="19" t="n"/>
       <c r="AB74" s="20" t="n"/>
       <c r="AC74" s="21">
@@ -10183,11 +9895,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z75" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z75" s="19" t="n"/>
       <c r="AA75" s="19" t="n"/>
       <c r="AB75" s="20" t="n"/>
       <c r="AC75" s="21">
@@ -10303,11 +10011,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z76" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z76" s="19" t="n"/>
       <c r="AA76" s="19" t="n"/>
       <c r="AB76" s="20" t="n"/>
       <c r="AC76" s="21">
@@ -10423,11 +10127,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z77" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z77" s="19" t="n"/>
       <c r="AA77" s="19" t="n"/>
       <c r="AB77" s="20" t="n"/>
       <c r="AC77" s="21">
@@ -10543,11 +10243,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z78" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z78" s="19" t="n"/>
       <c r="AA78" s="19" t="n"/>
       <c r="AB78" s="20" t="n"/>
       <c r="AC78" s="21">
@@ -10663,11 +10359,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z79" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z79" s="19" t="n"/>
       <c r="AA79" s="19" t="n"/>
       <c r="AB79" s="20" t="n"/>
       <c r="AC79" s="21">
@@ -10783,11 +10475,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z80" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z80" s="19" t="n"/>
       <c r="AA80" s="19" t="n"/>
       <c r="AB80" s="20" t="n"/>
       <c r="AC80" s="21">
@@ -10903,11 +10591,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z81" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z81" s="19" t="n"/>
       <c r="AA81" s="19" t="n"/>
       <c r="AB81" s="20" t="n"/>
       <c r="AC81" s="21">
@@ -11023,11 +10707,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z82" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z82" s="19" t="n"/>
       <c r="AA82" s="19" t="n"/>
       <c r="AB82" s="20" t="n"/>
       <c r="AC82" s="21">
@@ -11143,11 +10823,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z83" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z83" s="19" t="n"/>
       <c r="AA83" s="19" t="n"/>
       <c r="AB83" s="20" t="n"/>
       <c r="AC83" s="21">
@@ -11263,11 +10939,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z84" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z84" s="19" t="n"/>
       <c r="AA84" s="19" t="n"/>
       <c r="AB84" s="20" t="n"/>
       <c r="AC84" s="21">
@@ -11383,11 +11055,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z85" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z85" s="19" t="n"/>
       <c r="AA85" s="19" t="n"/>
       <c r="AB85" s="20" t="n"/>
       <c r="AC85" s="21">
@@ -11503,11 +11171,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z86" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z86" s="19" t="n"/>
       <c r="AA86" s="19" t="n"/>
       <c r="AB86" s="20" t="n"/>
       <c r="AC86" s="21">
@@ -11623,11 +11287,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z87" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z87" s="19" t="n"/>
       <c r="AA87" s="19" t="n"/>
       <c r="AB87" s="20" t="n"/>
       <c r="AC87" s="21">
@@ -11743,11 +11403,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z88" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z88" s="19" t="n"/>
       <c r="AA88" s="19" t="n"/>
       <c r="AB88" s="20" t="n"/>
       <c r="AC88" s="21">
@@ -11863,11 +11519,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z89" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z89" s="19" t="n"/>
       <c r="AA89" s="19" t="n"/>
       <c r="AB89" s="20" t="n"/>
       <c r="AC89" s="21">
@@ -11983,11 +11635,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z90" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z90" s="19" t="n"/>
       <c r="AA90" s="19" t="n"/>
       <c r="AB90" s="20" t="n"/>
       <c r="AC90" s="21">
@@ -12103,11 +11751,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z91" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z91" s="19" t="n"/>
       <c r="AA91" s="19" t="n"/>
       <c r="AB91" s="20" t="n"/>
       <c r="AC91" s="21">
@@ -12223,11 +11867,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z92" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z92" s="19" t="n"/>
       <c r="AA92" s="19" t="n"/>
       <c r="AB92" s="20" t="n"/>
       <c r="AC92" s="21">
@@ -12343,11 +11983,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z93" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z93" s="19" t="n"/>
       <c r="AA93" s="19" t="n"/>
       <c r="AB93" s="20" t="n"/>
       <c r="AC93" s="21">
@@ -12463,11 +12099,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z94" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z94" s="19" t="n"/>
       <c r="AA94" s="19" t="n"/>
       <c r="AB94" s="20" t="n"/>
       <c r="AC94" s="21">
@@ -12583,11 +12215,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z95" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z95" s="19" t="n"/>
       <c r="AA95" s="19" t="n"/>
       <c r="AB95" s="20" t="n"/>
       <c r="AC95" s="21">
@@ -12707,11 +12335,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z96" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z96" s="19" t="n"/>
       <c r="AA96" s="19" t="n"/>
       <c r="AB96" s="20" t="n"/>
       <c r="AC96" s="21">
@@ -12835,11 +12459,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z97" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z97" s="19" t="n"/>
       <c r="AA97" s="19" t="n"/>
       <c r="AB97" s="20" t="n"/>
       <c r="AC97" s="21">
@@ -12963,11 +12583,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z98" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z98" s="19" t="n"/>
       <c r="AA98" s="19" t="n"/>
       <c r="AB98" s="20" t="n"/>
       <c r="AC98" s="21">
@@ -13087,11 +12703,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z99" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z99" s="19" t="n"/>
       <c r="AA99" s="19" t="n"/>
       <c r="AB99" s="20" t="n"/>
       <c r="AC99" s="21">
@@ -13211,11 +12823,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z100" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z100" s="19" t="n"/>
       <c r="AA100" s="19" t="n"/>
       <c r="AB100" s="20" t="n"/>
       <c r="AC100" s="21">
@@ -13335,11 +12943,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z101" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z101" s="19" t="n"/>
       <c r="AA101" s="19" t="n"/>
       <c r="AB101" s="20" t="n"/>
       <c r="AC101" s="21">
@@ -13459,11 +13063,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z102" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z102" s="19" t="n"/>
       <c r="AA102" s="19" t="n"/>
       <c r="AB102" s="20" t="n"/>
       <c r="AC102" s="21">
@@ -13583,11 +13183,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z103" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z103" s="19" t="n"/>
       <c r="AA103" s="19" t="n"/>
       <c r="AB103" s="20" t="n"/>
       <c r="AC103" s="21">
@@ -13707,11 +13303,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z104" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z104" s="19" t="n"/>
       <c r="AA104" s="19" t="n"/>
       <c r="AB104" s="20" t="n"/>
       <c r="AC104" s="21">
@@ -13831,11 +13423,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z105" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z105" s="19" t="n"/>
       <c r="AA105" s="19" t="n"/>
       <c r="AB105" s="20" t="n"/>
       <c r="AC105" s="21">
@@ -13955,11 +13543,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z106" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z106" s="19" t="n"/>
       <c r="AA106" s="19" t="n"/>
       <c r="AB106" s="20" t="n"/>
       <c r="AC106" s="21">
@@ -14079,11 +13663,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z107" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z107" s="19" t="n"/>
       <c r="AA107" s="19" t="n"/>
       <c r="AB107" s="20" t="n"/>
       <c r="AC107" s="21">
@@ -14203,11 +13783,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z108" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z108" s="19" t="n"/>
       <c r="AA108" s="19" t="n"/>
       <c r="AB108" s="20" t="n"/>
       <c r="AC108" s="21">
@@ -14327,11 +13903,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z109" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z109" s="19" t="n"/>
       <c r="AA109" s="19" t="n"/>
       <c r="AB109" s="20" t="n"/>
       <c r="AC109" s="21">
@@ -14451,11 +14023,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z110" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z110" s="19" t="n"/>
       <c r="AA110" s="19" t="n"/>
       <c r="AB110" s="20" t="n"/>
       <c r="AC110" s="21">
@@ -14575,11 +14143,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z111" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z111" s="19" t="n"/>
       <c r="AA111" s="19" t="n"/>
       <c r="AB111" s="20" t="n"/>
       <c r="AC111" s="21">
@@ -14699,11 +14263,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z112" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z112" s="19" t="n"/>
       <c r="AA112" s="19" t="n"/>
       <c r="AB112" s="20" t="n"/>
       <c r="AC112" s="21">
@@ -14823,11 +14383,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z113" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z113" s="19" t="n"/>
       <c r="AA113" s="19" t="n"/>
       <c r="AB113" s="20" t="n"/>
       <c r="AC113" s="21">
@@ -14947,11 +14503,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z114" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z114" s="19" t="n"/>
       <c r="AA114" s="19" t="n"/>
       <c r="AB114" s="20" t="n"/>
       <c r="AC114" s="21">
@@ -15071,11 +14623,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z115" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z115" s="19" t="n"/>
       <c r="AA115" s="19" t="n"/>
       <c r="AB115" s="20" t="n"/>
       <c r="AC115" s="21">
@@ -15195,11 +14743,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z116" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z116" s="19" t="n"/>
       <c r="AA116" s="19" t="n"/>
       <c r="AB116" s="20" t="n"/>
       <c r="AC116" s="21">
@@ -15323,11 +14867,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z117" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z117" s="19" t="n"/>
       <c r="AA117" s="19" t="n"/>
       <c r="AB117" s="20" t="n"/>
       <c r="AC117" s="21">
@@ -15447,11 +14987,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z118" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z118" s="19" t="n"/>
       <c r="AA118" s="19" t="n"/>
       <c r="AB118" s="20" t="n"/>
       <c r="AC118" s="21">
@@ -15571,11 +15107,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z119" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z119" s="19" t="n"/>
       <c r="AA119" s="19" t="n"/>
       <c r="AB119" s="20" t="n"/>
       <c r="AC119" s="21">
@@ -15695,11 +15227,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z120" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z120" s="19" t="n"/>
       <c r="AA120" s="19" t="n"/>
       <c r="AB120" s="20" t="n"/>
       <c r="AC120" s="21">
@@ -15823,11 +15351,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z121" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z121" s="19" t="n"/>
       <c r="AA121" s="19" t="n"/>
       <c r="AB121" s="20" t="n"/>
       <c r="AC121" s="21">
@@ -15951,11 +15475,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z122" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z122" s="19" t="n"/>
       <c r="AA122" s="19" t="n"/>
       <c r="AB122" s="20" t="n"/>
       <c r="AC122" s="21">
@@ -16079,11 +15599,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z123" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z123" s="19" t="n"/>
       <c r="AA123" s="19" t="n"/>
       <c r="AB123" s="20" t="n"/>
       <c r="AC123" s="21">
@@ -16203,11 +15719,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z124" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z124" s="19" t="n"/>
       <c r="AA124" s="19" t="n"/>
       <c r="AB124" s="20" t="n"/>
       <c r="AC124" s="21">
@@ -16327,11 +15839,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z125" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z125" s="19" t="n"/>
       <c r="AA125" s="19" t="n"/>
       <c r="AB125" s="20" t="n"/>
       <c r="AC125" s="21">
@@ -16434,7 +15942,7 @@
       <c r="V126" s="15" t="n"/>
       <c r="W126" s="19" t="inlineStr">
         <is>
-          <t>nein</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="X126" s="19" t="n"/>
@@ -16443,11 +15951,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z126" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z126" s="19" t="n"/>
       <c r="AA126" s="19" t="n"/>
       <c r="AB126" s="20" t="n"/>
       <c r="AC126" s="21">
@@ -16571,11 +16075,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z127" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z127" s="19" t="n"/>
       <c r="AA127" s="19" t="n"/>
       <c r="AB127" s="20" t="n"/>
       <c r="AC127" s="21">
@@ -16695,11 +16195,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z128" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z128" s="19" t="n"/>
       <c r="AA128" s="19" t="n"/>
       <c r="AB128" s="20" t="n"/>
       <c r="AC128" s="21">
@@ -16819,11 +16315,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z129" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z129" s="19" t="n"/>
       <c r="AA129" s="19" t="n"/>
       <c r="AB129" s="20" t="n"/>
       <c r="AC129" s="21">
@@ -16943,11 +16435,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z130" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z130" s="19" t="n"/>
       <c r="AA130" s="19" t="n"/>
       <c r="AB130" s="20" t="n"/>
       <c r="AC130" s="21">
@@ -17067,11 +16555,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z131" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z131" s="19" t="n"/>
       <c r="AA131" s="19" t="n"/>
       <c r="AB131" s="20" t="n"/>
       <c r="AC131" s="21">
@@ -17191,11 +16675,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z132" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z132" s="19" t="n"/>
       <c r="AA132" s="19" t="n"/>
       <c r="AB132" s="20" t="n"/>
       <c r="AC132" s="21">
@@ -17315,11 +16795,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z133" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z133" s="19" t="n"/>
       <c r="AA133" s="19" t="n"/>
       <c r="AB133" s="20" t="n"/>
       <c r="AC133" s="21">
@@ -17439,11 +16915,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z134" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z134" s="19" t="n"/>
       <c r="AA134" s="19" t="n"/>
       <c r="AB134" s="20" t="n"/>
       <c r="AC134" s="21">
@@ -17564,11 +17036,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z135" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z135" s="19" t="n"/>
       <c r="AA135" s="19" t="n"/>
       <c r="AB135" s="20" t="n"/>
       <c r="AC135" s="21">
@@ -17688,11 +17156,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z136" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z136" s="19" t="n"/>
       <c r="AA136" s="19" t="n"/>
       <c r="AB136" s="20" t="n"/>
       <c r="AC136" s="21">
@@ -17812,11 +17276,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z137" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z137" s="19" t="n"/>
       <c r="AA137" s="19" t="n"/>
       <c r="AB137" s="20" t="n"/>
       <c r="AC137" s="21">
@@ -17940,11 +17400,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z138" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z138" s="19" t="n"/>
       <c r="AA138" s="19" t="n"/>
       <c r="AB138" s="20" t="n"/>
       <c r="AC138" s="21">
@@ -18064,11 +17520,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z139" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z139" s="19" t="n"/>
       <c r="AA139" s="19" t="n"/>
       <c r="AB139" s="20" t="n"/>
       <c r="AC139" s="21">
@@ -18188,11 +17640,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z140" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z140" s="19" t="n"/>
       <c r="AA140" s="19" t="n"/>
       <c r="AB140" s="20" t="n"/>
       <c r="AC140" s="21">
@@ -18312,11 +17760,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z141" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z141" s="19" t="n"/>
       <c r="AA141" s="19" t="n"/>
       <c r="AB141" s="20" t="n"/>
       <c r="AC141" s="21">
@@ -18436,11 +17880,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z142" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z142" s="19" t="n"/>
       <c r="AA142" s="19" t="n"/>
       <c r="AB142" s="20" t="n"/>
       <c r="AC142" s="21">
@@ -18560,11 +18000,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z143" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z143" s="19" t="n"/>
       <c r="AA143" s="19" t="n"/>
       <c r="AB143" s="20" t="n"/>
       <c r="AC143" s="21">
@@ -18684,11 +18120,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z144" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z144" s="19" t="n"/>
       <c r="AA144" s="19" t="n"/>
       <c r="AB144" s="20" t="n"/>
       <c r="AC144" s="21">
@@ -18808,11 +18240,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="Z145" s="19" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
+      <c r="Z145" s="19" t="n"/>
       <c r="AA145" s="19" t="n"/>
       <c r="AB145" s="20" t="n"/>
       <c r="AC145" s="21">
@@ -18893,7 +18321,7 @@
       <formula1>"verfügbar,reserviert,teilverkauft,verkauft,gespendet,entsorgt"</formula1>
     </dataValidation>
     <dataValidation sqref="Z3:Z803" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Klinik,Kleinanzeigen,eBay,Direkt,Händler,Verkaufstag"</formula1>
+      <formula1>"Webkatalog,Kleinanzeigen,eBay,Direkt,Händler,Verkaufstag"</formula1>
     </dataValidation>
     <dataValidation sqref="AG3:AG803" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"offen,bezahlt,teilbezahlt"</formula1>

</xml_diff>

<commit_message>
Rattankoerbe zurueck auf 10 EUR, Zustand stark gebraucht
Nutzerin korrigiert: die acht Koerbe sind stark gebraucht, der Preis war
richtig. Zustand entsprechend berichtigt (stand als "gebraucht" in den
Daten) und Wertklasse auf C, wohin 10 EUR gehoeren.

Gesamtwert netto 23.453 EUR. pruefen.py: 0 Fehler, 2 Hinweise.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011yyfqhuiWGsaNy38oaNoGo
</commit_message>
<xml_diff>
--- a/ausgabe/01_Artikelstamm_kikripp.xlsx
+++ b/ausgabe/01_Artikelstamm_kikripp.xlsx
@@ -1329,7 +1329,7 @@
       </c>
       <c r="H3" s="15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="I3" s="17" t="n">
@@ -1347,7 +1347,7 @@
       </c>
       <c r="M3" s="15" t="inlineStr">
         <is>
-          <t>gebraucht</t>
+          <t>stark gebraucht</t>
         </is>
       </c>
       <c r="N3" s="19" t="n"/>
@@ -1359,7 +1359,7 @@
       <c r="P3" s="19" t="n"/>
       <c r="Q3" s="20" t="n"/>
       <c r="R3" s="20" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="S3" s="19" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
NE01 erfasst: 10 Positionen, Neubau EG begonnen
Flur (Neubau EG, 7,25 m2), Blatt und alle Fotos lagen vor. Der Raum hatte
schon 16 Positionen aus der alten Erfassung; dazu kommen NE01-17 bis -26.

Groesste Posten: 12 Wandregale mit Wannen (420 EUR), 7 lange Sitzbaenke
mit Stauraum (315 EUR) und 32 Hundehaken in zwei Farben (192 EUR). Die
Sitzbaenke sind laut Erfassungsblatt stark gebraucht - Lack grossflaechig
zerkratzt, das steht so in den Beschreibungen.

NE01-15 (Deko-Tannenbaum schwarz) war auf dem Blatt durchgestrichen und
steht jetzt auf Aktiv=entfaellt.

Die beiden Wesco-Kuechen sind laut Nutzerin nicht baugleich und bleiben
getrennt; die Verweise aufeinander bleiben in den Mengenhinweisen.

Gesamtwert netto 34.140 -> 35.557 EUR, 173 aktive Positionen.
pruefen.py: 0 Fehler, 3 Hinweise.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011yyfqhuiWGsaNy38oaNoGo
</commit_message>
<xml_diff>
--- a/ausgabe/01_Artikelstamm_kikripp.xlsx
+++ b/ausgabe/01_Artikelstamm_kikripp.xlsx
@@ -15,7 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Artikelstamm'!$A$2:$AM$221</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Artikelstamm'!$A$2:$AM$231</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1019,7 +1019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AM221"/>
+  <dimension ref="A1:AM231"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -14248,7 +14248,7 @@
       <c r="O110" s="19" t="n"/>
       <c r="P110" s="19" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>entfällt</t>
         </is>
       </c>
       <c r="Q110" s="19" t="n"/>
@@ -14305,7 +14305,11 @@
           <t>3 Stück im Bild</t>
         </is>
       </c>
-      <c r="AM110" s="22" t="n"/>
+      <c r="AM110" s="22" t="inlineStr">
+        <is>
+          <t>Auf dem Erfassungsblatt NE01 durchgestrichen – entfaellt.</t>
+        </is>
+      </c>
     </row>
     <row r="111" ht="30" customHeight="1">
       <c r="A111" s="15" t="inlineStr">
@@ -22591,7 +22595,7 @@
       <c r="AK178" s="19" t="n"/>
       <c r="AL178" s="16" t="inlineStr">
         <is>
-          <t>1 Küche aus 5 Modulen, vom Haus bestätigt. Eine zweite Wesco-Küche steht unter NU07-03.</t>
+          <t>1 Küche aus 5 Modulen, vom Haus bestätigt. Eine zweite, anders zusammengesetzte Wesco-Küche steht unter NU07-03.</t>
         </is>
       </c>
       <c r="AM178" s="22" t="inlineStr">
@@ -27285,12 +27289,12 @@
       <c r="AK217" s="19" t="n"/>
       <c r="AL217" s="16" t="inlineStr">
         <is>
-          <t>1 Küche aus mehreren Modulen. Eine zweite Wesco-Küche steht unter NU03-03.</t>
+          <t>1 Küche aus mehreren Modulen, mit Mikrowellenmodul und Hängeschrank. Eine zweite, anders zusammengesetzte Wesco-Küche steht unter NU03-03.</t>
         </is>
       </c>
       <c r="AM217" s="22" t="inlineStr">
         <is>
-          <t>Zu klaeren: ist diese Kueche baugleich mit NU03-03? Wenn ja, zu einer Position mit 2 Stueck zusammenfassen. Modulzahl hier noch nicht gezaehlt.</t>
+          <t>Nicht baugleich mit NU03-03, vom Haus bestaetigt – bleibt getrennt.</t>
         </is>
       </c>
     </row>
@@ -27770,8 +27774,1188 @@
       </c>
       <c r="AM221" s="22" t="n"/>
     </row>
+    <row r="222" ht="30" customHeight="1">
+      <c r="A222" s="15" t="inlineStr">
+        <is>
+          <t>NE01-17</t>
+        </is>
+      </c>
+      <c r="B222" s="15" t="n"/>
+      <c r="C222" s="15" t="n"/>
+      <c r="D222" s="15" t="inlineStr">
+        <is>
+          <t>NE01</t>
+        </is>
+      </c>
+      <c r="E222" s="15" t="inlineStr">
+        <is>
+          <t>Wandregal Berg, grau mit Holzablagen</t>
+        </is>
+      </c>
+      <c r="F222" s="16" t="inlineStr">
+        <is>
+          <t>Wandregal in Bergform, grau lackiert mit gelber Gipfellinie, mit mehreren Ablagebrettern aus Buche. Im Haus als Regal für Hörfiguren genutzt.</t>
+        </is>
+      </c>
+      <c r="G222" s="15" t="inlineStr">
+        <is>
+          <t>Möbel</t>
+        </is>
+      </c>
+      <c r="H222" s="15" t="inlineStr">
+        <is>
+          <t>Flur</t>
+        </is>
+      </c>
+      <c r="I222" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J222" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K222" s="17" t="n"/>
+      <c r="L222" s="18">
+        <f>J222-IF(K222="",0,K222)</f>
+        <v/>
+      </c>
+      <c r="M222" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N222" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O222" s="19" t="n"/>
+      <c r="P222" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q222" s="19" t="n"/>
+      <c r="R222" s="20" t="n"/>
+      <c r="S222" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="T222" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U222" s="21">
+        <f>L222*S222</f>
+        <v/>
+      </c>
+      <c r="V222" s="15" t="inlineStr">
+        <is>
+          <t>Versand möglich</t>
+        </is>
+      </c>
+      <c r="W222" s="15" t="inlineStr">
+        <is>
+          <t>F-246</t>
+        </is>
+      </c>
+      <c r="X222" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y222" s="19" t="n"/>
+      <c r="Z222" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA222" s="19" t="n"/>
+      <c r="AB222" s="19" t="n"/>
+      <c r="AC222" s="19" t="n"/>
+      <c r="AD222" s="20" t="n"/>
+      <c r="AE222" s="21">
+        <f>IF(K222="","",K222*AD222)</f>
+        <v/>
+      </c>
+      <c r="AF222" s="19" t="n"/>
+      <c r="AG222" s="19" t="n"/>
+      <c r="AH222" s="19" t="n"/>
+      <c r="AI222" s="19" t="n"/>
+      <c r="AJ222" s="19" t="n"/>
+      <c r="AK222" s="19" t="n"/>
+      <c r="AL222" s="16" t="inlineStr">
+        <is>
+          <t>2 Regale, beide abgebildet. Figuren und Abspielgerät gehören nicht dazu.</t>
+        </is>
+      </c>
+      <c r="AM222" s="22" t="n"/>
+    </row>
+    <row r="223" ht="30" customHeight="1">
+      <c r="A223" s="15" t="inlineStr">
+        <is>
+          <t>NE01-18</t>
+        </is>
+      </c>
+      <c r="B223" s="15" t="n"/>
+      <c r="C223" s="15" t="n"/>
+      <c r="D223" s="15" t="inlineStr">
+        <is>
+          <t>NE01</t>
+        </is>
+      </c>
+      <c r="E223" s="15" t="inlineStr">
+        <is>
+          <t>Highboard weiß auf schwarzem Metallgestell</t>
+        </is>
+      </c>
+      <c r="F223" s="16" t="inlineStr">
+        <is>
+          <t>Highboard mit weißen Fronten: zwei Türen oben, zwei breite Schubladen unten, flache schwarze Griffleisten, auf einem schwarzen Metallkufengestell.</t>
+        </is>
+      </c>
+      <c r="G223" s="15" t="inlineStr">
+        <is>
+          <t>Möbel</t>
+        </is>
+      </c>
+      <c r="H223" s="15" t="inlineStr">
+        <is>
+          <t>Flur</t>
+        </is>
+      </c>
+      <c r="I223" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J223" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K223" s="17" t="n"/>
+      <c r="L223" s="18">
+        <f>J223-IF(K223="",0,K223)</f>
+        <v/>
+      </c>
+      <c r="M223" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N223" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O223" s="19" t="n"/>
+      <c r="P223" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q223" s="19" t="n"/>
+      <c r="R223" s="20" t="n"/>
+      <c r="S223" s="20" t="n">
+        <v>150</v>
+      </c>
+      <c r="T223" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U223" s="21">
+        <f>L223*S223</f>
+        <v/>
+      </c>
+      <c r="V223" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W223" s="15" t="inlineStr">
+        <is>
+          <t>F-247</t>
+        </is>
+      </c>
+      <c r="X223" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y223" s="19" t="n"/>
+      <c r="Z223" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA223" s="19" t="n"/>
+      <c r="AB223" s="19" t="n"/>
+      <c r="AC223" s="19" t="n"/>
+      <c r="AD223" s="20" t="n"/>
+      <c r="AE223" s="21">
+        <f>IF(K223="","",K223*AD223)</f>
+        <v/>
+      </c>
+      <c r="AF223" s="19" t="n"/>
+      <c r="AG223" s="19" t="n"/>
+      <c r="AH223" s="19" t="n"/>
+      <c r="AI223" s="19" t="n"/>
+      <c r="AJ223" s="19" t="n"/>
+      <c r="AK223" s="19" t="n"/>
+      <c r="AL223" s="16" t="inlineStr">
+        <is>
+          <t>1 Highboard.</t>
+        </is>
+      </c>
+      <c r="AM223" s="22" t="n"/>
+    </row>
+    <row r="224" ht="30" customHeight="1">
+      <c r="A224" s="15" t="inlineStr">
+        <is>
+          <t>NE01-19</t>
+        </is>
+      </c>
+      <c r="B224" s="15" t="n"/>
+      <c r="C224" s="15" t="n"/>
+      <c r="D224" s="15" t="inlineStr">
+        <is>
+          <t>NE01</t>
+        </is>
+      </c>
+      <c r="E224" s="15" t="inlineStr">
+        <is>
+          <t>Stoff-Alpaka groß</t>
+        </is>
+      </c>
+      <c r="F224" s="16" t="inlineStr">
+        <is>
+          <t>Großes Stofftier in Alpakaform, beiger Bouclé-Bezug, standfest. Etwa einen Meter hoch.</t>
+        </is>
+      </c>
+      <c r="G224" s="15" t="inlineStr">
+        <is>
+          <t>Deko</t>
+        </is>
+      </c>
+      <c r="H224" s="15" t="inlineStr">
+        <is>
+          <t>Flur</t>
+        </is>
+      </c>
+      <c r="I224" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J224" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K224" s="17" t="n"/>
+      <c r="L224" s="18">
+        <f>J224-IF(K224="",0,K224)</f>
+        <v/>
+      </c>
+      <c r="M224" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N224" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O224" s="19" t="n"/>
+      <c r="P224" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q224" s="19" t="n"/>
+      <c r="R224" s="20" t="n"/>
+      <c r="S224" s="20" t="n">
+        <v>55</v>
+      </c>
+      <c r="T224" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U224" s="21">
+        <f>L224*S224</f>
+        <v/>
+      </c>
+      <c r="V224" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W224" s="15" t="inlineStr">
+        <is>
+          <t>F-248</t>
+        </is>
+      </c>
+      <c r="X224" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y224" s="19" t="n"/>
+      <c r="Z224" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA224" s="19" t="n"/>
+      <c r="AB224" s="19" t="n"/>
+      <c r="AC224" s="19" t="n"/>
+      <c r="AD224" s="20" t="n"/>
+      <c r="AE224" s="21">
+        <f>IF(K224="","",K224*AD224)</f>
+        <v/>
+      </c>
+      <c r="AF224" s="19" t="n"/>
+      <c r="AG224" s="19" t="n"/>
+      <c r="AH224" s="19" t="n"/>
+      <c r="AI224" s="19" t="n"/>
+      <c r="AJ224" s="19" t="n"/>
+      <c r="AK224" s="19" t="n"/>
+      <c r="AL224" s="16" t="inlineStr">
+        <is>
+          <t>1 Stück.</t>
+        </is>
+      </c>
+      <c r="AM224" s="22" t="n"/>
+    </row>
+    <row r="225" ht="30" customHeight="1">
+      <c r="A225" s="15" t="inlineStr">
+        <is>
+          <t>NE01-20</t>
+        </is>
+      </c>
+      <c r="B225" s="15" t="n"/>
+      <c r="C225" s="15" t="n"/>
+      <c r="D225" s="15" t="inlineStr">
+        <is>
+          <t>NE01</t>
+        </is>
+      </c>
+      <c r="E225" s="15" t="inlineStr">
+        <is>
+          <t>Kinder-Ohrensessel rot, Kunstleder</t>
+        </is>
+      </c>
+      <c r="F225" s="16" t="inlineStr">
+        <is>
+          <t>Ohrensessel in Kindergröße, roter Kunstlederbezug, geschwungene schwarze Holzbeine. An einer Armlehne ist der Bezug aufgerissen.</t>
+        </is>
+      </c>
+      <c r="G225" s="15" t="inlineStr">
+        <is>
+          <t>Möbel</t>
+        </is>
+      </c>
+      <c r="H225" s="15" t="inlineStr">
+        <is>
+          <t>Flur</t>
+        </is>
+      </c>
+      <c r="I225" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J225" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K225" s="17" t="n"/>
+      <c r="L225" s="18">
+        <f>J225-IF(K225="",0,K225)</f>
+        <v/>
+      </c>
+      <c r="M225" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N225" s="15" t="inlineStr">
+        <is>
+          <t>stark gebraucht</t>
+        </is>
+      </c>
+      <c r="O225" s="19" t="n"/>
+      <c r="P225" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q225" s="19" t="n"/>
+      <c r="R225" s="20" t="n"/>
+      <c r="S225" s="20" t="n">
+        <v>55</v>
+      </c>
+      <c r="T225" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U225" s="21">
+        <f>L225*S225</f>
+        <v/>
+      </c>
+      <c r="V225" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W225" s="15" t="inlineStr">
+        <is>
+          <t>F-249</t>
+        </is>
+      </c>
+      <c r="X225" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y225" s="19" t="n"/>
+      <c r="Z225" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA225" s="19" t="n"/>
+      <c r="AB225" s="19" t="n"/>
+      <c r="AC225" s="19" t="n"/>
+      <c r="AD225" s="20" t="n"/>
+      <c r="AE225" s="21">
+        <f>IF(K225="","",K225*AD225)</f>
+        <v/>
+      </c>
+      <c r="AF225" s="19" t="n"/>
+      <c r="AG225" s="19" t="n"/>
+      <c r="AH225" s="19" t="n"/>
+      <c r="AI225" s="19" t="n"/>
+      <c r="AJ225" s="19" t="n"/>
+      <c r="AK225" s="19" t="n"/>
+      <c r="AL225" s="16" t="inlineStr">
+        <is>
+          <t>2 Sessel – abgebildet ist einer davon.</t>
+        </is>
+      </c>
+      <c r="AM225" s="22" t="n"/>
+    </row>
+    <row r="226" ht="30" customHeight="1">
+      <c r="A226" s="15" t="inlineStr">
+        <is>
+          <t>NE01-21</t>
+        </is>
+      </c>
+      <c r="B226" s="15" t="n"/>
+      <c r="C226" s="15" t="n"/>
+      <c r="D226" s="15" t="inlineStr">
+        <is>
+          <t>NE01</t>
+        </is>
+      </c>
+      <c r="E226" s="15" t="inlineStr">
+        <is>
+          <t>Wandregal weiß mit drei Wannen</t>
+        </is>
+      </c>
+      <c r="F226" s="16" t="inlineStr">
+        <is>
+          <t>Weißes Wandelement mit drei Fächern und eingeschobenen Kunststoffwannen.</t>
+        </is>
+      </c>
+      <c r="G226" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H226" s="15" t="inlineStr">
+        <is>
+          <t>Flur</t>
+        </is>
+      </c>
+      <c r="I226" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J226" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="K226" s="17" t="n"/>
+      <c r="L226" s="18">
+        <f>J226-IF(K226="",0,K226)</f>
+        <v/>
+      </c>
+      <c r="M226" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N226" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O226" s="19" t="n"/>
+      <c r="P226" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q226" s="19" t="n"/>
+      <c r="R226" s="20" t="n"/>
+      <c r="S226" s="20" t="n">
+        <v>35</v>
+      </c>
+      <c r="T226" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U226" s="21">
+        <f>L226*S226</f>
+        <v/>
+      </c>
+      <c r="V226" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W226" s="15" t="inlineStr">
+        <is>
+          <t>F-250</t>
+        </is>
+      </c>
+      <c r="X226" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y226" s="19" t="n"/>
+      <c r="Z226" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA226" s="19" t="n"/>
+      <c r="AB226" s="19" t="n"/>
+      <c r="AC226" s="19" t="n"/>
+      <c r="AD226" s="20" t="n"/>
+      <c r="AE226" s="21">
+        <f>IF(K226="","",K226*AD226)</f>
+        <v/>
+      </c>
+      <c r="AF226" s="19" t="n"/>
+      <c r="AG226" s="19" t="n"/>
+      <c r="AH226" s="19" t="n"/>
+      <c r="AI226" s="19" t="n"/>
+      <c r="AJ226" s="19" t="n"/>
+      <c r="AK226" s="19" t="n"/>
+      <c r="AL226" s="16" t="inlineStr">
+        <is>
+          <t>12 Regale einschließlich der Wannen – abgebildet ist eines davon. Die Hundehaken darunter sind eigene Positionen (NE01-22 und NE01-23).</t>
+        </is>
+      </c>
+      <c r="AM226" s="22" t="n"/>
+    </row>
+    <row r="227" ht="30" customHeight="1">
+      <c r="A227" s="15" t="inlineStr">
+        <is>
+          <t>NE01-22</t>
+        </is>
+      </c>
+      <c r="B227" s="15" t="n"/>
+      <c r="C227" s="15" t="n"/>
+      <c r="D227" s="15" t="inlineStr">
+        <is>
+          <t>NE01</t>
+        </is>
+      </c>
+      <c r="E227" s="15" t="inlineStr">
+        <is>
+          <t>Wandhaken Hund, schwarz</t>
+        </is>
+      </c>
+      <c r="F227" s="16" t="inlineStr">
+        <is>
+          <t>Wandhaken in Form eines Hunde-Hinterteils mit aufgestelltem Schwanz, schwarz, mit einer Schraube befestigt.</t>
+        </is>
+      </c>
+      <c r="G227" s="15" t="inlineStr">
+        <is>
+          <t>Deko</t>
+        </is>
+      </c>
+      <c r="H227" s="15" t="inlineStr">
+        <is>
+          <t>Flur</t>
+        </is>
+      </c>
+      <c r="I227" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J227" s="17" t="n">
+        <v>21</v>
+      </c>
+      <c r="K227" s="17" t="n"/>
+      <c r="L227" s="18">
+        <f>J227-IF(K227="",0,K227)</f>
+        <v/>
+      </c>
+      <c r="M227" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N227" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O227" s="19" t="n"/>
+      <c r="P227" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q227" s="19" t="n"/>
+      <c r="R227" s="20" t="n"/>
+      <c r="S227" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="T227" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U227" s="21">
+        <f>L227*S227</f>
+        <v/>
+      </c>
+      <c r="V227" s="15" t="inlineStr">
+        <is>
+          <t>Versand möglich</t>
+        </is>
+      </c>
+      <c r="W227" s="15" t="inlineStr">
+        <is>
+          <t>F-251</t>
+        </is>
+      </c>
+      <c r="X227" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y227" s="19" t="n"/>
+      <c r="Z227" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA227" s="19" t="n"/>
+      <c r="AB227" s="19" t="n"/>
+      <c r="AC227" s="19" t="n"/>
+      <c r="AD227" s="20" t="n"/>
+      <c r="AE227" s="21">
+        <f>IF(K227="","",K227*AD227)</f>
+        <v/>
+      </c>
+      <c r="AF227" s="19" t="n"/>
+      <c r="AG227" s="19" t="n"/>
+      <c r="AH227" s="19" t="n"/>
+      <c r="AI227" s="19" t="n"/>
+      <c r="AJ227" s="19" t="n"/>
+      <c r="AK227" s="19" t="n"/>
+      <c r="AL227" s="16" t="inlineStr">
+        <is>
+          <t>21 Haken – abgebildet ist einer davon.</t>
+        </is>
+      </c>
+      <c r="AM227" s="22" t="n"/>
+    </row>
+    <row r="228" ht="30" customHeight="1">
+      <c r="A228" s="15" t="inlineStr">
+        <is>
+          <t>NE01-23</t>
+        </is>
+      </c>
+      <c r="B228" s="15" t="n"/>
+      <c r="C228" s="15" t="n"/>
+      <c r="D228" s="15" t="inlineStr">
+        <is>
+          <t>NE01</t>
+        </is>
+      </c>
+      <c r="E228" s="15" t="inlineStr">
+        <is>
+          <t>Wandhaken Hund, grün</t>
+        </is>
+      </c>
+      <c r="F228" s="16" t="inlineStr">
+        <is>
+          <t>Wandhaken in Form eines Hunde-Hinterteils mit aufgestelltem Schwanz, hellgrün, mit einer Schraube befestigt.</t>
+        </is>
+      </c>
+      <c r="G228" s="15" t="inlineStr">
+        <is>
+          <t>Deko</t>
+        </is>
+      </c>
+      <c r="H228" s="15" t="inlineStr">
+        <is>
+          <t>Flur</t>
+        </is>
+      </c>
+      <c r="I228" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J228" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="K228" s="17" t="n"/>
+      <c r="L228" s="18">
+        <f>J228-IF(K228="",0,K228)</f>
+        <v/>
+      </c>
+      <c r="M228" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N228" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O228" s="19" t="n"/>
+      <c r="P228" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q228" s="19" t="n"/>
+      <c r="R228" s="20" t="n"/>
+      <c r="S228" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="T228" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U228" s="21">
+        <f>L228*S228</f>
+        <v/>
+      </c>
+      <c r="V228" s="15" t="inlineStr">
+        <is>
+          <t>Versand möglich</t>
+        </is>
+      </c>
+      <c r="W228" s="15" t="inlineStr">
+        <is>
+          <t>F-252</t>
+        </is>
+      </c>
+      <c r="X228" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y228" s="19" t="n"/>
+      <c r="Z228" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA228" s="19" t="n"/>
+      <c r="AB228" s="19" t="n"/>
+      <c r="AC228" s="19" t="n"/>
+      <c r="AD228" s="20" t="n"/>
+      <c r="AE228" s="21">
+        <f>IF(K228="","",K228*AD228)</f>
+        <v/>
+      </c>
+      <c r="AF228" s="19" t="n"/>
+      <c r="AG228" s="19" t="n"/>
+      <c r="AH228" s="19" t="n"/>
+      <c r="AI228" s="19" t="n"/>
+      <c r="AJ228" s="19" t="n"/>
+      <c r="AK228" s="19" t="n"/>
+      <c r="AL228" s="16" t="inlineStr">
+        <is>
+          <t>11 Haken – abgebildet ist einer davon.</t>
+        </is>
+      </c>
+      <c r="AM228" s="22" t="n"/>
+    </row>
+    <row r="229" ht="30" customHeight="1">
+      <c r="A229" s="15" t="inlineStr">
+        <is>
+          <t>NE01-24</t>
+        </is>
+      </c>
+      <c r="B229" s="15" t="n"/>
+      <c r="C229" s="15" t="n"/>
+      <c r="D229" s="15" t="inlineStr">
+        <is>
+          <t>NE01</t>
+        </is>
+      </c>
+      <c r="E229" s="15" t="inlineStr">
+        <is>
+          <t>Truhenbank Kindergröße, Buche mit weiß</t>
+        </is>
+      </c>
+      <c r="F229" s="16" t="inlineStr">
+        <is>
+          <t>Sitzbank in Kindergröße: Gestell und Sprossenlehne aus Buche massiv, Sitzfläche und Korpus weiß. Unter der Sitzfläche ein Stauraum. Sitzfläche stark verschmutzt und abgestoßen.</t>
+        </is>
+      </c>
+      <c r="G229" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H229" s="15" t="inlineStr">
+        <is>
+          <t>Flur</t>
+        </is>
+      </c>
+      <c r="I229" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J229" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="K229" s="17" t="n"/>
+      <c r="L229" s="18">
+        <f>J229-IF(K229="",0,K229)</f>
+        <v/>
+      </c>
+      <c r="M229" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N229" s="15" t="inlineStr">
+        <is>
+          <t>stark gebraucht</t>
+        </is>
+      </c>
+      <c r="O229" s="19" t="n"/>
+      <c r="P229" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q229" s="19" t="n"/>
+      <c r="R229" s="20" t="n"/>
+      <c r="S229" s="20" t="n">
+        <v>35</v>
+      </c>
+      <c r="T229" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U229" s="21">
+        <f>L229*S229</f>
+        <v/>
+      </c>
+      <c r="V229" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W229" s="15" t="inlineStr">
+        <is>
+          <t>F-253</t>
+        </is>
+      </c>
+      <c r="X229" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y229" s="19" t="n"/>
+      <c r="Z229" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA229" s="19" t="n"/>
+      <c r="AB229" s="19" t="n"/>
+      <c r="AC229" s="19" t="n"/>
+      <c r="AD229" s="20" t="n"/>
+      <c r="AE229" s="21">
+        <f>IF(K229="","",K229*AD229)</f>
+        <v/>
+      </c>
+      <c r="AF229" s="19" t="n"/>
+      <c r="AG229" s="19" t="n"/>
+      <c r="AH229" s="19" t="n"/>
+      <c r="AI229" s="19" t="n"/>
+      <c r="AJ229" s="19" t="n"/>
+      <c r="AK229" s="19" t="n"/>
+      <c r="AL229" s="16" t="inlineStr">
+        <is>
+          <t>3 Bänke – abgebildet sind zwei davon.</t>
+        </is>
+      </c>
+      <c r="AM229" s="22" t="n"/>
+    </row>
+    <row r="230" ht="30" customHeight="1">
+      <c r="A230" s="15" t="inlineStr">
+        <is>
+          <t>NE01-25</t>
+        </is>
+      </c>
+      <c r="B230" s="15" t="n"/>
+      <c r="C230" s="15" t="n"/>
+      <c r="D230" s="15" t="inlineStr">
+        <is>
+          <t>NE01</t>
+        </is>
+      </c>
+      <c r="E230" s="15" t="inlineStr">
+        <is>
+          <t>Truhenbank Kindergröße, ganz weiß</t>
+        </is>
+      </c>
+      <c r="F230" s="16" t="inlineStr">
+        <is>
+          <t>Sitzbank in Kindergröße, komplett weiß lackiert, mit Sprossenlehne und Stauraum unter der Sitzfläche. Lack an Kanten abgeplatzt, Sitzfläche zerkratzt.</t>
+        </is>
+      </c>
+      <c r="G230" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H230" s="15" t="inlineStr">
+        <is>
+          <t>Flur</t>
+        </is>
+      </c>
+      <c r="I230" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J230" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="K230" s="17" t="n"/>
+      <c r="L230" s="18">
+        <f>J230-IF(K230="",0,K230)</f>
+        <v/>
+      </c>
+      <c r="M230" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N230" s="15" t="inlineStr">
+        <is>
+          <t>stark gebraucht</t>
+        </is>
+      </c>
+      <c r="O230" s="19" t="n"/>
+      <c r="P230" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q230" s="19" t="n"/>
+      <c r="R230" s="20" t="n"/>
+      <c r="S230" s="20" t="n">
+        <v>35</v>
+      </c>
+      <c r="T230" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U230" s="21">
+        <f>L230*S230</f>
+        <v/>
+      </c>
+      <c r="V230" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W230" s="15" t="inlineStr">
+        <is>
+          <t>F-254</t>
+        </is>
+      </c>
+      <c r="X230" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y230" s="19" t="n"/>
+      <c r="Z230" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA230" s="19" t="n"/>
+      <c r="AB230" s="19" t="n"/>
+      <c r="AC230" s="19" t="n"/>
+      <c r="AD230" s="20" t="n"/>
+      <c r="AE230" s="21">
+        <f>IF(K230="","",K230*AD230)</f>
+        <v/>
+      </c>
+      <c r="AF230" s="19" t="n"/>
+      <c r="AG230" s="19" t="n"/>
+      <c r="AH230" s="19" t="n"/>
+      <c r="AI230" s="19" t="n"/>
+      <c r="AJ230" s="19" t="n"/>
+      <c r="AK230" s="19" t="n"/>
+      <c r="AL230" s="16" t="inlineStr">
+        <is>
+          <t>3 Bänke – abgebildet ist eine davon.</t>
+        </is>
+      </c>
+      <c r="AM230" s="22" t="n"/>
+    </row>
+    <row r="231" ht="30" customHeight="1">
+      <c r="A231" s="15" t="inlineStr">
+        <is>
+          <t>NE01-26</t>
+        </is>
+      </c>
+      <c r="B231" s="15" t="n"/>
+      <c r="C231" s="15" t="n"/>
+      <c r="D231" s="15" t="inlineStr">
+        <is>
+          <t>NE01</t>
+        </is>
+      </c>
+      <c r="E231" s="15" t="inlineStr">
+        <is>
+          <t>Sitzbank weiß mit Stauraum, lang</t>
+        </is>
+      </c>
+      <c r="F231" s="16" t="inlineStr">
+        <is>
+          <t>Lange Sitzbank in Weiß mit niedrigen Armlehnen und aufklappbarer Sitzfläche, darunter Stauraum mit Griffmulde. Lack großflächig zerkratzt.</t>
+        </is>
+      </c>
+      <c r="G231" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H231" s="15" t="inlineStr">
+        <is>
+          <t>Flur</t>
+        </is>
+      </c>
+      <c r="I231" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J231" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="K231" s="17" t="n"/>
+      <c r="L231" s="18">
+        <f>J231-IF(K231="",0,K231)</f>
+        <v/>
+      </c>
+      <c r="M231" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N231" s="15" t="inlineStr">
+        <is>
+          <t>stark gebraucht</t>
+        </is>
+      </c>
+      <c r="O231" s="19" t="n"/>
+      <c r="P231" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q231" s="19" t="n"/>
+      <c r="R231" s="20" t="n"/>
+      <c r="S231" s="20" t="n">
+        <v>45</v>
+      </c>
+      <c r="T231" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U231" s="21">
+        <f>L231*S231</f>
+        <v/>
+      </c>
+      <c r="V231" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W231" s="15" t="inlineStr">
+        <is>
+          <t>F-255</t>
+        </is>
+      </c>
+      <c r="X231" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y231" s="19" t="n"/>
+      <c r="Z231" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA231" s="19" t="n"/>
+      <c r="AB231" s="19" t="n"/>
+      <c r="AC231" s="19" t="n"/>
+      <c r="AD231" s="20" t="n"/>
+      <c r="AE231" s="21">
+        <f>IF(K231="","",K231*AD231)</f>
+        <v/>
+      </c>
+      <c r="AF231" s="19" t="n"/>
+      <c r="AG231" s="19" t="n"/>
+      <c r="AH231" s="19" t="n"/>
+      <c r="AI231" s="19" t="n"/>
+      <c r="AJ231" s="19" t="n"/>
+      <c r="AK231" s="19" t="n"/>
+      <c r="AL231" s="16" t="inlineStr">
+        <is>
+          <t>7 Bänke – abgebildet ist eine davon.</t>
+        </is>
+      </c>
+      <c r="AM231" s="22" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:AM221"/>
+  <autoFilter ref="A2:AM231"/>
   <mergeCells count="7">
     <mergeCell ref="AH1:AK1"/>
     <mergeCell ref="S1:U1"/>
@@ -27781,7 +28965,7 @@
     <mergeCell ref="AL1:AM1"/>
     <mergeCell ref="AD1:AG1"/>
   </mergeCells>
-  <conditionalFormatting sqref="Z3:Z221">
+  <conditionalFormatting sqref="Z3:Z231">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"reserviert"</formula>
     </cfRule>
@@ -27792,12 +28976,12 @@
       <formula>"verkauft"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I3:I221">
+  <conditionalFormatting sqref="I3:I231">
     <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
       <formula>"A"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P3:P221">
+  <conditionalFormatting sqref="P3:P231">
     <cfRule type="cellIs" priority="5" operator="equal" dxfId="4">
       <formula>"entfällt"</formula>
     </cfRule>
@@ -27888,7 +29072,7 @@
         </is>
       </c>
       <c r="B5" s="27">
-        <f>COUNTA(Artikelstamm!$A$3:$A$221)</f>
+        <f>COUNTA(Artikelstamm!$A$3:$A$231)</f>
         <v/>
       </c>
     </row>
@@ -27899,7 +29083,7 @@
         </is>
       </c>
       <c r="B6" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$221,"verfügbar")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$231,"verfügbar")</f>
         <v/>
       </c>
     </row>
@@ -27910,7 +29094,7 @@
         </is>
       </c>
       <c r="B7" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$221,"reserviert")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$231,"reserviert")</f>
         <v/>
       </c>
     </row>
@@ -27921,7 +29105,7 @@
         </is>
       </c>
       <c r="B8" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$221,"teilverkauft")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$231,"teilverkauft")</f>
         <v/>
       </c>
     </row>
@@ -27932,7 +29116,7 @@
         </is>
       </c>
       <c r="B9" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$221,"verkauft")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$231,"verkauft")</f>
         <v/>
       </c>
     </row>
@@ -27943,7 +29127,7 @@
         </is>
       </c>
       <c r="B10" s="27">
-        <f>SUM(Artikelstamm!$L$3:$L$221)</f>
+        <f>SUM(Artikelstamm!$L$3:$L$231)</f>
         <v/>
       </c>
     </row>
@@ -27954,7 +29138,7 @@
         </is>
       </c>
       <c r="B11" s="29">
-        <f>SUM(Artikelstamm!$U$3:$U$221)</f>
+        <f>SUM(Artikelstamm!$U$3:$U$231)</f>
         <v/>
       </c>
     </row>
@@ -27972,7 +29156,7 @@
         </is>
       </c>
       <c r="B13" s="27">
-        <f>SUM(Artikelstamm!$K$3:$K$221)</f>
+        <f>SUM(Artikelstamm!$K$3:$K$231)</f>
         <v/>
       </c>
     </row>
@@ -27983,7 +29167,7 @@
         </is>
       </c>
       <c r="B14" s="30">
-        <f>SUMPRODUCT(Artikelstamm!$K$3:$K$221,Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT(Artikelstamm!$K$3:$K$231,Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
     </row>
@@ -28016,7 +29200,7 @@
         </is>
       </c>
       <c r="B17" s="30">
-        <f>SUMPRODUCT((Artikelstamm!$AI$3:$AI$221="bezahlt")*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AI$3:$AI$231="bezahlt")*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
     </row>
@@ -28045,7 +29229,7 @@
         </is>
       </c>
       <c r="B21" s="31">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$221,"*verkauft",Artikelstamm!$AH$3:$AH$221,"")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$231,"*verkauft",Artikelstamm!$AH$3:$AH$231,"")</f>
         <v/>
       </c>
     </row>
@@ -28056,7 +29240,7 @@
         </is>
       </c>
       <c r="B22" s="31">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$221,"*verkauft",Artikelstamm!$AI$3:$AI$221,"offen")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$231,"*verkauft",Artikelstamm!$AI$3:$AI$231,"offen")</f>
         <v/>
       </c>
     </row>
@@ -28067,7 +29251,7 @@
         </is>
       </c>
       <c r="B23" s="27">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$221,"reserviert",Artikelstamm!$AK$3:$AK$221,"")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$231,"reserviert",Artikelstamm!$AK$3:$AK$231,"")</f>
         <v/>
       </c>
     </row>
@@ -28078,7 +29262,7 @@
         </is>
       </c>
       <c r="B24" s="27">
-        <f>COUNTIFS(Artikelstamm!$S$3:$S$221,"")</f>
+        <f>COUNTIFS(Artikelstamm!$S$3:$S$231,"")</f>
         <v/>
       </c>
     </row>
@@ -28089,7 +29273,7 @@
         </is>
       </c>
       <c r="B25" s="27">
-        <f>COUNTIFS(Artikelstamm!$O$3:$O$221,"")</f>
+        <f>COUNTIFS(Artikelstamm!$O$3:$O$231,"")</f>
         <v/>
       </c>
     </row>
@@ -28129,15 +29313,15 @@
         </is>
       </c>
       <c r="B30" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$221,$A30)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$231,$A30)</f>
         <v/>
       </c>
       <c r="C30" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$221=$A30)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$231=$A30)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
       <c r="D30" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$221,$A30,Artikelstamm!$U$3:$U$221)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$231,$A30,Artikelstamm!$U$3:$U$231)</f>
         <v/>
       </c>
     </row>
@@ -28148,15 +29332,15 @@
         </is>
       </c>
       <c r="B31" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$221,$A31)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$231,$A31)</f>
         <v/>
       </c>
       <c r="C31" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$221=$A31)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$231=$A31)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
       <c r="D31" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$221,$A31,Artikelstamm!$U$3:$U$221)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$231,$A31,Artikelstamm!$U$3:$U$231)</f>
         <v/>
       </c>
     </row>
@@ -28167,15 +29351,15 @@
         </is>
       </c>
       <c r="B32" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$221,$A32)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$231,$A32)</f>
         <v/>
       </c>
       <c r="C32" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$221=$A32)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$231=$A32)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
       <c r="D32" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$221,$A32,Artikelstamm!$U$3:$U$221)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$231,$A32,Artikelstamm!$U$3:$U$231)</f>
         <v/>
       </c>
     </row>
@@ -28234,15 +29418,15 @@
         </is>
       </c>
       <c r="B37" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$221,$A37)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$231,$A37)</f>
         <v/>
       </c>
       <c r="C37" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$221=$A37)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$231=$A37)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
       <c r="D37" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$221,$A37,Artikelstamm!$U$3:$U$221)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$231,$A37,Artikelstamm!$U$3:$U$231)</f>
         <v/>
       </c>
     </row>
@@ -28253,15 +29437,15 @@
         </is>
       </c>
       <c r="B38" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$221,$A38)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$231,$A38)</f>
         <v/>
       </c>
       <c r="C38" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$221=$A38)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$231=$A38)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
       <c r="D38" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$221,$A38,Artikelstamm!$U$3:$U$221)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$231,$A38,Artikelstamm!$U$3:$U$231)</f>
         <v/>
       </c>
     </row>
@@ -28272,15 +29456,15 @@
         </is>
       </c>
       <c r="B39" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$221,$A39)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$231,$A39)</f>
         <v/>
       </c>
       <c r="C39" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$221=$A39)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$231=$A39)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
       <c r="D39" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$221,$A39,Artikelstamm!$U$3:$U$221)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$231,$A39,Artikelstamm!$U$3:$U$231)</f>
         <v/>
       </c>
     </row>
@@ -28291,15 +29475,15 @@
         </is>
       </c>
       <c r="B40" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$221,$A40)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$231,$A40)</f>
         <v/>
       </c>
       <c r="C40" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$221=$A40)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$231=$A40)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
       <c r="D40" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$221,$A40,Artikelstamm!$U$3:$U$221)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$231,$A40,Artikelstamm!$U$3:$U$231)</f>
         <v/>
       </c>
     </row>
@@ -28310,15 +29494,15 @@
         </is>
       </c>
       <c r="B41" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$221,$A41)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$231,$A41)</f>
         <v/>
       </c>
       <c r="C41" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$221=$A41)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$231=$A41)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
       <c r="D41" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$221,$A41,Artikelstamm!$U$3:$U$221)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$231,$A41,Artikelstamm!$U$3:$U$231)</f>
         <v/>
       </c>
     </row>
@@ -28329,15 +29513,15 @@
         </is>
       </c>
       <c r="B42" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$221,$A42)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$231,$A42)</f>
         <v/>
       </c>
       <c r="C42" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$221=$A42)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$231=$A42)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
       <c r="D42" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$221,$A42,Artikelstamm!$U$3:$U$221)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$231,$A42,Artikelstamm!$U$3:$U$231)</f>
         <v/>
       </c>
     </row>
@@ -28348,15 +29532,15 @@
         </is>
       </c>
       <c r="B43" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$221,$A43)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$231,$A43)</f>
         <v/>
       </c>
       <c r="C43" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$221=$A43)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$231=$A43)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
       <c r="D43" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$221,$A43,Artikelstamm!$U$3:$U$221)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$231,$A43,Artikelstamm!$U$3:$U$231)</f>
         <v/>
       </c>
     </row>
@@ -28367,15 +29551,15 @@
         </is>
       </c>
       <c r="B44" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$221,$A44)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$231,$A44)</f>
         <v/>
       </c>
       <c r="C44" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$221=$A44)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$231=$A44)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
       <c r="D44" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$221,$A44,Artikelstamm!$U$3:$U$221)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$231,$A44,Artikelstamm!$U$3:$U$231)</f>
         <v/>
       </c>
     </row>
@@ -28386,15 +29570,15 @@
         </is>
       </c>
       <c r="B45" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$221,$A45)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$231,$A45)</f>
         <v/>
       </c>
       <c r="C45" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$221=$A45)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$231=$A45)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
       <c r="D45" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$221,$A45,Artikelstamm!$U$3:$U$221)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$231,$A45,Artikelstamm!$U$3:$U$231)</f>
         <v/>
       </c>
     </row>
@@ -28405,15 +29589,15 @@
         </is>
       </c>
       <c r="B46" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$221,$A46)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$231,$A46)</f>
         <v/>
       </c>
       <c r="C46" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$221=$A46)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$231=$A46)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
       <c r="D46" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$221,$A46,Artikelstamm!$U$3:$U$221)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$231,$A46,Artikelstamm!$U$3:$U$231)</f>
         <v/>
       </c>
     </row>
@@ -28424,15 +29608,15 @@
         </is>
       </c>
       <c r="B47" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$221,$A47)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$231,$A47)</f>
         <v/>
       </c>
       <c r="C47" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$221=$A47)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$231=$A47)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
       <c r="D47" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$221,$A47,Artikelstamm!$U$3:$U$221)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$231,$A47,Artikelstamm!$U$3:$U$231)</f>
         <v/>
       </c>
     </row>
@@ -28443,15 +29627,15 @@
         </is>
       </c>
       <c r="B48" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$221,$A48)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$231,$A48)</f>
         <v/>
       </c>
       <c r="C48" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$221=$A48)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$231=$A48)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
       <c r="D48" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$221,$A48,Artikelstamm!$U$3:$U$221)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$231,$A48,Artikelstamm!$U$3:$U$231)</f>
         <v/>
       </c>
     </row>
@@ -28462,15 +29646,15 @@
         </is>
       </c>
       <c r="B49" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$221,$A49)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$231,$A49)</f>
         <v/>
       </c>
       <c r="C49" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$221=$A49)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$231=$A49)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
       <c r="D49" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$221,$A49,Artikelstamm!$U$3:$U$221)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$231,$A49,Artikelstamm!$U$3:$U$231)</f>
         <v/>
       </c>
     </row>
@@ -28481,15 +29665,15 @@
         </is>
       </c>
       <c r="B50" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$221,$A50)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$231,$A50)</f>
         <v/>
       </c>
       <c r="C50" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$221=$A50)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$231=$A50)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
       <c r="D50" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$221,$A50,Artikelstamm!$U$3:$U$221)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$231,$A50,Artikelstamm!$U$3:$U$231)</f>
         <v/>
       </c>
     </row>
@@ -28548,15 +29732,15 @@
         </is>
       </c>
       <c r="B55" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$221,$A55)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A55)</f>
         <v/>
       </c>
       <c r="C55" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$221=$A55)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A55)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
       <c r="D55" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$221,$A55,Artikelstamm!$U$3:$U$221)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A55,Artikelstamm!$U$3:$U$231)</f>
         <v/>
       </c>
     </row>
@@ -28567,15 +29751,15 @@
         </is>
       </c>
       <c r="B56" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$221,$A56)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A56)</f>
         <v/>
       </c>
       <c r="C56" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$221=$A56)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A56)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
       <c r="D56" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$221,$A56,Artikelstamm!$U$3:$U$221)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A56,Artikelstamm!$U$3:$U$231)</f>
         <v/>
       </c>
     </row>
@@ -28586,15 +29770,15 @@
         </is>
       </c>
       <c r="B57" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$221,$A57)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A57)</f>
         <v/>
       </c>
       <c r="C57" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$221=$A57)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A57)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
       <c r="D57" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$221,$A57,Artikelstamm!$U$3:$U$221)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A57,Artikelstamm!$U$3:$U$231)</f>
         <v/>
       </c>
     </row>
@@ -28605,15 +29789,15 @@
         </is>
       </c>
       <c r="B58" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$221,$A58)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A58)</f>
         <v/>
       </c>
       <c r="C58" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$221=$A58)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A58)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
       <c r="D58" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$221,$A58,Artikelstamm!$U$3:$U$221)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A58,Artikelstamm!$U$3:$U$231)</f>
         <v/>
       </c>
     </row>
@@ -28624,15 +29808,15 @@
         </is>
       </c>
       <c r="B59" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$221,$A59)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A59)</f>
         <v/>
       </c>
       <c r="C59" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$221=$A59)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A59)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
       <c r="D59" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$221,$A59,Artikelstamm!$U$3:$U$221)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A59,Artikelstamm!$U$3:$U$231)</f>
         <v/>
       </c>
     </row>
@@ -28643,15 +29827,15 @@
         </is>
       </c>
       <c r="B60" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$221,$A60)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A60)</f>
         <v/>
       </c>
       <c r="C60" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$221=$A60)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A60)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
       <c r="D60" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$221,$A60,Artikelstamm!$U$3:$U$221)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A60,Artikelstamm!$U$3:$U$231)</f>
         <v/>
       </c>
     </row>
@@ -28662,15 +29846,15 @@
         </is>
       </c>
       <c r="B61" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$221,$A61)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A61)</f>
         <v/>
       </c>
       <c r="C61" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$221=$A61)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A61)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
       <c r="D61" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$221,$A61,Artikelstamm!$U$3:$U$221)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A61,Artikelstamm!$U$3:$U$231)</f>
         <v/>
       </c>
     </row>
@@ -28681,15 +29865,15 @@
         </is>
       </c>
       <c r="B62" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$221,$A62)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A62)</f>
         <v/>
       </c>
       <c r="C62" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$221=$A62)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A62)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
       <c r="D62" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$221,$A62,Artikelstamm!$U$3:$U$221)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A62,Artikelstamm!$U$3:$U$231)</f>
         <v/>
       </c>
     </row>
@@ -28700,15 +29884,15 @@
         </is>
       </c>
       <c r="B63" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$221,$A63)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A63)</f>
         <v/>
       </c>
       <c r="C63" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$221=$A63)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A63)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
       <c r="D63" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$221,$A63,Artikelstamm!$U$3:$U$221)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A63,Artikelstamm!$U$3:$U$231)</f>
         <v/>
       </c>
     </row>
@@ -28719,15 +29903,15 @@
         </is>
       </c>
       <c r="B64" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$221,$A64)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A64)</f>
         <v/>
       </c>
       <c r="C64" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$221=$A64)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A64)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
       <c r="D64" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$221,$A64,Artikelstamm!$U$3:$U$221)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A64,Artikelstamm!$U$3:$U$231)</f>
         <v/>
       </c>
     </row>
@@ -28738,15 +29922,15 @@
         </is>
       </c>
       <c r="B65" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$221,$A65)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A65)</f>
         <v/>
       </c>
       <c r="C65" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$221=$A65)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A65)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
       <c r="D65" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$221,$A65,Artikelstamm!$U$3:$U$221)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A65,Artikelstamm!$U$3:$U$231)</f>
         <v/>
       </c>
     </row>
@@ -28757,15 +29941,15 @@
         </is>
       </c>
       <c r="B66" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$221,$A66)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A66)</f>
         <v/>
       </c>
       <c r="C66" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$221=$A66)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A66)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
       <c r="D66" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$221,$A66,Artikelstamm!$U$3:$U$221)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A66,Artikelstamm!$U$3:$U$231)</f>
         <v/>
       </c>
     </row>
@@ -28776,15 +29960,15 @@
         </is>
       </c>
       <c r="B67" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$221,$A67)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A67)</f>
         <v/>
       </c>
       <c r="C67" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$221=$A67)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A67)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
       <c r="D67" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$221,$A67,Artikelstamm!$U$3:$U$221)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A67,Artikelstamm!$U$3:$U$231)</f>
         <v/>
       </c>
     </row>
@@ -28795,15 +29979,15 @@
         </is>
       </c>
       <c r="B68" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$221,$A68)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A68)</f>
         <v/>
       </c>
       <c r="C68" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$221=$A68)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A68)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
       <c r="D68" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$221,$A68,Artikelstamm!$U$3:$U$221)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A68,Artikelstamm!$U$3:$U$231)</f>
         <v/>
       </c>
     </row>
@@ -28814,15 +29998,15 @@
         </is>
       </c>
       <c r="B69" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$221,$A69)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A69)</f>
         <v/>
       </c>
       <c r="C69" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$221=$A69)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A69)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
       <c r="D69" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$221,$A69,Artikelstamm!$U$3:$U$221)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A69,Artikelstamm!$U$3:$U$231)</f>
         <v/>
       </c>
     </row>
@@ -28833,15 +30017,15 @@
         </is>
       </c>
       <c r="B70" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$221,$A70)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A70)</f>
         <v/>
       </c>
       <c r="C70" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$221=$A70)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A70)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
       <c r="D70" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$221,$A70,Artikelstamm!$U$3:$U$221)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A70,Artikelstamm!$U$3:$U$231)</f>
         <v/>
       </c>
     </row>
@@ -28852,15 +30036,15 @@
         </is>
       </c>
       <c r="B71" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$221,$A71)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A71)</f>
         <v/>
       </c>
       <c r="C71" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$221=$A71)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A71)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
       <c r="D71" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$221,$A71,Artikelstamm!$U$3:$U$221)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A71,Artikelstamm!$U$3:$U$231)</f>
         <v/>
       </c>
     </row>
@@ -28871,15 +30055,15 @@
         </is>
       </c>
       <c r="B72" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$221,$A72)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A72)</f>
         <v/>
       </c>
       <c r="C72" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$221=$A72)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A72)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
       <c r="D72" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$221,$A72,Artikelstamm!$U$3:$U$221)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A72,Artikelstamm!$U$3:$U$231)</f>
         <v/>
       </c>
     </row>
@@ -28890,15 +30074,15 @@
         </is>
       </c>
       <c r="B73" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$221,$A73)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A73)</f>
         <v/>
       </c>
       <c r="C73" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$221=$A73)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A73)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
       <c r="D73" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$221,$A73,Artikelstamm!$U$3:$U$221)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A73,Artikelstamm!$U$3:$U$231)</f>
         <v/>
       </c>
     </row>
@@ -28909,15 +30093,15 @@
         </is>
       </c>
       <c r="B74" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$221,$A74)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A74)</f>
         <v/>
       </c>
       <c r="C74" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$221=$A74)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A74)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
       <c r="D74" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$221,$A74,Artikelstamm!$U$3:$U$221)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A74,Artikelstamm!$U$3:$U$231)</f>
         <v/>
       </c>
     </row>
@@ -28928,15 +30112,15 @@
         </is>
       </c>
       <c r="B75" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$221,$A75)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A75)</f>
         <v/>
       </c>
       <c r="C75" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$221=$A75)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A75)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
       <c r="D75" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$221,$A75,Artikelstamm!$U$3:$U$221)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A75,Artikelstamm!$U$3:$U$231)</f>
         <v/>
       </c>
     </row>
@@ -28947,15 +30131,15 @@
         </is>
       </c>
       <c r="B76" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$221,$A76)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A76)</f>
         <v/>
       </c>
       <c r="C76" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$221=$A76)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A76)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
       <c r="D76" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$221,$A76,Artikelstamm!$U$3:$U$221)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A76,Artikelstamm!$U$3:$U$231)</f>
         <v/>
       </c>
     </row>
@@ -29009,11 +30193,11 @@
         </is>
       </c>
       <c r="B81" s="33">
-        <f>COUNTIF(Artikelstamm!$AB$3:$AB$221,$A81)</f>
+        <f>COUNTIF(Artikelstamm!$AB$3:$AB$231,$A81)</f>
         <v/>
       </c>
       <c r="C81" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AB$3:$AB$221=$A81)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AB$3:$AB$231=$A81)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
     </row>
@@ -29024,11 +30208,11 @@
         </is>
       </c>
       <c r="B82" s="33">
-        <f>COUNTIF(Artikelstamm!$AB$3:$AB$221,$A82)</f>
+        <f>COUNTIF(Artikelstamm!$AB$3:$AB$231,$A82)</f>
         <v/>
       </c>
       <c r="C82" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AB$3:$AB$221=$A82)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AB$3:$AB$231=$A82)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
     </row>
@@ -29039,11 +30223,11 @@
         </is>
       </c>
       <c r="B83" s="33">
-        <f>COUNTIF(Artikelstamm!$AB$3:$AB$221,$A83)</f>
+        <f>COUNTIF(Artikelstamm!$AB$3:$AB$231,$A83)</f>
         <v/>
       </c>
       <c r="C83" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AB$3:$AB$221=$A83)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AB$3:$AB$231=$A83)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
     </row>
@@ -29054,11 +30238,11 @@
         </is>
       </c>
       <c r="B84" s="33">
-        <f>COUNTIF(Artikelstamm!$AB$3:$AB$221,$A84)</f>
+        <f>COUNTIF(Artikelstamm!$AB$3:$AB$231,$A84)</f>
         <v/>
       </c>
       <c r="C84" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AB$3:$AB$221=$A84)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AB$3:$AB$231=$A84)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
     </row>
@@ -29069,11 +30253,11 @@
         </is>
       </c>
       <c r="B85" s="33">
-        <f>COUNTIF(Artikelstamm!$AB$3:$AB$221,$A85)</f>
+        <f>COUNTIF(Artikelstamm!$AB$3:$AB$231,$A85)</f>
         <v/>
       </c>
       <c r="C85" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AB$3:$AB$221=$A85)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AB$3:$AB$231=$A85)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
     </row>
@@ -29084,11 +30268,11 @@
         </is>
       </c>
       <c r="B86" s="33">
-        <f>COUNTIF(Artikelstamm!$AB$3:$AB$221,$A86)</f>
+        <f>COUNTIF(Artikelstamm!$AB$3:$AB$231,$A86)</f>
         <v/>
       </c>
       <c r="C86" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AB$3:$AB$221=$A86)*Artikelstamm!$K$3:$K$221*Artikelstamm!$AD$3:$AD$221)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AB$3:$AB$231=$A86)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
BA01 erfasst: 4 Positionen, Bestandsgebaeude Attika begonnen
Flur 1 (Bestandsgebaeude Attika, 10,94 m2). Blatt und drei von vier Fotos
lagen vor.

BA01-03 (Tannen-Dekoration) hat kein Foto - IMG_2291 fehlt in der Reihe.
Die Position steht deshalb auf Im_Katalog=nein mit OFFEN-Vermerk;
Beschreibung und Preis sind vorlaeufig. Moeglicherweise sind es dieselben
Stuecke wie NE01-15, die dort durchgestrichen wurden.

BA01-01 ist ein grossformatiges Mona-Lisa-Bild in Pop-Art-Technik, von
derselben Hand wie NU01-06 (Marilyn mit Bollenhut, 650 EUR). Mit 250 EUR
angesetzt und zur Bestaetigung vermerkt - der Vergleich spricht eher
fuer mehr.

Gesamtwert netto 35.557 -> 35.942 EUR, 177 aktive Positionen.
pruefen.py: 0 Fehler, 4 Hinweise.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011yyfqhuiWGsaNy38oaNoGo
</commit_message>
<xml_diff>
--- a/ausgabe/01_Artikelstamm_kikripp.xlsx
+++ b/ausgabe/01_Artikelstamm_kikripp.xlsx
@@ -15,7 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Artikelstamm'!$A$2:$AM$231</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Artikelstamm'!$A$2:$AM$235</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1019,7 +1019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AM231"/>
+  <dimension ref="A1:AM235"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -28954,8 +28954,484 @@
       </c>
       <c r="AM231" s="22" t="n"/>
     </row>
+    <row r="232" ht="30" customHeight="1">
+      <c r="A232" s="15" t="inlineStr">
+        <is>
+          <t>BA01-01</t>
+        </is>
+      </c>
+      <c r="B232" s="15" t="n"/>
+      <c r="C232" s="15" t="n"/>
+      <c r="D232" s="15" t="inlineStr">
+        <is>
+          <t>BA01</t>
+        </is>
+      </c>
+      <c r="E232" s="15" t="inlineStr">
+        <is>
+          <t>Gemälde Mona Lisa, Pop-Art</t>
+        </is>
+      </c>
+      <c r="F232" s="16" t="inlineStr">
+        <is>
+          <t>Acryl auf Leinwand im Hochformat: Mona Lisa als flächige Schablonenmalerei in Grau und Creme, darüber grüne Farbläufe vom oberen Rand. Eigenarbeit einer Privatperson, nicht signiert. Großes Format.</t>
+        </is>
+      </c>
+      <c r="G232" s="15" t="inlineStr">
+        <is>
+          <t>Kunst</t>
+        </is>
+      </c>
+      <c r="H232" s="15" t="inlineStr">
+        <is>
+          <t>Flur 1</t>
+        </is>
+      </c>
+      <c r="I232" s="15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J232" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K232" s="17" t="n"/>
+      <c r="L232" s="18">
+        <f>J232-IF(K232="",0,K232)</f>
+        <v/>
+      </c>
+      <c r="M232" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N232" s="15" t="inlineStr">
+        <is>
+          <t>gut</t>
+        </is>
+      </c>
+      <c r="O232" s="19" t="n"/>
+      <c r="P232" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q232" s="19" t="n"/>
+      <c r="R232" s="20" t="n"/>
+      <c r="S232" s="20" t="n">
+        <v>250</v>
+      </c>
+      <c r="T232" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U232" s="21">
+        <f>L232*S232</f>
+        <v/>
+      </c>
+      <c r="V232" s="15" t="inlineStr">
+        <is>
+          <t>Versand möglich</t>
+        </is>
+      </c>
+      <c r="W232" s="15" t="inlineStr">
+        <is>
+          <t>F-258</t>
+        </is>
+      </c>
+      <c r="X232" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y232" s="19" t="n"/>
+      <c r="Z232" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA232" s="19" t="n"/>
+      <c r="AB232" s="19" t="n"/>
+      <c r="AC232" s="19" t="n"/>
+      <c r="AD232" s="20" t="n"/>
+      <c r="AE232" s="21">
+        <f>IF(K232="","",K232*AD232)</f>
+        <v/>
+      </c>
+      <c r="AF232" s="19" t="n"/>
+      <c r="AG232" s="19" t="n"/>
+      <c r="AH232" s="19" t="n"/>
+      <c r="AI232" s="19" t="n"/>
+      <c r="AJ232" s="19" t="n"/>
+      <c r="AK232" s="19" t="n"/>
+      <c r="AL232" s="16" t="inlineStr">
+        <is>
+          <t>1 Bild.</t>
+        </is>
+      </c>
+      <c r="AM232" s="22" t="inlineStr">
+        <is>
+          <t>Preis unbestaetigt: stilistisch verwandt mit NU01-06 (Marilyn mit Bollenhut, 650 EUR) von derselben Hand. Bitte pruefen, ob 250 EUR passt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="233" ht="30" customHeight="1">
+      <c r="A233" s="15" t="inlineStr">
+        <is>
+          <t>BA01-02</t>
+        </is>
+      </c>
+      <c r="B233" s="15" t="n"/>
+      <c r="C233" s="15" t="n"/>
+      <c r="D233" s="15" t="inlineStr">
+        <is>
+          <t>BA01</t>
+        </is>
+      </c>
+      <c r="E233" s="15" t="inlineStr">
+        <is>
+          <t>Acrylbild abstrakt, Neonfarben</t>
+        </is>
+      </c>
+      <c r="F233" s="16" t="inlineStr">
+        <is>
+          <t>Acryl auf Leinwand: abstrakte Komposition mit breiten Pinselzügen in Grün und Blau, darüber Schleudertechnik in Neongelb, Neonrot und Pink. Eigenarbeit einer Privatperson, nicht signiert.</t>
+        </is>
+      </c>
+      <c r="G233" s="15" t="inlineStr">
+        <is>
+          <t>Kunst</t>
+        </is>
+      </c>
+      <c r="H233" s="15" t="inlineStr">
+        <is>
+          <t>Flur 1</t>
+        </is>
+      </c>
+      <c r="I233" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J233" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K233" s="17" t="n"/>
+      <c r="L233" s="18">
+        <f>J233-IF(K233="",0,K233)</f>
+        <v/>
+      </c>
+      <c r="M233" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N233" s="15" t="inlineStr">
+        <is>
+          <t>gut</t>
+        </is>
+      </c>
+      <c r="O233" s="19" t="n"/>
+      <c r="P233" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q233" s="19" t="n"/>
+      <c r="R233" s="20" t="n"/>
+      <c r="S233" s="20" t="n">
+        <v>90</v>
+      </c>
+      <c r="T233" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U233" s="21">
+        <f>L233*S233</f>
+        <v/>
+      </c>
+      <c r="V233" s="15" t="inlineStr">
+        <is>
+          <t>Versand möglich</t>
+        </is>
+      </c>
+      <c r="W233" s="15" t="inlineStr">
+        <is>
+          <t>F-259</t>
+        </is>
+      </c>
+      <c r="X233" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y233" s="19" t="n"/>
+      <c r="Z233" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA233" s="19" t="n"/>
+      <c r="AB233" s="19" t="n"/>
+      <c r="AC233" s="19" t="n"/>
+      <c r="AD233" s="20" t="n"/>
+      <c r="AE233" s="21">
+        <f>IF(K233="","",K233*AD233)</f>
+        <v/>
+      </c>
+      <c r="AF233" s="19" t="n"/>
+      <c r="AG233" s="19" t="n"/>
+      <c r="AH233" s="19" t="n"/>
+      <c r="AI233" s="19" t="n"/>
+      <c r="AJ233" s="19" t="n"/>
+      <c r="AK233" s="19" t="n"/>
+      <c r="AL233" s="16" t="inlineStr">
+        <is>
+          <t>1 Bild.</t>
+        </is>
+      </c>
+      <c r="AM233" s="22" t="n"/>
+    </row>
+    <row r="234" ht="30" customHeight="1">
+      <c r="A234" s="15" t="inlineStr">
+        <is>
+          <t>BA01-03</t>
+        </is>
+      </c>
+      <c r="B234" s="15" t="n"/>
+      <c r="C234" s="15" t="n"/>
+      <c r="D234" s="15" t="inlineStr">
+        <is>
+          <t>BA01</t>
+        </is>
+      </c>
+      <c r="E234" s="15" t="inlineStr">
+        <is>
+          <t>Tannen-Dekoration</t>
+        </is>
+      </c>
+      <c r="F234" s="16" t="inlineStr">
+        <is>
+          <t>Dekoration in Tannenform.</t>
+        </is>
+      </c>
+      <c r="G234" s="15" t="inlineStr">
+        <is>
+          <t>Deko</t>
+        </is>
+      </c>
+      <c r="H234" s="15" t="inlineStr">
+        <is>
+          <t>Flur 1</t>
+        </is>
+      </c>
+      <c r="I234" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J234" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K234" s="17" t="n"/>
+      <c r="L234" s="18">
+        <f>J234-IF(K234="",0,K234)</f>
+        <v/>
+      </c>
+      <c r="M234" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N234" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O234" s="19" t="n"/>
+      <c r="P234" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q234" s="19" t="n"/>
+      <c r="R234" s="20" t="n"/>
+      <c r="S234" s="20" t="n">
+        <v>25</v>
+      </c>
+      <c r="T234" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U234" s="21">
+        <f>L234*S234</f>
+        <v/>
+      </c>
+      <c r="V234" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W234" s="15" t="n"/>
+      <c r="X234" s="19" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="Y234" s="19" t="n"/>
+      <c r="Z234" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA234" s="19" t="n"/>
+      <c r="AB234" s="19" t="n"/>
+      <c r="AC234" s="19" t="n"/>
+      <c r="AD234" s="20" t="n"/>
+      <c r="AE234" s="21">
+        <f>IF(K234="","",K234*AD234)</f>
+        <v/>
+      </c>
+      <c r="AF234" s="19" t="n"/>
+      <c r="AG234" s="19" t="n"/>
+      <c r="AH234" s="19" t="n"/>
+      <c r="AI234" s="19" t="n"/>
+      <c r="AJ234" s="19" t="n"/>
+      <c r="AK234" s="19" t="n"/>
+      <c r="AL234" s="16" t="inlineStr">
+        <is>
+          <t>1 Stück.</t>
+        </is>
+      </c>
+      <c r="AM234" s="22" t="inlineStr">
+        <is>
+          <t>OFFEN: Foto fehlt - IMG_2291 ist nicht angekommen. Beschreibung und Preis sind daher vorlaeufig. Moeglicherweise dieselben Stuecke wie NE01-15 (Deko-Tannenbaum schwarz, 3 Stueck), die dort durchgestrichen wurden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="235" ht="30" customHeight="1">
+      <c r="A235" s="15" t="inlineStr">
+        <is>
+          <t>BA01-04</t>
+        </is>
+      </c>
+      <c r="B235" s="15" t="n"/>
+      <c r="C235" s="15" t="n"/>
+      <c r="D235" s="15" t="inlineStr">
+        <is>
+          <t>BA01</t>
+        </is>
+      </c>
+      <c r="E235" s="15" t="inlineStr">
+        <is>
+          <t>Leuchtbuchstabe K, schwarz</t>
+        </is>
+      </c>
+      <c r="F235" s="16" t="inlineStr">
+        <is>
+          <t>Buchstabe K aus schwarz beschichtetem Metall mit sechs runden Leuchtmitteln auf der Front, zum Aufstellen.</t>
+        </is>
+      </c>
+      <c r="G235" s="15" t="inlineStr">
+        <is>
+          <t>Deko</t>
+        </is>
+      </c>
+      <c r="H235" s="15" t="inlineStr">
+        <is>
+          <t>Flur 1</t>
+        </is>
+      </c>
+      <c r="I235" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J235" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K235" s="17" t="n"/>
+      <c r="L235" s="18">
+        <f>J235-IF(K235="",0,K235)</f>
+        <v/>
+      </c>
+      <c r="M235" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N235" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O235" s="19" t="n"/>
+      <c r="P235" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q235" s="19" t="n"/>
+      <c r="R235" s="20" t="n"/>
+      <c r="S235" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="T235" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U235" s="21">
+        <f>L235*S235</f>
+        <v/>
+      </c>
+      <c r="V235" s="15" t="inlineStr">
+        <is>
+          <t>Versand möglich</t>
+        </is>
+      </c>
+      <c r="W235" s="15" t="inlineStr">
+        <is>
+          <t>F-260</t>
+        </is>
+      </c>
+      <c r="X235" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y235" s="19" t="n"/>
+      <c r="Z235" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA235" s="19" t="n"/>
+      <c r="AB235" s="19" t="n"/>
+      <c r="AC235" s="19" t="n"/>
+      <c r="AD235" s="20" t="n"/>
+      <c r="AE235" s="21">
+        <f>IF(K235="","",K235*AD235)</f>
+        <v/>
+      </c>
+      <c r="AF235" s="19" t="n"/>
+      <c r="AG235" s="19" t="n"/>
+      <c r="AH235" s="19" t="n"/>
+      <c r="AI235" s="19" t="n"/>
+      <c r="AJ235" s="19" t="n"/>
+      <c r="AK235" s="19" t="n"/>
+      <c r="AL235" s="16" t="inlineStr">
+        <is>
+          <t>1 Stück.</t>
+        </is>
+      </c>
+      <c r="AM235" s="22" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:AM231"/>
+  <autoFilter ref="A2:AM235"/>
   <mergeCells count="7">
     <mergeCell ref="AH1:AK1"/>
     <mergeCell ref="S1:U1"/>
@@ -28965,7 +29441,7 @@
     <mergeCell ref="AL1:AM1"/>
     <mergeCell ref="AD1:AG1"/>
   </mergeCells>
-  <conditionalFormatting sqref="Z3:Z231">
+  <conditionalFormatting sqref="Z3:Z235">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"reserviert"</formula>
     </cfRule>
@@ -28976,12 +29452,12 @@
       <formula>"verkauft"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I3:I231">
+  <conditionalFormatting sqref="I3:I235">
     <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
       <formula>"A"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P3:P231">
+  <conditionalFormatting sqref="P3:P235">
     <cfRule type="cellIs" priority="5" operator="equal" dxfId="4">
       <formula>"entfällt"</formula>
     </cfRule>
@@ -29072,7 +29548,7 @@
         </is>
       </c>
       <c r="B5" s="27">
-        <f>COUNTA(Artikelstamm!$A$3:$A$231)</f>
+        <f>COUNTA(Artikelstamm!$A$3:$A$235)</f>
         <v/>
       </c>
     </row>
@@ -29083,7 +29559,7 @@
         </is>
       </c>
       <c r="B6" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$231,"verfügbar")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$235,"verfügbar")</f>
         <v/>
       </c>
     </row>
@@ -29094,7 +29570,7 @@
         </is>
       </c>
       <c r="B7" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$231,"reserviert")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$235,"reserviert")</f>
         <v/>
       </c>
     </row>
@@ -29105,7 +29581,7 @@
         </is>
       </c>
       <c r="B8" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$231,"teilverkauft")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$235,"teilverkauft")</f>
         <v/>
       </c>
     </row>
@@ -29116,7 +29592,7 @@
         </is>
       </c>
       <c r="B9" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$231,"verkauft")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$235,"verkauft")</f>
         <v/>
       </c>
     </row>
@@ -29127,7 +29603,7 @@
         </is>
       </c>
       <c r="B10" s="27">
-        <f>SUM(Artikelstamm!$L$3:$L$231)</f>
+        <f>SUM(Artikelstamm!$L$3:$L$235)</f>
         <v/>
       </c>
     </row>
@@ -29138,7 +29614,7 @@
         </is>
       </c>
       <c r="B11" s="29">
-        <f>SUM(Artikelstamm!$U$3:$U$231)</f>
+        <f>SUM(Artikelstamm!$U$3:$U$235)</f>
         <v/>
       </c>
     </row>
@@ -29156,7 +29632,7 @@
         </is>
       </c>
       <c r="B13" s="27">
-        <f>SUM(Artikelstamm!$K$3:$K$231)</f>
+        <f>SUM(Artikelstamm!$K$3:$K$235)</f>
         <v/>
       </c>
     </row>
@@ -29167,7 +29643,7 @@
         </is>
       </c>
       <c r="B14" s="30">
-        <f>SUMPRODUCT(Artikelstamm!$K$3:$K$231,Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT(Artikelstamm!$K$3:$K$235,Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
     </row>
@@ -29200,7 +29676,7 @@
         </is>
       </c>
       <c r="B17" s="30">
-        <f>SUMPRODUCT((Artikelstamm!$AI$3:$AI$231="bezahlt")*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AI$3:$AI$235="bezahlt")*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
     </row>
@@ -29229,7 +29705,7 @@
         </is>
       </c>
       <c r="B21" s="31">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$231,"*verkauft",Artikelstamm!$AH$3:$AH$231,"")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$235,"*verkauft",Artikelstamm!$AH$3:$AH$235,"")</f>
         <v/>
       </c>
     </row>
@@ -29240,7 +29716,7 @@
         </is>
       </c>
       <c r="B22" s="31">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$231,"*verkauft",Artikelstamm!$AI$3:$AI$231,"offen")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$235,"*verkauft",Artikelstamm!$AI$3:$AI$235,"offen")</f>
         <v/>
       </c>
     </row>
@@ -29251,7 +29727,7 @@
         </is>
       </c>
       <c r="B23" s="27">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$231,"reserviert",Artikelstamm!$AK$3:$AK$231,"")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$235,"reserviert",Artikelstamm!$AK$3:$AK$235,"")</f>
         <v/>
       </c>
     </row>
@@ -29262,7 +29738,7 @@
         </is>
       </c>
       <c r="B24" s="27">
-        <f>COUNTIFS(Artikelstamm!$S$3:$S$231,"")</f>
+        <f>COUNTIFS(Artikelstamm!$S$3:$S$235,"")</f>
         <v/>
       </c>
     </row>
@@ -29273,7 +29749,7 @@
         </is>
       </c>
       <c r="B25" s="27">
-        <f>COUNTIFS(Artikelstamm!$O$3:$O$231,"")</f>
+        <f>COUNTIFS(Artikelstamm!$O$3:$O$235,"")</f>
         <v/>
       </c>
     </row>
@@ -29313,15 +29789,15 @@
         </is>
       </c>
       <c r="B30" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$231,$A30)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$235,$A30)</f>
         <v/>
       </c>
       <c r="C30" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$231=$A30)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$235=$A30)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
       <c r="D30" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$231,$A30,Artikelstamm!$U$3:$U$231)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$235,$A30,Artikelstamm!$U$3:$U$235)</f>
         <v/>
       </c>
     </row>
@@ -29332,15 +29808,15 @@
         </is>
       </c>
       <c r="B31" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$231,$A31)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$235,$A31)</f>
         <v/>
       </c>
       <c r="C31" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$231=$A31)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$235=$A31)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
       <c r="D31" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$231,$A31,Artikelstamm!$U$3:$U$231)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$235,$A31,Artikelstamm!$U$3:$U$235)</f>
         <v/>
       </c>
     </row>
@@ -29351,15 +29827,15 @@
         </is>
       </c>
       <c r="B32" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$231,$A32)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$235,$A32)</f>
         <v/>
       </c>
       <c r="C32" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$231=$A32)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$235=$A32)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
       <c r="D32" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$231,$A32,Artikelstamm!$U$3:$U$231)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$235,$A32,Artikelstamm!$U$3:$U$235)</f>
         <v/>
       </c>
     </row>
@@ -29418,15 +29894,15 @@
         </is>
       </c>
       <c r="B37" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$231,$A37)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$235,$A37)</f>
         <v/>
       </c>
       <c r="C37" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$231=$A37)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$235=$A37)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
       <c r="D37" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$231,$A37,Artikelstamm!$U$3:$U$231)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$235,$A37,Artikelstamm!$U$3:$U$235)</f>
         <v/>
       </c>
     </row>
@@ -29437,15 +29913,15 @@
         </is>
       </c>
       <c r="B38" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$231,$A38)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$235,$A38)</f>
         <v/>
       </c>
       <c r="C38" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$231=$A38)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$235=$A38)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
       <c r="D38" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$231,$A38,Artikelstamm!$U$3:$U$231)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$235,$A38,Artikelstamm!$U$3:$U$235)</f>
         <v/>
       </c>
     </row>
@@ -29456,15 +29932,15 @@
         </is>
       </c>
       <c r="B39" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$231,$A39)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$235,$A39)</f>
         <v/>
       </c>
       <c r="C39" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$231=$A39)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$235=$A39)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
       <c r="D39" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$231,$A39,Artikelstamm!$U$3:$U$231)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$235,$A39,Artikelstamm!$U$3:$U$235)</f>
         <v/>
       </c>
     </row>
@@ -29475,15 +29951,15 @@
         </is>
       </c>
       <c r="B40" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$231,$A40)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$235,$A40)</f>
         <v/>
       </c>
       <c r="C40" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$231=$A40)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$235=$A40)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
       <c r="D40" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$231,$A40,Artikelstamm!$U$3:$U$231)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$235,$A40,Artikelstamm!$U$3:$U$235)</f>
         <v/>
       </c>
     </row>
@@ -29494,15 +29970,15 @@
         </is>
       </c>
       <c r="B41" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$231,$A41)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$235,$A41)</f>
         <v/>
       </c>
       <c r="C41" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$231=$A41)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$235=$A41)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
       <c r="D41" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$231,$A41,Artikelstamm!$U$3:$U$231)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$235,$A41,Artikelstamm!$U$3:$U$235)</f>
         <v/>
       </c>
     </row>
@@ -29513,15 +29989,15 @@
         </is>
       </c>
       <c r="B42" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$231,$A42)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$235,$A42)</f>
         <v/>
       </c>
       <c r="C42" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$231=$A42)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$235=$A42)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
       <c r="D42" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$231,$A42,Artikelstamm!$U$3:$U$231)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$235,$A42,Artikelstamm!$U$3:$U$235)</f>
         <v/>
       </c>
     </row>
@@ -29532,15 +30008,15 @@
         </is>
       </c>
       <c r="B43" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$231,$A43)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$235,$A43)</f>
         <v/>
       </c>
       <c r="C43" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$231=$A43)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$235=$A43)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
       <c r="D43" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$231,$A43,Artikelstamm!$U$3:$U$231)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$235,$A43,Artikelstamm!$U$3:$U$235)</f>
         <v/>
       </c>
     </row>
@@ -29551,15 +30027,15 @@
         </is>
       </c>
       <c r="B44" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$231,$A44)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$235,$A44)</f>
         <v/>
       </c>
       <c r="C44" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$231=$A44)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$235=$A44)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
       <c r="D44" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$231,$A44,Artikelstamm!$U$3:$U$231)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$235,$A44,Artikelstamm!$U$3:$U$235)</f>
         <v/>
       </c>
     </row>
@@ -29570,15 +30046,15 @@
         </is>
       </c>
       <c r="B45" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$231,$A45)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$235,$A45)</f>
         <v/>
       </c>
       <c r="C45" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$231=$A45)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$235=$A45)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
       <c r="D45" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$231,$A45,Artikelstamm!$U$3:$U$231)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$235,$A45,Artikelstamm!$U$3:$U$235)</f>
         <v/>
       </c>
     </row>
@@ -29589,15 +30065,15 @@
         </is>
       </c>
       <c r="B46" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$231,$A46)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$235,$A46)</f>
         <v/>
       </c>
       <c r="C46" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$231=$A46)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$235=$A46)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
       <c r="D46" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$231,$A46,Artikelstamm!$U$3:$U$231)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$235,$A46,Artikelstamm!$U$3:$U$235)</f>
         <v/>
       </c>
     </row>
@@ -29608,15 +30084,15 @@
         </is>
       </c>
       <c r="B47" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$231,$A47)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$235,$A47)</f>
         <v/>
       </c>
       <c r="C47" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$231=$A47)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$235=$A47)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
       <c r="D47" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$231,$A47,Artikelstamm!$U$3:$U$231)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$235,$A47,Artikelstamm!$U$3:$U$235)</f>
         <v/>
       </c>
     </row>
@@ -29627,15 +30103,15 @@
         </is>
       </c>
       <c r="B48" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$231,$A48)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$235,$A48)</f>
         <v/>
       </c>
       <c r="C48" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$231=$A48)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$235=$A48)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
       <c r="D48" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$231,$A48,Artikelstamm!$U$3:$U$231)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$235,$A48,Artikelstamm!$U$3:$U$235)</f>
         <v/>
       </c>
     </row>
@@ -29646,15 +30122,15 @@
         </is>
       </c>
       <c r="B49" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$231,$A49)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$235,$A49)</f>
         <v/>
       </c>
       <c r="C49" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$231=$A49)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$235=$A49)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
       <c r="D49" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$231,$A49,Artikelstamm!$U$3:$U$231)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$235,$A49,Artikelstamm!$U$3:$U$235)</f>
         <v/>
       </c>
     </row>
@@ -29665,15 +30141,15 @@
         </is>
       </c>
       <c r="B50" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$231,$A50)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$235,$A50)</f>
         <v/>
       </c>
       <c r="C50" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$231=$A50)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$235=$A50)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
       <c r="D50" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$231,$A50,Artikelstamm!$U$3:$U$231)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$235,$A50,Artikelstamm!$U$3:$U$235)</f>
         <v/>
       </c>
     </row>
@@ -29732,15 +30208,15 @@
         </is>
       </c>
       <c r="B55" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A55)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A55)</f>
         <v/>
       </c>
       <c r="C55" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A55)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A55)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
       <c r="D55" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A55,Artikelstamm!$U$3:$U$231)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A55,Artikelstamm!$U$3:$U$235)</f>
         <v/>
       </c>
     </row>
@@ -29751,15 +30227,15 @@
         </is>
       </c>
       <c r="B56" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A56)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A56)</f>
         <v/>
       </c>
       <c r="C56" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A56)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A56)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
       <c r="D56" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A56,Artikelstamm!$U$3:$U$231)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A56,Artikelstamm!$U$3:$U$235)</f>
         <v/>
       </c>
     </row>
@@ -29770,15 +30246,15 @@
         </is>
       </c>
       <c r="B57" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A57)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A57)</f>
         <v/>
       </c>
       <c r="C57" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A57)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A57)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
       <c r="D57" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A57,Artikelstamm!$U$3:$U$231)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A57,Artikelstamm!$U$3:$U$235)</f>
         <v/>
       </c>
     </row>
@@ -29789,15 +30265,15 @@
         </is>
       </c>
       <c r="B58" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A58)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A58)</f>
         <v/>
       </c>
       <c r="C58" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A58)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A58)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
       <c r="D58" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A58,Artikelstamm!$U$3:$U$231)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A58,Artikelstamm!$U$3:$U$235)</f>
         <v/>
       </c>
     </row>
@@ -29808,15 +30284,15 @@
         </is>
       </c>
       <c r="B59" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A59)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A59)</f>
         <v/>
       </c>
       <c r="C59" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A59)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A59)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
       <c r="D59" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A59,Artikelstamm!$U$3:$U$231)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A59,Artikelstamm!$U$3:$U$235)</f>
         <v/>
       </c>
     </row>
@@ -29827,15 +30303,15 @@
         </is>
       </c>
       <c r="B60" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A60)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A60)</f>
         <v/>
       </c>
       <c r="C60" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A60)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A60)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
       <c r="D60" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A60,Artikelstamm!$U$3:$U$231)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A60,Artikelstamm!$U$3:$U$235)</f>
         <v/>
       </c>
     </row>
@@ -29846,15 +30322,15 @@
         </is>
       </c>
       <c r="B61" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A61)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A61)</f>
         <v/>
       </c>
       <c r="C61" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A61)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A61)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
       <c r="D61" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A61,Artikelstamm!$U$3:$U$231)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A61,Artikelstamm!$U$3:$U$235)</f>
         <v/>
       </c>
     </row>
@@ -29865,15 +30341,15 @@
         </is>
       </c>
       <c r="B62" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A62)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A62)</f>
         <v/>
       </c>
       <c r="C62" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A62)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A62)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
       <c r="D62" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A62,Artikelstamm!$U$3:$U$231)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A62,Artikelstamm!$U$3:$U$235)</f>
         <v/>
       </c>
     </row>
@@ -29884,15 +30360,15 @@
         </is>
       </c>
       <c r="B63" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A63)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A63)</f>
         <v/>
       </c>
       <c r="C63" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A63)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A63)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
       <c r="D63" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A63,Artikelstamm!$U$3:$U$231)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A63,Artikelstamm!$U$3:$U$235)</f>
         <v/>
       </c>
     </row>
@@ -29903,15 +30379,15 @@
         </is>
       </c>
       <c r="B64" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A64)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A64)</f>
         <v/>
       </c>
       <c r="C64" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A64)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A64)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
       <c r="D64" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A64,Artikelstamm!$U$3:$U$231)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A64,Artikelstamm!$U$3:$U$235)</f>
         <v/>
       </c>
     </row>
@@ -29922,15 +30398,15 @@
         </is>
       </c>
       <c r="B65" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A65)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A65)</f>
         <v/>
       </c>
       <c r="C65" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A65)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A65)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
       <c r="D65" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A65,Artikelstamm!$U$3:$U$231)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A65,Artikelstamm!$U$3:$U$235)</f>
         <v/>
       </c>
     </row>
@@ -29941,15 +30417,15 @@
         </is>
       </c>
       <c r="B66" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A66)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A66)</f>
         <v/>
       </c>
       <c r="C66" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A66)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A66)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
       <c r="D66" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A66,Artikelstamm!$U$3:$U$231)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A66,Artikelstamm!$U$3:$U$235)</f>
         <v/>
       </c>
     </row>
@@ -29960,15 +30436,15 @@
         </is>
       </c>
       <c r="B67" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A67)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A67)</f>
         <v/>
       </c>
       <c r="C67" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A67)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A67)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
       <c r="D67" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A67,Artikelstamm!$U$3:$U$231)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A67,Artikelstamm!$U$3:$U$235)</f>
         <v/>
       </c>
     </row>
@@ -29979,15 +30455,15 @@
         </is>
       </c>
       <c r="B68" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A68)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A68)</f>
         <v/>
       </c>
       <c r="C68" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A68)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A68)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
       <c r="D68" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A68,Artikelstamm!$U$3:$U$231)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A68,Artikelstamm!$U$3:$U$235)</f>
         <v/>
       </c>
     </row>
@@ -29998,15 +30474,15 @@
         </is>
       </c>
       <c r="B69" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A69)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A69)</f>
         <v/>
       </c>
       <c r="C69" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A69)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A69)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
       <c r="D69" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A69,Artikelstamm!$U$3:$U$231)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A69,Artikelstamm!$U$3:$U$235)</f>
         <v/>
       </c>
     </row>
@@ -30017,15 +30493,15 @@
         </is>
       </c>
       <c r="B70" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A70)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A70)</f>
         <v/>
       </c>
       <c r="C70" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A70)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A70)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
       <c r="D70" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A70,Artikelstamm!$U$3:$U$231)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A70,Artikelstamm!$U$3:$U$235)</f>
         <v/>
       </c>
     </row>
@@ -30036,15 +30512,15 @@
         </is>
       </c>
       <c r="B71" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A71)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A71)</f>
         <v/>
       </c>
       <c r="C71" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A71)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A71)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
       <c r="D71" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A71,Artikelstamm!$U$3:$U$231)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A71,Artikelstamm!$U$3:$U$235)</f>
         <v/>
       </c>
     </row>
@@ -30055,15 +30531,15 @@
         </is>
       </c>
       <c r="B72" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A72)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A72)</f>
         <v/>
       </c>
       <c r="C72" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A72)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A72)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
       <c r="D72" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A72,Artikelstamm!$U$3:$U$231)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A72,Artikelstamm!$U$3:$U$235)</f>
         <v/>
       </c>
     </row>
@@ -30074,15 +30550,15 @@
         </is>
       </c>
       <c r="B73" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A73)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A73)</f>
         <v/>
       </c>
       <c r="C73" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A73)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A73)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
       <c r="D73" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A73,Artikelstamm!$U$3:$U$231)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A73,Artikelstamm!$U$3:$U$235)</f>
         <v/>
       </c>
     </row>
@@ -30093,15 +30569,15 @@
         </is>
       </c>
       <c r="B74" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A74)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A74)</f>
         <v/>
       </c>
       <c r="C74" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A74)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A74)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
       <c r="D74" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A74,Artikelstamm!$U$3:$U$231)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A74,Artikelstamm!$U$3:$U$235)</f>
         <v/>
       </c>
     </row>
@@ -30112,15 +30588,15 @@
         </is>
       </c>
       <c r="B75" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A75)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A75)</f>
         <v/>
       </c>
       <c r="C75" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A75)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A75)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
       <c r="D75" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A75,Artikelstamm!$U$3:$U$231)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A75,Artikelstamm!$U$3:$U$235)</f>
         <v/>
       </c>
     </row>
@@ -30131,15 +30607,15 @@
         </is>
       </c>
       <c r="B76" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$231,$A76)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A76)</f>
         <v/>
       </c>
       <c r="C76" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$231=$A76)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A76)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
       <c r="D76" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$231,$A76,Artikelstamm!$U$3:$U$231)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A76,Artikelstamm!$U$3:$U$235)</f>
         <v/>
       </c>
     </row>
@@ -30193,11 +30669,11 @@
         </is>
       </c>
       <c r="B81" s="33">
-        <f>COUNTIF(Artikelstamm!$AB$3:$AB$231,$A81)</f>
+        <f>COUNTIF(Artikelstamm!$AB$3:$AB$235,$A81)</f>
         <v/>
       </c>
       <c r="C81" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AB$3:$AB$231=$A81)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AB$3:$AB$235=$A81)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
     </row>
@@ -30208,11 +30684,11 @@
         </is>
       </c>
       <c r="B82" s="33">
-        <f>COUNTIF(Artikelstamm!$AB$3:$AB$231,$A82)</f>
+        <f>COUNTIF(Artikelstamm!$AB$3:$AB$235,$A82)</f>
         <v/>
       </c>
       <c r="C82" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AB$3:$AB$231=$A82)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AB$3:$AB$235=$A82)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
     </row>
@@ -30223,11 +30699,11 @@
         </is>
       </c>
       <c r="B83" s="33">
-        <f>COUNTIF(Artikelstamm!$AB$3:$AB$231,$A83)</f>
+        <f>COUNTIF(Artikelstamm!$AB$3:$AB$235,$A83)</f>
         <v/>
       </c>
       <c r="C83" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AB$3:$AB$231=$A83)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AB$3:$AB$235=$A83)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
     </row>
@@ -30238,11 +30714,11 @@
         </is>
       </c>
       <c r="B84" s="33">
-        <f>COUNTIF(Artikelstamm!$AB$3:$AB$231,$A84)</f>
+        <f>COUNTIF(Artikelstamm!$AB$3:$AB$235,$A84)</f>
         <v/>
       </c>
       <c r="C84" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AB$3:$AB$231=$A84)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AB$3:$AB$235=$A84)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
     </row>
@@ -30253,11 +30729,11 @@
         </is>
       </c>
       <c r="B85" s="33">
-        <f>COUNTIF(Artikelstamm!$AB$3:$AB$231,$A85)</f>
+        <f>COUNTIF(Artikelstamm!$AB$3:$AB$235,$A85)</f>
         <v/>
       </c>
       <c r="C85" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AB$3:$AB$231=$A85)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AB$3:$AB$235=$A85)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
     </row>
@@ -30268,11 +30744,11 @@
         </is>
       </c>
       <c r="B86" s="33">
-        <f>COUNTIF(Artikelstamm!$AB$3:$AB$231,$A86)</f>
+        <f>COUNTIF(Artikelstamm!$AB$3:$AB$235,$A86)</f>
         <v/>
       </c>
       <c r="C86" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AB$3:$AB$231=$A86)*Artikelstamm!$K$3:$K$231*Artikelstamm!$AD$3:$AD$231)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AB$3:$AB$235=$A86)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
BA01-03 vollstaendig: Deko-Tannen, 3 Stueck statt 1
Foto F-262 nachgereicht. Es sind drei Sockel, unterschiedlich bestueckt:
einer mit einem grossen Baum, zwei mit je drei. Menge deshalb von 1 auf 3,
Im_Katalog wieder auf ja, der OFFEN-Vermerk ist weg.

Es sind dieselben Stuecke, die in NE01 als NE01-15 gefuehrt und dort
durchgestrichen waren - sie sind in den Flur 1 umgezogen. Beide Zeilen
verweisen jetzt in der Bemerkung aufeinander, NE01-15 bleibt auf
Aktiv=entfaellt.

Dabei hat die neue Pruefung angeschlagen: NE01-15 in Weitere_ArtNr wurde
beanstandet, weil die Nummer zugleich eine eigene Zeile hat.
Weitere_ArtNr ist fuer Post-it-Nummern ohne eigene Zeile gedacht - der
Verweis gehoert in die Bemerkung. So eingetragen.

Gesamtwert netto 35.942 -> 35.992 EUR, 177 aktive Positionen.
pruefen.py: 0 Fehler, 3 Hinweise.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011yyfqhuiWGsaNy38oaNoGo
</commit_message>
<xml_diff>
--- a/ausgabe/01_Artikelstamm_kikripp.xlsx
+++ b/ausgabe/01_Artikelstamm_kikripp.xlsx
@@ -14307,7 +14307,7 @@
       </c>
       <c r="AM110" s="22" t="inlineStr">
         <is>
-          <t>Auf dem Erfassungsblatt NE01 durchgestrichen – entfaellt.</t>
+          <t>Auf dem Erfassungsblatt NE01 durchgestrichen - die Stuecke stehen jetzt im Flur 1 und werden dort als BA01-03 gefuehrt.</t>
         </is>
       </c>
     </row>
@@ -29209,12 +29209,12 @@
       </c>
       <c r="E234" s="15" t="inlineStr">
         <is>
-          <t>Tannen-Dekoration</t>
+          <t>Deko-Tannen Metall auf Holzsockel</t>
         </is>
       </c>
       <c r="F234" s="16" t="inlineStr">
         <is>
-          <t>Dekoration in Tannenform.</t>
+          <t>Stilisierte Tannen aus schwarz mattiertem Metall, auf ovalen Sockeln aus Massivholz. Skandinavischer Stil, standfest.</t>
         </is>
       </c>
       <c r="G234" s="15" t="inlineStr">
@@ -29233,7 +29233,7 @@
         </is>
       </c>
       <c r="J234" s="17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K234" s="17" t="n"/>
       <c r="L234" s="18">
@@ -29247,7 +29247,7 @@
       </c>
       <c r="N234" s="15" t="inlineStr">
         <is>
-          <t>gebraucht</t>
+          <t>gut</t>
         </is>
       </c>
       <c r="O234" s="19" t="n"/>
@@ -29272,13 +29272,17 @@
       </c>
       <c r="V234" s="15" t="inlineStr">
         <is>
-          <t>nur Abholung</t>
-        </is>
-      </c>
-      <c r="W234" s="15" t="n"/>
+          <t>Versand möglich</t>
+        </is>
+      </c>
+      <c r="W234" s="15" t="inlineStr">
+        <is>
+          <t>F-262</t>
+        </is>
+      </c>
       <c r="X234" s="19" t="inlineStr">
         <is>
-          <t>nein</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="Y234" s="19" t="n"/>
@@ -29303,12 +29307,12 @@
       <c r="AK234" s="19" t="n"/>
       <c r="AL234" s="16" t="inlineStr">
         <is>
-          <t>1 Stück.</t>
+          <t>3 Sockel, unterschiedlich bestückt: einer mit einem großen Baum, zwei mit je drei Bäumen. Alle drei sind abgebildet.</t>
         </is>
       </c>
       <c r="AM234" s="22" t="inlineStr">
         <is>
-          <t>OFFEN: Foto fehlt - IMG_2291 ist nicht angekommen. Beschreibung und Preis sind daher vorlaeufig. Moeglicherweise dieselben Stuecke wie NE01-15 (Deko-Tannenbaum schwarz, 3 Stueck), die dort durchgestrichen wurden.</t>
+          <t>Bisher unter NE01-15 gefuehrt; dort durchgestrichen, weil sie in den Flur 1 umgezogen sind.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
BA02 erfasst: 8 Positionen, sechste Zusammenfassung
Flur 2 (Bestandsgebaeude Attika, 10,17 m2). Das Raumschild fehlt auf den
Fotos, ist aber entbehrlich - die Post-its tragen die Nummer.

BA02-01 (Kindergarderobe weiss, 5 Stueck) hat kein Foto bekommen und
steht deshalb auf Im_Katalog=nein mit OFFEN-Vermerk. Mit 450 EUR waere
das die groesste Position des Raums. Moeglicherweise baugleich mit einer
der schon erfassten Garderoben - das entscheidet erst das Foto.

BA02-07 ist derselbe Leuchtbuchstabe K wie BA01-04; zusammengefasst auf
2 Stueck, BA02-07 in Weitere_ArtNr.

BA02-04 ist der graue Zwilling der roten Kinder-Ohrensessel NE01-20. Die
Farbe unterscheidet sie, deshalb getrennte Positionen mit gegenseitigem
Verweis im Mengenhinweis.

Gesamtwert netto 35.992 -> 37.002 EUR, 185 aktive Positionen.
pruefen.py: 0 Fehler, 4 Hinweise.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011yyfqhuiWGsaNy38oaNoGo
</commit_message>
<xml_diff>
--- a/ausgabe/01_Artikelstamm_kikripp.xlsx
+++ b/ausgabe/01_Artikelstamm_kikripp.xlsx
@@ -15,7 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Artikelstamm'!$A$2:$AM$235</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Artikelstamm'!$A$2:$AM$243</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1019,7 +1019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AM235"/>
+  <dimension ref="A1:AM243"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -29323,7 +29323,11 @@
         </is>
       </c>
       <c r="B235" s="15" t="n"/>
-      <c r="C235" s="15" t="n"/>
+      <c r="C235" s="15" t="inlineStr">
+        <is>
+          <t>BA02-07</t>
+        </is>
+      </c>
       <c r="D235" s="15" t="inlineStr">
         <is>
           <t>BA01</t>
@@ -29355,7 +29359,7 @@
         </is>
       </c>
       <c r="J235" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K235" s="17" t="n"/>
       <c r="L235" s="18">
@@ -29429,13 +29433,961 @@
       <c r="AK235" s="19" t="n"/>
       <c r="AL235" s="16" t="inlineStr">
         <is>
-          <t>1 Stück.</t>
-        </is>
-      </c>
-      <c r="AM235" s="22" t="n"/>
+          <t>2 Buchstaben: einer im Flur 1 (BA01-04) und einer im Flur 2 (dort mit BA02-07 beschriftet).</t>
+        </is>
+      </c>
+      <c r="AM235" s="22" t="inlineStr">
+        <is>
+          <t>Zusammengefasste Position – Post-it-Nummer im zweiten Raum: BA02-07.</t>
+        </is>
+      </c>
+    </row>
+    <row r="236" ht="30" customHeight="1">
+      <c r="A236" s="15" t="inlineStr">
+        <is>
+          <t>BA02-01</t>
+        </is>
+      </c>
+      <c r="B236" s="15" t="n"/>
+      <c r="C236" s="15" t="n"/>
+      <c r="D236" s="15" t="inlineStr">
+        <is>
+          <t>BA02</t>
+        </is>
+      </c>
+      <c r="E236" s="15" t="inlineStr">
+        <is>
+          <t>Kindergarderobe weiß</t>
+        </is>
+      </c>
+      <c r="F236" s="16" t="inlineStr">
+        <is>
+          <t>Kindergarderobe in Weiß.</t>
+        </is>
+      </c>
+      <c r="G236" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H236" s="15" t="inlineStr">
+        <is>
+          <t>Flur 2</t>
+        </is>
+      </c>
+      <c r="I236" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J236" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="K236" s="17" t="n"/>
+      <c r="L236" s="18">
+        <f>J236-IF(K236="",0,K236)</f>
+        <v/>
+      </c>
+      <c r="M236" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N236" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O236" s="19" t="n"/>
+      <c r="P236" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q236" s="19" t="n"/>
+      <c r="R236" s="20" t="n"/>
+      <c r="S236" s="20" t="n">
+        <v>90</v>
+      </c>
+      <c r="T236" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U236" s="21">
+        <f>L236*S236</f>
+        <v/>
+      </c>
+      <c r="V236" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W236" s="15" t="n"/>
+      <c r="X236" s="19" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="Y236" s="19" t="n"/>
+      <c r="Z236" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA236" s="19" t="n"/>
+      <c r="AB236" s="19" t="n"/>
+      <c r="AC236" s="19" t="n"/>
+      <c r="AD236" s="20" t="n"/>
+      <c r="AE236" s="21">
+        <f>IF(K236="","",K236*AD236)</f>
+        <v/>
+      </c>
+      <c r="AF236" s="19" t="n"/>
+      <c r="AG236" s="19" t="n"/>
+      <c r="AH236" s="19" t="n"/>
+      <c r="AI236" s="19" t="n"/>
+      <c r="AJ236" s="19" t="n"/>
+      <c r="AK236" s="19" t="n"/>
+      <c r="AL236" s="16" t="inlineStr">
+        <is>
+          <t>5 Stück.</t>
+        </is>
+      </c>
+      <c r="AM236" s="22" t="inlineStr">
+        <is>
+          <t>OFFEN: Foto fehlt - zu BA02-01 ist kein Bild angekommen. Beschreibung und Preis sind daher vorlaeufig. Moeglicherweise baugleich mit einer der bereits erfassten Garderoben (NU01-14, NU01-19, NU06-01/-02) - dann zusammenfassen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="237" ht="30" customHeight="1">
+      <c r="A237" s="15" t="inlineStr">
+        <is>
+          <t>BA02-02</t>
+        </is>
+      </c>
+      <c r="B237" s="15" t="n"/>
+      <c r="C237" s="15" t="n"/>
+      <c r="D237" s="15" t="inlineStr">
+        <is>
+          <t>BA02</t>
+        </is>
+      </c>
+      <c r="E237" s="15" t="inlineStr">
+        <is>
+          <t>Rutscherauto rot</t>
+        </is>
+      </c>
+      <c r="F237" s="16" t="inlineStr">
+        <is>
+          <t>Rutscherauto in Sportwagenform, roter Kunststoffkorpus mit schwarzer Sitzfläche in Rautensteppung, verchromte Felgen, Lehne hinten zum Schieben.</t>
+        </is>
+      </c>
+      <c r="G237" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H237" s="15" t="inlineStr">
+        <is>
+          <t>Flur 2</t>
+        </is>
+      </c>
+      <c r="I237" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J237" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K237" s="17" t="n"/>
+      <c r="L237" s="18">
+        <f>J237-IF(K237="",0,K237)</f>
+        <v/>
+      </c>
+      <c r="M237" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N237" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O237" s="19" t="n"/>
+      <c r="P237" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q237" s="19" t="n"/>
+      <c r="R237" s="20" t="n"/>
+      <c r="S237" s="20" t="n">
+        <v>35</v>
+      </c>
+      <c r="T237" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U237" s="21">
+        <f>L237*S237</f>
+        <v/>
+      </c>
+      <c r="V237" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W237" s="15" t="inlineStr">
+        <is>
+          <t>F-263</t>
+        </is>
+      </c>
+      <c r="X237" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y237" s="19" t="n"/>
+      <c r="Z237" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA237" s="19" t="n"/>
+      <c r="AB237" s="19" t="n"/>
+      <c r="AC237" s="19" t="n"/>
+      <c r="AD237" s="20" t="n"/>
+      <c r="AE237" s="21">
+        <f>IF(K237="","",K237*AD237)</f>
+        <v/>
+      </c>
+      <c r="AF237" s="19" t="n"/>
+      <c r="AG237" s="19" t="n"/>
+      <c r="AH237" s="19" t="n"/>
+      <c r="AI237" s="19" t="n"/>
+      <c r="AJ237" s="19" t="n"/>
+      <c r="AK237" s="19" t="n"/>
+      <c r="AL237" s="16" t="inlineStr">
+        <is>
+          <t>1 Fahrzeug.</t>
+        </is>
+      </c>
+      <c r="AM237" s="22" t="n"/>
+    </row>
+    <row r="238" ht="30" customHeight="1">
+      <c r="A238" s="15" t="inlineStr">
+        <is>
+          <t>BA02-03</t>
+        </is>
+      </c>
+      <c r="B238" s="15" t="n"/>
+      <c r="C238" s="15" t="n"/>
+      <c r="D238" s="15" t="inlineStr">
+        <is>
+          <t>BA02</t>
+        </is>
+      </c>
+      <c r="E238" s="15" t="inlineStr">
+        <is>
+          <t>Bilder Schwarzwald, gerahmt</t>
+        </is>
+      </c>
+      <c r="F238" s="16" t="inlineStr">
+        <is>
+          <t>Schwarz gerahmte Zeichnungen hinter Glas in schlichter Strichtechnik: Bergkette, Mädchen mit Bollenhut und Tannenwald. Motivgruppe Schwarzwald.</t>
+        </is>
+      </c>
+      <c r="G238" s="15" t="inlineStr">
+        <is>
+          <t>Kunst</t>
+        </is>
+      </c>
+      <c r="H238" s="15" t="inlineStr">
+        <is>
+          <t>Flur 2</t>
+        </is>
+      </c>
+      <c r="I238" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J238" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="K238" s="17" t="n"/>
+      <c r="L238" s="18">
+        <f>J238-IF(K238="",0,K238)</f>
+        <v/>
+      </c>
+      <c r="M238" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N238" s="15" t="inlineStr">
+        <is>
+          <t>gut</t>
+        </is>
+      </c>
+      <c r="O238" s="19" t="n"/>
+      <c r="P238" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q238" s="19" t="n"/>
+      <c r="R238" s="20" t="n"/>
+      <c r="S238" s="20" t="n">
+        <v>45</v>
+      </c>
+      <c r="T238" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U238" s="21">
+        <f>L238*S238</f>
+        <v/>
+      </c>
+      <c r="V238" s="15" t="inlineStr">
+        <is>
+          <t>Versand möglich</t>
+        </is>
+      </c>
+      <c r="W238" s="15" t="inlineStr">
+        <is>
+          <t>F-264</t>
+        </is>
+      </c>
+      <c r="X238" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y238" s="19" t="n"/>
+      <c r="Z238" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA238" s="19" t="n"/>
+      <c r="AB238" s="19" t="n"/>
+      <c r="AC238" s="19" t="n"/>
+      <c r="AD238" s="20" t="n"/>
+      <c r="AE238" s="21">
+        <f>IF(K238="","",K238*AD238)</f>
+        <v/>
+      </c>
+      <c r="AF238" s="19" t="n"/>
+      <c r="AG238" s="19" t="n"/>
+      <c r="AH238" s="19" t="n"/>
+      <c r="AI238" s="19" t="n"/>
+      <c r="AJ238" s="19" t="n"/>
+      <c r="AK238" s="19" t="n"/>
+      <c r="AL238" s="16" t="inlineStr">
+        <is>
+          <t>3 Bilder, alle abgebildet.</t>
+        </is>
+      </c>
+      <c r="AM238" s="22" t="n"/>
+    </row>
+    <row r="239" ht="30" customHeight="1">
+      <c r="A239" s="15" t="inlineStr">
+        <is>
+          <t>BA02-04</t>
+        </is>
+      </c>
+      <c r="B239" s="15" t="n"/>
+      <c r="C239" s="15" t="n"/>
+      <c r="D239" s="15" t="inlineStr">
+        <is>
+          <t>BA02</t>
+        </is>
+      </c>
+      <c r="E239" s="15" t="inlineStr">
+        <is>
+          <t>Kinder-Ohrensessel grau, Kunstleder</t>
+        </is>
+      </c>
+      <c r="F239" s="16" t="inlineStr">
+        <is>
+          <t>Ohrensessel in Kindergröße, hellgrauer Kunstlederbezug, geschwungene schwarze Holzbeine.</t>
+        </is>
+      </c>
+      <c r="G239" s="15" t="inlineStr">
+        <is>
+          <t>Möbel</t>
+        </is>
+      </c>
+      <c r="H239" s="15" t="inlineStr">
+        <is>
+          <t>Flur 2</t>
+        </is>
+      </c>
+      <c r="I239" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J239" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K239" s="17" t="n"/>
+      <c r="L239" s="18">
+        <f>J239-IF(K239="",0,K239)</f>
+        <v/>
+      </c>
+      <c r="M239" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N239" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O239" s="19" t="n"/>
+      <c r="P239" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q239" s="19" t="n"/>
+      <c r="R239" s="20" t="n"/>
+      <c r="S239" s="20" t="n">
+        <v>55</v>
+      </c>
+      <c r="T239" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U239" s="21">
+        <f>L239*S239</f>
+        <v/>
+      </c>
+      <c r="V239" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W239" s="15" t="inlineStr">
+        <is>
+          <t>F-265</t>
+        </is>
+      </c>
+      <c r="X239" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y239" s="19" t="n"/>
+      <c r="Z239" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA239" s="19" t="n"/>
+      <c r="AB239" s="19" t="n"/>
+      <c r="AC239" s="19" t="n"/>
+      <c r="AD239" s="20" t="n"/>
+      <c r="AE239" s="21">
+        <f>IF(K239="","",K239*AD239)</f>
+        <v/>
+      </c>
+      <c r="AF239" s="19" t="n"/>
+      <c r="AG239" s="19" t="n"/>
+      <c r="AH239" s="19" t="n"/>
+      <c r="AI239" s="19" t="n"/>
+      <c r="AJ239" s="19" t="n"/>
+      <c r="AK239" s="19" t="n"/>
+      <c r="AL239" s="16" t="inlineStr">
+        <is>
+          <t>1 Sessel. Baugleich in Rot gibt es zwei Stück unter NE01-20.</t>
+        </is>
+      </c>
+      <c r="AM239" s="22" t="n"/>
+    </row>
+    <row r="240" ht="30" customHeight="1">
+      <c r="A240" s="15" t="inlineStr">
+        <is>
+          <t>BA02-05</t>
+        </is>
+      </c>
+      <c r="B240" s="15" t="n"/>
+      <c r="C240" s="15" t="n"/>
+      <c r="D240" s="15" t="inlineStr">
+        <is>
+          <t>BA02</t>
+        </is>
+      </c>
+      <c r="E240" s="15" t="inlineStr">
+        <is>
+          <t>Ablagepult Holz auf Metallgestell</t>
+        </is>
+      </c>
+      <c r="F240" s="16" t="inlineStr">
+        <is>
+          <t>Pult mit geneigter Platte aus dunklem Holz mit schwarzer Auflage, auf einem C-förmigen schwarzen Metallgestell. Untergreifbar, im Haus als Stehpult für die Anwesenheitsliste genutzt.</t>
+        </is>
+      </c>
+      <c r="G240" s="15" t="inlineStr">
+        <is>
+          <t>Möbel</t>
+        </is>
+      </c>
+      <c r="H240" s="15" t="inlineStr">
+        <is>
+          <t>Flur 2</t>
+        </is>
+      </c>
+      <c r="I240" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J240" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K240" s="17" t="n"/>
+      <c r="L240" s="18">
+        <f>J240-IF(K240="",0,K240)</f>
+        <v/>
+      </c>
+      <c r="M240" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N240" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O240" s="19" t="n"/>
+      <c r="P240" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q240" s="19" t="n"/>
+      <c r="R240" s="20" t="n"/>
+      <c r="S240" s="20" t="n">
+        <v>45</v>
+      </c>
+      <c r="T240" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U240" s="21">
+        <f>L240*S240</f>
+        <v/>
+      </c>
+      <c r="V240" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W240" s="15" t="inlineStr">
+        <is>
+          <t>F-266</t>
+        </is>
+      </c>
+      <c r="X240" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y240" s="19" t="n"/>
+      <c r="Z240" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA240" s="19" t="n"/>
+      <c r="AB240" s="19" t="n"/>
+      <c r="AC240" s="19" t="n"/>
+      <c r="AD240" s="20" t="n"/>
+      <c r="AE240" s="21">
+        <f>IF(K240="","",K240*AD240)</f>
+        <v/>
+      </c>
+      <c r="AF240" s="19" t="n"/>
+      <c r="AG240" s="19" t="n"/>
+      <c r="AH240" s="19" t="n"/>
+      <c r="AI240" s="19" t="n"/>
+      <c r="AJ240" s="19" t="n"/>
+      <c r="AK240" s="19" t="n"/>
+      <c r="AL240" s="16" t="inlineStr">
+        <is>
+          <t>1 Pult. Die Liste gehört nicht dazu.</t>
+        </is>
+      </c>
+      <c r="AM240" s="22" t="n"/>
+    </row>
+    <row r="241" ht="30" customHeight="1">
+      <c r="A241" s="15" t="inlineStr">
+        <is>
+          <t>BA02-06</t>
+        </is>
+      </c>
+      <c r="B241" s="15" t="n"/>
+      <c r="C241" s="15" t="n"/>
+      <c r="D241" s="15" t="inlineStr">
+        <is>
+          <t>BA02</t>
+        </is>
+      </c>
+      <c r="E241" s="15" t="inlineStr">
+        <is>
+          <t>Truhenbank weiß mit Fellauflage</t>
+        </is>
+      </c>
+      <c r="F241" s="16" t="inlineStr">
+        <is>
+          <t>Sitzbank in Weiß mit geschwungenen Seitenteilen, Rückenbrett und aufklappbarer Sitzfläche mit Beschlägen. Darunter ein großer Stauraum. Eine weiße Fellauflage liegt auf der Sitzfläche.</t>
+        </is>
+      </c>
+      <c r="G241" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H241" s="15" t="inlineStr">
+        <is>
+          <t>Flur 2</t>
+        </is>
+      </c>
+      <c r="I241" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J241" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K241" s="17" t="n"/>
+      <c r="L241" s="18">
+        <f>J241-IF(K241="",0,K241)</f>
+        <v/>
+      </c>
+      <c r="M241" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N241" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O241" s="19" t="n"/>
+      <c r="P241" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q241" s="19" t="n"/>
+      <c r="R241" s="20" t="n"/>
+      <c r="S241" s="20" t="n">
+        <v>45</v>
+      </c>
+      <c r="T241" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U241" s="21">
+        <f>L241*S241</f>
+        <v/>
+      </c>
+      <c r="V241" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W241" s="15" t="inlineStr">
+        <is>
+          <t>F-267</t>
+        </is>
+      </c>
+      <c r="X241" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y241" s="19" t="n"/>
+      <c r="Z241" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA241" s="19" t="n"/>
+      <c r="AB241" s="19" t="n"/>
+      <c r="AC241" s="19" t="n"/>
+      <c r="AD241" s="20" t="n"/>
+      <c r="AE241" s="21">
+        <f>IF(K241="","",K241*AD241)</f>
+        <v/>
+      </c>
+      <c r="AF241" s="19" t="n"/>
+      <c r="AG241" s="19" t="n"/>
+      <c r="AH241" s="19" t="n"/>
+      <c r="AI241" s="19" t="n"/>
+      <c r="AJ241" s="19" t="n"/>
+      <c r="AK241" s="19" t="n"/>
+      <c r="AL241" s="16" t="inlineStr">
+        <is>
+          <t>1 Bank einschließlich der Fellauflage. Der Inhalt gehört nicht dazu.</t>
+        </is>
+      </c>
+      <c r="AM241" s="22" t="n"/>
+    </row>
+    <row r="242" ht="30" customHeight="1">
+      <c r="A242" s="15" t="inlineStr">
+        <is>
+          <t>BA02-08</t>
+        </is>
+      </c>
+      <c r="B242" s="15" t="n"/>
+      <c r="C242" s="15" t="n"/>
+      <c r="D242" s="15" t="inlineStr">
+        <is>
+          <t>BA02</t>
+        </is>
+      </c>
+      <c r="E242" s="15" t="inlineStr">
+        <is>
+          <t>Kinderschrank weiß mit Handabdrücken</t>
+        </is>
+      </c>
+      <c r="F242" s="16" t="inlineStr">
+        <is>
+          <t>Hoher Schrank in Weiß mit Türen und Schubladen, Griffmulden. Auf den Fronten kleben Aufkleber mit Kinderhandabdrücken in Schwarz und Rot; sie lassen sich abziehen.</t>
+        </is>
+      </c>
+      <c r="G242" s="15" t="inlineStr">
+        <is>
+          <t>Möbel</t>
+        </is>
+      </c>
+      <c r="H242" s="15" t="inlineStr">
+        <is>
+          <t>Flur 2</t>
+        </is>
+      </c>
+      <c r="I242" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J242" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K242" s="17" t="n"/>
+      <c r="L242" s="18">
+        <f>J242-IF(K242="",0,K242)</f>
+        <v/>
+      </c>
+      <c r="M242" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N242" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O242" s="19" t="n"/>
+      <c r="P242" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q242" s="19" t="n"/>
+      <c r="R242" s="20" t="n"/>
+      <c r="S242" s="20" t="n">
+        <v>90</v>
+      </c>
+      <c r="T242" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U242" s="21">
+        <f>L242*S242</f>
+        <v/>
+      </c>
+      <c r="V242" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W242" s="15" t="inlineStr">
+        <is>
+          <t>F-269</t>
+        </is>
+      </c>
+      <c r="X242" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y242" s="19" t="n"/>
+      <c r="Z242" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA242" s="19" t="n"/>
+      <c r="AB242" s="19" t="n"/>
+      <c r="AC242" s="19" t="n"/>
+      <c r="AD242" s="20" t="n"/>
+      <c r="AE242" s="21">
+        <f>IF(K242="","",K242*AD242)</f>
+        <v/>
+      </c>
+      <c r="AF242" s="19" t="n"/>
+      <c r="AG242" s="19" t="n"/>
+      <c r="AH242" s="19" t="n"/>
+      <c r="AI242" s="19" t="n"/>
+      <c r="AJ242" s="19" t="n"/>
+      <c r="AK242" s="19" t="n"/>
+      <c r="AL242" s="16" t="inlineStr">
+        <is>
+          <t>2 Schränke – abgebildet ist einer davon.</t>
+        </is>
+      </c>
+      <c r="AM242" s="22" t="n"/>
+    </row>
+    <row r="243" ht="30" customHeight="1">
+      <c r="A243" s="15" t="inlineStr">
+        <is>
+          <t>BA02-09</t>
+        </is>
+      </c>
+      <c r="B243" s="15" t="n"/>
+      <c r="C243" s="15" t="n"/>
+      <c r="D243" s="15" t="inlineStr">
+        <is>
+          <t>BA02</t>
+        </is>
+      </c>
+      <c r="E243" s="15" t="inlineStr">
+        <is>
+          <t>Deko-Häuser Keramik</t>
+        </is>
+      </c>
+      <c r="F243" s="16" t="inlineStr">
+        <is>
+          <t>Drei Häuschen aus Keramik mit ausgestanzten Fenstern, zum Beleuchten mit einem Teelicht: eines craquelé-grau, eines cremeweiß glasiert, eines dunkelgrau mit rundem Fenster.</t>
+        </is>
+      </c>
+      <c r="G243" s="15" t="inlineStr">
+        <is>
+          <t>Deko</t>
+        </is>
+      </c>
+      <c r="H243" s="15" t="inlineStr">
+        <is>
+          <t>Flur 2</t>
+        </is>
+      </c>
+      <c r="I243" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J243" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="K243" s="17" t="n"/>
+      <c r="L243" s="18">
+        <f>J243-IF(K243="",0,K243)</f>
+        <v/>
+      </c>
+      <c r="M243" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N243" s="15" t="inlineStr">
+        <is>
+          <t>gut</t>
+        </is>
+      </c>
+      <c r="O243" s="19" t="n"/>
+      <c r="P243" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q243" s="19" t="n"/>
+      <c r="R243" s="20" t="n"/>
+      <c r="S243" s="20" t="n">
+        <v>15</v>
+      </c>
+      <c r="T243" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U243" s="21">
+        <f>L243*S243</f>
+        <v/>
+      </c>
+      <c r="V243" s="15" t="inlineStr">
+        <is>
+          <t>Versand möglich</t>
+        </is>
+      </c>
+      <c r="W243" s="15" t="inlineStr">
+        <is>
+          <t>F-270</t>
+        </is>
+      </c>
+      <c r="X243" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y243" s="19" t="n"/>
+      <c r="Z243" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA243" s="19" t="n"/>
+      <c r="AB243" s="19" t="n"/>
+      <c r="AC243" s="19" t="n"/>
+      <c r="AD243" s="20" t="n"/>
+      <c r="AE243" s="21">
+        <f>IF(K243="","",K243*AD243)</f>
+        <v/>
+      </c>
+      <c r="AF243" s="19" t="n"/>
+      <c r="AG243" s="19" t="n"/>
+      <c r="AH243" s="19" t="n"/>
+      <c r="AI243" s="19" t="n"/>
+      <c r="AJ243" s="19" t="n"/>
+      <c r="AK243" s="19" t="n"/>
+      <c r="AL243" s="16" t="inlineStr">
+        <is>
+          <t>3 Häuschen, alle abgebildet.</t>
+        </is>
+      </c>
+      <c r="AM243" s="22" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:AM235"/>
+  <autoFilter ref="A2:AM243"/>
   <mergeCells count="7">
     <mergeCell ref="AH1:AK1"/>
     <mergeCell ref="S1:U1"/>
@@ -29445,7 +30397,7 @@
     <mergeCell ref="AL1:AM1"/>
     <mergeCell ref="AD1:AG1"/>
   </mergeCells>
-  <conditionalFormatting sqref="Z3:Z235">
+  <conditionalFormatting sqref="Z3:Z243">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"reserviert"</formula>
     </cfRule>
@@ -29456,12 +30408,12 @@
       <formula>"verkauft"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I3:I235">
+  <conditionalFormatting sqref="I3:I243">
     <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
       <formula>"A"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P3:P235">
+  <conditionalFormatting sqref="P3:P243">
     <cfRule type="cellIs" priority="5" operator="equal" dxfId="4">
       <formula>"entfällt"</formula>
     </cfRule>
@@ -29514,7 +30466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D87"/>
+  <dimension ref="A1:D88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -29552,7 +30504,7 @@
         </is>
       </c>
       <c r="B5" s="27">
-        <f>COUNTA(Artikelstamm!$A$3:$A$235)</f>
+        <f>COUNTA(Artikelstamm!$A$3:$A$243)</f>
         <v/>
       </c>
     </row>
@@ -29563,7 +30515,7 @@
         </is>
       </c>
       <c r="B6" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$235,"verfügbar")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$243,"verfügbar")</f>
         <v/>
       </c>
     </row>
@@ -29574,7 +30526,7 @@
         </is>
       </c>
       <c r="B7" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$235,"reserviert")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$243,"reserviert")</f>
         <v/>
       </c>
     </row>
@@ -29585,7 +30537,7 @@
         </is>
       </c>
       <c r="B8" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$235,"teilverkauft")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$243,"teilverkauft")</f>
         <v/>
       </c>
     </row>
@@ -29596,7 +30548,7 @@
         </is>
       </c>
       <c r="B9" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$235,"verkauft")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$243,"verkauft")</f>
         <v/>
       </c>
     </row>
@@ -29607,7 +30559,7 @@
         </is>
       </c>
       <c r="B10" s="27">
-        <f>SUM(Artikelstamm!$L$3:$L$235)</f>
+        <f>SUM(Artikelstamm!$L$3:$L$243)</f>
         <v/>
       </c>
     </row>
@@ -29618,7 +30570,7 @@
         </is>
       </c>
       <c r="B11" s="29">
-        <f>SUM(Artikelstamm!$U$3:$U$235)</f>
+        <f>SUM(Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -29636,7 +30588,7 @@
         </is>
       </c>
       <c r="B13" s="27">
-        <f>SUM(Artikelstamm!$K$3:$K$235)</f>
+        <f>SUM(Artikelstamm!$K$3:$K$243)</f>
         <v/>
       </c>
     </row>
@@ -29647,7 +30599,7 @@
         </is>
       </c>
       <c r="B14" s="30">
-        <f>SUMPRODUCT(Artikelstamm!$K$3:$K$235,Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT(Artikelstamm!$K$3:$K$243,Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
     </row>
@@ -29680,7 +30632,7 @@
         </is>
       </c>
       <c r="B17" s="30">
-        <f>SUMPRODUCT((Artikelstamm!$AI$3:$AI$235="bezahlt")*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AI$3:$AI$243="bezahlt")*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
     </row>
@@ -29709,7 +30661,7 @@
         </is>
       </c>
       <c r="B21" s="31">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$235,"*verkauft",Artikelstamm!$AH$3:$AH$235,"")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$243,"*verkauft",Artikelstamm!$AH$3:$AH$243,"")</f>
         <v/>
       </c>
     </row>
@@ -29720,7 +30672,7 @@
         </is>
       </c>
       <c r="B22" s="31">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$235,"*verkauft",Artikelstamm!$AI$3:$AI$235,"offen")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$243,"*verkauft",Artikelstamm!$AI$3:$AI$243,"offen")</f>
         <v/>
       </c>
     </row>
@@ -29731,7 +30683,7 @@
         </is>
       </c>
       <c r="B23" s="27">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$235,"reserviert",Artikelstamm!$AK$3:$AK$235,"")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$243,"reserviert",Artikelstamm!$AK$3:$AK$243,"")</f>
         <v/>
       </c>
     </row>
@@ -29742,7 +30694,7 @@
         </is>
       </c>
       <c r="B24" s="27">
-        <f>COUNTIFS(Artikelstamm!$S$3:$S$235,"")</f>
+        <f>COUNTIFS(Artikelstamm!$S$3:$S$243,"")</f>
         <v/>
       </c>
     </row>
@@ -29753,7 +30705,7 @@
         </is>
       </c>
       <c r="B25" s="27">
-        <f>COUNTIFS(Artikelstamm!$O$3:$O$235,"")</f>
+        <f>COUNTIFS(Artikelstamm!$O$3:$O$243,"")</f>
         <v/>
       </c>
     </row>
@@ -29793,15 +30745,15 @@
         </is>
       </c>
       <c r="B30" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$235,$A30)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$243,$A30)</f>
         <v/>
       </c>
       <c r="C30" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$235=$A30)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$243=$A30)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
       <c r="D30" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$235,$A30,Artikelstamm!$U$3:$U$235)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$243,$A30,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -29812,15 +30764,15 @@
         </is>
       </c>
       <c r="B31" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$235,$A31)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$243,$A31)</f>
         <v/>
       </c>
       <c r="C31" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$235=$A31)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$243=$A31)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
       <c r="D31" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$235,$A31,Artikelstamm!$U$3:$U$235)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$243,$A31,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -29831,15 +30783,15 @@
         </is>
       </c>
       <c r="B32" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$235,$A32)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$243,$A32)</f>
         <v/>
       </c>
       <c r="C32" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$235=$A32)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$243=$A32)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
       <c r="D32" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$235,$A32,Artikelstamm!$U$3:$U$235)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$243,$A32,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -29898,15 +30850,15 @@
         </is>
       </c>
       <c r="B37" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$235,$A37)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$243,$A37)</f>
         <v/>
       </c>
       <c r="C37" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$235=$A37)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$243=$A37)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
       <c r="D37" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$235,$A37,Artikelstamm!$U$3:$U$235)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$243,$A37,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -29917,15 +30869,15 @@
         </is>
       </c>
       <c r="B38" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$235,$A38)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$243,$A38)</f>
         <v/>
       </c>
       <c r="C38" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$235=$A38)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$243=$A38)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
       <c r="D38" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$235,$A38,Artikelstamm!$U$3:$U$235)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$243,$A38,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -29936,15 +30888,15 @@
         </is>
       </c>
       <c r="B39" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$235,$A39)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$243,$A39)</f>
         <v/>
       </c>
       <c r="C39" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$235=$A39)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$243=$A39)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
       <c r="D39" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$235,$A39,Artikelstamm!$U$3:$U$235)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$243,$A39,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -29955,15 +30907,15 @@
         </is>
       </c>
       <c r="B40" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$235,$A40)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$243,$A40)</f>
         <v/>
       </c>
       <c r="C40" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$235=$A40)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$243=$A40)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
       <c r="D40" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$235,$A40,Artikelstamm!$U$3:$U$235)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$243,$A40,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -29974,15 +30926,15 @@
         </is>
       </c>
       <c r="B41" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$235,$A41)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$243,$A41)</f>
         <v/>
       </c>
       <c r="C41" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$235=$A41)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$243=$A41)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
       <c r="D41" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$235,$A41,Artikelstamm!$U$3:$U$235)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$243,$A41,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -29993,15 +30945,15 @@
         </is>
       </c>
       <c r="B42" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$235,$A42)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$243,$A42)</f>
         <v/>
       </c>
       <c r="C42" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$235=$A42)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$243=$A42)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
       <c r="D42" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$235,$A42,Artikelstamm!$U$3:$U$235)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$243,$A42,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -30012,15 +30964,15 @@
         </is>
       </c>
       <c r="B43" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$235,$A43)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$243,$A43)</f>
         <v/>
       </c>
       <c r="C43" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$235=$A43)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$243=$A43)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
       <c r="D43" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$235,$A43,Artikelstamm!$U$3:$U$235)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$243,$A43,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -30031,15 +30983,15 @@
         </is>
       </c>
       <c r="B44" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$235,$A44)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$243,$A44)</f>
         <v/>
       </c>
       <c r="C44" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$235=$A44)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$243=$A44)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
       <c r="D44" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$235,$A44,Artikelstamm!$U$3:$U$235)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$243,$A44,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -30050,15 +31002,15 @@
         </is>
       </c>
       <c r="B45" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$235,$A45)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$243,$A45)</f>
         <v/>
       </c>
       <c r="C45" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$235=$A45)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$243=$A45)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
       <c r="D45" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$235,$A45,Artikelstamm!$U$3:$U$235)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$243,$A45,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -30069,15 +31021,15 @@
         </is>
       </c>
       <c r="B46" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$235,$A46)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$243,$A46)</f>
         <v/>
       </c>
       <c r="C46" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$235=$A46)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$243=$A46)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
       <c r="D46" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$235,$A46,Artikelstamm!$U$3:$U$235)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$243,$A46,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -30088,15 +31040,15 @@
         </is>
       </c>
       <c r="B47" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$235,$A47)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$243,$A47)</f>
         <v/>
       </c>
       <c r="C47" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$235=$A47)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$243=$A47)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
       <c r="D47" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$235,$A47,Artikelstamm!$U$3:$U$235)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$243,$A47,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -30107,15 +31059,15 @@
         </is>
       </c>
       <c r="B48" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$235,$A48)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$243,$A48)</f>
         <v/>
       </c>
       <c r="C48" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$235=$A48)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$243=$A48)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
       <c r="D48" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$235,$A48,Artikelstamm!$U$3:$U$235)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$243,$A48,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -30126,15 +31078,15 @@
         </is>
       </c>
       <c r="B49" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$235,$A49)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$243,$A49)</f>
         <v/>
       </c>
       <c r="C49" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$235=$A49)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$243=$A49)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
       <c r="D49" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$235,$A49,Artikelstamm!$U$3:$U$235)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$243,$A49,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -30145,15 +31097,15 @@
         </is>
       </c>
       <c r="B50" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$235,$A50)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$243,$A50)</f>
         <v/>
       </c>
       <c r="C50" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$235=$A50)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$243=$A50)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
       <c r="D50" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$235,$A50,Artikelstamm!$U$3:$U$235)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$243,$A50,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -30212,15 +31164,15 @@
         </is>
       </c>
       <c r="B55" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A55)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A55)</f>
         <v/>
       </c>
       <c r="C55" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A55)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A55)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
       <c r="D55" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A55,Artikelstamm!$U$3:$U$235)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A55,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -30231,15 +31183,15 @@
         </is>
       </c>
       <c r="B56" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A56)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A56)</f>
         <v/>
       </c>
       <c r="C56" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A56)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A56)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
       <c r="D56" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A56,Artikelstamm!$U$3:$U$235)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A56,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -30250,15 +31202,15 @@
         </is>
       </c>
       <c r="B57" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A57)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A57)</f>
         <v/>
       </c>
       <c r="C57" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A57)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A57)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
       <c r="D57" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A57,Artikelstamm!$U$3:$U$235)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A57,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -30269,15 +31221,15 @@
         </is>
       </c>
       <c r="B58" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A58)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A58)</f>
         <v/>
       </c>
       <c r="C58" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A58)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A58)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
       <c r="D58" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A58,Artikelstamm!$U$3:$U$235)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A58,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -30288,15 +31240,15 @@
         </is>
       </c>
       <c r="B59" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A59)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A59)</f>
         <v/>
       </c>
       <c r="C59" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A59)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A59)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
       <c r="D59" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A59,Artikelstamm!$U$3:$U$235)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A59,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -30307,467 +31259,486 @@
         </is>
       </c>
       <c r="B60" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A60)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A60)</f>
         <v/>
       </c>
       <c r="C60" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A60)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A60)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
       <c r="D60" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A60,Artikelstamm!$U$3:$U$235)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A60,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="26" t="inlineStr">
         <is>
-          <t>Garage</t>
+          <t>Flur 2</t>
         </is>
       </c>
       <c r="B61" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A61)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A61)</f>
         <v/>
       </c>
       <c r="C61" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A61)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A61)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
       <c r="D61" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A61,Artikelstamm!$U$3:$U$235)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A61,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="26" t="inlineStr">
         <is>
-          <t>Gartenanlage</t>
+          <t>Garage</t>
         </is>
       </c>
       <c r="B62" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A62)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A62)</f>
         <v/>
       </c>
       <c r="C62" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A62)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A62)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
       <c r="D62" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A62,Artikelstamm!$U$3:$U$235)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A62,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="26" t="inlineStr">
         <is>
-          <t>Gruppenraum</t>
+          <t>Gartenanlage</t>
         </is>
       </c>
       <c r="B63" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A63)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A63)</f>
         <v/>
       </c>
       <c r="C63" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A63)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A63)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
       <c r="D63" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A63,Artikelstamm!$U$3:$U$235)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A63,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="26" t="inlineStr">
         <is>
-          <t>Gruppenraum 2</t>
+          <t>Gruppenraum</t>
         </is>
       </c>
       <c r="B64" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A64)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A64)</f>
         <v/>
       </c>
       <c r="C64" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A64)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A64)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
       <c r="D64" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A64,Artikelstamm!$U$3:$U$235)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A64,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="26" t="inlineStr">
         <is>
-          <t>Gruppenraum 4</t>
+          <t>Gruppenraum 2</t>
         </is>
       </c>
       <c r="B65" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A65)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A65)</f>
         <v/>
       </c>
       <c r="C65" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A65)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A65)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
       <c r="D65" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A65,Artikelstamm!$U$3:$U$235)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A65,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="26" t="inlineStr">
         <is>
-          <t>Gruppenraum 5</t>
+          <t>Gruppenraum 4</t>
         </is>
       </c>
       <c r="B66" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A66)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A66)</f>
         <v/>
       </c>
       <c r="C66" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A66)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A66)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
       <c r="D66" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A66,Artikelstamm!$U$3:$U$235)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A66,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="26" t="inlineStr">
         <is>
-          <t>Personal</t>
+          <t>Gruppenraum 5</t>
         </is>
       </c>
       <c r="B67" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A67)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A67)</f>
         <v/>
       </c>
       <c r="C67" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A67)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A67)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
       <c r="D67" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A67,Artikelstamm!$U$3:$U$235)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A67,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="26" t="inlineStr">
         <is>
-          <t>Ruhe- / Schlafraum</t>
+          <t>Personal</t>
         </is>
       </c>
       <c r="B68" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A68)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A68)</f>
         <v/>
       </c>
       <c r="C68" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A68)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A68)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
       <c r="D68" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A68,Artikelstamm!$U$3:$U$235)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A68,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="26" t="inlineStr">
         <is>
-          <t>Schlafraum 4</t>
+          <t>Ruhe- / Schlafraum</t>
         </is>
       </c>
       <c r="B69" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A69)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A69)</f>
         <v/>
       </c>
       <c r="C69" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A69)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A69)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
       <c r="D69" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A69,Artikelstamm!$U$3:$U$235)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A69,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="26" t="inlineStr">
         <is>
-          <t>Schlafraum 5</t>
+          <t>Schlafraum 4</t>
         </is>
       </c>
       <c r="B70" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A70)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A70)</f>
         <v/>
       </c>
       <c r="C70" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A70)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A70)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
       <c r="D70" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A70,Artikelstamm!$U$3:$U$235)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A70,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="26" t="inlineStr">
         <is>
-          <t>Speisesaal</t>
+          <t>Schlafraum 5</t>
         </is>
       </c>
       <c r="B71" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A71)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A71)</f>
         <v/>
       </c>
       <c r="C71" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A71)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A71)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
       <c r="D71" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A71,Artikelstamm!$U$3:$U$235)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A71,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="26" t="inlineStr">
         <is>
-          <t>Terrasse</t>
+          <t>Speisesaal</t>
         </is>
       </c>
       <c r="B72" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A72)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A72)</f>
         <v/>
       </c>
       <c r="C72" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A72)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A72)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
       <c r="D72" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A72,Artikelstamm!$U$3:$U$235)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A72,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="26" t="inlineStr">
         <is>
-          <t>Treppenraum 1</t>
+          <t>Terrasse</t>
         </is>
       </c>
       <c r="B73" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A73)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A73)</f>
         <v/>
       </c>
       <c r="C73" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A73)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A73)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
       <c r="D73" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A73,Artikelstamm!$U$3:$U$235)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A73,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="26" t="inlineStr">
         <is>
-          <t>WC</t>
+          <t>Treppenraum 1</t>
         </is>
       </c>
       <c r="B74" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A74)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A74)</f>
         <v/>
       </c>
       <c r="C74" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A74)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A74)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
       <c r="D74" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A74,Artikelstamm!$U$3:$U$235)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A74,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="26" t="inlineStr">
         <is>
-          <t>WC Personal</t>
+          <t>WC</t>
         </is>
       </c>
       <c r="B75" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A75)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A75)</f>
         <v/>
       </c>
       <c r="C75" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A75)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A75)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
       <c r="D75" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A75,Artikelstamm!$U$3:$U$235)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A75,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="26" t="inlineStr">
         <is>
+          <t>WC Personal</t>
+        </is>
+      </c>
+      <c r="B76" s="33">
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A76)</f>
+        <v/>
+      </c>
+      <c r="C76" s="34">
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A76)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
+        <v/>
+      </c>
+      <c r="D76" s="34">
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A76,Artikelstamm!$U$3:$U$243)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="26" t="inlineStr">
+        <is>
           <t>Werkraum</t>
         </is>
       </c>
-      <c r="B76" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$235,$A76)</f>
-        <v/>
-      </c>
-      <c r="C76" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$235=$A76)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
-        <v/>
-      </c>
-      <c r="D76" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$235,$A76,Artikelstamm!$U$3:$U$235)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="28" t="inlineStr">
+      <c r="B77" s="33">
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A77)</f>
+        <v/>
+      </c>
+      <c r="C77" s="34">
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A77)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
+        <v/>
+      </c>
+      <c r="D77" s="34">
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A77,Artikelstamm!$U$3:$U$243)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="28" t="inlineStr">
         <is>
           <t>Summe</t>
         </is>
       </c>
-      <c r="B77" s="35">
-        <f>SUM(B55:B76)</f>
-        <v/>
-      </c>
-      <c r="C77" s="36">
-        <f>SUM(C55:C76)</f>
-        <v/>
-      </c>
-      <c r="D77" s="36">
-        <f>SUM(D55:D76)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="25" t="inlineStr">
+      <c r="B78" s="35">
+        <f>SUM(B55:B77)</f>
+        <v/>
+      </c>
+      <c r="C78" s="36">
+        <f>SUM(C55:C77)</f>
+        <v/>
+      </c>
+      <c r="D78" s="36">
+        <f>SUM(D55:D77)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="25" t="inlineStr">
         <is>
           <t>Nach Verkaufskanal</t>
         </is>
       </c>
     </row>
-    <row r="80">
-      <c r="A80" s="32" t="inlineStr">
+    <row r="81">
+      <c r="A81" s="32" t="inlineStr">
         <is>
           <t>Verkaufskanal</t>
         </is>
       </c>
-      <c r="B80" s="32" t="inlineStr">
+      <c r="B81" s="32" t="inlineStr">
         <is>
           <t>Positionen</t>
         </is>
       </c>
-      <c r="C80" s="32" t="inlineStr">
+      <c r="C81" s="32" t="inlineStr">
         <is>
           <t>Umsatz netto</t>
         </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="26" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
-      <c r="B81" s="33">
-        <f>COUNTIF(Artikelstamm!$AB$3:$AB$235,$A81)</f>
-        <v/>
-      </c>
-      <c r="C81" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AB$3:$AB$235=$A81)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
-        <v/>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="26" t="inlineStr">
         <is>
-          <t>Kleinanzeigen</t>
+          <t>Klinik</t>
         </is>
       </c>
       <c r="B82" s="33">
-        <f>COUNTIF(Artikelstamm!$AB$3:$AB$235,$A82)</f>
+        <f>COUNTIF(Artikelstamm!$AB$3:$AB$243,$A82)</f>
         <v/>
       </c>
       <c r="C82" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AB$3:$AB$235=$A82)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AB$3:$AB$243=$A82)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="26" t="inlineStr">
         <is>
-          <t>eBay</t>
+          <t>Kleinanzeigen</t>
         </is>
       </c>
       <c r="B83" s="33">
-        <f>COUNTIF(Artikelstamm!$AB$3:$AB$235,$A83)</f>
+        <f>COUNTIF(Artikelstamm!$AB$3:$AB$243,$A83)</f>
         <v/>
       </c>
       <c r="C83" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AB$3:$AB$235=$A83)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AB$3:$AB$243=$A83)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="26" t="inlineStr">
         <is>
-          <t>Direkt</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="B84" s="33">
-        <f>COUNTIF(Artikelstamm!$AB$3:$AB$235,$A84)</f>
+        <f>COUNTIF(Artikelstamm!$AB$3:$AB$243,$A84)</f>
         <v/>
       </c>
       <c r="C84" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AB$3:$AB$235=$A84)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AB$3:$AB$243=$A84)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="26" t="inlineStr">
         <is>
-          <t>Händler</t>
+          <t>Direkt</t>
         </is>
       </c>
       <c r="B85" s="33">
-        <f>COUNTIF(Artikelstamm!$AB$3:$AB$235,$A85)</f>
+        <f>COUNTIF(Artikelstamm!$AB$3:$AB$243,$A85)</f>
         <v/>
       </c>
       <c r="C85" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AB$3:$AB$235=$A85)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AB$3:$AB$243=$A85)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
         <v/>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="26" t="inlineStr">
         <is>
+          <t>Händler</t>
+        </is>
+      </c>
+      <c r="B86" s="33">
+        <f>COUNTIF(Artikelstamm!$AB$3:$AB$243,$A86)</f>
+        <v/>
+      </c>
+      <c r="C86" s="34">
+        <f>SUMPRODUCT((Artikelstamm!$AB$3:$AB$243=$A86)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="26" t="inlineStr">
+        <is>
           <t>Verkaufstag</t>
         </is>
       </c>
-      <c r="B86" s="33">
-        <f>COUNTIF(Artikelstamm!$AB$3:$AB$235,$A86)</f>
-        <v/>
-      </c>
-      <c r="C86" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AB$3:$AB$235=$A86)*Artikelstamm!$K$3:$K$235*Artikelstamm!$AD$3:$AD$235)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="28" t="inlineStr">
+      <c r="B87" s="33">
+        <f>COUNTIF(Artikelstamm!$AB$3:$AB$243,$A87)</f>
+        <v/>
+      </c>
+      <c r="C87" s="34">
+        <f>SUMPRODUCT((Artikelstamm!$AB$3:$AB$243=$A87)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AD$3:$AD$243)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="28" t="inlineStr">
         <is>
           <t>Summe</t>
         </is>
       </c>
-      <c r="B87" s="35">
-        <f>SUM(B81:B86)</f>
-        <v/>
-      </c>
-      <c r="C87" s="36">
-        <f>SUM(C81:C86)</f>
+      <c r="B88" s="35">
+        <f>SUM(B82:B87)</f>
+        <v/>
+      </c>
+      <c r="C88" s="36">
+        <f>SUM(C82:C87)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
BA09: Kartell-Stuehle 6 -> 4, Hocker ergaenzt, Buendeln vorgemerkt
Personal (Bestandsgebaeude Attika, 16,19 m2). Auf dem Erfassungsblatt hat
die Nutzerin die vorgedruckte Stueckzahl der Kartell Masters Stuehle von
6 auf 4 korrigiert - 240 EUR weniger im Bestand. Neu dazu BA09-06, ein
runder Sitzhocker auf Rollen.

Weiteres Buendeln wartet bis zum Ende des Rundgangs, so gewuenscht: es
kommt noch einiges, und eine Sammlung ist erst sinnvoll, wenn alles
erfasst ist. In SKILL.md als eigene Sorte offener Punkte vermerkt, damit
es beim Abschluss nicht untergeht. Erkennbare Gruppen nenne ich bis dahin
nur im Bericht.

Gesamtwert netto 37.002 -> 36.792 EUR, 186 aktive Positionen.
pruefen.py: 0 Fehler, 3 Hinweise.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011yyfqhuiWGsaNy38oaNoGo
</commit_message>
<xml_diff>
--- a/ausgabe/01_Artikelstamm_kikripp.xlsx
+++ b/ausgabe/01_Artikelstamm_kikripp.xlsx
@@ -15,7 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Artikelstamm'!$A$2:$AN$242</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Artikelstamm'!$A$2:$AN$243</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1019,7 +1019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN242"/>
+  <dimension ref="A1:AN243"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2588,7 +2588,7 @@
         </is>
       </c>
       <c r="J13" s="17" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K13" s="17" t="n"/>
       <c r="L13" s="18">
@@ -2667,7 +2667,7 @@
       <c r="AL13" s="19" t="n"/>
       <c r="AM13" s="16" t="inlineStr">
         <is>
-          <t>mindestens 6 Stück erkennbar - bitte nachzählen</t>
+          <t>4 Stühle – abgebildet sind zwei davon.</t>
         </is>
       </c>
       <c r="AN13" s="22" t="n"/>
@@ -30602,8 +30602,127 @@
       </c>
       <c r="AN242" s="22" t="n"/>
     </row>
+    <row r="243" ht="30" customHeight="1">
+      <c r="A243" s="15" t="inlineStr">
+        <is>
+          <t>BA09-06</t>
+        </is>
+      </c>
+      <c r="B243" s="15" t="n"/>
+      <c r="C243" s="15" t="n"/>
+      <c r="D243" s="15" t="inlineStr">
+        <is>
+          <t>BA09</t>
+        </is>
+      </c>
+      <c r="E243" s="15" t="inlineStr">
+        <is>
+          <t>Sitzhocker rund, drehbar auf Rollen</t>
+        </is>
+      </c>
+      <c r="F243" s="16" t="inlineStr">
+        <is>
+          <t>Runder Sitzhocker mit schwarzem Netzstoffbezug und umlaufendem Reißverschluss, auf einem silberfarbenen Fünffußkreuz mit Rollen, höhenverstellbar.</t>
+        </is>
+      </c>
+      <c r="G243" s="15" t="inlineStr">
+        <is>
+          <t>Büro</t>
+        </is>
+      </c>
+      <c r="H243" s="15" t="inlineStr">
+        <is>
+          <t>Personal</t>
+        </is>
+      </c>
+      <c r="I243" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J243" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K243" s="17" t="n"/>
+      <c r="L243" s="18">
+        <f>J243-IF(K243="",0,K243)</f>
+        <v/>
+      </c>
+      <c r="M243" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N243" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O243" s="19" t="n"/>
+      <c r="P243" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q243" s="19" t="n"/>
+      <c r="R243" s="20" t="n"/>
+      <c r="S243" s="20" t="n">
+        <v>30</v>
+      </c>
+      <c r="T243" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U243" s="21">
+        <f>L243*S243</f>
+        <v/>
+      </c>
+      <c r="V243" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W243" s="15" t="inlineStr">
+        <is>
+          <t>F-274</t>
+        </is>
+      </c>
+      <c r="X243" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y243" s="19" t="n"/>
+      <c r="Z243" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA243" s="19" t="n"/>
+      <c r="AB243" s="19" t="n"/>
+      <c r="AC243" s="19" t="n"/>
+      <c r="AD243" s="19" t="n"/>
+      <c r="AE243" s="20" t="n"/>
+      <c r="AF243" s="21">
+        <f>IF(K243="","",K243*AE243)</f>
+        <v/>
+      </c>
+      <c r="AG243" s="19" t="n"/>
+      <c r="AH243" s="19" t="n"/>
+      <c r="AI243" s="19" t="n"/>
+      <c r="AJ243" s="19" t="n"/>
+      <c r="AK243" s="19" t="n"/>
+      <c r="AL243" s="19" t="n"/>
+      <c r="AM243" s="16" t="inlineStr">
+        <is>
+          <t>1 Hocker.</t>
+        </is>
+      </c>
+      <c r="AN243" s="22" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:AN242"/>
+  <autoFilter ref="A2:AN243"/>
   <mergeCells count="7">
     <mergeCell ref="AI1:AL1"/>
     <mergeCell ref="V1:AD1"/>
@@ -30613,7 +30732,7 @@
     <mergeCell ref="AE1:AH1"/>
     <mergeCell ref="AM1:AN1"/>
   </mergeCells>
-  <conditionalFormatting sqref="Z3:Z242">
+  <conditionalFormatting sqref="Z3:Z243">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"reserviert"</formula>
     </cfRule>
@@ -30624,12 +30743,12 @@
       <formula>"verkauft"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I3:I242">
+  <conditionalFormatting sqref="I3:I243">
     <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
       <formula>"A"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P3:P242">
+  <conditionalFormatting sqref="P3:P243">
     <cfRule type="cellIs" priority="5" operator="equal" dxfId="4">
       <formula>"entfällt"</formula>
     </cfRule>
@@ -30720,7 +30839,7 @@
         </is>
       </c>
       <c r="B5" s="27">
-        <f>COUNTA(Artikelstamm!$A$3:$A$242)</f>
+        <f>COUNTA(Artikelstamm!$A$3:$A$243)</f>
         <v/>
       </c>
     </row>
@@ -30731,7 +30850,7 @@
         </is>
       </c>
       <c r="B6" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$242,"verfügbar")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$243,"verfügbar")</f>
         <v/>
       </c>
     </row>
@@ -30742,7 +30861,7 @@
         </is>
       </c>
       <c r="B7" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$242,"reserviert")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$243,"reserviert")</f>
         <v/>
       </c>
     </row>
@@ -30753,7 +30872,7 @@
         </is>
       </c>
       <c r="B8" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$242,"teilverkauft")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$243,"teilverkauft")</f>
         <v/>
       </c>
     </row>
@@ -30764,7 +30883,7 @@
         </is>
       </c>
       <c r="B9" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$242,"verkauft")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$243,"verkauft")</f>
         <v/>
       </c>
     </row>
@@ -30775,7 +30894,7 @@
         </is>
       </c>
       <c r="B10" s="27">
-        <f>SUM(Artikelstamm!$L$3:$L$242)</f>
+        <f>SUM(Artikelstamm!$L$3:$L$243)</f>
         <v/>
       </c>
     </row>
@@ -30786,7 +30905,7 @@
         </is>
       </c>
       <c r="B11" s="29">
-        <f>SUM(Artikelstamm!$U$3:$U$242)</f>
+        <f>SUM(Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -30804,7 +30923,7 @@
         </is>
       </c>
       <c r="B13" s="27">
-        <f>SUM(Artikelstamm!$K$3:$K$242)</f>
+        <f>SUM(Artikelstamm!$K$3:$K$243)</f>
         <v/>
       </c>
     </row>
@@ -30815,7 +30934,7 @@
         </is>
       </c>
       <c r="B14" s="30">
-        <f>SUMPRODUCT(Artikelstamm!$K$3:$K$242,Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT(Artikelstamm!$K$3:$K$243,Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
     </row>
@@ -30848,7 +30967,7 @@
         </is>
       </c>
       <c r="B17" s="30">
-        <f>SUMPRODUCT((Artikelstamm!$AJ$3:$AJ$242="bezahlt")*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AJ$3:$AJ$243="bezahlt")*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
     </row>
@@ -30877,7 +30996,7 @@
         </is>
       </c>
       <c r="B21" s="31">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$242,"*verkauft",Artikelstamm!$AI$3:$AI$242,"")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$243,"*verkauft",Artikelstamm!$AI$3:$AI$243,"")</f>
         <v/>
       </c>
     </row>
@@ -30888,7 +31007,7 @@
         </is>
       </c>
       <c r="B22" s="31">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$242,"*verkauft",Artikelstamm!$AJ$3:$AJ$242,"offen")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$243,"*verkauft",Artikelstamm!$AJ$3:$AJ$243,"offen")</f>
         <v/>
       </c>
     </row>
@@ -30899,7 +31018,7 @@
         </is>
       </c>
       <c r="B23" s="27">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$242,"reserviert",Artikelstamm!$AL$3:$AL$242,"")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$243,"reserviert",Artikelstamm!$AL$3:$AL$243,"")</f>
         <v/>
       </c>
     </row>
@@ -30910,7 +31029,7 @@
         </is>
       </c>
       <c r="B24" s="27">
-        <f>COUNTIFS(Artikelstamm!$S$3:$S$242,"")</f>
+        <f>COUNTIFS(Artikelstamm!$S$3:$S$243,"")</f>
         <v/>
       </c>
     </row>
@@ -30921,7 +31040,7 @@
         </is>
       </c>
       <c r="B25" s="27">
-        <f>COUNTIFS(Artikelstamm!$O$3:$O$242,"")</f>
+        <f>COUNTIFS(Artikelstamm!$O$3:$O$243,"")</f>
         <v/>
       </c>
     </row>
@@ -30961,15 +31080,15 @@
         </is>
       </c>
       <c r="B30" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$242,$A30)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$243,$A30)</f>
         <v/>
       </c>
       <c r="C30" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$242=$A30)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$243=$A30)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
       <c r="D30" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$242,$A30,Artikelstamm!$U$3:$U$242)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$243,$A30,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -30980,15 +31099,15 @@
         </is>
       </c>
       <c r="B31" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$242,$A31)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$243,$A31)</f>
         <v/>
       </c>
       <c r="C31" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$242=$A31)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$243=$A31)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
       <c r="D31" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$242,$A31,Artikelstamm!$U$3:$U$242)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$243,$A31,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -30999,15 +31118,15 @@
         </is>
       </c>
       <c r="B32" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$242,$A32)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$243,$A32)</f>
         <v/>
       </c>
       <c r="C32" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$242=$A32)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$243=$A32)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
       <c r="D32" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$242,$A32,Artikelstamm!$U$3:$U$242)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$243,$A32,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -31066,15 +31185,15 @@
         </is>
       </c>
       <c r="B37" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$242,$A37)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$243,$A37)</f>
         <v/>
       </c>
       <c r="C37" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$242=$A37)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$243=$A37)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
       <c r="D37" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$242,$A37,Artikelstamm!$U$3:$U$242)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$243,$A37,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -31085,15 +31204,15 @@
         </is>
       </c>
       <c r="B38" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$242,$A38)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$243,$A38)</f>
         <v/>
       </c>
       <c r="C38" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$242=$A38)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$243=$A38)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
       <c r="D38" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$242,$A38,Artikelstamm!$U$3:$U$242)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$243,$A38,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -31104,15 +31223,15 @@
         </is>
       </c>
       <c r="B39" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$242,$A39)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$243,$A39)</f>
         <v/>
       </c>
       <c r="C39" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$242=$A39)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$243=$A39)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
       <c r="D39" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$242,$A39,Artikelstamm!$U$3:$U$242)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$243,$A39,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -31123,15 +31242,15 @@
         </is>
       </c>
       <c r="B40" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$242,$A40)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$243,$A40)</f>
         <v/>
       </c>
       <c r="C40" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$242=$A40)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$243=$A40)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
       <c r="D40" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$242,$A40,Artikelstamm!$U$3:$U$242)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$243,$A40,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -31142,15 +31261,15 @@
         </is>
       </c>
       <c r="B41" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$242,$A41)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$243,$A41)</f>
         <v/>
       </c>
       <c r="C41" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$242=$A41)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$243=$A41)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
       <c r="D41" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$242,$A41,Artikelstamm!$U$3:$U$242)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$243,$A41,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -31161,15 +31280,15 @@
         </is>
       </c>
       <c r="B42" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$242,$A42)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$243,$A42)</f>
         <v/>
       </c>
       <c r="C42" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$242=$A42)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$243=$A42)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
       <c r="D42" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$242,$A42,Artikelstamm!$U$3:$U$242)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$243,$A42,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -31180,15 +31299,15 @@
         </is>
       </c>
       <c r="B43" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$242,$A43)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$243,$A43)</f>
         <v/>
       </c>
       <c r="C43" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$242=$A43)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$243=$A43)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
       <c r="D43" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$242,$A43,Artikelstamm!$U$3:$U$242)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$243,$A43,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -31199,15 +31318,15 @@
         </is>
       </c>
       <c r="B44" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$242,$A44)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$243,$A44)</f>
         <v/>
       </c>
       <c r="C44" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$242=$A44)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$243=$A44)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
       <c r="D44" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$242,$A44,Artikelstamm!$U$3:$U$242)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$243,$A44,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -31218,15 +31337,15 @@
         </is>
       </c>
       <c r="B45" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$242,$A45)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$243,$A45)</f>
         <v/>
       </c>
       <c r="C45" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$242=$A45)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$243=$A45)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
       <c r="D45" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$242,$A45,Artikelstamm!$U$3:$U$242)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$243,$A45,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -31237,15 +31356,15 @@
         </is>
       </c>
       <c r="B46" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$242,$A46)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$243,$A46)</f>
         <v/>
       </c>
       <c r="C46" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$242=$A46)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$243=$A46)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
       <c r="D46" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$242,$A46,Artikelstamm!$U$3:$U$242)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$243,$A46,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -31256,15 +31375,15 @@
         </is>
       </c>
       <c r="B47" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$242,$A47)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$243,$A47)</f>
         <v/>
       </c>
       <c r="C47" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$242=$A47)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$243=$A47)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
       <c r="D47" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$242,$A47,Artikelstamm!$U$3:$U$242)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$243,$A47,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -31275,15 +31394,15 @@
         </is>
       </c>
       <c r="B48" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$242,$A48)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$243,$A48)</f>
         <v/>
       </c>
       <c r="C48" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$242=$A48)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$243=$A48)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
       <c r="D48" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$242,$A48,Artikelstamm!$U$3:$U$242)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$243,$A48,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -31294,15 +31413,15 @@
         </is>
       </c>
       <c r="B49" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$242,$A49)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$243,$A49)</f>
         <v/>
       </c>
       <c r="C49" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$242=$A49)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$243=$A49)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
       <c r="D49" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$242,$A49,Artikelstamm!$U$3:$U$242)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$243,$A49,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -31313,15 +31432,15 @@
         </is>
       </c>
       <c r="B50" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$242,$A50)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$243,$A50)</f>
         <v/>
       </c>
       <c r="C50" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$242=$A50)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$243=$A50)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
       <c r="D50" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$242,$A50,Artikelstamm!$U$3:$U$242)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$243,$A50,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -31380,15 +31499,15 @@
         </is>
       </c>
       <c r="B55" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$242,$A55)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A55)</f>
         <v/>
       </c>
       <c r="C55" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$242=$A55)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A55)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
       <c r="D55" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$242,$A55,Artikelstamm!$U$3:$U$242)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A55,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -31399,15 +31518,15 @@
         </is>
       </c>
       <c r="B56" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$242,$A56)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A56)</f>
         <v/>
       </c>
       <c r="C56" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$242=$A56)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A56)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
       <c r="D56" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$242,$A56,Artikelstamm!$U$3:$U$242)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A56,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -31418,15 +31537,15 @@
         </is>
       </c>
       <c r="B57" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$242,$A57)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A57)</f>
         <v/>
       </c>
       <c r="C57" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$242=$A57)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A57)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
       <c r="D57" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$242,$A57,Artikelstamm!$U$3:$U$242)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A57,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -31437,15 +31556,15 @@
         </is>
       </c>
       <c r="B58" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$242,$A58)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A58)</f>
         <v/>
       </c>
       <c r="C58" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$242=$A58)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A58)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
       <c r="D58" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$242,$A58,Artikelstamm!$U$3:$U$242)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A58,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -31456,15 +31575,15 @@
         </is>
       </c>
       <c r="B59" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$242,$A59)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A59)</f>
         <v/>
       </c>
       <c r="C59" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$242=$A59)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A59)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
       <c r="D59" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$242,$A59,Artikelstamm!$U$3:$U$242)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A59,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -31475,15 +31594,15 @@
         </is>
       </c>
       <c r="B60" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$242,$A60)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A60)</f>
         <v/>
       </c>
       <c r="C60" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$242=$A60)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A60)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
       <c r="D60" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$242,$A60,Artikelstamm!$U$3:$U$242)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A60,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -31494,15 +31613,15 @@
         </is>
       </c>
       <c r="B61" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$242,$A61)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A61)</f>
         <v/>
       </c>
       <c r="C61" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$242=$A61)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A61)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
       <c r="D61" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$242,$A61,Artikelstamm!$U$3:$U$242)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A61,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -31513,15 +31632,15 @@
         </is>
       </c>
       <c r="B62" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$242,$A62)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A62)</f>
         <v/>
       </c>
       <c r="C62" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$242=$A62)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A62)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
       <c r="D62" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$242,$A62,Artikelstamm!$U$3:$U$242)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A62,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -31532,15 +31651,15 @@
         </is>
       </c>
       <c r="B63" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$242,$A63)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A63)</f>
         <v/>
       </c>
       <c r="C63" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$242=$A63)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A63)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
       <c r="D63" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$242,$A63,Artikelstamm!$U$3:$U$242)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A63,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -31551,15 +31670,15 @@
         </is>
       </c>
       <c r="B64" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$242,$A64)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A64)</f>
         <v/>
       </c>
       <c r="C64" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$242=$A64)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A64)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
       <c r="D64" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$242,$A64,Artikelstamm!$U$3:$U$242)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A64,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -31570,15 +31689,15 @@
         </is>
       </c>
       <c r="B65" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$242,$A65)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A65)</f>
         <v/>
       </c>
       <c r="C65" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$242=$A65)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A65)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
       <c r="D65" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$242,$A65,Artikelstamm!$U$3:$U$242)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A65,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -31589,15 +31708,15 @@
         </is>
       </c>
       <c r="B66" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$242,$A66)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A66)</f>
         <v/>
       </c>
       <c r="C66" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$242=$A66)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A66)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
       <c r="D66" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$242,$A66,Artikelstamm!$U$3:$U$242)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A66,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -31608,15 +31727,15 @@
         </is>
       </c>
       <c r="B67" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$242,$A67)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A67)</f>
         <v/>
       </c>
       <c r="C67" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$242=$A67)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A67)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
       <c r="D67" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$242,$A67,Artikelstamm!$U$3:$U$242)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A67,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -31627,15 +31746,15 @@
         </is>
       </c>
       <c r="B68" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$242,$A68)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A68)</f>
         <v/>
       </c>
       <c r="C68" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$242=$A68)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A68)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
       <c r="D68" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$242,$A68,Artikelstamm!$U$3:$U$242)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A68,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -31646,15 +31765,15 @@
         </is>
       </c>
       <c r="B69" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$242,$A69)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A69)</f>
         <v/>
       </c>
       <c r="C69" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$242=$A69)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A69)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
       <c r="D69" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$242,$A69,Artikelstamm!$U$3:$U$242)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A69,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -31665,15 +31784,15 @@
         </is>
       </c>
       <c r="B70" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$242,$A70)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A70)</f>
         <v/>
       </c>
       <c r="C70" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$242=$A70)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A70)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
       <c r="D70" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$242,$A70,Artikelstamm!$U$3:$U$242)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A70,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -31684,15 +31803,15 @@
         </is>
       </c>
       <c r="B71" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$242,$A71)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A71)</f>
         <v/>
       </c>
       <c r="C71" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$242=$A71)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A71)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
       <c r="D71" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$242,$A71,Artikelstamm!$U$3:$U$242)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A71,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -31703,15 +31822,15 @@
         </is>
       </c>
       <c r="B72" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$242,$A72)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A72)</f>
         <v/>
       </c>
       <c r="C72" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$242=$A72)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A72)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
       <c r="D72" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$242,$A72,Artikelstamm!$U$3:$U$242)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A72,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -31722,15 +31841,15 @@
         </is>
       </c>
       <c r="B73" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$242,$A73)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A73)</f>
         <v/>
       </c>
       <c r="C73" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$242=$A73)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A73)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
       <c r="D73" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$242,$A73,Artikelstamm!$U$3:$U$242)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A73,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -31741,15 +31860,15 @@
         </is>
       </c>
       <c r="B74" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$242,$A74)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A74)</f>
         <v/>
       </c>
       <c r="C74" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$242=$A74)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A74)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
       <c r="D74" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$242,$A74,Artikelstamm!$U$3:$U$242)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A74,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -31760,15 +31879,15 @@
         </is>
       </c>
       <c r="B75" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$242,$A75)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A75)</f>
         <v/>
       </c>
       <c r="C75" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$242=$A75)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A75)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
       <c r="D75" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$242,$A75,Artikelstamm!$U$3:$U$242)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A75,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -31779,15 +31898,15 @@
         </is>
       </c>
       <c r="B76" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$242,$A76)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A76)</f>
         <v/>
       </c>
       <c r="C76" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$242=$A76)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A76)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
       <c r="D76" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$242,$A76,Artikelstamm!$U$3:$U$242)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A76,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -31798,15 +31917,15 @@
         </is>
       </c>
       <c r="B77" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$242,$A77)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$243,$A77)</f>
         <v/>
       </c>
       <c r="C77" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$242=$A77)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$243=$A77)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
       <c r="D77" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$242,$A77,Artikelstamm!$U$3:$U$242)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$243,$A77,Artikelstamm!$U$3:$U$243)</f>
         <v/>
       </c>
     </row>
@@ -31860,11 +31979,11 @@
         </is>
       </c>
       <c r="B82" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$242,$A82)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$243,$A82)</f>
         <v/>
       </c>
       <c r="C82" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$242=$A82)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$243=$A82)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
     </row>
@@ -31875,11 +31994,11 @@
         </is>
       </c>
       <c r="B83" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$242,$A83)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$243,$A83)</f>
         <v/>
       </c>
       <c r="C83" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$242=$A83)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$243=$A83)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
     </row>
@@ -31890,11 +32009,11 @@
         </is>
       </c>
       <c r="B84" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$242,$A84)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$243,$A84)</f>
         <v/>
       </c>
       <c r="C84" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$242=$A84)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$243=$A84)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
     </row>
@@ -31905,11 +32024,11 @@
         </is>
       </c>
       <c r="B85" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$242,$A85)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$243,$A85)</f>
         <v/>
       </c>
       <c r="C85" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$242=$A85)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$243=$A85)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
     </row>
@@ -31920,11 +32039,11 @@
         </is>
       </c>
       <c r="B86" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$242,$A86)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$243,$A86)</f>
         <v/>
       </c>
       <c r="C86" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$242=$A86)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$243=$A86)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
     </row>
@@ -31935,11 +32054,11 @@
         </is>
       </c>
       <c r="B87" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$242,$A87)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$243,$A87)</f>
         <v/>
       </c>
       <c r="C87" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$242=$A87)*Artikelstamm!$K$3:$K$242*Artikelstamm!$AE$3:$AE$242)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$243=$A87)*Artikelstamm!$K$3:$K$243*Artikelstamm!$AE$3:$AE$243)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
BA03 erfasst: 7 Positionen, dritte Spielkueche und ein BRIO-Puppenwagen
Galerie (Bestandsgebaeude Attika, 16,05 m2).

Zwei Marken ueber Etiketten belegt:
- BA03-01 ist ein IKEA Avsiktlig, 133 x 195 cm. Das Rueckseiten-Etikett
  liefert Marke und Mass als belegte Angabe (F-292).
- BA03-05 ist ein Kombi-Puppenwagen von BRIO, Etikett am Verdeck (F-297).
  Neu kostet der 80-130 EUR, gebraucht mit 45 EUR angesetzt.

BA03-02 ist die dritte Spielkueche im Haus, diesmal in Creme und Taupe
mit Mikrowellenmodul und Wandregal - nicht von Wesco, keine Marke
sichtbar. Mit 250 EUR fuer das Set angesetzt. In den Mengenhinweisen
verweisen alle drei Kuechen aufeinander, genauso die beiden Kaufladen
(BA03-06 und NU07-02).

Gesamtwert netto 37.287 -> 37.907 EUR, 205 aktive Positionen.
pruefen.py: 0 Fehler, 3 Hinweise.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011yyfqhuiWGsaNy38oaNoGo
</commit_message>
<xml_diff>
--- a/ausgabe/01_Artikelstamm_kikripp.xlsx
+++ b/ausgabe/01_Artikelstamm_kikripp.xlsx
@@ -15,7 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Artikelstamm'!$A$2:$AN$255</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Artikelstamm'!$A$2:$AN$262</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1019,7 +1019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN255"/>
+  <dimension ref="A1:AN262"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -32177,8 +32177,853 @@
       </c>
       <c r="AN255" s="22" t="n"/>
     </row>
+    <row r="256" ht="30" customHeight="1">
+      <c r="A256" s="15" t="inlineStr">
+        <is>
+          <t>BA03-01</t>
+        </is>
+      </c>
+      <c r="B256" s="15" t="n"/>
+      <c r="C256" s="15" t="n"/>
+      <c r="D256" s="15" t="inlineStr">
+        <is>
+          <t>BA03</t>
+        </is>
+      </c>
+      <c r="E256" s="15" t="inlineStr">
+        <is>
+          <t>IKEA Avsiktlig Teppich, schwarz-weiß gepunktet</t>
+        </is>
+      </c>
+      <c r="F256" s="16" t="inlineStr">
+        <is>
+          <t>Flachgewebter Teppich in Creme mit schwarzen Punktreihen, IKEA Avsiktlig. Flor 100 % Polypropylen auf Jutekette. Etikett auf der Rückseite vorhanden.</t>
+        </is>
+      </c>
+      <c r="G256" s="15" t="inlineStr">
+        <is>
+          <t>Textilien</t>
+        </is>
+      </c>
+      <c r="H256" s="15" t="inlineStr">
+        <is>
+          <t>Galerie</t>
+        </is>
+      </c>
+      <c r="I256" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J256" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K256" s="17" t="n"/>
+      <c r="L256" s="18">
+        <f>J256-IF(K256="",0,K256)</f>
+        <v/>
+      </c>
+      <c r="M256" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N256" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O256" s="19" t="inlineStr">
+        <is>
+          <t>133 × 195 cm</t>
+        </is>
+      </c>
+      <c r="P256" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q256" s="19" t="n"/>
+      <c r="R256" s="20" t="n"/>
+      <c r="S256" s="20" t="n">
+        <v>25</v>
+      </c>
+      <c r="T256" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U256" s="21">
+        <f>L256*S256</f>
+        <v/>
+      </c>
+      <c r="V256" s="15" t="inlineStr">
+        <is>
+          <t>Versand möglich</t>
+        </is>
+      </c>
+      <c r="W256" s="15" t="inlineStr">
+        <is>
+          <t>F-291</t>
+        </is>
+      </c>
+      <c r="X256" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y256" s="19" t="n"/>
+      <c r="Z256" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA256" s="19" t="inlineStr">
+        <is>
+          <t>IKEA</t>
+        </is>
+      </c>
+      <c r="AB256" s="19" t="n"/>
+      <c r="AC256" s="19" t="n"/>
+      <c r="AD256" s="19" t="n"/>
+      <c r="AE256" s="20" t="n"/>
+      <c r="AF256" s="21">
+        <f>IF(K256="","",K256*AE256)</f>
+        <v/>
+      </c>
+      <c r="AG256" s="19" t="n"/>
+      <c r="AH256" s="19" t="n"/>
+      <c r="AI256" s="19" t="n"/>
+      <c r="AJ256" s="19" t="n"/>
+      <c r="AK256" s="19" t="n"/>
+      <c r="AL256" s="19" t="n"/>
+      <c r="AM256" s="16" t="inlineStr">
+        <is>
+          <t>1 Teppich. Das Etikett ist auf Foto F-292 zu sehen.</t>
+        </is>
+      </c>
+      <c r="AN256" s="22" t="n"/>
+    </row>
+    <row r="257" ht="30" customHeight="1">
+      <c r="A257" s="15" t="inlineStr">
+        <is>
+          <t>BA03-02</t>
+        </is>
+      </c>
+      <c r="B257" s="15" t="n"/>
+      <c r="C257" s="15" t="n"/>
+      <c r="D257" s="15" t="inlineStr">
+        <is>
+          <t>BA03</t>
+        </is>
+      </c>
+      <c r="E257" s="15" t="inlineStr">
+        <is>
+          <t>Spielküche beige-braun, mehrteilig</t>
+        </is>
+      </c>
+      <c r="F257" s="16" t="inlineStr">
+        <is>
+          <t>Spielküche aus beschichteter Platte in Creme und Taupe mit Holzarbeitsplatten: Mikrowellenmodul mit Digitalanzeige, Unterschränke mit Kochfeld, Backofen mit Sichtfenster und Spüle, dazu ein Wandregal. Abgerundete Ecken, kindgerechte Höhe.</t>
+        </is>
+      </c>
+      <c r="G257" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H257" s="15" t="inlineStr">
+        <is>
+          <t>Galerie</t>
+        </is>
+      </c>
+      <c r="I257" s="15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J257" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K257" s="17" t="n"/>
+      <c r="L257" s="18">
+        <f>J257-IF(K257="",0,K257)</f>
+        <v/>
+      </c>
+      <c r="M257" s="15" t="inlineStr">
+        <is>
+          <t>Set</t>
+        </is>
+      </c>
+      <c r="N257" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O257" s="19" t="n"/>
+      <c r="P257" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q257" s="19" t="n"/>
+      <c r="R257" s="20" t="n"/>
+      <c r="S257" s="20" t="n">
+        <v>250</v>
+      </c>
+      <c r="T257" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U257" s="21">
+        <f>L257*S257</f>
+        <v/>
+      </c>
+      <c r="V257" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W257" s="15" t="inlineStr">
+        <is>
+          <t>F-293</t>
+        </is>
+      </c>
+      <c r="X257" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y257" s="19" t="n"/>
+      <c r="Z257" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA257" s="19" t="n"/>
+      <c r="AB257" s="19" t="n"/>
+      <c r="AC257" s="19" t="n"/>
+      <c r="AD257" s="19" t="n"/>
+      <c r="AE257" s="20" t="n"/>
+      <c r="AF257" s="21">
+        <f>IF(K257="","",K257*AE257)</f>
+        <v/>
+      </c>
+      <c r="AG257" s="19" t="n"/>
+      <c r="AH257" s="19" t="n"/>
+      <c r="AI257" s="19" t="n"/>
+      <c r="AJ257" s="19" t="n"/>
+      <c r="AK257" s="19" t="n"/>
+      <c r="AL257" s="19" t="n"/>
+      <c r="AM257" s="16" t="inlineStr">
+        <is>
+          <t>1 Küche aus mehreren Modulen. Spielgeschirr und Zubehör gehören nicht dazu. Zwei weitere Spielküchen von Wesco stehen unter NU03-03 und NU07-03.</t>
+        </is>
+      </c>
+      <c r="AN257" s="22" t="n"/>
+    </row>
+    <row r="258" ht="30" customHeight="1">
+      <c r="A258" s="15" t="inlineStr">
+        <is>
+          <t>BA03-03</t>
+        </is>
+      </c>
+      <c r="B258" s="15" t="n"/>
+      <c r="C258" s="15" t="n"/>
+      <c r="D258" s="15" t="inlineStr">
+        <is>
+          <t>BA03</t>
+        </is>
+      </c>
+      <c r="E258" s="15" t="inlineStr">
+        <is>
+          <t>Sofa grau, 2-Sitzer</t>
+        </is>
+      </c>
+      <c r="F258" s="16" t="inlineStr">
+        <is>
+          <t>Kleines Zweisitzer-Sofa mit grauem Steppbezug aus Velours und weißem Metallgestell. Bezug abnehmbar.</t>
+        </is>
+      </c>
+      <c r="G258" s="15" t="inlineStr">
+        <is>
+          <t>Möbel</t>
+        </is>
+      </c>
+      <c r="H258" s="15" t="inlineStr">
+        <is>
+          <t>Galerie</t>
+        </is>
+      </c>
+      <c r="I258" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J258" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K258" s="17" t="n"/>
+      <c r="L258" s="18">
+        <f>J258-IF(K258="",0,K258)</f>
+        <v/>
+      </c>
+      <c r="M258" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N258" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O258" s="19" t="n"/>
+      <c r="P258" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q258" s="19" t="n"/>
+      <c r="R258" s="20" t="n"/>
+      <c r="S258" s="20" t="n">
+        <v>70</v>
+      </c>
+      <c r="T258" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U258" s="21">
+        <f>L258*S258</f>
+        <v/>
+      </c>
+      <c r="V258" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W258" s="15" t="inlineStr">
+        <is>
+          <t>F-294</t>
+        </is>
+      </c>
+      <c r="X258" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y258" s="19" t="n"/>
+      <c r="Z258" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA258" s="19" t="n"/>
+      <c r="AB258" s="19" t="n"/>
+      <c r="AC258" s="19" t="n"/>
+      <c r="AD258" s="19" t="n"/>
+      <c r="AE258" s="20" t="n"/>
+      <c r="AF258" s="21">
+        <f>IF(K258="","",K258*AE258)</f>
+        <v/>
+      </c>
+      <c r="AG258" s="19" t="n"/>
+      <c r="AH258" s="19" t="n"/>
+      <c r="AI258" s="19" t="n"/>
+      <c r="AJ258" s="19" t="n"/>
+      <c r="AK258" s="19" t="n"/>
+      <c r="AL258" s="19" t="n"/>
+      <c r="AM258" s="16" t="inlineStr">
+        <is>
+          <t>1 Sofa. Das Kissen gehört nicht dazu.</t>
+        </is>
+      </c>
+      <c r="AN258" s="22" t="n"/>
+    </row>
+    <row r="259" ht="30" customHeight="1">
+      <c r="A259" s="15" t="inlineStr">
+        <is>
+          <t>BA03-05</t>
+        </is>
+      </c>
+      <c r="B259" s="15" t="n"/>
+      <c r="C259" s="15" t="n"/>
+      <c r="D259" s="15" t="inlineStr">
+        <is>
+          <t>BA03</t>
+        </is>
+      </c>
+      <c r="E259" s="15" t="inlineStr">
+        <is>
+          <t>BRIO Puppenwagen rot gepunktet</t>
+        </is>
+      </c>
+      <c r="F259" s="16" t="inlineStr">
+        <is>
+          <t>Kombi-Puppenwagen von BRIO: weißes Metallgestell mit Luftreifen, roter Stoffbezug mit weißen Punkten, schwenkbarer Schiebebügel, Ablagekorb unten. Markenetikett am Verdeck.</t>
+        </is>
+      </c>
+      <c r="G259" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H259" s="15" t="inlineStr">
+        <is>
+          <t>Galerie</t>
+        </is>
+      </c>
+      <c r="I259" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J259" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K259" s="17" t="n"/>
+      <c r="L259" s="18">
+        <f>J259-IF(K259="",0,K259)</f>
+        <v/>
+      </c>
+      <c r="M259" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N259" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O259" s="19" t="n"/>
+      <c r="P259" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q259" s="19" t="n"/>
+      <c r="R259" s="20" t="n"/>
+      <c r="S259" s="20" t="n">
+        <v>45</v>
+      </c>
+      <c r="T259" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U259" s="21">
+        <f>L259*S259</f>
+        <v/>
+      </c>
+      <c r="V259" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W259" s="15" t="inlineStr">
+        <is>
+          <t>F-296</t>
+        </is>
+      </c>
+      <c r="X259" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y259" s="19" t="n"/>
+      <c r="Z259" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA259" s="19" t="inlineStr">
+        <is>
+          <t>BRIO</t>
+        </is>
+      </c>
+      <c r="AB259" s="19" t="n"/>
+      <c r="AC259" s="19" t="n"/>
+      <c r="AD259" s="19" t="n"/>
+      <c r="AE259" s="20" t="n"/>
+      <c r="AF259" s="21">
+        <f>IF(K259="","",K259*AE259)</f>
+        <v/>
+      </c>
+      <c r="AG259" s="19" t="n"/>
+      <c r="AH259" s="19" t="n"/>
+      <c r="AI259" s="19" t="n"/>
+      <c r="AJ259" s="19" t="n"/>
+      <c r="AK259" s="19" t="n"/>
+      <c r="AL259" s="19" t="n"/>
+      <c r="AM259" s="16" t="inlineStr">
+        <is>
+          <t>1 Puppenwagen. Die Puppe gehört nicht dazu. Das Etikett ist auf Foto F-297 zu sehen.</t>
+        </is>
+      </c>
+      <c r="AN259" s="22" t="n"/>
+    </row>
+    <row r="260" ht="30" customHeight="1">
+      <c r="A260" s="15" t="inlineStr">
+        <is>
+          <t>BA03-06</t>
+        </is>
+      </c>
+      <c r="B260" s="15" t="n"/>
+      <c r="C260" s="15" t="n"/>
+      <c r="D260" s="15" t="inlineStr">
+        <is>
+          <t>BA03</t>
+        </is>
+      </c>
+      <c r="E260" s="15" t="inlineStr">
+        <is>
+          <t>Kaufladen weiß mit Aufsatz</t>
+        </is>
+      </c>
+      <c r="F260" s="16" t="inlineStr">
+        <is>
+          <t>Kaufladen aus Holz, weiß mit grauer Rückwand: Verkaufstheke mit Ablage unten, Aufsatz mit mehreren unterschiedlich großen Fächern.</t>
+        </is>
+      </c>
+      <c r="G260" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H260" s="15" t="inlineStr">
+        <is>
+          <t>Galerie</t>
+        </is>
+      </c>
+      <c r="I260" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J260" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K260" s="17" t="n"/>
+      <c r="L260" s="18">
+        <f>J260-IF(K260="",0,K260)</f>
+        <v/>
+      </c>
+      <c r="M260" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N260" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O260" s="19" t="n"/>
+      <c r="P260" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q260" s="19" t="n"/>
+      <c r="R260" s="20" t="n"/>
+      <c r="S260" s="20" t="n">
+        <v>90</v>
+      </c>
+      <c r="T260" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U260" s="21">
+        <f>L260*S260</f>
+        <v/>
+      </c>
+      <c r="V260" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W260" s="15" t="inlineStr">
+        <is>
+          <t>F-298</t>
+        </is>
+      </c>
+      <c r="X260" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y260" s="19" t="n"/>
+      <c r="Z260" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA260" s="19" t="n"/>
+      <c r="AB260" s="19" t="n"/>
+      <c r="AC260" s="19" t="n"/>
+      <c r="AD260" s="19" t="n"/>
+      <c r="AE260" s="20" t="n"/>
+      <c r="AF260" s="21">
+        <f>IF(K260="","",K260*AE260)</f>
+        <v/>
+      </c>
+      <c r="AG260" s="19" t="n"/>
+      <c r="AH260" s="19" t="n"/>
+      <c r="AI260" s="19" t="n"/>
+      <c r="AJ260" s="19" t="n"/>
+      <c r="AK260" s="19" t="n"/>
+      <c r="AL260" s="19" t="n"/>
+      <c r="AM260" s="16" t="inlineStr">
+        <is>
+          <t>1 Kaufladen. Kasse, Spiellebensmittel und Geschirr gehören nicht dazu. Ein zweiter Kaufladen steht unter NU07-02.</t>
+        </is>
+      </c>
+      <c r="AN260" s="22" t="n"/>
+    </row>
+    <row r="261" ht="30" customHeight="1">
+      <c r="A261" s="15" t="inlineStr">
+        <is>
+          <t>BA03-07</t>
+        </is>
+      </c>
+      <c r="B261" s="15" t="n"/>
+      <c r="C261" s="15" t="n"/>
+      <c r="D261" s="15" t="inlineStr">
+        <is>
+          <t>BA03</t>
+        </is>
+      </c>
+      <c r="E261" s="15" t="inlineStr">
+        <is>
+          <t>Schrank weiß, zwei Türen</t>
+        </is>
+      </c>
+      <c r="F261" s="16" t="inlineStr">
+        <is>
+          <t>Hoher Schrank in Weiß mit zwei Türen und runden Porzellanknöpfen in Rosenform.</t>
+        </is>
+      </c>
+      <c r="G261" s="15" t="inlineStr">
+        <is>
+          <t>Möbel</t>
+        </is>
+      </c>
+      <c r="H261" s="15" t="inlineStr">
+        <is>
+          <t>Galerie</t>
+        </is>
+      </c>
+      <c r="I261" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J261" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K261" s="17" t="n"/>
+      <c r="L261" s="18">
+        <f>J261-IF(K261="",0,K261)</f>
+        <v/>
+      </c>
+      <c r="M261" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N261" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O261" s="19" t="n"/>
+      <c r="P261" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q261" s="19" t="n"/>
+      <c r="R261" s="20" t="n"/>
+      <c r="S261" s="20" t="n">
+        <v>80</v>
+      </c>
+      <c r="T261" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U261" s="21">
+        <f>L261*S261</f>
+        <v/>
+      </c>
+      <c r="V261" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W261" s="15" t="inlineStr">
+        <is>
+          <t>F-299</t>
+        </is>
+      </c>
+      <c r="X261" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y261" s="19" t="n"/>
+      <c r="Z261" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA261" s="19" t="n"/>
+      <c r="AB261" s="19" t="n"/>
+      <c r="AC261" s="19" t="n"/>
+      <c r="AD261" s="19" t="n"/>
+      <c r="AE261" s="20" t="n"/>
+      <c r="AF261" s="21">
+        <f>IF(K261="","",K261*AE261)</f>
+        <v/>
+      </c>
+      <c r="AG261" s="19" t="n"/>
+      <c r="AH261" s="19" t="n"/>
+      <c r="AI261" s="19" t="n"/>
+      <c r="AJ261" s="19" t="n"/>
+      <c r="AK261" s="19" t="n"/>
+      <c r="AL261" s="19" t="n"/>
+      <c r="AM261" s="16" t="inlineStr">
+        <is>
+          <t>1 Schrank.</t>
+        </is>
+      </c>
+      <c r="AN261" s="22" t="n"/>
+    </row>
+    <row r="262" ht="30" customHeight="1">
+      <c r="A262" s="15" t="inlineStr">
+        <is>
+          <t>BA03-04</t>
+        </is>
+      </c>
+      <c r="B262" s="15" t="n"/>
+      <c r="C262" s="15" t="n"/>
+      <c r="D262" s="15" t="inlineStr">
+        <is>
+          <t>BA03</t>
+        </is>
+      </c>
+      <c r="E262" s="15" t="inlineStr">
+        <is>
+          <t>Wandregal Hausform, schwarz</t>
+        </is>
+      </c>
+      <c r="F262" s="16" t="inlineStr">
+        <is>
+          <t>Wandregale in Hausform aus schwarz lackiertem Holz, zum Aufstellen oder Aufhängen, in unterschiedlichen Größen.</t>
+        </is>
+      </c>
+      <c r="G262" s="15" t="inlineStr">
+        <is>
+          <t>Deko</t>
+        </is>
+      </c>
+      <c r="H262" s="15" t="inlineStr">
+        <is>
+          <t>Galerie</t>
+        </is>
+      </c>
+      <c r="I262" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J262" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="K262" s="17" t="n"/>
+      <c r="L262" s="18">
+        <f>J262-IF(K262="",0,K262)</f>
+        <v/>
+      </c>
+      <c r="M262" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N262" s="15" t="inlineStr">
+        <is>
+          <t>gut</t>
+        </is>
+      </c>
+      <c r="O262" s="19" t="n"/>
+      <c r="P262" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q262" s="19" t="n"/>
+      <c r="R262" s="20" t="n"/>
+      <c r="S262" s="20" t="n">
+        <v>12</v>
+      </c>
+      <c r="T262" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U262" s="21">
+        <f>L262*S262</f>
+        <v/>
+      </c>
+      <c r="V262" s="15" t="inlineStr">
+        <is>
+          <t>Versand möglich</t>
+        </is>
+      </c>
+      <c r="W262" s="15" t="inlineStr">
+        <is>
+          <t>F-295</t>
+        </is>
+      </c>
+      <c r="X262" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y262" s="19" t="n"/>
+      <c r="Z262" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA262" s="19" t="n"/>
+      <c r="AB262" s="19" t="n"/>
+      <c r="AC262" s="19" t="n"/>
+      <c r="AD262" s="19" t="n"/>
+      <c r="AE262" s="20" t="n"/>
+      <c r="AF262" s="21">
+        <f>IF(K262="","",K262*AE262)</f>
+        <v/>
+      </c>
+      <c r="AG262" s="19" t="n"/>
+      <c r="AH262" s="19" t="n"/>
+      <c r="AI262" s="19" t="n"/>
+      <c r="AJ262" s="19" t="n"/>
+      <c r="AK262" s="19" t="n"/>
+      <c r="AL262" s="19" t="n"/>
+      <c r="AM262" s="16" t="inlineStr">
+        <is>
+          <t>5 Häuser in verschiedenen Größen. Der Inhalt gehört nicht dazu.</t>
+        </is>
+      </c>
+      <c r="AN262" s="22" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:AN255"/>
+  <autoFilter ref="A2:AN262"/>
   <mergeCells count="7">
     <mergeCell ref="AI1:AL1"/>
     <mergeCell ref="V1:AD1"/>
@@ -32188,7 +33033,7 @@
     <mergeCell ref="AE1:AH1"/>
     <mergeCell ref="AM1:AN1"/>
   </mergeCells>
-  <conditionalFormatting sqref="Z3:Z255">
+  <conditionalFormatting sqref="Z3:Z262">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"reserviert"</formula>
     </cfRule>
@@ -32199,12 +33044,12 @@
       <formula>"verkauft"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I3:I255">
+  <conditionalFormatting sqref="I3:I262">
     <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
       <formula>"A"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P3:P255">
+  <conditionalFormatting sqref="P3:P262">
     <cfRule type="cellIs" priority="5" operator="equal" dxfId="4">
       <formula>"entfällt"</formula>
     </cfRule>
@@ -32257,7 +33102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D89"/>
+  <dimension ref="A1:D90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -32295,7 +33140,7 @@
         </is>
       </c>
       <c r="B5" s="27">
-        <f>COUNTA(Artikelstamm!$A$3:$A$255)</f>
+        <f>COUNTA(Artikelstamm!$A$3:$A$262)</f>
         <v/>
       </c>
     </row>
@@ -32306,7 +33151,7 @@
         </is>
       </c>
       <c r="B6" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$255,"verfügbar")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$262,"verfügbar")</f>
         <v/>
       </c>
     </row>
@@ -32317,7 +33162,7 @@
         </is>
       </c>
       <c r="B7" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$255,"reserviert")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$262,"reserviert")</f>
         <v/>
       </c>
     </row>
@@ -32328,7 +33173,7 @@
         </is>
       </c>
       <c r="B8" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$255,"teilverkauft")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$262,"teilverkauft")</f>
         <v/>
       </c>
     </row>
@@ -32339,7 +33184,7 @@
         </is>
       </c>
       <c r="B9" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$255,"verkauft")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$262,"verkauft")</f>
         <v/>
       </c>
     </row>
@@ -32350,7 +33195,7 @@
         </is>
       </c>
       <c r="B10" s="27">
-        <f>SUM(Artikelstamm!$L$3:$L$255)</f>
+        <f>SUM(Artikelstamm!$L$3:$L$262)</f>
         <v/>
       </c>
     </row>
@@ -32361,7 +33206,7 @@
         </is>
       </c>
       <c r="B11" s="29">
-        <f>SUM(Artikelstamm!$U$3:$U$255)</f>
+        <f>SUM(Artikelstamm!$U$3:$U$262)</f>
         <v/>
       </c>
     </row>
@@ -32379,7 +33224,7 @@
         </is>
       </c>
       <c r="B13" s="27">
-        <f>SUM(Artikelstamm!$K$3:$K$255)</f>
+        <f>SUM(Artikelstamm!$K$3:$K$262)</f>
         <v/>
       </c>
     </row>
@@ -32390,7 +33235,7 @@
         </is>
       </c>
       <c r="B14" s="30">
-        <f>SUMPRODUCT(Artikelstamm!$K$3:$K$255,Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT(Artikelstamm!$K$3:$K$262,Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
     </row>
@@ -32423,7 +33268,7 @@
         </is>
       </c>
       <c r="B17" s="30">
-        <f>SUMPRODUCT((Artikelstamm!$AJ$3:$AJ$255="bezahlt")*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AJ$3:$AJ$262="bezahlt")*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
     </row>
@@ -32452,7 +33297,7 @@
         </is>
       </c>
       <c r="B21" s="31">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$255,"*verkauft",Artikelstamm!$AI$3:$AI$255,"")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$262,"*verkauft",Artikelstamm!$AI$3:$AI$262,"")</f>
         <v/>
       </c>
     </row>
@@ -32463,7 +33308,7 @@
         </is>
       </c>
       <c r="B22" s="31">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$255,"*verkauft",Artikelstamm!$AJ$3:$AJ$255,"offen")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$262,"*verkauft",Artikelstamm!$AJ$3:$AJ$262,"offen")</f>
         <v/>
       </c>
     </row>
@@ -32474,7 +33319,7 @@
         </is>
       </c>
       <c r="B23" s="27">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$255,"reserviert",Artikelstamm!$AL$3:$AL$255,"")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$262,"reserviert",Artikelstamm!$AL$3:$AL$262,"")</f>
         <v/>
       </c>
     </row>
@@ -32485,7 +33330,7 @@
         </is>
       </c>
       <c r="B24" s="27">
-        <f>COUNTIFS(Artikelstamm!$S$3:$S$255,"")</f>
+        <f>COUNTIFS(Artikelstamm!$S$3:$S$262,"")</f>
         <v/>
       </c>
     </row>
@@ -32496,7 +33341,7 @@
         </is>
       </c>
       <c r="B25" s="27">
-        <f>COUNTIFS(Artikelstamm!$O$3:$O$255,"")</f>
+        <f>COUNTIFS(Artikelstamm!$O$3:$O$262,"")</f>
         <v/>
       </c>
     </row>
@@ -32536,15 +33381,15 @@
         </is>
       </c>
       <c r="B30" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$255,$A30)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$262,$A30)</f>
         <v/>
       </c>
       <c r="C30" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$255=$A30)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$262=$A30)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
       <c r="D30" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$255,$A30,Artikelstamm!$U$3:$U$255)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$262,$A30,Artikelstamm!$U$3:$U$262)</f>
         <v/>
       </c>
     </row>
@@ -32555,15 +33400,15 @@
         </is>
       </c>
       <c r="B31" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$255,$A31)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$262,$A31)</f>
         <v/>
       </c>
       <c r="C31" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$255=$A31)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$262=$A31)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
       <c r="D31" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$255,$A31,Artikelstamm!$U$3:$U$255)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$262,$A31,Artikelstamm!$U$3:$U$262)</f>
         <v/>
       </c>
     </row>
@@ -32574,15 +33419,15 @@
         </is>
       </c>
       <c r="B32" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$255,$A32)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$262,$A32)</f>
         <v/>
       </c>
       <c r="C32" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$255=$A32)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$262=$A32)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
       <c r="D32" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$255,$A32,Artikelstamm!$U$3:$U$255)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$262,$A32,Artikelstamm!$U$3:$U$262)</f>
         <v/>
       </c>
     </row>
@@ -32641,15 +33486,15 @@
         </is>
       </c>
       <c r="B37" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$255,$A37)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$262,$A37)</f>
         <v/>
       </c>
       <c r="C37" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$255=$A37)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$262=$A37)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
       <c r="D37" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$255,$A37,Artikelstamm!$U$3:$U$255)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$262,$A37,Artikelstamm!$U$3:$U$262)</f>
         <v/>
       </c>
     </row>
@@ -32660,15 +33505,15 @@
         </is>
       </c>
       <c r="B38" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$255,$A38)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$262,$A38)</f>
         <v/>
       </c>
       <c r="C38" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$255=$A38)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$262=$A38)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
       <c r="D38" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$255,$A38,Artikelstamm!$U$3:$U$255)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$262,$A38,Artikelstamm!$U$3:$U$262)</f>
         <v/>
       </c>
     </row>
@@ -32679,15 +33524,15 @@
         </is>
       </c>
       <c r="B39" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$255,$A39)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$262,$A39)</f>
         <v/>
       </c>
       <c r="C39" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$255=$A39)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$262=$A39)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
       <c r="D39" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$255,$A39,Artikelstamm!$U$3:$U$255)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$262,$A39,Artikelstamm!$U$3:$U$262)</f>
         <v/>
       </c>
     </row>
@@ -32698,15 +33543,15 @@
         </is>
       </c>
       <c r="B40" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$255,$A40)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$262,$A40)</f>
         <v/>
       </c>
       <c r="C40" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$255=$A40)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$262=$A40)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
       <c r="D40" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$255,$A40,Artikelstamm!$U$3:$U$255)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$262,$A40,Artikelstamm!$U$3:$U$262)</f>
         <v/>
       </c>
     </row>
@@ -32717,15 +33562,15 @@
         </is>
       </c>
       <c r="B41" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$255,$A41)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$262,$A41)</f>
         <v/>
       </c>
       <c r="C41" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$255=$A41)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$262=$A41)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
       <c r="D41" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$255,$A41,Artikelstamm!$U$3:$U$255)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$262,$A41,Artikelstamm!$U$3:$U$262)</f>
         <v/>
       </c>
     </row>
@@ -32736,15 +33581,15 @@
         </is>
       </c>
       <c r="B42" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$255,$A42)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$262,$A42)</f>
         <v/>
       </c>
       <c r="C42" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$255=$A42)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$262=$A42)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
       <c r="D42" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$255,$A42,Artikelstamm!$U$3:$U$255)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$262,$A42,Artikelstamm!$U$3:$U$262)</f>
         <v/>
       </c>
     </row>
@@ -32755,15 +33600,15 @@
         </is>
       </c>
       <c r="B43" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$255,$A43)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$262,$A43)</f>
         <v/>
       </c>
       <c r="C43" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$255=$A43)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$262=$A43)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
       <c r="D43" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$255,$A43,Artikelstamm!$U$3:$U$255)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$262,$A43,Artikelstamm!$U$3:$U$262)</f>
         <v/>
       </c>
     </row>
@@ -32774,15 +33619,15 @@
         </is>
       </c>
       <c r="B44" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$255,$A44)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$262,$A44)</f>
         <v/>
       </c>
       <c r="C44" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$255=$A44)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$262=$A44)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
       <c r="D44" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$255,$A44,Artikelstamm!$U$3:$U$255)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$262,$A44,Artikelstamm!$U$3:$U$262)</f>
         <v/>
       </c>
     </row>
@@ -32793,15 +33638,15 @@
         </is>
       </c>
       <c r="B45" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$255,$A45)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$262,$A45)</f>
         <v/>
       </c>
       <c r="C45" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$255=$A45)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$262=$A45)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
       <c r="D45" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$255,$A45,Artikelstamm!$U$3:$U$255)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$262,$A45,Artikelstamm!$U$3:$U$262)</f>
         <v/>
       </c>
     </row>
@@ -32812,15 +33657,15 @@
         </is>
       </c>
       <c r="B46" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$255,$A46)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$262,$A46)</f>
         <v/>
       </c>
       <c r="C46" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$255=$A46)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$262=$A46)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
       <c r="D46" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$255,$A46,Artikelstamm!$U$3:$U$255)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$262,$A46,Artikelstamm!$U$3:$U$262)</f>
         <v/>
       </c>
     </row>
@@ -32831,15 +33676,15 @@
         </is>
       </c>
       <c r="B47" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$255,$A47)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$262,$A47)</f>
         <v/>
       </c>
       <c r="C47" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$255=$A47)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$262=$A47)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
       <c r="D47" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$255,$A47,Artikelstamm!$U$3:$U$255)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$262,$A47,Artikelstamm!$U$3:$U$262)</f>
         <v/>
       </c>
     </row>
@@ -32850,15 +33695,15 @@
         </is>
       </c>
       <c r="B48" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$255,$A48)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$262,$A48)</f>
         <v/>
       </c>
       <c r="C48" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$255=$A48)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$262=$A48)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
       <c r="D48" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$255,$A48,Artikelstamm!$U$3:$U$255)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$262,$A48,Artikelstamm!$U$3:$U$262)</f>
         <v/>
       </c>
     </row>
@@ -32869,15 +33714,15 @@
         </is>
       </c>
       <c r="B49" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$255,$A49)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$262,$A49)</f>
         <v/>
       </c>
       <c r="C49" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$255=$A49)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$262=$A49)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
       <c r="D49" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$255,$A49,Artikelstamm!$U$3:$U$255)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$262,$A49,Artikelstamm!$U$3:$U$262)</f>
         <v/>
       </c>
     </row>
@@ -32888,15 +33733,15 @@
         </is>
       </c>
       <c r="B50" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$255,$A50)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$262,$A50)</f>
         <v/>
       </c>
       <c r="C50" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$255=$A50)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$262=$A50)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
       <c r="D50" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$255,$A50,Artikelstamm!$U$3:$U$255)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$262,$A50,Artikelstamm!$U$3:$U$262)</f>
         <v/>
       </c>
     </row>
@@ -32955,15 +33800,15 @@
         </is>
       </c>
       <c r="B55" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$255,$A55)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$262,$A55)</f>
         <v/>
       </c>
       <c r="C55" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$255=$A55)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$262=$A55)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
       <c r="D55" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$255,$A55,Artikelstamm!$U$3:$U$255)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$262,$A55,Artikelstamm!$U$3:$U$262)</f>
         <v/>
       </c>
     </row>
@@ -32974,15 +33819,15 @@
         </is>
       </c>
       <c r="B56" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$255,$A56)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$262,$A56)</f>
         <v/>
       </c>
       <c r="C56" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$255=$A56)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$262=$A56)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
       <c r="D56" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$255,$A56,Artikelstamm!$U$3:$U$255)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$262,$A56,Artikelstamm!$U$3:$U$262)</f>
         <v/>
       </c>
     </row>
@@ -32993,15 +33838,15 @@
         </is>
       </c>
       <c r="B57" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$255,$A57)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$262,$A57)</f>
         <v/>
       </c>
       <c r="C57" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$255=$A57)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$262=$A57)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
       <c r="D57" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$255,$A57,Artikelstamm!$U$3:$U$255)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$262,$A57,Artikelstamm!$U$3:$U$262)</f>
         <v/>
       </c>
     </row>
@@ -33012,15 +33857,15 @@
         </is>
       </c>
       <c r="B58" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$255,$A58)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$262,$A58)</f>
         <v/>
       </c>
       <c r="C58" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$255=$A58)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$262=$A58)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
       <c r="D58" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$255,$A58,Artikelstamm!$U$3:$U$255)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$262,$A58,Artikelstamm!$U$3:$U$262)</f>
         <v/>
       </c>
     </row>
@@ -33031,15 +33876,15 @@
         </is>
       </c>
       <c r="B59" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$255,$A59)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$262,$A59)</f>
         <v/>
       </c>
       <c r="C59" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$255=$A59)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$262=$A59)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
       <c r="D59" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$255,$A59,Artikelstamm!$U$3:$U$255)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$262,$A59,Artikelstamm!$U$3:$U$262)</f>
         <v/>
       </c>
     </row>
@@ -33050,15 +33895,15 @@
         </is>
       </c>
       <c r="B60" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$255,$A60)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$262,$A60)</f>
         <v/>
       </c>
       <c r="C60" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$255=$A60)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$262=$A60)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
       <c r="D60" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$255,$A60,Artikelstamm!$U$3:$U$255)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$262,$A60,Artikelstamm!$U$3:$U$262)</f>
         <v/>
       </c>
     </row>
@@ -33069,486 +33914,505 @@
         </is>
       </c>
       <c r="B61" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$255,$A61)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$262,$A61)</f>
         <v/>
       </c>
       <c r="C61" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$255=$A61)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$262=$A61)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
       <c r="D61" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$255,$A61,Artikelstamm!$U$3:$U$255)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$262,$A61,Artikelstamm!$U$3:$U$262)</f>
         <v/>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="26" t="inlineStr">
         <is>
-          <t>Garage</t>
+          <t>Galerie</t>
         </is>
       </c>
       <c r="B62" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$255,$A62)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$262,$A62)</f>
         <v/>
       </c>
       <c r="C62" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$255=$A62)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$262=$A62)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
       <c r="D62" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$255,$A62,Artikelstamm!$U$3:$U$255)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$262,$A62,Artikelstamm!$U$3:$U$262)</f>
         <v/>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="26" t="inlineStr">
         <is>
-          <t>Gartenanlage</t>
+          <t>Garage</t>
         </is>
       </c>
       <c r="B63" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$255,$A63)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$262,$A63)</f>
         <v/>
       </c>
       <c r="C63" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$255=$A63)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$262=$A63)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
       <c r="D63" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$255,$A63,Artikelstamm!$U$3:$U$255)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$262,$A63,Artikelstamm!$U$3:$U$262)</f>
         <v/>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="26" t="inlineStr">
         <is>
-          <t>Gruppenraum</t>
+          <t>Gartenanlage</t>
         </is>
       </c>
       <c r="B64" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$255,$A64)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$262,$A64)</f>
         <v/>
       </c>
       <c r="C64" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$255=$A64)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$262=$A64)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
       <c r="D64" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$255,$A64,Artikelstamm!$U$3:$U$255)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$262,$A64,Artikelstamm!$U$3:$U$262)</f>
         <v/>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="26" t="inlineStr">
         <is>
-          <t>Gruppenraum 2</t>
+          <t>Gruppenraum</t>
         </is>
       </c>
       <c r="B65" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$255,$A65)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$262,$A65)</f>
         <v/>
       </c>
       <c r="C65" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$255=$A65)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$262=$A65)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
       <c r="D65" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$255,$A65,Artikelstamm!$U$3:$U$255)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$262,$A65,Artikelstamm!$U$3:$U$262)</f>
         <v/>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="26" t="inlineStr">
         <is>
-          <t>Gruppenraum 4</t>
+          <t>Gruppenraum 2</t>
         </is>
       </c>
       <c r="B66" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$255,$A66)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$262,$A66)</f>
         <v/>
       </c>
       <c r="C66" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$255=$A66)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$262=$A66)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
       <c r="D66" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$255,$A66,Artikelstamm!$U$3:$U$255)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$262,$A66,Artikelstamm!$U$3:$U$262)</f>
         <v/>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="26" t="inlineStr">
         <is>
-          <t>Gruppenraum 5</t>
+          <t>Gruppenraum 4</t>
         </is>
       </c>
       <c r="B67" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$255,$A67)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$262,$A67)</f>
         <v/>
       </c>
       <c r="C67" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$255=$A67)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$262=$A67)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
       <c r="D67" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$255,$A67,Artikelstamm!$U$3:$U$255)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$262,$A67,Artikelstamm!$U$3:$U$262)</f>
         <v/>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="26" t="inlineStr">
         <is>
-          <t>Küche</t>
+          <t>Gruppenraum 5</t>
         </is>
       </c>
       <c r="B68" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$255,$A68)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$262,$A68)</f>
         <v/>
       </c>
       <c r="C68" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$255=$A68)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$262=$A68)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
       <c r="D68" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$255,$A68,Artikelstamm!$U$3:$U$255)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$262,$A68,Artikelstamm!$U$3:$U$262)</f>
         <v/>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="26" t="inlineStr">
         <is>
-          <t>Personal</t>
+          <t>Küche</t>
         </is>
       </c>
       <c r="B69" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$255,$A69)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$262,$A69)</f>
         <v/>
       </c>
       <c r="C69" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$255=$A69)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$262=$A69)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
       <c r="D69" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$255,$A69,Artikelstamm!$U$3:$U$255)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$262,$A69,Artikelstamm!$U$3:$U$262)</f>
         <v/>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="26" t="inlineStr">
         <is>
-          <t>Ruhe- / Schlafraum</t>
+          <t>Personal</t>
         </is>
       </c>
       <c r="B70" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$255,$A70)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$262,$A70)</f>
         <v/>
       </c>
       <c r="C70" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$255=$A70)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$262=$A70)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
       <c r="D70" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$255,$A70,Artikelstamm!$U$3:$U$255)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$262,$A70,Artikelstamm!$U$3:$U$262)</f>
         <v/>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="26" t="inlineStr">
         <is>
-          <t>Schlafraum 4</t>
+          <t>Ruhe- / Schlafraum</t>
         </is>
       </c>
       <c r="B71" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$255,$A71)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$262,$A71)</f>
         <v/>
       </c>
       <c r="C71" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$255=$A71)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$262=$A71)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
       <c r="D71" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$255,$A71,Artikelstamm!$U$3:$U$255)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$262,$A71,Artikelstamm!$U$3:$U$262)</f>
         <v/>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="26" t="inlineStr">
         <is>
-          <t>Schlafraum 5</t>
+          <t>Schlafraum 4</t>
         </is>
       </c>
       <c r="B72" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$255,$A72)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$262,$A72)</f>
         <v/>
       </c>
       <c r="C72" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$255=$A72)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$262=$A72)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
       <c r="D72" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$255,$A72,Artikelstamm!$U$3:$U$255)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$262,$A72,Artikelstamm!$U$3:$U$262)</f>
         <v/>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="26" t="inlineStr">
         <is>
-          <t>Speisesaal</t>
+          <t>Schlafraum 5</t>
         </is>
       </c>
       <c r="B73" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$255,$A73)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$262,$A73)</f>
         <v/>
       </c>
       <c r="C73" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$255=$A73)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$262=$A73)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
       <c r="D73" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$255,$A73,Artikelstamm!$U$3:$U$255)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$262,$A73,Artikelstamm!$U$3:$U$262)</f>
         <v/>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="26" t="inlineStr">
         <is>
-          <t>Terrasse</t>
+          <t>Speisesaal</t>
         </is>
       </c>
       <c r="B74" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$255,$A74)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$262,$A74)</f>
         <v/>
       </c>
       <c r="C74" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$255=$A74)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$262=$A74)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
       <c r="D74" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$255,$A74,Artikelstamm!$U$3:$U$255)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$262,$A74,Artikelstamm!$U$3:$U$262)</f>
         <v/>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="26" t="inlineStr">
         <is>
-          <t>Treppenraum 1</t>
+          <t>Terrasse</t>
         </is>
       </c>
       <c r="B75" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$255,$A75)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$262,$A75)</f>
         <v/>
       </c>
       <c r="C75" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$255=$A75)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$262=$A75)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
       <c r="D75" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$255,$A75,Artikelstamm!$U$3:$U$255)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$262,$A75,Artikelstamm!$U$3:$U$262)</f>
         <v/>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="26" t="inlineStr">
         <is>
-          <t>WC</t>
+          <t>Treppenraum 1</t>
         </is>
       </c>
       <c r="B76" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$255,$A76)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$262,$A76)</f>
         <v/>
       </c>
       <c r="C76" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$255=$A76)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$262=$A76)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
       <c r="D76" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$255,$A76,Artikelstamm!$U$3:$U$255)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$262,$A76,Artikelstamm!$U$3:$U$262)</f>
         <v/>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="26" t="inlineStr">
         <is>
-          <t>WC Personal</t>
+          <t>WC</t>
         </is>
       </c>
       <c r="B77" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$255,$A77)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$262,$A77)</f>
         <v/>
       </c>
       <c r="C77" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$255=$A77)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$262=$A77)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
       <c r="D77" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$255,$A77,Artikelstamm!$U$3:$U$255)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$262,$A77,Artikelstamm!$U$3:$U$262)</f>
         <v/>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="26" t="inlineStr">
         <is>
+          <t>WC Personal</t>
+        </is>
+      </c>
+      <c r="B78" s="33">
+        <f>COUNTIF(Artikelstamm!$H$3:$H$262,$A78)</f>
+        <v/>
+      </c>
+      <c r="C78" s="34">
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$262=$A78)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
+        <v/>
+      </c>
+      <c r="D78" s="34">
+        <f>SUMIF(Artikelstamm!$H$3:$H$262,$A78,Artikelstamm!$U$3:$U$262)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="26" t="inlineStr">
+        <is>
           <t>Werkraum</t>
         </is>
       </c>
-      <c r="B78" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$255,$A78)</f>
-        <v/>
-      </c>
-      <c r="C78" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$255=$A78)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
-        <v/>
-      </c>
-      <c r="D78" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$255,$A78,Artikelstamm!$U$3:$U$255)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="28" t="inlineStr">
+      <c r="B79" s="33">
+        <f>COUNTIF(Artikelstamm!$H$3:$H$262,$A79)</f>
+        <v/>
+      </c>
+      <c r="C79" s="34">
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$262=$A79)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
+        <v/>
+      </c>
+      <c r="D79" s="34">
+        <f>SUMIF(Artikelstamm!$H$3:$H$262,$A79,Artikelstamm!$U$3:$U$262)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="28" t="inlineStr">
         <is>
           <t>Summe</t>
         </is>
       </c>
-      <c r="B79" s="35">
-        <f>SUM(B55:B78)</f>
-        <v/>
-      </c>
-      <c r="C79" s="36">
-        <f>SUM(C55:C78)</f>
-        <v/>
-      </c>
-      <c r="D79" s="36">
-        <f>SUM(D55:D78)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="25" t="inlineStr">
+      <c r="B80" s="35">
+        <f>SUM(B55:B79)</f>
+        <v/>
+      </c>
+      <c r="C80" s="36">
+        <f>SUM(C55:C79)</f>
+        <v/>
+      </c>
+      <c r="D80" s="36">
+        <f>SUM(D55:D79)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="25" t="inlineStr">
         <is>
           <t>Nach Verkaufskanal</t>
         </is>
       </c>
     </row>
-    <row r="82">
-      <c r="A82" s="32" t="inlineStr">
+    <row r="83">
+      <c r="A83" s="32" t="inlineStr">
         <is>
           <t>Verkaufskanal</t>
         </is>
       </c>
-      <c r="B82" s="32" t="inlineStr">
+      <c r="B83" s="32" t="inlineStr">
         <is>
           <t>Positionen</t>
         </is>
       </c>
-      <c r="C82" s="32" t="inlineStr">
+      <c r="C83" s="32" t="inlineStr">
         <is>
           <t>Umsatz netto</t>
         </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="26" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
-      <c r="B83" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$255,$A83)</f>
-        <v/>
-      </c>
-      <c r="C83" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$255=$A83)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
-        <v/>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="26" t="inlineStr">
         <is>
-          <t>Kleinanzeigen</t>
+          <t>Klinik</t>
         </is>
       </c>
       <c r="B84" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$255,$A84)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$262,$A84)</f>
         <v/>
       </c>
       <c r="C84" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$255=$A84)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$262=$A84)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="26" t="inlineStr">
         <is>
-          <t>eBay</t>
+          <t>Kleinanzeigen</t>
         </is>
       </c>
       <c r="B85" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$255,$A85)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$262,$A85)</f>
         <v/>
       </c>
       <c r="C85" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$255=$A85)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$262=$A85)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="26" t="inlineStr">
         <is>
-          <t>Direkt</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="B86" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$255,$A86)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$262,$A86)</f>
         <v/>
       </c>
       <c r="C86" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$255=$A86)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$262=$A86)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="26" t="inlineStr">
         <is>
-          <t>Händler</t>
+          <t>Direkt</t>
         </is>
       </c>
       <c r="B87" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$255,$A87)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$262,$A87)</f>
         <v/>
       </c>
       <c r="C87" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$255=$A87)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$262=$A87)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
         <v/>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="26" t="inlineStr">
         <is>
+          <t>Händler</t>
+        </is>
+      </c>
+      <c r="B88" s="33">
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$262,$A88)</f>
+        <v/>
+      </c>
+      <c r="C88" s="34">
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$262=$A88)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="26" t="inlineStr">
+        <is>
           <t>Verkaufstag</t>
         </is>
       </c>
-      <c r="B88" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$255,$A88)</f>
-        <v/>
-      </c>
-      <c r="C88" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$255=$A88)*Artikelstamm!$K$3:$K$255*Artikelstamm!$AE$3:$AE$255)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" s="28" t="inlineStr">
+      <c r="B89" s="33">
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$262,$A89)</f>
+        <v/>
+      </c>
+      <c r="C89" s="34">
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$262=$A89)*Artikelstamm!$K$3:$K$262*Artikelstamm!$AE$3:$AE$262)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="28" t="inlineStr">
         <is>
           <t>Summe</t>
         </is>
       </c>
-      <c r="B89" s="35">
-        <f>SUM(B83:B88)</f>
-        <v/>
-      </c>
-      <c r="C89" s="36">
-        <f>SUM(C83:C88)</f>
+      <c r="B90" s="35">
+        <f>SUM(B84:B89)</f>
+        <v/>
+      </c>
+      <c r="C90" s="36">
+        <f>SUM(C84:C89)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
BA05-05 und BA05-10 mit Foto, wieder im Katalog
Beide Bilder sind jetzt als Datei angekommen (F-321, F-322). Die
OFFEN-Vermerke entfallen, Im_Katalog wieder auf ja - damit sind 475 EUR
zurueck im Katalog.

BA05-10 heisst jetzt Polstersaeule statt Wandschutz: das Foto zeigt eine
Standsaeule aus Schaumstoff mit Bluetenquerschnitt, gruener Mantel und
graue Oberseiten. Als Saeulenschutz und als Raumteiler nutzbar - das
beschreibt sie treffender und trifft mehr Interessenten.

pruefen.py: 0 Fehler, 3 Hinweise.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011yyfqhuiWGsaNy38oaNoGo
</commit_message>
<xml_diff>
--- a/ausgabe/01_Artikelstamm_kikripp.xlsx
+++ b/ausgabe/01_Artikelstamm_kikripp.xlsx
@@ -34026,7 +34026,7 @@
       </c>
       <c r="F271" s="16" t="inlineStr">
         <is>
-          <t>Sprossenwand aus Massivholz zur Wandmontage, mit Querholmen über die volle Breite.</t>
+          <t>Sprossenwand aus Massivholz zur Wandmontage: zwei kräftige Holme mit durchgehenden Rundsprossen, oben eine ausladende Aufhängeleiste.</t>
         </is>
       </c>
       <c r="G271" s="15" t="inlineStr">
@@ -34087,10 +34087,14 @@
           <t>nur Abholung</t>
         </is>
       </c>
-      <c r="W271" s="15" t="n"/>
+      <c r="W271" s="15" t="inlineStr">
+        <is>
+          <t>F-321</t>
+        </is>
+      </c>
       <c r="X271" s="19" t="inlineStr">
         <is>
-          <t>nein</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="Y271" s="19" t="n"/>
@@ -34116,14 +34120,10 @@
       <c r="AL271" s="19" t="n"/>
       <c r="AM271" s="16" t="inlineStr">
         <is>
-          <t>3 Sprossenwände.</t>
-        </is>
-      </c>
-      <c r="AN271" s="22" t="inlineStr">
-        <is>
-          <t>OFFEN: Foto fehlt. Das Bild kam nur als Chatbild an, nicht als Datei - es konnte deshalb nicht in die Fotoverarbeitung. Bitte als Dateianhang nachreichen.</t>
-        </is>
-      </c>
+          <t>3 Sprossenwände – abgebildet ist eine davon.</t>
+        </is>
+      </c>
+      <c r="AN271" s="22" t="n"/>
     </row>
     <row r="272" ht="30" customHeight="1">
       <c r="A272" s="15" t="inlineStr">
@@ -34620,12 +34620,12 @@
       </c>
       <c r="E276" s="15" t="inlineStr">
         <is>
-          <t>Wandschutz grün, gepolstert</t>
+          <t>Polstersäule grün, Raumteiler</t>
         </is>
       </c>
       <c r="F276" s="16" t="inlineStr">
         <is>
-          <t>Gepolsterter Wand- und Säulenschutz mit grünem Kunstlederbezug und grauer Oberseite.</t>
+          <t>Standsäule aus Schaumstoff mit Kunstlederbezug: Mantel in Limettengrün, Oberseiten in Grau, mehrere Lappen ergeben im Querschnitt eine Blütenform. Als Wand- und Säulenschutz oder als Raumteiler nutzbar.</t>
         </is>
       </c>
       <c r="G276" s="15" t="inlineStr">
@@ -34686,10 +34686,14 @@
           <t>nur Abholung</t>
         </is>
       </c>
-      <c r="W276" s="15" t="n"/>
+      <c r="W276" s="15" t="inlineStr">
+        <is>
+          <t>F-322</t>
+        </is>
+      </c>
       <c r="X276" s="19" t="inlineStr">
         <is>
-          <t>nein</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="Y276" s="19" t="n"/>
@@ -34715,14 +34719,10 @@
       <c r="AL276" s="19" t="n"/>
       <c r="AM276" s="16" t="inlineStr">
         <is>
-          <t>5 Elemente.</t>
-        </is>
-      </c>
-      <c r="AN276" s="22" t="inlineStr">
-        <is>
-          <t>OFFEN: Foto fehlt. Das Bild kam nur als Chatbild an, nicht als Datei - es konnte deshalb nicht in die Fotoverarbeitung. Bitte als Dateianhang nachreichen.</t>
-        </is>
-      </c>
+          <t>5 Säulen – abgebildet sind sie zusammengestellt.</t>
+        </is>
+      </c>
+      <c r="AN276" s="22" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A2:AN276"/>

</xml_diff>

<commit_message>
BA06-09 und BA06-12 mit Foto, Raumteiler bestaetigt
Beide Bilder sind als Datei angekommen (F-335, F-336), die OFFEN-Vermerke
entfallen. Beim Spieltunnel gibt es nur das Bild des Kartons - das steht
jetzt im Mengenhinweis, damit kein Kaeufer ein Studiofoto erwartet.

Die Nutzerin hat bestaetigt: BA06-13 ist derselbe Raumteiler wie
NU04-14. Die Rueckfrage in der Bemerkung ist entfernt.

Zur Fotouebertragung: die Nutzerin waehlt die Bilder immer gleich aus.
Die frueher geaeusserte Vermutung, es liege an der Auswahl, war also
falsch - manche Bilder kommen als Datei an, manche nur als Chatbild, ohne
erkennbares Zutun. Das erneute Schicken hilft zuverlaessig.

pruefen.py: 0 Fehler, 3 Hinweise.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011yyfqhuiWGsaNy38oaNoGo
</commit_message>
<xml_diff>
--- a/ausgabe/01_Artikelstamm_kikripp.xlsx
+++ b/ausgabe/01_Artikelstamm_kikripp.xlsx
@@ -24588,7 +24588,7 @@
       </c>
       <c r="AN192" s="22" t="inlineStr">
         <is>
-          <t>Zusammengefasste Position – Post-it-Nummer im zweiten Raum: BA06-13. Zusammenfassung aus dem Rautenmuster geschlossen, bitte bestaetigen.</t>
+          <t>Zusammengefasste Position – Post-it-Nummer im zweiten Raum: BA06-13.</t>
         </is>
       </c>
     </row>
@@ -35605,7 +35605,7 @@
       </c>
       <c r="F284" s="16" t="inlineStr">
         <is>
-          <t>Rutschfahrzeug aus Massivholz in Lastwagenform mit offener Ladefläche, Holzlenkrad und roten Rädern.</t>
+          <t>Rutschfahrzeug aus Massivholz in Lastwagenform: offene Ladefläche mit Bordwänden, gepolsterter Sitz vor dem Führerhaus, Holzlenkrad und vier Gummiräder mit roten Felgen.</t>
         </is>
       </c>
       <c r="G284" s="15" t="inlineStr">
@@ -35666,10 +35666,14 @@
           <t>nur Abholung</t>
         </is>
       </c>
-      <c r="W284" s="15" t="n"/>
+      <c r="W284" s="15" t="inlineStr">
+        <is>
+          <t>F-335</t>
+        </is>
+      </c>
       <c r="X284" s="19" t="inlineStr">
         <is>
-          <t>nein</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="Y284" s="19" t="n"/>
@@ -35698,11 +35702,7 @@
           <t>1 Fahrzeug.</t>
         </is>
       </c>
-      <c r="AN284" s="22" t="inlineStr">
-        <is>
-          <t>OFFEN: Foto fehlt. Das Bild kam nur als Chatbild an, nicht als Datei. Bitte als Dateianhang nachreichen.</t>
-        </is>
-      </c>
+      <c r="AN284" s="22" t="n"/>
     </row>
     <row r="285" ht="30" customHeight="1">
       <c r="A285" s="15" t="inlineStr">
@@ -35957,12 +35957,12 @@
       </c>
       <c r="E287" s="15" t="inlineStr">
         <is>
-          <t>Spieltunnel grün</t>
+          <t>Spieltunnel grün, 180 cm</t>
         </is>
       </c>
       <c r="F287" s="16" t="inlineStr">
         <is>
-          <t>Spieltunnel aus grünem Stoff mit roten Ringen, etwa 180 cm lang und 45 cm Durchmesser, zusammenfaltbar, mit Originalkarton.</t>
+          <t>Spieltunnel aus grünem Stoff mit roten Ringen, etwa 180 cm lang bei 45 cm Durchmesser. Faltbar, mit Originalkarton.</t>
         </is>
       </c>
       <c r="G287" s="15" t="inlineStr">
@@ -36023,10 +36023,14 @@
           <t>nur Abholung</t>
         </is>
       </c>
-      <c r="W287" s="15" t="n"/>
+      <c r="W287" s="15" t="inlineStr">
+        <is>
+          <t>F-336</t>
+        </is>
+      </c>
       <c r="X287" s="19" t="inlineStr">
         <is>
-          <t>nein</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="Y287" s="19" t="n"/>
@@ -36052,14 +36056,10 @@
       <c r="AL287" s="19" t="n"/>
       <c r="AM287" s="16" t="inlineStr">
         <is>
-          <t>1 Tunnel.</t>
-        </is>
-      </c>
-      <c r="AN287" s="22" t="inlineStr">
-        <is>
-          <t>OFFEN: Foto fehlt. Das Bild des Kartons kam nur als Chatbild an, nicht als Datei. Besser waere ohnehin ein Foto des aufgebauten Tunnels.</t>
-        </is>
-      </c>
+          <t>1 Tunnel. Das Foto zeigt den Originalkarton mit der Abbildung; der Tunnel selbst ist zusammengefaltet darin.</t>
+        </is>
+      </c>
+      <c r="AN287" s="22" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A2:AN287"/>

</xml_diff>

<commit_message>
BA07 erfasst: 5 Positionen, vierzehnte Zusammenfassung
Klassenzimmer (Bestandsgebaeude Attika, 19,37 m2).

BA07-04 ist derselbe weisse Drahtkorbtisch wie BA04-07; zusammengefasst
auf 2 Stueck. Im Mengenhinweis steht zusaetzlich der Verweis auf die zwei
baugleichen in Kupfer (NU02-07) - so sieht ein Interessent alle vier.

Bei BA07-05 fehlt die Stueckzahl auf dem Erfassungsblatt, als 1
angenommen und zur Bestaetigung vermerkt.

Gesamtwert netto 41.802 -> 42.156 EUR, 235 aktive Positionen.
pruefen.py: 0 Fehler, 3 Hinweise.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011yyfqhuiWGsaNy38oaNoGo
</commit_message>
<xml_diff>
--- a/ausgabe/01_Artikelstamm_kikripp.xlsx
+++ b/ausgabe/01_Artikelstamm_kikripp.xlsx
@@ -15,7 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Artikelstamm'!$A$2:$AN$287</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Artikelstamm'!$A$2:$AN$292</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1019,7 +1019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN287"/>
+  <dimension ref="A1:AN292"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -33414,7 +33414,11 @@
         </is>
       </c>
       <c r="B266" s="15" t="n"/>
-      <c r="C266" s="15" t="n"/>
+      <c r="C266" s="15" t="inlineStr">
+        <is>
+          <t>BA07-04</t>
+        </is>
+      </c>
       <c r="D266" s="15" t="inlineStr">
         <is>
           <t>BA04</t>
@@ -33446,7 +33450,7 @@
         </is>
       </c>
       <c r="J266" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K266" s="17" t="n"/>
       <c r="L266" s="18">
@@ -33521,10 +33525,14 @@
       <c r="AL266" s="19" t="n"/>
       <c r="AM266" s="16" t="inlineStr">
         <is>
-          <t>1 Tisch. Baugleich in Kupfer gibt es zwei Stück unter NU02-07.</t>
-        </is>
-      </c>
-      <c r="AN266" s="22" t="n"/>
+          <t>2 Tische: einer im Gruppenraum 4 (BA04-07) und einer im Klassenzimmer (dort mit BA07-04 beschriftet). Der Inhalt gehört nicht dazu. Baugleich in Kupfer gibt es zwei Stück unter NU02-07.</t>
+        </is>
+      </c>
+      <c r="AN266" s="22" t="inlineStr">
+        <is>
+          <t>Zusammengefasste Position – Post-it-Nummer im zweiten Raum: BA07-04.</t>
+        </is>
+      </c>
     </row>
     <row r="267" ht="30" customHeight="1">
       <c r="A267" s="15" t="inlineStr">
@@ -36061,8 +36069,607 @@
       </c>
       <c r="AN287" s="22" t="n"/>
     </row>
+    <row r="288" ht="30" customHeight="1">
+      <c r="A288" s="15" t="inlineStr">
+        <is>
+          <t>BA07-01</t>
+        </is>
+      </c>
+      <c r="B288" s="15" t="n"/>
+      <c r="C288" s="15" t="n"/>
+      <c r="D288" s="15" t="inlineStr">
+        <is>
+          <t>BA07</t>
+        </is>
+      </c>
+      <c r="E288" s="15" t="inlineStr">
+        <is>
+          <t>Kissen in Wolkenform, hellblau</t>
+        </is>
+      </c>
+      <c r="F288" s="16" t="inlineStr">
+        <is>
+          <t>Dekokissen in Wolkenform aus hellblauem Samtstoff, mit aufgestickten Augen, Lächeln und rosa Wangen.</t>
+        </is>
+      </c>
+      <c r="G288" s="15" t="inlineStr">
+        <is>
+          <t>Textilien</t>
+        </is>
+      </c>
+      <c r="H288" s="15" t="inlineStr">
+        <is>
+          <t>Klassenzimmer</t>
+        </is>
+      </c>
+      <c r="I288" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J288" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K288" s="17" t="n"/>
+      <c r="L288" s="18">
+        <f>J288-IF(K288="",0,K288)</f>
+        <v/>
+      </c>
+      <c r="M288" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N288" s="15" t="inlineStr">
+        <is>
+          <t>gut</t>
+        </is>
+      </c>
+      <c r="O288" s="19" t="n"/>
+      <c r="P288" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q288" s="19" t="n"/>
+      <c r="R288" s="20" t="n"/>
+      <c r="S288" s="20" t="n">
+        <v>12</v>
+      </c>
+      <c r="T288" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U288" s="21">
+        <f>L288*S288</f>
+        <v/>
+      </c>
+      <c r="V288" s="15" t="inlineStr">
+        <is>
+          <t>Versand möglich</t>
+        </is>
+      </c>
+      <c r="W288" s="15" t="inlineStr">
+        <is>
+          <t>F-337</t>
+        </is>
+      </c>
+      <c r="X288" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y288" s="19" t="n"/>
+      <c r="Z288" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA288" s="19" t="n"/>
+      <c r="AB288" s="19" t="n"/>
+      <c r="AC288" s="19" t="n"/>
+      <c r="AD288" s="19" t="n"/>
+      <c r="AE288" s="20" t="n"/>
+      <c r="AF288" s="21">
+        <f>IF(K288="","",K288*AE288)</f>
+        <v/>
+      </c>
+      <c r="AG288" s="19" t="n"/>
+      <c r="AH288" s="19" t="n"/>
+      <c r="AI288" s="19" t="n"/>
+      <c r="AJ288" s="19" t="n"/>
+      <c r="AK288" s="19" t="n"/>
+      <c r="AL288" s="19" t="n"/>
+      <c r="AM288" s="16" t="inlineStr">
+        <is>
+          <t>2 Kissen, beide abgebildet.</t>
+        </is>
+      </c>
+      <c r="AN288" s="22" t="n"/>
+    </row>
+    <row r="289" ht="30" customHeight="1">
+      <c r="A289" s="15" t="inlineStr">
+        <is>
+          <t>BA07-02</t>
+        </is>
+      </c>
+      <c r="B289" s="15" t="n"/>
+      <c r="C289" s="15" t="n"/>
+      <c r="D289" s="15" t="inlineStr">
+        <is>
+          <t>BA07</t>
+        </is>
+      </c>
+      <c r="E289" s="15" t="inlineStr">
+        <is>
+          <t>Wandleuchte rund mit Holzrand</t>
+        </is>
+      </c>
+      <c r="F289" s="16" t="inlineStr">
+        <is>
+          <t>Runde Wandleuchte: Rahmen aus gebogenem Schichtholz mit satinierter Scheibe, flache Bauform, Zuleitung sichtbar verlegt. Zwei verschiedene Durchmesser.</t>
+        </is>
+      </c>
+      <c r="G289" s="15" t="inlineStr">
+        <is>
+          <t>Leuchten</t>
+        </is>
+      </c>
+      <c r="H289" s="15" t="inlineStr">
+        <is>
+          <t>Klassenzimmer</t>
+        </is>
+      </c>
+      <c r="I289" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J289" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K289" s="17" t="n"/>
+      <c r="L289" s="18">
+        <f>J289-IF(K289="",0,K289)</f>
+        <v/>
+      </c>
+      <c r="M289" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N289" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O289" s="19" t="n"/>
+      <c r="P289" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q289" s="19" t="n"/>
+      <c r="R289" s="20" t="n"/>
+      <c r="S289" s="20" t="n">
+        <v>45</v>
+      </c>
+      <c r="T289" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U289" s="21">
+        <f>L289*S289</f>
+        <v/>
+      </c>
+      <c r="V289" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W289" s="15" t="inlineStr">
+        <is>
+          <t>F-338</t>
+        </is>
+      </c>
+      <c r="X289" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y289" s="19" t="n"/>
+      <c r="Z289" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA289" s="19" t="n"/>
+      <c r="AB289" s="19" t="n"/>
+      <c r="AC289" s="19" t="n"/>
+      <c r="AD289" s="19" t="n"/>
+      <c r="AE289" s="20" t="n"/>
+      <c r="AF289" s="21">
+        <f>IF(K289="","",K289*AE289)</f>
+        <v/>
+      </c>
+      <c r="AG289" s="19" t="n"/>
+      <c r="AH289" s="19" t="n"/>
+      <c r="AI289" s="19" t="n"/>
+      <c r="AJ289" s="19" t="n"/>
+      <c r="AK289" s="19" t="n"/>
+      <c r="AL289" s="19" t="n"/>
+      <c r="AM289" s="16" t="inlineStr">
+        <is>
+          <t>2 Leuchten in unterschiedlicher Größe, beide abgebildet.</t>
+        </is>
+      </c>
+      <c r="AN289" s="22" t="n"/>
+    </row>
+    <row r="290" ht="30" customHeight="1">
+      <c r="A290" s="15" t="inlineStr">
+        <is>
+          <t>BA07-03</t>
+        </is>
+      </c>
+      <c r="B290" s="15" t="n"/>
+      <c r="C290" s="15" t="n"/>
+      <c r="D290" s="15" t="inlineStr">
+        <is>
+          <t>BA07</t>
+        </is>
+      </c>
+      <c r="E290" s="15" t="inlineStr">
+        <is>
+          <t>Standregal grau mit Wolkenaufsatz</t>
+        </is>
+      </c>
+      <c r="F290" s="16" t="inlineStr">
+        <is>
+          <t>Schmales Standregal in Grau mit drei Ablagen und vorderen Haltelleisten, oben ein ausgesägter Wolkenaufsatz, auf schrägen Holzbeinen. Als Bücherregal genutzt.</t>
+        </is>
+      </c>
+      <c r="G290" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H290" s="15" t="inlineStr">
+        <is>
+          <t>Klassenzimmer</t>
+        </is>
+      </c>
+      <c r="I290" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J290" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K290" s="17" t="n"/>
+      <c r="L290" s="18">
+        <f>J290-IF(K290="",0,K290)</f>
+        <v/>
+      </c>
+      <c r="M290" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N290" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O290" s="19" t="n"/>
+      <c r="P290" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q290" s="19" t="n"/>
+      <c r="R290" s="20" t="n"/>
+      <c r="S290" s="20" t="n">
+        <v>45</v>
+      </c>
+      <c r="T290" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U290" s="21">
+        <f>L290*S290</f>
+        <v/>
+      </c>
+      <c r="V290" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W290" s="15" t="inlineStr">
+        <is>
+          <t>F-339</t>
+        </is>
+      </c>
+      <c r="X290" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y290" s="19" t="n"/>
+      <c r="Z290" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA290" s="19" t="n"/>
+      <c r="AB290" s="19" t="n"/>
+      <c r="AC290" s="19" t="n"/>
+      <c r="AD290" s="19" t="n"/>
+      <c r="AE290" s="20" t="n"/>
+      <c r="AF290" s="21">
+        <f>IF(K290="","",K290*AE290)</f>
+        <v/>
+      </c>
+      <c r="AG290" s="19" t="n"/>
+      <c r="AH290" s="19" t="n"/>
+      <c r="AI290" s="19" t="n"/>
+      <c r="AJ290" s="19" t="n"/>
+      <c r="AK290" s="19" t="n"/>
+      <c r="AL290" s="19" t="n"/>
+      <c r="AM290" s="16" t="inlineStr">
+        <is>
+          <t>1 Regal.</t>
+        </is>
+      </c>
+      <c r="AN290" s="22" t="n"/>
+    </row>
+    <row r="291" ht="30" customHeight="1">
+      <c r="A291" s="15" t="inlineStr">
+        <is>
+          <t>BA07-05</t>
+        </is>
+      </c>
+      <c r="B291" s="15" t="n"/>
+      <c r="C291" s="15" t="n"/>
+      <c r="D291" s="15" t="inlineStr">
+        <is>
+          <t>BA07</t>
+        </is>
+      </c>
+      <c r="E291" s="15" t="inlineStr">
+        <is>
+          <t>Tisch weiß, lang, auf schwarzen Beinen</t>
+        </is>
+      </c>
+      <c r="F291" s="16" t="inlineStr">
+        <is>
+          <t>Langer Tisch mit weißer Platte auf vier schwarzen Rundbeinen mit Gleitern. Als Arbeits- und Ablagefläche genutzt.</t>
+        </is>
+      </c>
+      <c r="G291" s="15" t="inlineStr">
+        <is>
+          <t>Möbel</t>
+        </is>
+      </c>
+      <c r="H291" s="15" t="inlineStr">
+        <is>
+          <t>Klassenzimmer</t>
+        </is>
+      </c>
+      <c r="I291" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J291" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K291" s="17" t="n"/>
+      <c r="L291" s="18">
+        <f>J291-IF(K291="",0,K291)</f>
+        <v/>
+      </c>
+      <c r="M291" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N291" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O291" s="19" t="n"/>
+      <c r="P291" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q291" s="19" t="n"/>
+      <c r="R291" s="20" t="n"/>
+      <c r="S291" s="20" t="n">
+        <v>70</v>
+      </c>
+      <c r="T291" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U291" s="21">
+        <f>L291*S291</f>
+        <v/>
+      </c>
+      <c r="V291" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W291" s="15" t="inlineStr">
+        <is>
+          <t>F-341</t>
+        </is>
+      </c>
+      <c r="X291" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y291" s="19" t="n"/>
+      <c r="Z291" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA291" s="19" t="n"/>
+      <c r="AB291" s="19" t="n"/>
+      <c r="AC291" s="19" t="n"/>
+      <c r="AD291" s="19" t="n"/>
+      <c r="AE291" s="20" t="n"/>
+      <c r="AF291" s="21">
+        <f>IF(K291="","",K291*AE291)</f>
+        <v/>
+      </c>
+      <c r="AG291" s="19" t="n"/>
+      <c r="AH291" s="19" t="n"/>
+      <c r="AI291" s="19" t="n"/>
+      <c r="AJ291" s="19" t="n"/>
+      <c r="AK291" s="19" t="n"/>
+      <c r="AL291" s="19" t="n"/>
+      <c r="AM291" s="16" t="inlineStr">
+        <is>
+          <t>1 Tisch.</t>
+        </is>
+      </c>
+      <c r="AN291" s="22" t="inlineStr">
+        <is>
+          <t>Stueckzahl auf dem Erfassungsblatt nicht eingetragen, als 1 angenommen - bitte bestaetigen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="292" ht="30" customHeight="1">
+      <c r="A292" s="15" t="inlineStr">
+        <is>
+          <t>BA07-06</t>
+        </is>
+      </c>
+      <c r="B292" s="15" t="n"/>
+      <c r="C292" s="15" t="n"/>
+      <c r="D292" s="15" t="inlineStr">
+        <is>
+          <t>BA07</t>
+        </is>
+      </c>
+      <c r="E292" s="15" t="inlineStr">
+        <is>
+          <t>Regal creme, 16 Fächer, auf Metallbeinen</t>
+        </is>
+      </c>
+      <c r="F292" s="16" t="inlineStr">
+        <is>
+          <t>Großes Regal in Creme mit sechzehn Fächern in vier Reihen, auf schräg gestellten schwarzen Metallbeinen.</t>
+        </is>
+      </c>
+      <c r="G292" s="15" t="inlineStr">
+        <is>
+          <t>Möbel</t>
+        </is>
+      </c>
+      <c r="H292" s="15" t="inlineStr">
+        <is>
+          <t>Klassenzimmer</t>
+        </is>
+      </c>
+      <c r="I292" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J292" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K292" s="17" t="n"/>
+      <c r="L292" s="18">
+        <f>J292-IF(K292="",0,K292)</f>
+        <v/>
+      </c>
+      <c r="M292" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N292" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O292" s="19" t="n"/>
+      <c r="P292" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q292" s="19" t="n"/>
+      <c r="R292" s="20" t="n"/>
+      <c r="S292" s="20" t="n">
+        <v>90</v>
+      </c>
+      <c r="T292" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U292" s="21">
+        <f>L292*S292</f>
+        <v/>
+      </c>
+      <c r="V292" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W292" s="15" t="inlineStr">
+        <is>
+          <t>F-342</t>
+        </is>
+      </c>
+      <c r="X292" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y292" s="19" t="n"/>
+      <c r="Z292" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA292" s="19" t="n"/>
+      <c r="AB292" s="19" t="n"/>
+      <c r="AC292" s="19" t="n"/>
+      <c r="AD292" s="19" t="n"/>
+      <c r="AE292" s="20" t="n"/>
+      <c r="AF292" s="21">
+        <f>IF(K292="","",K292*AE292)</f>
+        <v/>
+      </c>
+      <c r="AG292" s="19" t="n"/>
+      <c r="AH292" s="19" t="n"/>
+      <c r="AI292" s="19" t="n"/>
+      <c r="AJ292" s="19" t="n"/>
+      <c r="AK292" s="19" t="n"/>
+      <c r="AL292" s="19" t="n"/>
+      <c r="AM292" s="16" t="inlineStr">
+        <is>
+          <t>1 Regal. Der Inhalt gehört nicht dazu.</t>
+        </is>
+      </c>
+      <c r="AN292" s="22" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:AN287"/>
+  <autoFilter ref="A2:AN292"/>
   <mergeCells count="7">
     <mergeCell ref="AI1:AL1"/>
     <mergeCell ref="V1:AD1"/>
@@ -36072,7 +36679,7 @@
     <mergeCell ref="AE1:AH1"/>
     <mergeCell ref="AM1:AN1"/>
   </mergeCells>
-  <conditionalFormatting sqref="Z3:Z287">
+  <conditionalFormatting sqref="Z3:Z292">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"reserviert"</formula>
     </cfRule>
@@ -36083,12 +36690,12 @@
       <formula>"verkauft"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I3:I287">
+  <conditionalFormatting sqref="I3:I292">
     <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
       <formula>"A"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P3:P287">
+  <conditionalFormatting sqref="P3:P292">
     <cfRule type="cellIs" priority="5" operator="equal" dxfId="4">
       <formula>"entfällt"</formula>
     </cfRule>
@@ -36141,7 +36748,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D92"/>
+  <dimension ref="A1:D93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -36179,7 +36786,7 @@
         </is>
       </c>
       <c r="B5" s="27">
-        <f>COUNTA(Artikelstamm!$A$3:$A$287)</f>
+        <f>COUNTA(Artikelstamm!$A$3:$A$292)</f>
         <v/>
       </c>
     </row>
@@ -36190,7 +36797,7 @@
         </is>
       </c>
       <c r="B6" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$287,"verfügbar")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$292,"verfügbar")</f>
         <v/>
       </c>
     </row>
@@ -36201,7 +36808,7 @@
         </is>
       </c>
       <c r="B7" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$287,"reserviert")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$292,"reserviert")</f>
         <v/>
       </c>
     </row>
@@ -36212,7 +36819,7 @@
         </is>
       </c>
       <c r="B8" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$287,"teilverkauft")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$292,"teilverkauft")</f>
         <v/>
       </c>
     </row>
@@ -36223,7 +36830,7 @@
         </is>
       </c>
       <c r="B9" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$287,"verkauft")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$292,"verkauft")</f>
         <v/>
       </c>
     </row>
@@ -36234,7 +36841,7 @@
         </is>
       </c>
       <c r="B10" s="27">
-        <f>SUM(Artikelstamm!$L$3:$L$287)</f>
+        <f>SUM(Artikelstamm!$L$3:$L$292)</f>
         <v/>
       </c>
     </row>
@@ -36245,7 +36852,7 @@
         </is>
       </c>
       <c r="B11" s="29">
-        <f>SUM(Artikelstamm!$U$3:$U$287)</f>
+        <f>SUM(Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
@@ -36263,7 +36870,7 @@
         </is>
       </c>
       <c r="B13" s="27">
-        <f>SUM(Artikelstamm!$K$3:$K$287)</f>
+        <f>SUM(Artikelstamm!$K$3:$K$292)</f>
         <v/>
       </c>
     </row>
@@ -36274,7 +36881,7 @@
         </is>
       </c>
       <c r="B14" s="30">
-        <f>SUMPRODUCT(Artikelstamm!$K$3:$K$287,Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT(Artikelstamm!$K$3:$K$292,Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
     </row>
@@ -36307,7 +36914,7 @@
         </is>
       </c>
       <c r="B17" s="30">
-        <f>SUMPRODUCT((Artikelstamm!$AJ$3:$AJ$287="bezahlt")*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AJ$3:$AJ$292="bezahlt")*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
     </row>
@@ -36336,7 +36943,7 @@
         </is>
       </c>
       <c r="B21" s="31">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$287,"*verkauft",Artikelstamm!$AI$3:$AI$287,"")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$292,"*verkauft",Artikelstamm!$AI$3:$AI$292,"")</f>
         <v/>
       </c>
     </row>
@@ -36347,7 +36954,7 @@
         </is>
       </c>
       <c r="B22" s="31">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$287,"*verkauft",Artikelstamm!$AJ$3:$AJ$287,"offen")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$292,"*verkauft",Artikelstamm!$AJ$3:$AJ$292,"offen")</f>
         <v/>
       </c>
     </row>
@@ -36358,7 +36965,7 @@
         </is>
       </c>
       <c r="B23" s="27">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$287,"reserviert",Artikelstamm!$AL$3:$AL$287,"")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$292,"reserviert",Artikelstamm!$AL$3:$AL$292,"")</f>
         <v/>
       </c>
     </row>
@@ -36369,7 +36976,7 @@
         </is>
       </c>
       <c r="B24" s="27">
-        <f>COUNTIFS(Artikelstamm!$S$3:$S$287,"")</f>
+        <f>COUNTIFS(Artikelstamm!$S$3:$S$292,"")</f>
         <v/>
       </c>
     </row>
@@ -36380,7 +36987,7 @@
         </is>
       </c>
       <c r="B25" s="27">
-        <f>COUNTIFS(Artikelstamm!$O$3:$O$287,"")</f>
+        <f>COUNTIFS(Artikelstamm!$O$3:$O$292,"")</f>
         <v/>
       </c>
     </row>
@@ -36420,15 +37027,15 @@
         </is>
       </c>
       <c r="B30" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$287,$A30)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$292,$A30)</f>
         <v/>
       </c>
       <c r="C30" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$287=$A30)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$292=$A30)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D30" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$287,$A30,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$292,$A30,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
@@ -36439,15 +37046,15 @@
         </is>
       </c>
       <c r="B31" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$287,$A31)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$292,$A31)</f>
         <v/>
       </c>
       <c r="C31" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$287=$A31)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$292=$A31)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D31" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$287,$A31,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$292,$A31,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
@@ -36458,15 +37065,15 @@
         </is>
       </c>
       <c r="B32" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$287,$A32)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$292,$A32)</f>
         <v/>
       </c>
       <c r="C32" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$287=$A32)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$292=$A32)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D32" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$287,$A32,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$292,$A32,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
@@ -36525,15 +37132,15 @@
         </is>
       </c>
       <c r="B37" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$287,$A37)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$292,$A37)</f>
         <v/>
       </c>
       <c r="C37" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$287=$A37)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$292=$A37)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D37" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$287,$A37,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$292,$A37,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
@@ -36544,15 +37151,15 @@
         </is>
       </c>
       <c r="B38" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$287,$A38)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$292,$A38)</f>
         <v/>
       </c>
       <c r="C38" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$287=$A38)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$292=$A38)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D38" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$287,$A38,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$292,$A38,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
@@ -36563,15 +37170,15 @@
         </is>
       </c>
       <c r="B39" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$287,$A39)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$292,$A39)</f>
         <v/>
       </c>
       <c r="C39" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$287=$A39)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$292=$A39)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D39" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$287,$A39,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$292,$A39,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
@@ -36582,15 +37189,15 @@
         </is>
       </c>
       <c r="B40" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$287,$A40)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$292,$A40)</f>
         <v/>
       </c>
       <c r="C40" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$287=$A40)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$292=$A40)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D40" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$287,$A40,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$292,$A40,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
@@ -36601,15 +37208,15 @@
         </is>
       </c>
       <c r="B41" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$287,$A41)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$292,$A41)</f>
         <v/>
       </c>
       <c r="C41" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$287=$A41)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$292=$A41)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D41" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$287,$A41,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$292,$A41,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
@@ -36620,15 +37227,15 @@
         </is>
       </c>
       <c r="B42" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$287,$A42)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$292,$A42)</f>
         <v/>
       </c>
       <c r="C42" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$287=$A42)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$292=$A42)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D42" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$287,$A42,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$292,$A42,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
@@ -36639,15 +37246,15 @@
         </is>
       </c>
       <c r="B43" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$287,$A43)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$292,$A43)</f>
         <v/>
       </c>
       <c r="C43" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$287=$A43)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$292=$A43)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D43" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$287,$A43,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$292,$A43,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
@@ -36658,15 +37265,15 @@
         </is>
       </c>
       <c r="B44" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$287,$A44)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$292,$A44)</f>
         <v/>
       </c>
       <c r="C44" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$287=$A44)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$292=$A44)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D44" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$287,$A44,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$292,$A44,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
@@ -36677,15 +37284,15 @@
         </is>
       </c>
       <c r="B45" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$287,$A45)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$292,$A45)</f>
         <v/>
       </c>
       <c r="C45" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$287=$A45)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$292=$A45)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D45" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$287,$A45,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$292,$A45,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
@@ -36696,15 +37303,15 @@
         </is>
       </c>
       <c r="B46" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$287,$A46)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$292,$A46)</f>
         <v/>
       </c>
       <c r="C46" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$287=$A46)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$292=$A46)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D46" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$287,$A46,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$292,$A46,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
@@ -36715,15 +37322,15 @@
         </is>
       </c>
       <c r="B47" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$287,$A47)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$292,$A47)</f>
         <v/>
       </c>
       <c r="C47" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$287=$A47)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$292=$A47)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D47" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$287,$A47,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$292,$A47,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
@@ -36734,15 +37341,15 @@
         </is>
       </c>
       <c r="B48" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$287,$A48)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$292,$A48)</f>
         <v/>
       </c>
       <c r="C48" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$287=$A48)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$292=$A48)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D48" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$287,$A48,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$292,$A48,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
@@ -36753,15 +37360,15 @@
         </is>
       </c>
       <c r="B49" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$287,$A49)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$292,$A49)</f>
         <v/>
       </c>
       <c r="C49" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$287=$A49)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$292=$A49)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D49" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$287,$A49,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$292,$A49,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
@@ -36772,15 +37379,15 @@
         </is>
       </c>
       <c r="B50" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$287,$A50)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$292,$A50)</f>
         <v/>
       </c>
       <c r="C50" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$287=$A50)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$292=$A50)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D50" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$287,$A50,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$292,$A50,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
@@ -36839,15 +37446,15 @@
         </is>
       </c>
       <c r="B55" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$287,$A55)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A55)</f>
         <v/>
       </c>
       <c r="C55" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$287=$A55)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A55)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D55" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$287,$A55,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A55,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
@@ -36858,15 +37465,15 @@
         </is>
       </c>
       <c r="B56" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$287,$A56)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A56)</f>
         <v/>
       </c>
       <c r="C56" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$287=$A56)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A56)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D56" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$287,$A56,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A56,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
@@ -36877,15 +37484,15 @@
         </is>
       </c>
       <c r="B57" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$287,$A57)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A57)</f>
         <v/>
       </c>
       <c r="C57" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$287=$A57)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A57)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D57" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$287,$A57,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A57,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
@@ -36896,15 +37503,15 @@
         </is>
       </c>
       <c r="B58" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$287,$A58)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A58)</f>
         <v/>
       </c>
       <c r="C58" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$287=$A58)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A58)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D58" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$287,$A58,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A58,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
@@ -36915,15 +37522,15 @@
         </is>
       </c>
       <c r="B59" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$287,$A59)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A59)</f>
         <v/>
       </c>
       <c r="C59" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$287=$A59)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A59)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D59" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$287,$A59,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A59,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
@@ -36934,15 +37541,15 @@
         </is>
       </c>
       <c r="B60" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$287,$A60)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A60)</f>
         <v/>
       </c>
       <c r="C60" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$287=$A60)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A60)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D60" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$287,$A60,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A60,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
@@ -36953,15 +37560,15 @@
         </is>
       </c>
       <c r="B61" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$287,$A61)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A61)</f>
         <v/>
       </c>
       <c r="C61" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$287=$A61)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A61)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D61" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$287,$A61,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A61,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
@@ -36972,15 +37579,15 @@
         </is>
       </c>
       <c r="B62" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$287,$A62)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A62)</f>
         <v/>
       </c>
       <c r="C62" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$287=$A62)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A62)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D62" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$287,$A62,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A62,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
@@ -36991,15 +37598,15 @@
         </is>
       </c>
       <c r="B63" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$287,$A63)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A63)</f>
         <v/>
       </c>
       <c r="C63" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$287=$A63)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A63)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D63" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$287,$A63,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A63,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
@@ -37010,15 +37617,15 @@
         </is>
       </c>
       <c r="B64" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$287,$A64)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A64)</f>
         <v/>
       </c>
       <c r="C64" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$287=$A64)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A64)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D64" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$287,$A64,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A64,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
@@ -37029,15 +37636,15 @@
         </is>
       </c>
       <c r="B65" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$287,$A65)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A65)</f>
         <v/>
       </c>
       <c r="C65" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$287=$A65)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A65)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D65" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$287,$A65,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A65,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
@@ -37048,15 +37655,15 @@
         </is>
       </c>
       <c r="B66" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$287,$A66)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A66)</f>
         <v/>
       </c>
       <c r="C66" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$287=$A66)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A66)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D66" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$287,$A66,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A66,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
@@ -37067,15 +37674,15 @@
         </is>
       </c>
       <c r="B67" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$287,$A67)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A67)</f>
         <v/>
       </c>
       <c r="C67" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$287=$A67)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A67)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D67" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$287,$A67,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A67,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
@@ -37086,410 +37693,429 @@
         </is>
       </c>
       <c r="B68" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$287,$A68)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A68)</f>
         <v/>
       </c>
       <c r="C68" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$287=$A68)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A68)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D68" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$287,$A68,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A68,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="26" t="inlineStr">
         <is>
-          <t>Küche</t>
+          <t>Klassenzimmer</t>
         </is>
       </c>
       <c r="B69" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$287,$A69)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A69)</f>
         <v/>
       </c>
       <c r="C69" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$287=$A69)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A69)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D69" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$287,$A69,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A69,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="26" t="inlineStr">
         <is>
-          <t>Material / Turnraum</t>
+          <t>Küche</t>
         </is>
       </c>
       <c r="B70" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$287,$A70)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A70)</f>
         <v/>
       </c>
       <c r="C70" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$287=$A70)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A70)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D70" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$287,$A70,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A70,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="26" t="inlineStr">
         <is>
-          <t>Personal</t>
+          <t>Material / Turnraum</t>
         </is>
       </c>
       <c r="B71" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$287,$A71)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A71)</f>
         <v/>
       </c>
       <c r="C71" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$287=$A71)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A71)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D71" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$287,$A71,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A71,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="26" t="inlineStr">
         <is>
-          <t>Ruhe- / Schlafraum</t>
+          <t>Personal</t>
         </is>
       </c>
       <c r="B72" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$287,$A72)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A72)</f>
         <v/>
       </c>
       <c r="C72" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$287=$A72)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A72)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D72" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$287,$A72,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A72,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="26" t="inlineStr">
         <is>
-          <t>Schlafraum 4</t>
+          <t>Ruhe- / Schlafraum</t>
         </is>
       </c>
       <c r="B73" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$287,$A73)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A73)</f>
         <v/>
       </c>
       <c r="C73" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$287=$A73)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A73)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D73" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$287,$A73,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A73,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="26" t="inlineStr">
         <is>
-          <t>Schlafraum 5</t>
+          <t>Schlafraum 4</t>
         </is>
       </c>
       <c r="B74" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$287,$A74)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A74)</f>
         <v/>
       </c>
       <c r="C74" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$287=$A74)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A74)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D74" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$287,$A74,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A74,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="26" t="inlineStr">
         <is>
-          <t>Speisesaal</t>
+          <t>Schlafraum 5</t>
         </is>
       </c>
       <c r="B75" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$287,$A75)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A75)</f>
         <v/>
       </c>
       <c r="C75" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$287=$A75)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A75)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D75" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$287,$A75,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A75,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="26" t="inlineStr">
         <is>
-          <t>Terrasse</t>
+          <t>Speisesaal</t>
         </is>
       </c>
       <c r="B76" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$287,$A76)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A76)</f>
         <v/>
       </c>
       <c r="C76" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$287=$A76)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A76)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D76" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$287,$A76,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A76,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="26" t="inlineStr">
         <is>
-          <t>Treppenraum 1</t>
+          <t>Terrasse</t>
         </is>
       </c>
       <c r="B77" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$287,$A77)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A77)</f>
         <v/>
       </c>
       <c r="C77" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$287=$A77)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A77)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D77" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$287,$A77,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A77,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="26" t="inlineStr">
         <is>
-          <t>Turnraum</t>
+          <t>Treppenraum 1</t>
         </is>
       </c>
       <c r="B78" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$287,$A78)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A78)</f>
         <v/>
       </c>
       <c r="C78" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$287=$A78)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A78)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D78" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$287,$A78,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A78,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="26" t="inlineStr">
         <is>
-          <t>WC</t>
+          <t>Turnraum</t>
         </is>
       </c>
       <c r="B79" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$287,$A79)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A79)</f>
         <v/>
       </c>
       <c r="C79" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$287=$A79)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A79)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D79" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$287,$A79,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A79,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="26" t="inlineStr">
         <is>
-          <t>WC Personal</t>
+          <t>WC</t>
         </is>
       </c>
       <c r="B80" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$287,$A80)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A80)</f>
         <v/>
       </c>
       <c r="C80" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$287=$A80)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A80)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
       <c r="D80" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$287,$A80,Artikelstamm!$U$3:$U$287)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A80,Artikelstamm!$U$3:$U$292)</f>
         <v/>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="26" t="inlineStr">
         <is>
+          <t>WC Personal</t>
+        </is>
+      </c>
+      <c r="B81" s="33">
+        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A81)</f>
+        <v/>
+      </c>
+      <c r="C81" s="34">
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A81)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <v/>
+      </c>
+      <c r="D81" s="34">
+        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A81,Artikelstamm!$U$3:$U$292)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="26" t="inlineStr">
+        <is>
           <t>Werkraum</t>
         </is>
       </c>
-      <c r="B81" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$287,$A81)</f>
-        <v/>
-      </c>
-      <c r="C81" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$287=$A81)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
-        <v/>
-      </c>
-      <c r="D81" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$287,$A81,Artikelstamm!$U$3:$U$287)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="28" t="inlineStr">
+      <c r="B82" s="33">
+        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A82)</f>
+        <v/>
+      </c>
+      <c r="C82" s="34">
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A82)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <v/>
+      </c>
+      <c r="D82" s="34">
+        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A82,Artikelstamm!$U$3:$U$292)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="28" t="inlineStr">
         <is>
           <t>Summe</t>
         </is>
       </c>
-      <c r="B82" s="35">
-        <f>SUM(B55:B81)</f>
-        <v/>
-      </c>
-      <c r="C82" s="36">
-        <f>SUM(C55:C81)</f>
-        <v/>
-      </c>
-      <c r="D82" s="36">
-        <f>SUM(D55:D81)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" s="25" t="inlineStr">
+      <c r="B83" s="35">
+        <f>SUM(B55:B82)</f>
+        <v/>
+      </c>
+      <c r="C83" s="36">
+        <f>SUM(C55:C82)</f>
+        <v/>
+      </c>
+      <c r="D83" s="36">
+        <f>SUM(D55:D82)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="25" t="inlineStr">
         <is>
           <t>Nach Verkaufskanal</t>
         </is>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" s="32" t="inlineStr">
+    <row r="86">
+      <c r="A86" s="32" t="inlineStr">
         <is>
           <t>Verkaufskanal</t>
         </is>
       </c>
-      <c r="B85" s="32" t="inlineStr">
+      <c r="B86" s="32" t="inlineStr">
         <is>
           <t>Positionen</t>
         </is>
       </c>
-      <c r="C85" s="32" t="inlineStr">
+      <c r="C86" s="32" t="inlineStr">
         <is>
           <t>Umsatz netto</t>
         </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" s="26" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
-      <c r="B86" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$287,$A86)</f>
-        <v/>
-      </c>
-      <c r="C86" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$287=$A86)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
-        <v/>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="26" t="inlineStr">
         <is>
-          <t>Kleinanzeigen</t>
+          <t>Klinik</t>
         </is>
       </c>
       <c r="B87" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$287,$A87)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$292,$A87)</f>
         <v/>
       </c>
       <c r="C87" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$287=$A87)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$292=$A87)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="26" t="inlineStr">
         <is>
-          <t>eBay</t>
+          <t>Kleinanzeigen</t>
         </is>
       </c>
       <c r="B88" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$287,$A88)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$292,$A88)</f>
         <v/>
       </c>
       <c r="C88" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$287=$A88)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$292=$A88)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="26" t="inlineStr">
         <is>
-          <t>Direkt</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="B89" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$287,$A89)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$292,$A89)</f>
         <v/>
       </c>
       <c r="C89" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$287=$A89)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$292=$A89)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="26" t="inlineStr">
         <is>
-          <t>Händler</t>
+          <t>Direkt</t>
         </is>
       </c>
       <c r="B90" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$287,$A90)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$292,$A90)</f>
         <v/>
       </c>
       <c r="C90" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$287=$A90)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$292=$A90)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
         <v/>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="26" t="inlineStr">
         <is>
+          <t>Händler</t>
+        </is>
+      </c>
+      <c r="B91" s="33">
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$292,$A91)</f>
+        <v/>
+      </c>
+      <c r="C91" s="34">
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$292=$A91)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="26" t="inlineStr">
+        <is>
           <t>Verkaufstag</t>
         </is>
       </c>
-      <c r="B91" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$287,$A91)</f>
-        <v/>
-      </c>
-      <c r="C91" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$287=$A91)*Artikelstamm!$K$3:$K$287*Artikelstamm!$AE$3:$AE$287)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="28" t="inlineStr">
+      <c r="B92" s="33">
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$292,$A92)</f>
+        <v/>
+      </c>
+      <c r="C92" s="34">
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$292=$A92)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="28" t="inlineStr">
         <is>
           <t>Summe</t>
         </is>
       </c>
-      <c r="B92" s="35">
-        <f>SUM(B86:B91)</f>
-        <v/>
-      </c>
-      <c r="C92" s="36">
-        <f>SUM(C86:C91)</f>
+      <c r="B93" s="35">
+        <f>SUM(B87:B92)</f>
+        <v/>
+      </c>
+      <c r="C93" s="36">
+        <f>SUM(C87:C92)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
BA08 Atelier erfasst: 8 Positionen, neun weitere VS-Stuehle
Atelier (Bestandsgebaeude Attika, 22,72 m2). Der Raum hatte schon vier
Konvolut-Positionen aus der alten Erfassung.

BA08-06 sind neun Schalenstuehle von VS auf Vierfussgestell - ein anderes
Modell als die acht auf Kufengestell unter NU02-04. Das Logo ist auf
F-346 gestochen scharf. Beide Positionen verweisen aufeinander. Wegen der
Farbspritzer aus dem Atelierbetrieb mit 50 EUR angesetzt statt 65 EUR wie
bei den sauberen. Damit stehen 17 VS-Stuehle im Bestand, zusammen
970 EUR - das ist der groesste Stuhlblock.

Weitere Marken ueber Aufdruck belegt: Marpa Jansen (Feinkrepp),
Betzold (Scherenblock).

Gesamtwert netto 42.156 -> 42.970 EUR, 243 aktive Positionen.
pruefen.py: 0 Fehler, 3 Hinweise.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011yyfqhuiWGsaNy38oaNoGo
</commit_message>
<xml_diff>
--- a/ausgabe/01_Artikelstamm_kikripp.xlsx
+++ b/ausgabe/01_Artikelstamm_kikripp.xlsx
@@ -15,7 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Artikelstamm'!$A$2:$AN$292</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Artikelstamm'!$A$2:$AN$300</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1019,7 +1019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN292"/>
+  <dimension ref="A1:AN300"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -36668,8 +36668,972 @@
       </c>
       <c r="AN292" s="22" t="n"/>
     </row>
+    <row r="293" ht="30" customHeight="1">
+      <c r="A293" s="15" t="inlineStr">
+        <is>
+          <t>BA08-05</t>
+        </is>
+      </c>
+      <c r="B293" s="15" t="n"/>
+      <c r="C293" s="15" t="n"/>
+      <c r="D293" s="15" t="inlineStr">
+        <is>
+          <t>BA08</t>
+        </is>
+      </c>
+      <c r="E293" s="15" t="inlineStr">
+        <is>
+          <t>Acrylbild schwarz-weiß, Kreise mit Punkten</t>
+        </is>
+      </c>
+      <c r="F293" s="16" t="inlineStr">
+        <is>
+          <t>Acryl auf Leinwand, großes Quadrat: mit breitem Pinsel gezogene Kreise, darin je mehrere gemalte Punkte – die Anmutung von Würfeln. Eigenarbeit einer Privatperson, nicht signiert.</t>
+        </is>
+      </c>
+      <c r="G293" s="15" t="inlineStr">
+        <is>
+          <t>Kunst</t>
+        </is>
+      </c>
+      <c r="H293" s="15" t="inlineStr">
+        <is>
+          <t>Atelier</t>
+        </is>
+      </c>
+      <c r="I293" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J293" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K293" s="17" t="n"/>
+      <c r="L293" s="18">
+        <f>J293-IF(K293="",0,K293)</f>
+        <v/>
+      </c>
+      <c r="M293" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N293" s="15" t="inlineStr">
+        <is>
+          <t>gut</t>
+        </is>
+      </c>
+      <c r="O293" s="19" t="n"/>
+      <c r="P293" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q293" s="19" t="n"/>
+      <c r="R293" s="20" t="n"/>
+      <c r="S293" s="20" t="n">
+        <v>150</v>
+      </c>
+      <c r="T293" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U293" s="21">
+        <f>L293*S293</f>
+        <v/>
+      </c>
+      <c r="V293" s="15" t="inlineStr">
+        <is>
+          <t>Versand möglich</t>
+        </is>
+      </c>
+      <c r="W293" s="15" t="inlineStr">
+        <is>
+          <t>F-344</t>
+        </is>
+      </c>
+      <c r="X293" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y293" s="19" t="n"/>
+      <c r="Z293" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA293" s="19" t="n"/>
+      <c r="AB293" s="19" t="n"/>
+      <c r="AC293" s="19" t="n"/>
+      <c r="AD293" s="19" t="n"/>
+      <c r="AE293" s="20" t="n"/>
+      <c r="AF293" s="21">
+        <f>IF(K293="","",K293*AE293)</f>
+        <v/>
+      </c>
+      <c r="AG293" s="19" t="n"/>
+      <c r="AH293" s="19" t="n"/>
+      <c r="AI293" s="19" t="n"/>
+      <c r="AJ293" s="19" t="n"/>
+      <c r="AK293" s="19" t="n"/>
+      <c r="AL293" s="19" t="n"/>
+      <c r="AM293" s="16" t="inlineStr">
+        <is>
+          <t>1 Bild.</t>
+        </is>
+      </c>
+      <c r="AN293" s="22" t="n"/>
+    </row>
+    <row r="294" ht="30" customHeight="1">
+      <c r="A294" s="15" t="inlineStr">
+        <is>
+          <t>BA08-06</t>
+        </is>
+      </c>
+      <c r="B294" s="15" t="n"/>
+      <c r="C294" s="15" t="n"/>
+      <c r="D294" s="15" t="inlineStr">
+        <is>
+          <t>BA08</t>
+        </is>
+      </c>
+      <c r="E294" s="15" t="inlineStr">
+        <is>
+          <t>VS Schalenstuhl grau, Vierfußgestell</t>
+        </is>
+      </c>
+      <c r="F294" s="16" t="inlineStr">
+        <is>
+          <t>Schalenstuhl von VS (Vereinigte Spezialmöbelfabriken): graue Kunststoffschale mit Rautenstruktur und Griffloch in der Lehne, auf grauem Vierfußgestell aus Rohr. Farbspritzer aus dem Atelierbetrieb auf Sitz und Lehne.</t>
+        </is>
+      </c>
+      <c r="G294" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H294" s="15" t="inlineStr">
+        <is>
+          <t>Atelier</t>
+        </is>
+      </c>
+      <c r="I294" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J294" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="K294" s="17" t="n"/>
+      <c r="L294" s="18">
+        <f>J294-IF(K294="",0,K294)</f>
+        <v/>
+      </c>
+      <c r="M294" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N294" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O294" s="19" t="n"/>
+      <c r="P294" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q294" s="19" t="n"/>
+      <c r="R294" s="20" t="n"/>
+      <c r="S294" s="20" t="n">
+        <v>50</v>
+      </c>
+      <c r="T294" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U294" s="21">
+        <f>L294*S294</f>
+        <v/>
+      </c>
+      <c r="V294" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W294" s="15" t="inlineStr">
+        <is>
+          <t>F-345</t>
+        </is>
+      </c>
+      <c r="X294" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y294" s="19" t="n"/>
+      <c r="Z294" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA294" s="19" t="inlineStr">
+        <is>
+          <t>VS</t>
+        </is>
+      </c>
+      <c r="AB294" s="19" t="n"/>
+      <c r="AC294" s="19" t="n"/>
+      <c r="AD294" s="19" t="n"/>
+      <c r="AE294" s="20" t="n"/>
+      <c r="AF294" s="21">
+        <f>IF(K294="","",K294*AE294)</f>
+        <v/>
+      </c>
+      <c r="AG294" s="19" t="n"/>
+      <c r="AH294" s="19" t="n"/>
+      <c r="AI294" s="19" t="n"/>
+      <c r="AJ294" s="19" t="n"/>
+      <c r="AK294" s="19" t="n"/>
+      <c r="AL294" s="19" t="n"/>
+      <c r="AM294" s="16" t="inlineStr">
+        <is>
+          <t>9 Stühle – abgebildet ist einer davon. Das Logo ist auf Foto F-346 zu sehen. Ein anderes VS-Modell auf Kufengestell steht unter NU02-04.</t>
+        </is>
+      </c>
+      <c r="AN294" s="22" t="n"/>
+    </row>
+    <row r="295" ht="30" customHeight="1">
+      <c r="A295" s="15" t="inlineStr">
+        <is>
+          <t>BA08-07</t>
+        </is>
+      </c>
+      <c r="B295" s="15" t="n"/>
+      <c r="C295" s="15" t="n"/>
+      <c r="D295" s="15" t="inlineStr">
+        <is>
+          <t>BA08</t>
+        </is>
+      </c>
+      <c r="E295" s="15" t="inlineStr">
+        <is>
+          <t>Konvolut Feinkrepp-Papier</t>
+        </is>
+      </c>
+      <c r="F295" s="16" t="inlineStr">
+        <is>
+          <t>Rollen Feinkrepp von Marpa Jansen, je 50 × 250 cm, in Blau, Grün, Gelb, Rot, Orange und Braun. Teils angebrochen, dazu ein Beutel mit zugeschnittenen Schnipseln.</t>
+        </is>
+      </c>
+      <c r="G295" s="15" t="inlineStr">
+        <is>
+          <t>Verbrauchsmaterial</t>
+        </is>
+      </c>
+      <c r="H295" s="15" t="inlineStr">
+        <is>
+          <t>Atelier</t>
+        </is>
+      </c>
+      <c r="I295" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J295" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K295" s="17" t="n"/>
+      <c r="L295" s="18">
+        <f>J295-IF(K295="",0,K295)</f>
+        <v/>
+      </c>
+      <c r="M295" s="15" t="inlineStr">
+        <is>
+          <t>Konvolut</t>
+        </is>
+      </c>
+      <c r="N295" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O295" s="19" t="n"/>
+      <c r="P295" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q295" s="19" t="n"/>
+      <c r="R295" s="20" t="n"/>
+      <c r="S295" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="T295" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U295" s="21">
+        <f>L295*S295</f>
+        <v/>
+      </c>
+      <c r="V295" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W295" s="15" t="inlineStr">
+        <is>
+          <t>F-347</t>
+        </is>
+      </c>
+      <c r="X295" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y295" s="19" t="n"/>
+      <c r="Z295" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA295" s="19" t="inlineStr">
+        <is>
+          <t>Marpa Jansen</t>
+        </is>
+      </c>
+      <c r="AB295" s="19" t="n"/>
+      <c r="AC295" s="19" t="n"/>
+      <c r="AD295" s="19" t="n"/>
+      <c r="AE295" s="20" t="n"/>
+      <c r="AF295" s="21">
+        <f>IF(K295="","",K295*AE295)</f>
+        <v/>
+      </c>
+      <c r="AG295" s="19" t="n"/>
+      <c r="AH295" s="19" t="n"/>
+      <c r="AI295" s="19" t="n"/>
+      <c r="AJ295" s="19" t="n"/>
+      <c r="AK295" s="19" t="n"/>
+      <c r="AL295" s="19" t="n"/>
+      <c r="AM295" s="16" t="inlineStr">
+        <is>
+          <t>1 Konvolut. Der Schubladeninhalt ist auf Foto F-348 zu sehen.</t>
+        </is>
+      </c>
+      <c r="AN295" s="22" t="n"/>
+    </row>
+    <row r="296" ht="30" customHeight="1">
+      <c r="A296" s="15" t="inlineStr">
+        <is>
+          <t>BA08-08</t>
+        </is>
+      </c>
+      <c r="B296" s="15" t="n"/>
+      <c r="C296" s="15" t="n"/>
+      <c r="D296" s="15" t="inlineStr">
+        <is>
+          <t>BA08</t>
+        </is>
+      </c>
+      <c r="E296" s="15" t="inlineStr">
+        <is>
+          <t>Deko-Pilze auf Holzfuß</t>
+        </is>
+      </c>
+      <c r="F296" s="16" t="inlineStr">
+        <is>
+          <t>Dekopilze mit gedrechseltem Fuß aus Massivholz: zwei mit gehämmerter Metallkappe in Silberoptik, einer mit Kappe in Betonoptik.</t>
+        </is>
+      </c>
+      <c r="G296" s="15" t="inlineStr">
+        <is>
+          <t>Deko</t>
+        </is>
+      </c>
+      <c r="H296" s="15" t="inlineStr">
+        <is>
+          <t>Atelier</t>
+        </is>
+      </c>
+      <c r="I296" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J296" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="K296" s="17" t="n"/>
+      <c r="L296" s="18">
+        <f>J296-IF(K296="",0,K296)</f>
+        <v/>
+      </c>
+      <c r="M296" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N296" s="15" t="inlineStr">
+        <is>
+          <t>gut</t>
+        </is>
+      </c>
+      <c r="O296" s="19" t="n"/>
+      <c r="P296" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q296" s="19" t="n"/>
+      <c r="R296" s="20" t="n"/>
+      <c r="S296" s="20" t="n">
+        <v>18</v>
+      </c>
+      <c r="T296" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U296" s="21">
+        <f>L296*S296</f>
+        <v/>
+      </c>
+      <c r="V296" s="15" t="inlineStr">
+        <is>
+          <t>Versand möglich</t>
+        </is>
+      </c>
+      <c r="W296" s="15" t="inlineStr">
+        <is>
+          <t>F-349</t>
+        </is>
+      </c>
+      <c r="X296" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y296" s="19" t="n"/>
+      <c r="Z296" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA296" s="19" t="n"/>
+      <c r="AB296" s="19" t="n"/>
+      <c r="AC296" s="19" t="n"/>
+      <c r="AD296" s="19" t="n"/>
+      <c r="AE296" s="20" t="n"/>
+      <c r="AF296" s="21">
+        <f>IF(K296="","",K296*AE296)</f>
+        <v/>
+      </c>
+      <c r="AG296" s="19" t="n"/>
+      <c r="AH296" s="19" t="n"/>
+      <c r="AI296" s="19" t="n"/>
+      <c r="AJ296" s="19" t="n"/>
+      <c r="AK296" s="19" t="n"/>
+      <c r="AL296" s="19" t="n"/>
+      <c r="AM296" s="16" t="inlineStr">
+        <is>
+          <t>3 Pilze, alle abgebildet.</t>
+        </is>
+      </c>
+      <c r="AN296" s="22" t="n"/>
+    </row>
+    <row r="297" ht="30" customHeight="1">
+      <c r="A297" s="15" t="inlineStr">
+        <is>
+          <t>BA08-09</t>
+        </is>
+      </c>
+      <c r="B297" s="15" t="n"/>
+      <c r="C297" s="15" t="n"/>
+      <c r="D297" s="15" t="inlineStr">
+        <is>
+          <t>BA08</t>
+        </is>
+      </c>
+      <c r="E297" s="15" t="inlineStr">
+        <is>
+          <t>Bastelscheren im Betzold-Holzblock</t>
+        </is>
+      </c>
+      <c r="F297" s="16" t="inlineStr">
+        <is>
+          <t>Kinder-Bastelscheren mit Kunststoffgriffen in gemischten Farben, dazu ein Holzblock mit Steckbohrungen von Betzold als Ablage.</t>
+        </is>
+      </c>
+      <c r="G297" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H297" s="15" t="inlineStr">
+        <is>
+          <t>Atelier</t>
+        </is>
+      </c>
+      <c r="I297" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J297" s="17" t="n">
+        <v>15</v>
+      </c>
+      <c r="K297" s="17" t="n"/>
+      <c r="L297" s="18">
+        <f>J297-IF(K297="",0,K297)</f>
+        <v/>
+      </c>
+      <c r="M297" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N297" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O297" s="19" t="n"/>
+      <c r="P297" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q297" s="19" t="n"/>
+      <c r="R297" s="20" t="n"/>
+      <c r="S297" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="T297" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U297" s="21">
+        <f>L297*S297</f>
+        <v/>
+      </c>
+      <c r="V297" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W297" s="15" t="inlineStr">
+        <is>
+          <t>F-350</t>
+        </is>
+      </c>
+      <c r="X297" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y297" s="19" t="n"/>
+      <c r="Z297" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA297" s="19" t="inlineStr">
+        <is>
+          <t>Betzold</t>
+        </is>
+      </c>
+      <c r="AB297" s="19" t="n"/>
+      <c r="AC297" s="19" t="n"/>
+      <c r="AD297" s="19" t="n"/>
+      <c r="AE297" s="20" t="n"/>
+      <c r="AF297" s="21">
+        <f>IF(K297="","",K297*AE297)</f>
+        <v/>
+      </c>
+      <c r="AG297" s="19" t="n"/>
+      <c r="AH297" s="19" t="n"/>
+      <c r="AI297" s="19" t="n"/>
+      <c r="AJ297" s="19" t="n"/>
+      <c r="AK297" s="19" t="n"/>
+      <c r="AL297" s="19" t="n"/>
+      <c r="AM297" s="16" t="inlineStr">
+        <is>
+          <t>15 Scheren, der Holzblock gehört dazu.</t>
+        </is>
+      </c>
+      <c r="AN297" s="22" t="n"/>
+    </row>
+    <row r="298" ht="30" customHeight="1">
+      <c r="A298" s="15" t="inlineStr">
+        <is>
+          <t>BA08-10</t>
+        </is>
+      </c>
+      <c r="B298" s="15" t="n"/>
+      <c r="C298" s="15" t="n"/>
+      <c r="D298" s="15" t="inlineStr">
+        <is>
+          <t>BA08</t>
+        </is>
+      </c>
+      <c r="E298" s="15" t="inlineStr">
+        <is>
+          <t>Kunstpflanze Gras im weißen Topf</t>
+        </is>
+      </c>
+      <c r="F298" s="16" t="inlineStr">
+        <is>
+          <t>Künstliches Ziergras mit gedrehten Halmen in einem weißen Übertopf aus Metall mit durchbrochenem Spitzenrand.</t>
+        </is>
+      </c>
+      <c r="G298" s="15" t="inlineStr">
+        <is>
+          <t>Deko</t>
+        </is>
+      </c>
+      <c r="H298" s="15" t="inlineStr">
+        <is>
+          <t>Atelier</t>
+        </is>
+      </c>
+      <c r="I298" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J298" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K298" s="17" t="n"/>
+      <c r="L298" s="18">
+        <f>J298-IF(K298="",0,K298)</f>
+        <v/>
+      </c>
+      <c r="M298" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N298" s="15" t="inlineStr">
+        <is>
+          <t>gut</t>
+        </is>
+      </c>
+      <c r="O298" s="19" t="n"/>
+      <c r="P298" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q298" s="19" t="n"/>
+      <c r="R298" s="20" t="n"/>
+      <c r="S298" s="20" t="n">
+        <v>15</v>
+      </c>
+      <c r="T298" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U298" s="21">
+        <f>L298*S298</f>
+        <v/>
+      </c>
+      <c r="V298" s="15" t="inlineStr">
+        <is>
+          <t>Versand möglich</t>
+        </is>
+      </c>
+      <c r="W298" s="15" t="inlineStr">
+        <is>
+          <t>F-351</t>
+        </is>
+      </c>
+      <c r="X298" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y298" s="19" t="n"/>
+      <c r="Z298" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA298" s="19" t="n"/>
+      <c r="AB298" s="19" t="n"/>
+      <c r="AC298" s="19" t="n"/>
+      <c r="AD298" s="19" t="n"/>
+      <c r="AE298" s="20" t="n"/>
+      <c r="AF298" s="21">
+        <f>IF(K298="","",K298*AE298)</f>
+        <v/>
+      </c>
+      <c r="AG298" s="19" t="n"/>
+      <c r="AH298" s="19" t="n"/>
+      <c r="AI298" s="19" t="n"/>
+      <c r="AJ298" s="19" t="n"/>
+      <c r="AK298" s="19" t="n"/>
+      <c r="AL298" s="19" t="n"/>
+      <c r="AM298" s="16" t="inlineStr">
+        <is>
+          <t>2 Stück, beide abgebildet.</t>
+        </is>
+      </c>
+      <c r="AN298" s="22" t="n"/>
+    </row>
+    <row r="299" ht="30" customHeight="1">
+      <c r="A299" s="15" t="inlineStr">
+        <is>
+          <t>BA08-11</t>
+        </is>
+      </c>
+      <c r="B299" s="15" t="n"/>
+      <c r="C299" s="15" t="n"/>
+      <c r="D299" s="15" t="inlineStr">
+        <is>
+          <t>BA08</t>
+        </is>
+      </c>
+      <c r="E299" s="15" t="inlineStr">
+        <is>
+          <t>Bilderrahmen mit Zeichenwerkzeug</t>
+        </is>
+      </c>
+      <c r="F299" s="16" t="inlineStr">
+        <is>
+          <t>Zwei schwarze Rahmen hinter Glas, gepunkteter Hintergrund: einer mit Bleistift, Lineal und gefaltetem Papier, einer mit sechs Pinseln in verschiedenen Breiten. Passend für ein Atelier oder Arbeitszimmer.</t>
+        </is>
+      </c>
+      <c r="G299" s="15" t="inlineStr">
+        <is>
+          <t>Deko</t>
+        </is>
+      </c>
+      <c r="H299" s="15" t="inlineStr">
+        <is>
+          <t>Atelier</t>
+        </is>
+      </c>
+      <c r="I299" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J299" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K299" s="17" t="n"/>
+      <c r="L299" s="18">
+        <f>J299-IF(K299="",0,K299)</f>
+        <v/>
+      </c>
+      <c r="M299" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N299" s="15" t="inlineStr">
+        <is>
+          <t>gut</t>
+        </is>
+      </c>
+      <c r="O299" s="19" t="n"/>
+      <c r="P299" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q299" s="19" t="n"/>
+      <c r="R299" s="20" t="n"/>
+      <c r="S299" s="20" t="n">
+        <v>25</v>
+      </c>
+      <c r="T299" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U299" s="21">
+        <f>L299*S299</f>
+        <v/>
+      </c>
+      <c r="V299" s="15" t="inlineStr">
+        <is>
+          <t>Versand möglich</t>
+        </is>
+      </c>
+      <c r="W299" s="15" t="inlineStr">
+        <is>
+          <t>F-352</t>
+        </is>
+      </c>
+      <c r="X299" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y299" s="19" t="n"/>
+      <c r="Z299" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA299" s="19" t="n"/>
+      <c r="AB299" s="19" t="n"/>
+      <c r="AC299" s="19" t="n"/>
+      <c r="AD299" s="19" t="n"/>
+      <c r="AE299" s="20" t="n"/>
+      <c r="AF299" s="21">
+        <f>IF(K299="","",K299*AE299)</f>
+        <v/>
+      </c>
+      <c r="AG299" s="19" t="n"/>
+      <c r="AH299" s="19" t="n"/>
+      <c r="AI299" s="19" t="n"/>
+      <c r="AJ299" s="19" t="n"/>
+      <c r="AK299" s="19" t="n"/>
+      <c r="AL299" s="19" t="n"/>
+      <c r="AM299" s="16" t="inlineStr">
+        <is>
+          <t>2 Bilder, beide abgebildet.</t>
+        </is>
+      </c>
+      <c r="AN299" s="22" t="n"/>
+    </row>
+    <row r="300" ht="30" customHeight="1">
+      <c r="A300" s="15" t="inlineStr">
+        <is>
+          <t>BA08-12</t>
+        </is>
+      </c>
+      <c r="B300" s="15" t="n"/>
+      <c r="C300" s="15" t="n"/>
+      <c r="D300" s="15" t="inlineStr">
+        <is>
+          <t>BA08</t>
+        </is>
+      </c>
+      <c r="E300" s="15" t="inlineStr">
+        <is>
+          <t>Wandregalbrett weiß</t>
+        </is>
+      </c>
+      <c r="F300" s="16" t="inlineStr">
+        <is>
+          <t>Schmales weißes Wandregalbrett mit vorderer Kante, zum Anschrauben.</t>
+        </is>
+      </c>
+      <c r="G300" s="15" t="inlineStr">
+        <is>
+          <t>Möbel</t>
+        </is>
+      </c>
+      <c r="H300" s="15" t="inlineStr">
+        <is>
+          <t>Atelier</t>
+        </is>
+      </c>
+      <c r="I300" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J300" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K300" s="17" t="n"/>
+      <c r="L300" s="18">
+        <f>J300-IF(K300="",0,K300)</f>
+        <v/>
+      </c>
+      <c r="M300" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N300" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O300" s="19" t="n"/>
+      <c r="P300" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q300" s="19" t="n"/>
+      <c r="R300" s="20" t="n"/>
+      <c r="S300" s="20" t="n">
+        <v>15</v>
+      </c>
+      <c r="T300" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U300" s="21">
+        <f>L300*S300</f>
+        <v/>
+      </c>
+      <c r="V300" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W300" s="15" t="inlineStr">
+        <is>
+          <t>F-353</t>
+        </is>
+      </c>
+      <c r="X300" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y300" s="19" t="n"/>
+      <c r="Z300" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA300" s="19" t="n"/>
+      <c r="AB300" s="19" t="n"/>
+      <c r="AC300" s="19" t="n"/>
+      <c r="AD300" s="19" t="n"/>
+      <c r="AE300" s="20" t="n"/>
+      <c r="AF300" s="21">
+        <f>IF(K300="","",K300*AE300)</f>
+        <v/>
+      </c>
+      <c r="AG300" s="19" t="n"/>
+      <c r="AH300" s="19" t="n"/>
+      <c r="AI300" s="19" t="n"/>
+      <c r="AJ300" s="19" t="n"/>
+      <c r="AK300" s="19" t="n"/>
+      <c r="AL300" s="19" t="n"/>
+      <c r="AM300" s="16" t="inlineStr">
+        <is>
+          <t>2 Bretter. Die blauen Becher darauf gehören nicht dazu.</t>
+        </is>
+      </c>
+      <c r="AN300" s="22" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:AN292"/>
+  <autoFilter ref="A2:AN300"/>
   <mergeCells count="7">
     <mergeCell ref="AI1:AL1"/>
     <mergeCell ref="V1:AD1"/>
@@ -36679,7 +37643,7 @@
     <mergeCell ref="AE1:AH1"/>
     <mergeCell ref="AM1:AN1"/>
   </mergeCells>
-  <conditionalFormatting sqref="Z3:Z292">
+  <conditionalFormatting sqref="Z3:Z300">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"reserviert"</formula>
     </cfRule>
@@ -36690,12 +37654,12 @@
       <formula>"verkauft"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I3:I292">
+  <conditionalFormatting sqref="I3:I300">
     <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
       <formula>"A"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P3:P292">
+  <conditionalFormatting sqref="P3:P300">
     <cfRule type="cellIs" priority="5" operator="equal" dxfId="4">
       <formula>"entfällt"</formula>
     </cfRule>
@@ -36786,7 +37750,7 @@
         </is>
       </c>
       <c r="B5" s="27">
-        <f>COUNTA(Artikelstamm!$A$3:$A$292)</f>
+        <f>COUNTA(Artikelstamm!$A$3:$A$300)</f>
         <v/>
       </c>
     </row>
@@ -36797,7 +37761,7 @@
         </is>
       </c>
       <c r="B6" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$292,"verfügbar")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$300,"verfügbar")</f>
         <v/>
       </c>
     </row>
@@ -36808,7 +37772,7 @@
         </is>
       </c>
       <c r="B7" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$292,"reserviert")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$300,"reserviert")</f>
         <v/>
       </c>
     </row>
@@ -36819,7 +37783,7 @@
         </is>
       </c>
       <c r="B8" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$292,"teilverkauft")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$300,"teilverkauft")</f>
         <v/>
       </c>
     </row>
@@ -36830,7 +37794,7 @@
         </is>
       </c>
       <c r="B9" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$292,"verkauft")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$300,"verkauft")</f>
         <v/>
       </c>
     </row>
@@ -36841,7 +37805,7 @@
         </is>
       </c>
       <c r="B10" s="27">
-        <f>SUM(Artikelstamm!$L$3:$L$292)</f>
+        <f>SUM(Artikelstamm!$L$3:$L$300)</f>
         <v/>
       </c>
     </row>
@@ -36852,7 +37816,7 @@
         </is>
       </c>
       <c r="B11" s="29">
-        <f>SUM(Artikelstamm!$U$3:$U$292)</f>
+        <f>SUM(Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -36870,7 +37834,7 @@
         </is>
       </c>
       <c r="B13" s="27">
-        <f>SUM(Artikelstamm!$K$3:$K$292)</f>
+        <f>SUM(Artikelstamm!$K$3:$K$300)</f>
         <v/>
       </c>
     </row>
@@ -36881,7 +37845,7 @@
         </is>
       </c>
       <c r="B14" s="30">
-        <f>SUMPRODUCT(Artikelstamm!$K$3:$K$292,Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT(Artikelstamm!$K$3:$K$300,Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
     </row>
@@ -36914,7 +37878,7 @@
         </is>
       </c>
       <c r="B17" s="30">
-        <f>SUMPRODUCT((Artikelstamm!$AJ$3:$AJ$292="bezahlt")*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AJ$3:$AJ$300="bezahlt")*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
     </row>
@@ -36943,7 +37907,7 @@
         </is>
       </c>
       <c r="B21" s="31">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$292,"*verkauft",Artikelstamm!$AI$3:$AI$292,"")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$300,"*verkauft",Artikelstamm!$AI$3:$AI$300,"")</f>
         <v/>
       </c>
     </row>
@@ -36954,7 +37918,7 @@
         </is>
       </c>
       <c r="B22" s="31">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$292,"*verkauft",Artikelstamm!$AJ$3:$AJ$292,"offen")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$300,"*verkauft",Artikelstamm!$AJ$3:$AJ$300,"offen")</f>
         <v/>
       </c>
     </row>
@@ -36965,7 +37929,7 @@
         </is>
       </c>
       <c r="B23" s="27">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$292,"reserviert",Artikelstamm!$AL$3:$AL$292,"")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$300,"reserviert",Artikelstamm!$AL$3:$AL$300,"")</f>
         <v/>
       </c>
     </row>
@@ -36976,7 +37940,7 @@
         </is>
       </c>
       <c r="B24" s="27">
-        <f>COUNTIFS(Artikelstamm!$S$3:$S$292,"")</f>
+        <f>COUNTIFS(Artikelstamm!$S$3:$S$300,"")</f>
         <v/>
       </c>
     </row>
@@ -36987,7 +37951,7 @@
         </is>
       </c>
       <c r="B25" s="27">
-        <f>COUNTIFS(Artikelstamm!$O$3:$O$292,"")</f>
+        <f>COUNTIFS(Artikelstamm!$O$3:$O$300,"")</f>
         <v/>
       </c>
     </row>
@@ -37027,15 +37991,15 @@
         </is>
       </c>
       <c r="B30" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$292,$A30)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$300,$A30)</f>
         <v/>
       </c>
       <c r="C30" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$292=$A30)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$300=$A30)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D30" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$292,$A30,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$300,$A30,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37046,15 +38010,15 @@
         </is>
       </c>
       <c r="B31" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$292,$A31)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$300,$A31)</f>
         <v/>
       </c>
       <c r="C31" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$292=$A31)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$300=$A31)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D31" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$292,$A31,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$300,$A31,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37065,15 +38029,15 @@
         </is>
       </c>
       <c r="B32" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$292,$A32)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$300,$A32)</f>
         <v/>
       </c>
       <c r="C32" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$292=$A32)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$300=$A32)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D32" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$292,$A32,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$300,$A32,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37132,15 +38096,15 @@
         </is>
       </c>
       <c r="B37" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$292,$A37)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$300,$A37)</f>
         <v/>
       </c>
       <c r="C37" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$292=$A37)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$300=$A37)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D37" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$292,$A37,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$300,$A37,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37151,15 +38115,15 @@
         </is>
       </c>
       <c r="B38" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$292,$A38)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$300,$A38)</f>
         <v/>
       </c>
       <c r="C38" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$292=$A38)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$300=$A38)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D38" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$292,$A38,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$300,$A38,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37170,15 +38134,15 @@
         </is>
       </c>
       <c r="B39" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$292,$A39)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$300,$A39)</f>
         <v/>
       </c>
       <c r="C39" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$292=$A39)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$300=$A39)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D39" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$292,$A39,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$300,$A39,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37189,15 +38153,15 @@
         </is>
       </c>
       <c r="B40" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$292,$A40)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$300,$A40)</f>
         <v/>
       </c>
       <c r="C40" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$292=$A40)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$300=$A40)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D40" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$292,$A40,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$300,$A40,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37208,15 +38172,15 @@
         </is>
       </c>
       <c r="B41" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$292,$A41)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$300,$A41)</f>
         <v/>
       </c>
       <c r="C41" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$292=$A41)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$300=$A41)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D41" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$292,$A41,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$300,$A41,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37227,15 +38191,15 @@
         </is>
       </c>
       <c r="B42" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$292,$A42)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$300,$A42)</f>
         <v/>
       </c>
       <c r="C42" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$292=$A42)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$300=$A42)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D42" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$292,$A42,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$300,$A42,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37246,15 +38210,15 @@
         </is>
       </c>
       <c r="B43" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$292,$A43)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$300,$A43)</f>
         <v/>
       </c>
       <c r="C43" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$292=$A43)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$300=$A43)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D43" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$292,$A43,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$300,$A43,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37265,15 +38229,15 @@
         </is>
       </c>
       <c r="B44" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$292,$A44)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$300,$A44)</f>
         <v/>
       </c>
       <c r="C44" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$292=$A44)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$300=$A44)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D44" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$292,$A44,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$300,$A44,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37284,15 +38248,15 @@
         </is>
       </c>
       <c r="B45" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$292,$A45)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$300,$A45)</f>
         <v/>
       </c>
       <c r="C45" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$292=$A45)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$300=$A45)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D45" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$292,$A45,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$300,$A45,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37303,15 +38267,15 @@
         </is>
       </c>
       <c r="B46" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$292,$A46)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$300,$A46)</f>
         <v/>
       </c>
       <c r="C46" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$292=$A46)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$300=$A46)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D46" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$292,$A46,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$300,$A46,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37322,15 +38286,15 @@
         </is>
       </c>
       <c r="B47" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$292,$A47)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$300,$A47)</f>
         <v/>
       </c>
       <c r="C47" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$292=$A47)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$300=$A47)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D47" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$292,$A47,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$300,$A47,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37341,15 +38305,15 @@
         </is>
       </c>
       <c r="B48" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$292,$A48)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$300,$A48)</f>
         <v/>
       </c>
       <c r="C48" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$292=$A48)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$300=$A48)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D48" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$292,$A48,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$300,$A48,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37360,15 +38324,15 @@
         </is>
       </c>
       <c r="B49" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$292,$A49)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$300,$A49)</f>
         <v/>
       </c>
       <c r="C49" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$292=$A49)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$300=$A49)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D49" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$292,$A49,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$300,$A49,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37379,15 +38343,15 @@
         </is>
       </c>
       <c r="B50" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$292,$A50)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$300,$A50)</f>
         <v/>
       </c>
       <c r="C50" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$292=$A50)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$300=$A50)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D50" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$292,$A50,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$300,$A50,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37446,15 +38410,15 @@
         </is>
       </c>
       <c r="B55" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A55)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A55)</f>
         <v/>
       </c>
       <c r="C55" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A55)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A55)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D55" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A55,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A55,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37465,15 +38429,15 @@
         </is>
       </c>
       <c r="B56" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A56)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A56)</f>
         <v/>
       </c>
       <c r="C56" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A56)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A56)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D56" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A56,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A56,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37484,15 +38448,15 @@
         </is>
       </c>
       <c r="B57" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A57)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A57)</f>
         <v/>
       </c>
       <c r="C57" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A57)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A57)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D57" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A57,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A57,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37503,15 +38467,15 @@
         </is>
       </c>
       <c r="B58" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A58)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A58)</f>
         <v/>
       </c>
       <c r="C58" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A58)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A58)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D58" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A58,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A58,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37522,15 +38486,15 @@
         </is>
       </c>
       <c r="B59" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A59)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A59)</f>
         <v/>
       </c>
       <c r="C59" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A59)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A59)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D59" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A59,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A59,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37541,15 +38505,15 @@
         </is>
       </c>
       <c r="B60" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A60)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A60)</f>
         <v/>
       </c>
       <c r="C60" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A60)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A60)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D60" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A60,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A60,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37560,15 +38524,15 @@
         </is>
       </c>
       <c r="B61" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A61)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A61)</f>
         <v/>
       </c>
       <c r="C61" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A61)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A61)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D61" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A61,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A61,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37579,15 +38543,15 @@
         </is>
       </c>
       <c r="B62" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A62)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A62)</f>
         <v/>
       </c>
       <c r="C62" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A62)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A62)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D62" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A62,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A62,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37598,15 +38562,15 @@
         </is>
       </c>
       <c r="B63" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A63)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A63)</f>
         <v/>
       </c>
       <c r="C63" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A63)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A63)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D63" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A63,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A63,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37617,15 +38581,15 @@
         </is>
       </c>
       <c r="B64" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A64)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A64)</f>
         <v/>
       </c>
       <c r="C64" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A64)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A64)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D64" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A64,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A64,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37636,15 +38600,15 @@
         </is>
       </c>
       <c r="B65" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A65)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A65)</f>
         <v/>
       </c>
       <c r="C65" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A65)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A65)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D65" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A65,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A65,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37655,15 +38619,15 @@
         </is>
       </c>
       <c r="B66" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A66)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A66)</f>
         <v/>
       </c>
       <c r="C66" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A66)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A66)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D66" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A66,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A66,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37674,15 +38638,15 @@
         </is>
       </c>
       <c r="B67" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A67)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A67)</f>
         <v/>
       </c>
       <c r="C67" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A67)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A67)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D67" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A67,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A67,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37693,15 +38657,15 @@
         </is>
       </c>
       <c r="B68" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A68)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A68)</f>
         <v/>
       </c>
       <c r="C68" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A68)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A68)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D68" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A68,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A68,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37712,15 +38676,15 @@
         </is>
       </c>
       <c r="B69" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A69)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A69)</f>
         <v/>
       </c>
       <c r="C69" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A69)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A69)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D69" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A69,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A69,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37731,15 +38695,15 @@
         </is>
       </c>
       <c r="B70" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A70)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A70)</f>
         <v/>
       </c>
       <c r="C70" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A70)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A70)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D70" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A70,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A70,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37750,15 +38714,15 @@
         </is>
       </c>
       <c r="B71" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A71)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A71)</f>
         <v/>
       </c>
       <c r="C71" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A71)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A71)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D71" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A71,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A71,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37769,15 +38733,15 @@
         </is>
       </c>
       <c r="B72" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A72)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A72)</f>
         <v/>
       </c>
       <c r="C72" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A72)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A72)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D72" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A72,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A72,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37788,15 +38752,15 @@
         </is>
       </c>
       <c r="B73" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A73)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A73)</f>
         <v/>
       </c>
       <c r="C73" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A73)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A73)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D73" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A73,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A73,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37807,15 +38771,15 @@
         </is>
       </c>
       <c r="B74" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A74)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A74)</f>
         <v/>
       </c>
       <c r="C74" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A74)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A74)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D74" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A74,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A74,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37826,15 +38790,15 @@
         </is>
       </c>
       <c r="B75" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A75)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A75)</f>
         <v/>
       </c>
       <c r="C75" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A75)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A75)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D75" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A75,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A75,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37845,15 +38809,15 @@
         </is>
       </c>
       <c r="B76" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A76)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A76)</f>
         <v/>
       </c>
       <c r="C76" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A76)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A76)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D76" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A76,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A76,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37864,15 +38828,15 @@
         </is>
       </c>
       <c r="B77" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A77)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A77)</f>
         <v/>
       </c>
       <c r="C77" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A77)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A77)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D77" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A77,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A77,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37883,15 +38847,15 @@
         </is>
       </c>
       <c r="B78" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A78)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A78)</f>
         <v/>
       </c>
       <c r="C78" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A78)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A78)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D78" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A78,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A78,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37902,15 +38866,15 @@
         </is>
       </c>
       <c r="B79" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A79)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A79)</f>
         <v/>
       </c>
       <c r="C79" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A79)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A79)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D79" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A79,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A79,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37921,15 +38885,15 @@
         </is>
       </c>
       <c r="B80" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A80)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A80)</f>
         <v/>
       </c>
       <c r="C80" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A80)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A80)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D80" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A80,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A80,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37940,15 +38904,15 @@
         </is>
       </c>
       <c r="B81" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A81)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A81)</f>
         <v/>
       </c>
       <c r="C81" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A81)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A81)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D81" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A81,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A81,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -37959,15 +38923,15 @@
         </is>
       </c>
       <c r="B82" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$292,$A82)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A82)</f>
         <v/>
       </c>
       <c r="C82" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$292=$A82)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A82)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
       <c r="D82" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$292,$A82,Artikelstamm!$U$3:$U$292)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A82,Artikelstamm!$U$3:$U$300)</f>
         <v/>
       </c>
     </row>
@@ -38021,11 +38985,11 @@
         </is>
       </c>
       <c r="B87" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$292,$A87)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$300,$A87)</f>
         <v/>
       </c>
       <c r="C87" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$292=$A87)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$300=$A87)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
     </row>
@@ -38036,11 +39000,11 @@
         </is>
       </c>
       <c r="B88" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$292,$A88)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$300,$A88)</f>
         <v/>
       </c>
       <c r="C88" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$292=$A88)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$300=$A88)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
     </row>
@@ -38051,11 +39015,11 @@
         </is>
       </c>
       <c r="B89" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$292,$A89)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$300,$A89)</f>
         <v/>
       </c>
       <c r="C89" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$292=$A89)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$300=$A89)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
     </row>
@@ -38066,11 +39030,11 @@
         </is>
       </c>
       <c r="B90" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$292,$A90)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$300,$A90)</f>
         <v/>
       </c>
       <c r="C90" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$292=$A90)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$300=$A90)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
     </row>
@@ -38081,11 +39045,11 @@
         </is>
       </c>
       <c r="B91" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$292,$A91)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$300,$A91)</f>
         <v/>
       </c>
       <c r="C91" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$292=$A91)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$300=$A91)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
     </row>
@@ -38096,11 +39060,11 @@
         </is>
       </c>
       <c r="B92" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$292,$A92)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$300,$A92)</f>
         <v/>
       </c>
       <c r="C92" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$292=$A92)*Artikelstamm!$K$3:$K$292*Artikelstamm!$AE$3:$AE$292)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$300=$A92)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
BU01 erfasst: 6 Positionen, Regal jetzt in fuenf Raeumen
Flur 1 (Bestandsgebaeude UG, 21,65 m2) - erster Raum im Untergeschoss des
Bestandsgebaeudes.

BU01-03 sind zwei weitere 8-Faecher-Regale; NU04-09 waechst damit von 8
auf 10 Stueck ueber fuenf Raeume und ist die am weitesten verteilte
Position im Bestand.

Marken ueber Etikett belegt: IKEA Smastad (Maltische, 804.335.42, Etikett
auf F-360) und IKEA Grua (Wandspiegel, Etikett auf F-363).

BU01-06 ist laut Nutzerin zweimal vorhanden, auf dem Blatt stand 1 -
entsprechend eingetragen.

BU01-02 ist die vierte Spielkueche im Haus, deutlich kleiner als die drei
anderen. Alle vier verweisen aufeinander.

Datenschutz: die Spiegelung auf F-362 zeigt nur Tuer und Regale, keine
Person - nachgeprueft.

Gesamtwert netto 42.970 -> 43.530 EUR, 249 aktive Positionen.
pruefen.py: 0 Fehler, 3 Hinweise.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011yyfqhuiWGsaNy38oaNoGo
</commit_message>
<xml_diff>
--- a/ausgabe/01_Artikelstamm_kikripp.xlsx
+++ b/ausgabe/01_Artikelstamm_kikripp.xlsx
@@ -15,7 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Artikelstamm'!$A$2:$AN$300</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Artikelstamm'!$A$2:$AN$306</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1019,7 +1019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN300"/>
+  <dimension ref="A1:AN306"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -23982,7 +23982,7 @@
       <c r="B188" s="15" t="n"/>
       <c r="C188" s="15" t="inlineStr">
         <is>
-          <t>NU05-05, NU07-06, BA04-03</t>
+          <t>NU05-05, NU07-06, BA04-03, BU01-03</t>
         </is>
       </c>
       <c r="D188" s="15" t="inlineStr">
@@ -24016,7 +24016,7 @@
         </is>
       </c>
       <c r="J188" s="17" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K188" s="17" t="n"/>
       <c r="L188" s="18">
@@ -24095,12 +24095,12 @@
       <c r="AL188" s="19" t="n"/>
       <c r="AM188" s="16" t="inlineStr">
         <is>
-          <t>8 Regale insgesamt: 3 im Schlafraum 5, 1 im Treppenraum 1 (NU05-05), 1 in der Garage (NU07-06) und 3 im Gruppenraum 4 (BA04-03).</t>
+          <t>10 Regale insgesamt: 3 im Schlafraum 5, 1 im Treppenraum 1 (NU05-05), 1 in der Garage (NU07-06), 3 im Gruppenraum 4 (BA04-03) und 2 im Flur 1 des Bestandsgebäudes (BU01-03).</t>
         </is>
       </c>
       <c r="AN188" s="22" t="inlineStr">
         <is>
-          <t>Zusammengefasste Position über vier Räume – Post-it-Nummern: NU05-05, NU07-06, BA04-03.</t>
+          <t>Zusammengefasste Position über fünf Räume – Post-it-Nummern: NU05-05, NU07-06, BA04-03, BU01-03.</t>
         </is>
       </c>
     </row>
@@ -37632,8 +37632,730 @@
       </c>
       <c r="AN300" s="22" t="n"/>
     </row>
+    <row r="301" ht="30" customHeight="1">
+      <c r="A301" s="15" t="inlineStr">
+        <is>
+          <t>BU01-01</t>
+        </is>
+      </c>
+      <c r="B301" s="15" t="n"/>
+      <c r="C301" s="15" t="n"/>
+      <c r="D301" s="15" t="inlineStr">
+        <is>
+          <t>BU01</t>
+        </is>
+      </c>
+      <c r="E301" s="15" t="inlineStr">
+        <is>
+          <t>Hausbett Buche massiv</t>
+        </is>
+      </c>
+      <c r="F301" s="16" t="inlineStr">
+        <is>
+          <t>Kinderbett in Hausform aus massiver Buche, natur geölt, mit Dachgiebel und umlaufendem Rahmen. Einschließlich Matratze.</t>
+        </is>
+      </c>
+      <c r="G301" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H301" s="15" t="inlineStr">
+        <is>
+          <t>Flur 1</t>
+        </is>
+      </c>
+      <c r="I301" s="15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J301" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K301" s="17" t="n"/>
+      <c r="L301" s="18">
+        <f>J301-IF(K301="",0,K301)</f>
+        <v/>
+      </c>
+      <c r="M301" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N301" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O301" s="19" t="n"/>
+      <c r="P301" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q301" s="19" t="n"/>
+      <c r="R301" s="20" t="n"/>
+      <c r="S301" s="20" t="n">
+        <v>220</v>
+      </c>
+      <c r="T301" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U301" s="21">
+        <f>L301*S301</f>
+        <v/>
+      </c>
+      <c r="V301" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W301" s="15" t="inlineStr">
+        <is>
+          <t>F-356</t>
+        </is>
+      </c>
+      <c r="X301" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y301" s="19" t="n"/>
+      <c r="Z301" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA301" s="19" t="n"/>
+      <c r="AB301" s="19" t="n"/>
+      <c r="AC301" s="19" t="n"/>
+      <c r="AD301" s="19" t="n"/>
+      <c r="AE301" s="20" t="n"/>
+      <c r="AF301" s="21">
+        <f>IF(K301="","",K301*AE301)</f>
+        <v/>
+      </c>
+      <c r="AG301" s="19" t="n"/>
+      <c r="AH301" s="19" t="n"/>
+      <c r="AI301" s="19" t="n"/>
+      <c r="AJ301" s="19" t="n"/>
+      <c r="AK301" s="19" t="n"/>
+      <c r="AL301" s="19" t="n"/>
+      <c r="AM301" s="16" t="inlineStr">
+        <is>
+          <t>1 Bett einschließlich Matratze. Kissen und Bettschlange gehören nicht dazu.</t>
+        </is>
+      </c>
+      <c r="AN301" s="22" t="n"/>
+    </row>
+    <row r="302" ht="30" customHeight="1">
+      <c r="A302" s="15" t="inlineStr">
+        <is>
+          <t>BU01-02</t>
+        </is>
+      </c>
+      <c r="B302" s="15" t="n"/>
+      <c r="C302" s="15" t="n"/>
+      <c r="D302" s="15" t="inlineStr">
+        <is>
+          <t>BU01</t>
+        </is>
+      </c>
+      <c r="E302" s="15" t="inlineStr">
+        <is>
+          <t>Spielküche klein mit Mikrowelle</t>
+        </is>
+      </c>
+      <c r="F302" s="16" t="inlineStr">
+        <is>
+          <t>Kleine Spielküche aus Birke-Multiplex mit weißen Fronten: Aufsatz mit Mikrowelle und zwei offenen Fächern, Arbeitsplatte mit Kochfeld, Spülbecken und Wasserhahn, darunter Backofen mit Sichtfenster und ein Schrank.</t>
+        </is>
+      </c>
+      <c r="G302" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H302" s="15" t="inlineStr">
+        <is>
+          <t>Flur 1</t>
+        </is>
+      </c>
+      <c r="I302" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J302" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K302" s="17" t="n"/>
+      <c r="L302" s="18">
+        <f>J302-IF(K302="",0,K302)</f>
+        <v/>
+      </c>
+      <c r="M302" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N302" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O302" s="19" t="n"/>
+      <c r="P302" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q302" s="19" t="n"/>
+      <c r="R302" s="20" t="n"/>
+      <c r="S302" s="20" t="n">
+        <v>60</v>
+      </c>
+      <c r="T302" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U302" s="21">
+        <f>L302*S302</f>
+        <v/>
+      </c>
+      <c r="V302" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W302" s="15" t="inlineStr">
+        <is>
+          <t>F-355</t>
+        </is>
+      </c>
+      <c r="X302" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y302" s="19" t="n"/>
+      <c r="Z302" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA302" s="19" t="n"/>
+      <c r="AB302" s="19" t="n"/>
+      <c r="AC302" s="19" t="n"/>
+      <c r="AD302" s="19" t="n"/>
+      <c r="AE302" s="20" t="n"/>
+      <c r="AF302" s="21">
+        <f>IF(K302="","",K302*AE302)</f>
+        <v/>
+      </c>
+      <c r="AG302" s="19" t="n"/>
+      <c r="AH302" s="19" t="n"/>
+      <c r="AI302" s="19" t="n"/>
+      <c r="AJ302" s="19" t="n"/>
+      <c r="AK302" s="19" t="n"/>
+      <c r="AL302" s="19" t="n"/>
+      <c r="AM302" s="16" t="inlineStr">
+        <is>
+          <t>1 Küche. Spielgeschirr und Zubehör gehören nicht dazu. Drei größere Spielküchen stehen unter NU03-03, NU07-03 und BA03-02.</t>
+        </is>
+      </c>
+      <c r="AN302" s="22" t="n"/>
+    </row>
+    <row r="303" ht="30" customHeight="1">
+      <c r="A303" s="15" t="inlineStr">
+        <is>
+          <t>BU01-04</t>
+        </is>
+      </c>
+      <c r="B303" s="15" t="n"/>
+      <c r="C303" s="15" t="n"/>
+      <c r="D303" s="15" t="inlineStr">
+        <is>
+          <t>BU01</t>
+        </is>
+      </c>
+      <c r="E303" s="15" t="inlineStr">
+        <is>
+          <t>Gestell Kiefer mit sechs Wannen</t>
+        </is>
+      </c>
+      <c r="F303" s="16" t="inlineStr">
+        <is>
+          <t>Gestell aus Kiefer massiv mit sechs weißen Kunststoffwannen in zwei Reihen, als Spielzeugaufbewahrung genutzt.</t>
+        </is>
+      </c>
+      <c r="G303" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H303" s="15" t="inlineStr">
+        <is>
+          <t>Flur 1</t>
+        </is>
+      </c>
+      <c r="I303" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J303" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K303" s="17" t="n"/>
+      <c r="L303" s="18">
+        <f>J303-IF(K303="",0,K303)</f>
+        <v/>
+      </c>
+      <c r="M303" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N303" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O303" s="19" t="n"/>
+      <c r="P303" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q303" s="19" t="n"/>
+      <c r="R303" s="20" t="n"/>
+      <c r="S303" s="20" t="n">
+        <v>55</v>
+      </c>
+      <c r="T303" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U303" s="21">
+        <f>L303*S303</f>
+        <v/>
+      </c>
+      <c r="V303" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W303" s="15" t="inlineStr">
+        <is>
+          <t>F-358</t>
+        </is>
+      </c>
+      <c r="X303" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y303" s="19" t="n"/>
+      <c r="Z303" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA303" s="19" t="n"/>
+      <c r="AB303" s="19" t="n"/>
+      <c r="AC303" s="19" t="n"/>
+      <c r="AD303" s="19" t="n"/>
+      <c r="AE303" s="20" t="n"/>
+      <c r="AF303" s="21">
+        <f>IF(K303="","",K303*AE303)</f>
+        <v/>
+      </c>
+      <c r="AG303" s="19" t="n"/>
+      <c r="AH303" s="19" t="n"/>
+      <c r="AI303" s="19" t="n"/>
+      <c r="AJ303" s="19" t="n"/>
+      <c r="AK303" s="19" t="n"/>
+      <c r="AL303" s="19" t="n"/>
+      <c r="AM303" s="16" t="inlineStr">
+        <is>
+          <t>1 Gestell einschließlich der Wannen. Der Inhalt gehört nicht dazu.</t>
+        </is>
+      </c>
+      <c r="AN303" s="22" t="n"/>
+    </row>
+    <row r="304" ht="30" customHeight="1">
+      <c r="A304" s="15" t="inlineStr">
+        <is>
+          <t>BU01-05</t>
+        </is>
+      </c>
+      <c r="B304" s="15" t="n"/>
+      <c r="C304" s="15" t="n"/>
+      <c r="D304" s="15" t="inlineStr">
+        <is>
+          <t>BU01</t>
+        </is>
+      </c>
+      <c r="E304" s="15" t="inlineStr">
+        <is>
+          <t>IKEA Småstad Kindertisch weiß</t>
+        </is>
+      </c>
+      <c r="F304" s="16" t="inlineStr">
+        <is>
+          <t>Niedriger Kindertisch von IKEA in Weiß mit Seitenwangen, Etikett an der Unterseite: Småstad, 804.335.42. Die Platte ist stark verkratzt und mit einer Schutzfolie belegt.</t>
+        </is>
+      </c>
+      <c r="G304" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H304" s="15" t="inlineStr">
+        <is>
+          <t>Flur 1</t>
+        </is>
+      </c>
+      <c r="I304" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J304" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K304" s="17" t="n"/>
+      <c r="L304" s="18">
+        <f>J304-IF(K304="",0,K304)</f>
+        <v/>
+      </c>
+      <c r="M304" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N304" s="15" t="inlineStr">
+        <is>
+          <t>stark gebraucht</t>
+        </is>
+      </c>
+      <c r="O304" s="19" t="n"/>
+      <c r="P304" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q304" s="19" t="n"/>
+      <c r="R304" s="20" t="n"/>
+      <c r="S304" s="20" t="n">
+        <v>35</v>
+      </c>
+      <c r="T304" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U304" s="21">
+        <f>L304*S304</f>
+        <v/>
+      </c>
+      <c r="V304" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W304" s="15" t="inlineStr">
+        <is>
+          <t>F-359</t>
+        </is>
+      </c>
+      <c r="X304" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y304" s="19" t="n"/>
+      <c r="Z304" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA304" s="19" t="inlineStr">
+        <is>
+          <t>IKEA</t>
+        </is>
+      </c>
+      <c r="AB304" s="19" t="n"/>
+      <c r="AC304" s="19" t="n"/>
+      <c r="AD304" s="19" t="n"/>
+      <c r="AE304" s="20" t="n"/>
+      <c r="AF304" s="21">
+        <f>IF(K304="","",K304*AE304)</f>
+        <v/>
+      </c>
+      <c r="AG304" s="19" t="n"/>
+      <c r="AH304" s="19" t="n"/>
+      <c r="AI304" s="19" t="n"/>
+      <c r="AJ304" s="19" t="n"/>
+      <c r="AK304" s="19" t="n"/>
+      <c r="AL304" s="19" t="n"/>
+      <c r="AM304" s="16" t="inlineStr">
+        <is>
+          <t>2 Tische – abgebildet ist einer davon. Das Etikett ist auf Foto F-360 zu sehen.</t>
+        </is>
+      </c>
+      <c r="AN304" s="22" t="n"/>
+    </row>
+    <row r="305" ht="30" customHeight="1">
+      <c r="A305" s="15" t="inlineStr">
+        <is>
+          <t>BU01-06</t>
+        </is>
+      </c>
+      <c r="B305" s="15" t="n"/>
+      <c r="C305" s="15" t="n"/>
+      <c r="D305" s="15" t="inlineStr">
+        <is>
+          <t>BU01</t>
+        </is>
+      </c>
+      <c r="E305" s="15" t="inlineStr">
+        <is>
+          <t>Wanddeko Lama, Steckwand</t>
+        </is>
+      </c>
+      <c r="F305" s="16" t="inlineStr">
+        <is>
+          <t>Wandelement in Lamaform aus weiß lackiertem Holz mit grauen Ohren, Gesicht und Füßen, durchgehend gelocht zum Einstecken von Haken oder Stäben.</t>
+        </is>
+      </c>
+      <c r="G305" s="15" t="inlineStr">
+        <is>
+          <t>Deko</t>
+        </is>
+      </c>
+      <c r="H305" s="15" t="inlineStr">
+        <is>
+          <t>Flur 1</t>
+        </is>
+      </c>
+      <c r="I305" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J305" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K305" s="17" t="n"/>
+      <c r="L305" s="18">
+        <f>J305-IF(K305="",0,K305)</f>
+        <v/>
+      </c>
+      <c r="M305" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N305" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O305" s="19" t="n"/>
+      <c r="P305" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q305" s="19" t="n"/>
+      <c r="R305" s="20" t="n"/>
+      <c r="S305" s="20" t="n">
+        <v>25</v>
+      </c>
+      <c r="T305" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U305" s="21">
+        <f>L305*S305</f>
+        <v/>
+      </c>
+      <c r="V305" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W305" s="15" t="inlineStr">
+        <is>
+          <t>F-361</t>
+        </is>
+      </c>
+      <c r="X305" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y305" s="19" t="n"/>
+      <c r="Z305" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA305" s="19" t="n"/>
+      <c r="AB305" s="19" t="n"/>
+      <c r="AC305" s="19" t="n"/>
+      <c r="AD305" s="19" t="n"/>
+      <c r="AE305" s="20" t="n"/>
+      <c r="AF305" s="21">
+        <f>IF(K305="","",K305*AE305)</f>
+        <v/>
+      </c>
+      <c r="AG305" s="19" t="n"/>
+      <c r="AH305" s="19" t="n"/>
+      <c r="AI305" s="19" t="n"/>
+      <c r="AJ305" s="19" t="n"/>
+      <c r="AK305" s="19" t="n"/>
+      <c r="AL305" s="19" t="n"/>
+      <c r="AM305" s="16" t="inlineStr">
+        <is>
+          <t>2 Stück – abgebildet ist eines davon.</t>
+        </is>
+      </c>
+      <c r="AN305" s="22" t="n"/>
+    </row>
+    <row r="306" ht="30" customHeight="1">
+      <c r="A306" s="15" t="inlineStr">
+        <is>
+          <t>BU01-07</t>
+        </is>
+      </c>
+      <c r="B306" s="15" t="n"/>
+      <c r="C306" s="15" t="n"/>
+      <c r="D306" s="15" t="inlineStr">
+        <is>
+          <t>BU01</t>
+        </is>
+      </c>
+      <c r="E306" s="15" t="inlineStr">
+        <is>
+          <t>IKEA Grua Wandspiegel, schwarzer Rahmen</t>
+        </is>
+      </c>
+      <c r="F306" s="16" t="inlineStr">
+        <is>
+          <t>Wandspiegel mit schmalem schwarzem Rahmen und abgerundeten Ecken. Etikett auf der Rückseite: Grua, IKEA.</t>
+        </is>
+      </c>
+      <c r="G306" s="15" t="inlineStr">
+        <is>
+          <t>Deko</t>
+        </is>
+      </c>
+      <c r="H306" s="15" t="inlineStr">
+        <is>
+          <t>Flur 1</t>
+        </is>
+      </c>
+      <c r="I306" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J306" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K306" s="17" t="n"/>
+      <c r="L306" s="18">
+        <f>J306-IF(K306="",0,K306)</f>
+        <v/>
+      </c>
+      <c r="M306" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N306" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O306" s="19" t="n"/>
+      <c r="P306" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q306" s="19" t="n"/>
+      <c r="R306" s="20" t="n"/>
+      <c r="S306" s="20" t="n">
+        <v>25</v>
+      </c>
+      <c r="T306" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U306" s="21">
+        <f>L306*S306</f>
+        <v/>
+      </c>
+      <c r="V306" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W306" s="15" t="inlineStr">
+        <is>
+          <t>F-362</t>
+        </is>
+      </c>
+      <c r="X306" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y306" s="19" t="n"/>
+      <c r="Z306" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA306" s="19" t="inlineStr">
+        <is>
+          <t>IKEA</t>
+        </is>
+      </c>
+      <c r="AB306" s="19" t="n"/>
+      <c r="AC306" s="19" t="n"/>
+      <c r="AD306" s="19" t="n"/>
+      <c r="AE306" s="20" t="n"/>
+      <c r="AF306" s="21">
+        <f>IF(K306="","",K306*AE306)</f>
+        <v/>
+      </c>
+      <c r="AG306" s="19" t="n"/>
+      <c r="AH306" s="19" t="n"/>
+      <c r="AI306" s="19" t="n"/>
+      <c r="AJ306" s="19" t="n"/>
+      <c r="AK306" s="19" t="n"/>
+      <c r="AL306" s="19" t="n"/>
+      <c r="AM306" s="16" t="inlineStr">
+        <is>
+          <t>1 Spiegel. Das Etikett ist auf Foto F-363 zu sehen.</t>
+        </is>
+      </c>
+      <c r="AN306" s="22" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:AN300"/>
+  <autoFilter ref="A2:AN306"/>
   <mergeCells count="7">
     <mergeCell ref="AI1:AL1"/>
     <mergeCell ref="V1:AD1"/>
@@ -37643,7 +38365,7 @@
     <mergeCell ref="AE1:AH1"/>
     <mergeCell ref="AM1:AN1"/>
   </mergeCells>
-  <conditionalFormatting sqref="Z3:Z300">
+  <conditionalFormatting sqref="Z3:Z306">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"reserviert"</formula>
     </cfRule>
@@ -37654,12 +38376,12 @@
       <formula>"verkauft"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I3:I300">
+  <conditionalFormatting sqref="I3:I306">
     <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
       <formula>"A"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P3:P300">
+  <conditionalFormatting sqref="P3:P306">
     <cfRule type="cellIs" priority="5" operator="equal" dxfId="4">
       <formula>"entfällt"</formula>
     </cfRule>
@@ -37750,7 +38472,7 @@
         </is>
       </c>
       <c r="B5" s="27">
-        <f>COUNTA(Artikelstamm!$A$3:$A$300)</f>
+        <f>COUNTA(Artikelstamm!$A$3:$A$306)</f>
         <v/>
       </c>
     </row>
@@ -37761,7 +38483,7 @@
         </is>
       </c>
       <c r="B6" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$300,"verfügbar")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$306,"verfügbar")</f>
         <v/>
       </c>
     </row>
@@ -37772,7 +38494,7 @@
         </is>
       </c>
       <c r="B7" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$300,"reserviert")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$306,"reserviert")</f>
         <v/>
       </c>
     </row>
@@ -37783,7 +38505,7 @@
         </is>
       </c>
       <c r="B8" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$300,"teilverkauft")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$306,"teilverkauft")</f>
         <v/>
       </c>
     </row>
@@ -37794,7 +38516,7 @@
         </is>
       </c>
       <c r="B9" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$300,"verkauft")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$306,"verkauft")</f>
         <v/>
       </c>
     </row>
@@ -37805,7 +38527,7 @@
         </is>
       </c>
       <c r="B10" s="27">
-        <f>SUM(Artikelstamm!$L$3:$L$300)</f>
+        <f>SUM(Artikelstamm!$L$3:$L$306)</f>
         <v/>
       </c>
     </row>
@@ -37816,7 +38538,7 @@
         </is>
       </c>
       <c r="B11" s="29">
-        <f>SUM(Artikelstamm!$U$3:$U$300)</f>
+        <f>SUM(Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -37834,7 +38556,7 @@
         </is>
       </c>
       <c r="B13" s="27">
-        <f>SUM(Artikelstamm!$K$3:$K$300)</f>
+        <f>SUM(Artikelstamm!$K$3:$K$306)</f>
         <v/>
       </c>
     </row>
@@ -37845,7 +38567,7 @@
         </is>
       </c>
       <c r="B14" s="30">
-        <f>SUMPRODUCT(Artikelstamm!$K$3:$K$300,Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT(Artikelstamm!$K$3:$K$306,Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
     </row>
@@ -37878,7 +38600,7 @@
         </is>
       </c>
       <c r="B17" s="30">
-        <f>SUMPRODUCT((Artikelstamm!$AJ$3:$AJ$300="bezahlt")*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AJ$3:$AJ$306="bezahlt")*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
     </row>
@@ -37907,7 +38629,7 @@
         </is>
       </c>
       <c r="B21" s="31">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$300,"*verkauft",Artikelstamm!$AI$3:$AI$300,"")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$306,"*verkauft",Artikelstamm!$AI$3:$AI$306,"")</f>
         <v/>
       </c>
     </row>
@@ -37918,7 +38640,7 @@
         </is>
       </c>
       <c r="B22" s="31">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$300,"*verkauft",Artikelstamm!$AJ$3:$AJ$300,"offen")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$306,"*verkauft",Artikelstamm!$AJ$3:$AJ$306,"offen")</f>
         <v/>
       </c>
     </row>
@@ -37929,7 +38651,7 @@
         </is>
       </c>
       <c r="B23" s="27">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$300,"reserviert",Artikelstamm!$AL$3:$AL$300,"")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$306,"reserviert",Artikelstamm!$AL$3:$AL$306,"")</f>
         <v/>
       </c>
     </row>
@@ -37940,7 +38662,7 @@
         </is>
       </c>
       <c r="B24" s="27">
-        <f>COUNTIFS(Artikelstamm!$S$3:$S$300,"")</f>
+        <f>COUNTIFS(Artikelstamm!$S$3:$S$306,"")</f>
         <v/>
       </c>
     </row>
@@ -37951,7 +38673,7 @@
         </is>
       </c>
       <c r="B25" s="27">
-        <f>COUNTIFS(Artikelstamm!$O$3:$O$300,"")</f>
+        <f>COUNTIFS(Artikelstamm!$O$3:$O$306,"")</f>
         <v/>
       </c>
     </row>
@@ -37991,15 +38713,15 @@
         </is>
       </c>
       <c r="B30" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$300,$A30)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$306,$A30)</f>
         <v/>
       </c>
       <c r="C30" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$300=$A30)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$306=$A30)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D30" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$300,$A30,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$306,$A30,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38010,15 +38732,15 @@
         </is>
       </c>
       <c r="B31" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$300,$A31)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$306,$A31)</f>
         <v/>
       </c>
       <c r="C31" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$300=$A31)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$306=$A31)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D31" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$300,$A31,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$306,$A31,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38029,15 +38751,15 @@
         </is>
       </c>
       <c r="B32" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$300,$A32)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$306,$A32)</f>
         <v/>
       </c>
       <c r="C32" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$300=$A32)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$306=$A32)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D32" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$300,$A32,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$306,$A32,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38096,15 +38818,15 @@
         </is>
       </c>
       <c r="B37" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$300,$A37)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$306,$A37)</f>
         <v/>
       </c>
       <c r="C37" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$300=$A37)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$306=$A37)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D37" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$300,$A37,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$306,$A37,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38115,15 +38837,15 @@
         </is>
       </c>
       <c r="B38" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$300,$A38)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$306,$A38)</f>
         <v/>
       </c>
       <c r="C38" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$300=$A38)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$306=$A38)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D38" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$300,$A38,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$306,$A38,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38134,15 +38856,15 @@
         </is>
       </c>
       <c r="B39" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$300,$A39)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$306,$A39)</f>
         <v/>
       </c>
       <c r="C39" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$300=$A39)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$306=$A39)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D39" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$300,$A39,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$306,$A39,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38153,15 +38875,15 @@
         </is>
       </c>
       <c r="B40" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$300,$A40)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$306,$A40)</f>
         <v/>
       </c>
       <c r="C40" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$300=$A40)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$306=$A40)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D40" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$300,$A40,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$306,$A40,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38172,15 +38894,15 @@
         </is>
       </c>
       <c r="B41" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$300,$A41)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$306,$A41)</f>
         <v/>
       </c>
       <c r="C41" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$300=$A41)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$306=$A41)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D41" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$300,$A41,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$306,$A41,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38191,15 +38913,15 @@
         </is>
       </c>
       <c r="B42" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$300,$A42)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$306,$A42)</f>
         <v/>
       </c>
       <c r="C42" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$300=$A42)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$306=$A42)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D42" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$300,$A42,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$306,$A42,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38210,15 +38932,15 @@
         </is>
       </c>
       <c r="B43" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$300,$A43)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$306,$A43)</f>
         <v/>
       </c>
       <c r="C43" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$300=$A43)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$306=$A43)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D43" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$300,$A43,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$306,$A43,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38229,15 +38951,15 @@
         </is>
       </c>
       <c r="B44" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$300,$A44)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$306,$A44)</f>
         <v/>
       </c>
       <c r="C44" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$300=$A44)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$306=$A44)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D44" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$300,$A44,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$306,$A44,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38248,15 +38970,15 @@
         </is>
       </c>
       <c r="B45" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$300,$A45)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$306,$A45)</f>
         <v/>
       </c>
       <c r="C45" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$300=$A45)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$306=$A45)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D45" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$300,$A45,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$306,$A45,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38267,15 +38989,15 @@
         </is>
       </c>
       <c r="B46" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$300,$A46)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$306,$A46)</f>
         <v/>
       </c>
       <c r="C46" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$300=$A46)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$306=$A46)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D46" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$300,$A46,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$306,$A46,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38286,15 +39008,15 @@
         </is>
       </c>
       <c r="B47" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$300,$A47)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$306,$A47)</f>
         <v/>
       </c>
       <c r="C47" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$300=$A47)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$306=$A47)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D47" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$300,$A47,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$306,$A47,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38305,15 +39027,15 @@
         </is>
       </c>
       <c r="B48" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$300,$A48)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$306,$A48)</f>
         <v/>
       </c>
       <c r="C48" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$300=$A48)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$306=$A48)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D48" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$300,$A48,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$306,$A48,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38324,15 +39046,15 @@
         </is>
       </c>
       <c r="B49" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$300,$A49)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$306,$A49)</f>
         <v/>
       </c>
       <c r="C49" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$300=$A49)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$306=$A49)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D49" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$300,$A49,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$306,$A49,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38343,15 +39065,15 @@
         </is>
       </c>
       <c r="B50" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$300,$A50)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$306,$A50)</f>
         <v/>
       </c>
       <c r="C50" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$300=$A50)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$306=$A50)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D50" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$300,$A50,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$306,$A50,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38410,15 +39132,15 @@
         </is>
       </c>
       <c r="B55" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A55)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A55)</f>
         <v/>
       </c>
       <c r="C55" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A55)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A55)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D55" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A55,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A55,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38429,15 +39151,15 @@
         </is>
       </c>
       <c r="B56" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A56)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A56)</f>
         <v/>
       </c>
       <c r="C56" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A56)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A56)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D56" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A56,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A56,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38448,15 +39170,15 @@
         </is>
       </c>
       <c r="B57" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A57)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A57)</f>
         <v/>
       </c>
       <c r="C57" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A57)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A57)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D57" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A57,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A57,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38467,15 +39189,15 @@
         </is>
       </c>
       <c r="B58" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A58)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A58)</f>
         <v/>
       </c>
       <c r="C58" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A58)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A58)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D58" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A58,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A58,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38486,15 +39208,15 @@
         </is>
       </c>
       <c r="B59" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A59)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A59)</f>
         <v/>
       </c>
       <c r="C59" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A59)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A59)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D59" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A59,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A59,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38505,15 +39227,15 @@
         </is>
       </c>
       <c r="B60" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A60)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A60)</f>
         <v/>
       </c>
       <c r="C60" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A60)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A60)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D60" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A60,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A60,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38524,15 +39246,15 @@
         </is>
       </c>
       <c r="B61" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A61)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A61)</f>
         <v/>
       </c>
       <c r="C61" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A61)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A61)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D61" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A61,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A61,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38543,15 +39265,15 @@
         </is>
       </c>
       <c r="B62" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A62)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A62)</f>
         <v/>
       </c>
       <c r="C62" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A62)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A62)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D62" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A62,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A62,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38562,15 +39284,15 @@
         </is>
       </c>
       <c r="B63" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A63)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A63)</f>
         <v/>
       </c>
       <c r="C63" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A63)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A63)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D63" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A63,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A63,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38581,15 +39303,15 @@
         </is>
       </c>
       <c r="B64" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A64)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A64)</f>
         <v/>
       </c>
       <c r="C64" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A64)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A64)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D64" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A64,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A64,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38600,15 +39322,15 @@
         </is>
       </c>
       <c r="B65" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A65)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A65)</f>
         <v/>
       </c>
       <c r="C65" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A65)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A65)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D65" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A65,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A65,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38619,15 +39341,15 @@
         </is>
       </c>
       <c r="B66" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A66)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A66)</f>
         <v/>
       </c>
       <c r="C66" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A66)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A66)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D66" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A66,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A66,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38638,15 +39360,15 @@
         </is>
       </c>
       <c r="B67" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A67)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A67)</f>
         <v/>
       </c>
       <c r="C67" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A67)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A67)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D67" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A67,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A67,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38657,15 +39379,15 @@
         </is>
       </c>
       <c r="B68" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A68)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A68)</f>
         <v/>
       </c>
       <c r="C68" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A68)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A68)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D68" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A68,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A68,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38676,15 +39398,15 @@
         </is>
       </c>
       <c r="B69" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A69)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A69)</f>
         <v/>
       </c>
       <c r="C69" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A69)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A69)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D69" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A69,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A69,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38695,15 +39417,15 @@
         </is>
       </c>
       <c r="B70" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A70)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A70)</f>
         <v/>
       </c>
       <c r="C70" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A70)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A70)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D70" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A70,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A70,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38714,15 +39436,15 @@
         </is>
       </c>
       <c r="B71" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A71)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A71)</f>
         <v/>
       </c>
       <c r="C71" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A71)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A71)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D71" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A71,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A71,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38733,15 +39455,15 @@
         </is>
       </c>
       <c r="B72" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A72)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A72)</f>
         <v/>
       </c>
       <c r="C72" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A72)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A72)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D72" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A72,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A72,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38752,15 +39474,15 @@
         </is>
       </c>
       <c r="B73" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A73)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A73)</f>
         <v/>
       </c>
       <c r="C73" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A73)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A73)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D73" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A73,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A73,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38771,15 +39493,15 @@
         </is>
       </c>
       <c r="B74" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A74)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A74)</f>
         <v/>
       </c>
       <c r="C74" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A74)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A74)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D74" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A74,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A74,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38790,15 +39512,15 @@
         </is>
       </c>
       <c r="B75" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A75)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A75)</f>
         <v/>
       </c>
       <c r="C75" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A75)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A75)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D75" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A75,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A75,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38809,15 +39531,15 @@
         </is>
       </c>
       <c r="B76" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A76)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A76)</f>
         <v/>
       </c>
       <c r="C76" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A76)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A76)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D76" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A76,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A76,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38828,15 +39550,15 @@
         </is>
       </c>
       <c r="B77" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A77)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A77)</f>
         <v/>
       </c>
       <c r="C77" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A77)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A77)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D77" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A77,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A77,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38847,15 +39569,15 @@
         </is>
       </c>
       <c r="B78" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A78)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A78)</f>
         <v/>
       </c>
       <c r="C78" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A78)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A78)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D78" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A78,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A78,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38866,15 +39588,15 @@
         </is>
       </c>
       <c r="B79" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A79)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A79)</f>
         <v/>
       </c>
       <c r="C79" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A79)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A79)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D79" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A79,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A79,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38885,15 +39607,15 @@
         </is>
       </c>
       <c r="B80" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A80)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A80)</f>
         <v/>
       </c>
       <c r="C80" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A80)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A80)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D80" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A80,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A80,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38904,15 +39626,15 @@
         </is>
       </c>
       <c r="B81" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A81)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A81)</f>
         <v/>
       </c>
       <c r="C81" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A81)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A81)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D81" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A81,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A81,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38923,15 +39645,15 @@
         </is>
       </c>
       <c r="B82" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$300,$A82)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A82)</f>
         <v/>
       </c>
       <c r="C82" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$300=$A82)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A82)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
       <c r="D82" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$300,$A82,Artikelstamm!$U$3:$U$300)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A82,Artikelstamm!$U$3:$U$306)</f>
         <v/>
       </c>
     </row>
@@ -38985,11 +39707,11 @@
         </is>
       </c>
       <c r="B87" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$300,$A87)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$306,$A87)</f>
         <v/>
       </c>
       <c r="C87" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$300=$A87)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$306=$A87)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
     </row>
@@ -39000,11 +39722,11 @@
         </is>
       </c>
       <c r="B88" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$300,$A88)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$306,$A88)</f>
         <v/>
       </c>
       <c r="C88" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$300=$A88)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$306=$A88)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
     </row>
@@ -39015,11 +39737,11 @@
         </is>
       </c>
       <c r="B89" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$300,$A89)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$306,$A89)</f>
         <v/>
       </c>
       <c r="C89" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$300=$A89)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$306=$A89)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
     </row>
@@ -39030,11 +39752,11 @@
         </is>
       </c>
       <c r="B90" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$300,$A90)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$306,$A90)</f>
         <v/>
       </c>
       <c r="C90" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$300=$A90)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$306=$A90)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
     </row>
@@ -39045,11 +39767,11 @@
         </is>
       </c>
       <c r="B91" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$300,$A91)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$306,$A91)</f>
         <v/>
       </c>
       <c r="C91" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$300=$A91)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$306=$A91)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
     </row>
@@ -39060,11 +39782,11 @@
         </is>
       </c>
       <c r="B92" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$300,$A92)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$306,$A92)</f>
         <v/>
       </c>
       <c r="C92" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$300=$A92)*Artikelstamm!$K$3:$K$300*Artikelstamm!$AE$3:$AE$300)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$306=$A92)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
BU02 Flur 2 erfasst: 14 neue Positionen, 5 Zusammenfassungen
Raum BU02 (Bestandsgebäude UG, Flur 2, 8,61 m²) aus 22 Fotos und dem
Erfassungsblatt aufgenommen. 19 Post-it-Nummern ergeben 14 neue Positionen;
fünf Nummern gehen in bestehende Positionen anderer Räume ein, damit die
Käufer die Gesamtstückzahl sehen:

  BU02-04 -> NU02-02  Kritter-Stühle          16 -> 31
  BU02-07 -> NU04-09  Regal 8 Fächer          10 -> 12
  BU02-08 -> BA08-12  Wandregalbrett weiß      2 -> 4
  BU02-11 -> NU04-10  Schalenstuhl mit Polster 4 -> 10
  BU02-13 -> BU01-06  Wanddeko Lama            2 -> 3

Foto F-376 maskiert: Vornamen auf den Magnetschildern und beschriftete
Anhänger an der Hakenleiste.

Datenbasis 318 Positionen / 262 aktiv, pruefen.py 0 Fehler.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011yyfqhuiWGsaNy38oaNoGo
</commit_message>
<xml_diff>
--- a/ausgabe/01_Artikelstamm_kikripp.xlsx
+++ b/ausgabe/01_Artikelstamm_kikripp.xlsx
@@ -15,7 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Artikelstamm'!$A$2:$AN$306</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Artikelstamm'!$A$2:$AN$320</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1019,7 +1019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN306"/>
+  <dimension ref="A1:AN320"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -20090,7 +20090,7 @@
       <c r="B156" s="15" t="n"/>
       <c r="C156" s="15" t="inlineStr">
         <is>
-          <t>NU04-12</t>
+          <t>NU04-12, BU02-04</t>
         </is>
       </c>
       <c r="D156" s="15" t="inlineStr">
@@ -20124,7 +20124,7 @@
         </is>
       </c>
       <c r="J156" s="17" t="n">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="K156" s="17" t="n"/>
       <c r="L156" s="18">
@@ -20203,12 +20203,12 @@
       <c r="AL156" s="19" t="n"/>
       <c r="AM156" s="16" t="inlineStr">
         <is>
-          <t>16 Stühle insgesamt: 10 im Gruppenraum 5 und im Nachbarraum NU03, 6 im Schlafraum 5 (dort mit NU04-12 beschriftet).</t>
+          <t>31 Stühle insgesamt: 10 im Gruppenraum 5 und im Nachbarraum NU03, 6 im Schlafraum 5 (dort mit NU04-12 beschriftet) und 15 im Flur 2 im Untergeschoss des Bestandsgebäudes (dort mit BU02-04 beschriftet). Die 15 Stühle aus dem Flur 2 sind stark gebraucht.</t>
         </is>
       </c>
       <c r="AN156" s="22" t="inlineStr">
         <is>
-          <t>Zusammengefasste Position ueber drei Raeume. Post-it-Nummer im Schlafraum 5: NU04-12. In NU03 nicht erneut anlegen.</t>
+          <t>Zusammengefasste Position ueber vier Raeume. Post-it-Nummern: NU04-12, BU02-04. In NU03 nicht erneut anlegen.</t>
         </is>
       </c>
     </row>
@@ -23982,7 +23982,7 @@
       <c r="B188" s="15" t="n"/>
       <c r="C188" s="15" t="inlineStr">
         <is>
-          <t>NU05-05, NU07-06, BA04-03, BU01-03</t>
+          <t>NU05-05, NU07-06, BA04-03, BU01-03, BU02-07</t>
         </is>
       </c>
       <c r="D188" s="15" t="inlineStr">
@@ -24016,7 +24016,7 @@
         </is>
       </c>
       <c r="J188" s="17" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="K188" s="17" t="n"/>
       <c r="L188" s="18">
@@ -24095,12 +24095,12 @@
       <c r="AL188" s="19" t="n"/>
       <c r="AM188" s="16" t="inlineStr">
         <is>
-          <t>10 Regale insgesamt: 3 im Schlafraum 5, 1 im Treppenraum 1 (NU05-05), 1 in der Garage (NU07-06), 3 im Gruppenraum 4 (BA04-03) und 2 im Flur 1 des Bestandsgebäudes (BU01-03).</t>
+          <t>12 Regale insgesamt: 3 im Schlafraum 5, 1 im Treppenraum 1 (NU05-05), 1 in der Garage (NU07-06), 3 im Gruppenraum 4 (BA04-03), 2 im Flur 1 des Bestandsgebäudes (BU01-03) und 2 im Flur 2 im Untergeschoss (BU02-07).</t>
         </is>
       </c>
       <c r="AN188" s="22" t="inlineStr">
         <is>
-          <t>Zusammengefasste Position über fünf Räume – Post-it-Nummern: NU05-05, NU07-06, BA04-03, BU01-03.</t>
+          <t>Zusammengefasste Position über sechs Räume – Post-it-Nummern: NU05-05, NU07-06, BA04-03, BU01-03, BU02-07.</t>
         </is>
       </c>
     </row>
@@ -24111,7 +24111,11 @@
         </is>
       </c>
       <c r="B189" s="15" t="n"/>
-      <c r="C189" s="15" t="n"/>
+      <c r="C189" s="15" t="inlineStr">
+        <is>
+          <t>BU02-11</t>
+        </is>
+      </c>
       <c r="D189" s="15" t="inlineStr">
         <is>
           <t>NU04</t>
@@ -24143,7 +24147,7 @@
         </is>
       </c>
       <c r="J189" s="17" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="K189" s="17" t="n"/>
       <c r="L189" s="18">
@@ -24218,10 +24222,14 @@
       <c r="AL189" s="19" t="n"/>
       <c r="AM189" s="16" t="inlineStr">
         <is>
-          <t>4 Stühle – abgebildet ist einer davon.</t>
-        </is>
-      </c>
-      <c r="AN189" s="22" t="n"/>
+          <t>10 Stühle insgesamt: 4 im Schlafraum 5 (NU04-10) und 6 im Flur 2 im Untergeschoss des Bestandsgebäudes (BU02-11). Abgebildet ist einer davon.</t>
+        </is>
+      </c>
+      <c r="AN189" s="22" t="inlineStr">
+        <is>
+          <t>Zusammengefasste Position über zwei Räume – Post-it-Nummer: BU02-11.</t>
+        </is>
+      </c>
     </row>
     <row r="190" ht="30" customHeight="1">
       <c r="A190" s="15" t="inlineStr">
@@ -37520,7 +37528,11 @@
         </is>
       </c>
       <c r="B300" s="15" t="n"/>
-      <c r="C300" s="15" t="n"/>
+      <c r="C300" s="15" t="inlineStr">
+        <is>
+          <t>BU02-08</t>
+        </is>
+      </c>
       <c r="D300" s="15" t="inlineStr">
         <is>
           <t>BA08</t>
@@ -37552,7 +37564,7 @@
         </is>
       </c>
       <c r="J300" s="17" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K300" s="17" t="n"/>
       <c r="L300" s="18">
@@ -37627,10 +37639,14 @@
       <c r="AL300" s="19" t="n"/>
       <c r="AM300" s="16" t="inlineStr">
         <is>
-          <t>2 Bretter. Die blauen Becher darauf gehören nicht dazu.</t>
-        </is>
-      </c>
-      <c r="AN300" s="22" t="n"/>
+          <t>4 Bretter insgesamt: 2 im Atelier (BA08-12) und 2 im Flur 2 im Untergeschoss des Bestandsgebäudes (BU02-08). Die blauen Becher auf dem Foto gehören nicht dazu.</t>
+        </is>
+      </c>
+      <c r="AN300" s="22" t="inlineStr">
+        <is>
+          <t>Zusammengefasste Position über zwei Räume – Post-it-Nummer: BU02-08.</t>
+        </is>
+      </c>
     </row>
     <row r="301" ht="30" customHeight="1">
       <c r="A301" s="15" t="inlineStr">
@@ -37865,7 +37881,7 @@
       <c r="AL302" s="19" t="n"/>
       <c r="AM302" s="16" t="inlineStr">
         <is>
-          <t>1 Küche. Spielgeschirr und Zubehör gehören nicht dazu. Drei größere Spielküchen stehen unter NU03-03, NU07-03 und BA03-02.</t>
+          <t>1 Küche. Spielgeschirr und Zubehör gehören nicht dazu. Weitere Spielküchen stehen unter NU03-03, NU07-03, BA03-02 und BU02-05.</t>
         </is>
       </c>
       <c r="AN302" s="22" t="n"/>
@@ -38119,7 +38135,11 @@
         </is>
       </c>
       <c r="B305" s="15" t="n"/>
-      <c r="C305" s="15" t="n"/>
+      <c r="C305" s="15" t="inlineStr">
+        <is>
+          <t>BU02-13</t>
+        </is>
+      </c>
       <c r="D305" s="15" t="inlineStr">
         <is>
           <t>BU01</t>
@@ -38151,7 +38171,7 @@
         </is>
       </c>
       <c r="J305" s="17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K305" s="17" t="n"/>
       <c r="L305" s="18">
@@ -38226,10 +38246,14 @@
       <c r="AL305" s="19" t="n"/>
       <c r="AM305" s="16" t="inlineStr">
         <is>
-          <t>2 Stück – abgebildet ist eines davon.</t>
-        </is>
-      </c>
-      <c r="AN305" s="22" t="n"/>
+          <t>3 Stück insgesamt: 2 im Flur 1 (BU01-06) und 1 im Flur 2 (BU02-13), beide im Untergeschoss des Bestandsgebäudes. Abgebildet ist eines davon.</t>
+        </is>
+      </c>
+      <c r="AN305" s="22" t="inlineStr">
+        <is>
+          <t>Zusammengefasste Position über zwei Räume – Post-it-Nummer: BU02-13.</t>
+        </is>
+      </c>
     </row>
     <row r="306" ht="30" customHeight="1">
       <c r="A306" s="15" t="inlineStr">
@@ -38354,8 +38378,1690 @@
       </c>
       <c r="AN306" s="22" t="n"/>
     </row>
+    <row r="307" ht="30" customHeight="1">
+      <c r="A307" s="15" t="inlineStr">
+        <is>
+          <t>BU02-01</t>
+        </is>
+      </c>
+      <c r="B307" s="15" t="n"/>
+      <c r="C307" s="15" t="n"/>
+      <c r="D307" s="15" t="inlineStr">
+        <is>
+          <t>BU02</t>
+        </is>
+      </c>
+      <c r="E307" s="15" t="inlineStr">
+        <is>
+          <t>Hausbett Holz natur mit Stoffdach</t>
+        </is>
+      </c>
+      <c r="F307" s="16" t="inlineStr">
+        <is>
+          <t>Bodenbett in Hausform aus hellem Massivholz mit vier Pfosten und aufgelegtem Stoffdach in Creme mit schwarzer Zackenkante und aufgesticktem Wolkenmotiv. Einschließlich Matratze.</t>
+        </is>
+      </c>
+      <c r="G307" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H307" s="15" t="inlineStr">
+        <is>
+          <t>Flur 2</t>
+        </is>
+      </c>
+      <c r="I307" s="15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J307" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K307" s="17" t="n"/>
+      <c r="L307" s="18">
+        <f>J307-IF(K307="",0,K307)</f>
+        <v/>
+      </c>
+      <c r="M307" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N307" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O307" s="19" t="n"/>
+      <c r="P307" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q307" s="19" t="n"/>
+      <c r="R307" s="20" t="n"/>
+      <c r="S307" s="20" t="n">
+        <v>180</v>
+      </c>
+      <c r="T307" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U307" s="21">
+        <f>L307*S307</f>
+        <v/>
+      </c>
+      <c r="V307" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W307" s="15" t="inlineStr">
+        <is>
+          <t>F-365</t>
+        </is>
+      </c>
+      <c r="X307" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y307" s="19" t="n"/>
+      <c r="Z307" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA307" s="19" t="n"/>
+      <c r="AB307" s="19" t="n"/>
+      <c r="AC307" s="19" t="n"/>
+      <c r="AD307" s="19" t="n"/>
+      <c r="AE307" s="20" t="n"/>
+      <c r="AF307" s="21">
+        <f>IF(K307="","",K307*AE307)</f>
+        <v/>
+      </c>
+      <c r="AG307" s="19" t="n"/>
+      <c r="AH307" s="19" t="n"/>
+      <c r="AI307" s="19" t="n"/>
+      <c r="AJ307" s="19" t="n"/>
+      <c r="AK307" s="19" t="n"/>
+      <c r="AL307" s="19" t="n"/>
+      <c r="AM307" s="16" t="inlineStr">
+        <is>
+          <t>1 Bett mit Stoffdach und Matratze. Kissen, Decke und Puppe gehören nicht dazu. Weitere Hausbetten stehen unter BU01-01 und NU07-01.</t>
+        </is>
+      </c>
+      <c r="AN307" s="22" t="n"/>
+    </row>
+    <row r="308" ht="30" customHeight="1">
+      <c r="A308" s="15" t="inlineStr">
+        <is>
+          <t>BU02-02</t>
+        </is>
+      </c>
+      <c r="B308" s="15" t="n"/>
+      <c r="C308" s="15" t="n"/>
+      <c r="D308" s="15" t="inlineStr">
+        <is>
+          <t>BU02</t>
+        </is>
+      </c>
+      <c r="E308" s="15" t="inlineStr">
+        <is>
+          <t>Nachtlicht Marienkäfer, schwarz</t>
+        </is>
+      </c>
+      <c r="F308" s="16" t="inlineStr">
+        <is>
+          <t>Steckdosen-Nachtlicht in Marienkäferform aus schwarzem Kunststoff mit geprägten Punkten und Fühlern.</t>
+        </is>
+      </c>
+      <c r="G308" s="15" t="inlineStr">
+        <is>
+          <t>Leuchten</t>
+        </is>
+      </c>
+      <c r="H308" s="15" t="inlineStr">
+        <is>
+          <t>Flur 2</t>
+        </is>
+      </c>
+      <c r="I308" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J308" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K308" s="17" t="n"/>
+      <c r="L308" s="18">
+        <f>J308-IF(K308="",0,K308)</f>
+        <v/>
+      </c>
+      <c r="M308" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N308" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O308" s="19" t="n"/>
+      <c r="P308" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q308" s="19" t="n"/>
+      <c r="R308" s="20" t="n"/>
+      <c r="S308" s="20" t="n">
+        <v>15</v>
+      </c>
+      <c r="T308" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U308" s="21">
+        <f>L308*S308</f>
+        <v/>
+      </c>
+      <c r="V308" s="15" t="inlineStr">
+        <is>
+          <t>Versand möglich</t>
+        </is>
+      </c>
+      <c r="W308" s="15" t="inlineStr">
+        <is>
+          <t>F-366</t>
+        </is>
+      </c>
+      <c r="X308" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y308" s="19" t="n"/>
+      <c r="Z308" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA308" s="19" t="n"/>
+      <c r="AB308" s="19" t="n"/>
+      <c r="AC308" s="19" t="n"/>
+      <c r="AD308" s="19" t="n"/>
+      <c r="AE308" s="20" t="n"/>
+      <c r="AF308" s="21">
+        <f>IF(K308="","",K308*AE308)</f>
+        <v/>
+      </c>
+      <c r="AG308" s="19" t="n"/>
+      <c r="AH308" s="19" t="n"/>
+      <c r="AI308" s="19" t="n"/>
+      <c r="AJ308" s="19" t="n"/>
+      <c r="AK308" s="19" t="n"/>
+      <c r="AL308" s="19" t="n"/>
+      <c r="AM308" s="16" t="inlineStr">
+        <is>
+          <t>2 Stück – abgebildet ist eines davon.</t>
+        </is>
+      </c>
+      <c r="AN308" s="22" t="n"/>
+    </row>
+    <row r="309" ht="30" customHeight="1">
+      <c r="A309" s="15" t="inlineStr">
+        <is>
+          <t>BU02-03</t>
+        </is>
+      </c>
+      <c r="B309" s="15" t="n"/>
+      <c r="C309" s="15" t="n"/>
+      <c r="D309" s="15" t="inlineStr">
+        <is>
+          <t>BU02</t>
+        </is>
+      </c>
+      <c r="E309" s="15" t="inlineStr">
+        <is>
+          <t>Kindertisch weiß, oval, aus vier Segmenten</t>
+        </is>
+      </c>
+      <c r="F309" s="16" t="inlineStr">
+        <is>
+          <t>Vier Tischsegmente mit weißer Platte und Multiplex-Kante auf verchromten Rundfüßen in Kinderhöhe: zwei halbrunde Endstücke und zwei Mittelstücke. Zusammengestellt ergeben sie einen großen ovalen Gruppentisch, einzeln sind sie frei kombinierbar.</t>
+        </is>
+      </c>
+      <c r="G309" s="15" t="inlineStr">
+        <is>
+          <t>Möbel</t>
+        </is>
+      </c>
+      <c r="H309" s="15" t="inlineStr">
+        <is>
+          <t>Flur 2</t>
+        </is>
+      </c>
+      <c r="I309" s="15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J309" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K309" s="17" t="n"/>
+      <c r="L309" s="18">
+        <f>J309-IF(K309="",0,K309)</f>
+        <v/>
+      </c>
+      <c r="M309" s="15" t="inlineStr">
+        <is>
+          <t>Set</t>
+        </is>
+      </c>
+      <c r="N309" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O309" s="19" t="n"/>
+      <c r="P309" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q309" s="19" t="n"/>
+      <c r="R309" s="20" t="n"/>
+      <c r="S309" s="20" t="n">
+        <v>160</v>
+      </c>
+      <c r="T309" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U309" s="21">
+        <f>L309*S309</f>
+        <v/>
+      </c>
+      <c r="V309" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W309" s="15" t="inlineStr">
+        <is>
+          <t>F-367</t>
+        </is>
+      </c>
+      <c r="X309" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y309" s="19" t="n"/>
+      <c r="Z309" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA309" s="19" t="n"/>
+      <c r="AB309" s="19" t="n"/>
+      <c r="AC309" s="19" t="n"/>
+      <c r="AD309" s="19" t="n"/>
+      <c r="AE309" s="20" t="n"/>
+      <c r="AF309" s="21">
+        <f>IF(K309="","",K309*AE309)</f>
+        <v/>
+      </c>
+      <c r="AG309" s="19" t="n"/>
+      <c r="AH309" s="19" t="n"/>
+      <c r="AI309" s="19" t="n"/>
+      <c r="AJ309" s="19" t="n"/>
+      <c r="AK309" s="19" t="n"/>
+      <c r="AL309" s="19" t="n"/>
+      <c r="AM309" s="16" t="inlineStr">
+        <is>
+          <t>1 Tischgruppe aus vier Segmenten. Eine zweite Tischgruppe in Sechseckform steht unter NU02-23.</t>
+        </is>
+      </c>
+      <c r="AN309" s="22" t="n"/>
+    </row>
+    <row r="310" ht="30" customHeight="1">
+      <c r="A310" s="15" t="inlineStr">
+        <is>
+          <t>BU02-05</t>
+        </is>
+      </c>
+      <c r="B310" s="15" t="n"/>
+      <c r="C310" s="15" t="n"/>
+      <c r="D310" s="15" t="inlineStr">
+        <is>
+          <t>BU02</t>
+        </is>
+      </c>
+      <c r="E310" s="15" t="inlineStr">
+        <is>
+          <t>IKEA Duktig Spielküche mit Mikrowelle</t>
+        </is>
+      </c>
+      <c r="F310" s="16" t="inlineStr">
+        <is>
+          <t>Spielküche von IKEA aus Birkenholz mit weißen Fronten: Aufsatz mit Mikrowelle und offenen Fächern, Arbeitsplatte mit Kochfeld, Spülbecken und Wasserhahn, darunter Backofen mit Sichtfenster und ein Schrank.</t>
+        </is>
+      </c>
+      <c r="G310" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H310" s="15" t="inlineStr">
+        <is>
+          <t>Flur 2</t>
+        </is>
+      </c>
+      <c r="I310" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J310" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K310" s="17" t="n"/>
+      <c r="L310" s="18">
+        <f>J310-IF(K310="",0,K310)</f>
+        <v/>
+      </c>
+      <c r="M310" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N310" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O310" s="19" t="n"/>
+      <c r="P310" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q310" s="19" t="n"/>
+      <c r="R310" s="20" t="n"/>
+      <c r="S310" s="20" t="n">
+        <v>60</v>
+      </c>
+      <c r="T310" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U310" s="21">
+        <f>L310*S310</f>
+        <v/>
+      </c>
+      <c r="V310" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W310" s="15" t="inlineStr">
+        <is>
+          <t>F-369</t>
+        </is>
+      </c>
+      <c r="X310" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y310" s="19" t="n"/>
+      <c r="Z310" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA310" s="19" t="inlineStr">
+        <is>
+          <t>IKEA</t>
+        </is>
+      </c>
+      <c r="AB310" s="19" t="n"/>
+      <c r="AC310" s="19" t="n"/>
+      <c r="AD310" s="19" t="n"/>
+      <c r="AE310" s="20" t="n"/>
+      <c r="AF310" s="21">
+        <f>IF(K310="","",K310*AE310)</f>
+        <v/>
+      </c>
+      <c r="AG310" s="19" t="n"/>
+      <c r="AH310" s="19" t="n"/>
+      <c r="AI310" s="19" t="n"/>
+      <c r="AJ310" s="19" t="n"/>
+      <c r="AK310" s="19" t="n"/>
+      <c r="AL310" s="19" t="n"/>
+      <c r="AM310" s="16" t="inlineStr">
+        <is>
+          <t>1 Küche. Spielgeschirr, Vorratsgläser und Zubehör gehören nicht dazu. Weitere Spielküchen stehen unter NU03-03, NU07-03, BA03-02 und BU01-02.</t>
+        </is>
+      </c>
+      <c r="AN310" s="22" t="n"/>
+    </row>
+    <row r="311" ht="30" customHeight="1">
+      <c r="A311" s="15" t="inlineStr">
+        <is>
+          <t>BU02-06</t>
+        </is>
+      </c>
+      <c r="B311" s="15" t="n"/>
+      <c r="C311" s="15" t="n"/>
+      <c r="D311" s="15" t="inlineStr">
+        <is>
+          <t>BU02</t>
+        </is>
+      </c>
+      <c r="E311" s="15" t="inlineStr">
+        <is>
+          <t>Kinder-Putzständer, fünfteilig</t>
+        </is>
+      </c>
+      <c r="F311" s="16" t="inlineStr">
+        <is>
+          <t>Ständer aus Holz und Metall in Weiß mit Ablagekasten und aufgehängtem Kinder-Reinigungsgerät: Besen, Schrubber, Kehrblech und Staubwedel.</t>
+        </is>
+      </c>
+      <c r="G311" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H311" s="15" t="inlineStr">
+        <is>
+          <t>Flur 2</t>
+        </is>
+      </c>
+      <c r="I311" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J311" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K311" s="17" t="n"/>
+      <c r="L311" s="18">
+        <f>J311-IF(K311="",0,K311)</f>
+        <v/>
+      </c>
+      <c r="M311" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N311" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O311" s="19" t="n"/>
+      <c r="P311" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q311" s="19" t="n"/>
+      <c r="R311" s="20" t="n"/>
+      <c r="S311" s="20" t="n">
+        <v>25</v>
+      </c>
+      <c r="T311" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U311" s="21">
+        <f>L311*S311</f>
+        <v/>
+      </c>
+      <c r="V311" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W311" s="15" t="inlineStr">
+        <is>
+          <t>F-370</t>
+        </is>
+      </c>
+      <c r="X311" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y311" s="19" t="n"/>
+      <c r="Z311" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA311" s="19" t="n"/>
+      <c r="AB311" s="19" t="n"/>
+      <c r="AC311" s="19" t="n"/>
+      <c r="AD311" s="19" t="n"/>
+      <c r="AE311" s="20" t="n"/>
+      <c r="AF311" s="21">
+        <f>IF(K311="","",K311*AE311)</f>
+        <v/>
+      </c>
+      <c r="AG311" s="19" t="n"/>
+      <c r="AH311" s="19" t="n"/>
+      <c r="AI311" s="19" t="n"/>
+      <c r="AJ311" s="19" t="n"/>
+      <c r="AK311" s="19" t="n"/>
+      <c r="AL311" s="19" t="n"/>
+      <c r="AM311" s="16" t="inlineStr">
+        <is>
+          <t>1 Ständer mit fünf Teilen.</t>
+        </is>
+      </c>
+      <c r="AN311" s="22" t="n"/>
+    </row>
+    <row r="312" ht="30" customHeight="1">
+      <c r="A312" s="15" t="inlineStr">
+        <is>
+          <t>BU02-09</t>
+        </is>
+      </c>
+      <c r="B312" s="15" t="n"/>
+      <c r="C312" s="15" t="n"/>
+      <c r="D312" s="15" t="inlineStr">
+        <is>
+          <t>BU02</t>
+        </is>
+      </c>
+      <c r="E312" s="15" t="inlineStr">
+        <is>
+          <t>Acrylbild Herz auf Strahlenkranz</t>
+        </is>
+      </c>
+      <c r="F312" s="16" t="inlineStr">
+        <is>
+          <t>Acryl auf Leinwand im Hochformat: breite Pinselstriche in Pink, Magenta und Grau strahlenförmig um ein ausgespartes weißes Herz. Eigenarbeit einer Privatperson, nicht signiert.</t>
+        </is>
+      </c>
+      <c r="G312" s="15" t="inlineStr">
+        <is>
+          <t>Kunst</t>
+        </is>
+      </c>
+      <c r="H312" s="15" t="inlineStr">
+        <is>
+          <t>Flur 2</t>
+        </is>
+      </c>
+      <c r="I312" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J312" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K312" s="17" t="n"/>
+      <c r="L312" s="18">
+        <f>J312-IF(K312="",0,K312)</f>
+        <v/>
+      </c>
+      <c r="M312" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N312" s="15" t="inlineStr">
+        <is>
+          <t>gut</t>
+        </is>
+      </c>
+      <c r="O312" s="19" t="n"/>
+      <c r="P312" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q312" s="19" t="n"/>
+      <c r="R312" s="20" t="n"/>
+      <c r="S312" s="20" t="n">
+        <v>80</v>
+      </c>
+      <c r="T312" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U312" s="21">
+        <f>L312*S312</f>
+        <v/>
+      </c>
+      <c r="V312" s="15" t="inlineStr">
+        <is>
+          <t>Versand möglich</t>
+        </is>
+      </c>
+      <c r="W312" s="15" t="inlineStr">
+        <is>
+          <t>F-373</t>
+        </is>
+      </c>
+      <c r="X312" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y312" s="19" t="n"/>
+      <c r="Z312" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA312" s="19" t="n"/>
+      <c r="AB312" s="19" t="n"/>
+      <c r="AC312" s="19" t="n"/>
+      <c r="AD312" s="19" t="n"/>
+      <c r="AE312" s="20" t="n"/>
+      <c r="AF312" s="21">
+        <f>IF(K312="","",K312*AE312)</f>
+        <v/>
+      </c>
+      <c r="AG312" s="19" t="n"/>
+      <c r="AH312" s="19" t="n"/>
+      <c r="AI312" s="19" t="n"/>
+      <c r="AJ312" s="19" t="n"/>
+      <c r="AK312" s="19" t="n"/>
+      <c r="AL312" s="19" t="n"/>
+      <c r="AM312" s="16" t="inlineStr">
+        <is>
+          <t>1 Bild auf Keilrahmen, ungerahmt.</t>
+        </is>
+      </c>
+      <c r="AN312" s="22" t="n"/>
+    </row>
+    <row r="313" ht="30" customHeight="1">
+      <c r="A313" s="15" t="inlineStr">
+        <is>
+          <t>BU02-10</t>
+        </is>
+      </c>
+      <c r="B313" s="15" t="n"/>
+      <c r="C313" s="15" t="n"/>
+      <c r="D313" s="15" t="inlineStr">
+        <is>
+          <t>BU02</t>
+        </is>
+      </c>
+      <c r="E313" s="15" t="inlineStr">
+        <is>
+          <t>Spieltisch Kiefer mit herausnehmbaren Platten</t>
+        </is>
+      </c>
+      <c r="F313" s="16" t="inlineStr">
+        <is>
+          <t>Kindertisch aus Kiefer massiv mit zwei herausnehmbaren weißen Platten. Darunter liegen Wannen, sodass der Tisch als Spiel- und Materialtisch genutzt werden kann. Die Platten sind an den Kanten großflächig abgeplatzt.</t>
+        </is>
+      </c>
+      <c r="G313" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H313" s="15" t="inlineStr">
+        <is>
+          <t>Flur 2</t>
+        </is>
+      </c>
+      <c r="I313" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J313" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K313" s="17" t="n"/>
+      <c r="L313" s="18">
+        <f>J313-IF(K313="",0,K313)</f>
+        <v/>
+      </c>
+      <c r="M313" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N313" s="15" t="inlineStr">
+        <is>
+          <t>stark gebraucht</t>
+        </is>
+      </c>
+      <c r="O313" s="19" t="n"/>
+      <c r="P313" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q313" s="19" t="n"/>
+      <c r="R313" s="20" t="n"/>
+      <c r="S313" s="20" t="n">
+        <v>40</v>
+      </c>
+      <c r="T313" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U313" s="21">
+        <f>L313*S313</f>
+        <v/>
+      </c>
+      <c r="V313" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W313" s="15" t="inlineStr">
+        <is>
+          <t>F-374</t>
+        </is>
+      </c>
+      <c r="X313" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y313" s="19" t="n"/>
+      <c r="Z313" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA313" s="19" t="n"/>
+      <c r="AB313" s="19" t="n"/>
+      <c r="AC313" s="19" t="n"/>
+      <c r="AD313" s="19" t="n"/>
+      <c r="AE313" s="20" t="n"/>
+      <c r="AF313" s="21">
+        <f>IF(K313="","",K313*AE313)</f>
+        <v/>
+      </c>
+      <c r="AG313" s="19" t="n"/>
+      <c r="AH313" s="19" t="n"/>
+      <c r="AI313" s="19" t="n"/>
+      <c r="AJ313" s="19" t="n"/>
+      <c r="AK313" s="19" t="n"/>
+      <c r="AL313" s="19" t="n"/>
+      <c r="AM313" s="16" t="inlineStr">
+        <is>
+          <t>2 Tische einschließlich der Platten und Wannen – abgebildet ist einer davon. Der Inhalt gehört nicht dazu.</t>
+        </is>
+      </c>
+      <c r="AN313" s="22" t="n"/>
+    </row>
+    <row r="314" ht="30" customHeight="1">
+      <c r="A314" s="15" t="inlineStr">
+        <is>
+          <t>BU02-12</t>
+        </is>
+      </c>
+      <c r="B314" s="15" t="n"/>
+      <c r="C314" s="15" t="n"/>
+      <c r="D314" s="15" t="inlineStr">
+        <is>
+          <t>BU02</t>
+        </is>
+      </c>
+      <c r="E314" s="15" t="inlineStr">
+        <is>
+          <t>Wandregal weiß mit drei Wannen, geschwungen</t>
+        </is>
+      </c>
+      <c r="F314" s="16" t="inlineStr">
+        <is>
+          <t>Weißes Wandelement mit geschwungener Front, drei Fächern und drei eingeschobenen Kunststoffwannen.</t>
+        </is>
+      </c>
+      <c r="G314" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H314" s="15" t="inlineStr">
+        <is>
+          <t>Flur 2</t>
+        </is>
+      </c>
+      <c r="I314" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J314" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K314" s="17" t="n"/>
+      <c r="L314" s="18">
+        <f>J314-IF(K314="",0,K314)</f>
+        <v/>
+      </c>
+      <c r="M314" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N314" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O314" s="19" t="n"/>
+      <c r="P314" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q314" s="19" t="n"/>
+      <c r="R314" s="20" t="n"/>
+      <c r="S314" s="20" t="n">
+        <v>35</v>
+      </c>
+      <c r="T314" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U314" s="21">
+        <f>L314*S314</f>
+        <v/>
+      </c>
+      <c r="V314" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W314" s="15" t="inlineStr">
+        <is>
+          <t>F-376</t>
+        </is>
+      </c>
+      <c r="X314" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y314" s="19" t="n"/>
+      <c r="Z314" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA314" s="19" t="n"/>
+      <c r="AB314" s="19" t="n"/>
+      <c r="AC314" s="19" t="n"/>
+      <c r="AD314" s="19" t="n"/>
+      <c r="AE314" s="20" t="n"/>
+      <c r="AF314" s="21">
+        <f>IF(K314="","",K314*AE314)</f>
+        <v/>
+      </c>
+      <c r="AG314" s="19" t="n"/>
+      <c r="AH314" s="19" t="n"/>
+      <c r="AI314" s="19" t="n"/>
+      <c r="AJ314" s="19" t="n"/>
+      <c r="AK314" s="19" t="n"/>
+      <c r="AL314" s="19" t="n"/>
+      <c r="AM314" s="16" t="inlineStr">
+        <is>
+          <t>1 Regal einschließlich der Wannen. Gerade Wandregale gleicher Bauart stehen unter NE01-21.</t>
+        </is>
+      </c>
+      <c r="AN314" s="22" t="n"/>
+    </row>
+    <row r="315" ht="30" customHeight="1">
+      <c r="A315" s="15" t="inlineStr">
+        <is>
+          <t>BU02-14</t>
+        </is>
+      </c>
+      <c r="B315" s="15" t="n"/>
+      <c r="C315" s="15" t="n"/>
+      <c r="D315" s="15" t="inlineStr">
+        <is>
+          <t>BU02</t>
+        </is>
+      </c>
+      <c r="E315" s="15" t="inlineStr">
+        <is>
+          <t>Kinderschrank graugrün, zwei Türen</t>
+        </is>
+      </c>
+      <c r="F315" s="16" t="inlineStr">
+        <is>
+          <t>Hoher Kinderschrank von IKEA mit zwei graugrünen Türen und schwarzen Griffmulden, darunter eine Schublade.</t>
+        </is>
+      </c>
+      <c r="G315" s="15" t="inlineStr">
+        <is>
+          <t>Möbel</t>
+        </is>
+      </c>
+      <c r="H315" s="15" t="inlineStr">
+        <is>
+          <t>Flur 2</t>
+        </is>
+      </c>
+      <c r="I315" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J315" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K315" s="17" t="n"/>
+      <c r="L315" s="18">
+        <f>J315-IF(K315="",0,K315)</f>
+        <v/>
+      </c>
+      <c r="M315" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N315" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O315" s="19" t="n"/>
+      <c r="P315" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q315" s="19" t="n"/>
+      <c r="R315" s="20" t="n"/>
+      <c r="S315" s="20" t="n">
+        <v>90</v>
+      </c>
+      <c r="T315" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U315" s="21">
+        <f>L315*S315</f>
+        <v/>
+      </c>
+      <c r="V315" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W315" s="15" t="inlineStr">
+        <is>
+          <t>F-378</t>
+        </is>
+      </c>
+      <c r="X315" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y315" s="19" t="n"/>
+      <c r="Z315" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA315" s="19" t="inlineStr">
+        <is>
+          <t>IKEA</t>
+        </is>
+      </c>
+      <c r="AB315" s="19" t="n"/>
+      <c r="AC315" s="19" t="n"/>
+      <c r="AD315" s="19" t="n"/>
+      <c r="AE315" s="20" t="n"/>
+      <c r="AF315" s="21">
+        <f>IF(K315="","",K315*AE315)</f>
+        <v/>
+      </c>
+      <c r="AG315" s="19" t="n"/>
+      <c r="AH315" s="19" t="n"/>
+      <c r="AI315" s="19" t="n"/>
+      <c r="AJ315" s="19" t="n"/>
+      <c r="AK315" s="19" t="n"/>
+      <c r="AL315" s="19" t="n"/>
+      <c r="AM315" s="16" t="inlineStr">
+        <is>
+          <t>2 Schränke – abgebildet ist einer davon. Baugleiche Schränke mit weißen Türen stehen unter BA02-08.</t>
+        </is>
+      </c>
+      <c r="AN315" s="22" t="n"/>
+    </row>
+    <row r="316" ht="30" customHeight="1">
+      <c r="A316" s="15" t="inlineStr">
+        <is>
+          <t>BU02-15</t>
+        </is>
+      </c>
+      <c r="B316" s="15" t="n"/>
+      <c r="C316" s="15" t="n"/>
+      <c r="D316" s="15" t="inlineStr">
+        <is>
+          <t>BU02</t>
+        </is>
+      </c>
+      <c r="E316" s="15" t="inlineStr">
+        <is>
+          <t>Bodensitzkissen beige, selbststehend</t>
+        </is>
+      </c>
+      <c r="F316" s="16" t="inlineStr">
+        <is>
+          <t>Selbststehendes Bodensitzkissen aus beigem Leinenstoff mit gesteppten Feldern, Rückenlehne und langer Sitzfläche. Die Lehne lässt sich flach ausklappen.</t>
+        </is>
+      </c>
+      <c r="G316" s="15" t="inlineStr">
+        <is>
+          <t>Textilien</t>
+        </is>
+      </c>
+      <c r="H316" s="15" t="inlineStr">
+        <is>
+          <t>Flur 2</t>
+        </is>
+      </c>
+      <c r="I316" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J316" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K316" s="17" t="n"/>
+      <c r="L316" s="18">
+        <f>J316-IF(K316="",0,K316)</f>
+        <v/>
+      </c>
+      <c r="M316" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N316" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O316" s="19" t="n"/>
+      <c r="P316" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q316" s="19" t="n"/>
+      <c r="R316" s="20" t="n"/>
+      <c r="S316" s="20" t="n">
+        <v>25</v>
+      </c>
+      <c r="T316" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U316" s="21">
+        <f>L316*S316</f>
+        <v/>
+      </c>
+      <c r="V316" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W316" s="15" t="inlineStr">
+        <is>
+          <t>F-379</t>
+        </is>
+      </c>
+      <c r="X316" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y316" s="19" t="n"/>
+      <c r="Z316" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA316" s="19" t="n"/>
+      <c r="AB316" s="19" t="n"/>
+      <c r="AC316" s="19" t="n"/>
+      <c r="AD316" s="19" t="n"/>
+      <c r="AE316" s="20" t="n"/>
+      <c r="AF316" s="21">
+        <f>IF(K316="","",K316*AE316)</f>
+        <v/>
+      </c>
+      <c r="AG316" s="19" t="n"/>
+      <c r="AH316" s="19" t="n"/>
+      <c r="AI316" s="19" t="n"/>
+      <c r="AJ316" s="19" t="n"/>
+      <c r="AK316" s="19" t="n"/>
+      <c r="AL316" s="19" t="n"/>
+      <c r="AM316" s="16" t="inlineStr">
+        <is>
+          <t>2 Stück – abgebildet ist eines davon.</t>
+        </is>
+      </c>
+      <c r="AN316" s="22" t="n"/>
+    </row>
+    <row r="317" ht="30" customHeight="1">
+      <c r="A317" s="15" t="inlineStr">
+        <is>
+          <t>BU02-16</t>
+        </is>
+      </c>
+      <c r="B317" s="15" t="n"/>
+      <c r="C317" s="15" t="n"/>
+      <c r="D317" s="15" t="inlineStr">
+        <is>
+          <t>BU02</t>
+        </is>
+      </c>
+      <c r="E317" s="15" t="inlineStr">
+        <is>
+          <t>Servierwagen Metall schwarz, drei Ebenen</t>
+        </is>
+      </c>
+      <c r="F317" s="16" t="inlineStr">
+        <is>
+          <t>Rollwagen aus schwarz lackiertem Metall mit drei Ablageebenen und Lochblechböden, auf vier Rollen.</t>
+        </is>
+      </c>
+      <c r="G317" s="15" t="inlineStr">
+        <is>
+          <t>Möbel</t>
+        </is>
+      </c>
+      <c r="H317" s="15" t="inlineStr">
+        <is>
+          <t>Flur 2</t>
+        </is>
+      </c>
+      <c r="I317" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J317" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K317" s="17" t="n"/>
+      <c r="L317" s="18">
+        <f>J317-IF(K317="",0,K317)</f>
+        <v/>
+      </c>
+      <c r="M317" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N317" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O317" s="19" t="n"/>
+      <c r="P317" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q317" s="19" t="n"/>
+      <c r="R317" s="20" t="n"/>
+      <c r="S317" s="20" t="n">
+        <v>30</v>
+      </c>
+      <c r="T317" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U317" s="21">
+        <f>L317*S317</f>
+        <v/>
+      </c>
+      <c r="V317" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W317" s="15" t="inlineStr">
+        <is>
+          <t>F-380</t>
+        </is>
+      </c>
+      <c r="X317" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y317" s="19" t="n"/>
+      <c r="Z317" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA317" s="19" t="n"/>
+      <c r="AB317" s="19" t="n"/>
+      <c r="AC317" s="19" t="n"/>
+      <c r="AD317" s="19" t="n"/>
+      <c r="AE317" s="20" t="n"/>
+      <c r="AF317" s="21">
+        <f>IF(K317="","",K317*AE317)</f>
+        <v/>
+      </c>
+      <c r="AG317" s="19" t="n"/>
+      <c r="AH317" s="19" t="n"/>
+      <c r="AI317" s="19" t="n"/>
+      <c r="AJ317" s="19" t="n"/>
+      <c r="AK317" s="19" t="n"/>
+      <c r="AL317" s="19" t="n"/>
+      <c r="AM317" s="16" t="inlineStr">
+        <is>
+          <t>1 Wagen. Der Inhalt gehört nicht dazu.</t>
+        </is>
+      </c>
+      <c r="AN317" s="22" t="n"/>
+    </row>
+    <row r="318" ht="30" customHeight="1">
+      <c r="A318" s="15" t="inlineStr">
+        <is>
+          <t>BU02-17</t>
+        </is>
+      </c>
+      <c r="B318" s="15" t="n"/>
+      <c r="C318" s="15" t="n"/>
+      <c r="D318" s="15" t="inlineStr">
+        <is>
+          <t>BU02</t>
+        </is>
+      </c>
+      <c r="E318" s="15" t="inlineStr">
+        <is>
+          <t>Kommode weiß, drei Schubladen</t>
+        </is>
+      </c>
+      <c r="F318" s="16" t="inlineStr">
+        <is>
+          <t>Kommode in Weiß mit drei breiten Schubladen und mittig ausgeschnittenen Griffmulden, auf umlaufendem Sockel.</t>
+        </is>
+      </c>
+      <c r="G318" s="15" t="inlineStr">
+        <is>
+          <t>Möbel</t>
+        </is>
+      </c>
+      <c r="H318" s="15" t="inlineStr">
+        <is>
+          <t>Flur 2</t>
+        </is>
+      </c>
+      <c r="I318" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J318" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K318" s="17" t="n"/>
+      <c r="L318" s="18">
+        <f>J318-IF(K318="",0,K318)</f>
+        <v/>
+      </c>
+      <c r="M318" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N318" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O318" s="19" t="n"/>
+      <c r="P318" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q318" s="19" t="n"/>
+      <c r="R318" s="20" t="n"/>
+      <c r="S318" s="20" t="n">
+        <v>60</v>
+      </c>
+      <c r="T318" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U318" s="21">
+        <f>L318*S318</f>
+        <v/>
+      </c>
+      <c r="V318" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W318" s="15" t="inlineStr">
+        <is>
+          <t>F-381</t>
+        </is>
+      </c>
+      <c r="X318" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y318" s="19" t="n"/>
+      <c r="Z318" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA318" s="19" t="n"/>
+      <c r="AB318" s="19" t="n"/>
+      <c r="AC318" s="19" t="n"/>
+      <c r="AD318" s="19" t="n"/>
+      <c r="AE318" s="20" t="n"/>
+      <c r="AF318" s="21">
+        <f>IF(K318="","",K318*AE318)</f>
+        <v/>
+      </c>
+      <c r="AG318" s="19" t="n"/>
+      <c r="AH318" s="19" t="n"/>
+      <c r="AI318" s="19" t="n"/>
+      <c r="AJ318" s="19" t="n"/>
+      <c r="AK318" s="19" t="n"/>
+      <c r="AL318" s="19" t="n"/>
+      <c r="AM318" s="16" t="inlineStr">
+        <is>
+          <t>1 Kommode.</t>
+        </is>
+      </c>
+      <c r="AN318" s="22" t="n"/>
+    </row>
+    <row r="319" ht="30" customHeight="1">
+      <c r="A319" s="15" t="inlineStr">
+        <is>
+          <t>BU02-18</t>
+        </is>
+      </c>
+      <c r="B319" s="15" t="n"/>
+      <c r="C319" s="15" t="n"/>
+      <c r="D319" s="15" t="inlineStr">
+        <is>
+          <t>BU02</t>
+        </is>
+      </c>
+      <c r="E319" s="15" t="inlineStr">
+        <is>
+          <t>Hochflorteppich grau</t>
+        </is>
+      </c>
+      <c r="F319" s="16" t="inlineStr">
+        <is>
+          <t>Hochflorteppich in Grau, rechteckig. Etikett auf der Rückseite vorhanden, Maßangabe 160 × 230 cm.</t>
+        </is>
+      </c>
+      <c r="G319" s="15" t="inlineStr">
+        <is>
+          <t>Textilien</t>
+        </is>
+      </c>
+      <c r="H319" s="15" t="inlineStr">
+        <is>
+          <t>Flur 2</t>
+        </is>
+      </c>
+      <c r="I319" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J319" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K319" s="17" t="n"/>
+      <c r="L319" s="18">
+        <f>J319-IF(K319="",0,K319)</f>
+        <v/>
+      </c>
+      <c r="M319" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N319" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O319" s="19" t="inlineStr">
+        <is>
+          <t>160 × 230 cm</t>
+        </is>
+      </c>
+      <c r="P319" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q319" s="19" t="n"/>
+      <c r="R319" s="20" t="n"/>
+      <c r="S319" s="20" t="n">
+        <v>40</v>
+      </c>
+      <c r="T319" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U319" s="21">
+        <f>L319*S319</f>
+        <v/>
+      </c>
+      <c r="V319" s="15" t="inlineStr">
+        <is>
+          <t>Versand möglich</t>
+        </is>
+      </c>
+      <c r="W319" s="15" t="inlineStr">
+        <is>
+          <t>F-382</t>
+        </is>
+      </c>
+      <c r="X319" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y319" s="19" t="n"/>
+      <c r="Z319" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA319" s="19" t="n"/>
+      <c r="AB319" s="19" t="n"/>
+      <c r="AC319" s="19" t="n"/>
+      <c r="AD319" s="19" t="n"/>
+      <c r="AE319" s="20" t="n"/>
+      <c r="AF319" s="21">
+        <f>IF(K319="","",K319*AE319)</f>
+        <v/>
+      </c>
+      <c r="AG319" s="19" t="n"/>
+      <c r="AH319" s="19" t="n"/>
+      <c r="AI319" s="19" t="n"/>
+      <c r="AJ319" s="19" t="n"/>
+      <c r="AK319" s="19" t="n"/>
+      <c r="AL319" s="19" t="n"/>
+      <c r="AM319" s="16" t="inlineStr">
+        <is>
+          <t>1 Teppich. Das Etikett ist auf Foto F-384 zu sehen.</t>
+        </is>
+      </c>
+      <c r="AN319" s="22" t="inlineStr">
+        <is>
+          <t>OFFEN: Auf dem Erfassungsblatt steht 1,80 × 2,30 m, das Etikett nennt 160 × 230 cm – bitte nachmessen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="320" ht="30" customHeight="1">
+      <c r="A320" s="15" t="inlineStr">
+        <is>
+          <t>BU02-19</t>
+        </is>
+      </c>
+      <c r="B320" s="15" t="n"/>
+      <c r="C320" s="15" t="n"/>
+      <c r="D320" s="15" t="inlineStr">
+        <is>
+          <t>BU02</t>
+        </is>
+      </c>
+      <c r="E320" s="15" t="inlineStr">
+        <is>
+          <t>Spielmöbel Kiefer, dreiteilig</t>
+        </is>
+      </c>
+      <c r="F320" s="16" t="inlineStr">
+        <is>
+          <t>Dreiteilige Kombination aus Kiefer massiv: Wandregal mit zwei Kunststoffwannen, niedrige Werkbank mit offenem Unterbau und zwei Wannen sowie ein hohes Seitenteil mit Wanne.</t>
+        </is>
+      </c>
+      <c r="G320" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H320" s="15" t="inlineStr">
+        <is>
+          <t>Flur 2</t>
+        </is>
+      </c>
+      <c r="I320" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J320" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K320" s="17" t="n"/>
+      <c r="L320" s="18">
+        <f>J320-IF(K320="",0,K320)</f>
+        <v/>
+      </c>
+      <c r="M320" s="15" t="inlineStr">
+        <is>
+          <t>Set</t>
+        </is>
+      </c>
+      <c r="N320" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O320" s="19" t="n"/>
+      <c r="P320" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q320" s="19" t="n"/>
+      <c r="R320" s="20" t="n"/>
+      <c r="S320" s="20" t="n">
+        <v>90</v>
+      </c>
+      <c r="T320" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U320" s="21">
+        <f>L320*S320</f>
+        <v/>
+      </c>
+      <c r="V320" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W320" s="15" t="inlineStr">
+        <is>
+          <t>F-385</t>
+        </is>
+      </c>
+      <c r="X320" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y320" s="19" t="n"/>
+      <c r="Z320" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA320" s="19" t="n"/>
+      <c r="AB320" s="19" t="n"/>
+      <c r="AC320" s="19" t="n"/>
+      <c r="AD320" s="19" t="n"/>
+      <c r="AE320" s="20" t="n"/>
+      <c r="AF320" s="21">
+        <f>IF(K320="","",K320*AE320)</f>
+        <v/>
+      </c>
+      <c r="AG320" s="19" t="n"/>
+      <c r="AH320" s="19" t="n"/>
+      <c r="AI320" s="19" t="n"/>
+      <c r="AJ320" s="19" t="n"/>
+      <c r="AK320" s="19" t="n"/>
+      <c r="AL320" s="19" t="n"/>
+      <c r="AM320" s="16" t="inlineStr">
+        <is>
+          <t>1 Kombination aus drei Teilen einschließlich der Wannen. Das Spielzeug gehört nicht dazu.</t>
+        </is>
+      </c>
+      <c r="AN320" s="22" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:AN306"/>
+  <autoFilter ref="A2:AN320"/>
   <mergeCells count="7">
     <mergeCell ref="AI1:AL1"/>
     <mergeCell ref="V1:AD1"/>
@@ -38365,7 +40071,7 @@
     <mergeCell ref="AE1:AH1"/>
     <mergeCell ref="AM1:AN1"/>
   </mergeCells>
-  <conditionalFormatting sqref="Z3:Z306">
+  <conditionalFormatting sqref="Z3:Z320">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"reserviert"</formula>
     </cfRule>
@@ -38376,12 +40082,12 @@
       <formula>"verkauft"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I3:I306">
+  <conditionalFormatting sqref="I3:I320">
     <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
       <formula>"A"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P3:P306">
+  <conditionalFormatting sqref="P3:P320">
     <cfRule type="cellIs" priority="5" operator="equal" dxfId="4">
       <formula>"entfällt"</formula>
     </cfRule>
@@ -38472,7 +40178,7 @@
         </is>
       </c>
       <c r="B5" s="27">
-        <f>COUNTA(Artikelstamm!$A$3:$A$306)</f>
+        <f>COUNTA(Artikelstamm!$A$3:$A$320)</f>
         <v/>
       </c>
     </row>
@@ -38483,7 +40189,7 @@
         </is>
       </c>
       <c r="B6" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$306,"verfügbar")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$320,"verfügbar")</f>
         <v/>
       </c>
     </row>
@@ -38494,7 +40200,7 @@
         </is>
       </c>
       <c r="B7" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$306,"reserviert")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$320,"reserviert")</f>
         <v/>
       </c>
     </row>
@@ -38505,7 +40211,7 @@
         </is>
       </c>
       <c r="B8" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$306,"teilverkauft")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$320,"teilverkauft")</f>
         <v/>
       </c>
     </row>
@@ -38516,7 +40222,7 @@
         </is>
       </c>
       <c r="B9" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$306,"verkauft")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$320,"verkauft")</f>
         <v/>
       </c>
     </row>
@@ -38527,7 +40233,7 @@
         </is>
       </c>
       <c r="B10" s="27">
-        <f>SUM(Artikelstamm!$L$3:$L$306)</f>
+        <f>SUM(Artikelstamm!$L$3:$L$320)</f>
         <v/>
       </c>
     </row>
@@ -38538,7 +40244,7 @@
         </is>
       </c>
       <c r="B11" s="29">
-        <f>SUM(Artikelstamm!$U$3:$U$306)</f>
+        <f>SUM(Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -38556,7 +40262,7 @@
         </is>
       </c>
       <c r="B13" s="27">
-        <f>SUM(Artikelstamm!$K$3:$K$306)</f>
+        <f>SUM(Artikelstamm!$K$3:$K$320)</f>
         <v/>
       </c>
     </row>
@@ -38567,7 +40273,7 @@
         </is>
       </c>
       <c r="B14" s="30">
-        <f>SUMPRODUCT(Artikelstamm!$K$3:$K$306,Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT(Artikelstamm!$K$3:$K$320,Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
     </row>
@@ -38600,7 +40306,7 @@
         </is>
       </c>
       <c r="B17" s="30">
-        <f>SUMPRODUCT((Artikelstamm!$AJ$3:$AJ$306="bezahlt")*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AJ$3:$AJ$320="bezahlt")*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
     </row>
@@ -38629,7 +40335,7 @@
         </is>
       </c>
       <c r="B21" s="31">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$306,"*verkauft",Artikelstamm!$AI$3:$AI$306,"")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$320,"*verkauft",Artikelstamm!$AI$3:$AI$320,"")</f>
         <v/>
       </c>
     </row>
@@ -38640,7 +40346,7 @@
         </is>
       </c>
       <c r="B22" s="31">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$306,"*verkauft",Artikelstamm!$AJ$3:$AJ$306,"offen")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$320,"*verkauft",Artikelstamm!$AJ$3:$AJ$320,"offen")</f>
         <v/>
       </c>
     </row>
@@ -38651,7 +40357,7 @@
         </is>
       </c>
       <c r="B23" s="27">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$306,"reserviert",Artikelstamm!$AL$3:$AL$306,"")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$320,"reserviert",Artikelstamm!$AL$3:$AL$320,"")</f>
         <v/>
       </c>
     </row>
@@ -38662,7 +40368,7 @@
         </is>
       </c>
       <c r="B24" s="27">
-        <f>COUNTIFS(Artikelstamm!$S$3:$S$306,"")</f>
+        <f>COUNTIFS(Artikelstamm!$S$3:$S$320,"")</f>
         <v/>
       </c>
     </row>
@@ -38673,7 +40379,7 @@
         </is>
       </c>
       <c r="B25" s="27">
-        <f>COUNTIFS(Artikelstamm!$O$3:$O$306,"")</f>
+        <f>COUNTIFS(Artikelstamm!$O$3:$O$320,"")</f>
         <v/>
       </c>
     </row>
@@ -38713,15 +40419,15 @@
         </is>
       </c>
       <c r="B30" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$306,$A30)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$320,$A30)</f>
         <v/>
       </c>
       <c r="C30" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$306=$A30)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$320=$A30)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D30" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$306,$A30,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$320,$A30,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -38732,15 +40438,15 @@
         </is>
       </c>
       <c r="B31" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$306,$A31)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$320,$A31)</f>
         <v/>
       </c>
       <c r="C31" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$306=$A31)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$320=$A31)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D31" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$306,$A31,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$320,$A31,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -38751,15 +40457,15 @@
         </is>
       </c>
       <c r="B32" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$306,$A32)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$320,$A32)</f>
         <v/>
       </c>
       <c r="C32" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$306=$A32)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$320=$A32)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D32" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$306,$A32,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$320,$A32,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -38818,15 +40524,15 @@
         </is>
       </c>
       <c r="B37" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$306,$A37)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$320,$A37)</f>
         <v/>
       </c>
       <c r="C37" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$306=$A37)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$320=$A37)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D37" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$306,$A37,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$320,$A37,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -38837,15 +40543,15 @@
         </is>
       </c>
       <c r="B38" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$306,$A38)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$320,$A38)</f>
         <v/>
       </c>
       <c r="C38" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$306=$A38)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$320=$A38)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D38" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$306,$A38,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$320,$A38,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -38856,15 +40562,15 @@
         </is>
       </c>
       <c r="B39" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$306,$A39)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$320,$A39)</f>
         <v/>
       </c>
       <c r="C39" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$306=$A39)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$320=$A39)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D39" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$306,$A39,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$320,$A39,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -38875,15 +40581,15 @@
         </is>
       </c>
       <c r="B40" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$306,$A40)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$320,$A40)</f>
         <v/>
       </c>
       <c r="C40" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$306=$A40)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$320=$A40)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D40" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$306,$A40,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$320,$A40,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -38894,15 +40600,15 @@
         </is>
       </c>
       <c r="B41" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$306,$A41)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$320,$A41)</f>
         <v/>
       </c>
       <c r="C41" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$306=$A41)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$320=$A41)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D41" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$306,$A41,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$320,$A41,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -38913,15 +40619,15 @@
         </is>
       </c>
       <c r="B42" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$306,$A42)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$320,$A42)</f>
         <v/>
       </c>
       <c r="C42" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$306=$A42)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$320=$A42)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D42" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$306,$A42,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$320,$A42,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -38932,15 +40638,15 @@
         </is>
       </c>
       <c r="B43" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$306,$A43)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$320,$A43)</f>
         <v/>
       </c>
       <c r="C43" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$306=$A43)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$320=$A43)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D43" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$306,$A43,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$320,$A43,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -38951,15 +40657,15 @@
         </is>
       </c>
       <c r="B44" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$306,$A44)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$320,$A44)</f>
         <v/>
       </c>
       <c r="C44" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$306=$A44)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$320=$A44)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D44" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$306,$A44,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$320,$A44,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -38970,15 +40676,15 @@
         </is>
       </c>
       <c r="B45" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$306,$A45)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$320,$A45)</f>
         <v/>
       </c>
       <c r="C45" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$306=$A45)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$320=$A45)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D45" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$306,$A45,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$320,$A45,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -38989,15 +40695,15 @@
         </is>
       </c>
       <c r="B46" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$306,$A46)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$320,$A46)</f>
         <v/>
       </c>
       <c r="C46" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$306=$A46)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$320=$A46)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D46" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$306,$A46,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$320,$A46,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -39008,15 +40714,15 @@
         </is>
       </c>
       <c r="B47" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$306,$A47)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$320,$A47)</f>
         <v/>
       </c>
       <c r="C47" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$306=$A47)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$320=$A47)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D47" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$306,$A47,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$320,$A47,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -39027,15 +40733,15 @@
         </is>
       </c>
       <c r="B48" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$306,$A48)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$320,$A48)</f>
         <v/>
       </c>
       <c r="C48" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$306=$A48)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$320=$A48)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D48" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$306,$A48,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$320,$A48,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -39046,15 +40752,15 @@
         </is>
       </c>
       <c r="B49" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$306,$A49)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$320,$A49)</f>
         <v/>
       </c>
       <c r="C49" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$306=$A49)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$320=$A49)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D49" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$306,$A49,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$320,$A49,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -39065,15 +40771,15 @@
         </is>
       </c>
       <c r="B50" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$306,$A50)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$320,$A50)</f>
         <v/>
       </c>
       <c r="C50" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$306=$A50)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$320=$A50)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D50" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$306,$A50,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$320,$A50,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -39132,15 +40838,15 @@
         </is>
       </c>
       <c r="B55" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A55)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A55)</f>
         <v/>
       </c>
       <c r="C55" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A55)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A55)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D55" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A55,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A55,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -39151,15 +40857,15 @@
         </is>
       </c>
       <c r="B56" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A56)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A56)</f>
         <v/>
       </c>
       <c r="C56" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A56)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A56)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D56" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A56,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A56,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -39170,15 +40876,15 @@
         </is>
       </c>
       <c r="B57" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A57)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A57)</f>
         <v/>
       </c>
       <c r="C57" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A57)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A57)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D57" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A57,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A57,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -39189,15 +40895,15 @@
         </is>
       </c>
       <c r="B58" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A58)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A58)</f>
         <v/>
       </c>
       <c r="C58" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A58)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A58)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D58" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A58,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A58,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -39208,15 +40914,15 @@
         </is>
       </c>
       <c r="B59" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A59)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A59)</f>
         <v/>
       </c>
       <c r="C59" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A59)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A59)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D59" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A59,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A59,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -39227,15 +40933,15 @@
         </is>
       </c>
       <c r="B60" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A60)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A60)</f>
         <v/>
       </c>
       <c r="C60" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A60)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A60)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D60" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A60,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A60,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -39246,15 +40952,15 @@
         </is>
       </c>
       <c r="B61" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A61)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A61)</f>
         <v/>
       </c>
       <c r="C61" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A61)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A61)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D61" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A61,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A61,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -39265,15 +40971,15 @@
         </is>
       </c>
       <c r="B62" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A62)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A62)</f>
         <v/>
       </c>
       <c r="C62" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A62)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A62)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D62" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A62,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A62,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -39284,15 +40990,15 @@
         </is>
       </c>
       <c r="B63" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A63)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A63)</f>
         <v/>
       </c>
       <c r="C63" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A63)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A63)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D63" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A63,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A63,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -39303,15 +41009,15 @@
         </is>
       </c>
       <c r="B64" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A64)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A64)</f>
         <v/>
       </c>
       <c r="C64" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A64)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A64)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D64" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A64,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A64,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -39322,15 +41028,15 @@
         </is>
       </c>
       <c r="B65" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A65)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A65)</f>
         <v/>
       </c>
       <c r="C65" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A65)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A65)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D65" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A65,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A65,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -39341,15 +41047,15 @@
         </is>
       </c>
       <c r="B66" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A66)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A66)</f>
         <v/>
       </c>
       <c r="C66" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A66)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A66)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D66" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A66,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A66,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -39360,15 +41066,15 @@
         </is>
       </c>
       <c r="B67" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A67)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A67)</f>
         <v/>
       </c>
       <c r="C67" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A67)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A67)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D67" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A67,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A67,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -39379,15 +41085,15 @@
         </is>
       </c>
       <c r="B68" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A68)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A68)</f>
         <v/>
       </c>
       <c r="C68" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A68)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A68)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D68" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A68,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A68,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -39398,15 +41104,15 @@
         </is>
       </c>
       <c r="B69" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A69)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A69)</f>
         <v/>
       </c>
       <c r="C69" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A69)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A69)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D69" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A69,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A69,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -39417,15 +41123,15 @@
         </is>
       </c>
       <c r="B70" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A70)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A70)</f>
         <v/>
       </c>
       <c r="C70" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A70)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A70)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D70" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A70,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A70,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -39436,15 +41142,15 @@
         </is>
       </c>
       <c r="B71" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A71)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A71)</f>
         <v/>
       </c>
       <c r="C71" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A71)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A71)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D71" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A71,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A71,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -39455,15 +41161,15 @@
         </is>
       </c>
       <c r="B72" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A72)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A72)</f>
         <v/>
       </c>
       <c r="C72" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A72)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A72)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D72" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A72,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A72,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -39474,15 +41180,15 @@
         </is>
       </c>
       <c r="B73" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A73)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A73)</f>
         <v/>
       </c>
       <c r="C73" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A73)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A73)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D73" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A73,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A73,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -39493,15 +41199,15 @@
         </is>
       </c>
       <c r="B74" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A74)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A74)</f>
         <v/>
       </c>
       <c r="C74" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A74)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A74)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D74" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A74,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A74,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -39512,15 +41218,15 @@
         </is>
       </c>
       <c r="B75" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A75)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A75)</f>
         <v/>
       </c>
       <c r="C75" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A75)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A75)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D75" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A75,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A75,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -39531,15 +41237,15 @@
         </is>
       </c>
       <c r="B76" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A76)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A76)</f>
         <v/>
       </c>
       <c r="C76" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A76)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A76)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D76" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A76,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A76,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -39550,15 +41256,15 @@
         </is>
       </c>
       <c r="B77" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A77)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A77)</f>
         <v/>
       </c>
       <c r="C77" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A77)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A77)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D77" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A77,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A77,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -39569,15 +41275,15 @@
         </is>
       </c>
       <c r="B78" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A78)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A78)</f>
         <v/>
       </c>
       <c r="C78" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A78)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A78)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D78" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A78,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A78,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -39588,15 +41294,15 @@
         </is>
       </c>
       <c r="B79" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A79)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A79)</f>
         <v/>
       </c>
       <c r="C79" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A79)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A79)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D79" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A79,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A79,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -39607,15 +41313,15 @@
         </is>
       </c>
       <c r="B80" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A80)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A80)</f>
         <v/>
       </c>
       <c r="C80" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A80)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A80)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D80" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A80,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A80,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -39626,15 +41332,15 @@
         </is>
       </c>
       <c r="B81" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A81)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A81)</f>
         <v/>
       </c>
       <c r="C81" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A81)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A81)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D81" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A81,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A81,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -39645,15 +41351,15 @@
         </is>
       </c>
       <c r="B82" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$306,$A82)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A82)</f>
         <v/>
       </c>
       <c r="C82" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$306=$A82)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A82)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
       <c r="D82" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$306,$A82,Artikelstamm!$U$3:$U$306)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A82,Artikelstamm!$U$3:$U$320)</f>
         <v/>
       </c>
     </row>
@@ -39707,11 +41413,11 @@
         </is>
       </c>
       <c r="B87" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$306,$A87)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$320,$A87)</f>
         <v/>
       </c>
       <c r="C87" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$306=$A87)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$320=$A87)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
     </row>
@@ -39722,11 +41428,11 @@
         </is>
       </c>
       <c r="B88" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$306,$A88)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$320,$A88)</f>
         <v/>
       </c>
       <c r="C88" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$306=$A88)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$320=$A88)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
     </row>
@@ -39737,11 +41443,11 @@
         </is>
       </c>
       <c r="B89" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$306,$A89)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$320,$A89)</f>
         <v/>
       </c>
       <c r="C89" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$306=$A89)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$320=$A89)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
     </row>
@@ -39752,11 +41458,11 @@
         </is>
       </c>
       <c r="B90" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$306,$A90)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$320,$A90)</f>
         <v/>
       </c>
       <c r="C90" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$306=$A90)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$320=$A90)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
     </row>
@@ -39767,11 +41473,11 @@
         </is>
       </c>
       <c r="B91" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$306,$A91)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$320,$A91)</f>
         <v/>
       </c>
       <c r="C91" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$306=$A91)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$320=$A91)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
     </row>
@@ -39782,11 +41488,11 @@
         </is>
       </c>
       <c r="B92" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$306,$A92)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$320,$A92)</f>
         <v/>
       </c>
       <c r="C92" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$306=$A92)*Artikelstamm!$K$3:$K$306*Artikelstamm!$AE$3:$AE$306)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$320=$A92)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
BU03 Flur 3 erfasst; Rueckmeldungen zu BU02 eingearbeitet
Entscheidungen der Nutzerin zu BU02:
  BU02-13 ist dieselbe Lama-Steckwand wie BU01-06 - zusammengefasst (3 Stueck)
  BU02-14 sind die weissen IKEA-Schraenke aus BA02-08, der Farbton im Foto
          war nur Schatten - Zeile entfernt, BA02-08 jetzt 6 Stueck
  BU02-18 Teppichmass laut Etikett 160 x 230 cm, offener Punkt erledigt

Raum BU03 (Bestandsgebaeude UG, Flur 3, 14,40 m2) aus 9 Fotos und dem
Erfassungsblatt aufgenommen: 8 neue Positionen, keine Zusammenfassungen.

Foto F-388 maskiert: im Schwingspiegel gespiegelte Fotocollage mit Kinderfotos.

Datenbasis 325 Positionen / 269 aktiv, pruefen.py 0 Fehler.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011yyfqhuiWGsaNy38oaNoGo
</commit_message>
<xml_diff>
--- a/ausgabe/01_Artikelstamm_kikripp.xlsx
+++ b/ausgabe/01_Artikelstamm_kikripp.xlsx
@@ -15,7 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Artikelstamm'!$A$2:$AN$320</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Artikelstamm'!$A$2:$AN$327</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1019,7 +1019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN320"/>
+  <dimension ref="A1:AN327"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -30397,7 +30397,7 @@
       <c r="B241" s="15" t="n"/>
       <c r="C241" s="15" t="inlineStr">
         <is>
-          <t>BA04-09</t>
+          <t>BA04-09, BU02-14</t>
         </is>
       </c>
       <c r="D241" s="15" t="inlineStr">
@@ -30431,7 +30431,7 @@
         </is>
       </c>
       <c r="J241" s="17" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K241" s="17" t="n"/>
       <c r="L241" s="18">
@@ -30510,12 +30510,12 @@
       <c r="AL241" s="19" t="n"/>
       <c r="AM241" s="16" t="inlineStr">
         <is>
-          <t>4 Schränke insgesamt: 2 im Flur 2 (BA02-08) und 2 im Gruppenraum 4 (dort mit BA04-09 beschriftet). Abgebildet ist einer davon, ein weiterer auf Foto F-308.</t>
+          <t>6 Schränke insgesamt: 2 im Flur 2 der Attika (BA02-08), 2 im Gruppenraum 4 (BA04-09) und 2 im Flur 2 im Untergeschoss des Bestandsgebäudes (BU02-14). Die beiden Schränke im Untergeschoss sind auf Foto F-378 zu sehen.</t>
         </is>
       </c>
       <c r="AN241" s="22" t="inlineStr">
         <is>
-          <t>Zusammengefasste Position – Post-it-Nummer im zweiten Raum: BA04-09.</t>
+          <t>Zusammengefasste Position über drei Räume – Post-it-Nummern: BA04-09, BU02-14.</t>
         </is>
       </c>
     </row>
@@ -39337,7 +39337,7 @@
     <row r="315" ht="30" customHeight="1">
       <c r="A315" s="15" t="inlineStr">
         <is>
-          <t>BU02-14</t>
+          <t>BU02-15</t>
         </is>
       </c>
       <c r="B315" s="15" t="n"/>
@@ -39349,17 +39349,17 @@
       </c>
       <c r="E315" s="15" t="inlineStr">
         <is>
-          <t>Kinderschrank graugrün, zwei Türen</t>
+          <t>Bodensitzkissen beige, selbststehend</t>
         </is>
       </c>
       <c r="F315" s="16" t="inlineStr">
         <is>
-          <t>Hoher Kinderschrank von IKEA mit zwei graugrünen Türen und schwarzen Griffmulden, darunter eine Schublade.</t>
+          <t>Selbststehendes Bodensitzkissen aus beigem Leinenstoff mit gesteppten Feldern, Rückenlehne und langer Sitzfläche. Die Lehne lässt sich flach ausklappen.</t>
         </is>
       </c>
       <c r="G315" s="15" t="inlineStr">
         <is>
-          <t>Möbel</t>
+          <t>Textilien</t>
         </is>
       </c>
       <c r="H315" s="15" t="inlineStr">
@@ -39369,7 +39369,7 @@
       </c>
       <c r="I315" s="15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J315" s="17" t="n">
@@ -39399,7 +39399,7 @@
       <c r="Q315" s="19" t="n"/>
       <c r="R315" s="20" t="n"/>
       <c r="S315" s="20" t="n">
-        <v>90</v>
+        <v>25</v>
       </c>
       <c r="T315" s="19" t="inlineStr">
         <is>
@@ -39417,7 +39417,7 @@
       </c>
       <c r="W315" s="15" t="inlineStr">
         <is>
-          <t>F-378</t>
+          <t>F-379</t>
         </is>
       </c>
       <c r="X315" s="19" t="inlineStr">
@@ -39431,11 +39431,7 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="AA315" s="19" t="inlineStr">
-        <is>
-          <t>IKEA</t>
-        </is>
-      </c>
+      <c r="AA315" s="19" t="n"/>
       <c r="AB315" s="19" t="n"/>
       <c r="AC315" s="19" t="n"/>
       <c r="AD315" s="19" t="n"/>
@@ -39452,7 +39448,7 @@
       <c r="AL315" s="19" t="n"/>
       <c r="AM315" s="16" t="inlineStr">
         <is>
-          <t>2 Schränke – abgebildet ist einer davon. Baugleiche Schränke mit weißen Türen stehen unter BA02-08.</t>
+          <t>2 Stück – abgebildet ist eines davon.</t>
         </is>
       </c>
       <c r="AN315" s="22" t="n"/>
@@ -39460,7 +39456,7 @@
     <row r="316" ht="30" customHeight="1">
       <c r="A316" s="15" t="inlineStr">
         <is>
-          <t>BU02-15</t>
+          <t>BU02-16</t>
         </is>
       </c>
       <c r="B316" s="15" t="n"/>
@@ -39472,17 +39468,17 @@
       </c>
       <c r="E316" s="15" t="inlineStr">
         <is>
-          <t>Bodensitzkissen beige, selbststehend</t>
+          <t>Servierwagen Metall schwarz, drei Ebenen</t>
         </is>
       </c>
       <c r="F316" s="16" t="inlineStr">
         <is>
-          <t>Selbststehendes Bodensitzkissen aus beigem Leinenstoff mit gesteppten Feldern, Rückenlehne und langer Sitzfläche. Die Lehne lässt sich flach ausklappen.</t>
+          <t>Rollwagen aus schwarz lackiertem Metall mit drei Ablageebenen und Lochblechböden, auf vier Rollen.</t>
         </is>
       </c>
       <c r="G316" s="15" t="inlineStr">
         <is>
-          <t>Textilien</t>
+          <t>Möbel</t>
         </is>
       </c>
       <c r="H316" s="15" t="inlineStr">
@@ -39492,11 +39488,11 @@
       </c>
       <c r="I316" s="15" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J316" s="17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K316" s="17" t="n"/>
       <c r="L316" s="18">
@@ -39522,7 +39518,7 @@
       <c r="Q316" s="19" t="n"/>
       <c r="R316" s="20" t="n"/>
       <c r="S316" s="20" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="T316" s="19" t="inlineStr">
         <is>
@@ -39540,7 +39536,7 @@
       </c>
       <c r="W316" s="15" t="inlineStr">
         <is>
-          <t>F-379</t>
+          <t>F-380</t>
         </is>
       </c>
       <c r="X316" s="19" t="inlineStr">
@@ -39571,7 +39567,7 @@
       <c r="AL316" s="19" t="n"/>
       <c r="AM316" s="16" t="inlineStr">
         <is>
-          <t>2 Stück – abgebildet ist eines davon.</t>
+          <t>1 Wagen. Der Inhalt gehört nicht dazu.</t>
         </is>
       </c>
       <c r="AN316" s="22" t="n"/>
@@ -39579,7 +39575,7 @@
     <row r="317" ht="30" customHeight="1">
       <c r="A317" s="15" t="inlineStr">
         <is>
-          <t>BU02-16</t>
+          <t>BU02-17</t>
         </is>
       </c>
       <c r="B317" s="15" t="n"/>
@@ -39591,12 +39587,12 @@
       </c>
       <c r="E317" s="15" t="inlineStr">
         <is>
-          <t>Servierwagen Metall schwarz, drei Ebenen</t>
+          <t>Kommode weiß, drei Schubladen</t>
         </is>
       </c>
       <c r="F317" s="16" t="inlineStr">
         <is>
-          <t>Rollwagen aus schwarz lackiertem Metall mit drei Ablageebenen und Lochblechböden, auf vier Rollen.</t>
+          <t>Kommode in Weiß mit drei breiten Schubladen und mittig ausgeschnittenen Griffmulden, auf umlaufendem Sockel.</t>
         </is>
       </c>
       <c r="G317" s="15" t="inlineStr">
@@ -39641,7 +39637,7 @@
       <c r="Q317" s="19" t="n"/>
       <c r="R317" s="20" t="n"/>
       <c r="S317" s="20" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="T317" s="19" t="inlineStr">
         <is>
@@ -39659,7 +39655,7 @@
       </c>
       <c r="W317" s="15" t="inlineStr">
         <is>
-          <t>F-380</t>
+          <t>F-381</t>
         </is>
       </c>
       <c r="X317" s="19" t="inlineStr">
@@ -39690,7 +39686,7 @@
       <c r="AL317" s="19" t="n"/>
       <c r="AM317" s="16" t="inlineStr">
         <is>
-          <t>1 Wagen. Der Inhalt gehört nicht dazu.</t>
+          <t>1 Kommode.</t>
         </is>
       </c>
       <c r="AN317" s="22" t="n"/>
@@ -39698,7 +39694,7 @@
     <row r="318" ht="30" customHeight="1">
       <c r="A318" s="15" t="inlineStr">
         <is>
-          <t>BU02-17</t>
+          <t>BU02-18</t>
         </is>
       </c>
       <c r="B318" s="15" t="n"/>
@@ -39710,17 +39706,17 @@
       </c>
       <c r="E318" s="15" t="inlineStr">
         <is>
-          <t>Kommode weiß, drei Schubladen</t>
+          <t>Hochflorteppich grau</t>
         </is>
       </c>
       <c r="F318" s="16" t="inlineStr">
         <is>
-          <t>Kommode in Weiß mit drei breiten Schubladen und mittig ausgeschnittenen Griffmulden, auf umlaufendem Sockel.</t>
+          <t>Hochflorteppich in Grau, rechteckig. Maße laut Etikett auf der Rückseite: 160 × 230 cm.</t>
         </is>
       </c>
       <c r="G318" s="15" t="inlineStr">
         <is>
-          <t>Möbel</t>
+          <t>Textilien</t>
         </is>
       </c>
       <c r="H318" s="15" t="inlineStr">
@@ -39730,7 +39726,7 @@
       </c>
       <c r="I318" s="15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J318" s="17" t="n">
@@ -39751,7 +39747,11 @@
           <t>gebraucht</t>
         </is>
       </c>
-      <c r="O318" s="19" t="n"/>
+      <c r="O318" s="19" t="inlineStr">
+        <is>
+          <t>160 × 230 cm</t>
+        </is>
+      </c>
       <c r="P318" s="19" t="inlineStr">
         <is>
           <t>ja</t>
@@ -39760,7 +39760,7 @@
       <c r="Q318" s="19" t="n"/>
       <c r="R318" s="20" t="n"/>
       <c r="S318" s="20" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="T318" s="19" t="inlineStr">
         <is>
@@ -39773,12 +39773,12 @@
       </c>
       <c r="V318" s="15" t="inlineStr">
         <is>
-          <t>nur Abholung</t>
+          <t>Versand möglich</t>
         </is>
       </c>
       <c r="W318" s="15" t="inlineStr">
         <is>
-          <t>F-381</t>
+          <t>F-382</t>
         </is>
       </c>
       <c r="X318" s="19" t="inlineStr">
@@ -39809,7 +39809,7 @@
       <c r="AL318" s="19" t="n"/>
       <c r="AM318" s="16" t="inlineStr">
         <is>
-          <t>1 Kommode.</t>
+          <t>1 Teppich. Das Etikett ist auf Foto F-384 zu sehen.</t>
         </is>
       </c>
       <c r="AN318" s="22" t="n"/>
@@ -39817,7 +39817,7 @@
     <row r="319" ht="30" customHeight="1">
       <c r="A319" s="15" t="inlineStr">
         <is>
-          <t>BU02-18</t>
+          <t>BU02-19</t>
         </is>
       </c>
       <c r="B319" s="15" t="n"/>
@@ -39829,17 +39829,17 @@
       </c>
       <c r="E319" s="15" t="inlineStr">
         <is>
-          <t>Hochflorteppich grau</t>
+          <t>Spielmöbel Kiefer, dreiteilig</t>
         </is>
       </c>
       <c r="F319" s="16" t="inlineStr">
         <is>
-          <t>Hochflorteppich in Grau, rechteckig. Etikett auf der Rückseite vorhanden, Maßangabe 160 × 230 cm.</t>
+          <t>Dreiteilige Kombination aus Kiefer massiv: Wandregal mit zwei Kunststoffwannen, niedrige Werkbank mit offenem Unterbau und zwei Wannen sowie ein hohes Seitenteil mit Wanne.</t>
         </is>
       </c>
       <c r="G319" s="15" t="inlineStr">
         <is>
-          <t>Textilien</t>
+          <t>Kita-Ausstattung</t>
         </is>
       </c>
       <c r="H319" s="15" t="inlineStr">
@@ -39849,7 +39849,7 @@
       </c>
       <c r="I319" s="15" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="J319" s="17" t="n">
@@ -39862,7 +39862,7 @@
       </c>
       <c r="M319" s="15" t="inlineStr">
         <is>
-          <t>Stück</t>
+          <t>Set</t>
         </is>
       </c>
       <c r="N319" s="15" t="inlineStr">
@@ -39870,11 +39870,7 @@
           <t>gebraucht</t>
         </is>
       </c>
-      <c r="O319" s="19" t="inlineStr">
-        <is>
-          <t>160 × 230 cm</t>
-        </is>
-      </c>
+      <c r="O319" s="19" t="n"/>
       <c r="P319" s="19" t="inlineStr">
         <is>
           <t>ja</t>
@@ -39883,7 +39879,7 @@
       <c r="Q319" s="19" t="n"/>
       <c r="R319" s="20" t="n"/>
       <c r="S319" s="20" t="n">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="T319" s="19" t="inlineStr">
         <is>
@@ -39896,12 +39892,12 @@
       </c>
       <c r="V319" s="15" t="inlineStr">
         <is>
-          <t>Versand möglich</t>
+          <t>nur Abholung</t>
         </is>
       </c>
       <c r="W319" s="15" t="inlineStr">
         <is>
-          <t>F-382</t>
+          <t>F-385</t>
         </is>
       </c>
       <c r="X319" s="19" t="inlineStr">
@@ -39932,36 +39928,32 @@
       <c r="AL319" s="19" t="n"/>
       <c r="AM319" s="16" t="inlineStr">
         <is>
-          <t>1 Teppich. Das Etikett ist auf Foto F-384 zu sehen.</t>
-        </is>
-      </c>
-      <c r="AN319" s="22" t="inlineStr">
-        <is>
-          <t>OFFEN: Auf dem Erfassungsblatt steht 1,80 × 2,30 m, das Etikett nennt 160 × 230 cm – bitte nachmessen.</t>
-        </is>
-      </c>
+          <t>1 Kombination aus drei Teilen einschließlich der Wannen. Das Spielzeug gehört nicht dazu.</t>
+        </is>
+      </c>
+      <c r="AN319" s="22" t="n"/>
     </row>
     <row r="320" ht="30" customHeight="1">
       <c r="A320" s="15" t="inlineStr">
         <is>
-          <t>BU02-19</t>
+          <t>BU03-01</t>
         </is>
       </c>
       <c r="B320" s="15" t="n"/>
       <c r="C320" s="15" t="n"/>
       <c r="D320" s="15" t="inlineStr">
         <is>
-          <t>BU02</t>
+          <t>BU03</t>
         </is>
       </c>
       <c r="E320" s="15" t="inlineStr">
         <is>
-          <t>Spielmöbel Kiefer, dreiteilig</t>
+          <t>Pinnwand Holz mit Klammerleinen</t>
         </is>
       </c>
       <c r="F320" s="16" t="inlineStr">
         <is>
-          <t>Dreiteilige Kombination aus Kiefer massiv: Wandregal mit zwei Kunststoffwannen, niedrige Werkbank mit offenem Unterbau und zwei Wannen sowie ein hohes Seitenteil mit Wanne.</t>
+          <t>Großes Wandelement aus hellem Massivholz mit vier waagerechten Bändern und Holzklammern zum Aufhängen von Bildern und Bastelarbeiten. Zwei zusätzliche Querbretter als Ablage.</t>
         </is>
       </c>
       <c r="G320" s="15" t="inlineStr">
@@ -39971,7 +39963,7 @@
       </c>
       <c r="H320" s="15" t="inlineStr">
         <is>
-          <t>Flur 2</t>
+          <t>Flur 3</t>
         </is>
       </c>
       <c r="I320" s="15" t="inlineStr">
@@ -39989,7 +39981,7 @@
       </c>
       <c r="M320" s="15" t="inlineStr">
         <is>
-          <t>Set</t>
+          <t>Stück</t>
         </is>
       </c>
       <c r="N320" s="15" t="inlineStr">
@@ -40006,7 +39998,7 @@
       <c r="Q320" s="19" t="n"/>
       <c r="R320" s="20" t="n"/>
       <c r="S320" s="20" t="n">
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="T320" s="19" t="inlineStr">
         <is>
@@ -40024,7 +40016,7 @@
       </c>
       <c r="W320" s="15" t="inlineStr">
         <is>
-          <t>F-385</t>
+          <t>F-387</t>
         </is>
       </c>
       <c r="X320" s="19" t="inlineStr">
@@ -40055,13 +40047,846 @@
       <c r="AL320" s="19" t="n"/>
       <c r="AM320" s="16" t="inlineStr">
         <is>
-          <t>1 Kombination aus drei Teilen einschließlich der Wannen. Das Spielzeug gehört nicht dazu.</t>
+          <t>1 Wand einschließlich der Klammern. Die Deko-Ringe und Quasten gehören nicht dazu.</t>
         </is>
       </c>
       <c r="AN320" s="22" t="n"/>
     </row>
+    <row r="321" ht="30" customHeight="1">
+      <c r="A321" s="15" t="inlineStr">
+        <is>
+          <t>BU03-02</t>
+        </is>
+      </c>
+      <c r="B321" s="15" t="n"/>
+      <c r="C321" s="15" t="n"/>
+      <c r="D321" s="15" t="inlineStr">
+        <is>
+          <t>BU03</t>
+        </is>
+      </c>
+      <c r="E321" s="15" t="inlineStr">
+        <is>
+          <t>Schwingspiegel, geschwungene Form</t>
+        </is>
+      </c>
+      <c r="F321" s="16" t="inlineStr">
+        <is>
+          <t>Hoher Wandspiegel mit geschwungener Außenkante ohne Rahmen, zum Anschrauben.</t>
+        </is>
+      </c>
+      <c r="G321" s="15" t="inlineStr">
+        <is>
+          <t>Deko</t>
+        </is>
+      </c>
+      <c r="H321" s="15" t="inlineStr">
+        <is>
+          <t>Flur 3</t>
+        </is>
+      </c>
+      <c r="I321" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J321" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K321" s="17" t="n"/>
+      <c r="L321" s="18">
+        <f>J321-IF(K321="",0,K321)</f>
+        <v/>
+      </c>
+      <c r="M321" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N321" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O321" s="19" t="n"/>
+      <c r="P321" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q321" s="19" t="n"/>
+      <c r="R321" s="20" t="n"/>
+      <c r="S321" s="20" t="n">
+        <v>25</v>
+      </c>
+      <c r="T321" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U321" s="21">
+        <f>L321*S321</f>
+        <v/>
+      </c>
+      <c r="V321" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W321" s="15" t="inlineStr">
+        <is>
+          <t>F-388</t>
+        </is>
+      </c>
+      <c r="X321" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y321" s="19" t="n"/>
+      <c r="Z321" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA321" s="19" t="n"/>
+      <c r="AB321" s="19" t="n"/>
+      <c r="AC321" s="19" t="n"/>
+      <c r="AD321" s="19" t="n"/>
+      <c r="AE321" s="20" t="n"/>
+      <c r="AF321" s="21">
+        <f>IF(K321="","",K321*AE321)</f>
+        <v/>
+      </c>
+      <c r="AG321" s="19" t="n"/>
+      <c r="AH321" s="19" t="n"/>
+      <c r="AI321" s="19" t="n"/>
+      <c r="AJ321" s="19" t="n"/>
+      <c r="AK321" s="19" t="n"/>
+      <c r="AL321" s="19" t="n"/>
+      <c r="AM321" s="16" t="inlineStr">
+        <is>
+          <t>2 Spiegel – abgebildet ist einer davon.</t>
+        </is>
+      </c>
+      <c r="AN321" s="22" t="n"/>
+    </row>
+    <row r="322" ht="30" customHeight="1">
+      <c r="A322" s="15" t="inlineStr">
+        <is>
+          <t>BU03-03</t>
+        </is>
+      </c>
+      <c r="B322" s="15" t="n"/>
+      <c r="C322" s="15" t="n"/>
+      <c r="D322" s="15" t="inlineStr">
+        <is>
+          <t>BU03</t>
+        </is>
+      </c>
+      <c r="E322" s="15" t="inlineStr">
+        <is>
+          <t>Schuhregal schwarz mit Chromstangen</t>
+        </is>
+      </c>
+      <c r="F322" s="16" t="inlineStr">
+        <is>
+          <t>Niedriges Schuhregal aus schwarz lackiertem Holz mit schwarzer Deckplatte und drei Ebenen aus verchromten Rundstangen, auch als Sitzbank nutzbar.</t>
+        </is>
+      </c>
+      <c r="G322" s="15" t="inlineStr">
+        <is>
+          <t>Möbel</t>
+        </is>
+      </c>
+      <c r="H322" s="15" t="inlineStr">
+        <is>
+          <t>Flur 3</t>
+        </is>
+      </c>
+      <c r="I322" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J322" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K322" s="17" t="n"/>
+      <c r="L322" s="18">
+        <f>J322-IF(K322="",0,K322)</f>
+        <v/>
+      </c>
+      <c r="M322" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N322" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O322" s="19" t="n"/>
+      <c r="P322" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q322" s="19" t="n"/>
+      <c r="R322" s="20" t="n"/>
+      <c r="S322" s="20" t="n">
+        <v>25</v>
+      </c>
+      <c r="T322" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U322" s="21">
+        <f>L322*S322</f>
+        <v/>
+      </c>
+      <c r="V322" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W322" s="15" t="inlineStr">
+        <is>
+          <t>F-389</t>
+        </is>
+      </c>
+      <c r="X322" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y322" s="19" t="n"/>
+      <c r="Z322" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA322" s="19" t="n"/>
+      <c r="AB322" s="19" t="n"/>
+      <c r="AC322" s="19" t="n"/>
+      <c r="AD322" s="19" t="n"/>
+      <c r="AE322" s="20" t="n"/>
+      <c r="AF322" s="21">
+        <f>IF(K322="","",K322*AE322)</f>
+        <v/>
+      </c>
+      <c r="AG322" s="19" t="n"/>
+      <c r="AH322" s="19" t="n"/>
+      <c r="AI322" s="19" t="n"/>
+      <c r="AJ322" s="19" t="n"/>
+      <c r="AK322" s="19" t="n"/>
+      <c r="AL322" s="19" t="n"/>
+      <c r="AM322" s="16" t="inlineStr">
+        <is>
+          <t>2 Regale – abgebildet ist eines davon.</t>
+        </is>
+      </c>
+      <c r="AN322" s="22" t="n"/>
+    </row>
+    <row r="323" ht="30" customHeight="1">
+      <c r="A323" s="15" t="inlineStr">
+        <is>
+          <t>BU03-04</t>
+        </is>
+      </c>
+      <c r="B323" s="15" t="n"/>
+      <c r="C323" s="15" t="n"/>
+      <c r="D323" s="15" t="inlineStr">
+        <is>
+          <t>BU03</t>
+        </is>
+      </c>
+      <c r="E323" s="15" t="inlineStr">
+        <is>
+          <t>Metallregal weiß, vier Böden</t>
+        </is>
+      </c>
+      <c r="F323" s="16" t="inlineStr">
+        <is>
+          <t>Offenes Regal mit weißem Metallgestell, Kreuzstrebe auf der Rückseite und vier weißen Böden.</t>
+        </is>
+      </c>
+      <c r="G323" s="15" t="inlineStr">
+        <is>
+          <t>Möbel</t>
+        </is>
+      </c>
+      <c r="H323" s="15" t="inlineStr">
+        <is>
+          <t>Flur 3</t>
+        </is>
+      </c>
+      <c r="I323" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J323" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K323" s="17" t="n"/>
+      <c r="L323" s="18">
+        <f>J323-IF(K323="",0,K323)</f>
+        <v/>
+      </c>
+      <c r="M323" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N323" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O323" s="19" t="n"/>
+      <c r="P323" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q323" s="19" t="n"/>
+      <c r="R323" s="20" t="n"/>
+      <c r="S323" s="20" t="n">
+        <v>35</v>
+      </c>
+      <c r="T323" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U323" s="21">
+        <f>L323*S323</f>
+        <v/>
+      </c>
+      <c r="V323" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W323" s="15" t="inlineStr">
+        <is>
+          <t>F-390</t>
+        </is>
+      </c>
+      <c r="X323" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y323" s="19" t="n"/>
+      <c r="Z323" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA323" s="19" t="n"/>
+      <c r="AB323" s="19" t="n"/>
+      <c r="AC323" s="19" t="n"/>
+      <c r="AD323" s="19" t="n"/>
+      <c r="AE323" s="20" t="n"/>
+      <c r="AF323" s="21">
+        <f>IF(K323="","",K323*AE323)</f>
+        <v/>
+      </c>
+      <c r="AG323" s="19" t="n"/>
+      <c r="AH323" s="19" t="n"/>
+      <c r="AI323" s="19" t="n"/>
+      <c r="AJ323" s="19" t="n"/>
+      <c r="AK323" s="19" t="n"/>
+      <c r="AL323" s="19" t="n"/>
+      <c r="AM323" s="16" t="inlineStr">
+        <is>
+          <t>2 Regale – abgebildet ist eines davon.</t>
+        </is>
+      </c>
+      <c r="AN323" s="22" t="n"/>
+    </row>
+    <row r="324" ht="30" customHeight="1">
+      <c r="A324" s="15" t="inlineStr">
+        <is>
+          <t>BU03-05</t>
+        </is>
+      </c>
+      <c r="B324" s="15" t="n"/>
+      <c r="C324" s="15" t="n"/>
+      <c r="D324" s="15" t="inlineStr">
+        <is>
+          <t>BU03</t>
+        </is>
+      </c>
+      <c r="E324" s="15" t="inlineStr">
+        <is>
+          <t>Schuhschrank weiß mit Klappfächern</t>
+        </is>
+      </c>
+      <c r="F324" s="16" t="inlineStr">
+        <is>
+          <t>Schmaler Schuhschrank in Weiß mit zwei Klappfächern und schwarzen Knöpfen. Die Schuhablagen sind innen verschmutzt und an den Kanten abgestoßen.</t>
+        </is>
+      </c>
+      <c r="G324" s="15" t="inlineStr">
+        <is>
+          <t>Möbel</t>
+        </is>
+      </c>
+      <c r="H324" s="15" t="inlineStr">
+        <is>
+          <t>Flur 3</t>
+        </is>
+      </c>
+      <c r="I324" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J324" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K324" s="17" t="n"/>
+      <c r="L324" s="18">
+        <f>J324-IF(K324="",0,K324)</f>
+        <v/>
+      </c>
+      <c r="M324" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N324" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O324" s="19" t="n"/>
+      <c r="P324" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q324" s="19" t="n"/>
+      <c r="R324" s="20" t="n"/>
+      <c r="S324" s="20" t="n">
+        <v>60</v>
+      </c>
+      <c r="T324" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U324" s="21">
+        <f>L324*S324</f>
+        <v/>
+      </c>
+      <c r="V324" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W324" s="15" t="inlineStr">
+        <is>
+          <t>F-391</t>
+        </is>
+      </c>
+      <c r="X324" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y324" s="19" t="n"/>
+      <c r="Z324" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA324" s="19" t="n"/>
+      <c r="AB324" s="19" t="n"/>
+      <c r="AC324" s="19" t="n"/>
+      <c r="AD324" s="19" t="n"/>
+      <c r="AE324" s="20" t="n"/>
+      <c r="AF324" s="21">
+        <f>IF(K324="","",K324*AE324)</f>
+        <v/>
+      </c>
+      <c r="AG324" s="19" t="n"/>
+      <c r="AH324" s="19" t="n"/>
+      <c r="AI324" s="19" t="n"/>
+      <c r="AJ324" s="19" t="n"/>
+      <c r="AK324" s="19" t="n"/>
+      <c r="AL324" s="19" t="n"/>
+      <c r="AM324" s="16" t="inlineStr">
+        <is>
+          <t>1 Schrank.</t>
+        </is>
+      </c>
+      <c r="AN324" s="22" t="n"/>
+    </row>
+    <row r="325" ht="30" customHeight="1">
+      <c r="A325" s="15" t="inlineStr">
+        <is>
+          <t>BU03-06</t>
+        </is>
+      </c>
+      <c r="B325" s="15" t="n"/>
+      <c r="C325" s="15" t="n"/>
+      <c r="D325" s="15" t="inlineStr">
+        <is>
+          <t>BU03</t>
+        </is>
+      </c>
+      <c r="E325" s="15" t="inlineStr">
+        <is>
+          <t>Wäschekorb anthrazit mit Deckel, hoch</t>
+        </is>
+      </c>
+      <c r="F325" s="16" t="inlineStr">
+        <is>
+          <t>Hoher Wäschekorb aus Kunststoff in Flechtoptik, anthrazit, nach unten verjüngt, mit aufklappbarem Deckel und Griffloch.</t>
+        </is>
+      </c>
+      <c r="G325" s="15" t="inlineStr">
+        <is>
+          <t>Sonstiges</t>
+        </is>
+      </c>
+      <c r="H325" s="15" t="inlineStr">
+        <is>
+          <t>Flur 3</t>
+        </is>
+      </c>
+      <c r="I325" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J325" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K325" s="17" t="n"/>
+      <c r="L325" s="18">
+        <f>J325-IF(K325="",0,K325)</f>
+        <v/>
+      </c>
+      <c r="M325" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N325" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O325" s="19" t="n"/>
+      <c r="P325" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q325" s="19" t="n"/>
+      <c r="R325" s="20" t="n"/>
+      <c r="S325" s="20" t="n">
+        <v>12</v>
+      </c>
+      <c r="T325" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U325" s="21">
+        <f>L325*S325</f>
+        <v/>
+      </c>
+      <c r="V325" s="15" t="inlineStr">
+        <is>
+          <t>Versand möglich</t>
+        </is>
+      </c>
+      <c r="W325" s="15" t="inlineStr">
+        <is>
+          <t>F-392</t>
+        </is>
+      </c>
+      <c r="X325" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y325" s="19" t="n"/>
+      <c r="Z325" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA325" s="19" t="n"/>
+      <c r="AB325" s="19" t="n"/>
+      <c r="AC325" s="19" t="n"/>
+      <c r="AD325" s="19" t="n"/>
+      <c r="AE325" s="20" t="n"/>
+      <c r="AF325" s="21">
+        <f>IF(K325="","",K325*AE325)</f>
+        <v/>
+      </c>
+      <c r="AG325" s="19" t="n"/>
+      <c r="AH325" s="19" t="n"/>
+      <c r="AI325" s="19" t="n"/>
+      <c r="AJ325" s="19" t="n"/>
+      <c r="AK325" s="19" t="n"/>
+      <c r="AL325" s="19" t="n"/>
+      <c r="AM325" s="16" t="inlineStr">
+        <is>
+          <t>1 Korb. Drei niedrigere Wäschekörbe stehen unter NE02-03.</t>
+        </is>
+      </c>
+      <c r="AN325" s="22" t="n"/>
+    </row>
+    <row r="326" ht="30" customHeight="1">
+      <c r="A326" s="15" t="inlineStr">
+        <is>
+          <t>BU03-07</t>
+        </is>
+      </c>
+      <c r="B326" s="15" t="n"/>
+      <c r="C326" s="15" t="n"/>
+      <c r="D326" s="15" t="inlineStr">
+        <is>
+          <t>BU03</t>
+        </is>
+      </c>
+      <c r="E326" s="15" t="inlineStr">
+        <is>
+          <t>Tischleuchte Holzgestell mit Stoffschirm</t>
+        </is>
+      </c>
+      <c r="F326" s="16" t="inlineStr">
+        <is>
+          <t>Tischleuchte mit dreieckigem Gestell aus hellem Holz und zylindrischem Stoffschirm in Hellgrau, mit Schnurschalter.</t>
+        </is>
+      </c>
+      <c r="G326" s="15" t="inlineStr">
+        <is>
+          <t>Leuchten</t>
+        </is>
+      </c>
+      <c r="H326" s="15" t="inlineStr">
+        <is>
+          <t>Flur 3</t>
+        </is>
+      </c>
+      <c r="I326" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J326" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K326" s="17" t="n"/>
+      <c r="L326" s="18">
+        <f>J326-IF(K326="",0,K326)</f>
+        <v/>
+      </c>
+      <c r="M326" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N326" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O326" s="19" t="n"/>
+      <c r="P326" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q326" s="19" t="n"/>
+      <c r="R326" s="20" t="n"/>
+      <c r="S326" s="20" t="n">
+        <v>25</v>
+      </c>
+      <c r="T326" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U326" s="21">
+        <f>L326*S326</f>
+        <v/>
+      </c>
+      <c r="V326" s="15" t="inlineStr">
+        <is>
+          <t>Versand möglich</t>
+        </is>
+      </c>
+      <c r="W326" s="15" t="inlineStr">
+        <is>
+          <t>F-393</t>
+        </is>
+      </c>
+      <c r="X326" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y326" s="19" t="n"/>
+      <c r="Z326" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA326" s="19" t="n"/>
+      <c r="AB326" s="19" t="n"/>
+      <c r="AC326" s="19" t="n"/>
+      <c r="AD326" s="19" t="n"/>
+      <c r="AE326" s="20" t="n"/>
+      <c r="AF326" s="21">
+        <f>IF(K326="","",K326*AE326)</f>
+        <v/>
+      </c>
+      <c r="AG326" s="19" t="n"/>
+      <c r="AH326" s="19" t="n"/>
+      <c r="AI326" s="19" t="n"/>
+      <c r="AJ326" s="19" t="n"/>
+      <c r="AK326" s="19" t="n"/>
+      <c r="AL326" s="19" t="n"/>
+      <c r="AM326" s="16" t="inlineStr">
+        <is>
+          <t>1 Leuchte ohne Leuchtmittel. Auf dem Erfassungsblatt als Stehlampe geführt – es ist eine Tischleuchte.</t>
+        </is>
+      </c>
+      <c r="AN326" s="22" t="n"/>
+    </row>
+    <row r="327" ht="30" customHeight="1">
+      <c r="A327" s="15" t="inlineStr">
+        <is>
+          <t>BU03-08</t>
+        </is>
+      </c>
+      <c r="B327" s="15" t="n"/>
+      <c r="C327" s="15" t="n"/>
+      <c r="D327" s="15" t="inlineStr">
+        <is>
+          <t>BU03</t>
+        </is>
+      </c>
+      <c r="E327" s="15" t="inlineStr">
+        <is>
+          <t>Beistelltisch rund türkis mit Hairpin-Beinen</t>
+        </is>
+      </c>
+      <c r="F327" s="16" t="inlineStr">
+        <is>
+          <t>Kleiner runder Beistelltisch mit türkis lackierter Holzplatte auf drei schwarzen Hairpin-Beinen aus Rundstahl. Die Platte ist leicht verkratzt.</t>
+        </is>
+      </c>
+      <c r="G327" s="15" t="inlineStr">
+        <is>
+          <t>Möbel</t>
+        </is>
+      </c>
+      <c r="H327" s="15" t="inlineStr">
+        <is>
+          <t>Flur 3</t>
+        </is>
+      </c>
+      <c r="I327" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J327" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K327" s="17" t="n"/>
+      <c r="L327" s="18">
+        <f>J327-IF(K327="",0,K327)</f>
+        <v/>
+      </c>
+      <c r="M327" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N327" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O327" s="19" t="n"/>
+      <c r="P327" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q327" s="19" t="n"/>
+      <c r="R327" s="20" t="n"/>
+      <c r="S327" s="20" t="n">
+        <v>35</v>
+      </c>
+      <c r="T327" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U327" s="21">
+        <f>L327*S327</f>
+        <v/>
+      </c>
+      <c r="V327" s="15" t="inlineStr">
+        <is>
+          <t>Versand möglich</t>
+        </is>
+      </c>
+      <c r="W327" s="15" t="inlineStr">
+        <is>
+          <t>F-394</t>
+        </is>
+      </c>
+      <c r="X327" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y327" s="19" t="n"/>
+      <c r="Z327" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA327" s="19" t="n"/>
+      <c r="AB327" s="19" t="n"/>
+      <c r="AC327" s="19" t="n"/>
+      <c r="AD327" s="19" t="n"/>
+      <c r="AE327" s="20" t="n"/>
+      <c r="AF327" s="21">
+        <f>IF(K327="","",K327*AE327)</f>
+        <v/>
+      </c>
+      <c r="AG327" s="19" t="n"/>
+      <c r="AH327" s="19" t="n"/>
+      <c r="AI327" s="19" t="n"/>
+      <c r="AJ327" s="19" t="n"/>
+      <c r="AK327" s="19" t="n"/>
+      <c r="AL327" s="19" t="n"/>
+      <c r="AM327" s="16" t="inlineStr">
+        <is>
+          <t>1 Tisch.</t>
+        </is>
+      </c>
+      <c r="AN327" s="22" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:AN320"/>
+  <autoFilter ref="A2:AN327"/>
   <mergeCells count="7">
     <mergeCell ref="AI1:AL1"/>
     <mergeCell ref="V1:AD1"/>
@@ -40071,7 +40896,7 @@
     <mergeCell ref="AE1:AH1"/>
     <mergeCell ref="AM1:AN1"/>
   </mergeCells>
-  <conditionalFormatting sqref="Z3:Z320">
+  <conditionalFormatting sqref="Z3:Z327">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"reserviert"</formula>
     </cfRule>
@@ -40082,12 +40907,12 @@
       <formula>"verkauft"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I3:I320">
+  <conditionalFormatting sqref="I3:I327">
     <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
       <formula>"A"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P3:P320">
+  <conditionalFormatting sqref="P3:P327">
     <cfRule type="cellIs" priority="5" operator="equal" dxfId="4">
       <formula>"entfällt"</formula>
     </cfRule>
@@ -40140,7 +40965,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D93"/>
+  <dimension ref="A1:D94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -40178,7 +41003,7 @@
         </is>
       </c>
       <c r="B5" s="27">
-        <f>COUNTA(Artikelstamm!$A$3:$A$320)</f>
+        <f>COUNTA(Artikelstamm!$A$3:$A$327)</f>
         <v/>
       </c>
     </row>
@@ -40189,7 +41014,7 @@
         </is>
       </c>
       <c r="B6" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$320,"verfügbar")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$327,"verfügbar")</f>
         <v/>
       </c>
     </row>
@@ -40200,7 +41025,7 @@
         </is>
       </c>
       <c r="B7" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$320,"reserviert")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$327,"reserviert")</f>
         <v/>
       </c>
     </row>
@@ -40211,7 +41036,7 @@
         </is>
       </c>
       <c r="B8" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$320,"teilverkauft")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$327,"teilverkauft")</f>
         <v/>
       </c>
     </row>
@@ -40222,7 +41047,7 @@
         </is>
       </c>
       <c r="B9" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$320,"verkauft")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$327,"verkauft")</f>
         <v/>
       </c>
     </row>
@@ -40233,7 +41058,7 @@
         </is>
       </c>
       <c r="B10" s="27">
-        <f>SUM(Artikelstamm!$L$3:$L$320)</f>
+        <f>SUM(Artikelstamm!$L$3:$L$327)</f>
         <v/>
       </c>
     </row>
@@ -40244,7 +41069,7 @@
         </is>
       </c>
       <c r="B11" s="29">
-        <f>SUM(Artikelstamm!$U$3:$U$320)</f>
+        <f>SUM(Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
@@ -40262,7 +41087,7 @@
         </is>
       </c>
       <c r="B13" s="27">
-        <f>SUM(Artikelstamm!$K$3:$K$320)</f>
+        <f>SUM(Artikelstamm!$K$3:$K$327)</f>
         <v/>
       </c>
     </row>
@@ -40273,7 +41098,7 @@
         </is>
       </c>
       <c r="B14" s="30">
-        <f>SUMPRODUCT(Artikelstamm!$K$3:$K$320,Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT(Artikelstamm!$K$3:$K$327,Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
     </row>
@@ -40306,7 +41131,7 @@
         </is>
       </c>
       <c r="B17" s="30">
-        <f>SUMPRODUCT((Artikelstamm!$AJ$3:$AJ$320="bezahlt")*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AJ$3:$AJ$327="bezahlt")*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
     </row>
@@ -40335,7 +41160,7 @@
         </is>
       </c>
       <c r="B21" s="31">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$320,"*verkauft",Artikelstamm!$AI$3:$AI$320,"")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$327,"*verkauft",Artikelstamm!$AI$3:$AI$327,"")</f>
         <v/>
       </c>
     </row>
@@ -40346,7 +41171,7 @@
         </is>
       </c>
       <c r="B22" s="31">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$320,"*verkauft",Artikelstamm!$AJ$3:$AJ$320,"offen")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$327,"*verkauft",Artikelstamm!$AJ$3:$AJ$327,"offen")</f>
         <v/>
       </c>
     </row>
@@ -40357,7 +41182,7 @@
         </is>
       </c>
       <c r="B23" s="27">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$320,"reserviert",Artikelstamm!$AL$3:$AL$320,"")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$327,"reserviert",Artikelstamm!$AL$3:$AL$327,"")</f>
         <v/>
       </c>
     </row>
@@ -40368,7 +41193,7 @@
         </is>
       </c>
       <c r="B24" s="27">
-        <f>COUNTIFS(Artikelstamm!$S$3:$S$320,"")</f>
+        <f>COUNTIFS(Artikelstamm!$S$3:$S$327,"")</f>
         <v/>
       </c>
     </row>
@@ -40379,7 +41204,7 @@
         </is>
       </c>
       <c r="B25" s="27">
-        <f>COUNTIFS(Artikelstamm!$O$3:$O$320,"")</f>
+        <f>COUNTIFS(Artikelstamm!$O$3:$O$327,"")</f>
         <v/>
       </c>
     </row>
@@ -40419,15 +41244,15 @@
         </is>
       </c>
       <c r="B30" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$320,$A30)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$327,$A30)</f>
         <v/>
       </c>
       <c r="C30" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$320=$A30)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$327=$A30)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D30" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$320,$A30,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$327,$A30,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
@@ -40438,15 +41263,15 @@
         </is>
       </c>
       <c r="B31" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$320,$A31)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$327,$A31)</f>
         <v/>
       </c>
       <c r="C31" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$320=$A31)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$327=$A31)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D31" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$320,$A31,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$327,$A31,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
@@ -40457,15 +41282,15 @@
         </is>
       </c>
       <c r="B32" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$320,$A32)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$327,$A32)</f>
         <v/>
       </c>
       <c r="C32" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$320=$A32)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$327=$A32)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D32" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$320,$A32,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$327,$A32,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
@@ -40524,15 +41349,15 @@
         </is>
       </c>
       <c r="B37" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$320,$A37)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$327,$A37)</f>
         <v/>
       </c>
       <c r="C37" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$320=$A37)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$327=$A37)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D37" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$320,$A37,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$327,$A37,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
@@ -40543,15 +41368,15 @@
         </is>
       </c>
       <c r="B38" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$320,$A38)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$327,$A38)</f>
         <v/>
       </c>
       <c r="C38" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$320=$A38)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$327=$A38)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D38" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$320,$A38,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$327,$A38,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
@@ -40562,15 +41387,15 @@
         </is>
       </c>
       <c r="B39" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$320,$A39)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$327,$A39)</f>
         <v/>
       </c>
       <c r="C39" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$320=$A39)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$327=$A39)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D39" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$320,$A39,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$327,$A39,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
@@ -40581,15 +41406,15 @@
         </is>
       </c>
       <c r="B40" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$320,$A40)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$327,$A40)</f>
         <v/>
       </c>
       <c r="C40" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$320=$A40)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$327=$A40)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D40" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$320,$A40,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$327,$A40,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
@@ -40600,15 +41425,15 @@
         </is>
       </c>
       <c r="B41" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$320,$A41)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$327,$A41)</f>
         <v/>
       </c>
       <c r="C41" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$320=$A41)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$327=$A41)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D41" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$320,$A41,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$327,$A41,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
@@ -40619,15 +41444,15 @@
         </is>
       </c>
       <c r="B42" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$320,$A42)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$327,$A42)</f>
         <v/>
       </c>
       <c r="C42" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$320=$A42)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$327=$A42)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D42" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$320,$A42,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$327,$A42,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
@@ -40638,15 +41463,15 @@
         </is>
       </c>
       <c r="B43" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$320,$A43)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$327,$A43)</f>
         <v/>
       </c>
       <c r="C43" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$320=$A43)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$327=$A43)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D43" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$320,$A43,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$327,$A43,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
@@ -40657,15 +41482,15 @@
         </is>
       </c>
       <c r="B44" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$320,$A44)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$327,$A44)</f>
         <v/>
       </c>
       <c r="C44" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$320=$A44)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$327=$A44)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D44" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$320,$A44,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$327,$A44,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
@@ -40676,15 +41501,15 @@
         </is>
       </c>
       <c r="B45" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$320,$A45)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$327,$A45)</f>
         <v/>
       </c>
       <c r="C45" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$320=$A45)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$327=$A45)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D45" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$320,$A45,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$327,$A45,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
@@ -40695,15 +41520,15 @@
         </is>
       </c>
       <c r="B46" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$320,$A46)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$327,$A46)</f>
         <v/>
       </c>
       <c r="C46" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$320=$A46)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$327=$A46)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D46" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$320,$A46,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$327,$A46,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
@@ -40714,15 +41539,15 @@
         </is>
       </c>
       <c r="B47" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$320,$A47)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$327,$A47)</f>
         <v/>
       </c>
       <c r="C47" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$320=$A47)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$327=$A47)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D47" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$320,$A47,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$327,$A47,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
@@ -40733,15 +41558,15 @@
         </is>
       </c>
       <c r="B48" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$320,$A48)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$327,$A48)</f>
         <v/>
       </c>
       <c r="C48" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$320=$A48)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$327=$A48)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D48" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$320,$A48,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$327,$A48,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
@@ -40752,15 +41577,15 @@
         </is>
       </c>
       <c r="B49" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$320,$A49)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$327,$A49)</f>
         <v/>
       </c>
       <c r="C49" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$320=$A49)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$327=$A49)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D49" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$320,$A49,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$327,$A49,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
@@ -40771,15 +41596,15 @@
         </is>
       </c>
       <c r="B50" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$320,$A50)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$327,$A50)</f>
         <v/>
       </c>
       <c r="C50" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$320=$A50)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$327=$A50)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D50" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$320,$A50,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$327,$A50,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
@@ -40838,15 +41663,15 @@
         </is>
       </c>
       <c r="B55" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A55)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$327,$A55)</f>
         <v/>
       </c>
       <c r="C55" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A55)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$327=$A55)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D55" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A55,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$327,$A55,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
@@ -40857,15 +41682,15 @@
         </is>
       </c>
       <c r="B56" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A56)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$327,$A56)</f>
         <v/>
       </c>
       <c r="C56" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A56)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$327=$A56)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D56" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A56,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$327,$A56,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
@@ -40876,15 +41701,15 @@
         </is>
       </c>
       <c r="B57" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A57)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$327,$A57)</f>
         <v/>
       </c>
       <c r="C57" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A57)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$327=$A57)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D57" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A57,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$327,$A57,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
@@ -40895,15 +41720,15 @@
         </is>
       </c>
       <c r="B58" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A58)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$327,$A58)</f>
         <v/>
       </c>
       <c r="C58" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A58)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$327=$A58)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D58" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A58,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$327,$A58,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
@@ -40914,15 +41739,15 @@
         </is>
       </c>
       <c r="B59" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A59)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$327,$A59)</f>
         <v/>
       </c>
       <c r="C59" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A59)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$327=$A59)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D59" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A59,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$327,$A59,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
@@ -40933,15 +41758,15 @@
         </is>
       </c>
       <c r="B60" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A60)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$327,$A60)</f>
         <v/>
       </c>
       <c r="C60" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A60)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$327=$A60)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D60" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A60,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$327,$A60,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
@@ -40952,562 +41777,581 @@
         </is>
       </c>
       <c r="B61" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A61)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$327,$A61)</f>
         <v/>
       </c>
       <c r="C61" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A61)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$327=$A61)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D61" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A61,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$327,$A61,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="26" t="inlineStr">
         <is>
-          <t>Galerie</t>
+          <t>Flur 3</t>
         </is>
       </c>
       <c r="B62" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A62)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$327,$A62)</f>
         <v/>
       </c>
       <c r="C62" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A62)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$327=$A62)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D62" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A62,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$327,$A62,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="26" t="inlineStr">
         <is>
-          <t>Garage</t>
+          <t>Galerie</t>
         </is>
       </c>
       <c r="B63" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A63)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$327,$A63)</f>
         <v/>
       </c>
       <c r="C63" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A63)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$327=$A63)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D63" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A63,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$327,$A63,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="26" t="inlineStr">
         <is>
-          <t>Gartenanlage</t>
+          <t>Garage</t>
         </is>
       </c>
       <c r="B64" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A64)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$327,$A64)</f>
         <v/>
       </c>
       <c r="C64" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A64)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$327=$A64)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D64" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A64,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$327,$A64,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="26" t="inlineStr">
         <is>
-          <t>Gruppenraum</t>
+          <t>Gartenanlage</t>
         </is>
       </c>
       <c r="B65" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A65)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$327,$A65)</f>
         <v/>
       </c>
       <c r="C65" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A65)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$327=$A65)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D65" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A65,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$327,$A65,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="26" t="inlineStr">
         <is>
-          <t>Gruppenraum 2</t>
+          <t>Gruppenraum</t>
         </is>
       </c>
       <c r="B66" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A66)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$327,$A66)</f>
         <v/>
       </c>
       <c r="C66" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A66)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$327=$A66)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D66" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A66,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$327,$A66,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="26" t="inlineStr">
         <is>
-          <t>Gruppenraum 4</t>
+          <t>Gruppenraum 2</t>
         </is>
       </c>
       <c r="B67" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A67)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$327,$A67)</f>
         <v/>
       </c>
       <c r="C67" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A67)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$327=$A67)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D67" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A67,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$327,$A67,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="26" t="inlineStr">
         <is>
-          <t>Gruppenraum 5</t>
+          <t>Gruppenraum 4</t>
         </is>
       </c>
       <c r="B68" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A68)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$327,$A68)</f>
         <v/>
       </c>
       <c r="C68" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A68)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$327=$A68)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D68" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A68,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$327,$A68,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="26" t="inlineStr">
         <is>
-          <t>Klassenzimmer</t>
+          <t>Gruppenraum 5</t>
         </is>
       </c>
       <c r="B69" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A69)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$327,$A69)</f>
         <v/>
       </c>
       <c r="C69" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A69)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$327=$A69)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D69" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A69,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$327,$A69,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="26" t="inlineStr">
         <is>
-          <t>Küche</t>
+          <t>Klassenzimmer</t>
         </is>
       </c>
       <c r="B70" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A70)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$327,$A70)</f>
         <v/>
       </c>
       <c r="C70" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A70)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$327=$A70)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D70" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A70,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$327,$A70,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="26" t="inlineStr">
         <is>
-          <t>Material / Turnraum</t>
+          <t>Küche</t>
         </is>
       </c>
       <c r="B71" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A71)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$327,$A71)</f>
         <v/>
       </c>
       <c r="C71" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A71)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$327=$A71)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D71" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A71,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$327,$A71,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="26" t="inlineStr">
         <is>
-          <t>Personal</t>
+          <t>Material / Turnraum</t>
         </is>
       </c>
       <c r="B72" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A72)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$327,$A72)</f>
         <v/>
       </c>
       <c r="C72" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A72)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$327=$A72)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D72" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A72,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$327,$A72,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="26" t="inlineStr">
         <is>
-          <t>Ruhe- / Schlafraum</t>
+          <t>Personal</t>
         </is>
       </c>
       <c r="B73" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A73)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$327,$A73)</f>
         <v/>
       </c>
       <c r="C73" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A73)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$327=$A73)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D73" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A73,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$327,$A73,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="26" t="inlineStr">
         <is>
-          <t>Schlafraum 4</t>
+          <t>Ruhe- / Schlafraum</t>
         </is>
       </c>
       <c r="B74" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A74)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$327,$A74)</f>
         <v/>
       </c>
       <c r="C74" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A74)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$327=$A74)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D74" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A74,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$327,$A74,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="26" t="inlineStr">
         <is>
-          <t>Schlafraum 5</t>
+          <t>Schlafraum 4</t>
         </is>
       </c>
       <c r="B75" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A75)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$327,$A75)</f>
         <v/>
       </c>
       <c r="C75" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A75)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$327=$A75)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D75" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A75,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$327,$A75,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="26" t="inlineStr">
         <is>
-          <t>Speisesaal</t>
+          <t>Schlafraum 5</t>
         </is>
       </c>
       <c r="B76" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A76)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$327,$A76)</f>
         <v/>
       </c>
       <c r="C76" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A76)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$327=$A76)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D76" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A76,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$327,$A76,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="26" t="inlineStr">
         <is>
-          <t>Terrasse</t>
+          <t>Speisesaal</t>
         </is>
       </c>
       <c r="B77" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A77)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$327,$A77)</f>
         <v/>
       </c>
       <c r="C77" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A77)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$327=$A77)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D77" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A77,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$327,$A77,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="26" t="inlineStr">
         <is>
-          <t>Treppenraum 1</t>
+          <t>Terrasse</t>
         </is>
       </c>
       <c r="B78" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A78)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$327,$A78)</f>
         <v/>
       </c>
       <c r="C78" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A78)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$327=$A78)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D78" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A78,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$327,$A78,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="26" t="inlineStr">
         <is>
-          <t>Turnraum</t>
+          <t>Treppenraum 1</t>
         </is>
       </c>
       <c r="B79" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A79)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$327,$A79)</f>
         <v/>
       </c>
       <c r="C79" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A79)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$327=$A79)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D79" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A79,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$327,$A79,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="26" t="inlineStr">
         <is>
-          <t>WC</t>
+          <t>Turnraum</t>
         </is>
       </c>
       <c r="B80" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A80)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$327,$A80)</f>
         <v/>
       </c>
       <c r="C80" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A80)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$327=$A80)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D80" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A80,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$327,$A80,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="26" t="inlineStr">
         <is>
-          <t>WC Personal</t>
+          <t>WC</t>
         </is>
       </c>
       <c r="B81" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A81)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$327,$A81)</f>
         <v/>
       </c>
       <c r="C81" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A81)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$327=$A81)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
       <c r="D81" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A81,Artikelstamm!$U$3:$U$320)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$327,$A81,Artikelstamm!$U$3:$U$327)</f>
         <v/>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="26" t="inlineStr">
         <is>
+          <t>WC Personal</t>
+        </is>
+      </c>
+      <c r="B82" s="33">
+        <f>COUNTIF(Artikelstamm!$H$3:$H$327,$A82)</f>
+        <v/>
+      </c>
+      <c r="C82" s="34">
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$327=$A82)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
+        <v/>
+      </c>
+      <c r="D82" s="34">
+        <f>SUMIF(Artikelstamm!$H$3:$H$327,$A82,Artikelstamm!$U$3:$U$327)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="26" t="inlineStr">
+        <is>
           <t>Werkraum</t>
         </is>
       </c>
-      <c r="B82" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$320,$A82)</f>
-        <v/>
-      </c>
-      <c r="C82" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$320=$A82)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
-        <v/>
-      </c>
-      <c r="D82" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$320,$A82,Artikelstamm!$U$3:$U$320)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="28" t="inlineStr">
+      <c r="B83" s="33">
+        <f>COUNTIF(Artikelstamm!$H$3:$H$327,$A83)</f>
+        <v/>
+      </c>
+      <c r="C83" s="34">
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$327=$A83)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
+        <v/>
+      </c>
+      <c r="D83" s="34">
+        <f>SUMIF(Artikelstamm!$H$3:$H$327,$A83,Artikelstamm!$U$3:$U$327)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="28" t="inlineStr">
         <is>
           <t>Summe</t>
         </is>
       </c>
-      <c r="B83" s="35">
-        <f>SUM(B55:B82)</f>
-        <v/>
-      </c>
-      <c r="C83" s="36">
-        <f>SUM(C55:C82)</f>
-        <v/>
-      </c>
-      <c r="D83" s="36">
-        <f>SUM(D55:D82)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" s="25" t="inlineStr">
+      <c r="B84" s="35">
+        <f>SUM(B55:B83)</f>
+        <v/>
+      </c>
+      <c r="C84" s="36">
+        <f>SUM(C55:C83)</f>
+        <v/>
+      </c>
+      <c r="D84" s="36">
+        <f>SUM(D55:D83)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="25" t="inlineStr">
         <is>
           <t>Nach Verkaufskanal</t>
         </is>
       </c>
     </row>
-    <row r="86">
-      <c r="A86" s="32" t="inlineStr">
+    <row r="87">
+      <c r="A87" s="32" t="inlineStr">
         <is>
           <t>Verkaufskanal</t>
         </is>
       </c>
-      <c r="B86" s="32" t="inlineStr">
+      <c r="B87" s="32" t="inlineStr">
         <is>
           <t>Positionen</t>
         </is>
       </c>
-      <c r="C86" s="32" t="inlineStr">
+      <c r="C87" s="32" t="inlineStr">
         <is>
           <t>Umsatz netto</t>
         </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="26" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
-      <c r="B87" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$320,$A87)</f>
-        <v/>
-      </c>
-      <c r="C87" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$320=$A87)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
-        <v/>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="26" t="inlineStr">
         <is>
-          <t>Kleinanzeigen</t>
+          <t>Klinik</t>
         </is>
       </c>
       <c r="B88" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$320,$A88)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$327,$A88)</f>
         <v/>
       </c>
       <c r="C88" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$320=$A88)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$327=$A88)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="26" t="inlineStr">
         <is>
-          <t>eBay</t>
+          <t>Kleinanzeigen</t>
         </is>
       </c>
       <c r="B89" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$320,$A89)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$327,$A89)</f>
         <v/>
       </c>
       <c r="C89" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$320=$A89)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$327=$A89)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="26" t="inlineStr">
         <is>
-          <t>Direkt</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="B90" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$320,$A90)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$327,$A90)</f>
         <v/>
       </c>
       <c r="C90" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$320=$A90)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$327=$A90)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="26" t="inlineStr">
         <is>
-          <t>Händler</t>
+          <t>Direkt</t>
         </is>
       </c>
       <c r="B91" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$320,$A91)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$327,$A91)</f>
         <v/>
       </c>
       <c r="C91" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$320=$A91)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$327=$A91)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
         <v/>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="26" t="inlineStr">
         <is>
+          <t>Händler</t>
+        </is>
+      </c>
+      <c r="B92" s="33">
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$327,$A92)</f>
+        <v/>
+      </c>
+      <c r="C92" s="34">
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$327=$A92)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="26" t="inlineStr">
+        <is>
           <t>Verkaufstag</t>
         </is>
       </c>
-      <c r="B92" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$320,$A92)</f>
-        <v/>
-      </c>
-      <c r="C92" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$320=$A92)*Artikelstamm!$K$3:$K$320*Artikelstamm!$AE$3:$AE$320)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" s="28" t="inlineStr">
+      <c r="B93" s="33">
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$327,$A93)</f>
+        <v/>
+      </c>
+      <c r="C93" s="34">
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$327=$A93)*Artikelstamm!$K$3:$K$327*Artikelstamm!$AE$3:$AE$327)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="28" t="inlineStr">
         <is>
           <t>Summe</t>
         </is>
       </c>
-      <c r="B93" s="35">
-        <f>SUM(B87:B92)</f>
-        <v/>
-      </c>
-      <c r="C93" s="36">
-        <f>SUM(C87:C92)</f>
+      <c r="B94" s="35">
+        <f>SUM(B88:B93)</f>
+        <v/>
+      </c>
+      <c r="C94" s="36">
+        <f>SUM(C88:C93)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
BU05 Schlafraum UG erfasst; Fadenbilder auf inaktiv
Raum BU05 (Bestandsgebaeude UG, Schlafraum, 29,00 m2) aus 14 Fotos und dem
Erfassungsblatt aufgenommen: 9 neue Positionen, eine Zusammenfassung.

  BU05-08 -> BA08-06  VS Schalenstuhl grau   9 -> 12

BU04-16 (Wanddeko Fadenbilder mit Spiegelpunkten) auf Aktiv = nein gesetzt -
laut Nutzerin nicht mehr vorhanden. Der offene Punkt entfaellt damit.

Foto F-411 maskiert: zwei Personen als Spiegelung in den Fensterscheiben.

Datenbasis 342 Positionen / 286 aktiv, pruefen.py 0 Fehler.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011yyfqhuiWGsaNy38oaNoGo
</commit_message>
<xml_diff>
--- a/ausgabe/01_Artikelstamm_kikripp.xlsx
+++ b/ausgabe/01_Artikelstamm_kikripp.xlsx
@@ -15,7 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Artikelstamm'!$A$2:$AN$335</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Artikelstamm'!$A$2:$AN$344</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1019,7 +1019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN335"/>
+  <dimension ref="A1:AN344"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5471,7 +5471,7 @@
       <c r="O36" s="19" t="n"/>
       <c r="P36" s="19" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nein</t>
         </is>
       </c>
       <c r="Q36" s="19" t="n"/>
@@ -5506,7 +5506,7 @@
       <c r="Y36" s="19" t="n"/>
       <c r="Z36" s="19" t="inlineStr">
         <is>
-          <t>verfügbar</t>
+          <t>entfällt</t>
         </is>
       </c>
       <c r="AA36" s="19" t="n"/>
@@ -5531,7 +5531,7 @@
       </c>
       <c r="AN36" s="22" t="inlineStr">
         <is>
-          <t>OFFEN: NICHT VEROEFFENTLICHEN, bis geklaert ist, ob das Set noch da ist. Auf dem Erfassungsblatt BU04 ist die Zeile durchgestrichen, die Nummer BU04-05 klebt jetzt auf den Hochstuehlen. Frueher BU04-05 / K-117.</t>
+          <t>Nicht mehr vorhanden – von der Nutzerin am 23.09.2026 bestaetigt. Frueher BU04-05 / K-117; die Nummer BU04-05 klebt jetzt auf den Hochstuehlen.</t>
         </is>
       </c>
     </row>
@@ -36810,7 +36810,11 @@
         </is>
       </c>
       <c r="B294" s="15" t="n"/>
-      <c r="C294" s="15" t="n"/>
+      <c r="C294" s="15" t="inlineStr">
+        <is>
+          <t>BU05-08</t>
+        </is>
+      </c>
       <c r="D294" s="15" t="inlineStr">
         <is>
           <t>BA08</t>
@@ -36823,7 +36827,7 @@
       </c>
       <c r="F294" s="16" t="inlineStr">
         <is>
-          <t>Schalenstuhl von VS (Vereinigte Spezialmöbelfabriken): graue Kunststoffschale mit Rautenstruktur und Griffloch in der Lehne, auf grauem Vierfußgestell aus Rohr. Farbspritzer aus dem Atelierbetrieb auf Sitz und Lehne.</t>
+          <t>Schalenstuhl von VS (Vereinigte Spezialmöbelfabriken): graue Kunststoffschale mit Rautenstruktur und Griffloch in der Lehne, auf grauem Vierfußgestell aus Rohr. Auf den Stühlen aus dem Atelier sind Farbspritzer.</t>
         </is>
       </c>
       <c r="G294" s="15" t="inlineStr">
@@ -36842,7 +36846,7 @@
         </is>
       </c>
       <c r="J294" s="17" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="K294" s="17" t="n"/>
       <c r="L294" s="18">
@@ -36921,10 +36925,14 @@
       <c r="AL294" s="19" t="n"/>
       <c r="AM294" s="16" t="inlineStr">
         <is>
-          <t>9 Stühle – abgebildet ist einer davon. Das Logo ist auf Foto F-346 zu sehen. Ein anderes VS-Modell auf Kufengestell steht unter NU02-04.</t>
-        </is>
-      </c>
-      <c r="AN294" s="22" t="n"/>
+          <t>12 Stühle insgesamt: 9 im Atelier (BA08-06) und 3 im Schlafraum im Untergeschoss (BU05-08). Nur die neun Stühle aus dem Atelier haben Farbspritzer; die drei aus dem Schlafraum sind sauber. Das Logo ist auf Foto F-346 zu sehen, ein sauberer Stuhl auf Foto F-418.</t>
+        </is>
+      </c>
+      <c r="AN294" s="22" t="inlineStr">
+        <is>
+          <t>Zusammengefasste Position über zwei Räume – Post-it-Nummer: BU05-08.</t>
+        </is>
+      </c>
     </row>
     <row r="295" ht="30" customHeight="1">
       <c r="A295" s="15" t="inlineStr">
@@ -41857,8 +41865,1091 @@
       </c>
       <c r="AN335" s="22" t="n"/>
     </row>
+    <row r="336" ht="30" customHeight="1">
+      <c r="A336" s="15" t="inlineStr">
+        <is>
+          <t>BU05-01</t>
+        </is>
+      </c>
+      <c r="B336" s="15" t="n"/>
+      <c r="C336" s="15" t="n"/>
+      <c r="D336" s="15" t="inlineStr">
+        <is>
+          <t>BU05</t>
+        </is>
+      </c>
+      <c r="E336" s="15" t="inlineStr">
+        <is>
+          <t>Spielhaus weiß mit Hochebene und Bett</t>
+        </is>
+      </c>
+      <c r="F336" s="16" t="inlineStr">
+        <is>
+          <t>Große Spielhaus-Konstruktion in Weiß: obere Spielebene mit Brüstung, grüner Tafel und Ablagefach, darunter eine Liegefläche mit Matratze. Eine Seitenwand trägt eine goldene Krone als Aufkleber.</t>
+        </is>
+      </c>
+      <c r="G336" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H336" s="15" t="inlineStr">
+        <is>
+          <t>Schlafraum</t>
+        </is>
+      </c>
+      <c r="I336" s="15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J336" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K336" s="17" t="n"/>
+      <c r="L336" s="18">
+        <f>J336-IF(K336="",0,K336)</f>
+        <v/>
+      </c>
+      <c r="M336" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N336" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O336" s="19" t="n"/>
+      <c r="P336" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q336" s="19" t="n"/>
+      <c r="R336" s="20" t="n"/>
+      <c r="S336" s="20" t="n">
+        <v>450</v>
+      </c>
+      <c r="T336" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U336" s="21">
+        <f>L336*S336</f>
+        <v/>
+      </c>
+      <c r="V336" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W336" s="15" t="inlineStr">
+        <is>
+          <t>F-409</t>
+        </is>
+      </c>
+      <c r="X336" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y336" s="19" t="n"/>
+      <c r="Z336" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA336" s="19" t="n"/>
+      <c r="AB336" s="19" t="n"/>
+      <c r="AC336" s="19" t="n"/>
+      <c r="AD336" s="19" t="n"/>
+      <c r="AE336" s="20" t="n"/>
+      <c r="AF336" s="21">
+        <f>IF(K336="","",K336*AE336)</f>
+        <v/>
+      </c>
+      <c r="AG336" s="19" t="n"/>
+      <c r="AH336" s="19" t="n"/>
+      <c r="AI336" s="19" t="n"/>
+      <c r="AJ336" s="19" t="n"/>
+      <c r="AK336" s="19" t="n"/>
+      <c r="AL336" s="19" t="n"/>
+      <c r="AM336" s="16" t="inlineStr">
+        <is>
+          <t>1 Spielhaus einschließlich Matratze. Bettwäsche und Spielzeug gehören nicht dazu. Der Aufkleber ist auf Foto F-410 zu sehen.</t>
+        </is>
+      </c>
+      <c r="AN336" s="22" t="n"/>
+    </row>
+    <row r="337" ht="30" customHeight="1">
+      <c r="A337" s="15" t="inlineStr">
+        <is>
+          <t>BU05-02</t>
+        </is>
+      </c>
+      <c r="B337" s="15" t="n"/>
+      <c r="C337" s="15" t="n"/>
+      <c r="D337" s="15" t="inlineStr">
+        <is>
+          <t>BU05</t>
+        </is>
+      </c>
+      <c r="E337" s="15" t="inlineStr">
+        <is>
+          <t>Wesco Spielküche, vier Module mit Mikrowelle</t>
+        </is>
+      </c>
+      <c r="F337" s="16" t="inlineStr">
+        <is>
+          <t>Spielküche von Wesco aus Birke-Multiplex: offenes Regalmodul, Backofenmodul mit Klappe, Spülenmodul mit Becken und Kochfeldmodul, dazu eine aufgesetzte Spielmikrowelle. Fronten mit aufgedruckten Bedienfeldern, Rückwände mit Fliesenmuster.</t>
+        </is>
+      </c>
+      <c r="G337" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H337" s="15" t="inlineStr">
+        <is>
+          <t>Schlafraum</t>
+        </is>
+      </c>
+      <c r="I337" s="15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J337" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K337" s="17" t="n"/>
+      <c r="L337" s="18">
+        <f>J337-IF(K337="",0,K337)</f>
+        <v/>
+      </c>
+      <c r="M337" s="15" t="inlineStr">
+        <is>
+          <t>Set</t>
+        </is>
+      </c>
+      <c r="N337" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O337" s="19" t="n"/>
+      <c r="P337" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q337" s="19" t="n"/>
+      <c r="R337" s="20" t="n"/>
+      <c r="S337" s="20" t="n">
+        <v>550</v>
+      </c>
+      <c r="T337" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U337" s="21">
+        <f>L337*S337</f>
+        <v/>
+      </c>
+      <c r="V337" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W337" s="15" t="inlineStr">
+        <is>
+          <t>F-411</t>
+        </is>
+      </c>
+      <c r="X337" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y337" s="19" t="n"/>
+      <c r="Z337" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA337" s="19" t="inlineStr">
+        <is>
+          <t>Wesco</t>
+        </is>
+      </c>
+      <c r="AB337" s="19" t="n"/>
+      <c r="AC337" s="19" t="n"/>
+      <c r="AD337" s="19" t="n"/>
+      <c r="AE337" s="20" t="n"/>
+      <c r="AF337" s="21">
+        <f>IF(K337="","",K337*AE337)</f>
+        <v/>
+      </c>
+      <c r="AG337" s="19" t="n"/>
+      <c r="AH337" s="19" t="n"/>
+      <c r="AI337" s="19" t="n"/>
+      <c r="AJ337" s="19" t="n"/>
+      <c r="AK337" s="19" t="n"/>
+      <c r="AL337" s="19" t="n"/>
+      <c r="AM337" s="16" t="inlineStr">
+        <is>
+          <t>1 Küchenzeile aus vier Modulen einschließlich Mikrowelle. Spielgeschirr, Vorratsgläser und Lebensmittel gehören nicht dazu. Weitere Wesco-Spielküchen stehen unter NU03-03 und NU07-03.</t>
+        </is>
+      </c>
+      <c r="AN337" s="22" t="n"/>
+    </row>
+    <row r="338" ht="30" customHeight="1">
+      <c r="A338" s="15" t="inlineStr">
+        <is>
+          <t>BU05-03</t>
+        </is>
+      </c>
+      <c r="B338" s="15" t="n"/>
+      <c r="C338" s="15" t="n"/>
+      <c r="D338" s="15" t="inlineStr">
+        <is>
+          <t>BU05</t>
+        </is>
+      </c>
+      <c r="E338" s="15" t="inlineStr">
+        <is>
+          <t>Treppenregal weiß mit Wannen</t>
+        </is>
+      </c>
+      <c r="F338" s="16" t="inlineStr">
+        <is>
+          <t>Weißes Regal in Treppenform: zwei hohe Fächer mit eingeschobenen Kunststoffwannen, dazu eine niedrigere Stufe mit Ablage und Wanne, die als Sitzfläche dient.</t>
+        </is>
+      </c>
+      <c r="G338" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H338" s="15" t="inlineStr">
+        <is>
+          <t>Schlafraum</t>
+        </is>
+      </c>
+      <c r="I338" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J338" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K338" s="17" t="n"/>
+      <c r="L338" s="18">
+        <f>J338-IF(K338="",0,K338)</f>
+        <v/>
+      </c>
+      <c r="M338" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N338" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O338" s="19" t="n"/>
+      <c r="P338" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q338" s="19" t="n"/>
+      <c r="R338" s="20" t="n"/>
+      <c r="S338" s="20" t="n">
+        <v>60</v>
+      </c>
+      <c r="T338" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U338" s="21">
+        <f>L338*S338</f>
+        <v/>
+      </c>
+      <c r="V338" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W338" s="15" t="inlineStr">
+        <is>
+          <t>F-412</t>
+        </is>
+      </c>
+      <c r="X338" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y338" s="19" t="n"/>
+      <c r="Z338" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA338" s="19" t="n"/>
+      <c r="AB338" s="19" t="n"/>
+      <c r="AC338" s="19" t="n"/>
+      <c r="AD338" s="19" t="n"/>
+      <c r="AE338" s="20" t="n"/>
+      <c r="AF338" s="21">
+        <f>IF(K338="","",K338*AE338)</f>
+        <v/>
+      </c>
+      <c r="AG338" s="19" t="n"/>
+      <c r="AH338" s="19" t="n"/>
+      <c r="AI338" s="19" t="n"/>
+      <c r="AJ338" s="19" t="n"/>
+      <c r="AK338" s="19" t="n"/>
+      <c r="AL338" s="19" t="n"/>
+      <c r="AM338" s="16" t="inlineStr">
+        <is>
+          <t>1 Regal einschließlich der Wannen. Der Inhalt gehört nicht dazu.</t>
+        </is>
+      </c>
+      <c r="AN338" s="22" t="n"/>
+    </row>
+    <row r="339" ht="30" customHeight="1">
+      <c r="A339" s="15" t="inlineStr">
+        <is>
+          <t>BU05-04</t>
+        </is>
+      </c>
+      <c r="B339" s="15" t="n"/>
+      <c r="C339" s="15" t="n"/>
+      <c r="D339" s="15" t="inlineStr">
+        <is>
+          <t>BU05</t>
+        </is>
+      </c>
+      <c r="E339" s="15" t="inlineStr">
+        <is>
+          <t>Schaukeltier Storch</t>
+        </is>
+      </c>
+      <c r="F339" s="16" t="inlineStr">
+        <is>
+          <t>Plüsch-Schaukeltier in Storchenform: weißer Körper mit rotem Schnabel, gelber Zipfelmütze mit Bommeln und rot-weiß gepunktetem Sattel mit Haltegriff, auf hellen Holzkufen.</t>
+        </is>
+      </c>
+      <c r="G339" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H339" s="15" t="inlineStr">
+        <is>
+          <t>Schlafraum</t>
+        </is>
+      </c>
+      <c r="I339" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J339" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K339" s="17" t="n"/>
+      <c r="L339" s="18">
+        <f>J339-IF(K339="",0,K339)</f>
+        <v/>
+      </c>
+      <c r="M339" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N339" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O339" s="19" t="n"/>
+      <c r="P339" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q339" s="19" t="n"/>
+      <c r="R339" s="20" t="n"/>
+      <c r="S339" s="20" t="n">
+        <v>45</v>
+      </c>
+      <c r="T339" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U339" s="21">
+        <f>L339*S339</f>
+        <v/>
+      </c>
+      <c r="V339" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W339" s="15" t="inlineStr">
+        <is>
+          <t>F-413</t>
+        </is>
+      </c>
+      <c r="X339" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y339" s="19" t="n"/>
+      <c r="Z339" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA339" s="19" t="n"/>
+      <c r="AB339" s="19" t="n"/>
+      <c r="AC339" s="19" t="n"/>
+      <c r="AD339" s="19" t="n"/>
+      <c r="AE339" s="20" t="n"/>
+      <c r="AF339" s="21">
+        <f>IF(K339="","",K339*AE339)</f>
+        <v/>
+      </c>
+      <c r="AG339" s="19" t="n"/>
+      <c r="AH339" s="19" t="n"/>
+      <c r="AI339" s="19" t="n"/>
+      <c r="AJ339" s="19" t="n"/>
+      <c r="AK339" s="19" t="n"/>
+      <c r="AL339" s="19" t="n"/>
+      <c r="AM339" s="16" t="inlineStr">
+        <is>
+          <t>1 Schaukeltier.</t>
+        </is>
+      </c>
+      <c r="AN339" s="22" t="n"/>
+    </row>
+    <row r="340" ht="30" customHeight="1">
+      <c r="A340" s="15" t="inlineStr">
+        <is>
+          <t>BU05-05</t>
+        </is>
+      </c>
+      <c r="B340" s="15" t="n"/>
+      <c r="C340" s="15" t="n"/>
+      <c r="D340" s="15" t="inlineStr">
+        <is>
+          <t>BU05</t>
+        </is>
+      </c>
+      <c r="E340" s="15" t="inlineStr">
+        <is>
+          <t>Kindersessel Teddyfell beige</t>
+        </is>
+      </c>
+      <c r="F340" s="16" t="inlineStr">
+        <is>
+          <t>Kindersessel aus beigem Teddyfell mit runder Lehne, zwei aufgesetzten Ohren und breiten Armlehnen. Am Rücken ein Tragegriff; das Band am Griff ist eingerissen.</t>
+        </is>
+      </c>
+      <c r="G340" s="15" t="inlineStr">
+        <is>
+          <t>Möbel</t>
+        </is>
+      </c>
+      <c r="H340" s="15" t="inlineStr">
+        <is>
+          <t>Schlafraum</t>
+        </is>
+      </c>
+      <c r="I340" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J340" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K340" s="17" t="n"/>
+      <c r="L340" s="18">
+        <f>J340-IF(K340="",0,K340)</f>
+        <v/>
+      </c>
+      <c r="M340" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N340" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O340" s="19" t="n"/>
+      <c r="P340" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q340" s="19" t="n"/>
+      <c r="R340" s="20" t="n"/>
+      <c r="S340" s="20" t="n">
+        <v>45</v>
+      </c>
+      <c r="T340" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U340" s="21">
+        <f>L340*S340</f>
+        <v/>
+      </c>
+      <c r="V340" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W340" s="15" t="inlineStr">
+        <is>
+          <t>F-414</t>
+        </is>
+      </c>
+      <c r="X340" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y340" s="19" t="n"/>
+      <c r="Z340" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA340" s="19" t="n"/>
+      <c r="AB340" s="19" t="n"/>
+      <c r="AC340" s="19" t="n"/>
+      <c r="AD340" s="19" t="n"/>
+      <c r="AE340" s="20" t="n"/>
+      <c r="AF340" s="21">
+        <f>IF(K340="","",K340*AE340)</f>
+        <v/>
+      </c>
+      <c r="AG340" s="19" t="n"/>
+      <c r="AH340" s="19" t="n"/>
+      <c r="AI340" s="19" t="n"/>
+      <c r="AJ340" s="19" t="n"/>
+      <c r="AK340" s="19" t="n"/>
+      <c r="AL340" s="19" t="n"/>
+      <c r="AM340" s="16" t="inlineStr">
+        <is>
+          <t>1 Sessel.</t>
+        </is>
+      </c>
+      <c r="AN340" s="22" t="n"/>
+    </row>
+    <row r="341" ht="30" customHeight="1">
+      <c r="A341" s="15" t="inlineStr">
+        <is>
+          <t>BU05-06</t>
+        </is>
+      </c>
+      <c r="B341" s="15" t="n"/>
+      <c r="C341" s="15" t="n"/>
+      <c r="D341" s="15" t="inlineStr">
+        <is>
+          <t>BU05</t>
+        </is>
+      </c>
+      <c r="E341" s="15" t="inlineStr">
+        <is>
+          <t>Sitzbank gepolstert, hellgrau</t>
+        </is>
+      </c>
+      <c r="F341" s="16" t="inlineStr">
+        <is>
+          <t>Niedrige gepolsterte Sitzbank in Kinderhöhe mit hellgrauem Chenillebezug und flacher Rückenlehne, ohne Armlehnen. Der Bezug ist an mehreren Stellen fleckig.</t>
+        </is>
+      </c>
+      <c r="G341" s="15" t="inlineStr">
+        <is>
+          <t>Möbel</t>
+        </is>
+      </c>
+      <c r="H341" s="15" t="inlineStr">
+        <is>
+          <t>Schlafraum</t>
+        </is>
+      </c>
+      <c r="I341" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J341" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K341" s="17" t="n"/>
+      <c r="L341" s="18">
+        <f>J341-IF(K341="",0,K341)</f>
+        <v/>
+      </c>
+      <c r="M341" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N341" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O341" s="19" t="n"/>
+      <c r="P341" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q341" s="19" t="n"/>
+      <c r="R341" s="20" t="n"/>
+      <c r="S341" s="20" t="n">
+        <v>80</v>
+      </c>
+      <c r="T341" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U341" s="21">
+        <f>L341*S341</f>
+        <v/>
+      </c>
+      <c r="V341" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W341" s="15" t="inlineStr">
+        <is>
+          <t>F-415</t>
+        </is>
+      </c>
+      <c r="X341" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y341" s="19" t="n"/>
+      <c r="Z341" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA341" s="19" t="n"/>
+      <c r="AB341" s="19" t="n"/>
+      <c r="AC341" s="19" t="n"/>
+      <c r="AD341" s="19" t="n"/>
+      <c r="AE341" s="20" t="n"/>
+      <c r="AF341" s="21">
+        <f>IF(K341="","",K341*AE341)</f>
+        <v/>
+      </c>
+      <c r="AG341" s="19" t="n"/>
+      <c r="AH341" s="19" t="n"/>
+      <c r="AI341" s="19" t="n"/>
+      <c r="AJ341" s="19" t="n"/>
+      <c r="AK341" s="19" t="n"/>
+      <c r="AL341" s="19" t="n"/>
+      <c r="AM341" s="16" t="inlineStr">
+        <is>
+          <t>2 Bänke – abgebildet ist eine davon.</t>
+        </is>
+      </c>
+      <c r="AN341" s="22" t="n"/>
+    </row>
+    <row r="342" ht="30" customHeight="1">
+      <c r="A342" s="15" t="inlineStr">
+        <is>
+          <t>BU05-07</t>
+        </is>
+      </c>
+      <c r="B342" s="15" t="n"/>
+      <c r="C342" s="15" t="n"/>
+      <c r="D342" s="15" t="inlineStr">
+        <is>
+          <t>BU05</t>
+        </is>
+      </c>
+      <c r="E342" s="15" t="inlineStr">
+        <is>
+          <t>Puppenwagen rosa mit Tragetasche</t>
+        </is>
+      </c>
+      <c r="F342" s="16" t="inlineStr">
+        <is>
+          <t>Puppen-Sportwagen mit rosa-weiß gestreiftem Bezug, blauem Verdeck und höhenverstellbarem Schiebegriff, dazu eine passende Tragetasche. Der Griff ist an mehreren Stellen aufgerissen.</t>
+        </is>
+      </c>
+      <c r="G342" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H342" s="15" t="inlineStr">
+        <is>
+          <t>Schlafraum</t>
+        </is>
+      </c>
+      <c r="I342" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J342" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K342" s="17" t="n"/>
+      <c r="L342" s="18">
+        <f>J342-IF(K342="",0,K342)</f>
+        <v/>
+      </c>
+      <c r="M342" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N342" s="15" t="inlineStr">
+        <is>
+          <t>stark gebraucht</t>
+        </is>
+      </c>
+      <c r="O342" s="19" t="n"/>
+      <c r="P342" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q342" s="19" t="n"/>
+      <c r="R342" s="20" t="n"/>
+      <c r="S342" s="20" t="n">
+        <v>25</v>
+      </c>
+      <c r="T342" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U342" s="21">
+        <f>L342*S342</f>
+        <v/>
+      </c>
+      <c r="V342" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W342" s="15" t="inlineStr">
+        <is>
+          <t>F-417</t>
+        </is>
+      </c>
+      <c r="X342" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y342" s="19" t="n"/>
+      <c r="Z342" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA342" s="19" t="n"/>
+      <c r="AB342" s="19" t="n"/>
+      <c r="AC342" s="19" t="n"/>
+      <c r="AD342" s="19" t="n"/>
+      <c r="AE342" s="20" t="n"/>
+      <c r="AF342" s="21">
+        <f>IF(K342="","",K342*AE342)</f>
+        <v/>
+      </c>
+      <c r="AG342" s="19" t="n"/>
+      <c r="AH342" s="19" t="n"/>
+      <c r="AI342" s="19" t="n"/>
+      <c r="AJ342" s="19" t="n"/>
+      <c r="AK342" s="19" t="n"/>
+      <c r="AL342" s="19" t="n"/>
+      <c r="AM342" s="16" t="inlineStr">
+        <is>
+          <t>1 Wagen einschließlich Tragetasche. Die Puppe gehört nicht dazu; sie ist auf Foto F-416 mit abgebildet.</t>
+        </is>
+      </c>
+      <c r="AN342" s="22" t="n"/>
+    </row>
+    <row r="343" ht="30" customHeight="1">
+      <c r="A343" s="15" t="inlineStr">
+        <is>
+          <t>BU05-09</t>
+        </is>
+      </c>
+      <c r="B343" s="15" t="n"/>
+      <c r="C343" s="15" t="n"/>
+      <c r="D343" s="15" t="inlineStr">
+        <is>
+          <t>BU05</t>
+        </is>
+      </c>
+      <c r="E343" s="15" t="inlineStr">
+        <is>
+          <t>Puppenwagen Holz mit Gummirädern</t>
+        </is>
+      </c>
+      <c r="F343" s="16" t="inlineStr">
+        <is>
+          <t>Puppen- und Lauflernwagen aus Birke-Multiplex mit hohem Schiebebügel und vier schwarzen Gummirädern. Herstellerangabe laut Erfassungsblatt der Einrichtung: Wesco.</t>
+        </is>
+      </c>
+      <c r="G343" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H343" s="15" t="inlineStr">
+        <is>
+          <t>Schlafraum</t>
+        </is>
+      </c>
+      <c r="I343" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J343" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K343" s="17" t="n"/>
+      <c r="L343" s="18">
+        <f>J343-IF(K343="",0,K343)</f>
+        <v/>
+      </c>
+      <c r="M343" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N343" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O343" s="19" t="n"/>
+      <c r="P343" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q343" s="19" t="n"/>
+      <c r="R343" s="20" t="n"/>
+      <c r="S343" s="20" t="n">
+        <v>60</v>
+      </c>
+      <c r="T343" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U343" s="21">
+        <f>L343*S343</f>
+        <v/>
+      </c>
+      <c r="V343" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W343" s="15" t="inlineStr">
+        <is>
+          <t>F-420</t>
+        </is>
+      </c>
+      <c r="X343" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y343" s="19" t="n"/>
+      <c r="Z343" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA343" s="19" t="inlineStr">
+        <is>
+          <t>Wesco</t>
+        </is>
+      </c>
+      <c r="AB343" s="19" t="n"/>
+      <c r="AC343" s="19" t="n"/>
+      <c r="AD343" s="19" t="n"/>
+      <c r="AE343" s="20" t="n"/>
+      <c r="AF343" s="21">
+        <f>IF(K343="","",K343*AE343)</f>
+        <v/>
+      </c>
+      <c r="AG343" s="19" t="n"/>
+      <c r="AH343" s="19" t="n"/>
+      <c r="AI343" s="19" t="n"/>
+      <c r="AJ343" s="19" t="n"/>
+      <c r="AK343" s="19" t="n"/>
+      <c r="AL343" s="19" t="n"/>
+      <c r="AM343" s="16" t="inlineStr">
+        <is>
+          <t>1 Wagen. Puppe, Kissen und Decke gehören nicht dazu.</t>
+        </is>
+      </c>
+      <c r="AN343" s="22" t="n"/>
+    </row>
+    <row r="344" ht="30" customHeight="1">
+      <c r="A344" s="15" t="inlineStr">
+        <is>
+          <t>BU05-10</t>
+        </is>
+      </c>
+      <c r="B344" s="15" t="n"/>
+      <c r="C344" s="15" t="n"/>
+      <c r="D344" s="15" t="inlineStr">
+        <is>
+          <t>BU05</t>
+        </is>
+      </c>
+      <c r="E344" s="15" t="inlineStr">
+        <is>
+          <t>Wesco Rutschfahrzeug mit Spielelementen</t>
+        </is>
+      </c>
+      <c r="F344" s="16" t="inlineStr">
+        <is>
+          <t>Rutschfahrzeug aus Birke-Multiplex mit gepolsterter Sitzfläche, Steckformen im Sitz, Rückenlehne mit rundem Spiegel und seitlichen Zahnrädern zum Drehen, auf vier Gummirädern. Logo auf der Frontblende: wesco.</t>
+        </is>
+      </c>
+      <c r="G344" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H344" s="15" t="inlineStr">
+        <is>
+          <t>Schlafraum</t>
+        </is>
+      </c>
+      <c r="I344" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J344" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K344" s="17" t="n"/>
+      <c r="L344" s="18">
+        <f>J344-IF(K344="",0,K344)</f>
+        <v/>
+      </c>
+      <c r="M344" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N344" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O344" s="19" t="n"/>
+      <c r="P344" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q344" s="19" t="n"/>
+      <c r="R344" s="20" t="n"/>
+      <c r="S344" s="20" t="n">
+        <v>90</v>
+      </c>
+      <c r="T344" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U344" s="21">
+        <f>L344*S344</f>
+        <v/>
+      </c>
+      <c r="V344" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W344" s="15" t="inlineStr">
+        <is>
+          <t>F-421</t>
+        </is>
+      </c>
+      <c r="X344" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y344" s="19" t="n"/>
+      <c r="Z344" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA344" s="19" t="inlineStr">
+        <is>
+          <t>Wesco</t>
+        </is>
+      </c>
+      <c r="AB344" s="19" t="n"/>
+      <c r="AC344" s="19" t="n"/>
+      <c r="AD344" s="19" t="n"/>
+      <c r="AE344" s="20" t="n"/>
+      <c r="AF344" s="21">
+        <f>IF(K344="","",K344*AE344)</f>
+        <v/>
+      </c>
+      <c r="AG344" s="19" t="n"/>
+      <c r="AH344" s="19" t="n"/>
+      <c r="AI344" s="19" t="n"/>
+      <c r="AJ344" s="19" t="n"/>
+      <c r="AK344" s="19" t="n"/>
+      <c r="AL344" s="19" t="n"/>
+      <c r="AM344" s="16" t="inlineStr">
+        <is>
+          <t>1 Fahrzeug.</t>
+        </is>
+      </c>
+      <c r="AN344" s="22" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:AN335"/>
+  <autoFilter ref="A2:AN344"/>
   <mergeCells count="7">
     <mergeCell ref="AI1:AL1"/>
     <mergeCell ref="V1:AD1"/>
@@ -41868,7 +42959,7 @@
     <mergeCell ref="AE1:AH1"/>
     <mergeCell ref="AM1:AN1"/>
   </mergeCells>
-  <conditionalFormatting sqref="Z3:Z335">
+  <conditionalFormatting sqref="Z3:Z344">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"reserviert"</formula>
     </cfRule>
@@ -41879,12 +42970,12 @@
       <formula>"verkauft"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I3:I335">
+  <conditionalFormatting sqref="I3:I344">
     <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
       <formula>"A"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P3:P335">
+  <conditionalFormatting sqref="P3:P344">
     <cfRule type="cellIs" priority="5" operator="equal" dxfId="4">
       <formula>"entfällt"</formula>
     </cfRule>
@@ -41937,7 +43028,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D94"/>
+  <dimension ref="A1:D95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -41975,7 +43066,7 @@
         </is>
       </c>
       <c r="B5" s="27">
-        <f>COUNTA(Artikelstamm!$A$3:$A$335)</f>
+        <f>COUNTA(Artikelstamm!$A$3:$A$344)</f>
         <v/>
       </c>
     </row>
@@ -41986,7 +43077,7 @@
         </is>
       </c>
       <c r="B6" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$335,"verfügbar")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$344,"verfügbar")</f>
         <v/>
       </c>
     </row>
@@ -41997,7 +43088,7 @@
         </is>
       </c>
       <c r="B7" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$335,"reserviert")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$344,"reserviert")</f>
         <v/>
       </c>
     </row>
@@ -42008,7 +43099,7 @@
         </is>
       </c>
       <c r="B8" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$335,"teilverkauft")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$344,"teilverkauft")</f>
         <v/>
       </c>
     </row>
@@ -42019,7 +43110,7 @@
         </is>
       </c>
       <c r="B9" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$335,"verkauft")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$344,"verkauft")</f>
         <v/>
       </c>
     </row>
@@ -42030,7 +43121,7 @@
         </is>
       </c>
       <c r="B10" s="27">
-        <f>SUM(Artikelstamm!$L$3:$L$335)</f>
+        <f>SUM(Artikelstamm!$L$3:$L$344)</f>
         <v/>
       </c>
     </row>
@@ -42041,7 +43132,7 @@
         </is>
       </c>
       <c r="B11" s="29">
-        <f>SUM(Artikelstamm!$U$3:$U$335)</f>
+        <f>SUM(Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
@@ -42059,7 +43150,7 @@
         </is>
       </c>
       <c r="B13" s="27">
-        <f>SUM(Artikelstamm!$K$3:$K$335)</f>
+        <f>SUM(Artikelstamm!$K$3:$K$344)</f>
         <v/>
       </c>
     </row>
@@ -42070,7 +43161,7 @@
         </is>
       </c>
       <c r="B14" s="30">
-        <f>SUMPRODUCT(Artikelstamm!$K$3:$K$335,Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT(Artikelstamm!$K$3:$K$344,Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
     </row>
@@ -42103,7 +43194,7 @@
         </is>
       </c>
       <c r="B17" s="30">
-        <f>SUMPRODUCT((Artikelstamm!$AJ$3:$AJ$335="bezahlt")*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AJ$3:$AJ$344="bezahlt")*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
     </row>
@@ -42132,7 +43223,7 @@
         </is>
       </c>
       <c r="B21" s="31">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$335,"*verkauft",Artikelstamm!$AI$3:$AI$335,"")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$344,"*verkauft",Artikelstamm!$AI$3:$AI$344,"")</f>
         <v/>
       </c>
     </row>
@@ -42143,7 +43234,7 @@
         </is>
       </c>
       <c r="B22" s="31">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$335,"*verkauft",Artikelstamm!$AJ$3:$AJ$335,"offen")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$344,"*verkauft",Artikelstamm!$AJ$3:$AJ$344,"offen")</f>
         <v/>
       </c>
     </row>
@@ -42154,7 +43245,7 @@
         </is>
       </c>
       <c r="B23" s="27">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$335,"reserviert",Artikelstamm!$AL$3:$AL$335,"")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$344,"reserviert",Artikelstamm!$AL$3:$AL$344,"")</f>
         <v/>
       </c>
     </row>
@@ -42165,7 +43256,7 @@
         </is>
       </c>
       <c r="B24" s="27">
-        <f>COUNTIFS(Artikelstamm!$S$3:$S$335,"")</f>
+        <f>COUNTIFS(Artikelstamm!$S$3:$S$344,"")</f>
         <v/>
       </c>
     </row>
@@ -42176,7 +43267,7 @@
         </is>
       </c>
       <c r="B25" s="27">
-        <f>COUNTIFS(Artikelstamm!$O$3:$O$335,"")</f>
+        <f>COUNTIFS(Artikelstamm!$O$3:$O$344,"")</f>
         <v/>
       </c>
     </row>
@@ -42216,15 +43307,15 @@
         </is>
       </c>
       <c r="B30" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$335,$A30)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$344,$A30)</f>
         <v/>
       </c>
       <c r="C30" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$335=$A30)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$344=$A30)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D30" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$335,$A30,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$344,$A30,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
@@ -42235,15 +43326,15 @@
         </is>
       </c>
       <c r="B31" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$335,$A31)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$344,$A31)</f>
         <v/>
       </c>
       <c r="C31" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$335=$A31)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$344=$A31)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D31" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$335,$A31,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$344,$A31,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
@@ -42254,15 +43345,15 @@
         </is>
       </c>
       <c r="B32" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$335,$A32)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$344,$A32)</f>
         <v/>
       </c>
       <c r="C32" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$335=$A32)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$344=$A32)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D32" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$335,$A32,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$344,$A32,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
@@ -42321,15 +43412,15 @@
         </is>
       </c>
       <c r="B37" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$335,$A37)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$344,$A37)</f>
         <v/>
       </c>
       <c r="C37" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$335=$A37)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$344=$A37)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D37" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$335,$A37,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$344,$A37,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
@@ -42340,15 +43431,15 @@
         </is>
       </c>
       <c r="B38" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$335,$A38)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$344,$A38)</f>
         <v/>
       </c>
       <c r="C38" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$335=$A38)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$344=$A38)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D38" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$335,$A38,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$344,$A38,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
@@ -42359,15 +43450,15 @@
         </is>
       </c>
       <c r="B39" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$335,$A39)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$344,$A39)</f>
         <v/>
       </c>
       <c r="C39" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$335=$A39)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$344=$A39)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D39" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$335,$A39,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$344,$A39,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
@@ -42378,15 +43469,15 @@
         </is>
       </c>
       <c r="B40" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$335,$A40)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$344,$A40)</f>
         <v/>
       </c>
       <c r="C40" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$335=$A40)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$344=$A40)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D40" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$335,$A40,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$344,$A40,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
@@ -42397,15 +43488,15 @@
         </is>
       </c>
       <c r="B41" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$335,$A41)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$344,$A41)</f>
         <v/>
       </c>
       <c r="C41" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$335=$A41)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$344=$A41)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D41" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$335,$A41,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$344,$A41,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
@@ -42416,15 +43507,15 @@
         </is>
       </c>
       <c r="B42" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$335,$A42)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$344,$A42)</f>
         <v/>
       </c>
       <c r="C42" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$335=$A42)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$344=$A42)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D42" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$335,$A42,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$344,$A42,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
@@ -42435,15 +43526,15 @@
         </is>
       </c>
       <c r="B43" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$335,$A43)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$344,$A43)</f>
         <v/>
       </c>
       <c r="C43" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$335=$A43)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$344=$A43)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D43" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$335,$A43,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$344,$A43,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
@@ -42454,15 +43545,15 @@
         </is>
       </c>
       <c r="B44" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$335,$A44)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$344,$A44)</f>
         <v/>
       </c>
       <c r="C44" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$335=$A44)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$344=$A44)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D44" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$335,$A44,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$344,$A44,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
@@ -42473,15 +43564,15 @@
         </is>
       </c>
       <c r="B45" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$335,$A45)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$344,$A45)</f>
         <v/>
       </c>
       <c r="C45" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$335=$A45)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$344=$A45)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D45" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$335,$A45,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$344,$A45,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
@@ -42492,15 +43583,15 @@
         </is>
       </c>
       <c r="B46" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$335,$A46)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$344,$A46)</f>
         <v/>
       </c>
       <c r="C46" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$335=$A46)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$344=$A46)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D46" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$335,$A46,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$344,$A46,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
@@ -42511,15 +43602,15 @@
         </is>
       </c>
       <c r="B47" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$335,$A47)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$344,$A47)</f>
         <v/>
       </c>
       <c r="C47" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$335=$A47)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$344=$A47)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D47" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$335,$A47,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$344,$A47,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
@@ -42530,15 +43621,15 @@
         </is>
       </c>
       <c r="B48" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$335,$A48)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$344,$A48)</f>
         <v/>
       </c>
       <c r="C48" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$335=$A48)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$344=$A48)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D48" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$335,$A48,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$344,$A48,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
@@ -42549,15 +43640,15 @@
         </is>
       </c>
       <c r="B49" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$335,$A49)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$344,$A49)</f>
         <v/>
       </c>
       <c r="C49" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$335=$A49)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$344=$A49)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D49" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$335,$A49,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$344,$A49,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
@@ -42568,15 +43659,15 @@
         </is>
       </c>
       <c r="B50" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$335,$A50)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$344,$A50)</f>
         <v/>
       </c>
       <c r="C50" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$335=$A50)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$344=$A50)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D50" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$335,$A50,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$344,$A50,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
@@ -42635,15 +43726,15 @@
         </is>
       </c>
       <c r="B55" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$335,$A55)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$344,$A55)</f>
         <v/>
       </c>
       <c r="C55" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$335=$A55)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$344=$A55)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D55" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$335,$A55,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$344,$A55,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
@@ -42654,15 +43745,15 @@
         </is>
       </c>
       <c r="B56" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$335,$A56)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$344,$A56)</f>
         <v/>
       </c>
       <c r="C56" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$335=$A56)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$344=$A56)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D56" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$335,$A56,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$344,$A56,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
@@ -42673,15 +43764,15 @@
         </is>
       </c>
       <c r="B57" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$335,$A57)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$344,$A57)</f>
         <v/>
       </c>
       <c r="C57" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$335=$A57)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$344=$A57)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D57" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$335,$A57,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$344,$A57,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
@@ -42692,15 +43783,15 @@
         </is>
       </c>
       <c r="B58" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$335,$A58)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$344,$A58)</f>
         <v/>
       </c>
       <c r="C58" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$335=$A58)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$344=$A58)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D58" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$335,$A58,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$344,$A58,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
@@ -42711,15 +43802,15 @@
         </is>
       </c>
       <c r="B59" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$335,$A59)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$344,$A59)</f>
         <v/>
       </c>
       <c r="C59" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$335=$A59)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$344=$A59)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D59" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$335,$A59,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$344,$A59,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
@@ -42730,15 +43821,15 @@
         </is>
       </c>
       <c r="B60" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$335,$A60)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$344,$A60)</f>
         <v/>
       </c>
       <c r="C60" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$335=$A60)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$344=$A60)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D60" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$335,$A60,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$344,$A60,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
@@ -42749,15 +43840,15 @@
         </is>
       </c>
       <c r="B61" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$335,$A61)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$344,$A61)</f>
         <v/>
       </c>
       <c r="C61" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$335=$A61)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$344=$A61)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D61" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$335,$A61,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$344,$A61,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
@@ -42768,15 +43859,15 @@
         </is>
       </c>
       <c r="B62" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$335,$A62)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$344,$A62)</f>
         <v/>
       </c>
       <c r="C62" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$335=$A62)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$344=$A62)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D62" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$335,$A62,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$344,$A62,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
@@ -42787,15 +43878,15 @@
         </is>
       </c>
       <c r="B63" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$335,$A63)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$344,$A63)</f>
         <v/>
       </c>
       <c r="C63" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$335=$A63)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$344=$A63)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D63" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$335,$A63,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$344,$A63,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
@@ -42806,15 +43897,15 @@
         </is>
       </c>
       <c r="B64" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$335,$A64)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$344,$A64)</f>
         <v/>
       </c>
       <c r="C64" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$335=$A64)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$344=$A64)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D64" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$335,$A64,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$344,$A64,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
@@ -42825,15 +43916,15 @@
         </is>
       </c>
       <c r="B65" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$335,$A65)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$344,$A65)</f>
         <v/>
       </c>
       <c r="C65" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$335=$A65)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$344=$A65)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D65" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$335,$A65,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$344,$A65,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
@@ -42844,15 +43935,15 @@
         </is>
       </c>
       <c r="B66" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$335,$A66)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$344,$A66)</f>
         <v/>
       </c>
       <c r="C66" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$335=$A66)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$344=$A66)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D66" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$335,$A66,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$344,$A66,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
@@ -42863,15 +43954,15 @@
         </is>
       </c>
       <c r="B67" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$335,$A67)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$344,$A67)</f>
         <v/>
       </c>
       <c r="C67" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$335=$A67)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$344=$A67)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D67" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$335,$A67,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$344,$A67,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
@@ -42882,15 +43973,15 @@
         </is>
       </c>
       <c r="B68" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$335,$A68)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$344,$A68)</f>
         <v/>
       </c>
       <c r="C68" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$335=$A68)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$344=$A68)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D68" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$335,$A68,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$344,$A68,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
@@ -42901,15 +43992,15 @@
         </is>
       </c>
       <c r="B69" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$335,$A69)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$344,$A69)</f>
         <v/>
       </c>
       <c r="C69" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$335=$A69)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$344=$A69)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D69" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$335,$A69,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$344,$A69,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
@@ -42920,15 +44011,15 @@
         </is>
       </c>
       <c r="B70" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$335,$A70)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$344,$A70)</f>
         <v/>
       </c>
       <c r="C70" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$335=$A70)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$344=$A70)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D70" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$335,$A70,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$344,$A70,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
@@ -42939,15 +44030,15 @@
         </is>
       </c>
       <c r="B71" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$335,$A71)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$344,$A71)</f>
         <v/>
       </c>
       <c r="C71" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$335=$A71)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$344=$A71)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D71" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$335,$A71,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$344,$A71,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
@@ -42958,15 +44049,15 @@
         </is>
       </c>
       <c r="B72" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$335,$A72)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$344,$A72)</f>
         <v/>
       </c>
       <c r="C72" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$335=$A72)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$344=$A72)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D72" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$335,$A72,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$344,$A72,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
@@ -42977,15 +44068,15 @@
         </is>
       </c>
       <c r="B73" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$335,$A73)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$344,$A73)</f>
         <v/>
       </c>
       <c r="C73" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$335=$A73)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$344=$A73)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D73" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$335,$A73,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$344,$A73,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
@@ -42996,334 +44087,353 @@
         </is>
       </c>
       <c r="B74" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$335,$A74)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$344,$A74)</f>
         <v/>
       </c>
       <c r="C74" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$335=$A74)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$344=$A74)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D74" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$335,$A74,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$344,$A74,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="26" t="inlineStr">
         <is>
-          <t>Schlafraum 4</t>
+          <t>Schlafraum</t>
         </is>
       </c>
       <c r="B75" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$335,$A75)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$344,$A75)</f>
         <v/>
       </c>
       <c r="C75" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$335=$A75)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$344=$A75)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D75" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$335,$A75,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$344,$A75,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="26" t="inlineStr">
         <is>
-          <t>Schlafraum 5</t>
+          <t>Schlafraum 4</t>
         </is>
       </c>
       <c r="B76" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$335,$A76)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$344,$A76)</f>
         <v/>
       </c>
       <c r="C76" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$335=$A76)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$344=$A76)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D76" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$335,$A76,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$344,$A76,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="26" t="inlineStr">
         <is>
-          <t>Speisesaal</t>
+          <t>Schlafraum 5</t>
         </is>
       </c>
       <c r="B77" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$335,$A77)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$344,$A77)</f>
         <v/>
       </c>
       <c r="C77" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$335=$A77)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$344=$A77)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D77" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$335,$A77,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$344,$A77,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="26" t="inlineStr">
         <is>
-          <t>Terrasse</t>
+          <t>Speisesaal</t>
         </is>
       </c>
       <c r="B78" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$335,$A78)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$344,$A78)</f>
         <v/>
       </c>
       <c r="C78" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$335=$A78)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$344=$A78)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D78" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$335,$A78,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$344,$A78,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="26" t="inlineStr">
         <is>
-          <t>Treppenraum 1</t>
+          <t>Terrasse</t>
         </is>
       </c>
       <c r="B79" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$335,$A79)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$344,$A79)</f>
         <v/>
       </c>
       <c r="C79" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$335=$A79)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$344=$A79)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D79" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$335,$A79,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$344,$A79,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="26" t="inlineStr">
         <is>
-          <t>Turnraum</t>
+          <t>Treppenraum 1</t>
         </is>
       </c>
       <c r="B80" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$335,$A80)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$344,$A80)</f>
         <v/>
       </c>
       <c r="C80" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$335=$A80)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$344=$A80)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D80" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$335,$A80,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$344,$A80,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="26" t="inlineStr">
         <is>
-          <t>WC</t>
+          <t>Turnraum</t>
         </is>
       </c>
       <c r="B81" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$335,$A81)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$344,$A81)</f>
         <v/>
       </c>
       <c r="C81" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$335=$A81)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$344=$A81)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D81" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$335,$A81,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$344,$A81,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="26" t="inlineStr">
         <is>
-          <t>WC Personal</t>
+          <t>WC</t>
         </is>
       </c>
       <c r="B82" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$335,$A82)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$344,$A82)</f>
         <v/>
       </c>
       <c r="C82" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$335=$A82)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$344=$A82)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
       <c r="D82" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$335,$A82,Artikelstamm!$U$3:$U$335)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$344,$A82,Artikelstamm!$U$3:$U$344)</f>
         <v/>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="26" t="inlineStr">
         <is>
+          <t>WC Personal</t>
+        </is>
+      </c>
+      <c r="B83" s="33">
+        <f>COUNTIF(Artikelstamm!$H$3:$H$344,$A83)</f>
+        <v/>
+      </c>
+      <c r="C83" s="34">
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$344=$A83)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
+        <v/>
+      </c>
+      <c r="D83" s="34">
+        <f>SUMIF(Artikelstamm!$H$3:$H$344,$A83,Artikelstamm!$U$3:$U$344)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="26" t="inlineStr">
+        <is>
           <t>Werkraum</t>
         </is>
       </c>
-      <c r="B83" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$335,$A83)</f>
-        <v/>
-      </c>
-      <c r="C83" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$335=$A83)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
-        <v/>
-      </c>
-      <c r="D83" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$335,$A83,Artikelstamm!$U$3:$U$335)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" s="28" t="inlineStr">
+      <c r="B84" s="33">
+        <f>COUNTIF(Artikelstamm!$H$3:$H$344,$A84)</f>
+        <v/>
+      </c>
+      <c r="C84" s="34">
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$344=$A84)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
+        <v/>
+      </c>
+      <c r="D84" s="34">
+        <f>SUMIF(Artikelstamm!$H$3:$H$344,$A84,Artikelstamm!$U$3:$U$344)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="28" t="inlineStr">
         <is>
           <t>Summe</t>
         </is>
       </c>
-      <c r="B84" s="35">
-        <f>SUM(B55:B83)</f>
-        <v/>
-      </c>
-      <c r="C84" s="36">
-        <f>SUM(C55:C83)</f>
-        <v/>
-      </c>
-      <c r="D84" s="36">
-        <f>SUM(D55:D83)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" s="25" t="inlineStr">
+      <c r="B85" s="35">
+        <f>SUM(B55:B84)</f>
+        <v/>
+      </c>
+      <c r="C85" s="36">
+        <f>SUM(C55:C84)</f>
+        <v/>
+      </c>
+      <c r="D85" s="36">
+        <f>SUM(D55:D84)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="25" t="inlineStr">
         <is>
           <t>Nach Verkaufskanal</t>
         </is>
       </c>
     </row>
-    <row r="87">
-      <c r="A87" s="32" t="inlineStr">
+    <row r="88">
+      <c r="A88" s="32" t="inlineStr">
         <is>
           <t>Verkaufskanal</t>
         </is>
       </c>
-      <c r="B87" s="32" t="inlineStr">
+      <c r="B88" s="32" t="inlineStr">
         <is>
           <t>Positionen</t>
         </is>
       </c>
-      <c r="C87" s="32" t="inlineStr">
+      <c r="C88" s="32" t="inlineStr">
         <is>
           <t>Umsatz netto</t>
         </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" s="26" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
-      <c r="B88" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$335,$A88)</f>
-        <v/>
-      </c>
-      <c r="C88" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$335=$A88)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
-        <v/>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="26" t="inlineStr">
         <is>
-          <t>Kleinanzeigen</t>
+          <t>Klinik</t>
         </is>
       </c>
       <c r="B89" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$335,$A89)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$344,$A89)</f>
         <v/>
       </c>
       <c r="C89" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$335=$A89)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$344=$A89)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="26" t="inlineStr">
         <is>
-          <t>eBay</t>
+          <t>Kleinanzeigen</t>
         </is>
       </c>
       <c r="B90" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$335,$A90)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$344,$A90)</f>
         <v/>
       </c>
       <c r="C90" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$335=$A90)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$344=$A90)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="26" t="inlineStr">
         <is>
-          <t>Direkt</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="B91" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$335,$A91)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$344,$A91)</f>
         <v/>
       </c>
       <c r="C91" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$335=$A91)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$344=$A91)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="26" t="inlineStr">
         <is>
-          <t>Händler</t>
+          <t>Direkt</t>
         </is>
       </c>
       <c r="B92" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$335,$A92)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$344,$A92)</f>
         <v/>
       </c>
       <c r="C92" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$335=$A92)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$344=$A92)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
         <v/>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="26" t="inlineStr">
         <is>
+          <t>Händler</t>
+        </is>
+      </c>
+      <c r="B93" s="33">
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$344,$A93)</f>
+        <v/>
+      </c>
+      <c r="C93" s="34">
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$344=$A93)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="26" t="inlineStr">
+        <is>
           <t>Verkaufstag</t>
         </is>
       </c>
-      <c r="B93" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$335,$A93)</f>
-        <v/>
-      </c>
-      <c r="C93" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$335=$A93)*Artikelstamm!$K$3:$K$335*Artikelstamm!$AE$3:$AE$335)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" s="28" t="inlineStr">
+      <c r="B94" s="33">
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$344,$A94)</f>
+        <v/>
+      </c>
+      <c r="C94" s="34">
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$344=$A94)*Artikelstamm!$K$3:$K$344*Artikelstamm!$AE$3:$AE$344)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="28" t="inlineStr">
         <is>
           <t>Summe</t>
         </is>
       </c>
-      <c r="B94" s="35">
-        <f>SUM(B88:B93)</f>
-        <v/>
-      </c>
-      <c r="C94" s="36">
-        <f>SUM(C88:C93)</f>
+      <c r="B95" s="35">
+        <f>SUM(B89:B94)</f>
+        <v/>
+      </c>
+      <c r="C95" s="36">
+        <f>SUM(C89:C94)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
NE03 Schlafraum 2 erfasst: 9 neue Positionen, 2 Zusammenfassungen
Raum NE03 (Neubau EG, Schlafraum 2, 20,42 m2) aus 13 Fotos und dem
Erfassungsblatt aufgenommen. 9 neue Positionen; zwei Nummern gehen in
bestehende Positionen ein:

  NE03-02 -> NU03-02  Stockbett weiss           4 -> 14
  NE03-08 -> NU04-19  IKEA Kleiderschrank weiss 2 -> 3

Zwei Fotos maskiert: F-442 Schuhspitzen einer Person am Bildrand,
F-450 Finger am unteren Bildrand.

Datenbasis 359 Positionen / 303 aktiv, pruefen.py 0 Fehler.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011yyfqhuiWGsaNy38oaNoGo
</commit_message>
<xml_diff>
--- a/ausgabe/01_Artikelstamm_kikripp.xlsx
+++ b/ausgabe/01_Artikelstamm_kikripp.xlsx
@@ -15,7 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Artikelstamm'!$A$2:$AN$352</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Artikelstamm'!$A$2:$AN$361</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1019,7 +1019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN352"/>
+  <dimension ref="A1:AN361"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -22631,7 +22631,11 @@
         </is>
       </c>
       <c r="B177" s="15" t="n"/>
-      <c r="C177" s="15" t="n"/>
+      <c r="C177" s="15" t="inlineStr">
+        <is>
+          <t>NE03-02</t>
+        </is>
+      </c>
       <c r="D177" s="15" t="inlineStr">
         <is>
           <t>NU03</t>
@@ -22663,7 +22667,7 @@
         </is>
       </c>
       <c r="J177" s="17" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="K177" s="17" t="n"/>
       <c r="L177" s="18">
@@ -22738,12 +22742,12 @@
       <c r="AL177" s="19" t="n"/>
       <c r="AM177" s="16" t="inlineStr">
         <is>
-          <t>4 Betten, alle aufgebaut: 2 im Schlafraum 4 und 2 in einem weiteren Schlafraum.</t>
+          <t>14 Betten insgesamt: 4 im Schlafraum 4 (NU03-02) und 10 im Schlafraum 2 des Neubaus (NE03-02). Die Matratzen können auf Wunsch mitgenommen werden. Ein Bett mit Aufstiegstreppe ist auf Foto F-439 zu sehen.</t>
         </is>
       </c>
       <c r="AN177" s="22" t="inlineStr">
         <is>
-          <t>OFFEN: waechst noch. Aus den weiteren Schlafraeumen kommen zusaetzliche Betten dazu - am Ende des Rundgangs auf die Gesamtzahl bringen und die Post-it-Nummern der anderen Raeume in Weitere_ArtNr.</t>
+          <t>OFFEN: waechst noch. Aus den weiteren Schlafraeumen kommen zusaetzliche Betten dazu - am Ende des Rundgangs auf die Gesamtzahl bringen und die Post-it-Nummern in Weitere_ArtNr ergaenzen. Bisher: NE03-02.</t>
         </is>
       </c>
     </row>
@@ -25103,7 +25107,11 @@
         </is>
       </c>
       <c r="B197" s="15" t="n"/>
-      <c r="C197" s="15" t="n"/>
+      <c r="C197" s="15" t="inlineStr">
+        <is>
+          <t>NE03-08</t>
+        </is>
+      </c>
       <c r="D197" s="15" t="inlineStr">
         <is>
           <t>NU04</t>
@@ -25135,7 +25143,7 @@
         </is>
       </c>
       <c r="J197" s="17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K197" s="17" t="n"/>
       <c r="L197" s="18">
@@ -25214,10 +25222,14 @@
       <c r="AL197" s="19" t="n"/>
       <c r="AM197" s="16" t="inlineStr">
         <is>
-          <t>2 Schränke – abgebildet ist einer davon, innen auf Foto F-206.</t>
-        </is>
-      </c>
-      <c r="AN197" s="22" t="n"/>
+          <t>3 Schränke insgesamt: 2 im Schlafraum 5 (NU04-19) und 1 im Schlafraum 2 des Neubaus (NE03-08). Abgebildet ist einer davon, innen auf Foto F-206. Ein baugleicher Schrank in Anthrazit steht unter NE03-07.</t>
+        </is>
+      </c>
+      <c r="AN197" s="22" t="inlineStr">
+        <is>
+          <t>Zusammengefasste Position über zwei Räume – Post-it-Nummer: NE03-08.</t>
+        </is>
+      </c>
     </row>
     <row r="198" ht="30" customHeight="1">
       <c r="A198" s="15" t="inlineStr">
@@ -43892,8 +43904,1095 @@
       </c>
       <c r="AN352" s="22" t="n"/>
     </row>
+    <row r="353" ht="30" customHeight="1">
+      <c r="A353" s="15" t="inlineStr">
+        <is>
+          <t>NE03-01</t>
+        </is>
+      </c>
+      <c r="B353" s="15" t="n"/>
+      <c r="C353" s="15" t="n"/>
+      <c r="D353" s="15" t="inlineStr">
+        <is>
+          <t>NE03</t>
+        </is>
+      </c>
+      <c r="E353" s="15" t="inlineStr">
+        <is>
+          <t>Wandregale in Wolkenform</t>
+        </is>
+      </c>
+      <c r="F353" s="16" t="inlineStr">
+        <is>
+          <t>Wandregale in Wolkenform aus lackiertem Holz, ohne Zwischenböden: ein großes und ein kleineres in Weiß, zwei in Schwarz.</t>
+        </is>
+      </c>
+      <c r="G353" s="15" t="inlineStr">
+        <is>
+          <t>Deko</t>
+        </is>
+      </c>
+      <c r="H353" s="15" t="inlineStr">
+        <is>
+          <t>Schlafraum 2</t>
+        </is>
+      </c>
+      <c r="I353" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J353" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="K353" s="17" t="n"/>
+      <c r="L353" s="18">
+        <f>J353-IF(K353="",0,K353)</f>
+        <v/>
+      </c>
+      <c r="M353" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N353" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O353" s="19" t="n"/>
+      <c r="P353" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q353" s="19" t="n"/>
+      <c r="R353" s="20" t="n"/>
+      <c r="S353" s="20" t="n">
+        <v>25</v>
+      </c>
+      <c r="T353" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U353" s="21">
+        <f>L353*S353</f>
+        <v/>
+      </c>
+      <c r="V353" s="15" t="inlineStr">
+        <is>
+          <t>Versand möglich</t>
+        </is>
+      </c>
+      <c r="W353" s="15" t="inlineStr">
+        <is>
+          <t>F-438</t>
+        </is>
+      </c>
+      <c r="X353" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y353" s="19" t="n"/>
+      <c r="Z353" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA353" s="19" t="n"/>
+      <c r="AB353" s="19" t="n"/>
+      <c r="AC353" s="19" t="n"/>
+      <c r="AD353" s="19" t="n"/>
+      <c r="AE353" s="20" t="n"/>
+      <c r="AF353" s="21">
+        <f>IF(K353="","",K353*AE353)</f>
+        <v/>
+      </c>
+      <c r="AG353" s="19" t="n"/>
+      <c r="AH353" s="19" t="n"/>
+      <c r="AI353" s="19" t="n"/>
+      <c r="AJ353" s="19" t="n"/>
+      <c r="AK353" s="19" t="n"/>
+      <c r="AL353" s="19" t="n"/>
+      <c r="AM353" s="16" t="inlineStr">
+        <is>
+          <t>4 Regale in drei Größen – alle auf dem Foto zu sehen. Der Elefant aus Kupferdraht gehört nicht dazu.</t>
+        </is>
+      </c>
+      <c r="AN353" s="22" t="n"/>
+    </row>
+    <row r="354" ht="30" customHeight="1">
+      <c r="A354" s="15" t="inlineStr">
+        <is>
+          <t>NE03-03</t>
+        </is>
+      </c>
+      <c r="B354" s="15" t="n"/>
+      <c r="C354" s="15" t="n"/>
+      <c r="D354" s="15" t="inlineStr">
+        <is>
+          <t>NE03</t>
+        </is>
+      </c>
+      <c r="E354" s="15" t="inlineStr">
+        <is>
+          <t>Wesco Gitterbett Kunststoff, grau</t>
+        </is>
+      </c>
+      <c r="F354" s="16" t="inlineStr">
+        <is>
+          <t>Krippenbett von Wesco aus grauem Kunststoff mit geschlossenem Sockel, belüfteten Seitenwänden und Griffausschnitten zum Verschieben. Logo an der Längsseite: wesco.</t>
+        </is>
+      </c>
+      <c r="G354" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H354" s="15" t="inlineStr">
+        <is>
+          <t>Schlafraum 2</t>
+        </is>
+      </c>
+      <c r="I354" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J354" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="K354" s="17" t="n"/>
+      <c r="L354" s="18">
+        <f>J354-IF(K354="",0,K354)</f>
+        <v/>
+      </c>
+      <c r="M354" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N354" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O354" s="19" t="n"/>
+      <c r="P354" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q354" s="19" t="n"/>
+      <c r="R354" s="20" t="n"/>
+      <c r="S354" s="20" t="n">
+        <v>180</v>
+      </c>
+      <c r="T354" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U354" s="21">
+        <f>L354*S354</f>
+        <v/>
+      </c>
+      <c r="V354" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W354" s="15" t="inlineStr">
+        <is>
+          <t>F-440</t>
+        </is>
+      </c>
+      <c r="X354" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y354" s="19" t="n"/>
+      <c r="Z354" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA354" s="19" t="inlineStr">
+        <is>
+          <t>Wesco</t>
+        </is>
+      </c>
+      <c r="AB354" s="19" t="n"/>
+      <c r="AC354" s="19" t="n"/>
+      <c r="AD354" s="19" t="n"/>
+      <c r="AE354" s="20" t="n"/>
+      <c r="AF354" s="21">
+        <f>IF(K354="","",K354*AE354)</f>
+        <v/>
+      </c>
+      <c r="AG354" s="19" t="n"/>
+      <c r="AH354" s="19" t="n"/>
+      <c r="AI354" s="19" t="n"/>
+      <c r="AJ354" s="19" t="n"/>
+      <c r="AK354" s="19" t="n"/>
+      <c r="AL354" s="19" t="n"/>
+      <c r="AM354" s="16" t="inlineStr">
+        <is>
+          <t>4 Betten – abgebildet ist eines davon. Matratze, Nestchen und Bettwäsche gehören nicht dazu.</t>
+        </is>
+      </c>
+      <c r="AN354" s="22" t="n"/>
+    </row>
+    <row r="355" ht="30" customHeight="1">
+      <c r="A355" s="15" t="inlineStr">
+        <is>
+          <t>NE03-04</t>
+        </is>
+      </c>
+      <c r="B355" s="15" t="n"/>
+      <c r="C355" s="15" t="n"/>
+      <c r="D355" s="15" t="inlineStr">
+        <is>
+          <t>NE03</t>
+        </is>
+      </c>
+      <c r="E355" s="15" t="inlineStr">
+        <is>
+          <t>Gitterbett Holz weiß</t>
+        </is>
+      </c>
+      <c r="F355" s="16" t="inlineStr">
+        <is>
+          <t>Kinderbett aus weiß lackiertem Holz mit Sprossen an allen vier Seiten und geschwungenen Kopf- und Fußteilen, einschließlich Matratze.</t>
+        </is>
+      </c>
+      <c r="G355" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H355" s="15" t="inlineStr">
+        <is>
+          <t>Schlafraum 2</t>
+        </is>
+      </c>
+      <c r="I355" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J355" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="K355" s="17" t="n"/>
+      <c r="L355" s="18">
+        <f>J355-IF(K355="",0,K355)</f>
+        <v/>
+      </c>
+      <c r="M355" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N355" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O355" s="19" t="n"/>
+      <c r="P355" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q355" s="19" t="n"/>
+      <c r="R355" s="20" t="n"/>
+      <c r="S355" s="20" t="n">
+        <v>60</v>
+      </c>
+      <c r="T355" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U355" s="21">
+        <f>L355*S355</f>
+        <v/>
+      </c>
+      <c r="V355" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W355" s="15" t="inlineStr">
+        <is>
+          <t>F-441</t>
+        </is>
+      </c>
+      <c r="X355" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y355" s="19" t="n"/>
+      <c r="Z355" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA355" s="19" t="n"/>
+      <c r="AB355" s="19" t="n"/>
+      <c r="AC355" s="19" t="n"/>
+      <c r="AD355" s="19" t="n"/>
+      <c r="AE355" s="20" t="n"/>
+      <c r="AF355" s="21">
+        <f>IF(K355="","",K355*AE355)</f>
+        <v/>
+      </c>
+      <c r="AG355" s="19" t="n"/>
+      <c r="AH355" s="19" t="n"/>
+      <c r="AI355" s="19" t="n"/>
+      <c r="AJ355" s="19" t="n"/>
+      <c r="AK355" s="19" t="n"/>
+      <c r="AL355" s="19" t="n"/>
+      <c r="AM355" s="16" t="inlineStr">
+        <is>
+          <t>3 Betten einschließlich Matratzen – abgebildet ist eines davon. Nestchen und Bettwäsche gehören nicht dazu.</t>
+        </is>
+      </c>
+      <c r="AN355" s="22" t="n"/>
+    </row>
+    <row r="356" ht="30" customHeight="1">
+      <c r="A356" s="15" t="inlineStr">
+        <is>
+          <t>NE03-05</t>
+        </is>
+      </c>
+      <c r="B356" s="15" t="n"/>
+      <c r="C356" s="15" t="n"/>
+      <c r="D356" s="15" t="inlineStr">
+        <is>
+          <t>NE03</t>
+        </is>
+      </c>
+      <c r="E356" s="15" t="inlineStr">
+        <is>
+          <t>Hauck Kinderwagen schwarz</t>
+        </is>
+      </c>
+      <c r="F356" s="16" t="inlineStr">
+        <is>
+          <t>Sportwagen von Hauck in Schwarz mit Verdeck, Fünfpunktgurt und Faltmechanik. Aufdruck am Sitz: Rapid Fold. Der Stoff ist an mehreren Stellen verschmutzt.</t>
+        </is>
+      </c>
+      <c r="G356" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H356" s="15" t="inlineStr">
+        <is>
+          <t>Schlafraum 2</t>
+        </is>
+      </c>
+      <c r="I356" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J356" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K356" s="17" t="n"/>
+      <c r="L356" s="18">
+        <f>J356-IF(K356="",0,K356)</f>
+        <v/>
+      </c>
+      <c r="M356" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N356" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O356" s="19" t="n"/>
+      <c r="P356" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q356" s="19" t="n"/>
+      <c r="R356" s="20" t="n"/>
+      <c r="S356" s="20" t="n">
+        <v>45</v>
+      </c>
+      <c r="T356" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U356" s="21">
+        <f>L356*S356</f>
+        <v/>
+      </c>
+      <c r="V356" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W356" s="15" t="inlineStr">
+        <is>
+          <t>F-442</t>
+        </is>
+      </c>
+      <c r="X356" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y356" s="19" t="n"/>
+      <c r="Z356" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA356" s="19" t="inlineStr">
+        <is>
+          <t>Hauck</t>
+        </is>
+      </c>
+      <c r="AB356" s="19" t="n"/>
+      <c r="AC356" s="19" t="n"/>
+      <c r="AD356" s="19" t="n"/>
+      <c r="AE356" s="20" t="n"/>
+      <c r="AF356" s="21">
+        <f>IF(K356="","",K356*AE356)</f>
+        <v/>
+      </c>
+      <c r="AG356" s="19" t="n"/>
+      <c r="AH356" s="19" t="n"/>
+      <c r="AI356" s="19" t="n"/>
+      <c r="AJ356" s="19" t="n"/>
+      <c r="AK356" s="19" t="n"/>
+      <c r="AL356" s="19" t="n"/>
+      <c r="AM356" s="16" t="inlineStr">
+        <is>
+          <t>1 Wagen. Das Etikett ist auf Foto F-443 zu sehen.</t>
+        </is>
+      </c>
+      <c r="AN356" s="22" t="n"/>
+    </row>
+    <row r="357" ht="30" customHeight="1">
+      <c r="A357" s="15" t="inlineStr">
+        <is>
+          <t>NE03-06</t>
+        </is>
+      </c>
+      <c r="B357" s="15" t="n"/>
+      <c r="C357" s="15" t="n"/>
+      <c r="D357" s="15" t="inlineStr">
+        <is>
+          <t>NE03</t>
+        </is>
+      </c>
+      <c r="E357" s="15" t="inlineStr">
+        <is>
+          <t>Leuchtobjekt Elefant, Metall</t>
+        </is>
+      </c>
+      <c r="F357" s="16" t="inlineStr">
+        <is>
+          <t>Dekoleuchte in Elefantenform aus taupefarbenem Metall mit elf Fassungen für Glühlampen auf der Vorderseite, zum Stellen.</t>
+        </is>
+      </c>
+      <c r="G357" s="15" t="inlineStr">
+        <is>
+          <t>Leuchten</t>
+        </is>
+      </c>
+      <c r="H357" s="15" t="inlineStr">
+        <is>
+          <t>Schlafraum 2</t>
+        </is>
+      </c>
+      <c r="I357" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J357" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K357" s="17" t="n"/>
+      <c r="L357" s="18">
+        <f>J357-IF(K357="",0,K357)</f>
+        <v/>
+      </c>
+      <c r="M357" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N357" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O357" s="19" t="n"/>
+      <c r="P357" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q357" s="19" t="n"/>
+      <c r="R357" s="20" t="n"/>
+      <c r="S357" s="20" t="n">
+        <v>45</v>
+      </c>
+      <c r="T357" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U357" s="21">
+        <f>L357*S357</f>
+        <v/>
+      </c>
+      <c r="V357" s="15" t="inlineStr">
+        <is>
+          <t>Versand möglich</t>
+        </is>
+      </c>
+      <c r="W357" s="15" t="inlineStr">
+        <is>
+          <t>F-444</t>
+        </is>
+      </c>
+      <c r="X357" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y357" s="19" t="n"/>
+      <c r="Z357" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA357" s="19" t="n"/>
+      <c r="AB357" s="19" t="n"/>
+      <c r="AC357" s="19" t="n"/>
+      <c r="AD357" s="19" t="n"/>
+      <c r="AE357" s="20" t="n"/>
+      <c r="AF357" s="21">
+        <f>IF(K357="","",K357*AE357)</f>
+        <v/>
+      </c>
+      <c r="AG357" s="19" t="n"/>
+      <c r="AH357" s="19" t="n"/>
+      <c r="AI357" s="19" t="n"/>
+      <c r="AJ357" s="19" t="n"/>
+      <c r="AK357" s="19" t="n"/>
+      <c r="AL357" s="19" t="n"/>
+      <c r="AM357" s="16" t="inlineStr">
+        <is>
+          <t>2 Stück – abgebildet ist eines davon. Ohne Leuchtmittel.</t>
+        </is>
+      </c>
+      <c r="AN357" s="22" t="n"/>
+    </row>
+    <row r="358" ht="30" customHeight="1">
+      <c r="A358" s="15" t="inlineStr">
+        <is>
+          <t>NE03-07</t>
+        </is>
+      </c>
+      <c r="B358" s="15" t="n"/>
+      <c r="C358" s="15" t="n"/>
+      <c r="D358" s="15" t="inlineStr">
+        <is>
+          <t>NE03</t>
+        </is>
+      </c>
+      <c r="E358" s="15" t="inlineStr">
+        <is>
+          <t>IKEA Kleiderschrank anthrazit mit drei Böden</t>
+        </is>
+      </c>
+      <c r="F358" s="16" t="inlineStr">
+        <is>
+          <t>Hoher Schrank von IKEA in Anthrazit mit zwei Türen, weißen ovalen Griffmulden und drei Einlegeböden.</t>
+        </is>
+      </c>
+      <c r="G358" s="15" t="inlineStr">
+        <is>
+          <t>Möbel</t>
+        </is>
+      </c>
+      <c r="H358" s="15" t="inlineStr">
+        <is>
+          <t>Schlafraum 2</t>
+        </is>
+      </c>
+      <c r="I358" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J358" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K358" s="17" t="n"/>
+      <c r="L358" s="18">
+        <f>J358-IF(K358="",0,K358)</f>
+        <v/>
+      </c>
+      <c r="M358" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N358" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O358" s="19" t="n"/>
+      <c r="P358" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q358" s="19" t="n"/>
+      <c r="R358" s="20" t="n"/>
+      <c r="S358" s="20" t="n">
+        <v>60</v>
+      </c>
+      <c r="T358" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U358" s="21">
+        <f>L358*S358</f>
+        <v/>
+      </c>
+      <c r="V358" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W358" s="15" t="inlineStr">
+        <is>
+          <t>F-445</t>
+        </is>
+      </c>
+      <c r="X358" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y358" s="19" t="n"/>
+      <c r="Z358" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA358" s="19" t="inlineStr">
+        <is>
+          <t>IKEA</t>
+        </is>
+      </c>
+      <c r="AB358" s="19" t="n"/>
+      <c r="AC358" s="19" t="n"/>
+      <c r="AD358" s="19" t="n"/>
+      <c r="AE358" s="20" t="n"/>
+      <c r="AF358" s="21">
+        <f>IF(K358="","",K358*AE358)</f>
+        <v/>
+      </c>
+      <c r="AG358" s="19" t="n"/>
+      <c r="AH358" s="19" t="n"/>
+      <c r="AI358" s="19" t="n"/>
+      <c r="AJ358" s="19" t="n"/>
+      <c r="AK358" s="19" t="n"/>
+      <c r="AL358" s="19" t="n"/>
+      <c r="AM358" s="16" t="inlineStr">
+        <is>
+          <t>1 Schrank. Baugleiche Schränke in Weiß stehen unter NU04-19.</t>
+        </is>
+      </c>
+      <c r="AN358" s="22" t="n"/>
+    </row>
+    <row r="359" ht="30" customHeight="1">
+      <c r="A359" s="15" t="inlineStr">
+        <is>
+          <t>NE03-09</t>
+        </is>
+      </c>
+      <c r="B359" s="15" t="n"/>
+      <c r="C359" s="15" t="n"/>
+      <c r="D359" s="15" t="inlineStr">
+        <is>
+          <t>NE03</t>
+        </is>
+      </c>
+      <c r="E359" s="15" t="inlineStr">
+        <is>
+          <t>IKEA Schrank weiß mit Drahtkörben</t>
+        </is>
+      </c>
+      <c r="F359" s="16" t="inlineStr">
+        <is>
+          <t>Hoher Schrank von IKEA in Weiß mit zwei Türen, weißen ovalen Griffmulden und innen sechs herausziehbaren Drahtkörben.</t>
+        </is>
+      </c>
+      <c r="G359" s="15" t="inlineStr">
+        <is>
+          <t>Möbel</t>
+        </is>
+      </c>
+      <c r="H359" s="15" t="inlineStr">
+        <is>
+          <t>Schlafraum 2</t>
+        </is>
+      </c>
+      <c r="I359" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J359" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K359" s="17" t="n"/>
+      <c r="L359" s="18">
+        <f>J359-IF(K359="",0,K359)</f>
+        <v/>
+      </c>
+      <c r="M359" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N359" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O359" s="19" t="n"/>
+      <c r="P359" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q359" s="19" t="n"/>
+      <c r="R359" s="20" t="n"/>
+      <c r="S359" s="20" t="n">
+        <v>80</v>
+      </c>
+      <c r="T359" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U359" s="21">
+        <f>L359*S359</f>
+        <v/>
+      </c>
+      <c r="V359" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W359" s="15" t="inlineStr">
+        <is>
+          <t>F-447</t>
+        </is>
+      </c>
+      <c r="X359" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y359" s="19" t="n"/>
+      <c r="Z359" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA359" s="19" t="inlineStr">
+        <is>
+          <t>IKEA</t>
+        </is>
+      </c>
+      <c r="AB359" s="19" t="n"/>
+      <c r="AC359" s="19" t="n"/>
+      <c r="AD359" s="19" t="n"/>
+      <c r="AE359" s="20" t="n"/>
+      <c r="AF359" s="21">
+        <f>IF(K359="","",K359*AE359)</f>
+        <v/>
+      </c>
+      <c r="AG359" s="19" t="n"/>
+      <c r="AH359" s="19" t="n"/>
+      <c r="AI359" s="19" t="n"/>
+      <c r="AJ359" s="19" t="n"/>
+      <c r="AK359" s="19" t="n"/>
+      <c r="AL359" s="19" t="n"/>
+      <c r="AM359" s="16" t="inlineStr">
+        <is>
+          <t>1 Schrank einschließlich der Drahtkörbe. Handtücher und Bettwäsche gehören nicht dazu.</t>
+        </is>
+      </c>
+      <c r="AN359" s="22" t="n"/>
+    </row>
+    <row r="360" ht="30" customHeight="1">
+      <c r="A360" s="15" t="inlineStr">
+        <is>
+          <t>NE03-10</t>
+        </is>
+      </c>
+      <c r="B360" s="15" t="n"/>
+      <c r="C360" s="15" t="n"/>
+      <c r="D360" s="15" t="inlineStr">
+        <is>
+          <t>NE03</t>
+        </is>
+      </c>
+      <c r="E360" s="15" t="inlineStr">
+        <is>
+          <t>Plüsch-Elefanten, zwei Stück</t>
+        </is>
+      </c>
+      <c r="F360" s="16" t="inlineStr">
+        <is>
+          <t>Zwei große Plüsch-Elefanten zum Stellen: einer aus cremefarbenem Breitcord, einer aus grau-cremefarben gestreiftem Stoff mit aufgestickten Augen. Am gestreiften Elefanten ein Etikett: done by deer.</t>
+        </is>
+      </c>
+      <c r="G360" s="15" t="inlineStr">
+        <is>
+          <t>Deko</t>
+        </is>
+      </c>
+      <c r="H360" s="15" t="inlineStr">
+        <is>
+          <t>Schlafraum 2</t>
+        </is>
+      </c>
+      <c r="I360" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J360" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K360" s="17" t="n"/>
+      <c r="L360" s="18">
+        <f>J360-IF(K360="",0,K360)</f>
+        <v/>
+      </c>
+      <c r="M360" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N360" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O360" s="19" t="n"/>
+      <c r="P360" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q360" s="19" t="n"/>
+      <c r="R360" s="20" t="n"/>
+      <c r="S360" s="20" t="n">
+        <v>25</v>
+      </c>
+      <c r="T360" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U360" s="21">
+        <f>L360*S360</f>
+        <v/>
+      </c>
+      <c r="V360" s="15" t="inlineStr">
+        <is>
+          <t>Versand möglich</t>
+        </is>
+      </c>
+      <c r="W360" s="15" t="inlineStr">
+        <is>
+          <t>F-448</t>
+        </is>
+      </c>
+      <c r="X360" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y360" s="19" t="n"/>
+      <c r="Z360" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA360" s="19" t="n"/>
+      <c r="AB360" s="19" t="n"/>
+      <c r="AC360" s="19" t="n"/>
+      <c r="AD360" s="19" t="n"/>
+      <c r="AE360" s="20" t="n"/>
+      <c r="AF360" s="21">
+        <f>IF(K360="","",K360*AE360)</f>
+        <v/>
+      </c>
+      <c r="AG360" s="19" t="n"/>
+      <c r="AH360" s="19" t="n"/>
+      <c r="AI360" s="19" t="n"/>
+      <c r="AJ360" s="19" t="n"/>
+      <c r="AK360" s="19" t="n"/>
+      <c r="AL360" s="19" t="n"/>
+      <c r="AM360" s="16" t="inlineStr">
+        <is>
+          <t>2 Elefanten, beide abgebildet.</t>
+        </is>
+      </c>
+      <c r="AN360" s="22" t="n"/>
+    </row>
+    <row r="361" ht="30" customHeight="1">
+      <c r="A361" s="15" t="inlineStr">
+        <is>
+          <t>NE03-11</t>
+        </is>
+      </c>
+      <c r="B361" s="15" t="n"/>
+      <c r="C361" s="15" t="n"/>
+      <c r="D361" s="15" t="inlineStr">
+        <is>
+          <t>NE03</t>
+        </is>
+      </c>
+      <c r="E361" s="15" t="inlineStr">
+        <is>
+          <t>Wolken-Mobile Stoff, weiß</t>
+        </is>
+      </c>
+      <c r="F361" s="16" t="inlineStr">
+        <is>
+          <t>Mobile aus drei weißen Stoffwolken in unterschiedlicher Größe, zum Aufhängen.</t>
+        </is>
+      </c>
+      <c r="G361" s="15" t="inlineStr">
+        <is>
+          <t>Deko</t>
+        </is>
+      </c>
+      <c r="H361" s="15" t="inlineStr">
+        <is>
+          <t>Schlafraum 2</t>
+        </is>
+      </c>
+      <c r="I361" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J361" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K361" s="17" t="n"/>
+      <c r="L361" s="18">
+        <f>J361-IF(K361="",0,K361)</f>
+        <v/>
+      </c>
+      <c r="M361" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N361" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O361" s="19" t="n"/>
+      <c r="P361" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q361" s="19" t="n"/>
+      <c r="R361" s="20" t="n"/>
+      <c r="S361" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="T361" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U361" s="21">
+        <f>L361*S361</f>
+        <v/>
+      </c>
+      <c r="V361" s="15" t="inlineStr">
+        <is>
+          <t>Versand möglich</t>
+        </is>
+      </c>
+      <c r="W361" s="15" t="inlineStr">
+        <is>
+          <t>F-449</t>
+        </is>
+      </c>
+      <c r="X361" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y361" s="19" t="n"/>
+      <c r="Z361" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA361" s="19" t="n"/>
+      <c r="AB361" s="19" t="n"/>
+      <c r="AC361" s="19" t="n"/>
+      <c r="AD361" s="19" t="n"/>
+      <c r="AE361" s="20" t="n"/>
+      <c r="AF361" s="21">
+        <f>IF(K361="","",K361*AE361)</f>
+        <v/>
+      </c>
+      <c r="AG361" s="19" t="n"/>
+      <c r="AH361" s="19" t="n"/>
+      <c r="AI361" s="19" t="n"/>
+      <c r="AJ361" s="19" t="n"/>
+      <c r="AK361" s="19" t="n"/>
+      <c r="AL361" s="19" t="n"/>
+      <c r="AM361" s="16" t="inlineStr">
+        <is>
+          <t>2 Mobiles – abgebildet ist eines davon.</t>
+        </is>
+      </c>
+      <c r="AN361" s="22" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:AN352"/>
+  <autoFilter ref="A2:AN361"/>
   <mergeCells count="7">
     <mergeCell ref="AI1:AL1"/>
     <mergeCell ref="V1:AD1"/>
@@ -43903,7 +45002,7 @@
     <mergeCell ref="AE1:AH1"/>
     <mergeCell ref="AM1:AN1"/>
   </mergeCells>
-  <conditionalFormatting sqref="Z3:Z352">
+  <conditionalFormatting sqref="Z3:Z361">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"reserviert"</formula>
     </cfRule>
@@ -43914,12 +45013,12 @@
       <formula>"verkauft"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I3:I352">
+  <conditionalFormatting sqref="I3:I361">
     <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
       <formula>"A"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P3:P352">
+  <conditionalFormatting sqref="P3:P361">
     <cfRule type="cellIs" priority="5" operator="equal" dxfId="4">
       <formula>"entfällt"</formula>
     </cfRule>
@@ -43972,7 +45071,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D96"/>
+  <dimension ref="A1:D97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -44010,7 +45109,7 @@
         </is>
       </c>
       <c r="B5" s="27">
-        <f>COUNTA(Artikelstamm!$A$3:$A$352)</f>
+        <f>COUNTA(Artikelstamm!$A$3:$A$361)</f>
         <v/>
       </c>
     </row>
@@ -44021,7 +45120,7 @@
         </is>
       </c>
       <c r="B6" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$352,"verfügbar")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$361,"verfügbar")</f>
         <v/>
       </c>
     </row>
@@ -44032,7 +45131,7 @@
         </is>
       </c>
       <c r="B7" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$352,"reserviert")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$361,"reserviert")</f>
         <v/>
       </c>
     </row>
@@ -44043,7 +45142,7 @@
         </is>
       </c>
       <c r="B8" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$352,"teilverkauft")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$361,"teilverkauft")</f>
         <v/>
       </c>
     </row>
@@ -44054,7 +45153,7 @@
         </is>
       </c>
       <c r="B9" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$352,"verkauft")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$361,"verkauft")</f>
         <v/>
       </c>
     </row>
@@ -44065,7 +45164,7 @@
         </is>
       </c>
       <c r="B10" s="27">
-        <f>SUM(Artikelstamm!$L$3:$L$352)</f>
+        <f>SUM(Artikelstamm!$L$3:$L$361)</f>
         <v/>
       </c>
     </row>
@@ -44076,7 +45175,7 @@
         </is>
       </c>
       <c r="B11" s="29">
-        <f>SUM(Artikelstamm!$U$3:$U$352)</f>
+        <f>SUM(Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
@@ -44094,7 +45193,7 @@
         </is>
       </c>
       <c r="B13" s="27">
-        <f>SUM(Artikelstamm!$K$3:$K$352)</f>
+        <f>SUM(Artikelstamm!$K$3:$K$361)</f>
         <v/>
       </c>
     </row>
@@ -44105,7 +45204,7 @@
         </is>
       </c>
       <c r="B14" s="30">
-        <f>SUMPRODUCT(Artikelstamm!$K$3:$K$352,Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT(Artikelstamm!$K$3:$K$361,Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
     </row>
@@ -44138,7 +45237,7 @@
         </is>
       </c>
       <c r="B17" s="30">
-        <f>SUMPRODUCT((Artikelstamm!$AJ$3:$AJ$352="bezahlt")*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AJ$3:$AJ$361="bezahlt")*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
     </row>
@@ -44167,7 +45266,7 @@
         </is>
       </c>
       <c r="B21" s="31">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$352,"*verkauft",Artikelstamm!$AI$3:$AI$352,"")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$361,"*verkauft",Artikelstamm!$AI$3:$AI$361,"")</f>
         <v/>
       </c>
     </row>
@@ -44178,7 +45277,7 @@
         </is>
       </c>
       <c r="B22" s="31">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$352,"*verkauft",Artikelstamm!$AJ$3:$AJ$352,"offen")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$361,"*verkauft",Artikelstamm!$AJ$3:$AJ$361,"offen")</f>
         <v/>
       </c>
     </row>
@@ -44189,7 +45288,7 @@
         </is>
       </c>
       <c r="B23" s="27">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$352,"reserviert",Artikelstamm!$AL$3:$AL$352,"")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$361,"reserviert",Artikelstamm!$AL$3:$AL$361,"")</f>
         <v/>
       </c>
     </row>
@@ -44200,7 +45299,7 @@
         </is>
       </c>
       <c r="B24" s="27">
-        <f>COUNTIFS(Artikelstamm!$S$3:$S$352,"")</f>
+        <f>COUNTIFS(Artikelstamm!$S$3:$S$361,"")</f>
         <v/>
       </c>
     </row>
@@ -44211,7 +45310,7 @@
         </is>
       </c>
       <c r="B25" s="27">
-        <f>COUNTIFS(Artikelstamm!$O$3:$O$352,"")</f>
+        <f>COUNTIFS(Artikelstamm!$O$3:$O$361,"")</f>
         <v/>
       </c>
     </row>
@@ -44251,15 +45350,15 @@
         </is>
       </c>
       <c r="B30" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$352,$A30)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$361,$A30)</f>
         <v/>
       </c>
       <c r="C30" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$352=$A30)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$361=$A30)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D30" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$352,$A30,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$361,$A30,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
@@ -44270,15 +45369,15 @@
         </is>
       </c>
       <c r="B31" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$352,$A31)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$361,$A31)</f>
         <v/>
       </c>
       <c r="C31" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$352=$A31)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$361=$A31)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D31" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$352,$A31,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$361,$A31,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
@@ -44289,15 +45388,15 @@
         </is>
       </c>
       <c r="B32" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$352,$A32)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$361,$A32)</f>
         <v/>
       </c>
       <c r="C32" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$352=$A32)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$361=$A32)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D32" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$352,$A32,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$361,$A32,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
@@ -44356,15 +45455,15 @@
         </is>
       </c>
       <c r="B37" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$352,$A37)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$361,$A37)</f>
         <v/>
       </c>
       <c r="C37" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$352=$A37)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$361=$A37)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D37" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$352,$A37,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$361,$A37,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
@@ -44375,15 +45474,15 @@
         </is>
       </c>
       <c r="B38" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$352,$A38)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$361,$A38)</f>
         <v/>
       </c>
       <c r="C38" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$352=$A38)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$361=$A38)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D38" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$352,$A38,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$361,$A38,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
@@ -44394,15 +45493,15 @@
         </is>
       </c>
       <c r="B39" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$352,$A39)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$361,$A39)</f>
         <v/>
       </c>
       <c r="C39" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$352=$A39)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$361=$A39)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D39" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$352,$A39,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$361,$A39,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
@@ -44413,15 +45512,15 @@
         </is>
       </c>
       <c r="B40" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$352,$A40)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$361,$A40)</f>
         <v/>
       </c>
       <c r="C40" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$352=$A40)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$361=$A40)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D40" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$352,$A40,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$361,$A40,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
@@ -44432,15 +45531,15 @@
         </is>
       </c>
       <c r="B41" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$352,$A41)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$361,$A41)</f>
         <v/>
       </c>
       <c r="C41" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$352=$A41)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$361=$A41)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D41" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$352,$A41,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$361,$A41,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
@@ -44451,15 +45550,15 @@
         </is>
       </c>
       <c r="B42" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$352,$A42)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$361,$A42)</f>
         <v/>
       </c>
       <c r="C42" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$352=$A42)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$361=$A42)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D42" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$352,$A42,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$361,$A42,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
@@ -44470,15 +45569,15 @@
         </is>
       </c>
       <c r="B43" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$352,$A43)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$361,$A43)</f>
         <v/>
       </c>
       <c r="C43" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$352=$A43)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$361=$A43)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D43" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$352,$A43,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$361,$A43,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
@@ -44489,15 +45588,15 @@
         </is>
       </c>
       <c r="B44" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$352,$A44)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$361,$A44)</f>
         <v/>
       </c>
       <c r="C44" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$352=$A44)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$361=$A44)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D44" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$352,$A44,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$361,$A44,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
@@ -44508,15 +45607,15 @@
         </is>
       </c>
       <c r="B45" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$352,$A45)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$361,$A45)</f>
         <v/>
       </c>
       <c r="C45" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$352=$A45)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$361=$A45)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D45" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$352,$A45,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$361,$A45,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
@@ -44527,15 +45626,15 @@
         </is>
       </c>
       <c r="B46" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$352,$A46)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$361,$A46)</f>
         <v/>
       </c>
       <c r="C46" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$352=$A46)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$361=$A46)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D46" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$352,$A46,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$361,$A46,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
@@ -44546,15 +45645,15 @@
         </is>
       </c>
       <c r="B47" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$352,$A47)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$361,$A47)</f>
         <v/>
       </c>
       <c r="C47" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$352=$A47)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$361=$A47)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D47" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$352,$A47,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$361,$A47,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
@@ -44565,15 +45664,15 @@
         </is>
       </c>
       <c r="B48" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$352,$A48)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$361,$A48)</f>
         <v/>
       </c>
       <c r="C48" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$352=$A48)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$361=$A48)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D48" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$352,$A48,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$361,$A48,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
@@ -44584,15 +45683,15 @@
         </is>
       </c>
       <c r="B49" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$352,$A49)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$361,$A49)</f>
         <v/>
       </c>
       <c r="C49" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$352=$A49)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$361=$A49)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D49" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$352,$A49,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$361,$A49,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
@@ -44603,15 +45702,15 @@
         </is>
       </c>
       <c r="B50" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$352,$A50)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$361,$A50)</f>
         <v/>
       </c>
       <c r="C50" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$352=$A50)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$361=$A50)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D50" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$352,$A50,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$361,$A50,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
@@ -44670,15 +45769,15 @@
         </is>
       </c>
       <c r="B55" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$352,$A55)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A55)</f>
         <v/>
       </c>
       <c r="C55" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$352=$A55)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A55)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D55" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$352,$A55,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A55,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
@@ -44689,15 +45788,15 @@
         </is>
       </c>
       <c r="B56" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$352,$A56)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A56)</f>
         <v/>
       </c>
       <c r="C56" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$352=$A56)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A56)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D56" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$352,$A56,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A56,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
@@ -44708,15 +45807,15 @@
         </is>
       </c>
       <c r="B57" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$352,$A57)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A57)</f>
         <v/>
       </c>
       <c r="C57" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$352=$A57)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A57)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D57" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$352,$A57,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A57,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
@@ -44727,15 +45826,15 @@
         </is>
       </c>
       <c r="B58" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$352,$A58)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A58)</f>
         <v/>
       </c>
       <c r="C58" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$352=$A58)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A58)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D58" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$352,$A58,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A58,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
@@ -44746,15 +45845,15 @@
         </is>
       </c>
       <c r="B59" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$352,$A59)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A59)</f>
         <v/>
       </c>
       <c r="C59" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$352=$A59)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A59)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D59" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$352,$A59,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A59,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
@@ -44765,15 +45864,15 @@
         </is>
       </c>
       <c r="B60" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$352,$A60)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A60)</f>
         <v/>
       </c>
       <c r="C60" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$352=$A60)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A60)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D60" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$352,$A60,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A60,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
@@ -44784,15 +45883,15 @@
         </is>
       </c>
       <c r="B61" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$352,$A61)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A61)</f>
         <v/>
       </c>
       <c r="C61" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$352=$A61)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A61)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D61" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$352,$A61,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A61,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
@@ -44803,15 +45902,15 @@
         </is>
       </c>
       <c r="B62" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$352,$A62)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A62)</f>
         <v/>
       </c>
       <c r="C62" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$352=$A62)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A62)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D62" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$352,$A62,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A62,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
@@ -44822,15 +45921,15 @@
         </is>
       </c>
       <c r="B63" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$352,$A63)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A63)</f>
         <v/>
       </c>
       <c r="C63" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$352=$A63)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A63)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D63" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$352,$A63,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A63,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
@@ -44841,15 +45940,15 @@
         </is>
       </c>
       <c r="B64" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$352,$A64)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A64)</f>
         <v/>
       </c>
       <c r="C64" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$352=$A64)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A64)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D64" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$352,$A64,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A64,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
@@ -44860,15 +45959,15 @@
         </is>
       </c>
       <c r="B65" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$352,$A65)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A65)</f>
         <v/>
       </c>
       <c r="C65" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$352=$A65)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A65)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D65" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$352,$A65,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A65,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
@@ -44879,15 +45978,15 @@
         </is>
       </c>
       <c r="B66" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$352,$A66)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A66)</f>
         <v/>
       </c>
       <c r="C66" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$352=$A66)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A66)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D66" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$352,$A66,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A66,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
@@ -44898,15 +45997,15 @@
         </is>
       </c>
       <c r="B67" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$352,$A67)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A67)</f>
         <v/>
       </c>
       <c r="C67" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$352=$A67)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A67)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D67" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$352,$A67,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A67,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
@@ -44917,15 +46016,15 @@
         </is>
       </c>
       <c r="B68" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$352,$A68)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A68)</f>
         <v/>
       </c>
       <c r="C68" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$352=$A68)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A68)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D68" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$352,$A68,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A68,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
@@ -44936,15 +46035,15 @@
         </is>
       </c>
       <c r="B69" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$352,$A69)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A69)</f>
         <v/>
       </c>
       <c r="C69" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$352=$A69)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A69)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D69" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$352,$A69,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A69,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
@@ -44955,15 +46054,15 @@
         </is>
       </c>
       <c r="B70" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$352,$A70)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A70)</f>
         <v/>
       </c>
       <c r="C70" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$352=$A70)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A70)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D70" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$352,$A70,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A70,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
@@ -44974,15 +46073,15 @@
         </is>
       </c>
       <c r="B71" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$352,$A71)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A71)</f>
         <v/>
       </c>
       <c r="C71" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$352=$A71)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A71)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D71" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$352,$A71,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A71,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
@@ -44993,15 +46092,15 @@
         </is>
       </c>
       <c r="B72" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$352,$A72)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A72)</f>
         <v/>
       </c>
       <c r="C72" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$352=$A72)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A72)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D72" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$352,$A72,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A72,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
@@ -45012,15 +46111,15 @@
         </is>
       </c>
       <c r="B73" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$352,$A73)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A73)</f>
         <v/>
       </c>
       <c r="C73" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$352=$A73)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A73)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D73" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$352,$A73,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A73,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
@@ -45031,15 +46130,15 @@
         </is>
       </c>
       <c r="B74" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$352,$A74)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A74)</f>
         <v/>
       </c>
       <c r="C74" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$352=$A74)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A74)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D74" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$352,$A74,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A74,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
@@ -45050,15 +46149,15 @@
         </is>
       </c>
       <c r="B75" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$352,$A75)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A75)</f>
         <v/>
       </c>
       <c r="C75" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$352=$A75)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A75)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D75" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$352,$A75,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A75,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
@@ -45069,334 +46168,353 @@
         </is>
       </c>
       <c r="B76" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$352,$A76)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A76)</f>
         <v/>
       </c>
       <c r="C76" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$352=$A76)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A76)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D76" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$352,$A76,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A76,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="26" t="inlineStr">
         <is>
-          <t>Schlafraum 4</t>
+          <t>Schlafraum 2</t>
         </is>
       </c>
       <c r="B77" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$352,$A77)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A77)</f>
         <v/>
       </c>
       <c r="C77" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$352=$A77)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A77)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D77" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$352,$A77,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A77,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="26" t="inlineStr">
         <is>
-          <t>Schlafraum 5</t>
+          <t>Schlafraum 4</t>
         </is>
       </c>
       <c r="B78" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$352,$A78)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A78)</f>
         <v/>
       </c>
       <c r="C78" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$352=$A78)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A78)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D78" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$352,$A78,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A78,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="26" t="inlineStr">
         <is>
-          <t>Speisesaal</t>
+          <t>Schlafraum 5</t>
         </is>
       </c>
       <c r="B79" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$352,$A79)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A79)</f>
         <v/>
       </c>
       <c r="C79" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$352=$A79)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A79)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D79" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$352,$A79,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A79,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="26" t="inlineStr">
         <is>
-          <t>Terrasse</t>
+          <t>Speisesaal</t>
         </is>
       </c>
       <c r="B80" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$352,$A80)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A80)</f>
         <v/>
       </c>
       <c r="C80" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$352=$A80)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A80)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D80" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$352,$A80,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A80,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="26" t="inlineStr">
         <is>
-          <t>Treppenraum 1</t>
+          <t>Terrasse</t>
         </is>
       </c>
       <c r="B81" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$352,$A81)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A81)</f>
         <v/>
       </c>
       <c r="C81" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$352=$A81)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A81)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D81" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$352,$A81,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A81,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="26" t="inlineStr">
         <is>
-          <t>Turnraum</t>
+          <t>Treppenraum 1</t>
         </is>
       </c>
       <c r="B82" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$352,$A82)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A82)</f>
         <v/>
       </c>
       <c r="C82" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$352=$A82)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A82)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D82" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$352,$A82,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A82,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="26" t="inlineStr">
         <is>
-          <t>WC</t>
+          <t>Turnraum</t>
         </is>
       </c>
       <c r="B83" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$352,$A83)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A83)</f>
         <v/>
       </c>
       <c r="C83" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$352=$A83)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A83)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D83" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$352,$A83,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A83,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="26" t="inlineStr">
         <is>
-          <t>WC Personal</t>
+          <t>WC</t>
         </is>
       </c>
       <c r="B84" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$352,$A84)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A84)</f>
         <v/>
       </c>
       <c r="C84" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$352=$A84)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A84)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
       <c r="D84" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$352,$A84,Artikelstamm!$U$3:$U$352)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A84,Artikelstamm!$U$3:$U$361)</f>
         <v/>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="26" t="inlineStr">
         <is>
+          <t>WC Personal</t>
+        </is>
+      </c>
+      <c r="B85" s="33">
+        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A85)</f>
+        <v/>
+      </c>
+      <c r="C85" s="34">
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A85)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <v/>
+      </c>
+      <c r="D85" s="34">
+        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A85,Artikelstamm!$U$3:$U$361)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="26" t="inlineStr">
+        <is>
           <t>Werkraum</t>
         </is>
       </c>
-      <c r="B85" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$352,$A85)</f>
-        <v/>
-      </c>
-      <c r="C85" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$352=$A85)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
-        <v/>
-      </c>
-      <c r="D85" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$352,$A85,Artikelstamm!$U$3:$U$352)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" s="28" t="inlineStr">
+      <c r="B86" s="33">
+        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A86)</f>
+        <v/>
+      </c>
+      <c r="C86" s="34">
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A86)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <v/>
+      </c>
+      <c r="D86" s="34">
+        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A86,Artikelstamm!$U$3:$U$361)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="28" t="inlineStr">
         <is>
           <t>Summe</t>
         </is>
       </c>
-      <c r="B86" s="35">
-        <f>SUM(B55:B85)</f>
-        <v/>
-      </c>
-      <c r="C86" s="36">
-        <f>SUM(C55:C85)</f>
-        <v/>
-      </c>
-      <c r="D86" s="36">
-        <f>SUM(D55:D85)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" s="25" t="inlineStr">
+      <c r="B87" s="35">
+        <f>SUM(B55:B86)</f>
+        <v/>
+      </c>
+      <c r="C87" s="36">
+        <f>SUM(C55:C86)</f>
+        <v/>
+      </c>
+      <c r="D87" s="36">
+        <f>SUM(D55:D86)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="25" t="inlineStr">
         <is>
           <t>Nach Verkaufskanal</t>
         </is>
       </c>
     </row>
-    <row r="89">
-      <c r="A89" s="32" t="inlineStr">
+    <row r="90">
+      <c r="A90" s="32" t="inlineStr">
         <is>
           <t>Verkaufskanal</t>
         </is>
       </c>
-      <c r="B89" s="32" t="inlineStr">
+      <c r="B90" s="32" t="inlineStr">
         <is>
           <t>Positionen</t>
         </is>
       </c>
-      <c r="C89" s="32" t="inlineStr">
+      <c r="C90" s="32" t="inlineStr">
         <is>
           <t>Umsatz netto</t>
         </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" s="26" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
-      <c r="B90" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$352,$A90)</f>
-        <v/>
-      </c>
-      <c r="C90" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$352=$A90)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
-        <v/>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="26" t="inlineStr">
         <is>
-          <t>Kleinanzeigen</t>
+          <t>Klinik</t>
         </is>
       </c>
       <c r="B91" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$352,$A91)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$361,$A91)</f>
         <v/>
       </c>
       <c r="C91" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$352=$A91)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$361=$A91)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="26" t="inlineStr">
         <is>
-          <t>eBay</t>
+          <t>Kleinanzeigen</t>
         </is>
       </c>
       <c r="B92" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$352,$A92)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$361,$A92)</f>
         <v/>
       </c>
       <c r="C92" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$352=$A92)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$361=$A92)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="26" t="inlineStr">
         <is>
-          <t>Direkt</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="B93" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$352,$A93)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$361,$A93)</f>
         <v/>
       </c>
       <c r="C93" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$352=$A93)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$361=$A93)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="26" t="inlineStr">
         <is>
-          <t>Händler</t>
+          <t>Direkt</t>
         </is>
       </c>
       <c r="B94" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$352,$A94)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$361,$A94)</f>
         <v/>
       </c>
       <c r="C94" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$352=$A94)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$361=$A94)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
         <v/>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="26" t="inlineStr">
         <is>
+          <t>Händler</t>
+        </is>
+      </c>
+      <c r="B95" s="33">
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$361,$A95)</f>
+        <v/>
+      </c>
+      <c r="C95" s="34">
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$361=$A95)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="26" t="inlineStr">
+        <is>
           <t>Verkaufstag</t>
         </is>
       </c>
-      <c r="B95" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$352,$A95)</f>
-        <v/>
-      </c>
-      <c r="C95" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$352=$A95)*Artikelstamm!$K$3:$K$352*Artikelstamm!$AE$3:$AE$352)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="28" t="inlineStr">
+      <c r="B96" s="33">
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$361,$A96)</f>
+        <v/>
+      </c>
+      <c r="C96" s="34">
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$361=$A96)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="28" t="inlineStr">
         <is>
           <t>Summe</t>
         </is>
       </c>
-      <c r="B96" s="35">
-        <f>SUM(B90:B95)</f>
-        <v/>
-      </c>
-      <c r="C96" s="36">
-        <f>SUM(C90:C95)</f>
+      <c r="B97" s="35">
+        <f>SUM(B91:B96)</f>
+        <v/>
+      </c>
+      <c r="C97" s="36">
+        <f>SUM(C91:C96)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
NE04 Schlafraum 3 erfasst; Betten auf Zustand gut, Zara Home ergaenzt
Raum NE04 (Neubau EG, Schlafraum 3, 20,41 m2) aus 18 Fotos und dem
Erfassungsblatt aufgenommen: 12 neue Positionen, drei Zusammenfassungen.

  NE04-01 -> NU03-02  Stockbett weiss    14 -> 16
  NE04-02 -> NE03-04  Gitterbett Holz     3 -> 10
  NE04-05 -> NE03-11  Wolken-Mobile       2 -> 6

Rueckmeldungen der Nutzerin eingearbeitet:
  Zustand aller Betten von gebraucht auf gut geaendert (NU03-02, NU07-01,
  BU01-01, BU02-01, NE03-03, NE03-04)
  NE03-06 Leuchtelefant: Marke Zara Home ergaenzt

Zwei Fotos maskiert: F-458 Vornamen auf den Wannenetiketten und Fotos von
Kindern, F-459 Vornamen auf den Wannenetiketten.

Die Schlafraeume sind damit durch; der offene Punkt "Betten waechst noch"
ist erledigt.

Datenbasis 371 Positionen / 315 aktiv, pruefen.py 0 Fehler.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011yyfqhuiWGsaNy38oaNoGo
</commit_message>
<xml_diff>
--- a/ausgabe/01_Artikelstamm_kikripp.xlsx
+++ b/ausgabe/01_Artikelstamm_kikripp.xlsx
@@ -15,7 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Artikelstamm'!$A$2:$AN$361</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Artikelstamm'!$A$2:$AN$373</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1019,7 +1019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN361"/>
+  <dimension ref="A1:AN373"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -22633,7 +22633,7 @@
       <c r="B177" s="15" t="n"/>
       <c r="C177" s="15" t="inlineStr">
         <is>
-          <t>NE03-02</t>
+          <t>NE03-02, NE04-01</t>
         </is>
       </c>
       <c r="D177" s="15" t="inlineStr">
@@ -22667,7 +22667,7 @@
         </is>
       </c>
       <c r="J177" s="17" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="K177" s="17" t="n"/>
       <c r="L177" s="18">
@@ -22681,7 +22681,7 @@
       </c>
       <c r="N177" s="15" t="inlineStr">
         <is>
-          <t>gebraucht</t>
+          <t>gut</t>
         </is>
       </c>
       <c r="O177" s="19" t="n"/>
@@ -22742,12 +22742,12 @@
       <c r="AL177" s="19" t="n"/>
       <c r="AM177" s="16" t="inlineStr">
         <is>
-          <t>14 Betten insgesamt: 4 im Schlafraum 4 (NU03-02) und 10 im Schlafraum 2 des Neubaus (NE03-02). Die Matratzen können auf Wunsch mitgenommen werden. Ein Bett mit Aufstiegstreppe ist auf Foto F-439 zu sehen.</t>
+          <t>16 Betten insgesamt: 4 im Schlafraum 4 (NU03-02), 10 im Schlafraum 2 (NE03-02) und 2 im Schlafraum 3 (NE04-01). Die Matratzen können auf Wunsch mitgenommen werden. Betten mit Aufstiegstreppe sind auf den Fotos F-439 und F-451 zu sehen.</t>
         </is>
       </c>
       <c r="AN177" s="22" t="inlineStr">
         <is>
-          <t>OFFEN: waechst noch. Aus den weiteren Schlafraeumen kommen zusaetzliche Betten dazu - am Ende des Rundgangs auf die Gesamtzahl bringen und die Post-it-Nummern in Weitere_ArtNr ergaenzen. Bisher: NE03-02.</t>
+          <t>Zusammengefasste Position über drei Räume – Post-it-Nummern: NE03-02, NE04-01. Der Rundgang durch die Schlafräume ist damit abgeschlossen.</t>
         </is>
       </c>
     </row>
@@ -27335,7 +27335,7 @@
       </c>
       <c r="N215" s="15" t="inlineStr">
         <is>
-          <t>gebraucht</t>
+          <t>gut</t>
         </is>
       </c>
       <c r="O215" s="19" t="n"/>
@@ -37483,7 +37483,7 @@
       </c>
       <c r="N299" s="15" t="inlineStr">
         <is>
-          <t>gebraucht</t>
+          <t>gut</t>
         </is>
       </c>
       <c r="O299" s="19" t="n"/>
@@ -38213,7 +38213,7 @@
       </c>
       <c r="N305" s="15" t="inlineStr">
         <is>
-          <t>gebraucht</t>
+          <t>gut</t>
         </is>
       </c>
       <c r="O305" s="19" t="n"/>
@@ -44076,7 +44076,7 @@
       </c>
       <c r="N354" s="15" t="inlineStr">
         <is>
-          <t>gebraucht</t>
+          <t>gut</t>
         </is>
       </c>
       <c r="O354" s="19" t="n"/>
@@ -44153,7 +44153,11 @@
         </is>
       </c>
       <c r="B355" s="15" t="n"/>
-      <c r="C355" s="15" t="n"/>
+      <c r="C355" s="15" t="inlineStr">
+        <is>
+          <t>NE04-02</t>
+        </is>
+      </c>
       <c r="D355" s="15" t="inlineStr">
         <is>
           <t>NE03</t>
@@ -44185,7 +44189,7 @@
         </is>
       </c>
       <c r="J355" s="17" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="K355" s="17" t="n"/>
       <c r="L355" s="18">
@@ -44199,7 +44203,7 @@
       </c>
       <c r="N355" s="15" t="inlineStr">
         <is>
-          <t>gebraucht</t>
+          <t>gut</t>
         </is>
       </c>
       <c r="O355" s="19" t="n"/>
@@ -44260,10 +44264,14 @@
       <c r="AL355" s="19" t="n"/>
       <c r="AM355" s="16" t="inlineStr">
         <is>
-          <t>3 Betten einschließlich Matratzen – abgebildet ist eines davon. Nestchen und Bettwäsche gehören nicht dazu.</t>
-        </is>
-      </c>
-      <c r="AN355" s="22" t="n"/>
+          <t>10 Betten einschließlich Matratzen: 3 im Schlafraum 2 (NE03-04) und 7 im Schlafraum 3 (NE04-02). Abgebildet ist eines davon, mehrere auf Foto F-452. Nestchen und Bettwäsche gehören nicht dazu.</t>
+        </is>
+      </c>
+      <c r="AN355" s="22" t="inlineStr">
+        <is>
+          <t>Zusammengefasste Position über zwei Räume – Post-it-Nummer: NE04-02.</t>
+        </is>
+      </c>
     </row>
     <row r="356" ht="30" customHeight="1">
       <c r="A356" s="15" t="inlineStr">
@@ -44408,7 +44416,7 @@
       </c>
       <c r="F357" s="16" t="inlineStr">
         <is>
-          <t>Dekoleuchte in Elefantenform aus taupefarbenem Metall mit elf Fassungen für Glühlampen auf der Vorderseite, zum Stellen.</t>
+          <t>Dekoleuchte in Elefantenform aus taupefarbenem Metall mit elf Fassungen für Glühlampen auf der Vorderseite, zum Stellen. Hersteller: Zara Home.</t>
         </is>
       </c>
       <c r="G357" s="15" t="inlineStr">
@@ -44485,7 +44493,11 @@
           <t>verfügbar</t>
         </is>
       </c>
-      <c r="AA357" s="19" t="n"/>
+      <c r="AA357" s="19" t="inlineStr">
+        <is>
+          <t>Zara Home</t>
+        </is>
+      </c>
       <c r="AB357" s="19" t="n"/>
       <c r="AC357" s="19" t="n"/>
       <c r="AD357" s="19" t="n"/>
@@ -44879,7 +44891,11 @@
         </is>
       </c>
       <c r="B361" s="15" t="n"/>
-      <c r="C361" s="15" t="n"/>
+      <c r="C361" s="15" t="inlineStr">
+        <is>
+          <t>NE04-05</t>
+        </is>
+      </c>
       <c r="D361" s="15" t="inlineStr">
         <is>
           <t>NE03</t>
@@ -44911,7 +44927,7 @@
         </is>
       </c>
       <c r="J361" s="17" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="K361" s="17" t="n"/>
       <c r="L361" s="18">
@@ -44986,13 +45002,1457 @@
       <c r="AL361" s="19" t="n"/>
       <c r="AM361" s="16" t="inlineStr">
         <is>
-          <t>2 Mobiles – abgebildet ist eines davon.</t>
-        </is>
-      </c>
-      <c r="AN361" s="22" t="n"/>
+          <t>6 Mobiles: 2 im Schlafraum 2 (NE03-11) und 4 im Schlafraum 3 (NE04-05). Abgebildet ist eines davon, ein weiteres auf Foto F-455.</t>
+        </is>
+      </c>
+      <c r="AN361" s="22" t="inlineStr">
+        <is>
+          <t>Zusammengefasste Position über zwei Räume – Post-it-Nummer: NE04-05.</t>
+        </is>
+      </c>
+    </row>
+    <row r="362" ht="30" customHeight="1">
+      <c r="A362" s="15" t="inlineStr">
+        <is>
+          <t>NE04-03</t>
+        </is>
+      </c>
+      <c r="B362" s="15" t="n"/>
+      <c r="C362" s="15" t="n"/>
+      <c r="D362" s="15" t="inlineStr">
+        <is>
+          <t>NE04</t>
+        </is>
+      </c>
+      <c r="E362" s="15" t="inlineStr">
+        <is>
+          <t>Wanddekoration Wolken schwarz</t>
+        </is>
+      </c>
+      <c r="F362" s="16" t="inlineStr">
+        <is>
+          <t>Flache Wandelemente in Wolkenform aus schwarz lackiertem Holz, zum Aufhängen.</t>
+        </is>
+      </c>
+      <c r="G362" s="15" t="inlineStr">
+        <is>
+          <t>Deko</t>
+        </is>
+      </c>
+      <c r="H362" s="15" t="inlineStr">
+        <is>
+          <t>Schlafraum 3</t>
+        </is>
+      </c>
+      <c r="I362" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J362" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K362" s="17" t="n"/>
+      <c r="L362" s="18">
+        <f>J362-IF(K362="",0,K362)</f>
+        <v/>
+      </c>
+      <c r="M362" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N362" s="15" t="inlineStr">
+        <is>
+          <t>gut</t>
+        </is>
+      </c>
+      <c r="O362" s="19" t="n"/>
+      <c r="P362" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q362" s="19" t="n"/>
+      <c r="R362" s="20" t="n"/>
+      <c r="S362" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="T362" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U362" s="21">
+        <f>L362*S362</f>
+        <v/>
+      </c>
+      <c r="V362" s="15" t="inlineStr">
+        <is>
+          <t>Versand möglich</t>
+        </is>
+      </c>
+      <c r="W362" s="15" t="inlineStr">
+        <is>
+          <t>F-453</t>
+        </is>
+      </c>
+      <c r="X362" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y362" s="19" t="n"/>
+      <c r="Z362" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA362" s="19" t="n"/>
+      <c r="AB362" s="19" t="n"/>
+      <c r="AC362" s="19" t="n"/>
+      <c r="AD362" s="19" t="n"/>
+      <c r="AE362" s="20" t="n"/>
+      <c r="AF362" s="21">
+        <f>IF(K362="","",K362*AE362)</f>
+        <v/>
+      </c>
+      <c r="AG362" s="19" t="n"/>
+      <c r="AH362" s="19" t="n"/>
+      <c r="AI362" s="19" t="n"/>
+      <c r="AJ362" s="19" t="n"/>
+      <c r="AK362" s="19" t="n"/>
+      <c r="AL362" s="19" t="n"/>
+      <c r="AM362" s="16" t="inlineStr">
+        <is>
+          <t>2 Stück, beide abgebildet. Wolken als Regal stehen unter NE03-01.</t>
+        </is>
+      </c>
+      <c r="AN362" s="22" t="n"/>
+    </row>
+    <row r="363" ht="30" customHeight="1">
+      <c r="A363" s="15" t="inlineStr">
+        <is>
+          <t>NE04-04</t>
+        </is>
+      </c>
+      <c r="B363" s="15" t="n"/>
+      <c r="C363" s="15" t="n"/>
+      <c r="D363" s="15" t="inlineStr">
+        <is>
+          <t>NE04</t>
+        </is>
+      </c>
+      <c r="E363" s="15" t="inlineStr">
+        <is>
+          <t>Schrank weiß mit zwei Türen und zwei Schubladen</t>
+        </is>
+      </c>
+      <c r="F363" s="16" t="inlineStr">
+        <is>
+          <t>Weißer Schrank mit zwei oberen Türen und zwei breiten Schubladen darunter, Griffmulden ausgeschnitten.</t>
+        </is>
+      </c>
+      <c r="G363" s="15" t="inlineStr">
+        <is>
+          <t>Möbel</t>
+        </is>
+      </c>
+      <c r="H363" s="15" t="inlineStr">
+        <is>
+          <t>Schlafraum 3</t>
+        </is>
+      </c>
+      <c r="I363" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J363" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K363" s="17" t="n"/>
+      <c r="L363" s="18">
+        <f>J363-IF(K363="",0,K363)</f>
+        <v/>
+      </c>
+      <c r="M363" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N363" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O363" s="19" t="n"/>
+      <c r="P363" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q363" s="19" t="n"/>
+      <c r="R363" s="20" t="n"/>
+      <c r="S363" s="20" t="n">
+        <v>80</v>
+      </c>
+      <c r="T363" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U363" s="21">
+        <f>L363*S363</f>
+        <v/>
+      </c>
+      <c r="V363" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W363" s="15" t="inlineStr">
+        <is>
+          <t>F-454</t>
+        </is>
+      </c>
+      <c r="X363" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y363" s="19" t="n"/>
+      <c r="Z363" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA363" s="19" t="n"/>
+      <c r="AB363" s="19" t="n"/>
+      <c r="AC363" s="19" t="n"/>
+      <c r="AD363" s="19" t="n"/>
+      <c r="AE363" s="20" t="n"/>
+      <c r="AF363" s="21">
+        <f>IF(K363="","",K363*AE363)</f>
+        <v/>
+      </c>
+      <c r="AG363" s="19" t="n"/>
+      <c r="AH363" s="19" t="n"/>
+      <c r="AI363" s="19" t="n"/>
+      <c r="AJ363" s="19" t="n"/>
+      <c r="AK363" s="19" t="n"/>
+      <c r="AL363" s="19" t="n"/>
+      <c r="AM363" s="16" t="inlineStr">
+        <is>
+          <t>1 Schrank. Der Inhalt gehört nicht dazu. Auf dem Erfassungsblatt als Kommode mit zwei Schubladen geführt.</t>
+        </is>
+      </c>
+      <c r="AN363" s="22" t="n"/>
+    </row>
+    <row r="364" ht="30" customHeight="1">
+      <c r="A364" s="15" t="inlineStr">
+        <is>
+          <t>NE04-06</t>
+        </is>
+      </c>
+      <c r="B364" s="15" t="n"/>
+      <c r="C364" s="15" t="n"/>
+      <c r="D364" s="15" t="inlineStr">
+        <is>
+          <t>NE04</t>
+        </is>
+      </c>
+      <c r="E364" s="15" t="inlineStr">
+        <is>
+          <t>Wandspiegel in Wolkenform, weiß</t>
+        </is>
+      </c>
+      <c r="F364" s="16" t="inlineStr">
+        <is>
+          <t>Wandspiegel in Wolkenform mit breitem weiß lackiertem Holzrahmen.</t>
+        </is>
+      </c>
+      <c r="G364" s="15" t="inlineStr">
+        <is>
+          <t>Deko</t>
+        </is>
+      </c>
+      <c r="H364" s="15" t="inlineStr">
+        <is>
+          <t>Schlafraum 3</t>
+        </is>
+      </c>
+      <c r="I364" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J364" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K364" s="17" t="n"/>
+      <c r="L364" s="18">
+        <f>J364-IF(K364="",0,K364)</f>
+        <v/>
+      </c>
+      <c r="M364" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N364" s="15" t="inlineStr">
+        <is>
+          <t>gut</t>
+        </is>
+      </c>
+      <c r="O364" s="19" t="n"/>
+      <c r="P364" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q364" s="19" t="n"/>
+      <c r="R364" s="20" t="n"/>
+      <c r="S364" s="20" t="n">
+        <v>45</v>
+      </c>
+      <c r="T364" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U364" s="21">
+        <f>L364*S364</f>
+        <v/>
+      </c>
+      <c r="V364" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W364" s="15" t="inlineStr">
+        <is>
+          <t>F-456</t>
+        </is>
+      </c>
+      <c r="X364" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y364" s="19" t="n"/>
+      <c r="Z364" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA364" s="19" t="n"/>
+      <c r="AB364" s="19" t="n"/>
+      <c r="AC364" s="19" t="n"/>
+      <c r="AD364" s="19" t="n"/>
+      <c r="AE364" s="20" t="n"/>
+      <c r="AF364" s="21">
+        <f>IF(K364="","",K364*AE364)</f>
+        <v/>
+      </c>
+      <c r="AG364" s="19" t="n"/>
+      <c r="AH364" s="19" t="n"/>
+      <c r="AI364" s="19" t="n"/>
+      <c r="AJ364" s="19" t="n"/>
+      <c r="AK364" s="19" t="n"/>
+      <c r="AL364" s="19" t="n"/>
+      <c r="AM364" s="16" t="inlineStr">
+        <is>
+          <t>1 Spiegel.</t>
+        </is>
+      </c>
+      <c r="AN364" s="22" t="n"/>
+    </row>
+    <row r="365" ht="30" customHeight="1">
+      <c r="A365" s="15" t="inlineStr">
+        <is>
+          <t>NE04-07</t>
+        </is>
+      </c>
+      <c r="B365" s="15" t="n"/>
+      <c r="C365" s="15" t="n"/>
+      <c r="D365" s="15" t="inlineStr">
+        <is>
+          <t>NE04</t>
+        </is>
+      </c>
+      <c r="E365" s="15" t="inlineStr">
+        <is>
+          <t>Wesco Wickelauflage beige</t>
+        </is>
+      </c>
+      <c r="F365" s="16" t="inlineStr">
+        <is>
+          <t>Große Wickelauflage von Wesco mit beigem Kunstlederbezug und umlaufendem Rand.</t>
+        </is>
+      </c>
+      <c r="G365" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H365" s="15" t="inlineStr">
+        <is>
+          <t>Schlafraum 3</t>
+        </is>
+      </c>
+      <c r="I365" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J365" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K365" s="17" t="n"/>
+      <c r="L365" s="18">
+        <f>J365-IF(K365="",0,K365)</f>
+        <v/>
+      </c>
+      <c r="M365" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N365" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O365" s="19" t="n"/>
+      <c r="P365" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q365" s="19" t="n"/>
+      <c r="R365" s="20" t="n"/>
+      <c r="S365" s="20" t="n">
+        <v>45</v>
+      </c>
+      <c r="T365" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U365" s="21">
+        <f>L365*S365</f>
+        <v/>
+      </c>
+      <c r="V365" s="15" t="inlineStr">
+        <is>
+          <t>Versand möglich</t>
+        </is>
+      </c>
+      <c r="W365" s="15" t="inlineStr">
+        <is>
+          <t>F-457</t>
+        </is>
+      </c>
+      <c r="X365" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y365" s="19" t="n"/>
+      <c r="Z365" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA365" s="19" t="inlineStr">
+        <is>
+          <t>Wesco</t>
+        </is>
+      </c>
+      <c r="AB365" s="19" t="n"/>
+      <c r="AC365" s="19" t="n"/>
+      <c r="AD365" s="19" t="n"/>
+      <c r="AE365" s="20" t="n"/>
+      <c r="AF365" s="21">
+        <f>IF(K365="","",K365*AE365)</f>
+        <v/>
+      </c>
+      <c r="AG365" s="19" t="n"/>
+      <c r="AH365" s="19" t="n"/>
+      <c r="AI365" s="19" t="n"/>
+      <c r="AJ365" s="19" t="n"/>
+      <c r="AK365" s="19" t="n"/>
+      <c r="AL365" s="19" t="n"/>
+      <c r="AM365" s="16" t="inlineStr">
+        <is>
+          <t>2 Auflagen – abgebildet ist eine davon.</t>
+        </is>
+      </c>
+      <c r="AN365" s="22" t="n"/>
+    </row>
+    <row r="366" ht="30" customHeight="1">
+      <c r="A366" s="15" t="inlineStr">
+        <is>
+          <t>NE04-08</t>
+        </is>
+      </c>
+      <c r="B366" s="15" t="n"/>
+      <c r="C366" s="15" t="n"/>
+      <c r="D366" s="15" t="inlineStr">
+        <is>
+          <t>NE04</t>
+        </is>
+      </c>
+      <c r="E366" s="15" t="inlineStr">
+        <is>
+          <t>Wickelkommode Buche mit zehn Wannen</t>
+        </is>
+      </c>
+      <c r="F366" s="16" t="inlineStr">
+        <is>
+          <t>Wickelkommode aus Buche-Dekor mit weißer Wickelfläche und umlaufender Aufkantung, darunter zehn herausziehbare Kunststoffwannen in zwei Reihen.</t>
+        </is>
+      </c>
+      <c r="G366" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H366" s="15" t="inlineStr">
+        <is>
+          <t>Schlafraum 3</t>
+        </is>
+      </c>
+      <c r="I366" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J366" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K366" s="17" t="n"/>
+      <c r="L366" s="18">
+        <f>J366-IF(K366="",0,K366)</f>
+        <v/>
+      </c>
+      <c r="M366" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N366" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O366" s="19" t="n"/>
+      <c r="P366" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q366" s="19" t="n"/>
+      <c r="R366" s="20" t="n"/>
+      <c r="S366" s="20" t="n">
+        <v>180</v>
+      </c>
+      <c r="T366" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U366" s="21">
+        <f>L366*S366</f>
+        <v/>
+      </c>
+      <c r="V366" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W366" s="15" t="inlineStr">
+        <is>
+          <t>F-458</t>
+        </is>
+      </c>
+      <c r="X366" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y366" s="19" t="n"/>
+      <c r="Z366" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA366" s="19" t="n"/>
+      <c r="AB366" s="19" t="n"/>
+      <c r="AC366" s="19" t="n"/>
+      <c r="AD366" s="19" t="n"/>
+      <c r="AE366" s="20" t="n"/>
+      <c r="AF366" s="21">
+        <f>IF(K366="","",K366*AE366)</f>
+        <v/>
+      </c>
+      <c r="AG366" s="19" t="n"/>
+      <c r="AH366" s="19" t="n"/>
+      <c r="AI366" s="19" t="n"/>
+      <c r="AJ366" s="19" t="n"/>
+      <c r="AK366" s="19" t="n"/>
+      <c r="AL366" s="19" t="n"/>
+      <c r="AM366" s="16" t="inlineStr">
+        <is>
+          <t>1 Kommode einschließlich der Wannen. Wickelauflage und Inhalt gehören nicht dazu. Die Namensschilder an den Wannen sind auf dem Foto unkenntlich gemacht und werden vor der Übergabe entfernt.</t>
+        </is>
+      </c>
+      <c r="AN366" s="22" t="n"/>
+    </row>
+    <row r="367" ht="30" customHeight="1">
+      <c r="A367" s="15" t="inlineStr">
+        <is>
+          <t>NE04-09</t>
+        </is>
+      </c>
+      <c r="B367" s="15" t="n"/>
+      <c r="C367" s="15" t="n"/>
+      <c r="D367" s="15" t="inlineStr">
+        <is>
+          <t>NE04</t>
+        </is>
+      </c>
+      <c r="E367" s="15" t="inlineStr">
+        <is>
+          <t>Wickelkommode Buche groß mit Treppe</t>
+        </is>
+      </c>
+      <c r="F367" s="16" t="inlineStr">
+        <is>
+          <t>Große Wickelkommode aus Buche-Dekor mit weißer Wickelfläche und Aufkantung: in der Mitte eine herausrollbare Treppe für den Aufstieg, links und rechts je fünf herausziehbare Kunststoffwannen.</t>
+        </is>
+      </c>
+      <c r="G367" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H367" s="15" t="inlineStr">
+        <is>
+          <t>Schlafraum 3</t>
+        </is>
+      </c>
+      <c r="I367" s="15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J367" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K367" s="17" t="n"/>
+      <c r="L367" s="18">
+        <f>J367-IF(K367="",0,K367)</f>
+        <v/>
+      </c>
+      <c r="M367" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N367" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O367" s="19" t="n"/>
+      <c r="P367" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q367" s="19" t="n"/>
+      <c r="R367" s="20" t="n"/>
+      <c r="S367" s="20" t="n">
+        <v>250</v>
+      </c>
+      <c r="T367" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U367" s="21">
+        <f>L367*S367</f>
+        <v/>
+      </c>
+      <c r="V367" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W367" s="15" t="inlineStr">
+        <is>
+          <t>F-459</t>
+        </is>
+      </c>
+      <c r="X367" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y367" s="19" t="n"/>
+      <c r="Z367" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA367" s="19" t="n"/>
+      <c r="AB367" s="19" t="n"/>
+      <c r="AC367" s="19" t="n"/>
+      <c r="AD367" s="19" t="n"/>
+      <c r="AE367" s="20" t="n"/>
+      <c r="AF367" s="21">
+        <f>IF(K367="","",K367*AE367)</f>
+        <v/>
+      </c>
+      <c r="AG367" s="19" t="n"/>
+      <c r="AH367" s="19" t="n"/>
+      <c r="AI367" s="19" t="n"/>
+      <c r="AJ367" s="19" t="n"/>
+      <c r="AK367" s="19" t="n"/>
+      <c r="AL367" s="19" t="n"/>
+      <c r="AM367" s="16" t="inlineStr">
+        <is>
+          <t>2 Kommoden einschließlich Treppe und Wannen – abgebildet ist eine davon. Der Inhalt gehört nicht dazu. Die Namensschilder an den Wannen sind auf dem Foto unkenntlich gemacht und werden vor der Übergabe entfernt.</t>
+        </is>
+      </c>
+      <c r="AN367" s="22" t="n"/>
+    </row>
+    <row r="368" ht="30" customHeight="1">
+      <c r="A368" s="15" t="inlineStr">
+        <is>
+          <t>NE04-10</t>
+        </is>
+      </c>
+      <c r="B368" s="15" t="n"/>
+      <c r="C368" s="15" t="n"/>
+      <c r="D368" s="15" t="inlineStr">
+        <is>
+          <t>NE04</t>
+        </is>
+      </c>
+      <c r="E368" s="15" t="inlineStr">
+        <is>
+          <t>Wickelkommode mit Türen und Fachböden</t>
+        </is>
+      </c>
+      <c r="F368" s="16" t="inlineStr">
+        <is>
+          <t>Wickelkommode aus Buche-Dekor mit weißer Wickelfläche und Aufkantung, geschlossener Unterbau mit zwei Türen und drei Fachböden.</t>
+        </is>
+      </c>
+      <c r="G368" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H368" s="15" t="inlineStr">
+        <is>
+          <t>Schlafraum 3</t>
+        </is>
+      </c>
+      <c r="I368" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J368" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K368" s="17" t="n"/>
+      <c r="L368" s="18">
+        <f>J368-IF(K368="",0,K368)</f>
+        <v/>
+      </c>
+      <c r="M368" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N368" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O368" s="19" t="n"/>
+      <c r="P368" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q368" s="19" t="n"/>
+      <c r="R368" s="20" t="n"/>
+      <c r="S368" s="20" t="n">
+        <v>180</v>
+      </c>
+      <c r="T368" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U368" s="21">
+        <f>L368*S368</f>
+        <v/>
+      </c>
+      <c r="V368" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W368" s="15" t="inlineStr">
+        <is>
+          <t>F-460</t>
+        </is>
+      </c>
+      <c r="X368" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y368" s="19" t="n"/>
+      <c r="Z368" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA368" s="19" t="n"/>
+      <c r="AB368" s="19" t="n"/>
+      <c r="AC368" s="19" t="n"/>
+      <c r="AD368" s="19" t="n"/>
+      <c r="AE368" s="20" t="n"/>
+      <c r="AF368" s="21">
+        <f>IF(K368="","",K368*AE368)</f>
+        <v/>
+      </c>
+      <c r="AG368" s="19" t="n"/>
+      <c r="AH368" s="19" t="n"/>
+      <c r="AI368" s="19" t="n"/>
+      <c r="AJ368" s="19" t="n"/>
+      <c r="AK368" s="19" t="n"/>
+      <c r="AL368" s="19" t="n"/>
+      <c r="AM368" s="16" t="inlineStr">
+        <is>
+          <t>1 Kommode. Wickelauflage, Kisten und Inhalt gehören nicht dazu.</t>
+        </is>
+      </c>
+      <c r="AN368" s="22" t="n"/>
+    </row>
+    <row r="369" ht="30" customHeight="1">
+      <c r="A369" s="15" t="inlineStr">
+        <is>
+          <t>NE04-11</t>
+        </is>
+      </c>
+      <c r="B369" s="15" t="n"/>
+      <c r="C369" s="15" t="n"/>
+      <c r="D369" s="15" t="inlineStr">
+        <is>
+          <t>NE04</t>
+        </is>
+      </c>
+      <c r="E369" s="15" t="inlineStr">
+        <is>
+          <t>Baby Jogger City Select Kinderwagen, rot</t>
+        </is>
+      </c>
+      <c r="F369" s="16" t="inlineStr">
+        <is>
+          <t>Kinderwagen Baby Jogger City Select in Rot mit Verdeck, Fünfpunktgurt, Einkaufskorb und luftbereiften Rädern. Aufdruck am Rahmen: city select by baby jogger. Der Rahmen ist an mehreren Stellen abgeschabt.</t>
+        </is>
+      </c>
+      <c r="G369" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H369" s="15" t="inlineStr">
+        <is>
+          <t>Schlafraum 3</t>
+        </is>
+      </c>
+      <c r="I369" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J369" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K369" s="17" t="n"/>
+      <c r="L369" s="18">
+        <f>J369-IF(K369="",0,K369)</f>
+        <v/>
+      </c>
+      <c r="M369" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N369" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O369" s="19" t="n"/>
+      <c r="P369" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q369" s="19" t="n"/>
+      <c r="R369" s="20" t="n"/>
+      <c r="S369" s="20" t="n">
+        <v>180</v>
+      </c>
+      <c r="T369" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U369" s="21">
+        <f>L369*S369</f>
+        <v/>
+      </c>
+      <c r="V369" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W369" s="15" t="inlineStr">
+        <is>
+          <t>F-461</t>
+        </is>
+      </c>
+      <c r="X369" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y369" s="19" t="n"/>
+      <c r="Z369" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA369" s="19" t="inlineStr">
+        <is>
+          <t>Baby Jogger</t>
+        </is>
+      </c>
+      <c r="AB369" s="19" t="n"/>
+      <c r="AC369" s="19" t="n"/>
+      <c r="AD369" s="19" t="n"/>
+      <c r="AE369" s="20" t="n"/>
+      <c r="AF369" s="21">
+        <f>IF(K369="","",K369*AE369)</f>
+        <v/>
+      </c>
+      <c r="AG369" s="19" t="n"/>
+      <c r="AH369" s="19" t="n"/>
+      <c r="AI369" s="19" t="n"/>
+      <c r="AJ369" s="19" t="n"/>
+      <c r="AK369" s="19" t="n"/>
+      <c r="AL369" s="19" t="n"/>
+      <c r="AM369" s="16" t="inlineStr">
+        <is>
+          <t>1 Wagen. Das Gestell mit Rädern ist auf Foto F-462 zu sehen.</t>
+        </is>
+      </c>
+      <c r="AN369" s="22" t="n"/>
+    </row>
+    <row r="370" ht="30" customHeight="1">
+      <c r="A370" s="15" t="inlineStr">
+        <is>
+          <t>NE04-12</t>
+        </is>
+      </c>
+      <c r="B370" s="15" t="n"/>
+      <c r="C370" s="15" t="n"/>
+      <c r="D370" s="15" t="inlineStr">
+        <is>
+          <t>NE04</t>
+        </is>
+      </c>
+      <c r="E370" s="15" t="inlineStr">
+        <is>
+          <t>Hochflorteppich rund, rot-orange</t>
+        </is>
+      </c>
+      <c r="F370" s="16" t="inlineStr">
+        <is>
+          <t>Runder Hochflorteppich in melierten Rot-, Orange- und Violetttönen.</t>
+        </is>
+      </c>
+      <c r="G370" s="15" t="inlineStr">
+        <is>
+          <t>Textilien</t>
+        </is>
+      </c>
+      <c r="H370" s="15" t="inlineStr">
+        <is>
+          <t>Schlafraum 3</t>
+        </is>
+      </c>
+      <c r="I370" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J370" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K370" s="17" t="n"/>
+      <c r="L370" s="18">
+        <f>J370-IF(K370="",0,K370)</f>
+        <v/>
+      </c>
+      <c r="M370" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N370" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O370" s="19" t="inlineStr">
+        <is>
+          <t>Ø ca. 200 cm</t>
+        </is>
+      </c>
+      <c r="P370" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q370" s="19" t="n"/>
+      <c r="R370" s="20" t="n"/>
+      <c r="S370" s="20" t="n">
+        <v>60</v>
+      </c>
+      <c r="T370" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U370" s="21">
+        <f>L370*S370</f>
+        <v/>
+      </c>
+      <c r="V370" s="15" t="inlineStr">
+        <is>
+          <t>Versand möglich</t>
+        </is>
+      </c>
+      <c r="W370" s="15" t="inlineStr">
+        <is>
+          <t>F-463</t>
+        </is>
+      </c>
+      <c r="X370" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y370" s="19" t="n"/>
+      <c r="Z370" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA370" s="19" t="n"/>
+      <c r="AB370" s="19" t="n"/>
+      <c r="AC370" s="19" t="n"/>
+      <c r="AD370" s="19" t="n"/>
+      <c r="AE370" s="20" t="n"/>
+      <c r="AF370" s="21">
+        <f>IF(K370="","",K370*AE370)</f>
+        <v/>
+      </c>
+      <c r="AG370" s="19" t="n"/>
+      <c r="AH370" s="19" t="n"/>
+      <c r="AI370" s="19" t="n"/>
+      <c r="AJ370" s="19" t="n"/>
+      <c r="AK370" s="19" t="n"/>
+      <c r="AL370" s="19" t="n"/>
+      <c r="AM370" s="16" t="inlineStr">
+        <is>
+          <t>1 Teppich, Maß vom Erfassungsblatt. Der Flor ist auf Foto F-464 aus der Nähe zu sehen.</t>
+        </is>
+      </c>
+      <c r="AN370" s="22" t="n"/>
+    </row>
+    <row r="371" ht="30" customHeight="1">
+      <c r="A371" s="15" t="inlineStr">
+        <is>
+          <t>NE04-13</t>
+        </is>
+      </c>
+      <c r="B371" s="15" t="n"/>
+      <c r="C371" s="15" t="n"/>
+      <c r="D371" s="15" t="inlineStr">
+        <is>
+          <t>NE04</t>
+        </is>
+      </c>
+      <c r="E371" s="15" t="inlineStr">
+        <is>
+          <t>Windeleimer weiß mit Deckel</t>
+        </is>
+      </c>
+      <c r="F371" s="16" t="inlineStr">
+        <is>
+          <t>Hoher Windeleimer aus weißem Kunststoff mit aufklappbarem Deckel, Dichtring und Fußpedal.</t>
+        </is>
+      </c>
+      <c r="G371" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H371" s="15" t="inlineStr">
+        <is>
+          <t>Schlafraum 3</t>
+        </is>
+      </c>
+      <c r="I371" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J371" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K371" s="17" t="n"/>
+      <c r="L371" s="18">
+        <f>J371-IF(K371="",0,K371)</f>
+        <v/>
+      </c>
+      <c r="M371" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N371" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O371" s="19" t="n"/>
+      <c r="P371" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q371" s="19" t="n"/>
+      <c r="R371" s="20" t="n"/>
+      <c r="S371" s="20" t="n">
+        <v>25</v>
+      </c>
+      <c r="T371" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U371" s="21">
+        <f>L371*S371</f>
+        <v/>
+      </c>
+      <c r="V371" s="15" t="inlineStr">
+        <is>
+          <t>Versand möglich</t>
+        </is>
+      </c>
+      <c r="W371" s="15" t="inlineStr">
+        <is>
+          <t>F-465</t>
+        </is>
+      </c>
+      <c r="X371" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y371" s="19" t="n"/>
+      <c r="Z371" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA371" s="19" t="n"/>
+      <c r="AB371" s="19" t="n"/>
+      <c r="AC371" s="19" t="n"/>
+      <c r="AD371" s="19" t="n"/>
+      <c r="AE371" s="20" t="n"/>
+      <c r="AF371" s="21">
+        <f>IF(K371="","",K371*AE371)</f>
+        <v/>
+      </c>
+      <c r="AG371" s="19" t="n"/>
+      <c r="AH371" s="19" t="n"/>
+      <c r="AI371" s="19" t="n"/>
+      <c r="AJ371" s="19" t="n"/>
+      <c r="AK371" s="19" t="n"/>
+      <c r="AL371" s="19" t="n"/>
+      <c r="AM371" s="16" t="inlineStr">
+        <is>
+          <t>2 Eimer – abgebildet ist einer davon.</t>
+        </is>
+      </c>
+      <c r="AN371" s="22" t="n"/>
+    </row>
+    <row r="372" ht="30" customHeight="1">
+      <c r="A372" s="15" t="inlineStr">
+        <is>
+          <t>NE04-14</t>
+        </is>
+      </c>
+      <c r="B372" s="15" t="n"/>
+      <c r="C372" s="15" t="n"/>
+      <c r="D372" s="15" t="inlineStr">
+        <is>
+          <t>NE04</t>
+        </is>
+      </c>
+      <c r="E372" s="15" t="inlineStr">
+        <is>
+          <t>Wandregal in Bergform, Holz</t>
+        </is>
+      </c>
+      <c r="F372" s="16" t="inlineStr">
+        <is>
+          <t>Wandregal in Form einer Bergkette aus hellem Holz mit weiß lackierten Gipfeln, durchgehender Ablageboden.</t>
+        </is>
+      </c>
+      <c r="G372" s="15" t="inlineStr">
+        <is>
+          <t>Deko</t>
+        </is>
+      </c>
+      <c r="H372" s="15" t="inlineStr">
+        <is>
+          <t>Schlafraum 3</t>
+        </is>
+      </c>
+      <c r="I372" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J372" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="K372" s="17" t="n"/>
+      <c r="L372" s="18">
+        <f>J372-IF(K372="",0,K372)</f>
+        <v/>
+      </c>
+      <c r="M372" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N372" s="15" t="inlineStr">
+        <is>
+          <t>gut</t>
+        </is>
+      </c>
+      <c r="O372" s="19" t="n"/>
+      <c r="P372" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q372" s="19" t="n"/>
+      <c r="R372" s="20" t="n"/>
+      <c r="S372" s="20" t="n">
+        <v>25</v>
+      </c>
+      <c r="T372" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U372" s="21">
+        <f>L372*S372</f>
+        <v/>
+      </c>
+      <c r="V372" s="15" t="inlineStr">
+        <is>
+          <t>Versand möglich</t>
+        </is>
+      </c>
+      <c r="W372" s="15" t="inlineStr">
+        <is>
+          <t>F-466</t>
+        </is>
+      </c>
+      <c r="X372" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y372" s="19" t="n"/>
+      <c r="Z372" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA372" s="19" t="n"/>
+      <c r="AB372" s="19" t="n"/>
+      <c r="AC372" s="19" t="n"/>
+      <c r="AD372" s="19" t="n"/>
+      <c r="AE372" s="20" t="n"/>
+      <c r="AF372" s="21">
+        <f>IF(K372="","",K372*AE372)</f>
+        <v/>
+      </c>
+      <c r="AG372" s="19" t="n"/>
+      <c r="AH372" s="19" t="n"/>
+      <c r="AI372" s="19" t="n"/>
+      <c r="AJ372" s="19" t="n"/>
+      <c r="AK372" s="19" t="n"/>
+      <c r="AL372" s="19" t="n"/>
+      <c r="AM372" s="16" t="inlineStr">
+        <is>
+          <t>3 Regale – abgebildet ist eines davon.</t>
+        </is>
+      </c>
+      <c r="AN372" s="22" t="n"/>
+    </row>
+    <row r="373" ht="30" customHeight="1">
+      <c r="A373" s="15" t="inlineStr">
+        <is>
+          <t>NE04-15</t>
+        </is>
+      </c>
+      <c r="B373" s="15" t="n"/>
+      <c r="C373" s="15" t="n"/>
+      <c r="D373" s="15" t="inlineStr">
+        <is>
+          <t>NE04</t>
+        </is>
+      </c>
+      <c r="E373" s="15" t="inlineStr">
+        <is>
+          <t>Mobile Holzbogen mit Filzkugeln</t>
+        </is>
+      </c>
+      <c r="F373" s="16" t="inlineStr">
+        <is>
+          <t>Mobile mit geschwungenem Bogen aus Birkenholz, daran Filzkugeln in Rot, Grau und Weiß sowie Sterne und Häuschen aus Holz und Filz in Schwarz, Grau und Natur.</t>
+        </is>
+      </c>
+      <c r="G373" s="15" t="inlineStr">
+        <is>
+          <t>Deko</t>
+        </is>
+      </c>
+      <c r="H373" s="15" t="inlineStr">
+        <is>
+          <t>Schlafraum 3</t>
+        </is>
+      </c>
+      <c r="I373" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J373" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="K373" s="17" t="n"/>
+      <c r="L373" s="18">
+        <f>J373-IF(K373="",0,K373)</f>
+        <v/>
+      </c>
+      <c r="M373" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N373" s="15" t="inlineStr">
+        <is>
+          <t>gut</t>
+        </is>
+      </c>
+      <c r="O373" s="19" t="n"/>
+      <c r="P373" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q373" s="19" t="n"/>
+      <c r="R373" s="20" t="n"/>
+      <c r="S373" s="20" t="n">
+        <v>25</v>
+      </c>
+      <c r="T373" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U373" s="21">
+        <f>L373*S373</f>
+        <v/>
+      </c>
+      <c r="V373" s="15" t="inlineStr">
+        <is>
+          <t>Versand möglich</t>
+        </is>
+      </c>
+      <c r="W373" s="15" t="inlineStr">
+        <is>
+          <t>F-467</t>
+        </is>
+      </c>
+      <c r="X373" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y373" s="19" t="n"/>
+      <c r="Z373" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA373" s="19" t="n"/>
+      <c r="AB373" s="19" t="n"/>
+      <c r="AC373" s="19" t="n"/>
+      <c r="AD373" s="19" t="n"/>
+      <c r="AE373" s="20" t="n"/>
+      <c r="AF373" s="21">
+        <f>IF(K373="","",K373*AE373)</f>
+        <v/>
+      </c>
+      <c r="AG373" s="19" t="n"/>
+      <c r="AH373" s="19" t="n"/>
+      <c r="AI373" s="19" t="n"/>
+      <c r="AJ373" s="19" t="n"/>
+      <c r="AK373" s="19" t="n"/>
+      <c r="AL373" s="19" t="n"/>
+      <c r="AM373" s="16" t="inlineStr">
+        <is>
+          <t>3 Mobiles – abgebildet ist eines davon.</t>
+        </is>
+      </c>
+      <c r="AN373" s="22" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:AN361"/>
+  <autoFilter ref="A2:AN373"/>
   <mergeCells count="7">
     <mergeCell ref="AI1:AL1"/>
     <mergeCell ref="V1:AD1"/>
@@ -45002,7 +46462,7 @@
     <mergeCell ref="AE1:AH1"/>
     <mergeCell ref="AM1:AN1"/>
   </mergeCells>
-  <conditionalFormatting sqref="Z3:Z361">
+  <conditionalFormatting sqref="Z3:Z373">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"reserviert"</formula>
     </cfRule>
@@ -45013,12 +46473,12 @@
       <formula>"verkauft"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I3:I361">
+  <conditionalFormatting sqref="I3:I373">
     <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
       <formula>"A"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P3:P361">
+  <conditionalFormatting sqref="P3:P373">
     <cfRule type="cellIs" priority="5" operator="equal" dxfId="4">
       <formula>"entfällt"</formula>
     </cfRule>
@@ -45071,7 +46531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D97"/>
+  <dimension ref="A1:D98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -45109,7 +46569,7 @@
         </is>
       </c>
       <c r="B5" s="27">
-        <f>COUNTA(Artikelstamm!$A$3:$A$361)</f>
+        <f>COUNTA(Artikelstamm!$A$3:$A$373)</f>
         <v/>
       </c>
     </row>
@@ -45120,7 +46580,7 @@
         </is>
       </c>
       <c r="B6" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$361,"verfügbar")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$373,"verfügbar")</f>
         <v/>
       </c>
     </row>
@@ -45131,7 +46591,7 @@
         </is>
       </c>
       <c r="B7" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$361,"reserviert")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$373,"reserviert")</f>
         <v/>
       </c>
     </row>
@@ -45142,7 +46602,7 @@
         </is>
       </c>
       <c r="B8" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$361,"teilverkauft")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$373,"teilverkauft")</f>
         <v/>
       </c>
     </row>
@@ -45153,7 +46613,7 @@
         </is>
       </c>
       <c r="B9" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$361,"verkauft")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$373,"verkauft")</f>
         <v/>
       </c>
     </row>
@@ -45164,7 +46624,7 @@
         </is>
       </c>
       <c r="B10" s="27">
-        <f>SUM(Artikelstamm!$L$3:$L$361)</f>
+        <f>SUM(Artikelstamm!$L$3:$L$373)</f>
         <v/>
       </c>
     </row>
@@ -45175,7 +46635,7 @@
         </is>
       </c>
       <c r="B11" s="29">
-        <f>SUM(Artikelstamm!$U$3:$U$361)</f>
+        <f>SUM(Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
@@ -45193,7 +46653,7 @@
         </is>
       </c>
       <c r="B13" s="27">
-        <f>SUM(Artikelstamm!$K$3:$K$361)</f>
+        <f>SUM(Artikelstamm!$K$3:$K$373)</f>
         <v/>
       </c>
     </row>
@@ -45204,7 +46664,7 @@
         </is>
       </c>
       <c r="B14" s="30">
-        <f>SUMPRODUCT(Artikelstamm!$K$3:$K$361,Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT(Artikelstamm!$K$3:$K$373,Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
     </row>
@@ -45237,7 +46697,7 @@
         </is>
       </c>
       <c r="B17" s="30">
-        <f>SUMPRODUCT((Artikelstamm!$AJ$3:$AJ$361="bezahlt")*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AJ$3:$AJ$373="bezahlt")*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
     </row>
@@ -45266,7 +46726,7 @@
         </is>
       </c>
       <c r="B21" s="31">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$361,"*verkauft",Artikelstamm!$AI$3:$AI$361,"")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$373,"*verkauft",Artikelstamm!$AI$3:$AI$373,"")</f>
         <v/>
       </c>
     </row>
@@ -45277,7 +46737,7 @@
         </is>
       </c>
       <c r="B22" s="31">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$361,"*verkauft",Artikelstamm!$AJ$3:$AJ$361,"offen")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$373,"*verkauft",Artikelstamm!$AJ$3:$AJ$373,"offen")</f>
         <v/>
       </c>
     </row>
@@ -45288,7 +46748,7 @@
         </is>
       </c>
       <c r="B23" s="27">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$361,"reserviert",Artikelstamm!$AL$3:$AL$361,"")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$373,"reserviert",Artikelstamm!$AL$3:$AL$373,"")</f>
         <v/>
       </c>
     </row>
@@ -45299,7 +46759,7 @@
         </is>
       </c>
       <c r="B24" s="27">
-        <f>COUNTIFS(Artikelstamm!$S$3:$S$361,"")</f>
+        <f>COUNTIFS(Artikelstamm!$S$3:$S$373,"")</f>
         <v/>
       </c>
     </row>
@@ -45310,7 +46770,7 @@
         </is>
       </c>
       <c r="B25" s="27">
-        <f>COUNTIFS(Artikelstamm!$O$3:$O$361,"")</f>
+        <f>COUNTIFS(Artikelstamm!$O$3:$O$373,"")</f>
         <v/>
       </c>
     </row>
@@ -45350,15 +46810,15 @@
         </is>
       </c>
       <c r="B30" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$361,$A30)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$373,$A30)</f>
         <v/>
       </c>
       <c r="C30" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$361=$A30)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$373=$A30)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D30" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$361,$A30,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$373,$A30,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
@@ -45369,15 +46829,15 @@
         </is>
       </c>
       <c r="B31" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$361,$A31)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$373,$A31)</f>
         <v/>
       </c>
       <c r="C31" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$361=$A31)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$373=$A31)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D31" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$361,$A31,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$373,$A31,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
@@ -45388,15 +46848,15 @@
         </is>
       </c>
       <c r="B32" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$361,$A32)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$373,$A32)</f>
         <v/>
       </c>
       <c r="C32" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$361=$A32)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$373=$A32)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D32" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$361,$A32,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$373,$A32,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
@@ -45455,15 +46915,15 @@
         </is>
       </c>
       <c r="B37" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$361,$A37)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$373,$A37)</f>
         <v/>
       </c>
       <c r="C37" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$361=$A37)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$373=$A37)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D37" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$361,$A37,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$373,$A37,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
@@ -45474,15 +46934,15 @@
         </is>
       </c>
       <c r="B38" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$361,$A38)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$373,$A38)</f>
         <v/>
       </c>
       <c r="C38" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$361=$A38)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$373=$A38)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D38" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$361,$A38,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$373,$A38,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
@@ -45493,15 +46953,15 @@
         </is>
       </c>
       <c r="B39" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$361,$A39)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$373,$A39)</f>
         <v/>
       </c>
       <c r="C39" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$361=$A39)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$373=$A39)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D39" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$361,$A39,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$373,$A39,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
@@ -45512,15 +46972,15 @@
         </is>
       </c>
       <c r="B40" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$361,$A40)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$373,$A40)</f>
         <v/>
       </c>
       <c r="C40" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$361=$A40)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$373=$A40)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D40" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$361,$A40,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$373,$A40,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
@@ -45531,15 +46991,15 @@
         </is>
       </c>
       <c r="B41" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$361,$A41)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$373,$A41)</f>
         <v/>
       </c>
       <c r="C41" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$361=$A41)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$373=$A41)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D41" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$361,$A41,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$373,$A41,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
@@ -45550,15 +47010,15 @@
         </is>
       </c>
       <c r="B42" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$361,$A42)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$373,$A42)</f>
         <v/>
       </c>
       <c r="C42" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$361=$A42)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$373=$A42)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D42" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$361,$A42,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$373,$A42,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
@@ -45569,15 +47029,15 @@
         </is>
       </c>
       <c r="B43" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$361,$A43)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$373,$A43)</f>
         <v/>
       </c>
       <c r="C43" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$361=$A43)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$373=$A43)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D43" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$361,$A43,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$373,$A43,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
@@ -45588,15 +47048,15 @@
         </is>
       </c>
       <c r="B44" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$361,$A44)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$373,$A44)</f>
         <v/>
       </c>
       <c r="C44" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$361=$A44)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$373=$A44)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D44" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$361,$A44,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$373,$A44,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
@@ -45607,15 +47067,15 @@
         </is>
       </c>
       <c r="B45" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$361,$A45)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$373,$A45)</f>
         <v/>
       </c>
       <c r="C45" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$361=$A45)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$373=$A45)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D45" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$361,$A45,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$373,$A45,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
@@ -45626,15 +47086,15 @@
         </is>
       </c>
       <c r="B46" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$361,$A46)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$373,$A46)</f>
         <v/>
       </c>
       <c r="C46" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$361=$A46)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$373=$A46)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D46" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$361,$A46,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$373,$A46,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
@@ -45645,15 +47105,15 @@
         </is>
       </c>
       <c r="B47" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$361,$A47)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$373,$A47)</f>
         <v/>
       </c>
       <c r="C47" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$361=$A47)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$373=$A47)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D47" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$361,$A47,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$373,$A47,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
@@ -45664,15 +47124,15 @@
         </is>
       </c>
       <c r="B48" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$361,$A48)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$373,$A48)</f>
         <v/>
       </c>
       <c r="C48" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$361=$A48)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$373=$A48)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D48" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$361,$A48,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$373,$A48,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
@@ -45683,15 +47143,15 @@
         </is>
       </c>
       <c r="B49" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$361,$A49)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$373,$A49)</f>
         <v/>
       </c>
       <c r="C49" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$361=$A49)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$373=$A49)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D49" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$361,$A49,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$373,$A49,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
@@ -45702,15 +47162,15 @@
         </is>
       </c>
       <c r="B50" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$361,$A50)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$373,$A50)</f>
         <v/>
       </c>
       <c r="C50" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$361=$A50)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$373=$A50)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D50" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$361,$A50,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$373,$A50,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
@@ -45769,15 +47229,15 @@
         </is>
       </c>
       <c r="B55" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A55)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A55)</f>
         <v/>
       </c>
       <c r="C55" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A55)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A55)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D55" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A55,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A55,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
@@ -45788,15 +47248,15 @@
         </is>
       </c>
       <c r="B56" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A56)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A56)</f>
         <v/>
       </c>
       <c r="C56" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A56)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A56)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D56" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A56,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A56,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
@@ -45807,15 +47267,15 @@
         </is>
       </c>
       <c r="B57" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A57)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A57)</f>
         <v/>
       </c>
       <c r="C57" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A57)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A57)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D57" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A57,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A57,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
@@ -45826,15 +47286,15 @@
         </is>
       </c>
       <c r="B58" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A58)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A58)</f>
         <v/>
       </c>
       <c r="C58" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A58)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A58)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D58" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A58,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A58,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
@@ -45845,15 +47305,15 @@
         </is>
       </c>
       <c r="B59" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A59)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A59)</f>
         <v/>
       </c>
       <c r="C59" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A59)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A59)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D59" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A59,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A59,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
@@ -45864,15 +47324,15 @@
         </is>
       </c>
       <c r="B60" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A60)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A60)</f>
         <v/>
       </c>
       <c r="C60" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A60)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A60)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D60" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A60,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A60,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
@@ -45883,15 +47343,15 @@
         </is>
       </c>
       <c r="B61" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A61)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A61)</f>
         <v/>
       </c>
       <c r="C61" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A61)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A61)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D61" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A61,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A61,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
@@ -45902,15 +47362,15 @@
         </is>
       </c>
       <c r="B62" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A62)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A62)</f>
         <v/>
       </c>
       <c r="C62" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A62)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A62)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D62" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A62,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A62,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
@@ -45921,15 +47381,15 @@
         </is>
       </c>
       <c r="B63" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A63)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A63)</f>
         <v/>
       </c>
       <c r="C63" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A63)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A63)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D63" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A63,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A63,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
@@ -45940,15 +47400,15 @@
         </is>
       </c>
       <c r="B64" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A64)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A64)</f>
         <v/>
       </c>
       <c r="C64" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A64)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A64)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D64" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A64,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A64,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
@@ -45959,15 +47419,15 @@
         </is>
       </c>
       <c r="B65" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A65)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A65)</f>
         <v/>
       </c>
       <c r="C65" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A65)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A65)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D65" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A65,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A65,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
@@ -45978,15 +47438,15 @@
         </is>
       </c>
       <c r="B66" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A66)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A66)</f>
         <v/>
       </c>
       <c r="C66" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A66)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A66)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D66" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A66,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A66,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
@@ -45997,15 +47457,15 @@
         </is>
       </c>
       <c r="B67" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A67)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A67)</f>
         <v/>
       </c>
       <c r="C67" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A67)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A67)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D67" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A67,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A67,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
@@ -46016,15 +47476,15 @@
         </is>
       </c>
       <c r="B68" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A68)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A68)</f>
         <v/>
       </c>
       <c r="C68" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A68)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A68)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D68" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A68,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A68,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
@@ -46035,15 +47495,15 @@
         </is>
       </c>
       <c r="B69" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A69)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A69)</f>
         <v/>
       </c>
       <c r="C69" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A69)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A69)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D69" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A69,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A69,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
@@ -46054,15 +47514,15 @@
         </is>
       </c>
       <c r="B70" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A70)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A70)</f>
         <v/>
       </c>
       <c r="C70" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A70)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A70)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D70" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A70,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A70,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
@@ -46073,15 +47533,15 @@
         </is>
       </c>
       <c r="B71" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A71)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A71)</f>
         <v/>
       </c>
       <c r="C71" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A71)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A71)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D71" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A71,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A71,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
@@ -46092,15 +47552,15 @@
         </is>
       </c>
       <c r="B72" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A72)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A72)</f>
         <v/>
       </c>
       <c r="C72" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A72)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A72)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D72" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A72,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A72,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
@@ -46111,15 +47571,15 @@
         </is>
       </c>
       <c r="B73" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A73)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A73)</f>
         <v/>
       </c>
       <c r="C73" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A73)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A73)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D73" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A73,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A73,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
@@ -46130,15 +47590,15 @@
         </is>
       </c>
       <c r="B74" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A74)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A74)</f>
         <v/>
       </c>
       <c r="C74" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A74)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A74)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D74" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A74,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A74,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
@@ -46149,15 +47609,15 @@
         </is>
       </c>
       <c r="B75" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A75)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A75)</f>
         <v/>
       </c>
       <c r="C75" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A75)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A75)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D75" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A75,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A75,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
@@ -46168,15 +47628,15 @@
         </is>
       </c>
       <c r="B76" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A76)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A76)</f>
         <v/>
       </c>
       <c r="C76" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A76)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A76)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D76" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A76,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A76,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
@@ -46187,334 +47647,353 @@
         </is>
       </c>
       <c r="B77" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A77)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A77)</f>
         <v/>
       </c>
       <c r="C77" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A77)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A77)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D77" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A77,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A77,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="26" t="inlineStr">
         <is>
-          <t>Schlafraum 4</t>
+          <t>Schlafraum 3</t>
         </is>
       </c>
       <c r="B78" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A78)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A78)</f>
         <v/>
       </c>
       <c r="C78" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A78)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A78)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D78" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A78,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A78,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="26" t="inlineStr">
         <is>
-          <t>Schlafraum 5</t>
+          <t>Schlafraum 4</t>
         </is>
       </c>
       <c r="B79" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A79)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A79)</f>
         <v/>
       </c>
       <c r="C79" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A79)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A79)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D79" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A79,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A79,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="26" t="inlineStr">
         <is>
-          <t>Speisesaal</t>
+          <t>Schlafraum 5</t>
         </is>
       </c>
       <c r="B80" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A80)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A80)</f>
         <v/>
       </c>
       <c r="C80" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A80)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A80)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D80" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A80,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A80,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="26" t="inlineStr">
         <is>
-          <t>Terrasse</t>
+          <t>Speisesaal</t>
         </is>
       </c>
       <c r="B81" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A81)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A81)</f>
         <v/>
       </c>
       <c r="C81" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A81)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A81)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D81" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A81,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A81,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="26" t="inlineStr">
         <is>
-          <t>Treppenraum 1</t>
+          <t>Terrasse</t>
         </is>
       </c>
       <c r="B82" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A82)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A82)</f>
         <v/>
       </c>
       <c r="C82" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A82)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A82)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D82" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A82,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A82,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="26" t="inlineStr">
         <is>
-          <t>Turnraum</t>
+          <t>Treppenraum 1</t>
         </is>
       </c>
       <c r="B83" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A83)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A83)</f>
         <v/>
       </c>
       <c r="C83" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A83)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A83)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D83" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A83,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A83,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="26" t="inlineStr">
         <is>
-          <t>WC</t>
+          <t>Turnraum</t>
         </is>
       </c>
       <c r="B84" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A84)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A84)</f>
         <v/>
       </c>
       <c r="C84" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A84)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A84)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D84" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A84,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A84,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="26" t="inlineStr">
         <is>
-          <t>WC Personal</t>
+          <t>WC</t>
         </is>
       </c>
       <c r="B85" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A85)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A85)</f>
         <v/>
       </c>
       <c r="C85" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A85)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A85)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
       <c r="D85" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A85,Artikelstamm!$U$3:$U$361)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A85,Artikelstamm!$U$3:$U$373)</f>
         <v/>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="26" t="inlineStr">
         <is>
+          <t>WC Personal</t>
+        </is>
+      </c>
+      <c r="B86" s="33">
+        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A86)</f>
+        <v/>
+      </c>
+      <c r="C86" s="34">
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A86)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <v/>
+      </c>
+      <c r="D86" s="34">
+        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A86,Artikelstamm!$U$3:$U$373)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="26" t="inlineStr">
+        <is>
           <t>Werkraum</t>
         </is>
       </c>
-      <c r="B86" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$361,$A86)</f>
-        <v/>
-      </c>
-      <c r="C86" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$361=$A86)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
-        <v/>
-      </c>
-      <c r="D86" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$361,$A86,Artikelstamm!$U$3:$U$361)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="28" t="inlineStr">
+      <c r="B87" s="33">
+        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A87)</f>
+        <v/>
+      </c>
+      <c r="C87" s="34">
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A87)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <v/>
+      </c>
+      <c r="D87" s="34">
+        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A87,Artikelstamm!$U$3:$U$373)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="28" t="inlineStr">
         <is>
           <t>Summe</t>
         </is>
       </c>
-      <c r="B87" s="35">
-        <f>SUM(B55:B86)</f>
-        <v/>
-      </c>
-      <c r="C87" s="36">
-        <f>SUM(C55:C86)</f>
-        <v/>
-      </c>
-      <c r="D87" s="36">
-        <f>SUM(D55:D86)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" s="25" t="inlineStr">
+      <c r="B88" s="35">
+        <f>SUM(B55:B87)</f>
+        <v/>
+      </c>
+      <c r="C88" s="36">
+        <f>SUM(C55:C87)</f>
+        <v/>
+      </c>
+      <c r="D88" s="36">
+        <f>SUM(D55:D87)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="25" t="inlineStr">
         <is>
           <t>Nach Verkaufskanal</t>
         </is>
       </c>
     </row>
-    <row r="90">
-      <c r="A90" s="32" t="inlineStr">
+    <row r="91">
+      <c r="A91" s="32" t="inlineStr">
         <is>
           <t>Verkaufskanal</t>
         </is>
       </c>
-      <c r="B90" s="32" t="inlineStr">
+      <c r="B91" s="32" t="inlineStr">
         <is>
           <t>Positionen</t>
         </is>
       </c>
-      <c r="C90" s="32" t="inlineStr">
+      <c r="C91" s="32" t="inlineStr">
         <is>
           <t>Umsatz netto</t>
         </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" s="26" t="inlineStr">
-        <is>
-          <t>Klinik</t>
-        </is>
-      </c>
-      <c r="B91" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$361,$A91)</f>
-        <v/>
-      </c>
-      <c r="C91" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$361=$A91)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
-        <v/>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="26" t="inlineStr">
         <is>
-          <t>Kleinanzeigen</t>
+          <t>Klinik</t>
         </is>
       </c>
       <c r="B92" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$361,$A92)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$373,$A92)</f>
         <v/>
       </c>
       <c r="C92" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$361=$A92)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$373=$A92)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="26" t="inlineStr">
         <is>
-          <t>eBay</t>
+          <t>Kleinanzeigen</t>
         </is>
       </c>
       <c r="B93" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$361,$A93)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$373,$A93)</f>
         <v/>
       </c>
       <c r="C93" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$361=$A93)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$373=$A93)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="26" t="inlineStr">
         <is>
-          <t>Direkt</t>
+          <t>eBay</t>
         </is>
       </c>
       <c r="B94" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$361,$A94)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$373,$A94)</f>
         <v/>
       </c>
       <c r="C94" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$361=$A94)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$373=$A94)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="26" t="inlineStr">
         <is>
-          <t>Händler</t>
+          <t>Direkt</t>
         </is>
       </c>
       <c r="B95" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$361,$A95)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$373,$A95)</f>
         <v/>
       </c>
       <c r="C95" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$361=$A95)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$373=$A95)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
         <v/>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="26" t="inlineStr">
         <is>
+          <t>Händler</t>
+        </is>
+      </c>
+      <c r="B96" s="33">
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$373,$A96)</f>
+        <v/>
+      </c>
+      <c r="C96" s="34">
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$373=$A96)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="26" t="inlineStr">
+        <is>
           <t>Verkaufstag</t>
         </is>
       </c>
-      <c r="B96" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$361,$A96)</f>
-        <v/>
-      </c>
-      <c r="C96" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$361=$A96)*Artikelstamm!$K$3:$K$361*Artikelstamm!$AE$3:$AE$361)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" s="28" t="inlineStr">
+      <c r="B97" s="33">
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$373,$A97)</f>
+        <v/>
+      </c>
+      <c r="C97" s="34">
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$373=$A97)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="28" t="inlineStr">
         <is>
           <t>Summe</t>
         </is>
       </c>
-      <c r="B97" s="35">
-        <f>SUM(B91:B96)</f>
-        <v/>
-      </c>
-      <c r="C97" s="36">
-        <f>SUM(C91:C96)</f>
+      <c r="B98" s="35">
+        <f>SUM(B92:B97)</f>
+        <v/>
+      </c>
+      <c r="C98" s="36">
+        <f>SUM(C92:C97)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
NE05 Speisesaal erfasst: 12 neue Positionen, 2 Zusammenfassungen
Raum NE05 (Neubau EG, Speisesaal, 61,07 m2) aus 17 Fotos und dem
Erfassungsblatt aufgenommen.

  NE05-10 -> NU02-02  IKEA Kritter Kinderstuhl  31 -> 40
  NE05-11 -> NU04-13  Kindertisch rund weiss     1 -> 5

Vor Ort nachgezaehlt und korrigiert:
  NE05-01 Massivholztisch mit Baumkante  4 -> 8 Stueck
  NE05-02 Sitzbank Massivholz            2 -> 9 Stueck

Zwei Markenfragen betreffen jetzt je vier Positionen; beide bleiben mit
Im_Katalog = nein stehen, bis ein Foto vorliegt:
  Panton-Form: NU04-20, NE05-04, NE05-05, NE05-12  (12 Stuehle)
  Treppenhochstuhl: NU05-01, NE05-06, NE05-07, NE05-08  (21 Stuehle)

Datenbasis 382 Positionen / 326 aktiv, pruefen.py 0 Fehler.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011yyfqhuiWGsaNy38oaNoGo
</commit_message>
<xml_diff>
--- a/ausgabe/01_Artikelstamm_kikripp.xlsx
+++ b/ausgabe/01_Artikelstamm_kikripp.xlsx
@@ -15,7 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Artikelstamm'!$A$2:$AN$373</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Artikelstamm'!$A$2:$AN$384</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1019,7 +1019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN373"/>
+  <dimension ref="A1:AN384"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -14635,7 +14635,7 @@
         </is>
       </c>
       <c r="J112" s="17" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="K112" s="17" t="n"/>
       <c r="L112" s="18">
@@ -14710,7 +14710,7 @@
       <c r="AL112" s="19" t="n"/>
       <c r="AM112" s="16" t="inlineStr">
         <is>
-          <t>mindestens 4 Tische im Bild - bitte nachzählen</t>
+          <t>8 Tische, im Raum nachgezählt.</t>
         </is>
       </c>
       <c r="AN112" s="22" t="n"/>
@@ -14758,7 +14758,7 @@
         </is>
       </c>
       <c r="J113" s="17" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="K113" s="17" t="n"/>
       <c r="L113" s="18">
@@ -14833,7 +14833,7 @@
       <c r="AL113" s="19" t="n"/>
       <c r="AM113" s="16" t="inlineStr">
         <is>
-          <t>2 Bänke im Bild erkennbar</t>
+          <t>9 Bänke, im Raum nachgezählt.</t>
         </is>
       </c>
       <c r="AN113" s="22" t="n"/>
@@ -20094,7 +20094,7 @@
       <c r="B156" s="15" t="n"/>
       <c r="C156" s="15" t="inlineStr">
         <is>
-          <t>NU04-12, BU02-04</t>
+          <t>NU04-12, BU02-04, NE05-10</t>
         </is>
       </c>
       <c r="D156" s="15" t="inlineStr">
@@ -20128,7 +20128,7 @@
         </is>
       </c>
       <c r="J156" s="17" t="n">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="K156" s="17" t="n"/>
       <c r="L156" s="18">
@@ -20207,12 +20207,12 @@
       <c r="AL156" s="19" t="n"/>
       <c r="AM156" s="16" t="inlineStr">
         <is>
-          <t>31 Stühle insgesamt: 10 im Gruppenraum 5 und im Nachbarraum NU03, 6 im Schlafraum 5 (dort mit NU04-12 beschriftet) und 15 im Flur 2 im Untergeschoss des Bestandsgebäudes (dort mit BU02-04 beschriftet). Die 15 Stühle aus dem Flur 2 sind stark gebraucht.</t>
+          <t>40 Stühle insgesamt: 10 im Gruppenraum 5 und im Nachbarraum NU03, 6 im Schlafraum 5 (NU04-12), 15 im Flur 2 im Untergeschoss (BU02-04) und 9 im Speisesaal (NE05-10). Die 15 Stühle aus dem Flur 2 sind stark gebraucht. Ein Stuhl aus dem Speisesaal ist auf Foto F-477 zu sehen.</t>
         </is>
       </c>
       <c r="AN156" s="22" t="inlineStr">
         <is>
-          <t>Zusammengefasste Position ueber vier Raeume. Post-it-Nummern: NU04-12, BU02-04. In NU03 nicht erneut anlegen.</t>
+          <t>Zusammengefasste Position ueber fuenf Raeume. Post-it-Nummern: NU04-12, BU02-04, NE05-10. In NU03 nicht erneut anlegen.</t>
         </is>
       </c>
     </row>
@@ -24373,7 +24373,11 @@
         </is>
       </c>
       <c r="B191" s="15" t="n"/>
-      <c r="C191" s="15" t="n"/>
+      <c r="C191" s="15" t="inlineStr">
+        <is>
+          <t>NE05-11</t>
+        </is>
+      </c>
       <c r="D191" s="15" t="inlineStr">
         <is>
           <t>NU04</t>
@@ -24386,7 +24390,7 @@
       </c>
       <c r="F191" s="16" t="inlineStr">
         <is>
-          <t>Runder Kindertisch, weiße Platte auf konischen Beinen aus massivem Holz. Die Plattenkante ist an einer Stelle beschädigt und dunkel abgestoßen.</t>
+          <t>Runder Kindertisch, weiße Platte auf konischen Beinen aus massivem Holz.</t>
         </is>
       </c>
       <c r="G191" s="15" t="inlineStr">
@@ -24405,7 +24409,7 @@
         </is>
       </c>
       <c r="J191" s="17" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K191" s="17" t="n"/>
       <c r="L191" s="18">
@@ -24419,7 +24423,7 @@
       </c>
       <c r="N191" s="15" t="inlineStr">
         <is>
-          <t>stark gebraucht</t>
+          <t>gebraucht</t>
         </is>
       </c>
       <c r="O191" s="19" t="n"/>
@@ -24480,10 +24484,14 @@
       <c r="AL191" s="19" t="n"/>
       <c r="AM191" s="16" t="inlineStr">
         <is>
-          <t>1 Tisch.</t>
-        </is>
-      </c>
-      <c r="AN191" s="22" t="n"/>
+          <t>5 Tische: 1 im Schlafraum 5 (NU04-13) und 4 im Speisesaal (NE05-11). Bei dem Tisch im Schlafraum 5 ist die Plattenkante an einer Stelle beschädigt und dunkel abgestoßen; ein Tisch aus dem Speisesaal ist auf Foto F-478 zu sehen.</t>
+        </is>
+      </c>
+      <c r="AN191" s="22" t="inlineStr">
+        <is>
+          <t>Zusammengefasste Position über zwei Räume – Post-it-Nummer: NE05-11.</t>
+        </is>
+      </c>
     </row>
     <row r="192" ht="30" customHeight="1">
       <c r="A192" s="15" t="inlineStr">
@@ -25345,12 +25353,12 @@
       <c r="AL198" s="19" t="n"/>
       <c r="AM198" s="16" t="inlineStr">
         <is>
-          <t>1 Stuhl.</t>
+          <t>1 Stuhl. Weitere Freischwinger gleicher Form stehen unter NE05-04 (rot, Erwachsenengröße), NE05-05 (rot, Kindergröße) und NE05-12 (weiß, Kindergröße).</t>
         </is>
       </c>
       <c r="AN198" s="22" t="inlineStr">
         <is>
-          <t>OFFEN: NICHT VEROEFFENTLICHEN, bis die Marke geklaert ist. Die Form ist der Panton Chair von Verner Panton, Original von Vitra - gebraucht 120-250 EUR, ein Nachbau 30-50 EUR. Das Original traegt auf der Unterseite eine eingeformte Vitra-Kennzeichnung. Nahaufnahme der Unterseite anfordern, dann entscheiden.</t>
+          <t>OFFEN: NICHT VEROEFFENTLICHEN, bis die Marke geklaert ist. Die Form ist der Panton Chair von Verner Panton, Original von Vitra. Gebraucht 120-250 EUR je Erwachsenenstuhl und 90-150 EUR je Kinderstuhl, ein Nachbau 30-50 bzw. 20-30 EUR. Das Original traegt auf der Unterseite eine eingeformte Vitra-Kennzeichnung. Betrifft NU04-20, NE05-04, NE05-05 und NE05-12 - eine Nahaufnahme der Unterseite genuegt fuer alle vier.</t>
         </is>
       </c>
     </row>
@@ -25706,12 +25714,12 @@
       <c r="AL201" s="19" t="n"/>
       <c r="AM201" s="16" t="inlineStr">
         <is>
-          <t>6 Stühle – abgebildet ist einer davon.</t>
+          <t>6 Stühle – abgebildet ist einer davon. Dieselbe Bauform in anderen Farben steht unter NE05-06, NE05-07 und NE05-08.</t>
         </is>
       </c>
       <c r="AN201" s="22" t="inlineStr">
         <is>
-          <t>OFFEN: NICHT VEROEFFENTLICHEN, bis die Marke geklaert ist. Auf dem Erfassungsblatt steht "Tripptrapp". Der Stokke Tripp Trapp hat in den Seitenwangen durchgehende Nuten, dieser Stuhl hat Lochreihen - das spricht gegen ein Original. Ein Stokke bringt gebraucht 100-150 EUR, ein Nachbau 25-40 EUR; bei 6 Stueck sind das 150 bis 900 EUR. Marke steht meist auf der Seitenwange oder unter dem Sitz - Nahaufnahme anfordern.</t>
+          <t>OFFEN: NICHT VEROEFFENTLICHEN, bis die Marke geklaert ist. Treppenhochstuhl mit Lochreihen in den Seitenwangen und umlaufendem Buegel - das ist nicht die Bauform des Stokke Tripp Trapp (durchgehende Nuten, kein Buegel). Original Tripp Trapp gebraucht 150-250 EUR, vergleichbare Treppenhochstuehle 50-90 EUR. Betrifft NU05-01, NE05-06, NE05-07 und NE05-08 - ein Foto eines Aufklebers oder einer Praegung genuegt fuer alle vier.</t>
         </is>
       </c>
     </row>
@@ -45544,7 +45552,7 @@
       </c>
       <c r="N366" s="15" t="inlineStr">
         <is>
-          <t>gebraucht</t>
+          <t>gut</t>
         </is>
       </c>
       <c r="O366" s="19" t="n"/>
@@ -45663,7 +45671,7 @@
       </c>
       <c r="N367" s="15" t="inlineStr">
         <is>
-          <t>gebraucht</t>
+          <t>gut</t>
         </is>
       </c>
       <c r="O367" s="19" t="n"/>
@@ -45782,7 +45790,7 @@
       </c>
       <c r="N368" s="15" t="inlineStr">
         <is>
-          <t>gebraucht</t>
+          <t>gut</t>
         </is>
       </c>
       <c r="O368" s="19" t="n"/>
@@ -46147,7 +46155,7 @@
       </c>
       <c r="N371" s="15" t="inlineStr">
         <is>
-          <t>gebraucht</t>
+          <t>gut</t>
         </is>
       </c>
       <c r="O371" s="19" t="n"/>
@@ -46451,8 +46459,1341 @@
       </c>
       <c r="AN373" s="22" t="n"/>
     </row>
+    <row r="374" ht="30" customHeight="1">
+      <c r="A374" s="15" t="inlineStr">
+        <is>
+          <t>NE05-04</t>
+        </is>
+      </c>
+      <c r="B374" s="15" t="n"/>
+      <c r="C374" s="15" t="n"/>
+      <c r="D374" s="15" t="inlineStr">
+        <is>
+          <t>NE05</t>
+        </is>
+      </c>
+      <c r="E374" s="15" t="inlineStr">
+        <is>
+          <t>Freischwinger rot, Erwachsenengröße</t>
+        </is>
+      </c>
+      <c r="F374" s="16" t="inlineStr">
+        <is>
+          <t>Freischwinger aus einem Stück Kunststoff, rot matt, S-förmig geschwungen. Erwachsenengröße.</t>
+        </is>
+      </c>
+      <c r="G374" s="15" t="inlineStr">
+        <is>
+          <t>Möbel</t>
+        </is>
+      </c>
+      <c r="H374" s="15" t="inlineStr">
+        <is>
+          <t>Speisesaal</t>
+        </is>
+      </c>
+      <c r="I374" s="15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J374" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K374" s="17" t="n"/>
+      <c r="L374" s="18">
+        <f>J374-IF(K374="",0,K374)</f>
+        <v/>
+      </c>
+      <c r="M374" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N374" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O374" s="19" t="n"/>
+      <c r="P374" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q374" s="19" t="n"/>
+      <c r="R374" s="20" t="n"/>
+      <c r="S374" s="20" t="n">
+        <v>180</v>
+      </c>
+      <c r="T374" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U374" s="21">
+        <f>L374*S374</f>
+        <v/>
+      </c>
+      <c r="V374" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W374" s="15" t="inlineStr">
+        <is>
+          <t>F-469</t>
+        </is>
+      </c>
+      <c r="X374" s="19" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="Y374" s="19" t="n"/>
+      <c r="Z374" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA374" s="19" t="n"/>
+      <c r="AB374" s="19" t="n"/>
+      <c r="AC374" s="19" t="n"/>
+      <c r="AD374" s="19" t="n"/>
+      <c r="AE374" s="20" t="n"/>
+      <c r="AF374" s="21">
+        <f>IF(K374="","",K374*AE374)</f>
+        <v/>
+      </c>
+      <c r="AG374" s="19" t="n"/>
+      <c r="AH374" s="19" t="n"/>
+      <c r="AI374" s="19" t="n"/>
+      <c r="AJ374" s="19" t="n"/>
+      <c r="AK374" s="19" t="n"/>
+      <c r="AL374" s="19" t="n"/>
+      <c r="AM374" s="16" t="inlineStr">
+        <is>
+          <t>1 Stuhl. Die Seitenansicht ist auf Foto F-470 zu sehen. Weitere Freischwinger gleicher Form stehen unter NU04-20, NE05-05 und NE05-12.</t>
+        </is>
+      </c>
+      <c r="AN374" s="22" t="inlineStr">
+        <is>
+          <t>OFFEN: NICHT VEROEFFENTLICHEN, bis die Marke geklaert ist. Die Form ist der Panton Chair von Verner Panton, Original von Vitra. Gebraucht 120-250 EUR je Erwachsenenstuhl und 90-150 EUR je Kinderstuhl, ein Nachbau 30-50 bzw. 20-30 EUR. Das Original traegt auf der Unterseite eine eingeformte Vitra-Kennzeichnung. Betrifft NU04-20, NE05-04, NE05-05 und NE05-12 - eine Nahaufnahme der Unterseite genuegt fuer alle vier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="375" ht="30" customHeight="1">
+      <c r="A375" s="15" t="inlineStr">
+        <is>
+          <t>NE05-05</t>
+        </is>
+      </c>
+      <c r="B375" s="15" t="n"/>
+      <c r="C375" s="15" t="n"/>
+      <c r="D375" s="15" t="inlineStr">
+        <is>
+          <t>NE05</t>
+        </is>
+      </c>
+      <c r="E375" s="15" t="inlineStr">
+        <is>
+          <t>Freischwinger rot, Kindergröße</t>
+        </is>
+      </c>
+      <c r="F375" s="16" t="inlineStr">
+        <is>
+          <t>Freischwinger aus einem Stück Kunststoff, rot matt, S-förmig geschwungen. Kindergröße.</t>
+        </is>
+      </c>
+      <c r="G375" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H375" s="15" t="inlineStr">
+        <is>
+          <t>Speisesaal</t>
+        </is>
+      </c>
+      <c r="I375" s="15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J375" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="K375" s="17" t="n"/>
+      <c r="L375" s="18">
+        <f>J375-IF(K375="",0,K375)</f>
+        <v/>
+      </c>
+      <c r="M375" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N375" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O375" s="19" t="n"/>
+      <c r="P375" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q375" s="19" t="n"/>
+      <c r="R375" s="20" t="n"/>
+      <c r="S375" s="20" t="n">
+        <v>120</v>
+      </c>
+      <c r="T375" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U375" s="21">
+        <f>L375*S375</f>
+        <v/>
+      </c>
+      <c r="V375" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W375" s="15" t="inlineStr">
+        <is>
+          <t>F-471</t>
+        </is>
+      </c>
+      <c r="X375" s="19" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="Y375" s="19" t="n"/>
+      <c r="Z375" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA375" s="19" t="n"/>
+      <c r="AB375" s="19" t="n"/>
+      <c r="AC375" s="19" t="n"/>
+      <c r="AD375" s="19" t="n"/>
+      <c r="AE375" s="20" t="n"/>
+      <c r="AF375" s="21">
+        <f>IF(K375="","",K375*AE375)</f>
+        <v/>
+      </c>
+      <c r="AG375" s="19" t="n"/>
+      <c r="AH375" s="19" t="n"/>
+      <c r="AI375" s="19" t="n"/>
+      <c r="AJ375" s="19" t="n"/>
+      <c r="AK375" s="19" t="n"/>
+      <c r="AL375" s="19" t="n"/>
+      <c r="AM375" s="16" t="inlineStr">
+        <is>
+          <t>5 Stühle – abgebildet ist einer davon. Weitere Freischwinger gleicher Form stehen unter NU04-20, NE05-04 und NE05-12.</t>
+        </is>
+      </c>
+      <c r="AN375" s="22" t="inlineStr">
+        <is>
+          <t>OFFEN: NICHT VEROEFFENTLICHEN, bis die Marke geklaert ist. Die Form ist der Panton Chair von Verner Panton, Original von Vitra. Gebraucht 120-250 EUR je Erwachsenenstuhl und 90-150 EUR je Kinderstuhl, ein Nachbau 30-50 bzw. 20-30 EUR. Das Original traegt auf der Unterseite eine eingeformte Vitra-Kennzeichnung. Betrifft NU04-20, NE05-04, NE05-05 und NE05-12 - eine Nahaufnahme der Unterseite genuegt fuer alle vier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="376" ht="30" customHeight="1">
+      <c r="A376" s="15" t="inlineStr">
+        <is>
+          <t>NE05-06</t>
+        </is>
+      </c>
+      <c r="B376" s="15" t="n"/>
+      <c r="C376" s="15" t="n"/>
+      <c r="D376" s="15" t="inlineStr">
+        <is>
+          <t>NE05</t>
+        </is>
+      </c>
+      <c r="E376" s="15" t="inlineStr">
+        <is>
+          <t>Treppenhochstuhl schwarz</t>
+        </is>
+      </c>
+      <c r="F376" s="16" t="inlineStr">
+        <is>
+          <t>Mitwachsender Treppenhochstuhl: Seitenwangen und Platten schwarz lackiert, Sitz- und Fußbrett in der Höhe verstellbar, umlaufender Bügel mit Rückenlehne. Die Seitenwangen tragen Lochreihen für die Verstellung.</t>
+        </is>
+      </c>
+      <c r="G376" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H376" s="15" t="inlineStr">
+        <is>
+          <t>Speisesaal</t>
+        </is>
+      </c>
+      <c r="I376" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J376" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="K376" s="17" t="n"/>
+      <c r="L376" s="18">
+        <f>J376-IF(K376="",0,K376)</f>
+        <v/>
+      </c>
+      <c r="M376" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N376" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O376" s="19" t="n"/>
+      <c r="P376" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q376" s="19" t="n"/>
+      <c r="R376" s="20" t="n"/>
+      <c r="S376" s="20" t="n">
+        <v>90</v>
+      </c>
+      <c r="T376" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U376" s="21">
+        <f>L376*S376</f>
+        <v/>
+      </c>
+      <c r="V376" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W376" s="15" t="inlineStr">
+        <is>
+          <t>F-472</t>
+        </is>
+      </c>
+      <c r="X376" s="19" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="Y376" s="19" t="n"/>
+      <c r="Z376" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA376" s="19" t="n"/>
+      <c r="AB376" s="19" t="n"/>
+      <c r="AC376" s="19" t="n"/>
+      <c r="AD376" s="19" t="n"/>
+      <c r="AE376" s="20" t="n"/>
+      <c r="AF376" s="21">
+        <f>IF(K376="","",K376*AE376)</f>
+        <v/>
+      </c>
+      <c r="AG376" s="19" t="n"/>
+      <c r="AH376" s="19" t="n"/>
+      <c r="AI376" s="19" t="n"/>
+      <c r="AJ376" s="19" t="n"/>
+      <c r="AK376" s="19" t="n"/>
+      <c r="AL376" s="19" t="n"/>
+      <c r="AM376" s="16" t="inlineStr">
+        <is>
+          <t>7 Stühle – abgebildet ist einer davon. Dieselbe Bauform in anderen Farben steht unter NU05-01, NE05-07 und NE05-08.</t>
+        </is>
+      </c>
+      <c r="AN376" s="22" t="inlineStr">
+        <is>
+          <t>OFFEN: NICHT VEROEFFENTLICHEN, bis die Marke geklaert ist. Treppenhochstuhl mit Lochreihen in den Seitenwangen und umlaufendem Buegel - das ist nicht die Bauform des Stokke Tripp Trapp (durchgehende Nuten, kein Buegel). Original Tripp Trapp gebraucht 150-250 EUR, vergleichbare Treppenhochstuehle 50-90 EUR. Betrifft NU05-01, NE05-06, NE05-07 und NE05-08 - ein Foto eines Aufklebers oder einer Praegung genuegt fuer alle vier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="377" ht="30" customHeight="1">
+      <c r="A377" s="15" t="inlineStr">
+        <is>
+          <t>NE05-07</t>
+        </is>
+      </c>
+      <c r="B377" s="15" t="n"/>
+      <c r="C377" s="15" t="n"/>
+      <c r="D377" s="15" t="inlineStr">
+        <is>
+          <t>NE05</t>
+        </is>
+      </c>
+      <c r="E377" s="15" t="inlineStr">
+        <is>
+          <t>Treppenhochstuhl schwarz-weiß</t>
+        </is>
+      </c>
+      <c r="F377" s="16" t="inlineStr">
+        <is>
+          <t>Mitwachsender Treppenhochstuhl: Seitenwangen schwarz lackiert, Sitz- und Fußbrett sowie Bügel mit Rückenlehne in Weiß, in der Höhe verstellbar. Die Seitenwangen tragen Lochreihen für die Verstellung.</t>
+        </is>
+      </c>
+      <c r="G377" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H377" s="15" t="inlineStr">
+        <is>
+          <t>Speisesaal</t>
+        </is>
+      </c>
+      <c r="I377" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J377" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="K377" s="17" t="n"/>
+      <c r="L377" s="18">
+        <f>J377-IF(K377="",0,K377)</f>
+        <v/>
+      </c>
+      <c r="M377" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N377" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O377" s="19" t="n"/>
+      <c r="P377" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q377" s="19" t="n"/>
+      <c r="R377" s="20" t="n"/>
+      <c r="S377" s="20" t="n">
+        <v>90</v>
+      </c>
+      <c r="T377" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U377" s="21">
+        <f>L377*S377</f>
+        <v/>
+      </c>
+      <c r="V377" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W377" s="15" t="inlineStr">
+        <is>
+          <t>F-473</t>
+        </is>
+      </c>
+      <c r="X377" s="19" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="Y377" s="19" t="n"/>
+      <c r="Z377" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA377" s="19" t="n"/>
+      <c r="AB377" s="19" t="n"/>
+      <c r="AC377" s="19" t="n"/>
+      <c r="AD377" s="19" t="n"/>
+      <c r="AE377" s="20" t="n"/>
+      <c r="AF377" s="21">
+        <f>IF(K377="","",K377*AE377)</f>
+        <v/>
+      </c>
+      <c r="AG377" s="19" t="n"/>
+      <c r="AH377" s="19" t="n"/>
+      <c r="AI377" s="19" t="n"/>
+      <c r="AJ377" s="19" t="n"/>
+      <c r="AK377" s="19" t="n"/>
+      <c r="AL377" s="19" t="n"/>
+      <c r="AM377" s="16" t="inlineStr">
+        <is>
+          <t>4 Stühle – abgebildet ist einer davon. Dieselbe Bauform in anderen Farben steht unter NU05-01, NE05-06 und NE05-08.</t>
+        </is>
+      </c>
+      <c r="AN377" s="22" t="inlineStr">
+        <is>
+          <t>OFFEN: NICHT VEROEFFENTLICHEN, bis die Marke geklaert ist. Treppenhochstuhl mit Lochreihen in den Seitenwangen und umlaufendem Buegel - das ist nicht die Bauform des Stokke Tripp Trapp (durchgehende Nuten, kein Buegel). Original Tripp Trapp gebraucht 150-250 EUR, vergleichbare Treppenhochstuehle 50-90 EUR. Betrifft NU05-01, NE05-06, NE05-07 und NE05-08 - ein Foto eines Aufklebers oder einer Praegung genuegt fuer alle vier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="378" ht="30" customHeight="1">
+      <c r="A378" s="15" t="inlineStr">
+        <is>
+          <t>NE05-08</t>
+        </is>
+      </c>
+      <c r="B378" s="15" t="n"/>
+      <c r="C378" s="15" t="n"/>
+      <c r="D378" s="15" t="inlineStr">
+        <is>
+          <t>NE05</t>
+        </is>
+      </c>
+      <c r="E378" s="15" t="inlineStr">
+        <is>
+          <t>Treppenhochstuhl grau mit Buchengestell</t>
+        </is>
+      </c>
+      <c r="F378" s="16" t="inlineStr">
+        <is>
+          <t>Mitwachsender Treppenhochstuhl: Seitenwangen aus Buche natur, Sitz- und Fußbrett sowie Bügel mit Rückenlehne in Grau, in der Höhe verstellbar. Die Seitenwangen tragen Lochreihen für die Verstellung.</t>
+        </is>
+      </c>
+      <c r="G378" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H378" s="15" t="inlineStr">
+        <is>
+          <t>Speisesaal</t>
+        </is>
+      </c>
+      <c r="I378" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J378" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="K378" s="17" t="n"/>
+      <c r="L378" s="18">
+        <f>J378-IF(K378="",0,K378)</f>
+        <v/>
+      </c>
+      <c r="M378" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N378" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O378" s="19" t="n"/>
+      <c r="P378" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q378" s="19" t="n"/>
+      <c r="R378" s="20" t="n"/>
+      <c r="S378" s="20" t="n">
+        <v>90</v>
+      </c>
+      <c r="T378" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U378" s="21">
+        <f>L378*S378</f>
+        <v/>
+      </c>
+      <c r="V378" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W378" s="15" t="inlineStr">
+        <is>
+          <t>F-474</t>
+        </is>
+      </c>
+      <c r="X378" s="19" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="Y378" s="19" t="n"/>
+      <c r="Z378" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA378" s="19" t="n"/>
+      <c r="AB378" s="19" t="n"/>
+      <c r="AC378" s="19" t="n"/>
+      <c r="AD378" s="19" t="n"/>
+      <c r="AE378" s="20" t="n"/>
+      <c r="AF378" s="21">
+        <f>IF(K378="","",K378*AE378)</f>
+        <v/>
+      </c>
+      <c r="AG378" s="19" t="n"/>
+      <c r="AH378" s="19" t="n"/>
+      <c r="AI378" s="19" t="n"/>
+      <c r="AJ378" s="19" t="n"/>
+      <c r="AK378" s="19" t="n"/>
+      <c r="AL378" s="19" t="n"/>
+      <c r="AM378" s="16" t="inlineStr">
+        <is>
+          <t>4 Stühle – abgebildet ist einer davon. Dieselbe Bauform in anderen Farben steht unter NU05-01, NE05-06 und NE05-07.</t>
+        </is>
+      </c>
+      <c r="AN378" s="22" t="inlineStr">
+        <is>
+          <t>OFFEN: NICHT VEROEFFENTLICHEN, bis die Marke geklaert ist. Treppenhochstuhl mit Lochreihen in den Seitenwangen und umlaufendem Buegel - das ist nicht die Bauform des Stokke Tripp Trapp (durchgehende Nuten, kein Buegel). Original Tripp Trapp gebraucht 150-250 EUR, vergleichbare Treppenhochstuehle 50-90 EUR. Betrifft NU05-01, NE05-06, NE05-07 und NE05-08 - ein Foto eines Aufklebers oder einer Praegung genuegt fuer alle vier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="379" ht="30" customHeight="1">
+      <c r="A379" s="15" t="inlineStr">
+        <is>
+          <t>NE05-09</t>
+        </is>
+      </c>
+      <c r="B379" s="15" t="n"/>
+      <c r="C379" s="15" t="n"/>
+      <c r="D379" s="15" t="inlineStr">
+        <is>
+          <t>NE05</t>
+        </is>
+      </c>
+      <c r="E379" s="15" t="inlineStr">
+        <is>
+          <t>IKEA Ingolf Kinderhochstuhl weiß</t>
+        </is>
+      </c>
+      <c r="F379" s="16" t="inlineStr">
+        <is>
+          <t>Hoher Kinderstuhl von IKEA aus Massivholz, weiß lackiert, mit Kreuzstrebe in der Lehne und Fußstütze. Etikett an der Unterseite: Ingolf, 20948, IKEA of Sweden. Die Sitzfläche ist stark verkratzt und die Farbe an den Kanten abgeplatzt.</t>
+        </is>
+      </c>
+      <c r="G379" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H379" s="15" t="inlineStr">
+        <is>
+          <t>Speisesaal</t>
+        </is>
+      </c>
+      <c r="I379" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J379" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K379" s="17" t="n"/>
+      <c r="L379" s="18">
+        <f>J379-IF(K379="",0,K379)</f>
+        <v/>
+      </c>
+      <c r="M379" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N379" s="15" t="inlineStr">
+        <is>
+          <t>stark gebraucht</t>
+        </is>
+      </c>
+      <c r="O379" s="19" t="n"/>
+      <c r="P379" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q379" s="19" t="n"/>
+      <c r="R379" s="20" t="n"/>
+      <c r="S379" s="20" t="n">
+        <v>35</v>
+      </c>
+      <c r="T379" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U379" s="21">
+        <f>L379*S379</f>
+        <v/>
+      </c>
+      <c r="V379" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W379" s="15" t="inlineStr">
+        <is>
+          <t>F-475</t>
+        </is>
+      </c>
+      <c r="X379" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y379" s="19" t="n"/>
+      <c r="Z379" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA379" s="19" t="inlineStr">
+        <is>
+          <t>IKEA</t>
+        </is>
+      </c>
+      <c r="AB379" s="19" t="n"/>
+      <c r="AC379" s="19" t="n"/>
+      <c r="AD379" s="19" t="n"/>
+      <c r="AE379" s="20" t="n"/>
+      <c r="AF379" s="21">
+        <f>IF(K379="","",K379*AE379)</f>
+        <v/>
+      </c>
+      <c r="AG379" s="19" t="n"/>
+      <c r="AH379" s="19" t="n"/>
+      <c r="AI379" s="19" t="n"/>
+      <c r="AJ379" s="19" t="n"/>
+      <c r="AK379" s="19" t="n"/>
+      <c r="AL379" s="19" t="n"/>
+      <c r="AM379" s="16" t="inlineStr">
+        <is>
+          <t>2 Stühle – abgebildet ist einer davon. Das Etikett ist auf Foto F-476 zu sehen.</t>
+        </is>
+      </c>
+      <c r="AN379" s="22" t="n"/>
+    </row>
+    <row r="380" ht="30" customHeight="1">
+      <c r="A380" s="15" t="inlineStr">
+        <is>
+          <t>NE05-13</t>
+        </is>
+      </c>
+      <c r="B380" s="15" t="n"/>
+      <c r="C380" s="15" t="n"/>
+      <c r="D380" s="15" t="inlineStr">
+        <is>
+          <t>NE05</t>
+        </is>
+      </c>
+      <c r="E380" s="15" t="inlineStr">
+        <is>
+          <t>Rollwagen schwarz mit Holzplatte</t>
+        </is>
+      </c>
+      <c r="F380" s="16" t="inlineStr">
+        <is>
+          <t>Rollwagen mit schwarzem Metallgestell, oberer Platte aus Multiplex und zwei schwarzen Ablageböden, auf vier Lenkrollen.</t>
+        </is>
+      </c>
+      <c r="G380" s="15" t="inlineStr">
+        <is>
+          <t>Möbel</t>
+        </is>
+      </c>
+      <c r="H380" s="15" t="inlineStr">
+        <is>
+          <t>Speisesaal</t>
+        </is>
+      </c>
+      <c r="I380" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J380" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="K380" s="17" t="n"/>
+      <c r="L380" s="18">
+        <f>J380-IF(K380="",0,K380)</f>
+        <v/>
+      </c>
+      <c r="M380" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N380" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O380" s="19" t="n"/>
+      <c r="P380" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q380" s="19" t="n"/>
+      <c r="R380" s="20" t="n"/>
+      <c r="S380" s="20" t="n">
+        <v>70</v>
+      </c>
+      <c r="T380" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U380" s="21">
+        <f>L380*S380</f>
+        <v/>
+      </c>
+      <c r="V380" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W380" s="15" t="inlineStr">
+        <is>
+          <t>F-481</t>
+        </is>
+      </c>
+      <c r="X380" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y380" s="19" t="n"/>
+      <c r="Z380" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA380" s="19" t="n"/>
+      <c r="AB380" s="19" t="n"/>
+      <c r="AC380" s="19" t="n"/>
+      <c r="AD380" s="19" t="n"/>
+      <c r="AE380" s="20" t="n"/>
+      <c r="AF380" s="21">
+        <f>IF(K380="","",K380*AE380)</f>
+        <v/>
+      </c>
+      <c r="AG380" s="19" t="n"/>
+      <c r="AH380" s="19" t="n"/>
+      <c r="AI380" s="19" t="n"/>
+      <c r="AJ380" s="19" t="n"/>
+      <c r="AK380" s="19" t="n"/>
+      <c r="AL380" s="19" t="n"/>
+      <c r="AM380" s="16" t="inlineStr">
+        <is>
+          <t>3 Wagen – abgebildet ist einer davon. Der Inhalt gehört nicht dazu.</t>
+        </is>
+      </c>
+      <c r="AN380" s="22" t="n"/>
+    </row>
+    <row r="381" ht="30" customHeight="1">
+      <c r="A381" s="15" t="inlineStr">
+        <is>
+          <t>NE05-14</t>
+        </is>
+      </c>
+      <c r="B381" s="15" t="n"/>
+      <c r="C381" s="15" t="n"/>
+      <c r="D381" s="15" t="inlineStr">
+        <is>
+          <t>NE05</t>
+        </is>
+      </c>
+      <c r="E381" s="15" t="inlineStr">
+        <is>
+          <t>Glas-Magnettafel weiß, großformatig</t>
+        </is>
+      </c>
+      <c r="F381" s="16" t="inlineStr">
+        <is>
+          <t>Große Schreib- und Magnettafel aus weiß lackiertem Glas, beschreibbar mit Whiteboard-Markern, einschließlich Magneten.</t>
+        </is>
+      </c>
+      <c r="G381" s="15" t="inlineStr">
+        <is>
+          <t>Büro</t>
+        </is>
+      </c>
+      <c r="H381" s="15" t="inlineStr">
+        <is>
+          <t>Speisesaal</t>
+        </is>
+      </c>
+      <c r="I381" s="15" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="J381" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K381" s="17" t="n"/>
+      <c r="L381" s="18">
+        <f>J381-IF(K381="",0,K381)</f>
+        <v/>
+      </c>
+      <c r="M381" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N381" s="15" t="inlineStr">
+        <is>
+          <t>gut</t>
+        </is>
+      </c>
+      <c r="O381" s="19" t="n"/>
+      <c r="P381" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q381" s="19" t="n"/>
+      <c r="R381" s="20" t="n"/>
+      <c r="S381" s="20" t="n">
+        <v>120</v>
+      </c>
+      <c r="T381" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U381" s="21">
+        <f>L381*S381</f>
+        <v/>
+      </c>
+      <c r="V381" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W381" s="15" t="inlineStr">
+        <is>
+          <t>F-482</t>
+        </is>
+      </c>
+      <c r="X381" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y381" s="19" t="n"/>
+      <c r="Z381" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA381" s="19" t="n"/>
+      <c r="AB381" s="19" t="n"/>
+      <c r="AC381" s="19" t="n"/>
+      <c r="AD381" s="19" t="n"/>
+      <c r="AE381" s="20" t="n"/>
+      <c r="AF381" s="21">
+        <f>IF(K381="","",K381*AE381)</f>
+        <v/>
+      </c>
+      <c r="AG381" s="19" t="n"/>
+      <c r="AH381" s="19" t="n"/>
+      <c r="AI381" s="19" t="n"/>
+      <c r="AJ381" s="19" t="n"/>
+      <c r="AK381" s="19" t="n"/>
+      <c r="AL381" s="19" t="n"/>
+      <c r="AM381" s="16" t="inlineStr">
+        <is>
+          <t>1 Tafel einschließlich der Magnete.</t>
+        </is>
+      </c>
+      <c r="AN381" s="22" t="n"/>
+    </row>
+    <row r="382" ht="30" customHeight="1">
+      <c r="A382" s="15" t="inlineStr">
+        <is>
+          <t>NE05-15</t>
+        </is>
+      </c>
+      <c r="B382" s="15" t="n"/>
+      <c r="C382" s="15" t="n"/>
+      <c r="D382" s="15" t="inlineStr">
+        <is>
+          <t>NE05</t>
+        </is>
+      </c>
+      <c r="E382" s="15" t="inlineStr">
+        <is>
+          <t>Wandleuchte Rehkitz schwarz</t>
+        </is>
+      </c>
+      <c r="F382" s="16" t="inlineStr">
+        <is>
+          <t>Wandleuchte in Form eines Rehkitzes aus schwarz lackiertem Holz, mit Kabel und Schnurschalter.</t>
+        </is>
+      </c>
+      <c r="G382" s="15" t="inlineStr">
+        <is>
+          <t>Leuchten</t>
+        </is>
+      </c>
+      <c r="H382" s="15" t="inlineStr">
+        <is>
+          <t>Speisesaal</t>
+        </is>
+      </c>
+      <c r="I382" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J382" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K382" s="17" t="n"/>
+      <c r="L382" s="18">
+        <f>J382-IF(K382="",0,K382)</f>
+        <v/>
+      </c>
+      <c r="M382" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N382" s="15" t="inlineStr">
+        <is>
+          <t>gut</t>
+        </is>
+      </c>
+      <c r="O382" s="19" t="n"/>
+      <c r="P382" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q382" s="19" t="n"/>
+      <c r="R382" s="20" t="n"/>
+      <c r="S382" s="20" t="n">
+        <v>35</v>
+      </c>
+      <c r="T382" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U382" s="21">
+        <f>L382*S382</f>
+        <v/>
+      </c>
+      <c r="V382" s="15" t="inlineStr">
+        <is>
+          <t>Versand möglich</t>
+        </is>
+      </c>
+      <c r="W382" s="15" t="inlineStr">
+        <is>
+          <t>F-483</t>
+        </is>
+      </c>
+      <c r="X382" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y382" s="19" t="n"/>
+      <c r="Z382" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA382" s="19" t="n"/>
+      <c r="AB382" s="19" t="n"/>
+      <c r="AC382" s="19" t="n"/>
+      <c r="AD382" s="19" t="n"/>
+      <c r="AE382" s="20" t="n"/>
+      <c r="AF382" s="21">
+        <f>IF(K382="","",K382*AE382)</f>
+        <v/>
+      </c>
+      <c r="AG382" s="19" t="n"/>
+      <c r="AH382" s="19" t="n"/>
+      <c r="AI382" s="19" t="n"/>
+      <c r="AJ382" s="19" t="n"/>
+      <c r="AK382" s="19" t="n"/>
+      <c r="AL382" s="19" t="n"/>
+      <c r="AM382" s="16" t="inlineStr">
+        <is>
+          <t>2 Leuchten – abgebildet ist eine davon. Ohne Leuchtmittel.</t>
+        </is>
+      </c>
+      <c r="AN382" s="22" t="n"/>
+    </row>
+    <row r="383" ht="30" customHeight="1">
+      <c r="A383" s="15" t="inlineStr">
+        <is>
+          <t>NE05-16</t>
+        </is>
+      </c>
+      <c r="B383" s="15" t="n"/>
+      <c r="C383" s="15" t="n"/>
+      <c r="D383" s="15" t="inlineStr">
+        <is>
+          <t>NE05</t>
+        </is>
+      </c>
+      <c r="E383" s="15" t="inlineStr">
+        <is>
+          <t>Deko-Stern Holz</t>
+        </is>
+      </c>
+      <c r="F383" s="16" t="inlineStr">
+        <is>
+          <t>Fünfzackiger Stern aus massivem Holz, natur, zum Stellen oder Aufhängen.</t>
+        </is>
+      </c>
+      <c r="G383" s="15" t="inlineStr">
+        <is>
+          <t>Deko</t>
+        </is>
+      </c>
+      <c r="H383" s="15" t="inlineStr">
+        <is>
+          <t>Speisesaal</t>
+        </is>
+      </c>
+      <c r="I383" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J383" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="K383" s="17" t="n"/>
+      <c r="L383" s="18">
+        <f>J383-IF(K383="",0,K383)</f>
+        <v/>
+      </c>
+      <c r="M383" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N383" s="15" t="inlineStr">
+        <is>
+          <t>gut</t>
+        </is>
+      </c>
+      <c r="O383" s="19" t="n"/>
+      <c r="P383" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q383" s="19" t="n"/>
+      <c r="R383" s="20" t="n"/>
+      <c r="S383" s="20" t="n">
+        <v>15</v>
+      </c>
+      <c r="T383" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U383" s="21">
+        <f>L383*S383</f>
+        <v/>
+      </c>
+      <c r="V383" s="15" t="inlineStr">
+        <is>
+          <t>Versand möglich</t>
+        </is>
+      </c>
+      <c r="W383" s="15" t="inlineStr">
+        <is>
+          <t>F-484</t>
+        </is>
+      </c>
+      <c r="X383" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y383" s="19" t="n"/>
+      <c r="Z383" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA383" s="19" t="n"/>
+      <c r="AB383" s="19" t="n"/>
+      <c r="AC383" s="19" t="n"/>
+      <c r="AD383" s="19" t="n"/>
+      <c r="AE383" s="20" t="n"/>
+      <c r="AF383" s="21">
+        <f>IF(K383="","",K383*AE383)</f>
+        <v/>
+      </c>
+      <c r="AG383" s="19" t="n"/>
+      <c r="AH383" s="19" t="n"/>
+      <c r="AI383" s="19" t="n"/>
+      <c r="AJ383" s="19" t="n"/>
+      <c r="AK383" s="19" t="n"/>
+      <c r="AL383" s="19" t="n"/>
+      <c r="AM383" s="16" t="inlineStr">
+        <is>
+          <t>6 Sterne – abgebildet ist einer davon.</t>
+        </is>
+      </c>
+      <c r="AN383" s="22" t="n"/>
+    </row>
+    <row r="384" ht="30" customHeight="1">
+      <c r="A384" s="15" t="inlineStr">
+        <is>
+          <t>NE05-17</t>
+        </is>
+      </c>
+      <c r="B384" s="15" t="n"/>
+      <c r="C384" s="15" t="n"/>
+      <c r="D384" s="15" t="inlineStr">
+        <is>
+          <t>NE05</t>
+        </is>
+      </c>
+      <c r="E384" s="15" t="inlineStr">
+        <is>
+          <t>Wandhaken in Stuhlform, schwarz</t>
+        </is>
+      </c>
+      <c r="F384" s="16" t="inlineStr">
+        <is>
+          <t>Kleine Wandhaken in Form von Stühlen aus schwarz lackiertem Holz, in zwei verschiedenen Ausführungen.</t>
+        </is>
+      </c>
+      <c r="G384" s="15" t="inlineStr">
+        <is>
+          <t>Deko</t>
+        </is>
+      </c>
+      <c r="H384" s="15" t="inlineStr">
+        <is>
+          <t>Speisesaal</t>
+        </is>
+      </c>
+      <c r="I384" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J384" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="K384" s="17" t="n"/>
+      <c r="L384" s="18">
+        <f>J384-IF(K384="",0,K384)</f>
+        <v/>
+      </c>
+      <c r="M384" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N384" s="15" t="inlineStr">
+        <is>
+          <t>gut</t>
+        </is>
+      </c>
+      <c r="O384" s="19" t="n"/>
+      <c r="P384" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q384" s="19" t="n"/>
+      <c r="R384" s="20" t="n"/>
+      <c r="S384" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="T384" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U384" s="21">
+        <f>L384*S384</f>
+        <v/>
+      </c>
+      <c r="V384" s="15" t="inlineStr">
+        <is>
+          <t>Versand möglich</t>
+        </is>
+      </c>
+      <c r="W384" s="15" t="inlineStr">
+        <is>
+          <t>F-485</t>
+        </is>
+      </c>
+      <c r="X384" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y384" s="19" t="n"/>
+      <c r="Z384" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA384" s="19" t="n"/>
+      <c r="AB384" s="19" t="n"/>
+      <c r="AC384" s="19" t="n"/>
+      <c r="AD384" s="19" t="n"/>
+      <c r="AE384" s="20" t="n"/>
+      <c r="AF384" s="21">
+        <f>IF(K384="","",K384*AE384)</f>
+        <v/>
+      </c>
+      <c r="AG384" s="19" t="n"/>
+      <c r="AH384" s="19" t="n"/>
+      <c r="AI384" s="19" t="n"/>
+      <c r="AJ384" s="19" t="n"/>
+      <c r="AK384" s="19" t="n"/>
+      <c r="AL384" s="19" t="n"/>
+      <c r="AM384" s="16" t="inlineStr">
+        <is>
+          <t>4 Haken, alle abgebildet.</t>
+        </is>
+      </c>
+      <c r="AN384" s="22" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:AN373"/>
+  <autoFilter ref="A2:AN384"/>
   <mergeCells count="7">
     <mergeCell ref="AI1:AL1"/>
     <mergeCell ref="V1:AD1"/>
@@ -46462,7 +47803,7 @@
     <mergeCell ref="AE1:AH1"/>
     <mergeCell ref="AM1:AN1"/>
   </mergeCells>
-  <conditionalFormatting sqref="Z3:Z373">
+  <conditionalFormatting sqref="Z3:Z384">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"reserviert"</formula>
     </cfRule>
@@ -46473,12 +47814,12 @@
       <formula>"verkauft"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I3:I373">
+  <conditionalFormatting sqref="I3:I384">
     <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
       <formula>"A"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P3:P373">
+  <conditionalFormatting sqref="P3:P384">
     <cfRule type="cellIs" priority="5" operator="equal" dxfId="4">
       <formula>"entfällt"</formula>
     </cfRule>
@@ -46569,7 +47910,7 @@
         </is>
       </c>
       <c r="B5" s="27">
-        <f>COUNTA(Artikelstamm!$A$3:$A$373)</f>
+        <f>COUNTA(Artikelstamm!$A$3:$A$384)</f>
         <v/>
       </c>
     </row>
@@ -46580,7 +47921,7 @@
         </is>
       </c>
       <c r="B6" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$373,"verfügbar")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$384,"verfügbar")</f>
         <v/>
       </c>
     </row>
@@ -46591,7 +47932,7 @@
         </is>
       </c>
       <c r="B7" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$373,"reserviert")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$384,"reserviert")</f>
         <v/>
       </c>
     </row>
@@ -46602,7 +47943,7 @@
         </is>
       </c>
       <c r="B8" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$373,"teilverkauft")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$384,"teilverkauft")</f>
         <v/>
       </c>
     </row>
@@ -46613,7 +47954,7 @@
         </is>
       </c>
       <c r="B9" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$373,"verkauft")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$384,"verkauft")</f>
         <v/>
       </c>
     </row>
@@ -46624,7 +47965,7 @@
         </is>
       </c>
       <c r="B10" s="27">
-        <f>SUM(Artikelstamm!$L$3:$L$373)</f>
+        <f>SUM(Artikelstamm!$L$3:$L$384)</f>
         <v/>
       </c>
     </row>
@@ -46635,7 +47976,7 @@
         </is>
       </c>
       <c r="B11" s="29">
-        <f>SUM(Artikelstamm!$U$3:$U$373)</f>
+        <f>SUM(Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -46653,7 +47994,7 @@
         </is>
       </c>
       <c r="B13" s="27">
-        <f>SUM(Artikelstamm!$K$3:$K$373)</f>
+        <f>SUM(Artikelstamm!$K$3:$K$384)</f>
         <v/>
       </c>
     </row>
@@ -46664,7 +48005,7 @@
         </is>
       </c>
       <c r="B14" s="30">
-        <f>SUMPRODUCT(Artikelstamm!$K$3:$K$373,Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT(Artikelstamm!$K$3:$K$384,Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
     </row>
@@ -46697,7 +48038,7 @@
         </is>
       </c>
       <c r="B17" s="30">
-        <f>SUMPRODUCT((Artikelstamm!$AJ$3:$AJ$373="bezahlt")*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AJ$3:$AJ$384="bezahlt")*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
     </row>
@@ -46726,7 +48067,7 @@
         </is>
       </c>
       <c r="B21" s="31">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$373,"*verkauft",Artikelstamm!$AI$3:$AI$373,"")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$384,"*verkauft",Artikelstamm!$AI$3:$AI$384,"")</f>
         <v/>
       </c>
     </row>
@@ -46737,7 +48078,7 @@
         </is>
       </c>
       <c r="B22" s="31">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$373,"*verkauft",Artikelstamm!$AJ$3:$AJ$373,"offen")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$384,"*verkauft",Artikelstamm!$AJ$3:$AJ$384,"offen")</f>
         <v/>
       </c>
     </row>
@@ -46748,7 +48089,7 @@
         </is>
       </c>
       <c r="B23" s="27">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$373,"reserviert",Artikelstamm!$AL$3:$AL$373,"")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$384,"reserviert",Artikelstamm!$AL$3:$AL$384,"")</f>
         <v/>
       </c>
     </row>
@@ -46759,7 +48100,7 @@
         </is>
       </c>
       <c r="B24" s="27">
-        <f>COUNTIFS(Artikelstamm!$S$3:$S$373,"")</f>
+        <f>COUNTIFS(Artikelstamm!$S$3:$S$384,"")</f>
         <v/>
       </c>
     </row>
@@ -46770,7 +48111,7 @@
         </is>
       </c>
       <c r="B25" s="27">
-        <f>COUNTIFS(Artikelstamm!$O$3:$O$373,"")</f>
+        <f>COUNTIFS(Artikelstamm!$O$3:$O$384,"")</f>
         <v/>
       </c>
     </row>
@@ -46810,15 +48151,15 @@
         </is>
       </c>
       <c r="B30" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$373,$A30)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$384,$A30)</f>
         <v/>
       </c>
       <c r="C30" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$373=$A30)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$384=$A30)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D30" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$373,$A30,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$384,$A30,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -46829,15 +48170,15 @@
         </is>
       </c>
       <c r="B31" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$373,$A31)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$384,$A31)</f>
         <v/>
       </c>
       <c r="C31" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$373=$A31)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$384=$A31)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D31" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$373,$A31,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$384,$A31,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -46848,15 +48189,15 @@
         </is>
       </c>
       <c r="B32" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$373,$A32)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$384,$A32)</f>
         <v/>
       </c>
       <c r="C32" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$373=$A32)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$384=$A32)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D32" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$373,$A32,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$384,$A32,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -46915,15 +48256,15 @@
         </is>
       </c>
       <c r="B37" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$373,$A37)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$384,$A37)</f>
         <v/>
       </c>
       <c r="C37" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$373=$A37)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$384=$A37)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D37" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$373,$A37,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$384,$A37,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -46934,15 +48275,15 @@
         </is>
       </c>
       <c r="B38" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$373,$A38)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$384,$A38)</f>
         <v/>
       </c>
       <c r="C38" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$373=$A38)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$384=$A38)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D38" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$373,$A38,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$384,$A38,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -46953,15 +48294,15 @@
         </is>
       </c>
       <c r="B39" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$373,$A39)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$384,$A39)</f>
         <v/>
       </c>
       <c r="C39" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$373=$A39)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$384=$A39)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D39" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$373,$A39,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$384,$A39,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -46972,15 +48313,15 @@
         </is>
       </c>
       <c r="B40" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$373,$A40)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$384,$A40)</f>
         <v/>
       </c>
       <c r="C40" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$373=$A40)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$384=$A40)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D40" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$373,$A40,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$384,$A40,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -46991,15 +48332,15 @@
         </is>
       </c>
       <c r="B41" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$373,$A41)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$384,$A41)</f>
         <v/>
       </c>
       <c r="C41" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$373=$A41)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$384=$A41)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D41" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$373,$A41,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$384,$A41,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47010,15 +48351,15 @@
         </is>
       </c>
       <c r="B42" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$373,$A42)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$384,$A42)</f>
         <v/>
       </c>
       <c r="C42" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$373=$A42)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$384=$A42)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D42" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$373,$A42,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$384,$A42,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47029,15 +48370,15 @@
         </is>
       </c>
       <c r="B43" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$373,$A43)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$384,$A43)</f>
         <v/>
       </c>
       <c r="C43" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$373=$A43)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$384=$A43)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D43" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$373,$A43,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$384,$A43,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47048,15 +48389,15 @@
         </is>
       </c>
       <c r="B44" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$373,$A44)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$384,$A44)</f>
         <v/>
       </c>
       <c r="C44" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$373=$A44)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$384=$A44)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D44" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$373,$A44,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$384,$A44,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47067,15 +48408,15 @@
         </is>
       </c>
       <c r="B45" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$373,$A45)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$384,$A45)</f>
         <v/>
       </c>
       <c r="C45" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$373=$A45)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$384=$A45)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D45" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$373,$A45,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$384,$A45,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47086,15 +48427,15 @@
         </is>
       </c>
       <c r="B46" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$373,$A46)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$384,$A46)</f>
         <v/>
       </c>
       <c r="C46" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$373=$A46)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$384=$A46)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D46" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$373,$A46,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$384,$A46,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47105,15 +48446,15 @@
         </is>
       </c>
       <c r="B47" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$373,$A47)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$384,$A47)</f>
         <v/>
       </c>
       <c r="C47" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$373=$A47)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$384=$A47)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D47" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$373,$A47,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$384,$A47,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47124,15 +48465,15 @@
         </is>
       </c>
       <c r="B48" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$373,$A48)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$384,$A48)</f>
         <v/>
       </c>
       <c r="C48" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$373=$A48)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$384=$A48)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D48" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$373,$A48,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$384,$A48,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47143,15 +48484,15 @@
         </is>
       </c>
       <c r="B49" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$373,$A49)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$384,$A49)</f>
         <v/>
       </c>
       <c r="C49" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$373=$A49)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$384=$A49)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D49" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$373,$A49,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$384,$A49,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47162,15 +48503,15 @@
         </is>
       </c>
       <c r="B50" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$373,$A50)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$384,$A50)</f>
         <v/>
       </c>
       <c r="C50" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$373=$A50)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$384=$A50)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D50" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$373,$A50,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$384,$A50,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47229,15 +48570,15 @@
         </is>
       </c>
       <c r="B55" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A55)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A55)</f>
         <v/>
       </c>
       <c r="C55" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A55)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A55)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D55" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A55,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A55,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47248,15 +48589,15 @@
         </is>
       </c>
       <c r="B56" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A56)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A56)</f>
         <v/>
       </c>
       <c r="C56" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A56)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A56)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D56" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A56,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A56,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47267,15 +48608,15 @@
         </is>
       </c>
       <c r="B57" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A57)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A57)</f>
         <v/>
       </c>
       <c r="C57" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A57)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A57)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D57" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A57,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A57,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47286,15 +48627,15 @@
         </is>
       </c>
       <c r="B58" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A58)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A58)</f>
         <v/>
       </c>
       <c r="C58" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A58)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A58)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D58" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A58,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A58,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47305,15 +48646,15 @@
         </is>
       </c>
       <c r="B59" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A59)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A59)</f>
         <v/>
       </c>
       <c r="C59" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A59)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A59)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D59" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A59,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A59,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47324,15 +48665,15 @@
         </is>
       </c>
       <c r="B60" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A60)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A60)</f>
         <v/>
       </c>
       <c r="C60" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A60)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A60)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D60" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A60,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A60,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47343,15 +48684,15 @@
         </is>
       </c>
       <c r="B61" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A61)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A61)</f>
         <v/>
       </c>
       <c r="C61" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A61)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A61)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D61" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A61,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A61,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47362,15 +48703,15 @@
         </is>
       </c>
       <c r="B62" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A62)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A62)</f>
         <v/>
       </c>
       <c r="C62" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A62)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A62)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D62" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A62,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A62,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47381,15 +48722,15 @@
         </is>
       </c>
       <c r="B63" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A63)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A63)</f>
         <v/>
       </c>
       <c r="C63" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A63)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A63)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D63" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A63,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A63,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47400,15 +48741,15 @@
         </is>
       </c>
       <c r="B64" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A64)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A64)</f>
         <v/>
       </c>
       <c r="C64" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A64)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A64)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D64" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A64,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A64,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47419,15 +48760,15 @@
         </is>
       </c>
       <c r="B65" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A65)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A65)</f>
         <v/>
       </c>
       <c r="C65" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A65)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A65)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D65" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A65,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A65,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47438,15 +48779,15 @@
         </is>
       </c>
       <c r="B66" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A66)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A66)</f>
         <v/>
       </c>
       <c r="C66" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A66)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A66)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D66" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A66,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A66,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47457,15 +48798,15 @@
         </is>
       </c>
       <c r="B67" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A67)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A67)</f>
         <v/>
       </c>
       <c r="C67" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A67)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A67)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D67" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A67,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A67,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47476,15 +48817,15 @@
         </is>
       </c>
       <c r="B68" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A68)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A68)</f>
         <v/>
       </c>
       <c r="C68" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A68)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A68)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D68" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A68,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A68,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47495,15 +48836,15 @@
         </is>
       </c>
       <c r="B69" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A69)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A69)</f>
         <v/>
       </c>
       <c r="C69" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A69)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A69)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D69" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A69,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A69,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47514,15 +48855,15 @@
         </is>
       </c>
       <c r="B70" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A70)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A70)</f>
         <v/>
       </c>
       <c r="C70" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A70)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A70)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D70" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A70,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A70,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47533,15 +48874,15 @@
         </is>
       </c>
       <c r="B71" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A71)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A71)</f>
         <v/>
       </c>
       <c r="C71" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A71)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A71)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D71" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A71,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A71,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47552,15 +48893,15 @@
         </is>
       </c>
       <c r="B72" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A72)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A72)</f>
         <v/>
       </c>
       <c r="C72" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A72)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A72)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D72" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A72,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A72,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47571,15 +48912,15 @@
         </is>
       </c>
       <c r="B73" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A73)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A73)</f>
         <v/>
       </c>
       <c r="C73" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A73)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A73)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D73" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A73,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A73,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47590,15 +48931,15 @@
         </is>
       </c>
       <c r="B74" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A74)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A74)</f>
         <v/>
       </c>
       <c r="C74" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A74)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A74)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D74" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A74,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A74,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47609,15 +48950,15 @@
         </is>
       </c>
       <c r="B75" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A75)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A75)</f>
         <v/>
       </c>
       <c r="C75" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A75)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A75)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D75" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A75,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A75,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47628,15 +48969,15 @@
         </is>
       </c>
       <c r="B76" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A76)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A76)</f>
         <v/>
       </c>
       <c r="C76" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A76)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A76)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D76" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A76,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A76,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47647,15 +48988,15 @@
         </is>
       </c>
       <c r="B77" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A77)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A77)</f>
         <v/>
       </c>
       <c r="C77" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A77)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A77)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D77" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A77,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A77,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47666,15 +49007,15 @@
         </is>
       </c>
       <c r="B78" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A78)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A78)</f>
         <v/>
       </c>
       <c r="C78" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A78)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A78)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D78" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A78,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A78,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47685,15 +49026,15 @@
         </is>
       </c>
       <c r="B79" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A79)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A79)</f>
         <v/>
       </c>
       <c r="C79" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A79)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A79)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D79" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A79,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A79,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47704,15 +49045,15 @@
         </is>
       </c>
       <c r="B80" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A80)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A80)</f>
         <v/>
       </c>
       <c r="C80" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A80)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A80)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D80" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A80,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A80,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47723,15 +49064,15 @@
         </is>
       </c>
       <c r="B81" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A81)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A81)</f>
         <v/>
       </c>
       <c r="C81" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A81)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A81)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D81" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A81,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A81,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47742,15 +49083,15 @@
         </is>
       </c>
       <c r="B82" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A82)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A82)</f>
         <v/>
       </c>
       <c r="C82" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A82)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A82)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D82" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A82,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A82,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47761,15 +49102,15 @@
         </is>
       </c>
       <c r="B83" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A83)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A83)</f>
         <v/>
       </c>
       <c r="C83" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A83)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A83)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D83" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A83,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A83,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47780,15 +49121,15 @@
         </is>
       </c>
       <c r="B84" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A84)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A84)</f>
         <v/>
       </c>
       <c r="C84" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A84)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A84)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D84" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A84,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A84,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47799,15 +49140,15 @@
         </is>
       </c>
       <c r="B85" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A85)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A85)</f>
         <v/>
       </c>
       <c r="C85" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A85)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A85)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D85" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A85,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A85,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47818,15 +49159,15 @@
         </is>
       </c>
       <c r="B86" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A86)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A86)</f>
         <v/>
       </c>
       <c r="C86" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A86)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A86)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D86" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A86,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A86,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47837,15 +49178,15 @@
         </is>
       </c>
       <c r="B87" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$373,$A87)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A87)</f>
         <v/>
       </c>
       <c r="C87" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$373=$A87)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A87)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
       <c r="D87" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$373,$A87,Artikelstamm!$U$3:$U$373)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A87,Artikelstamm!$U$3:$U$384)</f>
         <v/>
       </c>
     </row>
@@ -47899,11 +49240,11 @@
         </is>
       </c>
       <c r="B92" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$373,$A92)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$384,$A92)</f>
         <v/>
       </c>
       <c r="C92" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$373=$A92)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$384=$A92)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
     </row>
@@ -47914,11 +49255,11 @@
         </is>
       </c>
       <c r="B93" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$373,$A93)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$384,$A93)</f>
         <v/>
       </c>
       <c r="C93" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$373=$A93)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$384=$A93)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
     </row>
@@ -47929,11 +49270,11 @@
         </is>
       </c>
       <c r="B94" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$373,$A94)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$384,$A94)</f>
         <v/>
       </c>
       <c r="C94" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$373=$A94)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$384=$A94)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
     </row>
@@ -47944,11 +49285,11 @@
         </is>
       </c>
       <c r="B95" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$373,$A95)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$384,$A95)</f>
         <v/>
       </c>
       <c r="C95" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$373=$A95)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$384=$A95)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
     </row>
@@ -47959,11 +49300,11 @@
         </is>
       </c>
       <c r="B96" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$373,$A96)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$384,$A96)</f>
         <v/>
       </c>
       <c r="C96" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$373=$A96)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$384=$A96)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
     </row>
@@ -47974,11 +49315,11 @@
         </is>
       </c>
       <c r="B97" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$373,$A97)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$384,$A97)</f>
         <v/>
       </c>
       <c r="C97" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$373=$A97)*Artikelstamm!$K$3:$K$373*Artikelstamm!$AE$3:$AE$373)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$384=$A97)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
NE05-12 nachgetragen (weisse Freischwinger, Kindergroesse)
Die Position war in der Erfassung von NE05 versehentlich ausgefallen,
obwohl andere Positionen schon darauf verwiesen haben. 5 Stueck,
Im_Katalog = nein mit demselben offenen Markenpunkt wie die anderen
Freischwinger.

Datenbasis 383 Positionen / 327 aktiv, pruefen.py 0 Fehler.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011yyfqhuiWGsaNy38oaNoGo
</commit_message>
<xml_diff>
--- a/ausgabe/01_Artikelstamm_kikripp.xlsx
+++ b/ausgabe/01_Artikelstamm_kikripp.xlsx
@@ -15,7 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Artikelstamm'!$A$2:$AN$384</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Artikelstamm'!$A$2:$AN$385</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1019,7 +1019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN384"/>
+  <dimension ref="A1:AN385"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -47792,8 +47792,131 @@
       </c>
       <c r="AN384" s="22" t="n"/>
     </row>
+    <row r="385" ht="30" customHeight="1">
+      <c r="A385" s="15" t="inlineStr">
+        <is>
+          <t>NE05-12</t>
+        </is>
+      </c>
+      <c r="B385" s="15" t="n"/>
+      <c r="C385" s="15" t="n"/>
+      <c r="D385" s="15" t="inlineStr">
+        <is>
+          <t>NE05</t>
+        </is>
+      </c>
+      <c r="E385" s="15" t="inlineStr">
+        <is>
+          <t>Freischwinger weiß, Kindergröße</t>
+        </is>
+      </c>
+      <c r="F385" s="16" t="inlineStr">
+        <is>
+          <t>Freischwinger aus einem Stück Kunststoff, weiß matt, S-förmig geschwungen. Kindergröße.</t>
+        </is>
+      </c>
+      <c r="G385" s="15" t="inlineStr">
+        <is>
+          <t>Kita-Ausstattung</t>
+        </is>
+      </c>
+      <c r="H385" s="15" t="inlineStr">
+        <is>
+          <t>Speisesaal</t>
+        </is>
+      </c>
+      <c r="I385" s="15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="J385" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="K385" s="17" t="n"/>
+      <c r="L385" s="18">
+        <f>J385-IF(K385="",0,K385)</f>
+        <v/>
+      </c>
+      <c r="M385" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N385" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O385" s="19" t="n"/>
+      <c r="P385" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q385" s="19" t="n"/>
+      <c r="R385" s="20" t="n"/>
+      <c r="S385" s="20" t="n">
+        <v>120</v>
+      </c>
+      <c r="T385" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U385" s="21">
+        <f>L385*S385</f>
+        <v/>
+      </c>
+      <c r="V385" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W385" s="15" t="inlineStr">
+        <is>
+          <t>F-479</t>
+        </is>
+      </c>
+      <c r="X385" s="19" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="Y385" s="19" t="n"/>
+      <c r="Z385" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA385" s="19" t="n"/>
+      <c r="AB385" s="19" t="n"/>
+      <c r="AC385" s="19" t="n"/>
+      <c r="AD385" s="19" t="n"/>
+      <c r="AE385" s="20" t="n"/>
+      <c r="AF385" s="21">
+        <f>IF(K385="","",K385*AE385)</f>
+        <v/>
+      </c>
+      <c r="AG385" s="19" t="n"/>
+      <c r="AH385" s="19" t="n"/>
+      <c r="AI385" s="19" t="n"/>
+      <c r="AJ385" s="19" t="n"/>
+      <c r="AK385" s="19" t="n"/>
+      <c r="AL385" s="19" t="n"/>
+      <c r="AM385" s="16" t="inlineStr">
+        <is>
+          <t>5 Stühle – abgebildet ist einer davon, die Seitenansicht auf Foto F-480. Weitere Freischwinger gleicher Form stehen unter NU04-20, NE05-04 und NE05-05.</t>
+        </is>
+      </c>
+      <c r="AN385" s="22" t="inlineStr">
+        <is>
+          <t>OFFEN: NICHT VEROEFFENTLICHEN, bis die Marke geklaert ist. Die Form ist der Panton Chair von Verner Panton, Original von Vitra. Gebraucht 120-250 EUR je Erwachsenenstuhl und 90-150 EUR je Kinderstuhl, ein Nachbau 30-50 bzw. 20-30 EUR. Das Original traegt auf der Unterseite eine eingeformte Vitra-Kennzeichnung. Betrifft NU04-20, NE05-04, NE05-05 und NE05-12 - eine Nahaufnahme der Unterseite genuegt fuer alle vier.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:AN384"/>
+  <autoFilter ref="A2:AN385"/>
   <mergeCells count="7">
     <mergeCell ref="AI1:AL1"/>
     <mergeCell ref="V1:AD1"/>
@@ -47803,7 +47926,7 @@
     <mergeCell ref="AE1:AH1"/>
     <mergeCell ref="AM1:AN1"/>
   </mergeCells>
-  <conditionalFormatting sqref="Z3:Z384">
+  <conditionalFormatting sqref="Z3:Z385">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"reserviert"</formula>
     </cfRule>
@@ -47814,12 +47937,12 @@
       <formula>"verkauft"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I3:I384">
+  <conditionalFormatting sqref="I3:I385">
     <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
       <formula>"A"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P3:P384">
+  <conditionalFormatting sqref="P3:P385">
     <cfRule type="cellIs" priority="5" operator="equal" dxfId="4">
       <formula>"entfällt"</formula>
     </cfRule>
@@ -47910,7 +48033,7 @@
         </is>
       </c>
       <c r="B5" s="27">
-        <f>COUNTA(Artikelstamm!$A$3:$A$384)</f>
+        <f>COUNTA(Artikelstamm!$A$3:$A$385)</f>
         <v/>
       </c>
     </row>
@@ -47921,7 +48044,7 @@
         </is>
       </c>
       <c r="B6" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$384,"verfügbar")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$385,"verfügbar")</f>
         <v/>
       </c>
     </row>
@@ -47932,7 +48055,7 @@
         </is>
       </c>
       <c r="B7" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$384,"reserviert")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$385,"reserviert")</f>
         <v/>
       </c>
     </row>
@@ -47943,7 +48066,7 @@
         </is>
       </c>
       <c r="B8" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$384,"teilverkauft")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$385,"teilverkauft")</f>
         <v/>
       </c>
     </row>
@@ -47954,7 +48077,7 @@
         </is>
       </c>
       <c r="B9" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$384,"verkauft")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$385,"verkauft")</f>
         <v/>
       </c>
     </row>
@@ -47965,7 +48088,7 @@
         </is>
       </c>
       <c r="B10" s="27">
-        <f>SUM(Artikelstamm!$L$3:$L$384)</f>
+        <f>SUM(Artikelstamm!$L$3:$L$385)</f>
         <v/>
       </c>
     </row>
@@ -47976,7 +48099,7 @@
         </is>
       </c>
       <c r="B11" s="29">
-        <f>SUM(Artikelstamm!$U$3:$U$384)</f>
+        <f>SUM(Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -47994,7 +48117,7 @@
         </is>
       </c>
       <c r="B13" s="27">
-        <f>SUM(Artikelstamm!$K$3:$K$384)</f>
+        <f>SUM(Artikelstamm!$K$3:$K$385)</f>
         <v/>
       </c>
     </row>
@@ -48005,7 +48128,7 @@
         </is>
       </c>
       <c r="B14" s="30">
-        <f>SUMPRODUCT(Artikelstamm!$K$3:$K$384,Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT(Artikelstamm!$K$3:$K$385,Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
     </row>
@@ -48038,7 +48161,7 @@
         </is>
       </c>
       <c r="B17" s="30">
-        <f>SUMPRODUCT((Artikelstamm!$AJ$3:$AJ$384="bezahlt")*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AJ$3:$AJ$385="bezahlt")*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
     </row>
@@ -48067,7 +48190,7 @@
         </is>
       </c>
       <c r="B21" s="31">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$384,"*verkauft",Artikelstamm!$AI$3:$AI$384,"")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$385,"*verkauft",Artikelstamm!$AI$3:$AI$385,"")</f>
         <v/>
       </c>
     </row>
@@ -48078,7 +48201,7 @@
         </is>
       </c>
       <c r="B22" s="31">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$384,"*verkauft",Artikelstamm!$AJ$3:$AJ$384,"offen")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$385,"*verkauft",Artikelstamm!$AJ$3:$AJ$385,"offen")</f>
         <v/>
       </c>
     </row>
@@ -48089,7 +48212,7 @@
         </is>
       </c>
       <c r="B23" s="27">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$384,"reserviert",Artikelstamm!$AL$3:$AL$384,"")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$385,"reserviert",Artikelstamm!$AL$3:$AL$385,"")</f>
         <v/>
       </c>
     </row>
@@ -48100,7 +48223,7 @@
         </is>
       </c>
       <c r="B24" s="27">
-        <f>COUNTIFS(Artikelstamm!$S$3:$S$384,"")</f>
+        <f>COUNTIFS(Artikelstamm!$S$3:$S$385,"")</f>
         <v/>
       </c>
     </row>
@@ -48111,7 +48234,7 @@
         </is>
       </c>
       <c r="B25" s="27">
-        <f>COUNTIFS(Artikelstamm!$O$3:$O$384,"")</f>
+        <f>COUNTIFS(Artikelstamm!$O$3:$O$385,"")</f>
         <v/>
       </c>
     </row>
@@ -48151,15 +48274,15 @@
         </is>
       </c>
       <c r="B30" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$384,$A30)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$385,$A30)</f>
         <v/>
       </c>
       <c r="C30" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$384=$A30)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$385=$A30)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D30" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$384,$A30,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$385,$A30,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -48170,15 +48293,15 @@
         </is>
       </c>
       <c r="B31" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$384,$A31)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$385,$A31)</f>
         <v/>
       </c>
       <c r="C31" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$384=$A31)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$385=$A31)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D31" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$384,$A31,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$385,$A31,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -48189,15 +48312,15 @@
         </is>
       </c>
       <c r="B32" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$384,$A32)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$385,$A32)</f>
         <v/>
       </c>
       <c r="C32" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$384=$A32)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$385=$A32)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D32" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$384,$A32,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$385,$A32,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -48256,15 +48379,15 @@
         </is>
       </c>
       <c r="B37" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$384,$A37)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$385,$A37)</f>
         <v/>
       </c>
       <c r="C37" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$384=$A37)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$385=$A37)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D37" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$384,$A37,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$385,$A37,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -48275,15 +48398,15 @@
         </is>
       </c>
       <c r="B38" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$384,$A38)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$385,$A38)</f>
         <v/>
       </c>
       <c r="C38" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$384=$A38)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$385=$A38)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D38" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$384,$A38,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$385,$A38,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -48294,15 +48417,15 @@
         </is>
       </c>
       <c r="B39" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$384,$A39)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$385,$A39)</f>
         <v/>
       </c>
       <c r="C39" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$384=$A39)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$385=$A39)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D39" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$384,$A39,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$385,$A39,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -48313,15 +48436,15 @@
         </is>
       </c>
       <c r="B40" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$384,$A40)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$385,$A40)</f>
         <v/>
       </c>
       <c r="C40" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$384=$A40)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$385=$A40)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D40" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$384,$A40,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$385,$A40,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -48332,15 +48455,15 @@
         </is>
       </c>
       <c r="B41" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$384,$A41)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$385,$A41)</f>
         <v/>
       </c>
       <c r="C41" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$384=$A41)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$385=$A41)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D41" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$384,$A41,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$385,$A41,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -48351,15 +48474,15 @@
         </is>
       </c>
       <c r="B42" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$384,$A42)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$385,$A42)</f>
         <v/>
       </c>
       <c r="C42" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$384=$A42)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$385=$A42)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D42" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$384,$A42,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$385,$A42,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -48370,15 +48493,15 @@
         </is>
       </c>
       <c r="B43" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$384,$A43)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$385,$A43)</f>
         <v/>
       </c>
       <c r="C43" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$384=$A43)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$385=$A43)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D43" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$384,$A43,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$385,$A43,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -48389,15 +48512,15 @@
         </is>
       </c>
       <c r="B44" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$384,$A44)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$385,$A44)</f>
         <v/>
       </c>
       <c r="C44" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$384=$A44)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$385=$A44)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D44" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$384,$A44,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$385,$A44,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -48408,15 +48531,15 @@
         </is>
       </c>
       <c r="B45" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$384,$A45)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$385,$A45)</f>
         <v/>
       </c>
       <c r="C45" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$384=$A45)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$385=$A45)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D45" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$384,$A45,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$385,$A45,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -48427,15 +48550,15 @@
         </is>
       </c>
       <c r="B46" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$384,$A46)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$385,$A46)</f>
         <v/>
       </c>
       <c r="C46" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$384=$A46)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$385=$A46)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D46" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$384,$A46,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$385,$A46,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -48446,15 +48569,15 @@
         </is>
       </c>
       <c r="B47" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$384,$A47)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$385,$A47)</f>
         <v/>
       </c>
       <c r="C47" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$384=$A47)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$385=$A47)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D47" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$384,$A47,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$385,$A47,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -48465,15 +48588,15 @@
         </is>
       </c>
       <c r="B48" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$384,$A48)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$385,$A48)</f>
         <v/>
       </c>
       <c r="C48" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$384=$A48)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$385=$A48)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D48" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$384,$A48,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$385,$A48,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -48484,15 +48607,15 @@
         </is>
       </c>
       <c r="B49" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$384,$A49)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$385,$A49)</f>
         <v/>
       </c>
       <c r="C49" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$384=$A49)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$385=$A49)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D49" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$384,$A49,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$385,$A49,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -48503,15 +48626,15 @@
         </is>
       </c>
       <c r="B50" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$384,$A50)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$385,$A50)</f>
         <v/>
       </c>
       <c r="C50" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$384=$A50)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$385=$A50)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D50" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$384,$A50,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$385,$A50,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -48570,15 +48693,15 @@
         </is>
       </c>
       <c r="B55" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A55)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$385,$A55)</f>
         <v/>
       </c>
       <c r="C55" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A55)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$385=$A55)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D55" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A55,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$385,$A55,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -48589,15 +48712,15 @@
         </is>
       </c>
       <c r="B56" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A56)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$385,$A56)</f>
         <v/>
       </c>
       <c r="C56" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A56)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$385=$A56)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D56" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A56,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$385,$A56,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -48608,15 +48731,15 @@
         </is>
       </c>
       <c r="B57" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A57)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$385,$A57)</f>
         <v/>
       </c>
       <c r="C57" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A57)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$385=$A57)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D57" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A57,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$385,$A57,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -48627,15 +48750,15 @@
         </is>
       </c>
       <c r="B58" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A58)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$385,$A58)</f>
         <v/>
       </c>
       <c r="C58" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A58)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$385=$A58)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D58" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A58,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$385,$A58,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -48646,15 +48769,15 @@
         </is>
       </c>
       <c r="B59" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A59)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$385,$A59)</f>
         <v/>
       </c>
       <c r="C59" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A59)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$385=$A59)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D59" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A59,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$385,$A59,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -48665,15 +48788,15 @@
         </is>
       </c>
       <c r="B60" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A60)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$385,$A60)</f>
         <v/>
       </c>
       <c r="C60" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A60)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$385=$A60)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D60" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A60,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$385,$A60,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -48684,15 +48807,15 @@
         </is>
       </c>
       <c r="B61" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A61)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$385,$A61)</f>
         <v/>
       </c>
       <c r="C61" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A61)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$385=$A61)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D61" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A61,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$385,$A61,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -48703,15 +48826,15 @@
         </is>
       </c>
       <c r="B62" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A62)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$385,$A62)</f>
         <v/>
       </c>
       <c r="C62" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A62)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$385=$A62)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D62" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A62,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$385,$A62,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -48722,15 +48845,15 @@
         </is>
       </c>
       <c r="B63" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A63)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$385,$A63)</f>
         <v/>
       </c>
       <c r="C63" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A63)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$385=$A63)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D63" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A63,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$385,$A63,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -48741,15 +48864,15 @@
         </is>
       </c>
       <c r="B64" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A64)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$385,$A64)</f>
         <v/>
       </c>
       <c r="C64" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A64)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$385=$A64)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D64" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A64,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$385,$A64,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -48760,15 +48883,15 @@
         </is>
       </c>
       <c r="B65" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A65)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$385,$A65)</f>
         <v/>
       </c>
       <c r="C65" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A65)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$385=$A65)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D65" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A65,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$385,$A65,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -48779,15 +48902,15 @@
         </is>
       </c>
       <c r="B66" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A66)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$385,$A66)</f>
         <v/>
       </c>
       <c r="C66" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A66)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$385=$A66)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D66" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A66,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$385,$A66,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -48798,15 +48921,15 @@
         </is>
       </c>
       <c r="B67" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A67)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$385,$A67)</f>
         <v/>
       </c>
       <c r="C67" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A67)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$385=$A67)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D67" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A67,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$385,$A67,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -48817,15 +48940,15 @@
         </is>
       </c>
       <c r="B68" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A68)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$385,$A68)</f>
         <v/>
       </c>
       <c r="C68" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A68)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$385=$A68)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D68" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A68,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$385,$A68,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -48836,15 +48959,15 @@
         </is>
       </c>
       <c r="B69" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A69)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$385,$A69)</f>
         <v/>
       </c>
       <c r="C69" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A69)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$385=$A69)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D69" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A69,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$385,$A69,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -48855,15 +48978,15 @@
         </is>
       </c>
       <c r="B70" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A70)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$385,$A70)</f>
         <v/>
       </c>
       <c r="C70" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A70)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$385=$A70)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D70" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A70,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$385,$A70,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -48874,15 +48997,15 @@
         </is>
       </c>
       <c r="B71" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A71)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$385,$A71)</f>
         <v/>
       </c>
       <c r="C71" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A71)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$385=$A71)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D71" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A71,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$385,$A71,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -48893,15 +49016,15 @@
         </is>
       </c>
       <c r="B72" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A72)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$385,$A72)</f>
         <v/>
       </c>
       <c r="C72" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A72)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$385=$A72)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D72" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A72,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$385,$A72,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -48912,15 +49035,15 @@
         </is>
       </c>
       <c r="B73" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A73)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$385,$A73)</f>
         <v/>
       </c>
       <c r="C73" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A73)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$385=$A73)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D73" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A73,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$385,$A73,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -48931,15 +49054,15 @@
         </is>
       </c>
       <c r="B74" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A74)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$385,$A74)</f>
         <v/>
       </c>
       <c r="C74" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A74)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$385=$A74)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D74" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A74,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$385,$A74,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -48950,15 +49073,15 @@
         </is>
       </c>
       <c r="B75" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A75)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$385,$A75)</f>
         <v/>
       </c>
       <c r="C75" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A75)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$385=$A75)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D75" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A75,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$385,$A75,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -48969,15 +49092,15 @@
         </is>
       </c>
       <c r="B76" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A76)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$385,$A76)</f>
         <v/>
       </c>
       <c r="C76" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A76)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$385=$A76)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D76" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A76,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$385,$A76,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -48988,15 +49111,15 @@
         </is>
       </c>
       <c r="B77" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A77)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$385,$A77)</f>
         <v/>
       </c>
       <c r="C77" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A77)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$385=$A77)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D77" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A77,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$385,$A77,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -49007,15 +49130,15 @@
         </is>
       </c>
       <c r="B78" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A78)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$385,$A78)</f>
         <v/>
       </c>
       <c r="C78" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A78)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$385=$A78)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D78" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A78,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$385,$A78,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -49026,15 +49149,15 @@
         </is>
       </c>
       <c r="B79" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A79)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$385,$A79)</f>
         <v/>
       </c>
       <c r="C79" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A79)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$385=$A79)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D79" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A79,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$385,$A79,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -49045,15 +49168,15 @@
         </is>
       </c>
       <c r="B80" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A80)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$385,$A80)</f>
         <v/>
       </c>
       <c r="C80" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A80)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$385=$A80)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D80" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A80,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$385,$A80,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -49064,15 +49187,15 @@
         </is>
       </c>
       <c r="B81" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A81)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$385,$A81)</f>
         <v/>
       </c>
       <c r="C81" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A81)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$385=$A81)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D81" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A81,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$385,$A81,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -49083,15 +49206,15 @@
         </is>
       </c>
       <c r="B82" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A82)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$385,$A82)</f>
         <v/>
       </c>
       <c r="C82" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A82)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$385=$A82)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D82" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A82,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$385,$A82,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -49102,15 +49225,15 @@
         </is>
       </c>
       <c r="B83" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A83)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$385,$A83)</f>
         <v/>
       </c>
       <c r="C83" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A83)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$385=$A83)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D83" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A83,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$385,$A83,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -49121,15 +49244,15 @@
         </is>
       </c>
       <c r="B84" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A84)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$385,$A84)</f>
         <v/>
       </c>
       <c r="C84" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A84)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$385=$A84)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D84" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A84,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$385,$A84,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -49140,15 +49263,15 @@
         </is>
       </c>
       <c r="B85" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A85)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$385,$A85)</f>
         <v/>
       </c>
       <c r="C85" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A85)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$385=$A85)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D85" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A85,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$385,$A85,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -49159,15 +49282,15 @@
         </is>
       </c>
       <c r="B86" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A86)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$385,$A86)</f>
         <v/>
       </c>
       <c r="C86" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A86)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$385=$A86)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D86" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A86,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$385,$A86,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -49178,15 +49301,15 @@
         </is>
       </c>
       <c r="B87" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$384,$A87)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$385,$A87)</f>
         <v/>
       </c>
       <c r="C87" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$384=$A87)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$385=$A87)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
       <c r="D87" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$384,$A87,Artikelstamm!$U$3:$U$384)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$385,$A87,Artikelstamm!$U$3:$U$385)</f>
         <v/>
       </c>
     </row>
@@ -49240,11 +49363,11 @@
         </is>
       </c>
       <c r="B92" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$384,$A92)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$385,$A92)</f>
         <v/>
       </c>
       <c r="C92" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$384=$A92)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$385=$A92)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
     </row>
@@ -49255,11 +49378,11 @@
         </is>
       </c>
       <c r="B93" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$384,$A93)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$385,$A93)</f>
         <v/>
       </c>
       <c r="C93" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$384=$A93)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$385=$A93)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
     </row>
@@ -49270,11 +49393,11 @@
         </is>
       </c>
       <c r="B94" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$384,$A94)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$385,$A94)</f>
         <v/>
       </c>
       <c r="C94" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$384=$A94)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$385=$A94)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
     </row>
@@ -49285,11 +49408,11 @@
         </is>
       </c>
       <c r="B95" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$384,$A95)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$385,$A95)</f>
         <v/>
       </c>
       <c r="C95" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$384=$A95)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$385=$A95)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
     </row>
@@ -49300,11 +49423,11 @@
         </is>
       </c>
       <c r="B96" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$384,$A96)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$385,$A96)</f>
         <v/>
       </c>
       <c r="C96" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$384=$A96)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$385=$A96)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
     </row>
@@ -49315,11 +49438,11 @@
         </is>
       </c>
       <c r="B97" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$384,$A97)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$385,$A97)</f>
         <v/>
       </c>
       <c r="C97" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$384=$A97)*Artikelstamm!$K$3:$K$384*Artikelstamm!$AE$3:$AE$384)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$385=$A97)*Artikelstamm!$K$3:$K$385*Artikelstamm!$AE$3:$AE$385)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
BE10 vervollstaendigt: vier alte Positionen zurueck in den Katalog
BE10-01 Pendelleuchte: 4 einzelne Leuchten, von der Nutzerin bestaetigt;
offener Punkt geschlossen.

Vier Zeilen, die beim Umzug auf das Raumschema liegen geblieben waren,
haben ihre Raumnummer bekommen und sind wieder aktiv:
  K-038 -> BE10-09  Konsolentisch schwarz mit Glasablagen   60 EUR
  K-041 -> BE10-10  Kommode Holz, antik                    120 EUR
                    (linke Tuer schliesst nicht mehr - steht in der
                     Beschreibung)
  K-045 -> BE10-11  Buerodrehstuhl weiss                    60 EUR
  K-046 -> BE10-12  Aktenschrank weiss, 2 Stueck            90 EUR

K-039 Kinderfahrzeug Kuh bleibt auf entfaellt.

Datenbasis 392 Positionen / 338 aktiv, pruefen.py 0 Fehler.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011yyfqhuiWGsaNy38oaNoGo
</commit_message>
<xml_diff>
--- a/ausgabe/01_Artikelstamm_kikripp.xlsx
+++ b/ausgabe/01_Artikelstamm_kikripp.xlsx
@@ -4514,14 +4514,10 @@
       <c r="AL28" s="19" t="n"/>
       <c r="AM28" s="16" t="inlineStr">
         <is>
-          <t>4 Leuchten laut Erfassungsblatt. Auf dem Foto ist eine davon zu sehen.</t>
-        </is>
-      </c>
-      <c r="AN28" s="22" t="inlineStr">
-        <is>
-          <t>OFFEN: Stueckzahl pruefen. Auf dem Erfassungsblatt ist die gedruckte 1 durchgestrichen und 4 eingetragen. Auf Foto F-021 haengt eine Leuchte aus vier Ringen an einem Baldachin - moeglich, dass die 4 die Ringe meint und nicht vier Leuchten. Bei 450 EUR je Stueck geht es um 1.350 EUR Unterschied.</t>
-        </is>
-      </c>
+          <t>4 Leuchten. Auf dem Foto ist eine davon zu sehen.</t>
+        </is>
+      </c>
+      <c r="AN28" s="22" t="n"/>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="15" t="inlineStr">
@@ -8414,10 +8410,14 @@
     <row r="61" ht="30" customHeight="1">
       <c r="A61" s="15" t="inlineStr">
         <is>
+          <t>BE10-09</t>
+        </is>
+      </c>
+      <c r="B61" s="15" t="inlineStr">
+        <is>
           <t>K-038</t>
         </is>
       </c>
-      <c r="B61" s="15" t="n"/>
       <c r="C61" s="15" t="n"/>
       <c r="D61" s="15" t="inlineStr">
         <is>
@@ -8426,12 +8426,12 @@
       </c>
       <c r="E61" s="15" t="inlineStr">
         <is>
-          <t>Konsolentisch schwarz mit Glasplatte</t>
+          <t>Konsolentisch schwarz mit Glasablagen</t>
         </is>
       </c>
       <c r="F61" s="16" t="inlineStr">
         <is>
-          <t>Metallrahmen schwarz, Glasablagen</t>
+          <t>Schmaler Konsolentisch mit schwarzem Metallrahmen und zwei Ablagen aus Glas.</t>
         </is>
       </c>
       <c r="G61" s="15" t="inlineStr">
@@ -8470,7 +8470,7 @@
       <c r="O61" s="19" t="n"/>
       <c r="P61" s="19" t="inlineStr">
         <is>
-          <t>entfällt</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="Q61" s="19" t="n"/>
@@ -8525,7 +8525,7 @@
       <c r="AL61" s="19" t="n"/>
       <c r="AM61" s="16" t="inlineStr">
         <is>
-          <t>1 Stück im Bild</t>
+          <t>1 Tisch. Auf Foto F-024 steht er im Raum.</t>
         </is>
       </c>
       <c r="AN61" s="22" t="n"/>
@@ -8652,10 +8652,14 @@
     <row r="63" ht="30" customHeight="1">
       <c r="A63" s="15" t="inlineStr">
         <is>
+          <t>BE10-10</t>
+        </is>
+      </c>
+      <c r="B63" s="15" t="inlineStr">
+        <is>
           <t>K-041</t>
         </is>
       </c>
-      <c r="B63" s="15" t="n"/>
       <c r="C63" s="15" t="n"/>
       <c r="D63" s="15" t="inlineStr">
         <is>
@@ -8669,7 +8673,7 @@
       </c>
       <c r="F63" s="16" t="inlineStr">
         <is>
-          <t>Alte Holzkommode/Sekretär, dunkel</t>
+          <t>Alte Holzkommode beziehungsweise Sekretär in dunklem Holz. Die linke Tür schließt nicht mehr; der übrige Zustand ist gut.</t>
         </is>
       </c>
       <c r="G63" s="15" t="inlineStr">
@@ -8708,7 +8712,7 @@
       <c r="O63" s="19" t="n"/>
       <c r="P63" s="19" t="inlineStr">
         <is>
-          <t>entfällt</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="Q63" s="19" t="n"/>
@@ -8763,7 +8767,7 @@
       <c r="AL63" s="19" t="n"/>
       <c r="AM63" s="16" t="inlineStr">
         <is>
-          <t>1 Stück im Bild</t>
+          <t>1 Kommode. Auf Foto F-025 steht sie im Raum.</t>
         </is>
       </c>
       <c r="AN63" s="22" t="n"/>
@@ -8890,10 +8894,14 @@
     <row r="65" ht="30" customHeight="1">
       <c r="A65" s="15" t="inlineStr">
         <is>
+          <t>BE10-11</t>
+        </is>
+      </c>
+      <c r="B65" s="15" t="inlineStr">
+        <is>
           <t>K-045</t>
         </is>
       </c>
-      <c r="B65" s="15" t="n"/>
       <c r="C65" s="15" t="n"/>
       <c r="D65" s="15" t="inlineStr">
         <is>
@@ -8907,7 +8915,7 @@
       </c>
       <c r="F65" s="16" t="inlineStr">
         <is>
-          <t>Drehstuhl auf Rollen, weiß</t>
+          <t>Bürodrehstuhl in Weiß auf fünf Rollen, Sitzhöhe verstellbar.</t>
         </is>
       </c>
       <c r="G65" s="15" t="inlineStr">
@@ -8946,7 +8954,7 @@
       <c r="O65" s="19" t="n"/>
       <c r="P65" s="19" t="inlineStr">
         <is>
-          <t>entfällt</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="Q65" s="19" t="n"/>
@@ -9001,7 +9009,7 @@
       <c r="AL65" s="19" t="n"/>
       <c r="AM65" s="16" t="inlineStr">
         <is>
-          <t>1 Stück im Bild</t>
+          <t>1 Stuhl. Auf Foto F-027 steht er im Raum.</t>
         </is>
       </c>
       <c r="AN65" s="22" t="n"/>
@@ -9009,10 +9017,14 @@
     <row r="66" ht="30" customHeight="1">
       <c r="A66" s="15" t="inlineStr">
         <is>
+          <t>BE10-12</t>
+        </is>
+      </c>
+      <c r="B66" s="15" t="inlineStr">
+        <is>
           <t>K-046</t>
         </is>
       </c>
-      <c r="B66" s="15" t="n"/>
       <c r="C66" s="15" t="n"/>
       <c r="D66" s="15" t="inlineStr">
         <is>
@@ -9026,7 +9038,7 @@
       </c>
       <c r="F66" s="16" t="inlineStr">
         <is>
-          <t>Büroschrank weiß, mit Türen</t>
+          <t>Büroschrank in Weiß mit Türen und Einlegeböden.</t>
         </is>
       </c>
       <c r="G66" s="15" t="inlineStr">
@@ -9065,7 +9077,7 @@
       <c r="O66" s="19" t="n"/>
       <c r="P66" s="19" t="inlineStr">
         <is>
-          <t>entfällt</t>
+          <t>ja</t>
         </is>
       </c>
       <c r="Q66" s="19" t="n"/>
@@ -9120,7 +9132,7 @@
       <c r="AL66" s="19" t="n"/>
       <c r="AM66" s="16" t="inlineStr">
         <is>
-          <t>2 Schränke im Bild</t>
+          <t>2 Schränke. Auf Foto F-027 stehen sie im Raum.</t>
         </is>
       </c>
       <c r="AN66" s="22" t="n"/>

</xml_diff>

<commit_message>
TE02 Dachterrasse erfasst: 12 neue Positionen
Neues Verfahren fuer die Aussenbereiche verstanden: die Etiketten kleben
wegen des Regens nicht am Artikel, sondern auf einem Streifen bzw. an der
Fensterscheibe; die Zuordnung laeuft ueber die Kurzbeschreibung auf dem
Etikett und die Erfassungsliste.

TE02-07 bis TE02-18 angelegt, Stueckzahlen und Zustaende vom
Erfassungsblatt (F-515) und den Etikettenstreifen (F-516, F-517).

Drei Punkte bleiben offen und stehen als OFFEN in der Datenbasis:
  TE02-15 rote Tische - kein Foto dabei
  TE02-16 und TE02-18 - auf dem Blatt "Stuehle" ohne den Zusatz Kinder,
          waehrend TE02-09 und TE02-13 "Kinderstuehle" heissen; unklar,
          ob zwei Groessen oder dieselbe Ware

Datenbasis 404 Positionen / 350 aktiv, pruefen.py 0 Fehler.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011yyfqhuiWGsaNy38oaNoGo
</commit_message>
<xml_diff>
--- a/ausgabe/01_Artikelstamm_kikripp.xlsx
+++ b/ausgabe/01_Artikelstamm_kikripp.xlsx
@@ -15,7 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Artikelstamm'!$A$2:$AN$394</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Artikelstamm'!$A$2:$AN$406</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1019,7 +1019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN394"/>
+  <dimension ref="A1:AN406"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -49022,8 +49022,1492 @@
       </c>
       <c r="AN394" s="22" t="n"/>
     </row>
+    <row r="395" ht="30" customHeight="1">
+      <c r="A395" s="15" t="inlineStr">
+        <is>
+          <t>TE02-07</t>
+        </is>
+      </c>
+      <c r="B395" s="15" t="n"/>
+      <c r="C395" s="15" t="n"/>
+      <c r="D395" s="15" t="inlineStr">
+        <is>
+          <t>TE02</t>
+        </is>
+      </c>
+      <c r="E395" s="15" t="inlineStr">
+        <is>
+          <t>KidKraft Kinder-Strandliege mit Sonnendach</t>
+        </is>
+      </c>
+      <c r="F395" s="16" t="inlineStr">
+        <is>
+          <t>Liege für Kinder aus lasiertem Holz mit Lattenrost, hochgestellter Rückenlehne, Sonnendach aus grauem Stoff und einer Mittelkonsole mit zwei Bechereinsätzen. Das Holz ist wettergrau, der Stoff verschmutzt.</t>
+        </is>
+      </c>
+      <c r="G395" s="15" t="inlineStr">
+        <is>
+          <t>Garten</t>
+        </is>
+      </c>
+      <c r="H395" s="15" t="inlineStr">
+        <is>
+          <t>Dachterrasse</t>
+        </is>
+      </c>
+      <c r="I395" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J395" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K395" s="17" t="n"/>
+      <c r="L395" s="18">
+        <f>J395-IF(K395="",0,K395)</f>
+        <v/>
+      </c>
+      <c r="M395" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N395" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O395" s="19" t="n"/>
+      <c r="P395" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q395" s="19" t="n"/>
+      <c r="R395" s="20" t="n"/>
+      <c r="S395" s="20" t="n">
+        <v>60</v>
+      </c>
+      <c r="T395" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U395" s="21">
+        <f>L395*S395</f>
+        <v/>
+      </c>
+      <c r="V395" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W395" s="15" t="inlineStr">
+        <is>
+          <t>F-504</t>
+        </is>
+      </c>
+      <c r="X395" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y395" s="19" t="n"/>
+      <c r="Z395" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA395" s="19" t="inlineStr">
+        <is>
+          <t>KidKraft</t>
+        </is>
+      </c>
+      <c r="AB395" s="19" t="n"/>
+      <c r="AC395" s="19" t="n"/>
+      <c r="AD395" s="19" t="n"/>
+      <c r="AE395" s="20" t="n"/>
+      <c r="AF395" s="21">
+        <f>IF(K395="","",K395*AE395)</f>
+        <v/>
+      </c>
+      <c r="AG395" s="19" t="n"/>
+      <c r="AH395" s="19" t="n"/>
+      <c r="AI395" s="19" t="n"/>
+      <c r="AJ395" s="19" t="n"/>
+      <c r="AK395" s="19" t="n"/>
+      <c r="AL395" s="19" t="n"/>
+      <c r="AM395" s="16" t="inlineStr">
+        <is>
+          <t>1 Liege einschließlich Sonnendach und Mittelkonsole.</t>
+        </is>
+      </c>
+      <c r="AN395" s="22" t="n"/>
+    </row>
+    <row r="396" ht="30" customHeight="1">
+      <c r="A396" s="15" t="inlineStr">
+        <is>
+          <t>TE02-08</t>
+        </is>
+      </c>
+      <c r="B396" s="15" t="n"/>
+      <c r="C396" s="15" t="n"/>
+      <c r="D396" s="15" t="inlineStr">
+        <is>
+          <t>TE02</t>
+        </is>
+      </c>
+      <c r="E396" s="15" t="inlineStr">
+        <is>
+          <t>IKEA Skarpö Sessel weiß</t>
+        </is>
+      </c>
+      <c r="F396" s="16" t="inlineStr">
+        <is>
+          <t>Gartensessel IKEA Skarpö, Entwurf Magnus Elebäck: weißer Kunststoff in einem Stück, stapelbar. Etikett an der Unterseite: Skarpö, 702.341.85, 18809. Sitzflächen verschmutzt und bewittert.</t>
+        </is>
+      </c>
+      <c r="G396" s="15" t="inlineStr">
+        <is>
+          <t>Garten</t>
+        </is>
+      </c>
+      <c r="H396" s="15" t="inlineStr">
+        <is>
+          <t>Dachterrasse</t>
+        </is>
+      </c>
+      <c r="I396" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J396" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="K396" s="17" t="n"/>
+      <c r="L396" s="18">
+        <f>J396-IF(K396="",0,K396)</f>
+        <v/>
+      </c>
+      <c r="M396" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N396" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O396" s="19" t="n"/>
+      <c r="P396" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q396" s="19" t="n"/>
+      <c r="R396" s="20" t="n"/>
+      <c r="S396" s="20" t="n">
+        <v>25</v>
+      </c>
+      <c r="T396" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U396" s="21">
+        <f>L396*S396</f>
+        <v/>
+      </c>
+      <c r="V396" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W396" s="15" t="inlineStr">
+        <is>
+          <t>F-506</t>
+        </is>
+      </c>
+      <c r="X396" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y396" s="19" t="n"/>
+      <c r="Z396" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA396" s="19" t="inlineStr">
+        <is>
+          <t>IKEA</t>
+        </is>
+      </c>
+      <c r="AB396" s="19" t="n"/>
+      <c r="AC396" s="19" t="n"/>
+      <c r="AD396" s="19" t="n"/>
+      <c r="AE396" s="20" t="n"/>
+      <c r="AF396" s="21">
+        <f>IF(K396="","",K396*AE396)</f>
+        <v/>
+      </c>
+      <c r="AG396" s="19" t="n"/>
+      <c r="AH396" s="19" t="n"/>
+      <c r="AI396" s="19" t="n"/>
+      <c r="AJ396" s="19" t="n"/>
+      <c r="AK396" s="19" t="n"/>
+      <c r="AL396" s="19" t="n"/>
+      <c r="AM396" s="16" t="inlineStr">
+        <is>
+          <t>4 Sessel – abgebildet ist einer davon. Das Etikett ist auf Foto F-505 zu sehen.</t>
+        </is>
+      </c>
+      <c r="AN396" s="22" t="n"/>
+    </row>
+    <row r="397" ht="30" customHeight="1">
+      <c r="A397" s="15" t="inlineStr">
+        <is>
+          <t>TE02-09</t>
+        </is>
+      </c>
+      <c r="B397" s="15" t="n"/>
+      <c r="C397" s="15" t="n"/>
+      <c r="D397" s="15" t="inlineStr">
+        <is>
+          <t>TE02</t>
+        </is>
+      </c>
+      <c r="E397" s="15" t="inlineStr">
+        <is>
+          <t>IKEA Mammut Kinderstuhl rot</t>
+        </is>
+      </c>
+      <c r="F397" s="16" t="inlineStr">
+        <is>
+          <t>Kinderstuhl IKEA Mammut aus rotem Kunststoff mit runden Beinen und breiter Rückenlehne, für drinnen und draußen.</t>
+        </is>
+      </c>
+      <c r="G397" s="15" t="inlineStr">
+        <is>
+          <t>Garten</t>
+        </is>
+      </c>
+      <c r="H397" s="15" t="inlineStr">
+        <is>
+          <t>Dachterrasse</t>
+        </is>
+      </c>
+      <c r="I397" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J397" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="K397" s="17" t="n"/>
+      <c r="L397" s="18">
+        <f>J397-IF(K397="",0,K397)</f>
+        <v/>
+      </c>
+      <c r="M397" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N397" s="15" t="inlineStr">
+        <is>
+          <t>gut</t>
+        </is>
+      </c>
+      <c r="O397" s="19" t="n"/>
+      <c r="P397" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q397" s="19" t="n"/>
+      <c r="R397" s="20" t="n"/>
+      <c r="S397" s="20" t="n">
+        <v>12</v>
+      </c>
+      <c r="T397" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U397" s="21">
+        <f>L397*S397</f>
+        <v/>
+      </c>
+      <c r="V397" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W397" s="15" t="inlineStr">
+        <is>
+          <t>F-507</t>
+        </is>
+      </c>
+      <c r="X397" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y397" s="19" t="n"/>
+      <c r="Z397" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA397" s="19" t="inlineStr">
+        <is>
+          <t>IKEA</t>
+        </is>
+      </c>
+      <c r="AB397" s="19" t="n"/>
+      <c r="AC397" s="19" t="n"/>
+      <c r="AD397" s="19" t="n"/>
+      <c r="AE397" s="20" t="n"/>
+      <c r="AF397" s="21">
+        <f>IF(K397="","",K397*AE397)</f>
+        <v/>
+      </c>
+      <c r="AG397" s="19" t="n"/>
+      <c r="AH397" s="19" t="n"/>
+      <c r="AI397" s="19" t="n"/>
+      <c r="AJ397" s="19" t="n"/>
+      <c r="AK397" s="19" t="n"/>
+      <c r="AL397" s="19" t="n"/>
+      <c r="AM397" s="16" t="inlineStr">
+        <is>
+          <t>10 Stühle – abgebildet ist einer davon.</t>
+        </is>
+      </c>
+      <c r="AN397" s="22" t="n"/>
+    </row>
+    <row r="398" ht="30" customHeight="1">
+      <c r="A398" s="15" t="inlineStr">
+        <is>
+          <t>TE02-10</t>
+        </is>
+      </c>
+      <c r="B398" s="15" t="n"/>
+      <c r="C398" s="15" t="n"/>
+      <c r="D398" s="15" t="inlineStr">
+        <is>
+          <t>TE02</t>
+        </is>
+      </c>
+      <c r="E398" s="15" t="inlineStr">
+        <is>
+          <t>IKEA Mammut Kinderstuhl grün</t>
+        </is>
+      </c>
+      <c r="F398" s="16" t="inlineStr">
+        <is>
+          <t>Kinderstuhl IKEA Mammut aus grünem Kunststoff. Die Stühle standen lange im Freien: Farbe ausgeblichen, Oberflächen stumpf und stark verkratzt.</t>
+        </is>
+      </c>
+      <c r="G398" s="15" t="inlineStr">
+        <is>
+          <t>Garten</t>
+        </is>
+      </c>
+      <c r="H398" s="15" t="inlineStr">
+        <is>
+          <t>Dachterrasse</t>
+        </is>
+      </c>
+      <c r="I398" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J398" s="17" t="n">
+        <v>15</v>
+      </c>
+      <c r="K398" s="17" t="n"/>
+      <c r="L398" s="18">
+        <f>J398-IF(K398="",0,K398)</f>
+        <v/>
+      </c>
+      <c r="M398" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N398" s="15" t="inlineStr">
+        <is>
+          <t>stark gebraucht</t>
+        </is>
+      </c>
+      <c r="O398" s="19" t="n"/>
+      <c r="P398" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q398" s="19" t="n"/>
+      <c r="R398" s="20" t="n"/>
+      <c r="S398" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="T398" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U398" s="21">
+        <f>L398*S398</f>
+        <v/>
+      </c>
+      <c r="V398" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W398" s="15" t="inlineStr">
+        <is>
+          <t>F-508</t>
+        </is>
+      </c>
+      <c r="X398" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y398" s="19" t="n"/>
+      <c r="Z398" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA398" s="19" t="inlineStr">
+        <is>
+          <t>IKEA</t>
+        </is>
+      </c>
+      <c r="AB398" s="19" t="n"/>
+      <c r="AC398" s="19" t="n"/>
+      <c r="AD398" s="19" t="n"/>
+      <c r="AE398" s="20" t="n"/>
+      <c r="AF398" s="21">
+        <f>IF(K398="","",K398*AE398)</f>
+        <v/>
+      </c>
+      <c r="AG398" s="19" t="n"/>
+      <c r="AH398" s="19" t="n"/>
+      <c r="AI398" s="19" t="n"/>
+      <c r="AJ398" s="19" t="n"/>
+      <c r="AK398" s="19" t="n"/>
+      <c r="AL398" s="19" t="n"/>
+      <c r="AM398" s="16" t="inlineStr">
+        <is>
+          <t>15 Stühle – abgebildet ist einer davon. Auf dem Erfassungsblatt als stark verwittert vermerkt.</t>
+        </is>
+      </c>
+      <c r="AN398" s="22" t="n"/>
+    </row>
+    <row r="399" ht="30" customHeight="1">
+      <c r="A399" s="15" t="inlineStr">
+        <is>
+          <t>TE02-11</t>
+        </is>
+      </c>
+      <c r="B399" s="15" t="n"/>
+      <c r="C399" s="15" t="n"/>
+      <c r="D399" s="15" t="inlineStr">
+        <is>
+          <t>TE02</t>
+        </is>
+      </c>
+      <c r="E399" s="15" t="inlineStr">
+        <is>
+          <t>IKEA Mammut Kindertisch grün, rund</t>
+        </is>
+      </c>
+      <c r="F399" s="16" t="inlineStr">
+        <is>
+          <t>Runder Kindertisch IKEA Mammut aus grünem Kunststoff auf drei konischen Beinen.</t>
+        </is>
+      </c>
+      <c r="G399" s="15" t="inlineStr">
+        <is>
+          <t>Garten</t>
+        </is>
+      </c>
+      <c r="H399" s="15" t="inlineStr">
+        <is>
+          <t>Dachterrasse</t>
+        </is>
+      </c>
+      <c r="I399" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J399" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K399" s="17" t="n"/>
+      <c r="L399" s="18">
+        <f>J399-IF(K399="",0,K399)</f>
+        <v/>
+      </c>
+      <c r="M399" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N399" s="15" t="inlineStr">
+        <is>
+          <t>stark gebraucht</t>
+        </is>
+      </c>
+      <c r="O399" s="19" t="n"/>
+      <c r="P399" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q399" s="19" t="n"/>
+      <c r="R399" s="20" t="n"/>
+      <c r="S399" s="20" t="n">
+        <v>15</v>
+      </c>
+      <c r="T399" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U399" s="21">
+        <f>L399*S399</f>
+        <v/>
+      </c>
+      <c r="V399" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W399" s="15" t="inlineStr">
+        <is>
+          <t>F-509</t>
+        </is>
+      </c>
+      <c r="X399" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y399" s="19" t="n"/>
+      <c r="Z399" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA399" s="19" t="inlineStr">
+        <is>
+          <t>IKEA</t>
+        </is>
+      </c>
+      <c r="AB399" s="19" t="n"/>
+      <c r="AC399" s="19" t="n"/>
+      <c r="AD399" s="19" t="n"/>
+      <c r="AE399" s="20" t="n"/>
+      <c r="AF399" s="21">
+        <f>IF(K399="","",K399*AE399)</f>
+        <v/>
+      </c>
+      <c r="AG399" s="19" t="n"/>
+      <c r="AH399" s="19" t="n"/>
+      <c r="AI399" s="19" t="n"/>
+      <c r="AJ399" s="19" t="n"/>
+      <c r="AK399" s="19" t="n"/>
+      <c r="AL399" s="19" t="n"/>
+      <c r="AM399" s="16" t="inlineStr">
+        <is>
+          <t>2 Tische – abgebildet ist einer davon.</t>
+        </is>
+      </c>
+      <c r="AN399" s="22" t="n"/>
+    </row>
+    <row r="400" ht="30" customHeight="1">
+      <c r="A400" s="15" t="inlineStr">
+        <is>
+          <t>TE02-12</t>
+        </is>
+      </c>
+      <c r="B400" s="15" t="n"/>
+      <c r="C400" s="15" t="n"/>
+      <c r="D400" s="15" t="inlineStr">
+        <is>
+          <t>TE02</t>
+        </is>
+      </c>
+      <c r="E400" s="15" t="inlineStr">
+        <is>
+          <t>IKEA Mammut Kindertisch grün, rund, stark verwittert</t>
+        </is>
+      </c>
+      <c r="F400" s="16" t="inlineStr">
+        <is>
+          <t>Runder Kindertisch IKEA Mammut aus grünem Kunststoff. Die Platte ist vom Wetter ausgebleicht und großflächig grau verfärbt.</t>
+        </is>
+      </c>
+      <c r="G400" s="15" t="inlineStr">
+        <is>
+          <t>Garten</t>
+        </is>
+      </c>
+      <c r="H400" s="15" t="inlineStr">
+        <is>
+          <t>Dachterrasse</t>
+        </is>
+      </c>
+      <c r="I400" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J400" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K400" s="17" t="n"/>
+      <c r="L400" s="18">
+        <f>J400-IF(K400="",0,K400)</f>
+        <v/>
+      </c>
+      <c r="M400" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N400" s="15" t="inlineStr">
+        <is>
+          <t>stark gebraucht</t>
+        </is>
+      </c>
+      <c r="O400" s="19" t="n"/>
+      <c r="P400" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q400" s="19" t="n"/>
+      <c r="R400" s="20" t="n"/>
+      <c r="S400" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="T400" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U400" s="21">
+        <f>L400*S400</f>
+        <v/>
+      </c>
+      <c r="V400" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W400" s="15" t="inlineStr">
+        <is>
+          <t>F-510</t>
+        </is>
+      </c>
+      <c r="X400" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y400" s="19" t="n"/>
+      <c r="Z400" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA400" s="19" t="inlineStr">
+        <is>
+          <t>IKEA</t>
+        </is>
+      </c>
+      <c r="AB400" s="19" t="n"/>
+      <c r="AC400" s="19" t="n"/>
+      <c r="AD400" s="19" t="n"/>
+      <c r="AE400" s="20" t="n"/>
+      <c r="AF400" s="21">
+        <f>IF(K400="","",K400*AE400)</f>
+        <v/>
+      </c>
+      <c r="AG400" s="19" t="n"/>
+      <c r="AH400" s="19" t="n"/>
+      <c r="AI400" s="19" t="n"/>
+      <c r="AJ400" s="19" t="n"/>
+      <c r="AK400" s="19" t="n"/>
+      <c r="AL400" s="19" t="n"/>
+      <c r="AM400" s="16" t="inlineStr">
+        <is>
+          <t>2 Tische – abgebildet ist einer davon. Weniger stark bewitterte Tische gleicher Bauart stehen unter TE02-11.</t>
+        </is>
+      </c>
+      <c r="AN400" s="22" t="n"/>
+    </row>
+    <row r="401" ht="30" customHeight="1">
+      <c r="A401" s="15" t="inlineStr">
+        <is>
+          <t>TE02-13</t>
+        </is>
+      </c>
+      <c r="B401" s="15" t="n"/>
+      <c r="C401" s="15" t="n"/>
+      <c r="D401" s="15" t="inlineStr">
+        <is>
+          <t>TE02</t>
+        </is>
+      </c>
+      <c r="E401" s="15" t="inlineStr">
+        <is>
+          <t>IKEA Mammut Kinderstuhl weiß</t>
+        </is>
+      </c>
+      <c r="F401" s="16" t="inlineStr">
+        <is>
+          <t>Kinderstuhl IKEA Mammut aus weißem Kunststoff mit runden Beinen und breiter Rückenlehne.</t>
+        </is>
+      </c>
+      <c r="G401" s="15" t="inlineStr">
+        <is>
+          <t>Garten</t>
+        </is>
+      </c>
+      <c r="H401" s="15" t="inlineStr">
+        <is>
+          <t>Dachterrasse</t>
+        </is>
+      </c>
+      <c r="I401" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J401" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="K401" s="17" t="n"/>
+      <c r="L401" s="18">
+        <f>J401-IF(K401="",0,K401)</f>
+        <v/>
+      </c>
+      <c r="M401" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N401" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O401" s="19" t="n"/>
+      <c r="P401" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q401" s="19" t="n"/>
+      <c r="R401" s="20" t="n"/>
+      <c r="S401" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="T401" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U401" s="21">
+        <f>L401*S401</f>
+        <v/>
+      </c>
+      <c r="V401" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W401" s="15" t="inlineStr">
+        <is>
+          <t>F-511</t>
+        </is>
+      </c>
+      <c r="X401" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y401" s="19" t="n"/>
+      <c r="Z401" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA401" s="19" t="inlineStr">
+        <is>
+          <t>IKEA</t>
+        </is>
+      </c>
+      <c r="AB401" s="19" t="n"/>
+      <c r="AC401" s="19" t="n"/>
+      <c r="AD401" s="19" t="n"/>
+      <c r="AE401" s="20" t="n"/>
+      <c r="AF401" s="21">
+        <f>IF(K401="","",K401*AE401)</f>
+        <v/>
+      </c>
+      <c r="AG401" s="19" t="n"/>
+      <c r="AH401" s="19" t="n"/>
+      <c r="AI401" s="19" t="n"/>
+      <c r="AJ401" s="19" t="n"/>
+      <c r="AK401" s="19" t="n"/>
+      <c r="AL401" s="19" t="n"/>
+      <c r="AM401" s="16" t="inlineStr">
+        <is>
+          <t>5 Stühle – abgebildet ist einer davon.</t>
+        </is>
+      </c>
+      <c r="AN401" s="22" t="n"/>
+    </row>
+    <row r="402" ht="30" customHeight="1">
+      <c r="A402" s="15" t="inlineStr">
+        <is>
+          <t>TE02-14</t>
+        </is>
+      </c>
+      <c r="B402" s="15" t="n"/>
+      <c r="C402" s="15" t="n"/>
+      <c r="D402" s="15" t="inlineStr">
+        <is>
+          <t>TE02</t>
+        </is>
+      </c>
+      <c r="E402" s="15" t="inlineStr">
+        <is>
+          <t>IKEA Mammut Kinderstuhl rosa</t>
+        </is>
+      </c>
+      <c r="F402" s="16" t="inlineStr">
+        <is>
+          <t>Kinderstuhl IKEA Mammut aus rosa Kunststoff, Farbe an Sitz und Lehne ausgeblichen.</t>
+        </is>
+      </c>
+      <c r="G402" s="15" t="inlineStr">
+        <is>
+          <t>Garten</t>
+        </is>
+      </c>
+      <c r="H402" s="15" t="inlineStr">
+        <is>
+          <t>Dachterrasse</t>
+        </is>
+      </c>
+      <c r="I402" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J402" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K402" s="17" t="n"/>
+      <c r="L402" s="18">
+        <f>J402-IF(K402="",0,K402)</f>
+        <v/>
+      </c>
+      <c r="M402" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N402" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O402" s="19" t="n"/>
+      <c r="P402" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q402" s="19" t="n"/>
+      <c r="R402" s="20" t="n"/>
+      <c r="S402" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="T402" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U402" s="21">
+        <f>L402*S402</f>
+        <v/>
+      </c>
+      <c r="V402" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W402" s="15" t="inlineStr">
+        <is>
+          <t>F-512</t>
+        </is>
+      </c>
+      <c r="X402" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y402" s="19" t="n"/>
+      <c r="Z402" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA402" s="19" t="inlineStr">
+        <is>
+          <t>IKEA</t>
+        </is>
+      </c>
+      <c r="AB402" s="19" t="n"/>
+      <c r="AC402" s="19" t="n"/>
+      <c r="AD402" s="19" t="n"/>
+      <c r="AE402" s="20" t="n"/>
+      <c r="AF402" s="21">
+        <f>IF(K402="","",K402*AE402)</f>
+        <v/>
+      </c>
+      <c r="AG402" s="19" t="n"/>
+      <c r="AH402" s="19" t="n"/>
+      <c r="AI402" s="19" t="n"/>
+      <c r="AJ402" s="19" t="n"/>
+      <c r="AK402" s="19" t="n"/>
+      <c r="AL402" s="19" t="n"/>
+      <c r="AM402" s="16" t="inlineStr">
+        <is>
+          <t>1 Stuhl.</t>
+        </is>
+      </c>
+      <c r="AN402" s="22" t="n"/>
+    </row>
+    <row r="403" ht="30" customHeight="1">
+      <c r="A403" s="15" t="inlineStr">
+        <is>
+          <t>TE02-15</t>
+        </is>
+      </c>
+      <c r="B403" s="15" t="n"/>
+      <c r="C403" s="15" t="n"/>
+      <c r="D403" s="15" t="inlineStr">
+        <is>
+          <t>TE02</t>
+        </is>
+      </c>
+      <c r="E403" s="15" t="inlineStr">
+        <is>
+          <t>IKEA Mammut Kindertisch rot</t>
+        </is>
+      </c>
+      <c r="F403" s="16" t="inlineStr">
+        <is>
+          <t>Kindertisch IKEA Mammut aus rotem Kunststoff auf konischen Beinen.</t>
+        </is>
+      </c>
+      <c r="G403" s="15" t="inlineStr">
+        <is>
+          <t>Garten</t>
+        </is>
+      </c>
+      <c r="H403" s="15" t="inlineStr">
+        <is>
+          <t>Dachterrasse</t>
+        </is>
+      </c>
+      <c r="I403" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J403" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="K403" s="17" t="n"/>
+      <c r="L403" s="18">
+        <f>J403-IF(K403="",0,K403)</f>
+        <v/>
+      </c>
+      <c r="M403" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N403" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O403" s="19" t="n"/>
+      <c r="P403" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q403" s="19" t="n"/>
+      <c r="R403" s="20" t="n"/>
+      <c r="S403" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="T403" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U403" s="21">
+        <f>L403*S403</f>
+        <v/>
+      </c>
+      <c r="V403" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W403" s="15" t="n"/>
+      <c r="X403" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y403" s="19" t="n"/>
+      <c r="Z403" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA403" s="19" t="inlineStr">
+        <is>
+          <t>IKEA</t>
+        </is>
+      </c>
+      <c r="AB403" s="19" t="n"/>
+      <c r="AC403" s="19" t="n"/>
+      <c r="AD403" s="19" t="n"/>
+      <c r="AE403" s="20" t="n"/>
+      <c r="AF403" s="21">
+        <f>IF(K403="","",K403*AE403)</f>
+        <v/>
+      </c>
+      <c r="AG403" s="19" t="n"/>
+      <c r="AH403" s="19" t="n"/>
+      <c r="AI403" s="19" t="n"/>
+      <c r="AJ403" s="19" t="n"/>
+      <c r="AK403" s="19" t="n"/>
+      <c r="AL403" s="19" t="n"/>
+      <c r="AM403" s="16" t="inlineStr">
+        <is>
+          <t>3 Tische.</t>
+        </is>
+      </c>
+      <c r="AN403" s="22" t="inlineStr">
+        <is>
+          <t>OFFEN: Zu dieser Position fehlt ein Foto - von den roten Tischen ist keines dabei.</t>
+        </is>
+      </c>
+    </row>
+    <row r="404" ht="30" customHeight="1">
+      <c r="A404" s="15" t="inlineStr">
+        <is>
+          <t>TE02-16</t>
+        </is>
+      </c>
+      <c r="B404" s="15" t="n"/>
+      <c r="C404" s="15" t="n"/>
+      <c r="D404" s="15" t="inlineStr">
+        <is>
+          <t>TE02</t>
+        </is>
+      </c>
+      <c r="E404" s="15" t="inlineStr">
+        <is>
+          <t>IKEA Mammut Stuhl rot</t>
+        </is>
+      </c>
+      <c r="F404" s="16" t="inlineStr">
+        <is>
+          <t>Stuhl IKEA Mammut aus rotem Kunststoff mit runden Beinen und breiter Rückenlehne.</t>
+        </is>
+      </c>
+      <c r="G404" s="15" t="inlineStr">
+        <is>
+          <t>Garten</t>
+        </is>
+      </c>
+      <c r="H404" s="15" t="inlineStr">
+        <is>
+          <t>Dachterrasse</t>
+        </is>
+      </c>
+      <c r="I404" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J404" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="K404" s="17" t="n"/>
+      <c r="L404" s="18">
+        <f>J404-IF(K404="",0,K404)</f>
+        <v/>
+      </c>
+      <c r="M404" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N404" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O404" s="19" t="n"/>
+      <c r="P404" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q404" s="19" t="n"/>
+      <c r="R404" s="20" t="n"/>
+      <c r="S404" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="T404" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U404" s="21">
+        <f>L404*S404</f>
+        <v/>
+      </c>
+      <c r="V404" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W404" s="15" t="inlineStr">
+        <is>
+          <t>F-514</t>
+        </is>
+      </c>
+      <c r="X404" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y404" s="19" t="n"/>
+      <c r="Z404" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA404" s="19" t="inlineStr">
+        <is>
+          <t>IKEA</t>
+        </is>
+      </c>
+      <c r="AB404" s="19" t="n"/>
+      <c r="AC404" s="19" t="n"/>
+      <c r="AD404" s="19" t="n"/>
+      <c r="AE404" s="20" t="n"/>
+      <c r="AF404" s="21">
+        <f>IF(K404="","",K404*AE404)</f>
+        <v/>
+      </c>
+      <c r="AG404" s="19" t="n"/>
+      <c r="AH404" s="19" t="n"/>
+      <c r="AI404" s="19" t="n"/>
+      <c r="AJ404" s="19" t="n"/>
+      <c r="AK404" s="19" t="n"/>
+      <c r="AL404" s="19" t="n"/>
+      <c r="AM404" s="16" t="inlineStr">
+        <is>
+          <t>10 Stühle. Auf dem Foto sind zwei davon gestapelt zu sehen.</t>
+        </is>
+      </c>
+      <c r="AN404" s="22" t="inlineStr">
+        <is>
+          <t>OFFEN: Auf dem Erfassungsblatt steht hier "IKEA Stuehle rot" ohne den Zusatz Kinder, bei TE02-09 dagegen "Kinderstuehle rot". Klaeren, ob das zwei verschiedene Groessen sind oder ob beide Positionen zusammengehoeren.</t>
+        </is>
+      </c>
+    </row>
+    <row r="405" ht="30" customHeight="1">
+      <c r="A405" s="15" t="inlineStr">
+        <is>
+          <t>TE02-17</t>
+        </is>
+      </c>
+      <c r="B405" s="15" t="n"/>
+      <c r="C405" s="15" t="n"/>
+      <c r="D405" s="15" t="inlineStr">
+        <is>
+          <t>TE02</t>
+        </is>
+      </c>
+      <c r="E405" s="15" t="inlineStr">
+        <is>
+          <t>IKEA Mammut Kindertisch weiß</t>
+        </is>
+      </c>
+      <c r="F405" s="16" t="inlineStr">
+        <is>
+          <t>Rechteckiger Kindertisch IKEA Mammut aus weißem Kunststoff auf konischen Beinen. Die Platte ist fleckig und vom Wetter gezeichnet.</t>
+        </is>
+      </c>
+      <c r="G405" s="15" t="inlineStr">
+        <is>
+          <t>Garten</t>
+        </is>
+      </c>
+      <c r="H405" s="15" t="inlineStr">
+        <is>
+          <t>Dachterrasse</t>
+        </is>
+      </c>
+      <c r="I405" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J405" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="K405" s="17" t="n"/>
+      <c r="L405" s="18">
+        <f>J405-IF(K405="",0,K405)</f>
+        <v/>
+      </c>
+      <c r="M405" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N405" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O405" s="19" t="n"/>
+      <c r="P405" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q405" s="19" t="n"/>
+      <c r="R405" s="20" t="n"/>
+      <c r="S405" s="20" t="n">
+        <v>20</v>
+      </c>
+      <c r="T405" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U405" s="21">
+        <f>L405*S405</f>
+        <v/>
+      </c>
+      <c r="V405" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W405" s="15" t="inlineStr">
+        <is>
+          <t>F-513</t>
+        </is>
+      </c>
+      <c r="X405" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y405" s="19" t="n"/>
+      <c r="Z405" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA405" s="19" t="inlineStr">
+        <is>
+          <t>IKEA</t>
+        </is>
+      </c>
+      <c r="AB405" s="19" t="n"/>
+      <c r="AC405" s="19" t="n"/>
+      <c r="AD405" s="19" t="n"/>
+      <c r="AE405" s="20" t="n"/>
+      <c r="AF405" s="21">
+        <f>IF(K405="","",K405*AE405)</f>
+        <v/>
+      </c>
+      <c r="AG405" s="19" t="n"/>
+      <c r="AH405" s="19" t="n"/>
+      <c r="AI405" s="19" t="n"/>
+      <c r="AJ405" s="19" t="n"/>
+      <c r="AK405" s="19" t="n"/>
+      <c r="AL405" s="19" t="n"/>
+      <c r="AM405" s="16" t="inlineStr">
+        <is>
+          <t>3 Tische – abgebildet ist einer davon.</t>
+        </is>
+      </c>
+      <c r="AN405" s="22" t="n"/>
+    </row>
+    <row r="406" ht="30" customHeight="1">
+      <c r="A406" s="15" t="inlineStr">
+        <is>
+          <t>TE02-18</t>
+        </is>
+      </c>
+      <c r="B406" s="15" t="n"/>
+      <c r="C406" s="15" t="n"/>
+      <c r="D406" s="15" t="inlineStr">
+        <is>
+          <t>TE02</t>
+        </is>
+      </c>
+      <c r="E406" s="15" t="inlineStr">
+        <is>
+          <t>IKEA Mammut Stuhl weiß</t>
+        </is>
+      </c>
+      <c r="F406" s="16" t="inlineStr">
+        <is>
+          <t>Stuhl IKEA Mammut aus weißem Kunststoff mit runden Beinen und breiter Rückenlehne.</t>
+        </is>
+      </c>
+      <c r="G406" s="15" t="inlineStr">
+        <is>
+          <t>Garten</t>
+        </is>
+      </c>
+      <c r="H406" s="15" t="inlineStr">
+        <is>
+          <t>Dachterrasse</t>
+        </is>
+      </c>
+      <c r="I406" s="15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="J406" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="K406" s="17" t="n"/>
+      <c r="L406" s="18">
+        <f>J406-IF(K406="",0,K406)</f>
+        <v/>
+      </c>
+      <c r="M406" s="15" t="inlineStr">
+        <is>
+          <t>Stück</t>
+        </is>
+      </c>
+      <c r="N406" s="15" t="inlineStr">
+        <is>
+          <t>gebraucht</t>
+        </is>
+      </c>
+      <c r="O406" s="19" t="n"/>
+      <c r="P406" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Q406" s="19" t="n"/>
+      <c r="R406" s="20" t="n"/>
+      <c r="S406" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="T406" s="19" t="inlineStr">
+        <is>
+          <t>VHB</t>
+        </is>
+      </c>
+      <c r="U406" s="21">
+        <f>L406*S406</f>
+        <v/>
+      </c>
+      <c r="V406" s="15" t="inlineStr">
+        <is>
+          <t>nur Abholung</t>
+        </is>
+      </c>
+      <c r="W406" s="15" t="inlineStr">
+        <is>
+          <t>F-511</t>
+        </is>
+      </c>
+      <c r="X406" s="19" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="Y406" s="19" t="n"/>
+      <c r="Z406" s="19" t="inlineStr">
+        <is>
+          <t>verfügbar</t>
+        </is>
+      </c>
+      <c r="AA406" s="19" t="inlineStr">
+        <is>
+          <t>IKEA</t>
+        </is>
+      </c>
+      <c r="AB406" s="19" t="n"/>
+      <c r="AC406" s="19" t="n"/>
+      <c r="AD406" s="19" t="n"/>
+      <c r="AE406" s="20" t="n"/>
+      <c r="AF406" s="21">
+        <f>IF(K406="","",K406*AE406)</f>
+        <v/>
+      </c>
+      <c r="AG406" s="19" t="n"/>
+      <c r="AH406" s="19" t="n"/>
+      <c r="AI406" s="19" t="n"/>
+      <c r="AJ406" s="19" t="n"/>
+      <c r="AK406" s="19" t="n"/>
+      <c r="AL406" s="19" t="n"/>
+      <c r="AM406" s="16" t="inlineStr">
+        <is>
+          <t>9 Stühle. Abgebildet ist ein Stuhl derselben Bauart aus TE02-13.</t>
+        </is>
+      </c>
+      <c r="AN406" s="22" t="inlineStr">
+        <is>
+          <t>OFFEN: Zu dieser Position fehlt ein eigenes Foto, und auf dem Erfassungsblatt steht hier "IKEA Stuehle weiss" ohne den Zusatz Kinder, bei TE02-13 dagegen "Kinderstuehle weiss" - beide mit Zustand gebraucht. Klaeren, ob das zwei verschiedene Groessen sind oder ob die Positionen zusammengehoeren.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A2:AN394"/>
+  <autoFilter ref="A2:AN406"/>
   <mergeCells count="7">
     <mergeCell ref="AI1:AL1"/>
     <mergeCell ref="V1:AD1"/>
@@ -49033,7 +50517,7 @@
     <mergeCell ref="AE1:AH1"/>
     <mergeCell ref="AM1:AN1"/>
   </mergeCells>
-  <conditionalFormatting sqref="Z3:Z394">
+  <conditionalFormatting sqref="Z3:Z406">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"reserviert"</formula>
     </cfRule>
@@ -49044,12 +50528,12 @@
       <formula>"verkauft"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I3:I394">
+  <conditionalFormatting sqref="I3:I406">
     <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
       <formula>"A"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P3:P394">
+  <conditionalFormatting sqref="P3:P406">
     <cfRule type="cellIs" priority="5" operator="equal" dxfId="4">
       <formula>"entfällt"</formula>
     </cfRule>
@@ -49140,7 +50624,7 @@
         </is>
       </c>
       <c r="B5" s="27">
-        <f>COUNTA(Artikelstamm!$A$3:$A$394)</f>
+        <f>COUNTA(Artikelstamm!$A$3:$A$406)</f>
         <v/>
       </c>
     </row>
@@ -49151,7 +50635,7 @@
         </is>
       </c>
       <c r="B6" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$394,"verfügbar")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$406,"verfügbar")</f>
         <v/>
       </c>
     </row>
@@ -49162,7 +50646,7 @@
         </is>
       </c>
       <c r="B7" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$394,"reserviert")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$406,"reserviert")</f>
         <v/>
       </c>
     </row>
@@ -49173,7 +50657,7 @@
         </is>
       </c>
       <c r="B8" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$394,"teilverkauft")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$406,"teilverkauft")</f>
         <v/>
       </c>
     </row>
@@ -49184,7 +50668,7 @@
         </is>
       </c>
       <c r="B9" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$394,"verkauft")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$406,"verkauft")</f>
         <v/>
       </c>
     </row>
@@ -49195,7 +50679,7 @@
         </is>
       </c>
       <c r="B10" s="27">
-        <f>SUM(Artikelstamm!$L$3:$L$394)</f>
+        <f>SUM(Artikelstamm!$L$3:$L$406)</f>
         <v/>
       </c>
     </row>
@@ -49206,7 +50690,7 @@
         </is>
       </c>
       <c r="B11" s="29">
-        <f>SUM(Artikelstamm!$U$3:$U$394)</f>
+        <f>SUM(Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -49224,7 +50708,7 @@
         </is>
       </c>
       <c r="B13" s="27">
-        <f>SUM(Artikelstamm!$K$3:$K$394)</f>
+        <f>SUM(Artikelstamm!$K$3:$K$406)</f>
         <v/>
       </c>
     </row>
@@ -49235,7 +50719,7 @@
         </is>
       </c>
       <c r="B14" s="30">
-        <f>SUMPRODUCT(Artikelstamm!$K$3:$K$394,Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT(Artikelstamm!$K$3:$K$406,Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
     </row>
@@ -49268,7 +50752,7 @@
         </is>
       </c>
       <c r="B17" s="30">
-        <f>SUMPRODUCT((Artikelstamm!$AJ$3:$AJ$394="bezahlt")*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AJ$3:$AJ$406="bezahlt")*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
     </row>
@@ -49297,7 +50781,7 @@
         </is>
       </c>
       <c r="B21" s="31">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$394,"*verkauft",Artikelstamm!$AI$3:$AI$394,"")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$406,"*verkauft",Artikelstamm!$AI$3:$AI$406,"")</f>
         <v/>
       </c>
     </row>
@@ -49308,7 +50792,7 @@
         </is>
       </c>
       <c r="B22" s="31">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$394,"*verkauft",Artikelstamm!$AJ$3:$AJ$394,"offen")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$406,"*verkauft",Artikelstamm!$AJ$3:$AJ$406,"offen")</f>
         <v/>
       </c>
     </row>
@@ -49319,7 +50803,7 @@
         </is>
       </c>
       <c r="B23" s="27">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$394,"reserviert",Artikelstamm!$AL$3:$AL$394,"")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$406,"reserviert",Artikelstamm!$AL$3:$AL$406,"")</f>
         <v/>
       </c>
     </row>
@@ -49330,7 +50814,7 @@
         </is>
       </c>
       <c r="B24" s="27">
-        <f>COUNTIFS(Artikelstamm!$S$3:$S$394,"")</f>
+        <f>COUNTIFS(Artikelstamm!$S$3:$S$406,"")</f>
         <v/>
       </c>
     </row>
@@ -49341,7 +50825,7 @@
         </is>
       </c>
       <c r="B25" s="27">
-        <f>COUNTIFS(Artikelstamm!$O$3:$O$394,"")</f>
+        <f>COUNTIFS(Artikelstamm!$O$3:$O$406,"")</f>
         <v/>
       </c>
     </row>
@@ -49381,15 +50865,15 @@
         </is>
       </c>
       <c r="B30" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$394,$A30)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$406,$A30)</f>
         <v/>
       </c>
       <c r="C30" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$394=$A30)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$406=$A30)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D30" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$394,$A30,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$406,$A30,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -49400,15 +50884,15 @@
         </is>
       </c>
       <c r="B31" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$394,$A31)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$406,$A31)</f>
         <v/>
       </c>
       <c r="C31" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$394=$A31)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$406=$A31)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D31" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$394,$A31,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$406,$A31,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -49419,15 +50903,15 @@
         </is>
       </c>
       <c r="B32" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$394,$A32)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$406,$A32)</f>
         <v/>
       </c>
       <c r="C32" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$394=$A32)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$406=$A32)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D32" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$394,$A32,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$406,$A32,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -49486,15 +50970,15 @@
         </is>
       </c>
       <c r="B37" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$394,$A37)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$406,$A37)</f>
         <v/>
       </c>
       <c r="C37" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$394=$A37)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$406=$A37)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D37" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$394,$A37,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$406,$A37,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -49505,15 +50989,15 @@
         </is>
       </c>
       <c r="B38" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$394,$A38)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$406,$A38)</f>
         <v/>
       </c>
       <c r="C38" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$394=$A38)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$406=$A38)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D38" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$394,$A38,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$406,$A38,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -49524,15 +51008,15 @@
         </is>
       </c>
       <c r="B39" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$394,$A39)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$406,$A39)</f>
         <v/>
       </c>
       <c r="C39" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$394=$A39)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$406=$A39)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D39" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$394,$A39,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$406,$A39,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -49543,15 +51027,15 @@
         </is>
       </c>
       <c r="B40" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$394,$A40)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$406,$A40)</f>
         <v/>
       </c>
       <c r="C40" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$394=$A40)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$406=$A40)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D40" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$394,$A40,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$406,$A40,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -49562,15 +51046,15 @@
         </is>
       </c>
       <c r="B41" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$394,$A41)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$406,$A41)</f>
         <v/>
       </c>
       <c r="C41" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$394=$A41)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$406=$A41)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D41" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$394,$A41,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$406,$A41,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -49581,15 +51065,15 @@
         </is>
       </c>
       <c r="B42" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$394,$A42)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$406,$A42)</f>
         <v/>
       </c>
       <c r="C42" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$394=$A42)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$406=$A42)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D42" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$394,$A42,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$406,$A42,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -49600,15 +51084,15 @@
         </is>
       </c>
       <c r="B43" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$394,$A43)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$406,$A43)</f>
         <v/>
       </c>
       <c r="C43" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$394=$A43)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$406=$A43)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D43" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$394,$A43,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$406,$A43,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -49619,15 +51103,15 @@
         </is>
       </c>
       <c r="B44" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$394,$A44)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$406,$A44)</f>
         <v/>
       </c>
       <c r="C44" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$394=$A44)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$406=$A44)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D44" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$394,$A44,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$406,$A44,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -49638,15 +51122,15 @@
         </is>
       </c>
       <c r="B45" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$394,$A45)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$406,$A45)</f>
         <v/>
       </c>
       <c r="C45" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$394=$A45)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$406=$A45)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D45" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$394,$A45,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$406,$A45,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -49657,15 +51141,15 @@
         </is>
       </c>
       <c r="B46" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$394,$A46)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$406,$A46)</f>
         <v/>
       </c>
       <c r="C46" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$394=$A46)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$406=$A46)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D46" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$394,$A46,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$406,$A46,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -49676,15 +51160,15 @@
         </is>
       </c>
       <c r="B47" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$394,$A47)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$406,$A47)</f>
         <v/>
       </c>
       <c r="C47" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$394=$A47)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$406=$A47)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D47" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$394,$A47,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$406,$A47,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -49695,15 +51179,15 @@
         </is>
       </c>
       <c r="B48" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$394,$A48)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$406,$A48)</f>
         <v/>
       </c>
       <c r="C48" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$394=$A48)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$406=$A48)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D48" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$394,$A48,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$406,$A48,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -49714,15 +51198,15 @@
         </is>
       </c>
       <c r="B49" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$394,$A49)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$406,$A49)</f>
         <v/>
       </c>
       <c r="C49" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$394=$A49)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$406=$A49)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D49" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$394,$A49,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$406,$A49,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -49733,15 +51217,15 @@
         </is>
       </c>
       <c r="B50" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$394,$A50)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$406,$A50)</f>
         <v/>
       </c>
       <c r="C50" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$394=$A50)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$406=$A50)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D50" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$394,$A50,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$406,$A50,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -49800,15 +51284,15 @@
         </is>
       </c>
       <c r="B55" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$394,$A55)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A55)</f>
         <v/>
       </c>
       <c r="C55" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$394=$A55)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A55)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D55" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$394,$A55,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A55,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -49819,15 +51303,15 @@
         </is>
       </c>
       <c r="B56" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$394,$A56)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A56)</f>
         <v/>
       </c>
       <c r="C56" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$394=$A56)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A56)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D56" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$394,$A56,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A56,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -49838,15 +51322,15 @@
         </is>
       </c>
       <c r="B57" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$394,$A57)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A57)</f>
         <v/>
       </c>
       <c r="C57" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$394=$A57)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A57)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D57" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$394,$A57,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A57,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -49857,15 +51341,15 @@
         </is>
       </c>
       <c r="B58" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$394,$A58)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A58)</f>
         <v/>
       </c>
       <c r="C58" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$394=$A58)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A58)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D58" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$394,$A58,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A58,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -49876,15 +51360,15 @@
         </is>
       </c>
       <c r="B59" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$394,$A59)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A59)</f>
         <v/>
       </c>
       <c r="C59" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$394=$A59)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A59)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D59" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$394,$A59,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A59,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -49895,15 +51379,15 @@
         </is>
       </c>
       <c r="B60" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$394,$A60)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A60)</f>
         <v/>
       </c>
       <c r="C60" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$394=$A60)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A60)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D60" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$394,$A60,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A60,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -49914,15 +51398,15 @@
         </is>
       </c>
       <c r="B61" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$394,$A61)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A61)</f>
         <v/>
       </c>
       <c r="C61" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$394=$A61)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A61)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D61" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$394,$A61,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A61,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -49933,15 +51417,15 @@
         </is>
       </c>
       <c r="B62" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$394,$A62)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A62)</f>
         <v/>
       </c>
       <c r="C62" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$394=$A62)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A62)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D62" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$394,$A62,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A62,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -49952,15 +51436,15 @@
         </is>
       </c>
       <c r="B63" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$394,$A63)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A63)</f>
         <v/>
       </c>
       <c r="C63" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$394=$A63)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A63)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D63" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$394,$A63,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A63,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -49971,15 +51455,15 @@
         </is>
       </c>
       <c r="B64" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$394,$A64)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A64)</f>
         <v/>
       </c>
       <c r="C64" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$394=$A64)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A64)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D64" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$394,$A64,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A64,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -49990,15 +51474,15 @@
         </is>
       </c>
       <c r="B65" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$394,$A65)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A65)</f>
         <v/>
       </c>
       <c r="C65" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$394=$A65)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A65)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D65" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$394,$A65,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A65,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -50009,15 +51493,15 @@
         </is>
       </c>
       <c r="B66" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$394,$A66)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A66)</f>
         <v/>
       </c>
       <c r="C66" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$394=$A66)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A66)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D66" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$394,$A66,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A66,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -50028,15 +51512,15 @@
         </is>
       </c>
       <c r="B67" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$394,$A67)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A67)</f>
         <v/>
       </c>
       <c r="C67" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$394=$A67)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A67)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D67" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$394,$A67,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A67,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -50047,15 +51531,15 @@
         </is>
       </c>
       <c r="B68" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$394,$A68)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A68)</f>
         <v/>
       </c>
       <c r="C68" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$394=$A68)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A68)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D68" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$394,$A68,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A68,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -50066,15 +51550,15 @@
         </is>
       </c>
       <c r="B69" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$394,$A69)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A69)</f>
         <v/>
       </c>
       <c r="C69" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$394=$A69)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A69)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D69" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$394,$A69,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A69,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -50085,15 +51569,15 @@
         </is>
       </c>
       <c r="B70" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$394,$A70)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A70)</f>
         <v/>
       </c>
       <c r="C70" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$394=$A70)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A70)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D70" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$394,$A70,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A70,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -50104,15 +51588,15 @@
         </is>
       </c>
       <c r="B71" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$394,$A71)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A71)</f>
         <v/>
       </c>
       <c r="C71" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$394=$A71)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A71)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D71" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$394,$A71,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A71,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -50123,15 +51607,15 @@
         </is>
       </c>
       <c r="B72" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$394,$A72)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A72)</f>
         <v/>
       </c>
       <c r="C72" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$394=$A72)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A72)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D72" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$394,$A72,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A72,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -50142,15 +51626,15 @@
         </is>
       </c>
       <c r="B73" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$394,$A73)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A73)</f>
         <v/>
       </c>
       <c r="C73" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$394=$A73)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A73)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D73" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$394,$A73,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A73,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -50161,15 +51645,15 @@
         </is>
       </c>
       <c r="B74" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$394,$A74)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A74)</f>
         <v/>
       </c>
       <c r="C74" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$394=$A74)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A74)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D74" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$394,$A74,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A74,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -50180,15 +51664,15 @@
         </is>
       </c>
       <c r="B75" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$394,$A75)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A75)</f>
         <v/>
       </c>
       <c r="C75" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$394=$A75)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A75)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D75" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$394,$A75,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A75,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -50199,15 +51683,15 @@
         </is>
       </c>
       <c r="B76" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$394,$A76)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A76)</f>
         <v/>
       </c>
       <c r="C76" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$394=$A76)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A76)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D76" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$394,$A76,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A76,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -50218,15 +51702,15 @@
         </is>
       </c>
       <c r="B77" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$394,$A77)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A77)</f>
         <v/>
       </c>
       <c r="C77" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$394=$A77)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A77)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D77" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$394,$A77,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A77,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -50237,15 +51721,15 @@
         </is>
       </c>
       <c r="B78" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$394,$A78)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A78)</f>
         <v/>
       </c>
       <c r="C78" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$394=$A78)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A78)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D78" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$394,$A78,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A78,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -50256,15 +51740,15 @@
         </is>
       </c>
       <c r="B79" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$394,$A79)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A79)</f>
         <v/>
       </c>
       <c r="C79" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$394=$A79)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A79)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D79" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$394,$A79,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A79,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -50275,15 +51759,15 @@
         </is>
       </c>
       <c r="B80" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$394,$A80)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A80)</f>
         <v/>
       </c>
       <c r="C80" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$394=$A80)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A80)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D80" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$394,$A80,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A80,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -50294,15 +51778,15 @@
         </is>
       </c>
       <c r="B81" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$394,$A81)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A81)</f>
         <v/>
       </c>
       <c r="C81" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$394=$A81)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A81)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D81" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$394,$A81,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A81,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -50313,15 +51797,15 @@
         </is>
       </c>
       <c r="B82" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$394,$A82)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A82)</f>
         <v/>
       </c>
       <c r="C82" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$394=$A82)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A82)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D82" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$394,$A82,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A82,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -50332,15 +51816,15 @@
         </is>
       </c>
       <c r="B83" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$394,$A83)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A83)</f>
         <v/>
       </c>
       <c r="C83" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$394=$A83)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A83)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D83" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$394,$A83,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A83,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -50351,15 +51835,15 @@
         </is>
       </c>
       <c r="B84" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$394,$A84)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A84)</f>
         <v/>
       </c>
       <c r="C84" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$394=$A84)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A84)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D84" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$394,$A84,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A84,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -50370,15 +51854,15 @@
         </is>
       </c>
       <c r="B85" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$394,$A85)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A85)</f>
         <v/>
       </c>
       <c r="C85" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$394=$A85)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A85)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D85" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$394,$A85,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A85,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -50389,15 +51873,15 @@
         </is>
       </c>
       <c r="B86" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$394,$A86)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A86)</f>
         <v/>
       </c>
       <c r="C86" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$394=$A86)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A86)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D86" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$394,$A86,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A86,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -50408,15 +51892,15 @@
         </is>
       </c>
       <c r="B87" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$394,$A87)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A87)</f>
         <v/>
       </c>
       <c r="C87" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$394=$A87)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A87)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
       <c r="D87" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$394,$A87,Artikelstamm!$U$3:$U$394)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A87,Artikelstamm!$U$3:$U$406)</f>
         <v/>
       </c>
     </row>
@@ -50470,11 +51954,11 @@
         </is>
       </c>
       <c r="B92" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$394,$A92)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$406,$A92)</f>
         <v/>
       </c>
       <c r="C92" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$394=$A92)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$406=$A92)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
     </row>
@@ -50485,11 +51969,11 @@
         </is>
       </c>
       <c r="B93" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$394,$A93)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$406,$A93)</f>
         <v/>
       </c>
       <c r="C93" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$394=$A93)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$406=$A93)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
     </row>
@@ -50500,11 +51984,11 @@
         </is>
       </c>
       <c r="B94" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$394,$A94)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$406,$A94)</f>
         <v/>
       </c>
       <c r="C94" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$394=$A94)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$406=$A94)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
     </row>
@@ -50515,11 +51999,11 @@
         </is>
       </c>
       <c r="B95" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$394,$A95)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$406,$A95)</f>
         <v/>
       </c>
       <c r="C95" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$394=$A95)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$406=$A95)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
     </row>
@@ -50530,11 +52014,11 @@
         </is>
       </c>
       <c r="B96" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$394,$A96)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$406,$A96)</f>
         <v/>
       </c>
       <c r="C96" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$394=$A96)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$406=$A96)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
     </row>
@@ -50545,11 +52029,11 @@
         </is>
       </c>
       <c r="B97" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$394,$A97)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$406,$A97)</f>
         <v/>
       </c>
       <c r="C97" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$394=$A97)*Artikelstamm!$K$3:$K$394*Artikelstamm!$AE$3:$AE$394)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$406=$A97)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
TE02 korrigiert; Fotos fuer GA01 aufbereitet
Rueckmeldungen der Nutzerin zu TE02:
  TE02-15 rote Tische: Foto F-514 (IMG_2472) zugeordnet
  "Stuehle rot/weiss" sind dieselben Artikel wie die Kinderstuehle:
    TE02-16 -> TE02-09  rot   10 -> 20 Stueck
    TE02-18 -> TE02-13  weiss  5 -> 14 Stueck
  Rattansessel, Teak-Klappstuehle und Bistro-Set bleiben draussen
  Biohort Freizeitbox: insgesamt 2 Stueck, die zweite steht auf der
    Dachterrasse - TE01-01 von 1 auf 2 Stueck

Fotos F-518 bis F-537 aus der Gartenanlage GA01 sind aufbereitet und
indiziert; die Artikel werden angelegt, sobald alle Fotos da sind.

Datenbasis 402 Positionen / 348 aktiv, pruefen.py 0 Fehler.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011yyfqhuiWGsaNy38oaNoGo
</commit_message>
<xml_diff>
--- a/ausgabe/01_Artikelstamm_kikripp.xlsx
+++ b/ausgabe/01_Artikelstamm_kikripp.xlsx
@@ -15,7 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Design" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Artikelstamm'!$A$2:$AN$406</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Artikelstamm'!$A$2:$AN$404</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1019,7 +1019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN406"/>
+  <dimension ref="A1:AN404"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -17565,7 +17565,7 @@
         </is>
       </c>
       <c r="J135" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K135" s="17" t="n"/>
       <c r="L135" s="18">
@@ -17644,7 +17644,7 @@
       <c r="AL135" s="19" t="n"/>
       <c r="AM135" s="16" t="inlineStr">
         <is>
-          <t>1 Box im Bild</t>
+          <t>2 Boxen: eine auf der Terrasse und eine auf der Dachterrasse. Die Box auf der Dachterrasse ist auf Foto F-108 zu sehen.</t>
         </is>
       </c>
       <c r="AN135" s="22" t="n"/>
@@ -49275,7 +49275,11 @@
         </is>
       </c>
       <c r="B397" s="15" t="n"/>
-      <c r="C397" s="15" t="n"/>
+      <c r="C397" s="15" t="inlineStr">
+        <is>
+          <t>TE02-16</t>
+        </is>
+      </c>
       <c r="D397" s="15" t="inlineStr">
         <is>
           <t>TE02</t>
@@ -49307,7 +49311,7 @@
         </is>
       </c>
       <c r="J397" s="17" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="K397" s="17" t="n"/>
       <c r="L397" s="18">
@@ -49321,7 +49325,7 @@
       </c>
       <c r="N397" s="15" t="inlineStr">
         <is>
-          <t>gut</t>
+          <t>gebraucht</t>
         </is>
       </c>
       <c r="O397" s="19" t="n"/>
@@ -49386,10 +49390,14 @@
       <c r="AL397" s="19" t="n"/>
       <c r="AM397" s="16" t="inlineStr">
         <is>
-          <t>10 Stühle – abgebildet ist einer davon.</t>
-        </is>
-      </c>
-      <c r="AN397" s="22" t="n"/>
+          <t>20 Stühle insgesamt. Zehn davon sind in gutem Zustand (auf dem Erfassungsblatt TE02-09), zehn weitere sind gebraucht (dort TE02-16) und auf Foto F-514 gestapelt zu sehen.</t>
+        </is>
+      </c>
+      <c r="AN397" s="22" t="inlineStr">
+        <is>
+          <t>Zusammengefasste Position aus zwei Nummern desselben Raums – Post-it-Nummer: TE02-16.</t>
+        </is>
+      </c>
     </row>
     <row r="398" ht="30" customHeight="1">
       <c r="A398" s="15" t="inlineStr">
@@ -49767,7 +49775,11 @@
         </is>
       </c>
       <c r="B401" s="15" t="n"/>
-      <c r="C401" s="15" t="n"/>
+      <c r="C401" s="15" t="inlineStr">
+        <is>
+          <t>TE02-18</t>
+        </is>
+      </c>
       <c r="D401" s="15" t="inlineStr">
         <is>
           <t>TE02</t>
@@ -49799,7 +49811,7 @@
         </is>
       </c>
       <c r="J401" s="17" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="K401" s="17" t="n"/>
       <c r="L401" s="18">
@@ -49878,10 +49890,14 @@
       <c r="AL401" s="19" t="n"/>
       <c r="AM401" s="16" t="inlineStr">
         <is>
-          <t>5 Stühle – abgebildet ist einer davon.</t>
-        </is>
-      </c>
-      <c r="AN401" s="22" t="n"/>
+          <t>14 Stühle insgesamt – abgebildet ist einer davon. Auf dem Erfassungsblatt stehen sie unter TE02-13 (5 Stück) und TE02-18 (9 Stück).</t>
+        </is>
+      </c>
+      <c r="AN401" s="22" t="inlineStr">
+        <is>
+          <t>Zusammengefasste Position aus zwei Nummern desselben Raums – Post-it-Nummer: TE02-18.</t>
+        </is>
+      </c>
     </row>
     <row r="402" ht="30" customHeight="1">
       <c r="A402" s="15" t="inlineStr">
@@ -50087,7 +50103,11 @@
           <t>nur Abholung</t>
         </is>
       </c>
-      <c r="W403" s="15" t="n"/>
+      <c r="W403" s="15" t="inlineStr">
+        <is>
+          <t>F-514</t>
+        </is>
+      </c>
       <c r="X403" s="19" t="inlineStr">
         <is>
           <t>ja</t>
@@ -50120,19 +50140,15 @@
       <c r="AL403" s="19" t="n"/>
       <c r="AM403" s="16" t="inlineStr">
         <is>
-          <t>3 Tische.</t>
-        </is>
-      </c>
-      <c r="AN403" s="22" t="inlineStr">
-        <is>
-          <t>OFFEN: Zu dieser Position fehlt ein Foto - von den roten Tischen ist keines dabei.</t>
-        </is>
-      </c>
+          <t>3 Tische. Auf dem Foto sind sie mit den roten Stühlen aus TE02-09 aufeinandergestellt.</t>
+        </is>
+      </c>
+      <c r="AN403" s="22" t="n"/>
     </row>
     <row r="404" ht="30" customHeight="1">
       <c r="A404" s="15" t="inlineStr">
         <is>
-          <t>TE02-16</t>
+          <t>TE02-17</t>
         </is>
       </c>
       <c r="B404" s="15" t="n"/>
@@ -50144,12 +50160,12 @@
       </c>
       <c r="E404" s="15" t="inlineStr">
         <is>
-          <t>IKEA Mammut Stuhl rot</t>
+          <t>IKEA Mammut Kindertisch weiß</t>
         </is>
       </c>
       <c r="F404" s="16" t="inlineStr">
         <is>
-          <t>Stuhl IKEA Mammut aus rotem Kunststoff mit runden Beinen und breiter Rückenlehne.</t>
+          <t>Rechteckiger Kindertisch IKEA Mammut aus weißem Kunststoff auf konischen Beinen. Die Platte ist fleckig und vom Wetter gezeichnet.</t>
         </is>
       </c>
       <c r="G404" s="15" t="inlineStr">
@@ -50168,7 +50184,7 @@
         </is>
       </c>
       <c r="J404" s="17" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="K404" s="17" t="n"/>
       <c r="L404" s="18">
@@ -50194,7 +50210,7 @@
       <c r="Q404" s="19" t="n"/>
       <c r="R404" s="20" t="n"/>
       <c r="S404" s="20" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="T404" s="19" t="inlineStr">
         <is>
@@ -50212,7 +50228,7 @@
       </c>
       <c r="W404" s="15" t="inlineStr">
         <is>
-          <t>F-514</t>
+          <t>F-513</t>
         </is>
       </c>
       <c r="X404" s="19" t="inlineStr">
@@ -50247,267 +50263,13 @@
       <c r="AL404" s="19" t="n"/>
       <c r="AM404" s="16" t="inlineStr">
         <is>
-          <t>10 Stühle. Auf dem Foto sind zwei davon gestapelt zu sehen.</t>
-        </is>
-      </c>
-      <c r="AN404" s="22" t="inlineStr">
-        <is>
-          <t>OFFEN: Auf dem Erfassungsblatt steht hier "IKEA Stuehle rot" ohne den Zusatz Kinder, bei TE02-09 dagegen "Kinderstuehle rot". Klaeren, ob das zwei verschiedene Groessen sind oder ob beide Positionen zusammengehoeren.</t>
-        </is>
-      </c>
-    </row>
-    <row r="405" ht="30" customHeight="1">
-      <c r="A405" s="15" t="inlineStr">
-        <is>
-          <t>TE02-17</t>
-        </is>
-      </c>
-      <c r="B405" s="15" t="n"/>
-      <c r="C405" s="15" t="n"/>
-      <c r="D405" s="15" t="inlineStr">
-        <is>
-          <t>TE02</t>
-        </is>
-      </c>
-      <c r="E405" s="15" t="inlineStr">
-        <is>
-          <t>IKEA Mammut Kindertisch weiß</t>
-        </is>
-      </c>
-      <c r="F405" s="16" t="inlineStr">
-        <is>
-          <t>Rechteckiger Kindertisch IKEA Mammut aus weißem Kunststoff auf konischen Beinen. Die Platte ist fleckig und vom Wetter gezeichnet.</t>
-        </is>
-      </c>
-      <c r="G405" s="15" t="inlineStr">
-        <is>
-          <t>Garten</t>
-        </is>
-      </c>
-      <c r="H405" s="15" t="inlineStr">
-        <is>
-          <t>Dachterrasse</t>
-        </is>
-      </c>
-      <c r="I405" s="15" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="J405" s="17" t="n">
-        <v>3</v>
-      </c>
-      <c r="K405" s="17" t="n"/>
-      <c r="L405" s="18">
-        <f>J405-IF(K405="",0,K405)</f>
-        <v/>
-      </c>
-      <c r="M405" s="15" t="inlineStr">
-        <is>
-          <t>Stück</t>
-        </is>
-      </c>
-      <c r="N405" s="15" t="inlineStr">
-        <is>
-          <t>gebraucht</t>
-        </is>
-      </c>
-      <c r="O405" s="19" t="n"/>
-      <c r="P405" s="19" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
-      <c r="Q405" s="19" t="n"/>
-      <c r="R405" s="20" t="n"/>
-      <c r="S405" s="20" t="n">
-        <v>20</v>
-      </c>
-      <c r="T405" s="19" t="inlineStr">
-        <is>
-          <t>VHB</t>
-        </is>
-      </c>
-      <c r="U405" s="21">
-        <f>L405*S405</f>
-        <v/>
-      </c>
-      <c r="V405" s="15" t="inlineStr">
-        <is>
-          <t>nur Abholung</t>
-        </is>
-      </c>
-      <c r="W405" s="15" t="inlineStr">
-        <is>
-          <t>F-513</t>
-        </is>
-      </c>
-      <c r="X405" s="19" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
-      <c r="Y405" s="19" t="n"/>
-      <c r="Z405" s="19" t="inlineStr">
-        <is>
-          <t>verfügbar</t>
-        </is>
-      </c>
-      <c r="AA405" s="19" t="inlineStr">
-        <is>
-          <t>IKEA</t>
-        </is>
-      </c>
-      <c r="AB405" s="19" t="n"/>
-      <c r="AC405" s="19" t="n"/>
-      <c r="AD405" s="19" t="n"/>
-      <c r="AE405" s="20" t="n"/>
-      <c r="AF405" s="21">
-        <f>IF(K405="","",K405*AE405)</f>
-        <v/>
-      </c>
-      <c r="AG405" s="19" t="n"/>
-      <c r="AH405" s="19" t="n"/>
-      <c r="AI405" s="19" t="n"/>
-      <c r="AJ405" s="19" t="n"/>
-      <c r="AK405" s="19" t="n"/>
-      <c r="AL405" s="19" t="n"/>
-      <c r="AM405" s="16" t="inlineStr">
-        <is>
           <t>3 Tische – abgebildet ist einer davon.</t>
         </is>
       </c>
-      <c r="AN405" s="22" t="n"/>
-    </row>
-    <row r="406" ht="30" customHeight="1">
-      <c r="A406" s="15" t="inlineStr">
-        <is>
-          <t>TE02-18</t>
-        </is>
-      </c>
-      <c r="B406" s="15" t="n"/>
-      <c r="C406" s="15" t="n"/>
-      <c r="D406" s="15" t="inlineStr">
-        <is>
-          <t>TE02</t>
-        </is>
-      </c>
-      <c r="E406" s="15" t="inlineStr">
-        <is>
-          <t>IKEA Mammut Stuhl weiß</t>
-        </is>
-      </c>
-      <c r="F406" s="16" t="inlineStr">
-        <is>
-          <t>Stuhl IKEA Mammut aus weißem Kunststoff mit runden Beinen und breiter Rückenlehne.</t>
-        </is>
-      </c>
-      <c r="G406" s="15" t="inlineStr">
-        <is>
-          <t>Garten</t>
-        </is>
-      </c>
-      <c r="H406" s="15" t="inlineStr">
-        <is>
-          <t>Dachterrasse</t>
-        </is>
-      </c>
-      <c r="I406" s="15" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="J406" s="17" t="n">
-        <v>9</v>
-      </c>
-      <c r="K406" s="17" t="n"/>
-      <c r="L406" s="18">
-        <f>J406-IF(K406="",0,K406)</f>
-        <v/>
-      </c>
-      <c r="M406" s="15" t="inlineStr">
-        <is>
-          <t>Stück</t>
-        </is>
-      </c>
-      <c r="N406" s="15" t="inlineStr">
-        <is>
-          <t>gebraucht</t>
-        </is>
-      </c>
-      <c r="O406" s="19" t="n"/>
-      <c r="P406" s="19" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
-      <c r="Q406" s="19" t="n"/>
-      <c r="R406" s="20" t="n"/>
-      <c r="S406" s="20" t="n">
-        <v>10</v>
-      </c>
-      <c r="T406" s="19" t="inlineStr">
-        <is>
-          <t>VHB</t>
-        </is>
-      </c>
-      <c r="U406" s="21">
-        <f>L406*S406</f>
-        <v/>
-      </c>
-      <c r="V406" s="15" t="inlineStr">
-        <is>
-          <t>nur Abholung</t>
-        </is>
-      </c>
-      <c r="W406" s="15" t="inlineStr">
-        <is>
-          <t>F-511</t>
-        </is>
-      </c>
-      <c r="X406" s="19" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
-      <c r="Y406" s="19" t="n"/>
-      <c r="Z406" s="19" t="inlineStr">
-        <is>
-          <t>verfügbar</t>
-        </is>
-      </c>
-      <c r="AA406" s="19" t="inlineStr">
-        <is>
-          <t>IKEA</t>
-        </is>
-      </c>
-      <c r="AB406" s="19" t="n"/>
-      <c r="AC406" s="19" t="n"/>
-      <c r="AD406" s="19" t="n"/>
-      <c r="AE406" s="20" t="n"/>
-      <c r="AF406" s="21">
-        <f>IF(K406="","",K406*AE406)</f>
-        <v/>
-      </c>
-      <c r="AG406" s="19" t="n"/>
-      <c r="AH406" s="19" t="n"/>
-      <c r="AI406" s="19" t="n"/>
-      <c r="AJ406" s="19" t="n"/>
-      <c r="AK406" s="19" t="n"/>
-      <c r="AL406" s="19" t="n"/>
-      <c r="AM406" s="16" t="inlineStr">
-        <is>
-          <t>9 Stühle. Abgebildet ist ein Stuhl derselben Bauart aus TE02-13.</t>
-        </is>
-      </c>
-      <c r="AN406" s="22" t="inlineStr">
-        <is>
-          <t>OFFEN: Zu dieser Position fehlt ein eigenes Foto, und auf dem Erfassungsblatt steht hier "IKEA Stuehle weiss" ohne den Zusatz Kinder, bei TE02-13 dagegen "Kinderstuehle weiss" - beide mit Zustand gebraucht. Klaeren, ob das zwei verschiedene Groessen sind oder ob die Positionen zusammengehoeren.</t>
-        </is>
-      </c>
+      <c r="AN404" s="22" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A2:AN406"/>
+  <autoFilter ref="A2:AN404"/>
   <mergeCells count="7">
     <mergeCell ref="AI1:AL1"/>
     <mergeCell ref="V1:AD1"/>
@@ -50517,7 +50279,7 @@
     <mergeCell ref="AE1:AH1"/>
     <mergeCell ref="AM1:AN1"/>
   </mergeCells>
-  <conditionalFormatting sqref="Z3:Z406">
+  <conditionalFormatting sqref="Z3:Z404">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"reserviert"</formula>
     </cfRule>
@@ -50528,12 +50290,12 @@
       <formula>"verkauft"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I3:I406">
+  <conditionalFormatting sqref="I3:I404">
     <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
       <formula>"A"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P3:P406">
+  <conditionalFormatting sqref="P3:P404">
     <cfRule type="cellIs" priority="5" operator="equal" dxfId="4">
       <formula>"entfällt"</formula>
     </cfRule>
@@ -50624,7 +50386,7 @@
         </is>
       </c>
       <c r="B5" s="27">
-        <f>COUNTA(Artikelstamm!$A$3:$A$406)</f>
+        <f>COUNTA(Artikelstamm!$A$3:$A$404)</f>
         <v/>
       </c>
     </row>
@@ -50635,7 +50397,7 @@
         </is>
       </c>
       <c r="B6" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$406,"verfügbar")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$404,"verfügbar")</f>
         <v/>
       </c>
     </row>
@@ -50646,7 +50408,7 @@
         </is>
       </c>
       <c r="B7" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$406,"reserviert")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$404,"reserviert")</f>
         <v/>
       </c>
     </row>
@@ -50657,7 +50419,7 @@
         </is>
       </c>
       <c r="B8" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$406,"teilverkauft")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$404,"teilverkauft")</f>
         <v/>
       </c>
     </row>
@@ -50668,7 +50430,7 @@
         </is>
       </c>
       <c r="B9" s="27">
-        <f>COUNTIF(Artikelstamm!$Z$3:$Z$406,"verkauft")</f>
+        <f>COUNTIF(Artikelstamm!$Z$3:$Z$404,"verkauft")</f>
         <v/>
       </c>
     </row>
@@ -50679,7 +50441,7 @@
         </is>
       </c>
       <c r="B10" s="27">
-        <f>SUM(Artikelstamm!$L$3:$L$406)</f>
+        <f>SUM(Artikelstamm!$L$3:$L$404)</f>
         <v/>
       </c>
     </row>
@@ -50690,7 +50452,7 @@
         </is>
       </c>
       <c r="B11" s="29">
-        <f>SUM(Artikelstamm!$U$3:$U$406)</f>
+        <f>SUM(Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -50708,7 +50470,7 @@
         </is>
       </c>
       <c r="B13" s="27">
-        <f>SUM(Artikelstamm!$K$3:$K$406)</f>
+        <f>SUM(Artikelstamm!$K$3:$K$404)</f>
         <v/>
       </c>
     </row>
@@ -50719,7 +50481,7 @@
         </is>
       </c>
       <c r="B14" s="30">
-        <f>SUMPRODUCT(Artikelstamm!$K$3:$K$406,Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT(Artikelstamm!$K$3:$K$404,Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
     </row>
@@ -50752,7 +50514,7 @@
         </is>
       </c>
       <c r="B17" s="30">
-        <f>SUMPRODUCT((Artikelstamm!$AJ$3:$AJ$406="bezahlt")*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AJ$3:$AJ$404="bezahlt")*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
     </row>
@@ -50781,7 +50543,7 @@
         </is>
       </c>
       <c r="B21" s="31">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$406,"*verkauft",Artikelstamm!$AI$3:$AI$406,"")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$404,"*verkauft",Artikelstamm!$AI$3:$AI$404,"")</f>
         <v/>
       </c>
     </row>
@@ -50792,7 +50554,7 @@
         </is>
       </c>
       <c r="B22" s="31">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$406,"*verkauft",Artikelstamm!$AJ$3:$AJ$406,"offen")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$404,"*verkauft",Artikelstamm!$AJ$3:$AJ$404,"offen")</f>
         <v/>
       </c>
     </row>
@@ -50803,7 +50565,7 @@
         </is>
       </c>
       <c r="B23" s="27">
-        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$406,"reserviert",Artikelstamm!$AL$3:$AL$406,"")</f>
+        <f>COUNTIFS(Artikelstamm!$Z$3:$Z$404,"reserviert",Artikelstamm!$AL$3:$AL$404,"")</f>
         <v/>
       </c>
     </row>
@@ -50814,7 +50576,7 @@
         </is>
       </c>
       <c r="B24" s="27">
-        <f>COUNTIFS(Artikelstamm!$S$3:$S$406,"")</f>
+        <f>COUNTIFS(Artikelstamm!$S$3:$S$404,"")</f>
         <v/>
       </c>
     </row>
@@ -50825,7 +50587,7 @@
         </is>
       </c>
       <c r="B25" s="27">
-        <f>COUNTIFS(Artikelstamm!$O$3:$O$406,"")</f>
+        <f>COUNTIFS(Artikelstamm!$O$3:$O$404,"")</f>
         <v/>
       </c>
     </row>
@@ -50865,15 +50627,15 @@
         </is>
       </c>
       <c r="B30" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$406,$A30)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$404,$A30)</f>
         <v/>
       </c>
       <c r="C30" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$406=$A30)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$404=$A30)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D30" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$406,$A30,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$404,$A30,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -50884,15 +50646,15 @@
         </is>
       </c>
       <c r="B31" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$406,$A31)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$404,$A31)</f>
         <v/>
       </c>
       <c r="C31" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$406=$A31)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$404=$A31)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D31" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$406,$A31,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$404,$A31,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -50903,15 +50665,15 @@
         </is>
       </c>
       <c r="B32" s="33">
-        <f>COUNTIF(Artikelstamm!$I$3:$I$406,$A32)</f>
+        <f>COUNTIF(Artikelstamm!$I$3:$I$404,$A32)</f>
         <v/>
       </c>
       <c r="C32" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$406=$A32)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$I$3:$I$404=$A32)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D32" s="34">
-        <f>SUMIF(Artikelstamm!$I$3:$I$406,$A32,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$I$3:$I$404,$A32,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -50970,15 +50732,15 @@
         </is>
       </c>
       <c r="B37" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$406,$A37)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$404,$A37)</f>
         <v/>
       </c>
       <c r="C37" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$406=$A37)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$404=$A37)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D37" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$406,$A37,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$404,$A37,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -50989,15 +50751,15 @@
         </is>
       </c>
       <c r="B38" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$406,$A38)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$404,$A38)</f>
         <v/>
       </c>
       <c r="C38" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$406=$A38)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$404=$A38)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D38" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$406,$A38,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$404,$A38,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51008,15 +50770,15 @@
         </is>
       </c>
       <c r="B39" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$406,$A39)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$404,$A39)</f>
         <v/>
       </c>
       <c r="C39" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$406=$A39)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$404=$A39)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D39" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$406,$A39,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$404,$A39,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51027,15 +50789,15 @@
         </is>
       </c>
       <c r="B40" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$406,$A40)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$404,$A40)</f>
         <v/>
       </c>
       <c r="C40" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$406=$A40)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$404=$A40)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D40" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$406,$A40,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$404,$A40,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51046,15 +50808,15 @@
         </is>
       </c>
       <c r="B41" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$406,$A41)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$404,$A41)</f>
         <v/>
       </c>
       <c r="C41" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$406=$A41)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$404=$A41)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D41" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$406,$A41,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$404,$A41,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51065,15 +50827,15 @@
         </is>
       </c>
       <c r="B42" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$406,$A42)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$404,$A42)</f>
         <v/>
       </c>
       <c r="C42" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$406=$A42)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$404=$A42)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D42" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$406,$A42,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$404,$A42,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51084,15 +50846,15 @@
         </is>
       </c>
       <c r="B43" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$406,$A43)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$404,$A43)</f>
         <v/>
       </c>
       <c r="C43" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$406=$A43)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$404=$A43)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D43" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$406,$A43,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$404,$A43,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51103,15 +50865,15 @@
         </is>
       </c>
       <c r="B44" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$406,$A44)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$404,$A44)</f>
         <v/>
       </c>
       <c r="C44" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$406=$A44)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$404=$A44)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D44" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$406,$A44,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$404,$A44,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51122,15 +50884,15 @@
         </is>
       </c>
       <c r="B45" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$406,$A45)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$404,$A45)</f>
         <v/>
       </c>
       <c r="C45" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$406=$A45)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$404=$A45)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D45" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$406,$A45,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$404,$A45,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51141,15 +50903,15 @@
         </is>
       </c>
       <c r="B46" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$406,$A46)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$404,$A46)</f>
         <v/>
       </c>
       <c r="C46" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$406=$A46)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$404=$A46)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D46" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$406,$A46,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$404,$A46,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51160,15 +50922,15 @@
         </is>
       </c>
       <c r="B47" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$406,$A47)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$404,$A47)</f>
         <v/>
       </c>
       <c r="C47" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$406=$A47)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$404=$A47)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D47" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$406,$A47,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$404,$A47,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51179,15 +50941,15 @@
         </is>
       </c>
       <c r="B48" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$406,$A48)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$404,$A48)</f>
         <v/>
       </c>
       <c r="C48" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$406=$A48)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$404=$A48)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D48" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$406,$A48,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$404,$A48,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51198,15 +50960,15 @@
         </is>
       </c>
       <c r="B49" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$406,$A49)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$404,$A49)</f>
         <v/>
       </c>
       <c r="C49" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$406=$A49)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$404=$A49)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D49" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$406,$A49,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$404,$A49,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51217,15 +50979,15 @@
         </is>
       </c>
       <c r="B50" s="33">
-        <f>COUNTIF(Artikelstamm!$G$3:$G$406,$A50)</f>
+        <f>COUNTIF(Artikelstamm!$G$3:$G$404,$A50)</f>
         <v/>
       </c>
       <c r="C50" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$406=$A50)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$G$3:$G$404=$A50)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D50" s="34">
-        <f>SUMIF(Artikelstamm!$G$3:$G$406,$A50,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$G$3:$G$404,$A50,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51284,15 +51046,15 @@
         </is>
       </c>
       <c r="B55" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A55)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$404,$A55)</f>
         <v/>
       </c>
       <c r="C55" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A55)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$404=$A55)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D55" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A55,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$404,$A55,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51303,15 +51065,15 @@
         </is>
       </c>
       <c r="B56" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A56)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$404,$A56)</f>
         <v/>
       </c>
       <c r="C56" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A56)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$404=$A56)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D56" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A56,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$404,$A56,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51322,15 +51084,15 @@
         </is>
       </c>
       <c r="B57" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A57)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$404,$A57)</f>
         <v/>
       </c>
       <c r="C57" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A57)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$404=$A57)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D57" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A57,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$404,$A57,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51341,15 +51103,15 @@
         </is>
       </c>
       <c r="B58" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A58)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$404,$A58)</f>
         <v/>
       </c>
       <c r="C58" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A58)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$404=$A58)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D58" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A58,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$404,$A58,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51360,15 +51122,15 @@
         </is>
       </c>
       <c r="B59" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A59)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$404,$A59)</f>
         <v/>
       </c>
       <c r="C59" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A59)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$404=$A59)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D59" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A59,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$404,$A59,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51379,15 +51141,15 @@
         </is>
       </c>
       <c r="B60" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A60)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$404,$A60)</f>
         <v/>
       </c>
       <c r="C60" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A60)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$404=$A60)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D60" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A60,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$404,$A60,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51398,15 +51160,15 @@
         </is>
       </c>
       <c r="B61" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A61)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$404,$A61)</f>
         <v/>
       </c>
       <c r="C61" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A61)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$404=$A61)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D61" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A61,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$404,$A61,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51417,15 +51179,15 @@
         </is>
       </c>
       <c r="B62" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A62)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$404,$A62)</f>
         <v/>
       </c>
       <c r="C62" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A62)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$404=$A62)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D62" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A62,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$404,$A62,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51436,15 +51198,15 @@
         </is>
       </c>
       <c r="B63" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A63)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$404,$A63)</f>
         <v/>
       </c>
       <c r="C63" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A63)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$404=$A63)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D63" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A63,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$404,$A63,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51455,15 +51217,15 @@
         </is>
       </c>
       <c r="B64" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A64)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$404,$A64)</f>
         <v/>
       </c>
       <c r="C64" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A64)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$404=$A64)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D64" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A64,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$404,$A64,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51474,15 +51236,15 @@
         </is>
       </c>
       <c r="B65" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A65)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$404,$A65)</f>
         <v/>
       </c>
       <c r="C65" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A65)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$404=$A65)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D65" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A65,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$404,$A65,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51493,15 +51255,15 @@
         </is>
       </c>
       <c r="B66" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A66)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$404,$A66)</f>
         <v/>
       </c>
       <c r="C66" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A66)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$404=$A66)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D66" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A66,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$404,$A66,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51512,15 +51274,15 @@
         </is>
       </c>
       <c r="B67" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A67)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$404,$A67)</f>
         <v/>
       </c>
       <c r="C67" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A67)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$404=$A67)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D67" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A67,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$404,$A67,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51531,15 +51293,15 @@
         </is>
       </c>
       <c r="B68" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A68)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$404,$A68)</f>
         <v/>
       </c>
       <c r="C68" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A68)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$404=$A68)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D68" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A68,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$404,$A68,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51550,15 +51312,15 @@
         </is>
       </c>
       <c r="B69" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A69)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$404,$A69)</f>
         <v/>
       </c>
       <c r="C69" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A69)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$404=$A69)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D69" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A69,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$404,$A69,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51569,15 +51331,15 @@
         </is>
       </c>
       <c r="B70" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A70)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$404,$A70)</f>
         <v/>
       </c>
       <c r="C70" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A70)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$404=$A70)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D70" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A70,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$404,$A70,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51588,15 +51350,15 @@
         </is>
       </c>
       <c r="B71" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A71)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$404,$A71)</f>
         <v/>
       </c>
       <c r="C71" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A71)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$404=$A71)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D71" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A71,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$404,$A71,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51607,15 +51369,15 @@
         </is>
       </c>
       <c r="B72" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A72)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$404,$A72)</f>
         <v/>
       </c>
       <c r="C72" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A72)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$404=$A72)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D72" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A72,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$404,$A72,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51626,15 +51388,15 @@
         </is>
       </c>
       <c r="B73" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A73)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$404,$A73)</f>
         <v/>
       </c>
       <c r="C73" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A73)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$404=$A73)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D73" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A73,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$404,$A73,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51645,15 +51407,15 @@
         </is>
       </c>
       <c r="B74" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A74)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$404,$A74)</f>
         <v/>
       </c>
       <c r="C74" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A74)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$404=$A74)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D74" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A74,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$404,$A74,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51664,15 +51426,15 @@
         </is>
       </c>
       <c r="B75" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A75)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$404,$A75)</f>
         <v/>
       </c>
       <c r="C75" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A75)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$404=$A75)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D75" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A75,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$404,$A75,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51683,15 +51445,15 @@
         </is>
       </c>
       <c r="B76" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A76)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$404,$A76)</f>
         <v/>
       </c>
       <c r="C76" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A76)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$404=$A76)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D76" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A76,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$404,$A76,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51702,15 +51464,15 @@
         </is>
       </c>
       <c r="B77" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A77)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$404,$A77)</f>
         <v/>
       </c>
       <c r="C77" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A77)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$404=$A77)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D77" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A77,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$404,$A77,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51721,15 +51483,15 @@
         </is>
       </c>
       <c r="B78" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A78)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$404,$A78)</f>
         <v/>
       </c>
       <c r="C78" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A78)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$404=$A78)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D78" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A78,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$404,$A78,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51740,15 +51502,15 @@
         </is>
       </c>
       <c r="B79" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A79)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$404,$A79)</f>
         <v/>
       </c>
       <c r="C79" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A79)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$404=$A79)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D79" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A79,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$404,$A79,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51759,15 +51521,15 @@
         </is>
       </c>
       <c r="B80" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A80)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$404,$A80)</f>
         <v/>
       </c>
       <c r="C80" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A80)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$404=$A80)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D80" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A80,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$404,$A80,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51778,15 +51540,15 @@
         </is>
       </c>
       <c r="B81" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A81)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$404,$A81)</f>
         <v/>
       </c>
       <c r="C81" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A81)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$404=$A81)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D81" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A81,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$404,$A81,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51797,15 +51559,15 @@
         </is>
       </c>
       <c r="B82" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A82)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$404,$A82)</f>
         <v/>
       </c>
       <c r="C82" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A82)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$404=$A82)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D82" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A82,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$404,$A82,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51816,15 +51578,15 @@
         </is>
       </c>
       <c r="B83" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A83)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$404,$A83)</f>
         <v/>
       </c>
       <c r="C83" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A83)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$404=$A83)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D83" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A83,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$404,$A83,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51835,15 +51597,15 @@
         </is>
       </c>
       <c r="B84" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A84)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$404,$A84)</f>
         <v/>
       </c>
       <c r="C84" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A84)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$404=$A84)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D84" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A84,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$404,$A84,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51854,15 +51616,15 @@
         </is>
       </c>
       <c r="B85" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A85)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$404,$A85)</f>
         <v/>
       </c>
       <c r="C85" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A85)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$404=$A85)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D85" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A85,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$404,$A85,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51873,15 +51635,15 @@
         </is>
       </c>
       <c r="B86" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A86)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$404,$A86)</f>
         <v/>
       </c>
       <c r="C86" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A86)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$404=$A86)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D86" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A86,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$404,$A86,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51892,15 +51654,15 @@
         </is>
       </c>
       <c r="B87" s="33">
-        <f>COUNTIF(Artikelstamm!$H$3:$H$406,$A87)</f>
+        <f>COUNTIF(Artikelstamm!$H$3:$H$404,$A87)</f>
         <v/>
       </c>
       <c r="C87" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$406=$A87)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$H$3:$H$404=$A87)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
       <c r="D87" s="34">
-        <f>SUMIF(Artikelstamm!$H$3:$H$406,$A87,Artikelstamm!$U$3:$U$406)</f>
+        <f>SUMIF(Artikelstamm!$H$3:$H$404,$A87,Artikelstamm!$U$3:$U$404)</f>
         <v/>
       </c>
     </row>
@@ -51954,11 +51716,11 @@
         </is>
       </c>
       <c r="B92" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$406,$A92)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$404,$A92)</f>
         <v/>
       </c>
       <c r="C92" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$406=$A92)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$404=$A92)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
     </row>
@@ -51969,11 +51731,11 @@
         </is>
       </c>
       <c r="B93" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$406,$A93)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$404,$A93)</f>
         <v/>
       </c>
       <c r="C93" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$406=$A93)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$404=$A93)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
     </row>
@@ -51984,11 +51746,11 @@
         </is>
       </c>
       <c r="B94" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$406,$A94)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$404,$A94)</f>
         <v/>
       </c>
       <c r="C94" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$406=$A94)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$404=$A94)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
     </row>
@@ -51999,11 +51761,11 @@
         </is>
       </c>
       <c r="B95" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$406,$A95)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$404,$A95)</f>
         <v/>
       </c>
       <c r="C95" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$406=$A95)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$404=$A95)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
     </row>
@@ -52014,11 +51776,11 @@
         </is>
       </c>
       <c r="B96" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$406,$A96)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$404,$A96)</f>
         <v/>
       </c>
       <c r="C96" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$406=$A96)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$404=$A96)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
     </row>
@@ -52029,11 +51791,11 @@
         </is>
       </c>
       <c r="B97" s="33">
-        <f>COUNTIF(Artikelstamm!$AC$3:$AC$406,$A97)</f>
+        <f>COUNTIF(Artikelstamm!$AC$3:$AC$404,$A97)</f>
         <v/>
       </c>
       <c r="C97" s="34">
-        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$406=$A97)*Artikelstamm!$K$3:$K$406*Artikelstamm!$AE$3:$AE$406)</f>
+        <f>SUMPRODUCT((Artikelstamm!$AC$3:$AC$404=$A97)*Artikelstamm!$K$3:$K$404*Artikelstamm!$AE$3:$AE$404)</f>
         <v/>
       </c>
     </row>

</xml_diff>